<commit_message>
Inicio de modificaciones para la creacion de Exp_Controller
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D78780-0884-4D38-B0D3-793A5EA3748D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0ED791-A8C8-49FA-9127-CD4D27FA30B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="205">
   <si>
     <t>OpCode</t>
   </si>
@@ -630,13 +630,34 @@
   </si>
   <si>
     <t>Se activa cuando se requiere llamar al kernel, o regresar del kernel</t>
+  </si>
+  <si>
+    <t>Alignment Fault</t>
+  </si>
+  <si>
+    <t>Error de aliniamiento en memoria, los accesos deben terminar en 00</t>
+  </si>
+  <si>
+    <t>Flags de paginas</t>
+  </si>
+  <si>
+    <t>Present</t>
+  </si>
+  <si>
+    <t>ReadOnly</t>
+  </si>
+  <si>
+    <t>KernelOnly</t>
+  </si>
+  <si>
+    <t>Global</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -653,6 +674,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1622,7 +1651,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="180">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1882,6 +1911,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1957,6 +1989,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1966,21 +2004,39 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1990,6 +2046,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2005,67 +2097,7 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -2153,6 +2185,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2444,7 +2479,8 @@
     <col min="5" max="6" width="19.85546875" style="15" customWidth="1"/>
     <col min="7" max="10" width="13.85546875" style="15" customWidth="1"/>
     <col min="11" max="11" width="13.5703125" style="15" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="9.140625" style="15"/>
+    <col min="12" max="12" width="9.140625" style="15"/>
+    <col min="13" max="13" width="13" style="15" customWidth="1"/>
     <col min="14" max="14" width="22.28515625" style="15" customWidth="1"/>
     <col min="15" max="15" width="18.7109375" style="15" customWidth="1"/>
     <col min="16" max="16" width="20" style="15" customWidth="1"/>
@@ -2461,62 +2497,62 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="140" t="s">
+      <c r="B2" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="126" t="s">
+      <c r="C2" s="147" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="127"/>
-      <c r="E2" s="128" t="s">
+      <c r="D2" s="148"/>
+      <c r="E2" s="127" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="128"/>
-      <c r="G2" s="129" t="s">
+      <c r="F2" s="127"/>
+      <c r="G2" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="128"/>
-      <c r="I2" s="128" t="s">
+      <c r="H2" s="127"/>
+      <c r="I2" s="127" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="128"/>
-      <c r="K2" s="133" t="s">
+      <c r="J2" s="127"/>
+      <c r="K2" s="126" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="128"/>
-      <c r="M2" s="128"/>
-      <c r="N2" s="128"/>
-      <c r="O2" s="128"/>
-      <c r="P2" s="134"/>
-      <c r="R2" s="153" t="s">
+      <c r="L2" s="127"/>
+      <c r="M2" s="127"/>
+      <c r="N2" s="127"/>
+      <c r="O2" s="127"/>
+      <c r="P2" s="128"/>
+      <c r="R2" s="154" t="s">
         <v>66</v>
       </c>
-      <c r="S2" s="88" t="s">
+      <c r="S2" s="89" t="s">
         <v>67</v>
       </c>
-      <c r="T2" s="157" t="s">
+      <c r="T2" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="158"/>
-      <c r="V2" s="158"/>
-      <c r="W2" s="158"/>
-      <c r="X2" s="158"/>
-      <c r="Y2" s="158"/>
-      <c r="Z2" s="158"/>
-      <c r="AA2" s="158"/>
-      <c r="AB2" s="158" t="s">
+      <c r="U2" s="159"/>
+      <c r="V2" s="159"/>
+      <c r="W2" s="159"/>
+      <c r="X2" s="159"/>
+      <c r="Y2" s="159"/>
+      <c r="Z2" s="159"/>
+      <c r="AA2" s="159"/>
+      <c r="AB2" s="159" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="158"/>
-      <c r="AD2" s="158"/>
-      <c r="AE2" s="158"/>
-      <c r="AF2" s="158"/>
-      <c r="AG2" s="158"/>
-      <c r="AH2" s="158"/>
-      <c r="AI2" s="159"/>
+      <c r="AC2" s="159"/>
+      <c r="AD2" s="159"/>
+      <c r="AE2" s="159"/>
+      <c r="AF2" s="159"/>
+      <c r="AG2" s="159"/>
+      <c r="AH2" s="159"/>
+      <c r="AI2" s="160"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="141"/>
+      <c r="B3" s="136"/>
       <c r="C3" s="16" t="s">
         <v>80</v>
       </c>
@@ -2541,21 +2577,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="123"/>
-      <c r="L3" s="124"/>
-      <c r="M3" s="124"/>
-      <c r="N3" s="124"/>
-      <c r="O3" s="124"/>
-      <c r="P3" s="125"/>
-      <c r="R3" s="154"/>
-      <c r="S3" s="151"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="145"/>
+      <c r="M3" s="145"/>
+      <c r="N3" s="145"/>
+      <c r="O3" s="145"/>
+      <c r="P3" s="146"/>
+      <c r="R3" s="155"/>
+      <c r="S3" s="152"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="112" t="s">
+      <c r="U3" s="115" t="s">
         <v>84</v>
       </c>
-      <c r="V3" s="112"/>
+      <c r="V3" s="115"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -2568,10 +2604,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="156" t="s">
+      <c r="AA3" s="157" t="s">
         <v>75</v>
       </c>
-      <c r="AB3" s="156"/>
+      <c r="AB3" s="157"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -2595,21 +2631,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="142"/>
+      <c r="B4" s="137"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="113" t="s">
+      <c r="E4" s="116" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="120"/>
-      <c r="G4" s="120"/>
-      <c r="H4" s="120"/>
-      <c r="I4" s="120"/>
-      <c r="J4" s="121"/>
+      <c r="F4" s="129"/>
+      <c r="G4" s="129"/>
+      <c r="H4" s="129"/>
+      <c r="I4" s="129"/>
+      <c r="J4" s="130"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -2619,20 +2655,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="113" t="s">
+      <c r="N4" s="116" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="120"/>
-      <c r="P4" s="121"/>
-      <c r="R4" s="155"/>
-      <c r="S4" s="152"/>
+      <c r="O4" s="129"/>
+      <c r="P4" s="130"/>
+      <c r="R4" s="156"/>
+      <c r="S4" s="153"/>
       <c r="T4" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="U4" s="113" t="s">
+      <c r="U4" s="116" t="s">
         <v>76</v>
       </c>
-      <c r="V4" s="114"/>
+      <c r="V4" s="117"/>
       <c r="W4" s="7" t="s">
         <v>72</v>
       </c>
@@ -2645,10 +2681,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="113" t="s">
+      <c r="AA4" s="116" t="s">
         <v>73</v>
       </c>
-      <c r="AB4" s="114"/>
+      <c r="AB4" s="117"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -2680,22 +2716,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="137"/>
-      <c r="F5" s="138"/>
-      <c r="G5" s="138"/>
-      <c r="H5" s="138"/>
-      <c r="I5" s="138"/>
-      <c r="J5" s="139"/>
+      <c r="E5" s="132"/>
+      <c r="F5" s="133"/>
+      <c r="G5" s="133"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="133"/>
+      <c r="J5" s="134"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="122" t="s">
+      <c r="N5" s="131" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="89"/>
-      <c r="P5" s="90"/>
+      <c r="O5" s="90"/>
+      <c r="P5" s="91"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -2705,10 +2741,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="117" t="s">
+      <c r="U5" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V5" s="118"/>
+      <c r="V5" s="119"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -2721,10 +2757,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="117" t="s">
+      <c r="AA5" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB5" s="118"/>
+      <c r="AB5" s="119"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -2756,12 +2792,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="136"/>
-      <c r="F6" s="131"/>
-      <c r="G6" s="131"/>
-      <c r="H6" s="131"/>
-      <c r="I6" s="131"/>
-      <c r="J6" s="132"/>
+      <c r="E6" s="124"/>
+      <c r="F6" s="122"/>
+      <c r="G6" s="122"/>
+      <c r="H6" s="122"/>
+      <c r="I6" s="122"/>
+      <c r="J6" s="123"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -2769,11 +2805,11 @@
         <v>156</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="119" t="s">
+      <c r="N6" s="125" t="s">
         <v>96</v>
       </c>
-      <c r="O6" s="91"/>
-      <c r="P6" s="92"/>
+      <c r="O6" s="92"/>
+      <c r="P6" s="93"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -2783,10 +2819,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="115" t="s">
+      <c r="U6" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V6" s="116"/>
+      <c r="V6" s="114"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -2799,10 +2835,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="115" t="s">
+      <c r="AA6" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB6" s="116"/>
+      <c r="AB6" s="114"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -2843,9 +2879,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="130"/>
-      <c r="I7" s="131"/>
-      <c r="J7" s="132"/>
+      <c r="H7" s="121"/>
+      <c r="I7" s="122"/>
+      <c r="J7" s="123"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -2853,11 +2889,11 @@
       <c r="M7" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N7" s="119" t="s">
+      <c r="N7" s="125" t="s">
         <v>53</v>
       </c>
-      <c r="O7" s="91"/>
-      <c r="P7" s="92"/>
+      <c r="O7" s="92"/>
+      <c r="P7" s="93"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -2867,10 +2903,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="115" t="s">
+      <c r="U7" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V7" s="116"/>
+      <c r="V7" s="114"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -2883,10 +2919,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="115" t="s">
+      <c r="AA7" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB7" s="116"/>
+      <c r="AB7" s="114"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -2927,9 +2963,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="130"/>
-      <c r="I8" s="131"/>
-      <c r="J8" s="132"/>
+      <c r="H8" s="121"/>
+      <c r="I8" s="122"/>
+      <c r="J8" s="123"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -2937,11 +2973,11 @@
       <c r="M8" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N8" s="119" t="s">
+      <c r="N8" s="125" t="s">
         <v>54</v>
       </c>
-      <c r="O8" s="91"/>
-      <c r="P8" s="92"/>
+      <c r="O8" s="92"/>
+      <c r="P8" s="93"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -2951,10 +2987,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="115" t="s">
+      <c r="U8" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V8" s="116"/>
+      <c r="V8" s="114"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -2967,10 +3003,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="115" t="s">
+      <c r="AA8" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB8" s="116"/>
+      <c r="AB8" s="114"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -3011,9 +3047,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="130"/>
-      <c r="I9" s="131"/>
-      <c r="J9" s="132"/>
+      <c r="H9" s="121"/>
+      <c r="I9" s="122"/>
+      <c r="J9" s="123"/>
       <c r="K9" s="37" t="s">
         <v>48</v>
       </c>
@@ -3021,11 +3057,11 @@
       <c r="M9" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N9" s="119" t="s">
+      <c r="N9" s="125" t="s">
         <v>55</v>
       </c>
-      <c r="O9" s="91"/>
-      <c r="P9" s="92"/>
+      <c r="O9" s="92"/>
+      <c r="P9" s="93"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -3035,10 +3071,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="115" t="s">
+      <c r="U9" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V9" s="116"/>
+      <c r="V9" s="114"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -3051,10 +3087,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="115" t="s">
+      <c r="AA9" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB9" s="116"/>
+      <c r="AB9" s="114"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -3095,9 +3131,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="130"/>
-      <c r="I10" s="131"/>
-      <c r="J10" s="132"/>
+      <c r="H10" s="121"/>
+      <c r="I10" s="122"/>
+      <c r="J10" s="123"/>
       <c r="K10" s="37" t="s">
         <v>49</v>
       </c>
@@ -3105,11 +3141,11 @@
       <c r="M10" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N10" s="119" t="s">
+      <c r="N10" s="125" t="s">
         <v>56</v>
       </c>
-      <c r="O10" s="91"/>
-      <c r="P10" s="92"/>
+      <c r="O10" s="92"/>
+      <c r="P10" s="93"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -3119,10 +3155,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="115" t="s">
+      <c r="U10" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V10" s="116"/>
+      <c r="V10" s="114"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -3135,10 +3171,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="115" t="s">
+      <c r="AA10" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB10" s="116"/>
+      <c r="AB10" s="114"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -3179,9 +3215,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="130"/>
-      <c r="I11" s="131"/>
-      <c r="J11" s="132"/>
+      <c r="H11" s="121"/>
+      <c r="I11" s="122"/>
+      <c r="J11" s="123"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -3189,11 +3225,11 @@
       <c r="M11" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N11" s="119" t="s">
+      <c r="N11" s="125" t="s">
         <v>57</v>
       </c>
-      <c r="O11" s="91"/>
-      <c r="P11" s="92"/>
+      <c r="O11" s="92"/>
+      <c r="P11" s="93"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -3203,10 +3239,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="115" t="s">
+      <c r="U11" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V11" s="116"/>
+      <c r="V11" s="114"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -3219,10 +3255,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="115" t="s">
+      <c r="AA11" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB11" s="116"/>
+      <c r="AB11" s="114"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -3263,9 +3299,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="130"/>
-      <c r="I12" s="131"/>
-      <c r="J12" s="132"/>
+      <c r="H12" s="121"/>
+      <c r="I12" s="122"/>
+      <c r="J12" s="123"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -3273,11 +3309,11 @@
       <c r="M12" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N12" s="119" t="s">
+      <c r="N12" s="125" t="s">
         <v>58</v>
       </c>
-      <c r="O12" s="91"/>
-      <c r="P12" s="92"/>
+      <c r="O12" s="92"/>
+      <c r="P12" s="93"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -3287,10 +3323,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="115" t="s">
+      <c r="U12" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V12" s="116"/>
+      <c r="V12" s="114"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -3303,10 +3339,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="115" t="s">
+      <c r="AA12" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB12" s="116"/>
+      <c r="AB12" s="114"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -3347,9 +3383,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="130"/>
-      <c r="I13" s="131"/>
-      <c r="J13" s="132"/>
+      <c r="H13" s="121"/>
+      <c r="I13" s="122"/>
+      <c r="J13" s="123"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -3357,11 +3393,11 @@
       <c r="M13" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N13" s="119" t="s">
+      <c r="N13" s="125" t="s">
         <v>59</v>
       </c>
-      <c r="O13" s="91"/>
-      <c r="P13" s="92"/>
+      <c r="O13" s="92"/>
+      <c r="P13" s="93"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -3371,10 +3407,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="115" t="s">
+      <c r="U13" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V13" s="116"/>
+      <c r="V13" s="114"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -3387,10 +3423,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="115" t="s">
+      <c r="AA13" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB13" s="116"/>
+      <c r="AB13" s="114"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -3431,9 +3467,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="130"/>
-      <c r="I14" s="131"/>
-      <c r="J14" s="132"/>
+      <c r="H14" s="121"/>
+      <c r="I14" s="122"/>
+      <c r="J14" s="123"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -3441,11 +3477,11 @@
       <c r="M14" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N14" s="119" t="s">
+      <c r="N14" s="125" t="s">
         <v>60</v>
       </c>
-      <c r="O14" s="91"/>
-      <c r="P14" s="92"/>
+      <c r="O14" s="92"/>
+      <c r="P14" s="93"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -3455,10 +3491,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="115" t="s">
+      <c r="U14" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V14" s="116"/>
+      <c r="V14" s="114"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -3471,10 +3507,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="115" t="s">
+      <c r="AA14" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB14" s="116"/>
+      <c r="AB14" s="114"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -3515,9 +3551,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="130"/>
-      <c r="I15" s="131"/>
-      <c r="J15" s="132"/>
+      <c r="H15" s="121"/>
+      <c r="I15" s="122"/>
+      <c r="J15" s="123"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -3525,11 +3561,11 @@
       <c r="M15" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N15" s="119" t="s">
+      <c r="N15" s="125" t="s">
         <v>61</v>
       </c>
-      <c r="O15" s="91"/>
-      <c r="P15" s="92"/>
+      <c r="O15" s="92"/>
+      <c r="P15" s="93"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -3539,10 +3575,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="115" t="s">
+      <c r="U15" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V15" s="116"/>
+      <c r="V15" s="114"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -3555,10 +3591,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="115" t="s">
+      <c r="AA15" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB15" s="116"/>
+      <c r="AB15" s="114"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -3593,21 +3629,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="130"/>
-      <c r="G16" s="131"/>
-      <c r="H16" s="131"/>
-      <c r="I16" s="131"/>
-      <c r="J16" s="132"/>
+      <c r="F16" s="121"/>
+      <c r="G16" s="122"/>
+      <c r="H16" s="122"/>
+      <c r="I16" s="122"/>
+      <c r="J16" s="123"/>
       <c r="K16" s="40" t="s">
         <v>50</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="119" t="s">
+      <c r="N16" s="125" t="s">
         <v>51</v>
       </c>
-      <c r="O16" s="91"/>
-      <c r="P16" s="92"/>
+      <c r="O16" s="92"/>
+      <c r="P16" s="93"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -3617,10 +3653,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="115" t="s">
+      <c r="U16" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V16" s="116"/>
+      <c r="V16" s="114"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -3633,10 +3669,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="115" t="s">
+      <c r="AA16" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB16" s="116"/>
+      <c r="AB16" s="114"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -3672,22 +3708,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="135" t="s">
+      <c r="G17" s="120" t="s">
         <v>77</v>
       </c>
-      <c r="H17" s="91"/>
-      <c r="I17" s="91"/>
-      <c r="J17" s="92"/>
+      <c r="H17" s="92"/>
+      <c r="I17" s="92"/>
+      <c r="J17" s="93"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="119" t="s">
+      <c r="N17" s="125" t="s">
         <v>65</v>
       </c>
-      <c r="O17" s="91"/>
-      <c r="P17" s="92"/>
+      <c r="O17" s="92"/>
+      <c r="P17" s="93"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -3697,10 +3733,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="115" t="s">
+      <c r="U17" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V17" s="116"/>
+      <c r="V17" s="114"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -3713,10 +3749,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="115" t="s">
+      <c r="AA17" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB17" s="116"/>
+      <c r="AB17" s="114"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -3752,12 +3788,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="135" t="s">
+      <c r="G18" s="120" t="s">
         <v>77</v>
       </c>
-      <c r="H18" s="91"/>
-      <c r="I18" s="91"/>
-      <c r="J18" s="92"/>
+      <c r="H18" s="92"/>
+      <c r="I18" s="92"/>
+      <c r="J18" s="93"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -3765,11 +3801,11 @@
       <c r="M18" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N18" s="119" t="s">
+      <c r="N18" s="125" t="s">
         <v>62</v>
       </c>
-      <c r="O18" s="91"/>
-      <c r="P18" s="92"/>
+      <c r="O18" s="92"/>
+      <c r="P18" s="93"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -3779,10 +3815,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="115" t="s">
+      <c r="U18" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V18" s="116"/>
+      <c r="V18" s="114"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -3795,10 +3831,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="115" t="s">
+      <c r="AA18" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB18" s="116"/>
+      <c r="AB18" s="114"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -3836,20 +3872,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="130"/>
-      <c r="H19" s="131"/>
-      <c r="I19" s="131"/>
-      <c r="J19" s="132"/>
+      <c r="G19" s="121"/>
+      <c r="H19" s="122"/>
+      <c r="I19" s="122"/>
+      <c r="J19" s="123"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="119" t="s">
+      <c r="N19" s="125" t="s">
         <v>94</v>
       </c>
-      <c r="O19" s="91"/>
-      <c r="P19" s="92"/>
+      <c r="O19" s="92"/>
+      <c r="P19" s="93"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -3859,10 +3895,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="115" t="s">
+      <c r="U19" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V19" s="116"/>
+      <c r="V19" s="114"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -3875,10 +3911,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="115" t="s">
+      <c r="AA19" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB19" s="116"/>
+      <c r="AB19" s="114"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -3918,20 +3954,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="130"/>
-      <c r="H20" s="131"/>
-      <c r="I20" s="131"/>
-      <c r="J20" s="132"/>
+      <c r="G20" s="121"/>
+      <c r="H20" s="122"/>
+      <c r="I20" s="122"/>
+      <c r="J20" s="123"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="119" t="s">
+      <c r="N20" s="125" t="s">
         <v>95</v>
       </c>
-      <c r="O20" s="91"/>
-      <c r="P20" s="92"/>
+      <c r="O20" s="92"/>
+      <c r="P20" s="93"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -3941,10 +3977,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="115" t="s">
+      <c r="U20" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V20" s="116"/>
+      <c r="V20" s="114"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -3957,10 +3993,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="115" t="s">
+      <c r="AA20" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB20" s="116"/>
+      <c r="AB20" s="114"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -3998,20 +4034,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="130"/>
-      <c r="H21" s="131"/>
-      <c r="I21" s="131"/>
-      <c r="J21" s="132"/>
+      <c r="G21" s="121"/>
+      <c r="H21" s="122"/>
+      <c r="I21" s="122"/>
+      <c r="J21" s="123"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="119" t="s">
+      <c r="N21" s="125" t="s">
         <v>63</v>
       </c>
-      <c r="O21" s="91"/>
-      <c r="P21" s="92"/>
+      <c r="O21" s="92"/>
+      <c r="P21" s="93"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -4021,10 +4057,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="115" t="s">
+      <c r="U21" s="113" t="s">
         <v>97</v>
       </c>
-      <c r="V21" s="116"/>
+      <c r="V21" s="114"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -4037,10 +4073,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="115" t="s">
+      <c r="AA21" s="113" t="s">
         <v>99</v>
       </c>
-      <c r="AB21" s="116"/>
+      <c r="AB21" s="114"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -4074,22 +4110,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="136"/>
-      <c r="F22" s="131"/>
-      <c r="G22" s="131"/>
-      <c r="H22" s="131"/>
-      <c r="I22" s="131"/>
-      <c r="J22" s="132"/>
+      <c r="E22" s="124"/>
+      <c r="F22" s="122"/>
+      <c r="G22" s="122"/>
+      <c r="H22" s="122"/>
+      <c r="I22" s="122"/>
+      <c r="J22" s="123"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="119" t="s">
+      <c r="N22" s="125" t="s">
         <v>64</v>
       </c>
-      <c r="O22" s="91"/>
-      <c r="P22" s="92"/>
+      <c r="O22" s="92"/>
+      <c r="P22" s="93"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -4099,10 +4135,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="115" t="s">
+      <c r="U22" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V22" s="116"/>
+      <c r="V22" s="114"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -4115,10 +4151,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="115" t="s">
+      <c r="AA22" s="113" t="s">
         <v>97</v>
       </c>
-      <c r="AB22" s="116"/>
+      <c r="AB22" s="114"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -4158,22 +4194,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="135" t="s">
+      <c r="G23" s="120" t="s">
         <v>78</v>
       </c>
-      <c r="H23" s="91"/>
-      <c r="I23" s="91"/>
-      <c r="J23" s="92"/>
+      <c r="H23" s="92"/>
+      <c r="I23" s="92"/>
+      <c r="J23" s="93"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="119" t="s">
+      <c r="N23" s="125" t="s">
         <v>83</v>
       </c>
-      <c r="O23" s="91"/>
-      <c r="P23" s="92"/>
+      <c r="O23" s="92"/>
+      <c r="P23" s="93"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -4183,10 +4219,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="115" t="s">
+      <c r="U23" s="113" t="s">
         <v>98</v>
       </c>
-      <c r="V23" s="116"/>
+      <c r="V23" s="114"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -4199,10 +4235,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="115" t="s">
+      <c r="AA23" s="113" t="s">
         <v>97</v>
       </c>
-      <c r="AB23" s="116"/>
+      <c r="AB23" s="114"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -4242,22 +4278,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="135" t="s">
+      <c r="G24" s="120" t="s">
         <v>78</v>
       </c>
-      <c r="H24" s="91"/>
-      <c r="I24" s="91"/>
-      <c r="J24" s="92"/>
+      <c r="H24" s="92"/>
+      <c r="I24" s="92"/>
+      <c r="J24" s="93"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="119" t="s">
+      <c r="N24" s="125" t="s">
         <v>82</v>
       </c>
-      <c r="O24" s="91"/>
-      <c r="P24" s="92"/>
+      <c r="O24" s="92"/>
+      <c r="P24" s="93"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -4267,10 +4303,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="115" t="s">
+      <c r="U24" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V24" s="116"/>
+      <c r="V24" s="114"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -4283,10 +4319,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="115" t="s">
+      <c r="AA24" s="113" t="s">
         <v>99</v>
       </c>
-      <c r="AB24" s="116"/>
+      <c r="AB24" s="114"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -4324,10 +4360,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="130"/>
-      <c r="H25" s="131"/>
-      <c r="I25" s="131"/>
-      <c r="J25" s="132"/>
+      <c r="G25" s="121"/>
+      <c r="H25" s="122"/>
+      <c r="I25" s="122"/>
+      <c r="J25" s="123"/>
       <c r="K25" s="49" t="s">
         <v>40</v>
       </c>
@@ -4335,11 +4371,11 @@
         <v>156</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="119" t="s">
+      <c r="N25" s="125" t="s">
         <v>42</v>
       </c>
-      <c r="O25" s="91"/>
-      <c r="P25" s="92"/>
+      <c r="O25" s="92"/>
+      <c r="P25" s="93"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -4349,10 +4385,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="115" t="s">
+      <c r="U25" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V25" s="116"/>
+      <c r="V25" s="114"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -4365,10 +4401,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="115" t="s">
+      <c r="AA25" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB25" s="116"/>
+      <c r="AB25" s="114"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -4406,10 +4442,10 @@
       <c r="F26" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="G26" s="130"/>
-      <c r="H26" s="131"/>
-      <c r="I26" s="131"/>
-      <c r="J26" s="132"/>
+      <c r="G26" s="121"/>
+      <c r="H26" s="122"/>
+      <c r="I26" s="122"/>
+      <c r="J26" s="123"/>
       <c r="K26" s="31" t="s">
         <v>41</v>
       </c>
@@ -4417,11 +4453,11 @@
         <v>156</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="119" t="s">
+      <c r="N26" s="125" t="s">
         <v>43</v>
       </c>
-      <c r="O26" s="91"/>
-      <c r="P26" s="92"/>
+      <c r="O26" s="92"/>
+      <c r="P26" s="93"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -4431,10 +4467,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="115" t="s">
+      <c r="U26" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V26" s="116"/>
+      <c r="V26" s="114"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -4447,10 +4483,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="115" t="s">
+      <c r="AA26" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB26" s="116"/>
+      <c r="AB26" s="114"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -4482,22 +4518,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="136"/>
-      <c r="F27" s="131"/>
-      <c r="G27" s="131"/>
-      <c r="H27" s="131"/>
-      <c r="I27" s="131"/>
-      <c r="J27" s="132"/>
+      <c r="E27" s="124"/>
+      <c r="F27" s="122"/>
+      <c r="G27" s="122"/>
+      <c r="H27" s="122"/>
+      <c r="I27" s="122"/>
+      <c r="J27" s="123"/>
       <c r="K27" s="25" t="s">
         <v>45</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="119" t="s">
+      <c r="N27" s="125" t="s">
         <v>47</v>
       </c>
-      <c r="O27" s="91"/>
-      <c r="P27" s="92"/>
+      <c r="O27" s="92"/>
+      <c r="P27" s="93"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -4507,10 +4543,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="115" t="s">
+      <c r="U27" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="V27" s="116"/>
+      <c r="V27" s="114"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -4523,10 +4559,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="115" t="s">
+      <c r="AA27" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="AB27" s="116"/>
+      <c r="AB27" s="114"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -4558,12 +4594,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="146"/>
-      <c r="F28" s="147"/>
-      <c r="G28" s="147"/>
-      <c r="H28" s="147"/>
-      <c r="I28" s="147"/>
-      <c r="J28" s="148"/>
+      <c r="E28" s="141"/>
+      <c r="F28" s="142"/>
+      <c r="G28" s="142"/>
+      <c r="H28" s="142"/>
+      <c r="I28" s="142"/>
+      <c r="J28" s="143"/>
       <c r="K28" s="52" t="s">
         <v>46</v>
       </c>
@@ -4571,11 +4607,11 @@
         <v>156</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="143" t="s">
+      <c r="N28" s="138" t="s">
         <v>93</v>
       </c>
-      <c r="O28" s="144"/>
-      <c r="P28" s="145"/>
+      <c r="O28" s="139"/>
+      <c r="P28" s="140"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -4585,10 +4621,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="149" t="s">
+      <c r="U28" s="150" t="s">
         <v>74</v>
       </c>
-      <c r="V28" s="150"/>
+      <c r="V28" s="151"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -4601,10 +4637,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="149" t="s">
+      <c r="AA28" s="150" t="s">
         <v>74</v>
       </c>
-      <c r="AB28" s="150"/>
+      <c r="AB28" s="151"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -4681,18 +4717,18 @@
       <c r="S30" s="75" t="s">
         <v>157</v>
       </c>
-      <c r="T30" s="87" t="s">
+      <c r="T30" s="88" t="s">
         <v>158</v>
       </c>
-      <c r="U30" s="87"/>
-      <c r="V30" s="87"/>
-      <c r="W30" s="87"/>
-      <c r="X30" s="87"/>
-      <c r="Y30" s="87"/>
-      <c r="Z30" s="87"/>
-      <c r="AA30" s="87"/>
-      <c r="AB30" s="87"/>
-      <c r="AC30" s="88"/>
+      <c r="U30" s="88"/>
+      <c r="V30" s="88"/>
+      <c r="W30" s="88"/>
+      <c r="X30" s="88"/>
+      <c r="Y30" s="88"/>
+      <c r="Z30" s="88"/>
+      <c r="AA30" s="88"/>
+      <c r="AB30" s="88"/>
+      <c r="AC30" s="89"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="67" t="s">
@@ -4733,18 +4769,18 @@
       <c r="S31" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="T31" s="89" t="s">
+      <c r="T31" s="90" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="89"/>
-      <c r="V31" s="89"/>
-      <c r="W31" s="89"/>
-      <c r="X31" s="89"/>
-      <c r="Y31" s="89"/>
-      <c r="Z31" s="89"/>
-      <c r="AA31" s="89"/>
-      <c r="AB31" s="89"/>
-      <c r="AC31" s="90"/>
+      <c r="U31" s="90"/>
+      <c r="V31" s="90"/>
+      <c r="W31" s="90"/>
+      <c r="X31" s="90"/>
+      <c r="Y31" s="90"/>
+      <c r="Z31" s="90"/>
+      <c r="AA31" s="90"/>
+      <c r="AB31" s="90"/>
+      <c r="AC31" s="91"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="4" t="s">
@@ -4768,72 +4804,118 @@
       <c r="S32" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="T32" s="91" t="s">
+      <c r="T32" s="92" t="s">
         <v>164</v>
       </c>
-      <c r="U32" s="91"/>
-      <c r="V32" s="91"/>
-      <c r="W32" s="91"/>
-      <c r="X32" s="91"/>
-      <c r="Y32" s="91"/>
-      <c r="Z32" s="91"/>
-      <c r="AA32" s="91"/>
-      <c r="AB32" s="91"/>
-      <c r="AC32" s="92"/>
-    </row>
-    <row r="33" spans="2:29" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U32" s="92"/>
+      <c r="V32" s="92"/>
+      <c r="W32" s="92"/>
+      <c r="X32" s="92"/>
+      <c r="Y32" s="92"/>
+      <c r="Z32" s="92"/>
+      <c r="AA32" s="92"/>
+      <c r="AB32" s="92"/>
+      <c r="AC32" s="93"/>
+    </row>
+    <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H33" s="87" t="s">
+        <v>200</v>
+      </c>
+      <c r="I33" s="73">
+        <v>7</v>
+      </c>
+      <c r="J33" s="74">
+        <v>6</v>
+      </c>
+      <c r="K33" s="74">
+        <v>5</v>
+      </c>
+      <c r="L33" s="74">
+        <v>4</v>
+      </c>
+      <c r="M33" s="74">
+        <v>3</v>
+      </c>
+      <c r="N33" s="74">
+        <v>2</v>
+      </c>
+      <c r="O33" s="74">
+        <v>1</v>
+      </c>
+      <c r="P33" s="72">
+        <v>0</v>
+      </c>
       <c r="R33" s="2">
         <v>2</v>
       </c>
       <c r="S33" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T33" s="91" t="s">
+      <c r="T33" s="92" t="s">
         <v>165</v>
       </c>
-      <c r="U33" s="91"/>
-      <c r="V33" s="91"/>
-      <c r="W33" s="91"/>
-      <c r="X33" s="91"/>
-      <c r="Y33" s="91"/>
-      <c r="Z33" s="91"/>
-      <c r="AA33" s="91"/>
-      <c r="AB33" s="91"/>
-      <c r="AC33" s="92"/>
+      <c r="U33" s="92"/>
+      <c r="V33" s="92"/>
+      <c r="W33" s="92"/>
+      <c r="X33" s="92"/>
+      <c r="Y33" s="92"/>
+      <c r="Z33" s="92"/>
+      <c r="AA33" s="92"/>
+      <c r="AB33" s="92"/>
+      <c r="AC33" s="93"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="168" t="s">
+      <c r="B34" s="169" t="s">
         <v>109</v>
       </c>
-      <c r="C34" s="123" t="s">
+      <c r="C34" s="144" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="125"/>
-      <c r="E34" s="123" t="s">
+      <c r="D34" s="146"/>
+      <c r="E34" s="144" t="s">
         <v>116</v>
       </c>
-      <c r="F34" s="125"/>
+      <c r="F34" s="146"/>
+      <c r="H34" s="77" t="s">
+        <v>66</v>
+      </c>
+      <c r="I34" s="78"/>
+      <c r="J34" s="79"/>
+      <c r="K34" s="79"/>
+      <c r="L34" s="79"/>
+      <c r="M34" s="79" t="s">
+        <v>204</v>
+      </c>
+      <c r="N34" s="79" t="s">
+        <v>203</v>
+      </c>
+      <c r="O34" s="79" t="s">
+        <v>202</v>
+      </c>
+      <c r="P34" s="80" t="s">
+        <v>201</v>
+      </c>
       <c r="R34" s="2">
         <v>3</v>
       </c>
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="91" t="s">
+      <c r="T34" s="92" t="s">
         <v>166</v>
       </c>
-      <c r="U34" s="91"/>
-      <c r="V34" s="91"/>
-      <c r="W34" s="91"/>
-      <c r="X34" s="91"/>
-      <c r="Y34" s="91"/>
-      <c r="Z34" s="91"/>
-      <c r="AA34" s="91"/>
-      <c r="AB34" s="91"/>
-      <c r="AC34" s="92"/>
+      <c r="U34" s="92"/>
+      <c r="V34" s="92"/>
+      <c r="W34" s="92"/>
+      <c r="X34" s="92"/>
+      <c r="Y34" s="92"/>
+      <c r="Z34" s="92"/>
+      <c r="AA34" s="92"/>
+      <c r="AB34" s="92"/>
+      <c r="AC34" s="93"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="169"/>
+      <c r="B35" s="170"/>
       <c r="C35" s="64" t="s">
         <v>100</v>
       </c>
@@ -4852,18 +4934,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="91" t="s">
+      <c r="T35" s="92" t="s">
         <v>167</v>
       </c>
-      <c r="U35" s="91"/>
-      <c r="V35" s="91"/>
-      <c r="W35" s="91"/>
-      <c r="X35" s="91"/>
-      <c r="Y35" s="91"/>
-      <c r="Z35" s="91"/>
-      <c r="AA35" s="91"/>
-      <c r="AB35" s="91"/>
-      <c r="AC35" s="92"/>
+      <c r="U35" s="92"/>
+      <c r="V35" s="92"/>
+      <c r="W35" s="92"/>
+      <c r="X35" s="92"/>
+      <c r="Y35" s="92"/>
+      <c r="Z35" s="92"/>
+      <c r="AA35" s="92"/>
+      <c r="AB35" s="92"/>
+      <c r="AC35" s="93"/>
     </row>
     <row r="36" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B36" s="1">
@@ -4887,18 +4969,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="91" t="s">
+      <c r="T36" s="92" t="s">
         <v>168</v>
       </c>
-      <c r="U36" s="91"/>
-      <c r="V36" s="91"/>
-      <c r="W36" s="91"/>
-      <c r="X36" s="91"/>
-      <c r="Y36" s="91"/>
-      <c r="Z36" s="91"/>
-      <c r="AA36" s="91"/>
-      <c r="AB36" s="91"/>
-      <c r="AC36" s="92"/>
+      <c r="U36" s="92"/>
+      <c r="V36" s="92"/>
+      <c r="W36" s="92"/>
+      <c r="X36" s="92"/>
+      <c r="Y36" s="92"/>
+      <c r="Z36" s="92"/>
+      <c r="AA36" s="92"/>
+      <c r="AB36" s="92"/>
+      <c r="AC36" s="93"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="2">
@@ -4916,24 +4998,25 @@
       <c r="F37" s="35" t="s">
         <v>110</v>
       </c>
+      <c r="N37" s="179"/>
       <c r="R37" s="2">
         <v>6</v>
       </c>
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="91" t="s">
+      <c r="T37" s="92" t="s">
         <v>197</v>
       </c>
-      <c r="U37" s="91"/>
-      <c r="V37" s="91"/>
-      <c r="W37" s="91"/>
-      <c r="X37" s="91"/>
-      <c r="Y37" s="91"/>
-      <c r="Z37" s="91"/>
-      <c r="AA37" s="91"/>
-      <c r="AB37" s="91"/>
-      <c r="AC37" s="92"/>
+      <c r="U37" s="92"/>
+      <c r="V37" s="92"/>
+      <c r="W37" s="92"/>
+      <c r="X37" s="92"/>
+      <c r="Y37" s="92"/>
+      <c r="Z37" s="92"/>
+      <c r="AA37" s="92"/>
+      <c r="AB37" s="92"/>
+      <c r="AC37" s="93"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="2">
@@ -4954,21 +5037,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="99" t="s">
+      <c r="S38" s="100" t="s">
         <v>73</v>
       </c>
-      <c r="T38" s="101" t="s">
+      <c r="T38" s="102" t="s">
         <v>169</v>
       </c>
-      <c r="U38" s="102"/>
-      <c r="V38" s="102"/>
-      <c r="W38" s="102"/>
-      <c r="X38" s="102"/>
-      <c r="Y38" s="102"/>
-      <c r="Z38" s="102"/>
-      <c r="AA38" s="102"/>
-      <c r="AB38" s="102"/>
-      <c r="AC38" s="103"/>
+      <c r="U38" s="103"/>
+      <c r="V38" s="103"/>
+      <c r="W38" s="103"/>
+      <c r="X38" s="103"/>
+      <c r="Y38" s="103"/>
+      <c r="Z38" s="103"/>
+      <c r="AA38" s="103"/>
+      <c r="AB38" s="103"/>
+      <c r="AC38" s="104"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="2">
@@ -4986,26 +5069,26 @@
       <c r="F39" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G39" s="107" t="s">
+      <c r="G39" s="108" t="s">
         <v>182</v>
       </c>
-      <c r="H39" s="93"/>
-      <c r="I39" s="93"/>
-      <c r="J39" s="94"/>
+      <c r="H39" s="94"/>
+      <c r="I39" s="94"/>
+      <c r="J39" s="95"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="100"/>
-      <c r="T39" s="104"/>
-      <c r="U39" s="105"/>
-      <c r="V39" s="105"/>
-      <c r="W39" s="105"/>
-      <c r="X39" s="105"/>
-      <c r="Y39" s="105"/>
-      <c r="Z39" s="105"/>
-      <c r="AA39" s="105"/>
-      <c r="AB39" s="105"/>
-      <c r="AC39" s="106"/>
+      <c r="S39" s="101"/>
+      <c r="T39" s="105"/>
+      <c r="U39" s="106"/>
+      <c r="V39" s="106"/>
+      <c r="W39" s="106"/>
+      <c r="X39" s="106"/>
+      <c r="Y39" s="106"/>
+      <c r="Z39" s="106"/>
+      <c r="AA39" s="106"/>
+      <c r="AB39" s="106"/>
+      <c r="AC39" s="107"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="2">
@@ -5023,28 +5106,28 @@
       <c r="F40" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G40" s="109"/>
-      <c r="H40" s="110"/>
-      <c r="I40" s="110"/>
-      <c r="J40" s="111"/>
+      <c r="G40" s="110"/>
+      <c r="H40" s="111"/>
+      <c r="I40" s="111"/>
+      <c r="J40" s="112"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="91" t="s">
+      <c r="T40" s="92" t="s">
         <v>170</v>
       </c>
-      <c r="U40" s="91"/>
-      <c r="V40" s="91"/>
-      <c r="W40" s="91"/>
-      <c r="X40" s="91"/>
-      <c r="Y40" s="91"/>
-      <c r="Z40" s="91"/>
-      <c r="AA40" s="91"/>
-      <c r="AB40" s="91"/>
-      <c r="AC40" s="92"/>
+      <c r="U40" s="92"/>
+      <c r="V40" s="92"/>
+      <c r="W40" s="92"/>
+      <c r="X40" s="92"/>
+      <c r="Y40" s="92"/>
+      <c r="Z40" s="92"/>
+      <c r="AA40" s="92"/>
+      <c r="AB40" s="92"/>
+      <c r="AC40" s="93"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="2">
@@ -5062,28 +5145,28 @@
       <c r="F41" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="G41" s="109"/>
-      <c r="H41" s="110"/>
-      <c r="I41" s="110"/>
-      <c r="J41" s="111"/>
+      <c r="G41" s="110"/>
+      <c r="H41" s="111"/>
+      <c r="I41" s="111"/>
+      <c r="J41" s="112"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="91" t="s">
+      <c r="T41" s="92" t="s">
         <v>171</v>
       </c>
-      <c r="U41" s="91"/>
-      <c r="V41" s="91"/>
-      <c r="W41" s="91"/>
-      <c r="X41" s="91"/>
-      <c r="Y41" s="91"/>
-      <c r="Z41" s="91"/>
-      <c r="AA41" s="91"/>
-      <c r="AB41" s="91"/>
-      <c r="AC41" s="92"/>
+      <c r="U41" s="92"/>
+      <c r="V41" s="92"/>
+      <c r="W41" s="92"/>
+      <c r="X41" s="92"/>
+      <c r="Y41" s="92"/>
+      <c r="Z41" s="92"/>
+      <c r="AA41" s="92"/>
+      <c r="AB41" s="92"/>
+      <c r="AC41" s="93"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="2">
@@ -5101,28 +5184,28 @@
       <c r="F42" s="76" t="s">
         <v>176</v>
       </c>
-      <c r="G42" s="108"/>
-      <c r="H42" s="95"/>
-      <c r="I42" s="95"/>
-      <c r="J42" s="96"/>
+      <c r="G42" s="109"/>
+      <c r="H42" s="96"/>
+      <c r="I42" s="96"/>
+      <c r="J42" s="97"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="T42" s="91" t="s">
+      <c r="T42" s="92" t="s">
         <v>172</v>
       </c>
-      <c r="U42" s="91"/>
-      <c r="V42" s="91"/>
-      <c r="W42" s="91"/>
-      <c r="X42" s="91"/>
-      <c r="Y42" s="91"/>
-      <c r="Z42" s="91"/>
-      <c r="AA42" s="91"/>
-      <c r="AB42" s="91"/>
-      <c r="AC42" s="92"/>
+      <c r="U42" s="92"/>
+      <c r="V42" s="92"/>
+      <c r="W42" s="92"/>
+      <c r="X42" s="92"/>
+      <c r="Y42" s="92"/>
+      <c r="Z42" s="92"/>
+      <c r="AA42" s="92"/>
+      <c r="AB42" s="92"/>
+      <c r="AC42" s="93"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="2">
@@ -5140,30 +5223,30 @@
       <c r="F43" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="G43" s="173" t="s">
+      <c r="G43" s="174" t="s">
         <v>194</v>
       </c>
-      <c r="H43" s="97"/>
-      <c r="I43" s="97"/>
-      <c r="J43" s="98"/>
+      <c r="H43" s="98"/>
+      <c r="I43" s="98"/>
+      <c r="J43" s="99"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="T43" s="91" t="s">
+      <c r="T43" s="92" t="s">
         <v>173</v>
       </c>
-      <c r="U43" s="91"/>
-      <c r="V43" s="91"/>
-      <c r="W43" s="91"/>
-      <c r="X43" s="91"/>
-      <c r="Y43" s="91"/>
-      <c r="Z43" s="91"/>
-      <c r="AA43" s="91"/>
-      <c r="AB43" s="91"/>
-      <c r="AC43" s="92"/>
+      <c r="U43" s="92"/>
+      <c r="V43" s="92"/>
+      <c r="W43" s="92"/>
+      <c r="X43" s="92"/>
+      <c r="Y43" s="92"/>
+      <c r="Z43" s="92"/>
+      <c r="AA43" s="92"/>
+      <c r="AB43" s="92"/>
+      <c r="AC43" s="93"/>
     </row>
     <row r="44" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="2">
@@ -5184,21 +5267,21 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="99" t="s">
+      <c r="S44" s="100" t="s">
         <v>76</v>
       </c>
-      <c r="T44" s="101" t="s">
+      <c r="T44" s="102" t="s">
         <v>174</v>
       </c>
-      <c r="U44" s="102"/>
-      <c r="V44" s="102"/>
-      <c r="W44" s="102"/>
-      <c r="X44" s="102"/>
-      <c r="Y44" s="102"/>
-      <c r="Z44" s="102"/>
-      <c r="AA44" s="102"/>
-      <c r="AB44" s="102"/>
-      <c r="AC44" s="103"/>
+      <c r="U44" s="103"/>
+      <c r="V44" s="103"/>
+      <c r="W44" s="103"/>
+      <c r="X44" s="103"/>
+      <c r="Y44" s="103"/>
+      <c r="Z44" s="103"/>
+      <c r="AA44" s="103"/>
+      <c r="AB44" s="103"/>
+      <c r="AC44" s="104"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="2">
@@ -5216,26 +5299,26 @@
       <c r="F45" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="G45" s="107" t="s">
+      <c r="G45" s="108" t="s">
         <v>181</v>
       </c>
-      <c r="H45" s="93"/>
-      <c r="I45" s="93"/>
-      <c r="J45" s="94"/>
+      <c r="H45" s="94"/>
+      <c r="I45" s="94"/>
+      <c r="J45" s="95"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="100"/>
-      <c r="T45" s="104"/>
-      <c r="U45" s="105"/>
-      <c r="V45" s="105"/>
-      <c r="W45" s="105"/>
-      <c r="X45" s="105"/>
-      <c r="Y45" s="105"/>
-      <c r="Z45" s="105"/>
-      <c r="AA45" s="105"/>
-      <c r="AB45" s="105"/>
-      <c r="AC45" s="106"/>
+      <c r="S45" s="101"/>
+      <c r="T45" s="105"/>
+      <c r="U45" s="106"/>
+      <c r="V45" s="106"/>
+      <c r="W45" s="106"/>
+      <c r="X45" s="106"/>
+      <c r="Y45" s="106"/>
+      <c r="Z45" s="106"/>
+      <c r="AA45" s="106"/>
+      <c r="AB45" s="106"/>
+      <c r="AC45" s="107"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B46" s="2">
@@ -5253,28 +5336,28 @@
       <c r="F46" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G46" s="108"/>
-      <c r="H46" s="95"/>
-      <c r="I46" s="95"/>
-      <c r="J46" s="96"/>
+      <c r="G46" s="109"/>
+      <c r="H46" s="96"/>
+      <c r="I46" s="96"/>
+      <c r="J46" s="97"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="T46" s="91" t="s">
+      <c r="T46" s="92" t="s">
         <v>175</v>
       </c>
-      <c r="U46" s="91"/>
-      <c r="V46" s="91"/>
-      <c r="W46" s="91"/>
-      <c r="X46" s="91"/>
-      <c r="Y46" s="91"/>
-      <c r="Z46" s="91"/>
-      <c r="AA46" s="91"/>
-      <c r="AB46" s="91"/>
-      <c r="AC46" s="92"/>
+      <c r="U46" s="92"/>
+      <c r="V46" s="92"/>
+      <c r="W46" s="92"/>
+      <c r="X46" s="92"/>
+      <c r="Y46" s="92"/>
+      <c r="Z46" s="92"/>
+      <c r="AA46" s="92"/>
+      <c r="AB46" s="92"/>
+      <c r="AC46" s="93"/>
     </row>
     <row r="47" spans="2:29" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="2">
@@ -5292,12 +5375,12 @@
       <c r="F47" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="G47" s="97" t="s">
+      <c r="G47" s="98" t="s">
         <v>152</v>
       </c>
-      <c r="H47" s="97"/>
-      <c r="I47" s="97"/>
-      <c r="J47" s="98"/>
+      <c r="H47" s="98"/>
+      <c r="I47" s="98"/>
+      <c r="J47" s="99"/>
     </row>
     <row r="48" spans="2:29" ht="30" x14ac:dyDescent="0.25">
       <c r="B48" s="2">
@@ -5349,12 +5432,12 @@
       <c r="F50" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="G50" s="93" t="s">
+      <c r="G50" s="94" t="s">
         <v>155</v>
       </c>
-      <c r="H50" s="93"/>
-      <c r="I50" s="93"/>
-      <c r="J50" s="94"/>
+      <c r="H50" s="94"/>
+      <c r="I50" s="94"/>
+      <c r="J50" s="95"/>
     </row>
     <row r="51" spans="2:10" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" s="4">
@@ -5372,38 +5455,38 @@
       <c r="F51" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="G51" s="95"/>
-      <c r="H51" s="95"/>
-      <c r="I51" s="95"/>
-      <c r="J51" s="96"/>
+      <c r="G51" s="96"/>
+      <c r="H51" s="96"/>
+      <c r="I51" s="96"/>
+      <c r="J51" s="97"/>
     </row>
     <row r="52" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="170" t="s">
+      <c r="B52" s="171" t="s">
         <v>142</v>
       </c>
-      <c r="C52" s="120"/>
-      <c r="D52" s="120"/>
-      <c r="E52" s="120"/>
-      <c r="F52" s="121"/>
+      <c r="C52" s="129"/>
+      <c r="D52" s="129"/>
+      <c r="E52" s="129"/>
+      <c r="F52" s="130"/>
     </row>
     <row r="54" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B55" s="162" t="s">
+      <c r="B55" s="163" t="s">
         <v>183</v>
       </c>
-      <c r="C55" s="160" t="s">
+      <c r="C55" s="161" t="s">
         <v>185</v>
       </c>
-      <c r="D55" s="174" t="s">
+      <c r="D55" s="175" t="s">
         <v>184</v>
       </c>
-      <c r="E55" s="175"/>
+      <c r="E55" s="176"/>
     </row>
     <row r="56" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="163"/>
-      <c r="C56" s="161"/>
-      <c r="D56" s="176"/>
-      <c r="E56" s="177"/>
+      <c r="B56" s="164"/>
+      <c r="C56" s="162"/>
+      <c r="D56" s="177"/>
+      <c r="E56" s="178"/>
     </row>
     <row r="57" spans="2:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="81">
@@ -5412,10 +5495,10 @@
       <c r="C57" s="84" t="s">
         <v>186</v>
       </c>
-      <c r="D57" s="164" t="s">
+      <c r="D57" s="165" t="s">
         <v>190</v>
       </c>
-      <c r="E57" s="165"/>
+      <c r="E57" s="166"/>
     </row>
     <row r="58" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B58" s="82">
@@ -5424,10 +5507,10 @@
       <c r="C58" s="85" t="s">
         <v>187</v>
       </c>
-      <c r="D58" s="166" t="s">
+      <c r="D58" s="167" t="s">
         <v>191</v>
       </c>
-      <c r="E58" s="167"/>
+      <c r="E58" s="168"/>
     </row>
     <row r="59" spans="2:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="82">
@@ -5436,10 +5519,10 @@
       <c r="C59" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="D59" s="166" t="s">
+      <c r="D59" s="167" t="s">
         <v>192</v>
       </c>
-      <c r="E59" s="167"/>
+      <c r="E59" s="168"/>
     </row>
     <row r="60" spans="2:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="82">
@@ -5448,106 +5531,110 @@
       <c r="C60" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="D60" s="166" t="s">
+      <c r="D60" s="167" t="s">
         <v>193</v>
       </c>
-      <c r="E60" s="167"/>
-    </row>
-    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="E60" s="168"/>
+    </row>
+    <row r="61" spans="2:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="82">
         <v>4</v>
       </c>
-      <c r="C61" s="85"/>
-      <c r="D61" s="166"/>
-      <c r="E61" s="167"/>
+      <c r="C61" s="85" t="s">
+        <v>198</v>
+      </c>
+      <c r="D61" s="167" t="s">
+        <v>199</v>
+      </c>
+      <c r="E61" s="168"/>
     </row>
     <row r="62" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B62" s="82">
         <v>5</v>
       </c>
       <c r="C62" s="85"/>
-      <c r="D62" s="166"/>
-      <c r="E62" s="167"/>
+      <c r="D62" s="167"/>
+      <c r="E62" s="168"/>
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B63" s="82">
         <v>6</v>
       </c>
       <c r="C63" s="85"/>
-      <c r="D63" s="166"/>
-      <c r="E63" s="167"/>
+      <c r="D63" s="167"/>
+      <c r="E63" s="168"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B64" s="82">
         <v>7</v>
       </c>
       <c r="C64" s="85"/>
-      <c r="D64" s="166"/>
-      <c r="E64" s="167"/>
+      <c r="D64" s="167"/>
+      <c r="E64" s="168"/>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="82">
         <v>8</v>
       </c>
       <c r="C65" s="85"/>
-      <c r="D65" s="166"/>
-      <c r="E65" s="167"/>
+      <c r="D65" s="167"/>
+      <c r="E65" s="168"/>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" s="82">
         <v>9</v>
       </c>
       <c r="C66" s="85"/>
-      <c r="D66" s="166"/>
-      <c r="E66" s="167"/>
+      <c r="D66" s="167"/>
+      <c r="E66" s="168"/>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" s="82">
         <v>10</v>
       </c>
       <c r="C67" s="85"/>
-      <c r="D67" s="166"/>
-      <c r="E67" s="167"/>
+      <c r="D67" s="167"/>
+      <c r="E67" s="168"/>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" s="82">
         <v>11</v>
       </c>
       <c r="C68" s="85"/>
-      <c r="D68" s="166"/>
-      <c r="E68" s="167"/>
+      <c r="D68" s="167"/>
+      <c r="E68" s="168"/>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69" s="82">
         <v>12</v>
       </c>
       <c r="C69" s="85"/>
-      <c r="D69" s="166"/>
-      <c r="E69" s="167"/>
+      <c r="D69" s="167"/>
+      <c r="E69" s="168"/>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B70" s="82">
         <v>13</v>
       </c>
       <c r="C70" s="85"/>
-      <c r="D70" s="166"/>
-      <c r="E70" s="167"/>
+      <c r="D70" s="167"/>
+      <c r="E70" s="168"/>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B71" s="82">
         <v>14</v>
       </c>
       <c r="C71" s="85"/>
-      <c r="D71" s="166"/>
-      <c r="E71" s="167"/>
+      <c r="D71" s="167"/>
+      <c r="E71" s="168"/>
     </row>
     <row r="72" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B72" s="83">
         <v>15</v>
       </c>
       <c r="C72" s="86"/>
-      <c r="D72" s="171"/>
-      <c r="E72" s="172"/>
+      <c r="D72" s="172"/>
+      <c r="E72" s="173"/>
     </row>
   </sheetData>
   <mergeCells count="158">
@@ -5575,7 +5662,6 @@
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="B34:B35"/>
     <mergeCell ref="B52:F52"/>
-    <mergeCell ref="AA23:AB23"/>
     <mergeCell ref="S2:S4"/>
     <mergeCell ref="R2:R4"/>
     <mergeCell ref="AA6:AB6"/>
@@ -5615,11 +5701,7 @@
     <mergeCell ref="U26:V26"/>
     <mergeCell ref="N26:P26"/>
     <mergeCell ref="N25:P25"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="N22:P22"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="N28:P28"/>
     <mergeCell ref="N27:P27"/>
@@ -5639,9 +5721,6 @@
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="G21:J21"/>
     <mergeCell ref="F16:J16"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="H15:J15"/>
     <mergeCell ref="K2:P2"/>
     <mergeCell ref="N7:P7"/>
     <mergeCell ref="N8:P8"/>
@@ -5649,6 +5728,10 @@
     <mergeCell ref="E4:J4"/>
     <mergeCell ref="N10:P10"/>
     <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="H9:J9"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G19:J19"/>
@@ -5660,12 +5743,15 @@
     <mergeCell ref="AA18:AB18"/>
     <mergeCell ref="N18:P18"/>
     <mergeCell ref="N16:P16"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
     <mergeCell ref="N6:P6"/>
     <mergeCell ref="N12:P12"/>
     <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H14:J14"/>
     <mergeCell ref="AA20:AB20"/>
     <mergeCell ref="AA21:AB21"/>
     <mergeCell ref="AA22:AB22"/>
@@ -5688,6 +5774,7 @@
     <mergeCell ref="U19:V19"/>
     <mergeCell ref="U10:V10"/>
     <mergeCell ref="U11:V11"/>
+    <mergeCell ref="AA23:AB23"/>
     <mergeCell ref="T30:AC30"/>
     <mergeCell ref="T31:AC31"/>
     <mergeCell ref="T32:AC32"/>

</xml_diff>

<commit_message>
Se implemento el sistema que guarda los EPC y Cause en una excepción. Faltaria el sistema que genera el doblefault y el sistema de alignamentfault
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0ED791-A8C8-49FA-9127-CD4D27FA30B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{635EA803-B12D-4441-BEE8-1D33FF932DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="208">
   <si>
     <t>OpCode</t>
   </si>
@@ -596,9 +596,6 @@
     <t>Nombre</t>
   </si>
   <si>
-    <t>Page Fault</t>
-  </si>
-  <si>
     <t>General Protection Fault</t>
   </si>
   <si>
@@ -608,9 +605,6 @@
     <t>Double Fault</t>
   </si>
   <si>
-    <t xml:space="preserve">Lanzada en el momento exacto en el que la MMU detecta un error de cualquier tipo </t>
-  </si>
-  <si>
     <t>Error lanzado cuando una instrucción privilegiada se intenta usar sin permisos</t>
   </si>
   <si>
@@ -651,6 +645,21 @@
   </si>
   <si>
     <t>Global</t>
+  </si>
+  <si>
+    <t>Page Fault LOD</t>
+  </si>
+  <si>
+    <t>Page Fault STR</t>
+  </si>
+  <si>
+    <t>Lanzada en el momento exacto en el que la MMU detecta un error en STR</t>
+  </si>
+  <si>
+    <t>Lanzada en el momento exacto en el que la MMU detecta un error en LOD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Excepción </t>
   </si>
 </sst>
 </file>
@@ -1651,7 +1660,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="180">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1902,28 +1911,28 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1974,6 +1983,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2025,9 +2043,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2043,9 +2058,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2064,15 +2076,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2100,27 +2103,27 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2144,15 +2147,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2166,9 +2160,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2187,7 +2178,22 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2497,62 +2503,62 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="135" t="s">
+      <c r="B2" s="136" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="147" t="s">
+      <c r="C2" s="145" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="148"/>
-      <c r="E2" s="127" t="s">
+      <c r="D2" s="146"/>
+      <c r="E2" s="129" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="127"/>
-      <c r="G2" s="149" t="s">
+      <c r="F2" s="129"/>
+      <c r="G2" s="147" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="127"/>
-      <c r="I2" s="127" t="s">
+      <c r="H2" s="129"/>
+      <c r="I2" s="129" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="127"/>
-      <c r="K2" s="126" t="s">
+      <c r="J2" s="129"/>
+      <c r="K2" s="128" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="127"/>
-      <c r="M2" s="127"/>
-      <c r="N2" s="127"/>
-      <c r="O2" s="127"/>
-      <c r="P2" s="128"/>
-      <c r="R2" s="154" t="s">
+      <c r="L2" s="129"/>
+      <c r="M2" s="129"/>
+      <c r="N2" s="129"/>
+      <c r="O2" s="129"/>
+      <c r="P2" s="130"/>
+      <c r="R2" s="150" t="s">
         <v>66</v>
       </c>
-      <c r="S2" s="89" t="s">
+      <c r="S2" s="87" t="s">
         <v>67</v>
       </c>
-      <c r="T2" s="158" t="s">
+      <c r="T2" s="156" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="159"/>
-      <c r="V2" s="159"/>
-      <c r="W2" s="159"/>
-      <c r="X2" s="159"/>
-      <c r="Y2" s="159"/>
-      <c r="Z2" s="159"/>
-      <c r="AA2" s="159"/>
-      <c r="AB2" s="159" t="s">
+      <c r="U2" s="157"/>
+      <c r="V2" s="157"/>
+      <c r="W2" s="157"/>
+      <c r="X2" s="157"/>
+      <c r="Y2" s="157"/>
+      <c r="Z2" s="157"/>
+      <c r="AA2" s="157"/>
+      <c r="AB2" s="157" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="159"/>
-      <c r="AD2" s="159"/>
-      <c r="AE2" s="159"/>
-      <c r="AF2" s="159"/>
-      <c r="AG2" s="159"/>
-      <c r="AH2" s="159"/>
-      <c r="AI2" s="160"/>
+      <c r="AC2" s="157"/>
+      <c r="AD2" s="157"/>
+      <c r="AE2" s="157"/>
+      <c r="AF2" s="157"/>
+      <c r="AG2" s="157"/>
+      <c r="AH2" s="157"/>
+      <c r="AI2" s="158"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="136"/>
+      <c r="B3" s="137"/>
       <c r="C3" s="16" t="s">
         <v>80</v>
       </c>
@@ -2577,21 +2583,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="144"/>
-      <c r="L3" s="145"/>
-      <c r="M3" s="145"/>
-      <c r="N3" s="145"/>
-      <c r="O3" s="145"/>
-      <c r="P3" s="146"/>
-      <c r="R3" s="155"/>
-      <c r="S3" s="152"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="143"/>
+      <c r="M3" s="143"/>
+      <c r="N3" s="143"/>
+      <c r="O3" s="143"/>
+      <c r="P3" s="144"/>
+      <c r="R3" s="151"/>
+      <c r="S3" s="148"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="115" t="s">
+      <c r="U3" s="118" t="s">
         <v>84</v>
       </c>
-      <c r="V3" s="115"/>
+      <c r="V3" s="118"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -2604,10 +2610,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="157" t="s">
+      <c r="AA3" s="155" t="s">
         <v>75</v>
       </c>
-      <c r="AB3" s="157"/>
+      <c r="AB3" s="155"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -2631,21 +2637,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="137"/>
+      <c r="B4" s="138"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="116" t="s">
+      <c r="E4" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="129"/>
-      <c r="G4" s="129"/>
-      <c r="H4" s="129"/>
-      <c r="I4" s="129"/>
-      <c r="J4" s="130"/>
+      <c r="F4" s="131"/>
+      <c r="G4" s="131"/>
+      <c r="H4" s="131"/>
+      <c r="I4" s="131"/>
+      <c r="J4" s="132"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -2655,20 +2661,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="116" t="s">
+      <c r="N4" s="119" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="129"/>
-      <c r="P4" s="130"/>
-      <c r="R4" s="156"/>
-      <c r="S4" s="153"/>
+      <c r="O4" s="131"/>
+      <c r="P4" s="132"/>
+      <c r="R4" s="152"/>
+      <c r="S4" s="149"/>
       <c r="T4" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="U4" s="116" t="s">
+      <c r="U4" s="119" t="s">
         <v>76</v>
       </c>
-      <c r="V4" s="117"/>
+      <c r="V4" s="120"/>
       <c r="W4" s="7" t="s">
         <v>72</v>
       </c>
@@ -2681,10 +2687,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="116" t="s">
+      <c r="AA4" s="119" t="s">
         <v>73</v>
       </c>
-      <c r="AB4" s="117"/>
+      <c r="AB4" s="120"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -2716,22 +2722,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="132"/>
-      <c r="F5" s="133"/>
-      <c r="G5" s="133"/>
-      <c r="H5" s="133"/>
-      <c r="I5" s="133"/>
-      <c r="J5" s="134"/>
+      <c r="E5" s="133"/>
+      <c r="F5" s="134"/>
+      <c r="G5" s="134"/>
+      <c r="H5" s="134"/>
+      <c r="I5" s="134"/>
+      <c r="J5" s="135"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="131" t="s">
+      <c r="N5" s="88" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="90"/>
-      <c r="P5" s="91"/>
+      <c r="O5" s="89"/>
+      <c r="P5" s="90"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -2741,10 +2747,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="118" t="s">
+      <c r="U5" s="121" t="s">
         <v>74</v>
       </c>
-      <c r="V5" s="119"/>
+      <c r="V5" s="122"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -2757,10 +2763,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="118" t="s">
+      <c r="AA5" s="121" t="s">
         <v>74</v>
       </c>
-      <c r="AB5" s="119"/>
+      <c r="AB5" s="122"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -2792,12 +2798,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="124"/>
-      <c r="F6" s="122"/>
-      <c r="G6" s="122"/>
-      <c r="H6" s="122"/>
-      <c r="I6" s="122"/>
-      <c r="J6" s="123"/>
+      <c r="E6" s="127"/>
+      <c r="F6" s="125"/>
+      <c r="G6" s="125"/>
+      <c r="H6" s="125"/>
+      <c r="I6" s="125"/>
+      <c r="J6" s="126"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -2805,7 +2811,7 @@
         <v>156</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="125" t="s">
+      <c r="N6" s="91" t="s">
         <v>96</v>
       </c>
       <c r="O6" s="92"/>
@@ -2819,10 +2825,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="113" t="s">
+      <c r="U6" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V6" s="114"/>
+      <c r="V6" s="117"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -2835,10 +2841,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="113" t="s">
+      <c r="AA6" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB6" s="114"/>
+      <c r="AB6" s="117"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -2879,9 +2885,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="121"/>
-      <c r="I7" s="122"/>
-      <c r="J7" s="123"/>
+      <c r="H7" s="124"/>
+      <c r="I7" s="125"/>
+      <c r="J7" s="126"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -2889,7 +2895,7 @@
       <c r="M7" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N7" s="125" t="s">
+      <c r="N7" s="91" t="s">
         <v>53</v>
       </c>
       <c r="O7" s="92"/>
@@ -2903,10 +2909,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="113" t="s">
+      <c r="U7" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V7" s="114"/>
+      <c r="V7" s="117"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -2919,10 +2925,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="113" t="s">
+      <c r="AA7" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB7" s="114"/>
+      <c r="AB7" s="117"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -2963,9 +2969,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="121"/>
-      <c r="I8" s="122"/>
-      <c r="J8" s="123"/>
+      <c r="H8" s="124"/>
+      <c r="I8" s="125"/>
+      <c r="J8" s="126"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -2973,7 +2979,7 @@
       <c r="M8" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N8" s="125" t="s">
+      <c r="N8" s="91" t="s">
         <v>54</v>
       </c>
       <c r="O8" s="92"/>
@@ -2987,10 +2993,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="113" t="s">
+      <c r="U8" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V8" s="114"/>
+      <c r="V8" s="117"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -3003,10 +3009,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="113" t="s">
+      <c r="AA8" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB8" s="114"/>
+      <c r="AB8" s="117"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -3047,9 +3053,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="121"/>
-      <c r="I9" s="122"/>
-      <c r="J9" s="123"/>
+      <c r="H9" s="124"/>
+      <c r="I9" s="125"/>
+      <c r="J9" s="126"/>
       <c r="K9" s="37" t="s">
         <v>48</v>
       </c>
@@ -3057,7 +3063,7 @@
       <c r="M9" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N9" s="125" t="s">
+      <c r="N9" s="91" t="s">
         <v>55</v>
       </c>
       <c r="O9" s="92"/>
@@ -3071,10 +3077,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="113" t="s">
+      <c r="U9" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V9" s="114"/>
+      <c r="V9" s="117"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -3087,10 +3093,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="113" t="s">
+      <c r="AA9" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB9" s="114"/>
+      <c r="AB9" s="117"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -3131,9 +3137,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="121"/>
-      <c r="I10" s="122"/>
-      <c r="J10" s="123"/>
+      <c r="H10" s="124"/>
+      <c r="I10" s="125"/>
+      <c r="J10" s="126"/>
       <c r="K10" s="37" t="s">
         <v>49</v>
       </c>
@@ -3141,7 +3147,7 @@
       <c r="M10" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N10" s="125" t="s">
+      <c r="N10" s="91" t="s">
         <v>56</v>
       </c>
       <c r="O10" s="92"/>
@@ -3155,10 +3161,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="113" t="s">
+      <c r="U10" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V10" s="114"/>
+      <c r="V10" s="117"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -3171,10 +3177,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="113" t="s">
+      <c r="AA10" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB10" s="114"/>
+      <c r="AB10" s="117"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -3215,9 +3221,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="121"/>
-      <c r="I11" s="122"/>
-      <c r="J11" s="123"/>
+      <c r="H11" s="124"/>
+      <c r="I11" s="125"/>
+      <c r="J11" s="126"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -3225,7 +3231,7 @@
       <c r="M11" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N11" s="125" t="s">
+      <c r="N11" s="91" t="s">
         <v>57</v>
       </c>
       <c r="O11" s="92"/>
@@ -3239,10 +3245,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="113" t="s">
+      <c r="U11" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V11" s="114"/>
+      <c r="V11" s="117"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -3255,10 +3261,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="113" t="s">
+      <c r="AA11" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB11" s="114"/>
+      <c r="AB11" s="117"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -3299,9 +3305,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="121"/>
-      <c r="I12" s="122"/>
-      <c r="J12" s="123"/>
+      <c r="H12" s="124"/>
+      <c r="I12" s="125"/>
+      <c r="J12" s="126"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -3309,7 +3315,7 @@
       <c r="M12" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N12" s="125" t="s">
+      <c r="N12" s="91" t="s">
         <v>58</v>
       </c>
       <c r="O12" s="92"/>
@@ -3323,10 +3329,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="113" t="s">
+      <c r="U12" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V12" s="114"/>
+      <c r="V12" s="117"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -3339,10 +3345,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="113" t="s">
+      <c r="AA12" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB12" s="114"/>
+      <c r="AB12" s="117"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -3383,9 +3389,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="121"/>
-      <c r="I13" s="122"/>
-      <c r="J13" s="123"/>
+      <c r="H13" s="124"/>
+      <c r="I13" s="125"/>
+      <c r="J13" s="126"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -3393,7 +3399,7 @@
       <c r="M13" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N13" s="125" t="s">
+      <c r="N13" s="91" t="s">
         <v>59</v>
       </c>
       <c r="O13" s="92"/>
@@ -3407,10 +3413,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="113" t="s">
+      <c r="U13" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V13" s="114"/>
+      <c r="V13" s="117"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -3423,10 +3429,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="113" t="s">
+      <c r="AA13" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB13" s="114"/>
+      <c r="AB13" s="117"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -3467,9 +3473,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="121"/>
-      <c r="I14" s="122"/>
-      <c r="J14" s="123"/>
+      <c r="H14" s="124"/>
+      <c r="I14" s="125"/>
+      <c r="J14" s="126"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -3477,7 +3483,7 @@
       <c r="M14" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N14" s="125" t="s">
+      <c r="N14" s="91" t="s">
         <v>60</v>
       </c>
       <c r="O14" s="92"/>
@@ -3491,10 +3497,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="113" t="s">
+      <c r="U14" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V14" s="114"/>
+      <c r="V14" s="117"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -3507,10 +3513,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="113" t="s">
+      <c r="AA14" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB14" s="114"/>
+      <c r="AB14" s="117"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -3551,9 +3557,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="121"/>
-      <c r="I15" s="122"/>
-      <c r="J15" s="123"/>
+      <c r="H15" s="124"/>
+      <c r="I15" s="125"/>
+      <c r="J15" s="126"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -3561,7 +3567,7 @@
       <c r="M15" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N15" s="125" t="s">
+      <c r="N15" s="91" t="s">
         <v>61</v>
       </c>
       <c r="O15" s="92"/>
@@ -3575,10 +3581,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="113" t="s">
+      <c r="U15" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V15" s="114"/>
+      <c r="V15" s="117"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -3591,10 +3597,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="113" t="s">
+      <c r="AA15" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB15" s="114"/>
+      <c r="AB15" s="117"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -3629,17 +3635,17 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="121"/>
-      <c r="G16" s="122"/>
-      <c r="H16" s="122"/>
-      <c r="I16" s="122"/>
-      <c r="J16" s="123"/>
+      <c r="F16" s="124"/>
+      <c r="G16" s="125"/>
+      <c r="H16" s="125"/>
+      <c r="I16" s="125"/>
+      <c r="J16" s="126"/>
       <c r="K16" s="40" t="s">
         <v>50</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="125" t="s">
+      <c r="N16" s="91" t="s">
         <v>51</v>
       </c>
       <c r="O16" s="92"/>
@@ -3653,10 +3659,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="113" t="s">
+      <c r="U16" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V16" s="114"/>
+      <c r="V16" s="117"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -3669,10 +3675,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="113" t="s">
+      <c r="AA16" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB16" s="114"/>
+      <c r="AB16" s="117"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -3708,7 +3714,7 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="120" t="s">
+      <c r="G17" s="123" t="s">
         <v>77</v>
       </c>
       <c r="H17" s="92"/>
@@ -3719,7 +3725,7 @@
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="125" t="s">
+      <c r="N17" s="91" t="s">
         <v>65</v>
       </c>
       <c r="O17" s="92"/>
@@ -3733,10 +3739,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="113" t="s">
+      <c r="U17" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V17" s="114"/>
+      <c r="V17" s="117"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -3749,10 +3755,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="113" t="s">
+      <c r="AA17" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB17" s="114"/>
+      <c r="AB17" s="117"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -3788,7 +3794,7 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="120" t="s">
+      <c r="G18" s="123" t="s">
         <v>77</v>
       </c>
       <c r="H18" s="92"/>
@@ -3801,7 +3807,7 @@
       <c r="M18" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N18" s="125" t="s">
+      <c r="N18" s="91" t="s">
         <v>62</v>
       </c>
       <c r="O18" s="92"/>
@@ -3815,10 +3821,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="113" t="s">
+      <c r="U18" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V18" s="114"/>
+      <c r="V18" s="117"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -3831,10 +3837,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="113" t="s">
+      <c r="AA18" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB18" s="114"/>
+      <c r="AB18" s="117"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -3872,16 +3878,16 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="121"/>
-      <c r="H19" s="122"/>
-      <c r="I19" s="122"/>
-      <c r="J19" s="123"/>
+      <c r="G19" s="124"/>
+      <c r="H19" s="125"/>
+      <c r="I19" s="125"/>
+      <c r="J19" s="126"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="125" t="s">
+      <c r="N19" s="91" t="s">
         <v>94</v>
       </c>
       <c r="O19" s="92"/>
@@ -3895,10 +3901,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="113" t="s">
+      <c r="U19" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V19" s="114"/>
+      <c r="V19" s="117"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -3911,10 +3917,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="113" t="s">
+      <c r="AA19" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB19" s="114"/>
+      <c r="AB19" s="117"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -3954,16 +3960,16 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="121"/>
-      <c r="H20" s="122"/>
-      <c r="I20" s="122"/>
-      <c r="J20" s="123"/>
+      <c r="G20" s="124"/>
+      <c r="H20" s="125"/>
+      <c r="I20" s="125"/>
+      <c r="J20" s="126"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="125" t="s">
+      <c r="N20" s="91" t="s">
         <v>95</v>
       </c>
       <c r="O20" s="92"/>
@@ -3977,10 +3983,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="113" t="s">
+      <c r="U20" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V20" s="114"/>
+      <c r="V20" s="117"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -3993,10 +3999,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="113" t="s">
+      <c r="AA20" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB20" s="114"/>
+      <c r="AB20" s="117"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -4034,16 +4040,16 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="121"/>
-      <c r="H21" s="122"/>
-      <c r="I21" s="122"/>
-      <c r="J21" s="123"/>
+      <c r="G21" s="124"/>
+      <c r="H21" s="125"/>
+      <c r="I21" s="125"/>
+      <c r="J21" s="126"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="125" t="s">
+      <c r="N21" s="91" t="s">
         <v>63</v>
       </c>
       <c r="O21" s="92"/>
@@ -4057,10 +4063,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="113" t="s">
+      <c r="U21" s="116" t="s">
         <v>97</v>
       </c>
-      <c r="V21" s="114"/>
+      <c r="V21" s="117"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -4073,10 +4079,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="113" t="s">
+      <c r="AA21" s="116" t="s">
         <v>99</v>
       </c>
-      <c r="AB21" s="114"/>
+      <c r="AB21" s="117"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -4110,18 +4116,18 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="124"/>
-      <c r="F22" s="122"/>
-      <c r="G22" s="122"/>
-      <c r="H22" s="122"/>
-      <c r="I22" s="122"/>
-      <c r="J22" s="123"/>
+      <c r="E22" s="127"/>
+      <c r="F22" s="125"/>
+      <c r="G22" s="125"/>
+      <c r="H22" s="125"/>
+      <c r="I22" s="125"/>
+      <c r="J22" s="126"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="125" t="s">
+      <c r="N22" s="91" t="s">
         <v>64</v>
       </c>
       <c r="O22" s="92"/>
@@ -4135,10 +4141,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="113" t="s">
+      <c r="U22" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V22" s="114"/>
+      <c r="V22" s="117"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -4151,10 +4157,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="113" t="s">
+      <c r="AA22" s="116" t="s">
         <v>97</v>
       </c>
-      <c r="AB22" s="114"/>
+      <c r="AB22" s="117"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -4194,7 +4200,7 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="120" t="s">
+      <c r="G23" s="123" t="s">
         <v>78</v>
       </c>
       <c r="H23" s="92"/>
@@ -4205,7 +4211,7 @@
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="125" t="s">
+      <c r="N23" s="91" t="s">
         <v>83</v>
       </c>
       <c r="O23" s="92"/>
@@ -4219,10 +4225,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="113" t="s">
+      <c r="U23" s="116" t="s">
         <v>98</v>
       </c>
-      <c r="V23" s="114"/>
+      <c r="V23" s="117"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -4235,10 +4241,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="113" t="s">
+      <c r="AA23" s="116" t="s">
         <v>97</v>
       </c>
-      <c r="AB23" s="114"/>
+      <c r="AB23" s="117"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -4278,7 +4284,7 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="120" t="s">
+      <c r="G24" s="123" t="s">
         <v>78</v>
       </c>
       <c r="H24" s="92"/>
@@ -4289,7 +4295,7 @@
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="125" t="s">
+      <c r="N24" s="91" t="s">
         <v>82</v>
       </c>
       <c r="O24" s="92"/>
@@ -4303,10 +4309,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="113" t="s">
+      <c r="U24" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V24" s="114"/>
+      <c r="V24" s="117"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -4319,10 +4325,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="113" t="s">
+      <c r="AA24" s="116" t="s">
         <v>99</v>
       </c>
-      <c r="AB24" s="114"/>
+      <c r="AB24" s="117"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -4360,10 +4366,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="121"/>
-      <c r="H25" s="122"/>
-      <c r="I25" s="122"/>
-      <c r="J25" s="123"/>
+      <c r="G25" s="124"/>
+      <c r="H25" s="125"/>
+      <c r="I25" s="125"/>
+      <c r="J25" s="126"/>
       <c r="K25" s="49" t="s">
         <v>40</v>
       </c>
@@ -4371,7 +4377,7 @@
         <v>156</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="125" t="s">
+      <c r="N25" s="91" t="s">
         <v>42</v>
       </c>
       <c r="O25" s="92"/>
@@ -4385,10 +4391,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="113" t="s">
+      <c r="U25" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V25" s="114"/>
+      <c r="V25" s="117"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -4401,10 +4407,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="113" t="s">
+      <c r="AA25" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB25" s="114"/>
+      <c r="AB25" s="117"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -4442,10 +4448,10 @@
       <c r="F26" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="G26" s="121"/>
-      <c r="H26" s="122"/>
-      <c r="I26" s="122"/>
-      <c r="J26" s="123"/>
+      <c r="G26" s="124"/>
+      <c r="H26" s="125"/>
+      <c r="I26" s="125"/>
+      <c r="J26" s="126"/>
       <c r="K26" s="31" t="s">
         <v>41</v>
       </c>
@@ -4453,7 +4459,7 @@
         <v>156</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="125" t="s">
+      <c r="N26" s="91" t="s">
         <v>43</v>
       </c>
       <c r="O26" s="92"/>
@@ -4467,10 +4473,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="113" t="s">
+      <c r="U26" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V26" s="114"/>
+      <c r="V26" s="117"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -4483,10 +4489,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="113" t="s">
+      <c r="AA26" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB26" s="114"/>
+      <c r="AB26" s="117"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -4518,18 +4524,18 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="124"/>
-      <c r="F27" s="122"/>
-      <c r="G27" s="122"/>
-      <c r="H27" s="122"/>
-      <c r="I27" s="122"/>
-      <c r="J27" s="123"/>
+      <c r="E27" s="127"/>
+      <c r="F27" s="125"/>
+      <c r="G27" s="125"/>
+      <c r="H27" s="125"/>
+      <c r="I27" s="125"/>
+      <c r="J27" s="126"/>
       <c r="K27" s="25" t="s">
         <v>45</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="125" t="s">
+      <c r="N27" s="91" t="s">
         <v>47</v>
       </c>
       <c r="O27" s="92"/>
@@ -4543,10 +4549,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="113" t="s">
+      <c r="U27" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="V27" s="114"/>
+      <c r="V27" s="117"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -4559,10 +4565,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="113" t="s">
+      <c r="AA27" s="116" t="s">
         <v>74</v>
       </c>
-      <c r="AB27" s="114"/>
+      <c r="AB27" s="117"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -4594,12 +4600,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="141"/>
-      <c r="F28" s="142"/>
-      <c r="G28" s="142"/>
-      <c r="H28" s="142"/>
-      <c r="I28" s="142"/>
-      <c r="J28" s="143"/>
+      <c r="E28" s="139"/>
+      <c r="F28" s="140"/>
+      <c r="G28" s="140"/>
+      <c r="H28" s="140"/>
+      <c r="I28" s="140"/>
+      <c r="J28" s="141"/>
       <c r="K28" s="52" t="s">
         <v>46</v>
       </c>
@@ -4607,11 +4613,11 @@
         <v>156</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="138" t="s">
+      <c r="N28" s="108" t="s">
         <v>93</v>
       </c>
-      <c r="O28" s="139"/>
-      <c r="P28" s="140"/>
+      <c r="O28" s="109"/>
+      <c r="P28" s="110"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -4621,10 +4627,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="150" t="s">
+      <c r="U28" s="153" t="s">
         <v>74</v>
       </c>
-      <c r="V28" s="151"/>
+      <c r="V28" s="154"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -4637,10 +4643,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="150" t="s">
+      <c r="AA28" s="153" t="s">
         <v>74</v>
       </c>
-      <c r="AB28" s="151"/>
+      <c r="AB28" s="154"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -4717,18 +4723,18 @@
       <c r="S30" s="75" t="s">
         <v>157</v>
       </c>
-      <c r="T30" s="88" t="s">
+      <c r="T30" s="86" t="s">
         <v>158</v>
       </c>
-      <c r="U30" s="88"/>
-      <c r="V30" s="88"/>
-      <c r="W30" s="88"/>
-      <c r="X30" s="88"/>
-      <c r="Y30" s="88"/>
-      <c r="Z30" s="88"/>
-      <c r="AA30" s="88"/>
-      <c r="AB30" s="88"/>
-      <c r="AC30" s="89"/>
+      <c r="U30" s="86"/>
+      <c r="V30" s="86"/>
+      <c r="W30" s="86"/>
+      <c r="X30" s="86"/>
+      <c r="Y30" s="86"/>
+      <c r="Z30" s="86"/>
+      <c r="AA30" s="86"/>
+      <c r="AB30" s="86"/>
+      <c r="AC30" s="87"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="67" t="s">
@@ -4769,18 +4775,18 @@
       <c r="S31" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="T31" s="90" t="s">
+      <c r="T31" s="88" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="90"/>
-      <c r="V31" s="90"/>
-      <c r="W31" s="90"/>
-      <c r="X31" s="90"/>
-      <c r="Y31" s="90"/>
-      <c r="Z31" s="90"/>
-      <c r="AA31" s="90"/>
-      <c r="AB31" s="90"/>
-      <c r="AC31" s="91"/>
+      <c r="U31" s="89"/>
+      <c r="V31" s="89"/>
+      <c r="W31" s="89"/>
+      <c r="X31" s="89"/>
+      <c r="Y31" s="89"/>
+      <c r="Z31" s="89"/>
+      <c r="AA31" s="89"/>
+      <c r="AB31" s="89"/>
+      <c r="AC31" s="90"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="4" t="s">
@@ -4804,7 +4810,7 @@
       <c r="S32" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="T32" s="92" t="s">
+      <c r="T32" s="91" t="s">
         <v>164</v>
       </c>
       <c r="U32" s="92"/>
@@ -4818,8 +4824,8 @@
       <c r="AC32" s="93"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="H33" s="87" t="s">
-        <v>200</v>
+      <c r="H33" s="84" t="s">
+        <v>198</v>
       </c>
       <c r="I33" s="73">
         <v>7</v>
@@ -4851,7 +4857,7 @@
       <c r="S33" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T33" s="92" t="s">
+      <c r="T33" s="91" t="s">
         <v>165</v>
       </c>
       <c r="U33" s="92"/>
@@ -4865,17 +4871,17 @@
       <c r="AC33" s="93"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="169" t="s">
+      <c r="B34" s="164" t="s">
         <v>109</v>
       </c>
-      <c r="C34" s="144" t="s">
+      <c r="C34" s="142" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="146"/>
-      <c r="E34" s="144" t="s">
+      <c r="D34" s="144"/>
+      <c r="E34" s="142" t="s">
         <v>116</v>
       </c>
-      <c r="F34" s="146"/>
+      <c r="F34" s="144"/>
       <c r="H34" s="77" t="s">
         <v>66</v>
       </c>
@@ -4884,16 +4890,16 @@
       <c r="K34" s="79"/>
       <c r="L34" s="79"/>
       <c r="M34" s="79" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="N34" s="79" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="O34" s="79" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="P34" s="80" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="R34" s="2">
         <v>3</v>
@@ -4901,7 +4907,7 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="92" t="s">
+      <c r="T34" s="91" t="s">
         <v>166</v>
       </c>
       <c r="U34" s="92"/>
@@ -4915,7 +4921,7 @@
       <c r="AC34" s="93"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="170"/>
+      <c r="B35" s="165"/>
       <c r="C35" s="64" t="s">
         <v>100</v>
       </c>
@@ -4934,7 +4940,7 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="92" t="s">
+      <c r="T35" s="91" t="s">
         <v>167</v>
       </c>
       <c r="U35" s="92"/>
@@ -4969,7 +4975,7 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="92" t="s">
+      <c r="T36" s="91" t="s">
         <v>168</v>
       </c>
       <c r="U36" s="92"/>
@@ -4998,15 +5004,15 @@
       <c r="F37" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="N37" s="179"/>
+      <c r="N37" s="85"/>
       <c r="R37" s="2">
         <v>6</v>
       </c>
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="92" t="s">
-        <v>197</v>
+      <c r="T37" s="91" t="s">
+        <v>195</v>
       </c>
       <c r="U37" s="92"/>
       <c r="V37" s="92"/>
@@ -5069,7 +5075,7 @@
       <c r="F39" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G39" s="108" t="s">
+      <c r="G39" s="111" t="s">
         <v>182</v>
       </c>
       <c r="H39" s="94"/>
@@ -5106,17 +5112,17 @@
       <c r="F40" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G40" s="110"/>
-      <c r="H40" s="111"/>
-      <c r="I40" s="111"/>
-      <c r="J40" s="112"/>
+      <c r="G40" s="113"/>
+      <c r="H40" s="114"/>
+      <c r="I40" s="114"/>
+      <c r="J40" s="115"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="92" t="s">
+      <c r="T40" s="91" t="s">
         <v>170</v>
       </c>
       <c r="U40" s="92"/>
@@ -5145,17 +5151,17 @@
       <c r="F41" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="G41" s="110"/>
-      <c r="H41" s="111"/>
-      <c r="I41" s="111"/>
-      <c r="J41" s="112"/>
+      <c r="G41" s="113"/>
+      <c r="H41" s="114"/>
+      <c r="I41" s="114"/>
+      <c r="J41" s="115"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="92" t="s">
+      <c r="T41" s="91" t="s">
         <v>171</v>
       </c>
       <c r="U41" s="92"/>
@@ -5184,7 +5190,7 @@
       <c r="F42" s="76" t="s">
         <v>176</v>
       </c>
-      <c r="G42" s="109"/>
+      <c r="G42" s="112"/>
       <c r="H42" s="96"/>
       <c r="I42" s="96"/>
       <c r="J42" s="97"/>
@@ -5194,7 +5200,7 @@
       <c r="S42" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="T42" s="92" t="s">
+      <c r="T42" s="91" t="s">
         <v>172</v>
       </c>
       <c r="U42" s="92"/>
@@ -5223,8 +5229,8 @@
       <c r="F43" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="G43" s="174" t="s">
-        <v>194</v>
+      <c r="G43" s="168" t="s">
+        <v>192</v>
       </c>
       <c r="H43" s="98"/>
       <c r="I43" s="98"/>
@@ -5235,7 +5241,7 @@
       <c r="S43" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="T43" s="92" t="s">
+      <c r="T43" s="91" t="s">
         <v>173</v>
       </c>
       <c r="U43" s="92"/>
@@ -5299,7 +5305,7 @@
       <c r="F45" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="G45" s="108" t="s">
+      <c r="G45" s="111" t="s">
         <v>181</v>
       </c>
       <c r="H45" s="94"/>
@@ -5336,7 +5342,7 @@
       <c r="F46" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G46" s="109"/>
+      <c r="G46" s="112"/>
       <c r="H46" s="96"/>
       <c r="I46" s="96"/>
       <c r="J46" s="97"/>
@@ -5346,18 +5352,18 @@
       <c r="S46" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="T46" s="92" t="s">
+      <c r="T46" s="108" t="s">
         <v>175</v>
       </c>
-      <c r="U46" s="92"/>
-      <c r="V46" s="92"/>
-      <c r="W46" s="92"/>
-      <c r="X46" s="92"/>
-      <c r="Y46" s="92"/>
-      <c r="Z46" s="92"/>
-      <c r="AA46" s="92"/>
-      <c r="AB46" s="92"/>
-      <c r="AC46" s="93"/>
+      <c r="U46" s="109"/>
+      <c r="V46" s="109"/>
+      <c r="W46" s="109"/>
+      <c r="X46" s="109"/>
+      <c r="Y46" s="109"/>
+      <c r="Z46" s="109"/>
+      <c r="AA46" s="109"/>
+      <c r="AB46" s="109"/>
+      <c r="AC46" s="110"/>
     </row>
     <row r="47" spans="2:29" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="2">
@@ -5390,13 +5396,13 @@
         <v>138</v>
       </c>
       <c r="D48" s="69" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E48" s="9" t="s">
         <v>129</v>
       </c>
       <c r="F48" s="35" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="49" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5461,180 +5467,188 @@
       <c r="J51" s="97"/>
     </row>
     <row r="52" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="171" t="s">
+      <c r="B52" s="166" t="s">
         <v>142</v>
       </c>
-      <c r="C52" s="129"/>
-      <c r="D52" s="129"/>
-      <c r="E52" s="129"/>
-      <c r="F52" s="130"/>
+      <c r="C52" s="131"/>
+      <c r="D52" s="131"/>
+      <c r="E52" s="131"/>
+      <c r="F52" s="132"/>
     </row>
     <row r="54" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B55" s="163" t="s">
+      <c r="B55" s="161" t="s">
         <v>183</v>
       </c>
-      <c r="C55" s="161" t="s">
+      <c r="C55" s="159" t="s">
         <v>185</v>
       </c>
-      <c r="D55" s="175" t="s">
+      <c r="D55" s="169" t="s">
         <v>184</v>
       </c>
-      <c r="E55" s="176"/>
+      <c r="E55" s="170"/>
     </row>
     <row r="56" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="164"/>
-      <c r="C56" s="162"/>
-      <c r="D56" s="177"/>
-      <c r="E56" s="178"/>
+      <c r="B56" s="162"/>
+      <c r="C56" s="160"/>
+      <c r="D56" s="171"/>
+      <c r="E56" s="172"/>
     </row>
     <row r="57" spans="2:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="81">
         <v>0</v>
       </c>
-      <c r="C57" s="84" t="s">
-        <v>186</v>
-      </c>
-      <c r="D57" s="165" t="s">
-        <v>190</v>
-      </c>
-      <c r="E57" s="166"/>
-    </row>
-    <row r="58" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="C57" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D57" s="177" t="s">
+        <v>207</v>
+      </c>
+      <c r="E57" s="178"/>
+    </row>
+    <row r="58" spans="2:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="82">
         <v>1</v>
       </c>
-      <c r="C58" s="85" t="s">
-        <v>187</v>
-      </c>
-      <c r="D58" s="167" t="s">
-        <v>191</v>
-      </c>
-      <c r="E58" s="168"/>
+      <c r="C58" s="173" t="s">
+        <v>203</v>
+      </c>
+      <c r="D58" s="175" t="s">
+        <v>206</v>
+      </c>
+      <c r="E58" s="163"/>
     </row>
     <row r="59" spans="2:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="82">
         <v>2</v>
       </c>
-      <c r="C59" s="37" t="s">
-        <v>188</v>
-      </c>
-      <c r="D59" s="167" t="s">
-        <v>192</v>
-      </c>
-      <c r="E59" s="168"/>
+      <c r="C59" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="D59" s="175" t="s">
+        <v>205</v>
+      </c>
+      <c r="E59" s="163"/>
     </row>
     <row r="60" spans="2:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="82">
         <v>3</v>
       </c>
-      <c r="C60" s="37" t="s">
+      <c r="C60" s="173" t="s">
+        <v>186</v>
+      </c>
+      <c r="D60" s="175" t="s">
         <v>189</v>
       </c>
-      <c r="D60" s="167" t="s">
-        <v>193</v>
-      </c>
-      <c r="E60" s="168"/>
+      <c r="E60" s="163"/>
     </row>
     <row r="61" spans="2:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="82">
         <v>4</v>
       </c>
-      <c r="C61" s="85" t="s">
-        <v>198</v>
-      </c>
-      <c r="D61" s="167" t="s">
-        <v>199</v>
-      </c>
-      <c r="E61" s="168"/>
-    </row>
-    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C61" s="38" t="s">
+        <v>187</v>
+      </c>
+      <c r="D61" s="175" t="s">
+        <v>190</v>
+      </c>
+      <c r="E61" s="163"/>
+    </row>
+    <row r="62" spans="2:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="82">
         <v>5</v>
       </c>
-      <c r="C62" s="85"/>
-      <c r="D62" s="167"/>
-      <c r="E62" s="168"/>
-    </row>
-    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C62" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="D62" s="175" t="s">
+        <v>191</v>
+      </c>
+      <c r="E62" s="163"/>
+    </row>
+    <row r="63" spans="2:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="82">
         <v>6</v>
       </c>
-      <c r="C63" s="85"/>
-      <c r="D63" s="167"/>
-      <c r="E63" s="168"/>
+      <c r="C63" s="173" t="s">
+        <v>196</v>
+      </c>
+      <c r="D63" s="175" t="s">
+        <v>197</v>
+      </c>
+      <c r="E63" s="163"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B64" s="82">
         <v>7</v>
       </c>
-      <c r="C64" s="85"/>
-      <c r="D64" s="167"/>
-      <c r="E64" s="168"/>
+      <c r="C64" s="173"/>
+      <c r="D64" s="175"/>
+      <c r="E64" s="163"/>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="82">
         <v>8</v>
       </c>
-      <c r="C65" s="85"/>
-      <c r="D65" s="167"/>
-      <c r="E65" s="168"/>
+      <c r="C65" s="173"/>
+      <c r="D65" s="175"/>
+      <c r="E65" s="163"/>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" s="82">
         <v>9</v>
       </c>
-      <c r="C66" s="85"/>
-      <c r="D66" s="167"/>
-      <c r="E66" s="168"/>
+      <c r="C66" s="173"/>
+      <c r="D66" s="175"/>
+      <c r="E66" s="163"/>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" s="82">
         <v>10</v>
       </c>
-      <c r="C67" s="85"/>
-      <c r="D67" s="167"/>
-      <c r="E67" s="168"/>
+      <c r="C67" s="173"/>
+      <c r="D67" s="175"/>
+      <c r="E67" s="163"/>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" s="82">
         <v>11</v>
       </c>
-      <c r="C68" s="85"/>
-      <c r="D68" s="167"/>
-      <c r="E68" s="168"/>
+      <c r="C68" s="173"/>
+      <c r="D68" s="175"/>
+      <c r="E68" s="163"/>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69" s="82">
         <v>12</v>
       </c>
-      <c r="C69" s="85"/>
-      <c r="D69" s="167"/>
-      <c r="E69" s="168"/>
+      <c r="C69" s="173"/>
+      <c r="D69" s="175"/>
+      <c r="E69" s="163"/>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B70" s="82">
         <v>13</v>
       </c>
-      <c r="C70" s="85"/>
-      <c r="D70" s="167"/>
-      <c r="E70" s="168"/>
+      <c r="C70" s="173"/>
+      <c r="D70" s="175"/>
+      <c r="E70" s="163"/>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B71" s="82">
         <v>14</v>
       </c>
-      <c r="C71" s="85"/>
-      <c r="D71" s="167"/>
-      <c r="E71" s="168"/>
+      <c r="C71" s="173"/>
+      <c r="D71" s="175"/>
+      <c r="E71" s="163"/>
     </row>
     <row r="72" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B72" s="83">
         <v>15</v>
       </c>
-      <c r="C72" s="86"/>
-      <c r="D72" s="172"/>
-      <c r="E72" s="173"/>
+      <c r="C72" s="174"/>
+      <c r="D72" s="176"/>
+      <c r="E72" s="167"/>
     </row>
   </sheetData>
   <mergeCells count="158">
@@ -5651,20 +5665,17 @@
     <mergeCell ref="D69:E69"/>
     <mergeCell ref="D70:E70"/>
     <mergeCell ref="D55:E56"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D57:E57"/>
     <mergeCell ref="C55:C56"/>
     <mergeCell ref="B55:B56"/>
-    <mergeCell ref="D57:E57"/>
     <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D61:E61"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="B34:B35"/>
     <mergeCell ref="B52:F52"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="AA6:AB6"/>
     <mergeCell ref="AA7:AB7"/>
     <mergeCell ref="AA28:AB28"/>
     <mergeCell ref="AA3:AB3"/>
@@ -5686,9 +5697,6 @@
     <mergeCell ref="U12:V12"/>
     <mergeCell ref="AA14:AB14"/>
     <mergeCell ref="U28:V28"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
     <mergeCell ref="N17:P17"/>
     <mergeCell ref="N19:P19"/>
     <mergeCell ref="N20:P20"/>
@@ -5696,6 +5704,8 @@
     <mergeCell ref="N23:P23"/>
     <mergeCell ref="U13:V13"/>
     <mergeCell ref="U14:V14"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="R2:R4"/>
     <mergeCell ref="U24:V24"/>
     <mergeCell ref="U25:V25"/>
     <mergeCell ref="U26:V26"/>
@@ -5720,7 +5730,6 @@
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="G21:J21"/>
-    <mergeCell ref="F16:J16"/>
     <mergeCell ref="K2:P2"/>
     <mergeCell ref="N7:P7"/>
     <mergeCell ref="N8:P8"/>
@@ -5752,6 +5761,10 @@
     <mergeCell ref="H13:J13"/>
     <mergeCell ref="H12:J12"/>
     <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="N13:P13"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
     <mergeCell ref="AA20:AB20"/>
     <mergeCell ref="AA21:AB21"/>
     <mergeCell ref="AA22:AB22"/>
@@ -5775,6 +5788,7 @@
     <mergeCell ref="U10:V10"/>
     <mergeCell ref="U11:V11"/>
     <mergeCell ref="AA23:AB23"/>
+    <mergeCell ref="AA6:AB6"/>
     <mergeCell ref="T30:AC30"/>
     <mergeCell ref="T31:AC31"/>
     <mergeCell ref="T32:AC32"/>

</xml_diff>

<commit_message>
Excepciones minimas completadas. Queda union con sistema de interrupciónes
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{635EA803-B12D-4441-BEE8-1D33FF932DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F57E3F6-5411-4067-9536-379F3D8BD3A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1660,7 +1660,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="179">
+  <cellXfs count="177">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1917,6 +1917,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2028,27 +2034,72 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2058,51 +2109,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2118,12 +2124,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2147,6 +2147,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2160,6 +2163,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2176,24 +2188,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2503,37 +2497,37 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="136" t="s">
+      <c r="B2" s="133" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="145" t="s">
+      <c r="C2" s="142" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="146"/>
-      <c r="E2" s="129" t="s">
+      <c r="D2" s="143"/>
+      <c r="E2" s="144" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="129"/>
-      <c r="G2" s="147" t="s">
+      <c r="F2" s="144"/>
+      <c r="G2" s="145" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="129"/>
-      <c r="I2" s="129" t="s">
+      <c r="H2" s="144"/>
+      <c r="I2" s="144" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="129"/>
-      <c r="K2" s="128" t="s">
+      <c r="J2" s="144"/>
+      <c r="K2" s="146" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="129"/>
-      <c r="M2" s="129"/>
-      <c r="N2" s="129"/>
-      <c r="O2" s="129"/>
-      <c r="P2" s="130"/>
-      <c r="R2" s="150" t="s">
+      <c r="L2" s="144"/>
+      <c r="M2" s="144"/>
+      <c r="N2" s="144"/>
+      <c r="O2" s="144"/>
+      <c r="P2" s="147"/>
+      <c r="R2" s="152" t="s">
         <v>66</v>
       </c>
-      <c r="S2" s="87" t="s">
+      <c r="S2" s="89" t="s">
         <v>67</v>
       </c>
       <c r="T2" s="156" t="s">
@@ -2558,7 +2552,7 @@
       <c r="AI2" s="158"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="137"/>
+      <c r="B3" s="134"/>
       <c r="C3" s="16" t="s">
         <v>80</v>
       </c>
@@ -2583,21 +2577,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="142"/>
-      <c r="L3" s="143"/>
-      <c r="M3" s="143"/>
-      <c r="N3" s="143"/>
-      <c r="O3" s="143"/>
-      <c r="P3" s="144"/>
-      <c r="R3" s="151"/>
-      <c r="S3" s="148"/>
+      <c r="K3" s="139"/>
+      <c r="L3" s="140"/>
+      <c r="M3" s="140"/>
+      <c r="N3" s="140"/>
+      <c r="O3" s="140"/>
+      <c r="P3" s="141"/>
+      <c r="R3" s="153"/>
+      <c r="S3" s="150"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="118" t="s">
+      <c r="U3" s="120" t="s">
         <v>84</v>
       </c>
-      <c r="V3" s="118"/>
+      <c r="V3" s="120"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -2637,21 +2631,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="138"/>
+      <c r="B4" s="135"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="119" t="s">
+      <c r="E4" s="121" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="131"/>
-      <c r="G4" s="131"/>
-      <c r="H4" s="131"/>
-      <c r="I4" s="131"/>
-      <c r="J4" s="132"/>
+      <c r="F4" s="148"/>
+      <c r="G4" s="148"/>
+      <c r="H4" s="148"/>
+      <c r="I4" s="148"/>
+      <c r="J4" s="149"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -2661,20 +2655,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="119" t="s">
+      <c r="N4" s="121" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="131"/>
-      <c r="P4" s="132"/>
-      <c r="R4" s="152"/>
-      <c r="S4" s="149"/>
+      <c r="O4" s="148"/>
+      <c r="P4" s="149"/>
+      <c r="R4" s="154"/>
+      <c r="S4" s="151"/>
       <c r="T4" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="U4" s="119" t="s">
+      <c r="U4" s="121" t="s">
         <v>76</v>
       </c>
-      <c r="V4" s="120"/>
+      <c r="V4" s="122"/>
       <c r="W4" s="7" t="s">
         <v>72</v>
       </c>
@@ -2687,10 +2681,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="119" t="s">
+      <c r="AA4" s="121" t="s">
         <v>73</v>
       </c>
-      <c r="AB4" s="120"/>
+      <c r="AB4" s="122"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -2722,22 +2716,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="133"/>
-      <c r="F5" s="134"/>
-      <c r="G5" s="134"/>
-      <c r="H5" s="134"/>
-      <c r="I5" s="134"/>
-      <c r="J5" s="135"/>
+      <c r="E5" s="125"/>
+      <c r="F5" s="126"/>
+      <c r="G5" s="126"/>
+      <c r="H5" s="126"/>
+      <c r="I5" s="126"/>
+      <c r="J5" s="127"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="88" t="s">
+      <c r="N5" s="90" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="89"/>
-      <c r="P5" s="90"/>
+      <c r="O5" s="91"/>
+      <c r="P5" s="92"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -2747,10 +2741,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="121" t="s">
+      <c r="U5" s="123" t="s">
         <v>74</v>
       </c>
-      <c r="V5" s="122"/>
+      <c r="V5" s="124"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -2763,10 +2757,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="121" t="s">
+      <c r="AA5" s="123" t="s">
         <v>74</v>
       </c>
-      <c r="AB5" s="122"/>
+      <c r="AB5" s="124"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -2798,12 +2792,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="127"/>
-      <c r="F6" s="125"/>
-      <c r="G6" s="125"/>
-      <c r="H6" s="125"/>
-      <c r="I6" s="125"/>
-      <c r="J6" s="126"/>
+      <c r="E6" s="132"/>
+      <c r="F6" s="129"/>
+      <c r="G6" s="129"/>
+      <c r="H6" s="129"/>
+      <c r="I6" s="129"/>
+      <c r="J6" s="130"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -2811,11 +2805,11 @@
         <v>156</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="91" t="s">
+      <c r="N6" s="93" t="s">
         <v>96</v>
       </c>
-      <c r="O6" s="92"/>
-      <c r="P6" s="93"/>
+      <c r="O6" s="94"/>
+      <c r="P6" s="95"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -2825,10 +2819,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="116" t="s">
+      <c r="U6" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V6" s="117"/>
+      <c r="V6" s="119"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -2841,10 +2835,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="116" t="s">
+      <c r="AA6" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB6" s="117"/>
+      <c r="AB6" s="119"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -2885,9 +2879,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="124"/>
-      <c r="I7" s="125"/>
-      <c r="J7" s="126"/>
+      <c r="H7" s="128"/>
+      <c r="I7" s="129"/>
+      <c r="J7" s="130"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -2895,11 +2889,11 @@
       <c r="M7" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N7" s="91" t="s">
+      <c r="N7" s="93" t="s">
         <v>53</v>
       </c>
-      <c r="O7" s="92"/>
-      <c r="P7" s="93"/>
+      <c r="O7" s="94"/>
+      <c r="P7" s="95"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -2909,10 +2903,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="116" t="s">
+      <c r="U7" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V7" s="117"/>
+      <c r="V7" s="119"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -2925,10 +2919,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="116" t="s">
+      <c r="AA7" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB7" s="117"/>
+      <c r="AB7" s="119"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -2969,9 +2963,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="124"/>
-      <c r="I8" s="125"/>
-      <c r="J8" s="126"/>
+      <c r="H8" s="128"/>
+      <c r="I8" s="129"/>
+      <c r="J8" s="130"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -2979,11 +2973,11 @@
       <c r="M8" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N8" s="91" t="s">
+      <c r="N8" s="93" t="s">
         <v>54</v>
       </c>
-      <c r="O8" s="92"/>
-      <c r="P8" s="93"/>
+      <c r="O8" s="94"/>
+      <c r="P8" s="95"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -2993,10 +2987,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="116" t="s">
+      <c r="U8" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V8" s="117"/>
+      <c r="V8" s="119"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -3009,10 +3003,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="116" t="s">
+      <c r="AA8" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB8" s="117"/>
+      <c r="AB8" s="119"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -3053,9 +3047,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="124"/>
-      <c r="I9" s="125"/>
-      <c r="J9" s="126"/>
+      <c r="H9" s="128"/>
+      <c r="I9" s="129"/>
+      <c r="J9" s="130"/>
       <c r="K9" s="37" t="s">
         <v>48</v>
       </c>
@@ -3063,11 +3057,11 @@
       <c r="M9" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N9" s="91" t="s">
+      <c r="N9" s="93" t="s">
         <v>55</v>
       </c>
-      <c r="O9" s="92"/>
-      <c r="P9" s="93"/>
+      <c r="O9" s="94"/>
+      <c r="P9" s="95"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -3077,10 +3071,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="116" t="s">
+      <c r="U9" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V9" s="117"/>
+      <c r="V9" s="119"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -3093,10 +3087,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="116" t="s">
+      <c r="AA9" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB9" s="117"/>
+      <c r="AB9" s="119"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -3137,9 +3131,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="124"/>
-      <c r="I10" s="125"/>
-      <c r="J10" s="126"/>
+      <c r="H10" s="128"/>
+      <c r="I10" s="129"/>
+      <c r="J10" s="130"/>
       <c r="K10" s="37" t="s">
         <v>49</v>
       </c>
@@ -3147,11 +3141,11 @@
       <c r="M10" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N10" s="91" t="s">
+      <c r="N10" s="93" t="s">
         <v>56</v>
       </c>
-      <c r="O10" s="92"/>
-      <c r="P10" s="93"/>
+      <c r="O10" s="94"/>
+      <c r="P10" s="95"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -3161,10 +3155,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="116" t="s">
+      <c r="U10" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V10" s="117"/>
+      <c r="V10" s="119"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -3177,10 +3171,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="116" t="s">
+      <c r="AA10" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB10" s="117"/>
+      <c r="AB10" s="119"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -3221,9 +3215,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="124"/>
-      <c r="I11" s="125"/>
-      <c r="J11" s="126"/>
+      <c r="H11" s="128"/>
+      <c r="I11" s="129"/>
+      <c r="J11" s="130"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -3231,11 +3225,11 @@
       <c r="M11" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N11" s="91" t="s">
+      <c r="N11" s="93" t="s">
         <v>57</v>
       </c>
-      <c r="O11" s="92"/>
-      <c r="P11" s="93"/>
+      <c r="O11" s="94"/>
+      <c r="P11" s="95"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -3245,10 +3239,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="116" t="s">
+      <c r="U11" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V11" s="117"/>
+      <c r="V11" s="119"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -3261,10 +3255,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="116" t="s">
+      <c r="AA11" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB11" s="117"/>
+      <c r="AB11" s="119"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -3305,9 +3299,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="124"/>
-      <c r="I12" s="125"/>
-      <c r="J12" s="126"/>
+      <c r="H12" s="128"/>
+      <c r="I12" s="129"/>
+      <c r="J12" s="130"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -3315,11 +3309,11 @@
       <c r="M12" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N12" s="91" t="s">
+      <c r="N12" s="93" t="s">
         <v>58</v>
       </c>
-      <c r="O12" s="92"/>
-      <c r="P12" s="93"/>
+      <c r="O12" s="94"/>
+      <c r="P12" s="95"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -3329,10 +3323,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="116" t="s">
+      <c r="U12" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V12" s="117"/>
+      <c r="V12" s="119"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -3345,10 +3339,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="116" t="s">
+      <c r="AA12" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB12" s="117"/>
+      <c r="AB12" s="119"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -3389,9 +3383,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="124"/>
-      <c r="I13" s="125"/>
-      <c r="J13" s="126"/>
+      <c r="H13" s="128"/>
+      <c r="I13" s="129"/>
+      <c r="J13" s="130"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -3399,11 +3393,11 @@
       <c r="M13" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N13" s="91" t="s">
+      <c r="N13" s="93" t="s">
         <v>59</v>
       </c>
-      <c r="O13" s="92"/>
-      <c r="P13" s="93"/>
+      <c r="O13" s="94"/>
+      <c r="P13" s="95"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -3413,10 +3407,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="116" t="s">
+      <c r="U13" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V13" s="117"/>
+      <c r="V13" s="119"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -3429,10 +3423,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="116" t="s">
+      <c r="AA13" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB13" s="117"/>
+      <c r="AB13" s="119"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -3473,9 +3467,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="124"/>
-      <c r="I14" s="125"/>
-      <c r="J14" s="126"/>
+      <c r="H14" s="128"/>
+      <c r="I14" s="129"/>
+      <c r="J14" s="130"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -3483,11 +3477,11 @@
       <c r="M14" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N14" s="91" t="s">
+      <c r="N14" s="93" t="s">
         <v>60</v>
       </c>
-      <c r="O14" s="92"/>
-      <c r="P14" s="93"/>
+      <c r="O14" s="94"/>
+      <c r="P14" s="95"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -3497,10 +3491,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="116" t="s">
+      <c r="U14" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V14" s="117"/>
+      <c r="V14" s="119"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -3513,10 +3507,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="116" t="s">
+      <c r="AA14" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB14" s="117"/>
+      <c r="AB14" s="119"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -3557,9 +3551,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="124"/>
-      <c r="I15" s="125"/>
-      <c r="J15" s="126"/>
+      <c r="H15" s="128"/>
+      <c r="I15" s="129"/>
+      <c r="J15" s="130"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -3567,11 +3561,11 @@
       <c r="M15" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N15" s="91" t="s">
+      <c r="N15" s="93" t="s">
         <v>61</v>
       </c>
-      <c r="O15" s="92"/>
-      <c r="P15" s="93"/>
+      <c r="O15" s="94"/>
+      <c r="P15" s="95"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -3581,10 +3575,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="116" t="s">
+      <c r="U15" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V15" s="117"/>
+      <c r="V15" s="119"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -3597,10 +3591,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="116" t="s">
+      <c r="AA15" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB15" s="117"/>
+      <c r="AB15" s="119"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -3635,21 +3629,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="124"/>
-      <c r="G16" s="125"/>
-      <c r="H16" s="125"/>
-      <c r="I16" s="125"/>
-      <c r="J16" s="126"/>
+      <c r="F16" s="128"/>
+      <c r="G16" s="129"/>
+      <c r="H16" s="129"/>
+      <c r="I16" s="129"/>
+      <c r="J16" s="130"/>
       <c r="K16" s="40" t="s">
         <v>50</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="91" t="s">
+      <c r="N16" s="93" t="s">
         <v>51</v>
       </c>
-      <c r="O16" s="92"/>
-      <c r="P16" s="93"/>
+      <c r="O16" s="94"/>
+      <c r="P16" s="95"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -3659,10 +3653,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="116" t="s">
+      <c r="U16" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V16" s="117"/>
+      <c r="V16" s="119"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -3675,10 +3669,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="116" t="s">
+      <c r="AA16" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB16" s="117"/>
+      <c r="AB16" s="119"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -3714,22 +3708,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="123" t="s">
+      <c r="G17" s="131" t="s">
         <v>77</v>
       </c>
-      <c r="H17" s="92"/>
-      <c r="I17" s="92"/>
-      <c r="J17" s="93"/>
+      <c r="H17" s="94"/>
+      <c r="I17" s="94"/>
+      <c r="J17" s="95"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="91" t="s">
+      <c r="N17" s="93" t="s">
         <v>65</v>
       </c>
-      <c r="O17" s="92"/>
-      <c r="P17" s="93"/>
+      <c r="O17" s="94"/>
+      <c r="P17" s="95"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -3739,10 +3733,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="116" t="s">
+      <c r="U17" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V17" s="117"/>
+      <c r="V17" s="119"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -3755,10 +3749,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="116" t="s">
+      <c r="AA17" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB17" s="117"/>
+      <c r="AB17" s="119"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -3794,12 +3788,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="123" t="s">
+      <c r="G18" s="131" t="s">
         <v>77</v>
       </c>
-      <c r="H18" s="92"/>
-      <c r="I18" s="92"/>
-      <c r="J18" s="93"/>
+      <c r="H18" s="94"/>
+      <c r="I18" s="94"/>
+      <c r="J18" s="95"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -3807,11 +3801,11 @@
       <c r="M18" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N18" s="91" t="s">
+      <c r="N18" s="93" t="s">
         <v>62</v>
       </c>
-      <c r="O18" s="92"/>
-      <c r="P18" s="93"/>
+      <c r="O18" s="94"/>
+      <c r="P18" s="95"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -3821,10 +3815,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="116" t="s">
+      <c r="U18" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V18" s="117"/>
+      <c r="V18" s="119"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -3837,10 +3831,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="116" t="s">
+      <c r="AA18" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB18" s="117"/>
+      <c r="AB18" s="119"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -3878,20 +3872,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="124"/>
-      <c r="H19" s="125"/>
-      <c r="I19" s="125"/>
-      <c r="J19" s="126"/>
+      <c r="G19" s="128"/>
+      <c r="H19" s="129"/>
+      <c r="I19" s="129"/>
+      <c r="J19" s="130"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="91" t="s">
+      <c r="N19" s="93" t="s">
         <v>94</v>
       </c>
-      <c r="O19" s="92"/>
-      <c r="P19" s="93"/>
+      <c r="O19" s="94"/>
+      <c r="P19" s="95"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -3901,10 +3895,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="116" t="s">
+      <c r="U19" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V19" s="117"/>
+      <c r="V19" s="119"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -3917,10 +3911,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="116" t="s">
+      <c r="AA19" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB19" s="117"/>
+      <c r="AB19" s="119"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -3960,20 +3954,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="124"/>
-      <c r="H20" s="125"/>
-      <c r="I20" s="125"/>
-      <c r="J20" s="126"/>
+      <c r="G20" s="128"/>
+      <c r="H20" s="129"/>
+      <c r="I20" s="129"/>
+      <c r="J20" s="130"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="91" t="s">
+      <c r="N20" s="93" t="s">
         <v>95</v>
       </c>
-      <c r="O20" s="92"/>
-      <c r="P20" s="93"/>
+      <c r="O20" s="94"/>
+      <c r="P20" s="95"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -3983,10 +3977,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="116" t="s">
+      <c r="U20" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V20" s="117"/>
+      <c r="V20" s="119"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -3999,10 +3993,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="116" t="s">
+      <c r="AA20" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB20" s="117"/>
+      <c r="AB20" s="119"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -4040,20 +4034,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="124"/>
-      <c r="H21" s="125"/>
-      <c r="I21" s="125"/>
-      <c r="J21" s="126"/>
+      <c r="G21" s="128"/>
+      <c r="H21" s="129"/>
+      <c r="I21" s="129"/>
+      <c r="J21" s="130"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="91" t="s">
+      <c r="N21" s="93" t="s">
         <v>63</v>
       </c>
-      <c r="O21" s="92"/>
-      <c r="P21" s="93"/>
+      <c r="O21" s="94"/>
+      <c r="P21" s="95"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -4063,10 +4057,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="116" t="s">
+      <c r="U21" s="118" t="s">
         <v>97</v>
       </c>
-      <c r="V21" s="117"/>
+      <c r="V21" s="119"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -4079,10 +4073,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="116" t="s">
+      <c r="AA21" s="118" t="s">
         <v>99</v>
       </c>
-      <c r="AB21" s="117"/>
+      <c r="AB21" s="119"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -4116,22 +4110,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="127"/>
-      <c r="F22" s="125"/>
-      <c r="G22" s="125"/>
-      <c r="H22" s="125"/>
-      <c r="I22" s="125"/>
-      <c r="J22" s="126"/>
+      <c r="E22" s="132"/>
+      <c r="F22" s="129"/>
+      <c r="G22" s="129"/>
+      <c r="H22" s="129"/>
+      <c r="I22" s="129"/>
+      <c r="J22" s="130"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="91" t="s">
+      <c r="N22" s="93" t="s">
         <v>64</v>
       </c>
-      <c r="O22" s="92"/>
-      <c r="P22" s="93"/>
+      <c r="O22" s="94"/>
+      <c r="P22" s="95"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -4141,10 +4135,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="116" t="s">
+      <c r="U22" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V22" s="117"/>
+      <c r="V22" s="119"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -4157,10 +4151,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="116" t="s">
+      <c r="AA22" s="118" t="s">
         <v>97</v>
       </c>
-      <c r="AB22" s="117"/>
+      <c r="AB22" s="119"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -4200,22 +4194,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="123" t="s">
+      <c r="G23" s="131" t="s">
         <v>78</v>
       </c>
-      <c r="H23" s="92"/>
-      <c r="I23" s="92"/>
-      <c r="J23" s="93"/>
+      <c r="H23" s="94"/>
+      <c r="I23" s="94"/>
+      <c r="J23" s="95"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="91" t="s">
+      <c r="N23" s="93" t="s">
         <v>83</v>
       </c>
-      <c r="O23" s="92"/>
-      <c r="P23" s="93"/>
+      <c r="O23" s="94"/>
+      <c r="P23" s="95"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -4225,10 +4219,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="116" t="s">
+      <c r="U23" s="118" t="s">
         <v>98</v>
       </c>
-      <c r="V23" s="117"/>
+      <c r="V23" s="119"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -4241,10 +4235,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="116" t="s">
+      <c r="AA23" s="118" t="s">
         <v>97</v>
       </c>
-      <c r="AB23" s="117"/>
+      <c r="AB23" s="119"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -4284,22 +4278,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="123" t="s">
+      <c r="G24" s="131" t="s">
         <v>78</v>
       </c>
-      <c r="H24" s="92"/>
-      <c r="I24" s="92"/>
-      <c r="J24" s="93"/>
+      <c r="H24" s="94"/>
+      <c r="I24" s="94"/>
+      <c r="J24" s="95"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="91" t="s">
+      <c r="N24" s="93" t="s">
         <v>82</v>
       </c>
-      <c r="O24" s="92"/>
-      <c r="P24" s="93"/>
+      <c r="O24" s="94"/>
+      <c r="P24" s="95"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -4309,10 +4303,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="116" t="s">
+      <c r="U24" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V24" s="117"/>
+      <c r="V24" s="119"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -4325,10 +4319,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="116" t="s">
+      <c r="AA24" s="118" t="s">
         <v>99</v>
       </c>
-      <c r="AB24" s="117"/>
+      <c r="AB24" s="119"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -4366,10 +4360,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="124"/>
-      <c r="H25" s="125"/>
-      <c r="I25" s="125"/>
-      <c r="J25" s="126"/>
+      <c r="G25" s="128"/>
+      <c r="H25" s="129"/>
+      <c r="I25" s="129"/>
+      <c r="J25" s="130"/>
       <c r="K25" s="49" t="s">
         <v>40</v>
       </c>
@@ -4377,11 +4371,11 @@
         <v>156</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="91" t="s">
+      <c r="N25" s="93" t="s">
         <v>42</v>
       </c>
-      <c r="O25" s="92"/>
-      <c r="P25" s="93"/>
+      <c r="O25" s="94"/>
+      <c r="P25" s="95"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -4391,10 +4385,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="116" t="s">
+      <c r="U25" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V25" s="117"/>
+      <c r="V25" s="119"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -4407,10 +4401,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="116" t="s">
+      <c r="AA25" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB25" s="117"/>
+      <c r="AB25" s="119"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -4448,10 +4442,10 @@
       <c r="F26" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="G26" s="124"/>
-      <c r="H26" s="125"/>
-      <c r="I26" s="125"/>
-      <c r="J26" s="126"/>
+      <c r="G26" s="128"/>
+      <c r="H26" s="129"/>
+      <c r="I26" s="129"/>
+      <c r="J26" s="130"/>
       <c r="K26" s="31" t="s">
         <v>41</v>
       </c>
@@ -4459,11 +4453,11 @@
         <v>156</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="91" t="s">
+      <c r="N26" s="93" t="s">
         <v>43</v>
       </c>
-      <c r="O26" s="92"/>
-      <c r="P26" s="93"/>
+      <c r="O26" s="94"/>
+      <c r="P26" s="95"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -4473,10 +4467,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="116" t="s">
+      <c r="U26" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V26" s="117"/>
+      <c r="V26" s="119"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -4489,10 +4483,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="116" t="s">
+      <c r="AA26" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB26" s="117"/>
+      <c r="AB26" s="119"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -4524,22 +4518,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="127"/>
-      <c r="F27" s="125"/>
-      <c r="G27" s="125"/>
-      <c r="H27" s="125"/>
-      <c r="I27" s="125"/>
-      <c r="J27" s="126"/>
+      <c r="E27" s="132"/>
+      <c r="F27" s="129"/>
+      <c r="G27" s="129"/>
+      <c r="H27" s="129"/>
+      <c r="I27" s="129"/>
+      <c r="J27" s="130"/>
       <c r="K27" s="25" t="s">
         <v>45</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="91" t="s">
+      <c r="N27" s="93" t="s">
         <v>47</v>
       </c>
-      <c r="O27" s="92"/>
-      <c r="P27" s="93"/>
+      <c r="O27" s="94"/>
+      <c r="P27" s="95"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -4549,10 +4543,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="116" t="s">
+      <c r="U27" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="V27" s="117"/>
+      <c r="V27" s="119"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -4565,10 +4559,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="116" t="s">
+      <c r="AA27" s="118" t="s">
         <v>74</v>
       </c>
-      <c r="AB27" s="117"/>
+      <c r="AB27" s="119"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -4600,12 +4594,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="139"/>
-      <c r="F28" s="140"/>
-      <c r="G28" s="140"/>
-      <c r="H28" s="140"/>
-      <c r="I28" s="140"/>
-      <c r="J28" s="141"/>
+      <c r="E28" s="136"/>
+      <c r="F28" s="137"/>
+      <c r="G28" s="137"/>
+      <c r="H28" s="137"/>
+      <c r="I28" s="137"/>
+      <c r="J28" s="138"/>
       <c r="K28" s="52" t="s">
         <v>46</v>
       </c>
@@ -4613,11 +4607,11 @@
         <v>156</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="108" t="s">
+      <c r="N28" s="110" t="s">
         <v>93</v>
       </c>
-      <c r="O28" s="109"/>
-      <c r="P28" s="110"/>
+      <c r="O28" s="111"/>
+      <c r="P28" s="112"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -4627,10 +4621,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="153" t="s">
+      <c r="U28" s="168" t="s">
         <v>74</v>
       </c>
-      <c r="V28" s="154"/>
+      <c r="V28" s="169"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -4643,10 +4637,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="153" t="s">
+      <c r="AA28" s="168" t="s">
         <v>74</v>
       </c>
-      <c r="AB28" s="154"/>
+      <c r="AB28" s="169"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -4723,18 +4717,18 @@
       <c r="S30" s="75" t="s">
         <v>157</v>
       </c>
-      <c r="T30" s="86" t="s">
+      <c r="T30" s="88" t="s">
         <v>158</v>
       </c>
-      <c r="U30" s="86"/>
-      <c r="V30" s="86"/>
-      <c r="W30" s="86"/>
-      <c r="X30" s="86"/>
-      <c r="Y30" s="86"/>
-      <c r="Z30" s="86"/>
-      <c r="AA30" s="86"/>
-      <c r="AB30" s="86"/>
-      <c r="AC30" s="87"/>
+      <c r="U30" s="88"/>
+      <c r="V30" s="88"/>
+      <c r="W30" s="88"/>
+      <c r="X30" s="88"/>
+      <c r="Y30" s="88"/>
+      <c r="Z30" s="88"/>
+      <c r="AA30" s="88"/>
+      <c r="AB30" s="88"/>
+      <c r="AC30" s="89"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="67" t="s">
@@ -4775,18 +4769,18 @@
       <c r="S31" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="T31" s="88" t="s">
+      <c r="T31" s="90" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="89"/>
-      <c r="V31" s="89"/>
-      <c r="W31" s="89"/>
-      <c r="X31" s="89"/>
-      <c r="Y31" s="89"/>
-      <c r="Z31" s="89"/>
-      <c r="AA31" s="89"/>
-      <c r="AB31" s="89"/>
-      <c r="AC31" s="90"/>
+      <c r="U31" s="91"/>
+      <c r="V31" s="91"/>
+      <c r="W31" s="91"/>
+      <c r="X31" s="91"/>
+      <c r="Y31" s="91"/>
+      <c r="Z31" s="91"/>
+      <c r="AA31" s="91"/>
+      <c r="AB31" s="91"/>
+      <c r="AC31" s="92"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="4" t="s">
@@ -4810,18 +4804,18 @@
       <c r="S32" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="T32" s="91" t="s">
+      <c r="T32" s="93" t="s">
         <v>164</v>
       </c>
-      <c r="U32" s="92"/>
-      <c r="V32" s="92"/>
-      <c r="W32" s="92"/>
-      <c r="X32" s="92"/>
-      <c r="Y32" s="92"/>
-      <c r="Z32" s="92"/>
-      <c r="AA32" s="92"/>
-      <c r="AB32" s="92"/>
-      <c r="AC32" s="93"/>
+      <c r="U32" s="94"/>
+      <c r="V32" s="94"/>
+      <c r="W32" s="94"/>
+      <c r="X32" s="94"/>
+      <c r="Y32" s="94"/>
+      <c r="Z32" s="94"/>
+      <c r="AA32" s="94"/>
+      <c r="AB32" s="94"/>
+      <c r="AC32" s="95"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H33" s="84" t="s">
@@ -4857,31 +4851,31 @@
       <c r="S33" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T33" s="91" t="s">
+      <c r="T33" s="93" t="s">
         <v>165</v>
       </c>
-      <c r="U33" s="92"/>
-      <c r="V33" s="92"/>
-      <c r="W33" s="92"/>
-      <c r="X33" s="92"/>
-      <c r="Y33" s="92"/>
-      <c r="Z33" s="92"/>
-      <c r="AA33" s="92"/>
-      <c r="AB33" s="92"/>
-      <c r="AC33" s="93"/>
+      <c r="U33" s="94"/>
+      <c r="V33" s="94"/>
+      <c r="W33" s="94"/>
+      <c r="X33" s="94"/>
+      <c r="Y33" s="94"/>
+      <c r="Z33" s="94"/>
+      <c r="AA33" s="94"/>
+      <c r="AB33" s="94"/>
+      <c r="AC33" s="95"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="164" t="s">
+      <c r="B34" s="165" t="s">
         <v>109</v>
       </c>
-      <c r="C34" s="142" t="s">
+      <c r="C34" s="139" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="144"/>
-      <c r="E34" s="142" t="s">
+      <c r="D34" s="141"/>
+      <c r="E34" s="139" t="s">
         <v>116</v>
       </c>
-      <c r="F34" s="144"/>
+      <c r="F34" s="141"/>
       <c r="H34" s="77" t="s">
         <v>66</v>
       </c>
@@ -4907,21 +4901,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="91" t="s">
+      <c r="T34" s="93" t="s">
         <v>166</v>
       </c>
-      <c r="U34" s="92"/>
-      <c r="V34" s="92"/>
-      <c r="W34" s="92"/>
-      <c r="X34" s="92"/>
-      <c r="Y34" s="92"/>
-      <c r="Z34" s="92"/>
-      <c r="AA34" s="92"/>
-      <c r="AB34" s="92"/>
-      <c r="AC34" s="93"/>
+      <c r="U34" s="94"/>
+      <c r="V34" s="94"/>
+      <c r="W34" s="94"/>
+      <c r="X34" s="94"/>
+      <c r="Y34" s="94"/>
+      <c r="Z34" s="94"/>
+      <c r="AA34" s="94"/>
+      <c r="AB34" s="94"/>
+      <c r="AC34" s="95"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="165"/>
+      <c r="B35" s="166"/>
       <c r="C35" s="64" t="s">
         <v>100</v>
       </c>
@@ -4940,18 +4934,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="91" t="s">
+      <c r="T35" s="93" t="s">
         <v>167</v>
       </c>
-      <c r="U35" s="92"/>
-      <c r="V35" s="92"/>
-      <c r="W35" s="92"/>
-      <c r="X35" s="92"/>
-      <c r="Y35" s="92"/>
-      <c r="Z35" s="92"/>
-      <c r="AA35" s="92"/>
-      <c r="AB35" s="92"/>
-      <c r="AC35" s="93"/>
+      <c r="U35" s="94"/>
+      <c r="V35" s="94"/>
+      <c r="W35" s="94"/>
+      <c r="X35" s="94"/>
+      <c r="Y35" s="94"/>
+      <c r="Z35" s="94"/>
+      <c r="AA35" s="94"/>
+      <c r="AB35" s="94"/>
+      <c r="AC35" s="95"/>
     </row>
     <row r="36" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B36" s="1">
@@ -4975,18 +4969,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="91" t="s">
+      <c r="T36" s="93" t="s">
         <v>168</v>
       </c>
-      <c r="U36" s="92"/>
-      <c r="V36" s="92"/>
-      <c r="W36" s="92"/>
-      <c r="X36" s="92"/>
-      <c r="Y36" s="92"/>
-      <c r="Z36" s="92"/>
-      <c r="AA36" s="92"/>
-      <c r="AB36" s="92"/>
-      <c r="AC36" s="93"/>
+      <c r="U36" s="94"/>
+      <c r="V36" s="94"/>
+      <c r="W36" s="94"/>
+      <c r="X36" s="94"/>
+      <c r="Y36" s="94"/>
+      <c r="Z36" s="94"/>
+      <c r="AA36" s="94"/>
+      <c r="AB36" s="94"/>
+      <c r="AC36" s="95"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="2">
@@ -5011,18 +5005,18 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="91" t="s">
+      <c r="T37" s="93" t="s">
         <v>195</v>
       </c>
-      <c r="U37" s="92"/>
-      <c r="V37" s="92"/>
-      <c r="W37" s="92"/>
-      <c r="X37" s="92"/>
-      <c r="Y37" s="92"/>
-      <c r="Z37" s="92"/>
-      <c r="AA37" s="92"/>
-      <c r="AB37" s="92"/>
-      <c r="AC37" s="93"/>
+      <c r="U37" s="94"/>
+      <c r="V37" s="94"/>
+      <c r="W37" s="94"/>
+      <c r="X37" s="94"/>
+      <c r="Y37" s="94"/>
+      <c r="Z37" s="94"/>
+      <c r="AA37" s="94"/>
+      <c r="AB37" s="94"/>
+      <c r="AC37" s="95"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="2">
@@ -5043,21 +5037,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="100" t="s">
+      <c r="S38" s="102" t="s">
         <v>73</v>
       </c>
-      <c r="T38" s="102" t="s">
+      <c r="T38" s="104" t="s">
         <v>169</v>
       </c>
-      <c r="U38" s="103"/>
-      <c r="V38" s="103"/>
-      <c r="W38" s="103"/>
-      <c r="X38" s="103"/>
-      <c r="Y38" s="103"/>
-      <c r="Z38" s="103"/>
-      <c r="AA38" s="103"/>
-      <c r="AB38" s="103"/>
-      <c r="AC38" s="104"/>
+      <c r="U38" s="105"/>
+      <c r="V38" s="105"/>
+      <c r="W38" s="105"/>
+      <c r="X38" s="105"/>
+      <c r="Y38" s="105"/>
+      <c r="Z38" s="105"/>
+      <c r="AA38" s="105"/>
+      <c r="AB38" s="105"/>
+      <c r="AC38" s="106"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="2">
@@ -5075,26 +5069,26 @@
       <c r="F39" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G39" s="111" t="s">
+      <c r="G39" s="113" t="s">
         <v>182</v>
       </c>
-      <c r="H39" s="94"/>
-      <c r="I39" s="94"/>
-      <c r="J39" s="95"/>
+      <c r="H39" s="96"/>
+      <c r="I39" s="96"/>
+      <c r="J39" s="97"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="101"/>
-      <c r="T39" s="105"/>
-      <c r="U39" s="106"/>
-      <c r="V39" s="106"/>
-      <c r="W39" s="106"/>
-      <c r="X39" s="106"/>
-      <c r="Y39" s="106"/>
-      <c r="Z39" s="106"/>
-      <c r="AA39" s="106"/>
-      <c r="AB39" s="106"/>
-      <c r="AC39" s="107"/>
+      <c r="S39" s="103"/>
+      <c r="T39" s="107"/>
+      <c r="U39" s="108"/>
+      <c r="V39" s="108"/>
+      <c r="W39" s="108"/>
+      <c r="X39" s="108"/>
+      <c r="Y39" s="108"/>
+      <c r="Z39" s="108"/>
+      <c r="AA39" s="108"/>
+      <c r="AB39" s="108"/>
+      <c r="AC39" s="109"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="2">
@@ -5112,28 +5106,28 @@
       <c r="F40" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G40" s="113"/>
-      <c r="H40" s="114"/>
-      <c r="I40" s="114"/>
-      <c r="J40" s="115"/>
+      <c r="G40" s="115"/>
+      <c r="H40" s="116"/>
+      <c r="I40" s="116"/>
+      <c r="J40" s="117"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="91" t="s">
+      <c r="T40" s="93" t="s">
         <v>170</v>
       </c>
-      <c r="U40" s="92"/>
-      <c r="V40" s="92"/>
-      <c r="W40" s="92"/>
-      <c r="X40" s="92"/>
-      <c r="Y40" s="92"/>
-      <c r="Z40" s="92"/>
-      <c r="AA40" s="92"/>
-      <c r="AB40" s="92"/>
-      <c r="AC40" s="93"/>
+      <c r="U40" s="94"/>
+      <c r="V40" s="94"/>
+      <c r="W40" s="94"/>
+      <c r="X40" s="94"/>
+      <c r="Y40" s="94"/>
+      <c r="Z40" s="94"/>
+      <c r="AA40" s="94"/>
+      <c r="AB40" s="94"/>
+      <c r="AC40" s="95"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="2">
@@ -5151,28 +5145,28 @@
       <c r="F41" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="G41" s="113"/>
-      <c r="H41" s="114"/>
-      <c r="I41" s="114"/>
-      <c r="J41" s="115"/>
+      <c r="G41" s="115"/>
+      <c r="H41" s="116"/>
+      <c r="I41" s="116"/>
+      <c r="J41" s="117"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="91" t="s">
+      <c r="T41" s="93" t="s">
         <v>171</v>
       </c>
-      <c r="U41" s="92"/>
-      <c r="V41" s="92"/>
-      <c r="W41" s="92"/>
-      <c r="X41" s="92"/>
-      <c r="Y41" s="92"/>
-      <c r="Z41" s="92"/>
-      <c r="AA41" s="92"/>
-      <c r="AB41" s="92"/>
-      <c r="AC41" s="93"/>
+      <c r="U41" s="94"/>
+      <c r="V41" s="94"/>
+      <c r="W41" s="94"/>
+      <c r="X41" s="94"/>
+      <c r="Y41" s="94"/>
+      <c r="Z41" s="94"/>
+      <c r="AA41" s="94"/>
+      <c r="AB41" s="94"/>
+      <c r="AC41" s="95"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="2">
@@ -5190,28 +5184,28 @@
       <c r="F42" s="76" t="s">
         <v>176</v>
       </c>
-      <c r="G42" s="112"/>
-      <c r="H42" s="96"/>
-      <c r="I42" s="96"/>
-      <c r="J42" s="97"/>
+      <c r="G42" s="114"/>
+      <c r="H42" s="98"/>
+      <c r="I42" s="98"/>
+      <c r="J42" s="99"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="T42" s="91" t="s">
+      <c r="T42" s="93" t="s">
         <v>172</v>
       </c>
-      <c r="U42" s="92"/>
-      <c r="V42" s="92"/>
-      <c r="W42" s="92"/>
-      <c r="X42" s="92"/>
-      <c r="Y42" s="92"/>
-      <c r="Z42" s="92"/>
-      <c r="AA42" s="92"/>
-      <c r="AB42" s="92"/>
-      <c r="AC42" s="93"/>
+      <c r="U42" s="94"/>
+      <c r="V42" s="94"/>
+      <c r="W42" s="94"/>
+      <c r="X42" s="94"/>
+      <c r="Y42" s="94"/>
+      <c r="Z42" s="94"/>
+      <c r="AA42" s="94"/>
+      <c r="AB42" s="94"/>
+      <c r="AC42" s="95"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="2">
@@ -5229,30 +5223,30 @@
       <c r="F43" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="G43" s="168" t="s">
+      <c r="G43" s="172" t="s">
         <v>192</v>
       </c>
-      <c r="H43" s="98"/>
-      <c r="I43" s="98"/>
-      <c r="J43" s="99"/>
+      <c r="H43" s="100"/>
+      <c r="I43" s="100"/>
+      <c r="J43" s="101"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="T43" s="91" t="s">
+      <c r="T43" s="93" t="s">
         <v>173</v>
       </c>
-      <c r="U43" s="92"/>
-      <c r="V43" s="92"/>
-      <c r="W43" s="92"/>
-      <c r="X43" s="92"/>
-      <c r="Y43" s="92"/>
-      <c r="Z43" s="92"/>
-      <c r="AA43" s="92"/>
-      <c r="AB43" s="92"/>
-      <c r="AC43" s="93"/>
+      <c r="U43" s="94"/>
+      <c r="V43" s="94"/>
+      <c r="W43" s="94"/>
+      <c r="X43" s="94"/>
+      <c r="Y43" s="94"/>
+      <c r="Z43" s="94"/>
+      <c r="AA43" s="94"/>
+      <c r="AB43" s="94"/>
+      <c r="AC43" s="95"/>
     </row>
     <row r="44" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="2">
@@ -5273,21 +5267,21 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="100" t="s">
+      <c r="S44" s="102" t="s">
         <v>76</v>
       </c>
-      <c r="T44" s="102" t="s">
+      <c r="T44" s="104" t="s">
         <v>174</v>
       </c>
-      <c r="U44" s="103"/>
-      <c r="V44" s="103"/>
-      <c r="W44" s="103"/>
-      <c r="X44" s="103"/>
-      <c r="Y44" s="103"/>
-      <c r="Z44" s="103"/>
-      <c r="AA44" s="103"/>
-      <c r="AB44" s="103"/>
-      <c r="AC44" s="104"/>
+      <c r="U44" s="105"/>
+      <c r="V44" s="105"/>
+      <c r="W44" s="105"/>
+      <c r="X44" s="105"/>
+      <c r="Y44" s="105"/>
+      <c r="Z44" s="105"/>
+      <c r="AA44" s="105"/>
+      <c r="AB44" s="105"/>
+      <c r="AC44" s="106"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="2">
@@ -5305,26 +5299,26 @@
       <c r="F45" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="G45" s="111" t="s">
+      <c r="G45" s="113" t="s">
         <v>181</v>
       </c>
-      <c r="H45" s="94"/>
-      <c r="I45" s="94"/>
-      <c r="J45" s="95"/>
+      <c r="H45" s="96"/>
+      <c r="I45" s="96"/>
+      <c r="J45" s="97"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="101"/>
-      <c r="T45" s="105"/>
-      <c r="U45" s="106"/>
-      <c r="V45" s="106"/>
-      <c r="W45" s="106"/>
-      <c r="X45" s="106"/>
-      <c r="Y45" s="106"/>
-      <c r="Z45" s="106"/>
-      <c r="AA45" s="106"/>
-      <c r="AB45" s="106"/>
-      <c r="AC45" s="107"/>
+      <c r="S45" s="103"/>
+      <c r="T45" s="107"/>
+      <c r="U45" s="108"/>
+      <c r="V45" s="108"/>
+      <c r="W45" s="108"/>
+      <c r="X45" s="108"/>
+      <c r="Y45" s="108"/>
+      <c r="Z45" s="108"/>
+      <c r="AA45" s="108"/>
+      <c r="AB45" s="108"/>
+      <c r="AC45" s="109"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B46" s="2">
@@ -5342,28 +5336,28 @@
       <c r="F46" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G46" s="112"/>
-      <c r="H46" s="96"/>
-      <c r="I46" s="96"/>
-      <c r="J46" s="97"/>
+      <c r="G46" s="114"/>
+      <c r="H46" s="98"/>
+      <c r="I46" s="98"/>
+      <c r="J46" s="99"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="T46" s="108" t="s">
+      <c r="T46" s="110" t="s">
         <v>175</v>
       </c>
-      <c r="U46" s="109"/>
-      <c r="V46" s="109"/>
-      <c r="W46" s="109"/>
-      <c r="X46" s="109"/>
-      <c r="Y46" s="109"/>
-      <c r="Z46" s="109"/>
-      <c r="AA46" s="109"/>
-      <c r="AB46" s="109"/>
-      <c r="AC46" s="110"/>
+      <c r="U46" s="111"/>
+      <c r="V46" s="111"/>
+      <c r="W46" s="111"/>
+      <c r="X46" s="111"/>
+      <c r="Y46" s="111"/>
+      <c r="Z46" s="111"/>
+      <c r="AA46" s="111"/>
+      <c r="AB46" s="111"/>
+      <c r="AC46" s="112"/>
     </row>
     <row r="47" spans="2:29" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="2">
@@ -5381,12 +5375,12 @@
       <c r="F47" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="G47" s="98" t="s">
+      <c r="G47" s="100" t="s">
         <v>152</v>
       </c>
-      <c r="H47" s="98"/>
-      <c r="I47" s="98"/>
-      <c r="J47" s="99"/>
+      <c r="H47" s="100"/>
+      <c r="I47" s="100"/>
+      <c r="J47" s="101"/>
     </row>
     <row r="48" spans="2:29" ht="30" x14ac:dyDescent="0.25">
       <c r="B48" s="2">
@@ -5438,12 +5432,12 @@
       <c r="F50" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="G50" s="94" t="s">
+      <c r="G50" s="96" t="s">
         <v>155</v>
       </c>
-      <c r="H50" s="94"/>
-      <c r="I50" s="94"/>
-      <c r="J50" s="95"/>
+      <c r="H50" s="96"/>
+      <c r="I50" s="96"/>
+      <c r="J50" s="97"/>
     </row>
     <row r="51" spans="2:10" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" s="4">
@@ -5461,19 +5455,19 @@
       <c r="F51" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="G51" s="96"/>
-      <c r="H51" s="96"/>
-      <c r="I51" s="96"/>
-      <c r="J51" s="97"/>
+      <c r="G51" s="98"/>
+      <c r="H51" s="98"/>
+      <c r="I51" s="98"/>
+      <c r="J51" s="99"/>
     </row>
     <row r="52" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="166" t="s">
+      <c r="B52" s="167" t="s">
         <v>142</v>
       </c>
-      <c r="C52" s="131"/>
-      <c r="D52" s="131"/>
-      <c r="E52" s="131"/>
-      <c r="F52" s="132"/>
+      <c r="C52" s="148"/>
+      <c r="D52" s="148"/>
+      <c r="E52" s="148"/>
+      <c r="F52" s="149"/>
     </row>
     <row r="54" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
@@ -5483,16 +5477,16 @@
       <c r="C55" s="159" t="s">
         <v>185</v>
       </c>
-      <c r="D55" s="169" t="s">
+      <c r="D55" s="173" t="s">
         <v>184</v>
       </c>
-      <c r="E55" s="170"/>
+      <c r="E55" s="174"/>
     </row>
     <row r="56" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B56" s="162"/>
       <c r="C56" s="160"/>
-      <c r="D56" s="171"/>
-      <c r="E56" s="172"/>
+      <c r="D56" s="175"/>
+      <c r="E56" s="176"/>
     </row>
     <row r="57" spans="2:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="81">
@@ -5501,22 +5495,22 @@
       <c r="C57" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D57" s="177" t="s">
+      <c r="D57" s="90" t="s">
         <v>207</v>
       </c>
-      <c r="E57" s="178"/>
+      <c r="E57" s="92"/>
     </row>
     <row r="58" spans="2:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="82">
         <v>1</v>
       </c>
-      <c r="C58" s="173" t="s">
+      <c r="C58" s="86" t="s">
         <v>203</v>
       </c>
-      <c r="D58" s="175" t="s">
+      <c r="D58" s="163" t="s">
         <v>206</v>
       </c>
-      <c r="E58" s="163"/>
+      <c r="E58" s="164"/>
     </row>
     <row r="59" spans="2:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="82">
@@ -5525,22 +5519,22 @@
       <c r="C59" s="38" t="s">
         <v>204</v>
       </c>
-      <c r="D59" s="175" t="s">
+      <c r="D59" s="163" t="s">
         <v>205</v>
       </c>
-      <c r="E59" s="163"/>
+      <c r="E59" s="164"/>
     </row>
     <row r="60" spans="2:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="82">
         <v>3</v>
       </c>
-      <c r="C60" s="173" t="s">
+      <c r="C60" s="86" t="s">
         <v>186</v>
       </c>
-      <c r="D60" s="175" t="s">
+      <c r="D60" s="163" t="s">
         <v>189</v>
       </c>
-      <c r="E60" s="163"/>
+      <c r="E60" s="164"/>
     </row>
     <row r="61" spans="2:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="82">
@@ -5549,10 +5543,10 @@
       <c r="C61" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="D61" s="175" t="s">
+      <c r="D61" s="163" t="s">
         <v>190</v>
       </c>
-      <c r="E61" s="163"/>
+      <c r="E61" s="164"/>
     </row>
     <row r="62" spans="2:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="82">
@@ -5561,94 +5555,94 @@
       <c r="C62" s="38" t="s">
         <v>188</v>
       </c>
-      <c r="D62" s="175" t="s">
+      <c r="D62" s="163" t="s">
         <v>191</v>
       </c>
-      <c r="E62" s="163"/>
+      <c r="E62" s="164"/>
     </row>
     <row r="63" spans="2:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="82">
         <v>6</v>
       </c>
-      <c r="C63" s="173" t="s">
+      <c r="C63" s="86" t="s">
         <v>196</v>
       </c>
-      <c r="D63" s="175" t="s">
+      <c r="D63" s="163" t="s">
         <v>197</v>
       </c>
-      <c r="E63" s="163"/>
+      <c r="E63" s="164"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B64" s="82">
         <v>7</v>
       </c>
-      <c r="C64" s="173"/>
-      <c r="D64" s="175"/>
-      <c r="E64" s="163"/>
+      <c r="C64" s="86"/>
+      <c r="D64" s="163"/>
+      <c r="E64" s="164"/>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="82">
         <v>8</v>
       </c>
-      <c r="C65" s="173"/>
-      <c r="D65" s="175"/>
-      <c r="E65" s="163"/>
+      <c r="C65" s="86"/>
+      <c r="D65" s="163"/>
+      <c r="E65" s="164"/>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" s="82">
         <v>9</v>
       </c>
-      <c r="C66" s="173"/>
-      <c r="D66" s="175"/>
-      <c r="E66" s="163"/>
+      <c r="C66" s="86"/>
+      <c r="D66" s="163"/>
+      <c r="E66" s="164"/>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" s="82">
         <v>10</v>
       </c>
-      <c r="C67" s="173"/>
-      <c r="D67" s="175"/>
-      <c r="E67" s="163"/>
+      <c r="C67" s="86"/>
+      <c r="D67" s="163"/>
+      <c r="E67" s="164"/>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" s="82">
         <v>11</v>
       </c>
-      <c r="C68" s="173"/>
-      <c r="D68" s="175"/>
-      <c r="E68" s="163"/>
+      <c r="C68" s="86"/>
+      <c r="D68" s="163"/>
+      <c r="E68" s="164"/>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69" s="82">
         <v>12</v>
       </c>
-      <c r="C69" s="173"/>
-      <c r="D69" s="175"/>
-      <c r="E69" s="163"/>
+      <c r="C69" s="86"/>
+      <c r="D69" s="163"/>
+      <c r="E69" s="164"/>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B70" s="82">
         <v>13</v>
       </c>
-      <c r="C70" s="173"/>
-      <c r="D70" s="175"/>
-      <c r="E70" s="163"/>
+      <c r="C70" s="86"/>
+      <c r="D70" s="163"/>
+      <c r="E70" s="164"/>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B71" s="82">
         <v>14</v>
       </c>
-      <c r="C71" s="173"/>
-      <c r="D71" s="175"/>
-      <c r="E71" s="163"/>
+      <c r="C71" s="86"/>
+      <c r="D71" s="163"/>
+      <c r="E71" s="164"/>
     </row>
     <row r="72" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B72" s="83">
         <v>15</v>
       </c>
-      <c r="C72" s="174"/>
-      <c r="D72" s="176"/>
-      <c r="E72" s="167"/>
+      <c r="C72" s="87"/>
+      <c r="D72" s="170"/>
+      <c r="E72" s="171"/>
     </row>
   </sheetData>
   <mergeCells count="158">
@@ -5678,15 +5672,6 @@
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="AA7:AB7"/>
     <mergeCell ref="AA28:AB28"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AA11:AB11"/>
     <mergeCell ref="AA12:AB12"/>
     <mergeCell ref="AA13:AB13"/>
     <mergeCell ref="AA24:AB24"/>
@@ -5702,6 +5687,15 @@
     <mergeCell ref="N20:P20"/>
     <mergeCell ref="N21:P21"/>
     <mergeCell ref="N23:P23"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AA11:AB11"/>
     <mergeCell ref="U13:V13"/>
     <mergeCell ref="U14:V14"/>
     <mergeCell ref="S2:S4"/>
@@ -5712,6 +5706,11 @@
     <mergeCell ref="N26:P26"/>
     <mergeCell ref="N25:P25"/>
     <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="N28:P28"/>
     <mergeCell ref="N27:P27"/>
@@ -5736,9 +5735,6 @@
     <mergeCell ref="N11:P11"/>
     <mergeCell ref="E4:J4"/>
     <mergeCell ref="N10:P10"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
     <mergeCell ref="E5:J5"/>
     <mergeCell ref="H9:J9"/>
     <mergeCell ref="G17:J17"/>
@@ -5763,8 +5759,6 @@
     <mergeCell ref="H14:J14"/>
     <mergeCell ref="F16:J16"/>
     <mergeCell ref="N13:P13"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
     <mergeCell ref="AA20:AB20"/>
     <mergeCell ref="AA21:AB21"/>
     <mergeCell ref="AA22:AB22"/>

</xml_diff>

<commit_message>
Se actualizo la información sobre Ints, ademas se arreglo errores con SP en RET
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F57E3F6-5411-4067-9536-379F3D8BD3A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BA19C1-875F-463A-86B6-57AFA879B049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1660,7 +1660,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="177">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1923,28 +1923,220 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1959,12 +2151,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1987,15 +2173,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2013,182 +2190,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2497,62 +2500,62 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="133" t="s">
+      <c r="B2" s="134" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="142" t="s">
+      <c r="C2" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="143"/>
-      <c r="E2" s="144" t="s">
+      <c r="D2" s="150"/>
+      <c r="E2" s="151" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="144"/>
-      <c r="G2" s="145" t="s">
+      <c r="F2" s="151"/>
+      <c r="G2" s="152" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="144"/>
-      <c r="I2" s="144" t="s">
+      <c r="H2" s="151"/>
+      <c r="I2" s="151" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="144"/>
-      <c r="K2" s="146" t="s">
+      <c r="J2" s="151"/>
+      <c r="K2" s="153" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="144"/>
-      <c r="M2" s="144"/>
-      <c r="N2" s="144"/>
-      <c r="O2" s="144"/>
-      <c r="P2" s="147"/>
-      <c r="R2" s="152" t="s">
+      <c r="L2" s="151"/>
+      <c r="M2" s="151"/>
+      <c r="N2" s="151"/>
+      <c r="O2" s="151"/>
+      <c r="P2" s="154"/>
+      <c r="R2" s="130" t="s">
         <v>66</v>
       </c>
-      <c r="S2" s="89" t="s">
+      <c r="S2" s="127" t="s">
         <v>67</v>
       </c>
-      <c r="T2" s="156" t="s">
+      <c r="T2" s="120" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="157"/>
-      <c r="V2" s="157"/>
-      <c r="W2" s="157"/>
-      <c r="X2" s="157"/>
-      <c r="Y2" s="157"/>
-      <c r="Z2" s="157"/>
-      <c r="AA2" s="157"/>
-      <c r="AB2" s="157" t="s">
+      <c r="U2" s="121"/>
+      <c r="V2" s="121"/>
+      <c r="W2" s="121"/>
+      <c r="X2" s="121"/>
+      <c r="Y2" s="121"/>
+      <c r="Z2" s="121"/>
+      <c r="AA2" s="121"/>
+      <c r="AB2" s="121" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="157"/>
-      <c r="AD2" s="157"/>
-      <c r="AE2" s="157"/>
-      <c r="AF2" s="157"/>
-      <c r="AG2" s="157"/>
-      <c r="AH2" s="157"/>
-      <c r="AI2" s="158"/>
+      <c r="AC2" s="121"/>
+      <c r="AD2" s="121"/>
+      <c r="AE2" s="121"/>
+      <c r="AF2" s="121"/>
+      <c r="AG2" s="121"/>
+      <c r="AH2" s="121"/>
+      <c r="AI2" s="122"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="134"/>
+      <c r="B3" s="135"/>
       <c r="C3" s="16" t="s">
         <v>80</v>
       </c>
@@ -2577,21 +2580,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="139"/>
-      <c r="L3" s="140"/>
-      <c r="M3" s="140"/>
-      <c r="N3" s="140"/>
-      <c r="O3" s="140"/>
-      <c r="P3" s="141"/>
-      <c r="R3" s="153"/>
-      <c r="S3" s="150"/>
+      <c r="K3" s="105"/>
+      <c r="L3" s="148"/>
+      <c r="M3" s="148"/>
+      <c r="N3" s="148"/>
+      <c r="O3" s="148"/>
+      <c r="P3" s="106"/>
+      <c r="R3" s="131"/>
+      <c r="S3" s="128"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="120" t="s">
+      <c r="U3" s="158" t="s">
         <v>84</v>
       </c>
-      <c r="V3" s="120"/>
+      <c r="V3" s="158"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -2604,10 +2607,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="155" t="s">
+      <c r="AA3" s="119" t="s">
         <v>75</v>
       </c>
-      <c r="AB3" s="155"/>
+      <c r="AB3" s="119"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -2631,21 +2634,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="135"/>
+      <c r="B4" s="136"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="121" t="s">
+      <c r="E4" s="123" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="148"/>
-      <c r="G4" s="148"/>
-      <c r="H4" s="148"/>
-      <c r="I4" s="148"/>
-      <c r="J4" s="149"/>
+      <c r="F4" s="110"/>
+      <c r="G4" s="110"/>
+      <c r="H4" s="110"/>
+      <c r="I4" s="110"/>
+      <c r="J4" s="111"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -2655,20 +2658,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="121" t="s">
+      <c r="N4" s="123" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="148"/>
-      <c r="P4" s="149"/>
-      <c r="R4" s="154"/>
-      <c r="S4" s="151"/>
+      <c r="O4" s="110"/>
+      <c r="P4" s="111"/>
+      <c r="R4" s="132"/>
+      <c r="S4" s="129"/>
       <c r="T4" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="U4" s="121" t="s">
+      <c r="U4" s="123" t="s">
         <v>76</v>
       </c>
-      <c r="V4" s="122"/>
+      <c r="V4" s="124"/>
       <c r="W4" s="7" t="s">
         <v>72</v>
       </c>
@@ -2681,10 +2684,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="121" t="s">
+      <c r="AA4" s="123" t="s">
         <v>73</v>
       </c>
-      <c r="AB4" s="122"/>
+      <c r="AB4" s="124"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -2716,22 +2719,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="125"/>
-      <c r="F5" s="126"/>
-      <c r="G5" s="126"/>
-      <c r="H5" s="126"/>
-      <c r="I5" s="126"/>
-      <c r="J5" s="127"/>
+      <c r="E5" s="155"/>
+      <c r="F5" s="156"/>
+      <c r="G5" s="156"/>
+      <c r="H5" s="156"/>
+      <c r="I5" s="156"/>
+      <c r="J5" s="157"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="90" t="s">
+      <c r="N5" s="99" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="91"/>
-      <c r="P5" s="92"/>
+      <c r="O5" s="133"/>
+      <c r="P5" s="100"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -2741,10 +2744,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="123" t="s">
+      <c r="U5" s="125" t="s">
         <v>74</v>
       </c>
-      <c r="V5" s="124"/>
+      <c r="V5" s="126"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -2757,10 +2760,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="123" t="s">
+      <c r="AA5" s="125" t="s">
         <v>74</v>
       </c>
-      <c r="AB5" s="124"/>
+      <c r="AB5" s="126"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -2792,12 +2795,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="132"/>
-      <c r="F6" s="129"/>
-      <c r="G6" s="129"/>
-      <c r="H6" s="129"/>
-      <c r="I6" s="129"/>
-      <c r="J6" s="130"/>
+      <c r="E6" s="146"/>
+      <c r="F6" s="141"/>
+      <c r="G6" s="141"/>
+      <c r="H6" s="141"/>
+      <c r="I6" s="141"/>
+      <c r="J6" s="142"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -2805,11 +2808,11 @@
         <v>156</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="93" t="s">
+      <c r="N6" s="116" t="s">
         <v>96</v>
       </c>
-      <c r="O6" s="94"/>
-      <c r="P6" s="95"/>
+      <c r="O6" s="117"/>
+      <c r="P6" s="118"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -2819,10 +2822,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="118" t="s">
+      <c r="U6" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V6" s="119"/>
+      <c r="V6" s="113"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -2835,10 +2838,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="118" t="s">
+      <c r="AA6" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB6" s="119"/>
+      <c r="AB6" s="113"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -2879,9 +2882,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="128"/>
-      <c r="I7" s="129"/>
-      <c r="J7" s="130"/>
+      <c r="H7" s="140"/>
+      <c r="I7" s="141"/>
+      <c r="J7" s="142"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -2889,11 +2892,11 @@
       <c r="M7" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N7" s="93" t="s">
+      <c r="N7" s="116" t="s">
         <v>53</v>
       </c>
-      <c r="O7" s="94"/>
-      <c r="P7" s="95"/>
+      <c r="O7" s="117"/>
+      <c r="P7" s="118"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -2903,10 +2906,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="118" t="s">
+      <c r="U7" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V7" s="119"/>
+      <c r="V7" s="113"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -2919,10 +2922,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="118" t="s">
+      <c r="AA7" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB7" s="119"/>
+      <c r="AB7" s="113"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -2963,9 +2966,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="128"/>
-      <c r="I8" s="129"/>
-      <c r="J8" s="130"/>
+      <c r="H8" s="140"/>
+      <c r="I8" s="141"/>
+      <c r="J8" s="142"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -2973,11 +2976,11 @@
       <c r="M8" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N8" s="93" t="s">
+      <c r="N8" s="116" t="s">
         <v>54</v>
       </c>
-      <c r="O8" s="94"/>
-      <c r="P8" s="95"/>
+      <c r="O8" s="117"/>
+      <c r="P8" s="118"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -2987,10 +2990,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="118" t="s">
+      <c r="U8" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V8" s="119"/>
+      <c r="V8" s="113"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -3003,10 +3006,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="118" t="s">
+      <c r="AA8" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB8" s="119"/>
+      <c r="AB8" s="113"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -3047,9 +3050,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="128"/>
-      <c r="I9" s="129"/>
-      <c r="J9" s="130"/>
+      <c r="H9" s="140"/>
+      <c r="I9" s="141"/>
+      <c r="J9" s="142"/>
       <c r="K9" s="37" t="s">
         <v>48</v>
       </c>
@@ -3057,11 +3060,11 @@
       <c r="M9" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N9" s="93" t="s">
+      <c r="N9" s="116" t="s">
         <v>55</v>
       </c>
-      <c r="O9" s="94"/>
-      <c r="P9" s="95"/>
+      <c r="O9" s="117"/>
+      <c r="P9" s="118"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -3071,10 +3074,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="118" t="s">
+      <c r="U9" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V9" s="119"/>
+      <c r="V9" s="113"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -3087,10 +3090,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="118" t="s">
+      <c r="AA9" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB9" s="119"/>
+      <c r="AB9" s="113"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -3131,9 +3134,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="128"/>
-      <c r="I10" s="129"/>
-      <c r="J10" s="130"/>
+      <c r="H10" s="140"/>
+      <c r="I10" s="141"/>
+      <c r="J10" s="142"/>
       <c r="K10" s="37" t="s">
         <v>49</v>
       </c>
@@ -3141,11 +3144,11 @@
       <c r="M10" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N10" s="93" t="s">
+      <c r="N10" s="116" t="s">
         <v>56</v>
       </c>
-      <c r="O10" s="94"/>
-      <c r="P10" s="95"/>
+      <c r="O10" s="117"/>
+      <c r="P10" s="118"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -3155,10 +3158,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="118" t="s">
+      <c r="U10" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V10" s="119"/>
+      <c r="V10" s="113"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -3171,10 +3174,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="118" t="s">
+      <c r="AA10" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB10" s="119"/>
+      <c r="AB10" s="113"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -3215,9 +3218,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="128"/>
-      <c r="I11" s="129"/>
-      <c r="J11" s="130"/>
+      <c r="H11" s="140"/>
+      <c r="I11" s="141"/>
+      <c r="J11" s="142"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -3225,11 +3228,11 @@
       <c r="M11" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N11" s="93" t="s">
+      <c r="N11" s="116" t="s">
         <v>57</v>
       </c>
-      <c r="O11" s="94"/>
-      <c r="P11" s="95"/>
+      <c r="O11" s="117"/>
+      <c r="P11" s="118"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -3239,10 +3242,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="118" t="s">
+      <c r="U11" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V11" s="119"/>
+      <c r="V11" s="113"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -3255,10 +3258,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="118" t="s">
+      <c r="AA11" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB11" s="119"/>
+      <c r="AB11" s="113"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -3299,9 +3302,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="128"/>
-      <c r="I12" s="129"/>
-      <c r="J12" s="130"/>
+      <c r="H12" s="140"/>
+      <c r="I12" s="141"/>
+      <c r="J12" s="142"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -3309,11 +3312,11 @@
       <c r="M12" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N12" s="93" t="s">
+      <c r="N12" s="116" t="s">
         <v>58</v>
       </c>
-      <c r="O12" s="94"/>
-      <c r="P12" s="95"/>
+      <c r="O12" s="117"/>
+      <c r="P12" s="118"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -3323,10 +3326,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="118" t="s">
+      <c r="U12" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V12" s="119"/>
+      <c r="V12" s="113"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -3339,10 +3342,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="118" t="s">
+      <c r="AA12" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB12" s="119"/>
+      <c r="AB12" s="113"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -3383,9 +3386,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="128"/>
-      <c r="I13" s="129"/>
-      <c r="J13" s="130"/>
+      <c r="H13" s="140"/>
+      <c r="I13" s="141"/>
+      <c r="J13" s="142"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -3393,11 +3396,11 @@
       <c r="M13" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N13" s="93" t="s">
+      <c r="N13" s="116" t="s">
         <v>59</v>
       </c>
-      <c r="O13" s="94"/>
-      <c r="P13" s="95"/>
+      <c r="O13" s="117"/>
+      <c r="P13" s="118"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -3407,10 +3410,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="118" t="s">
+      <c r="U13" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V13" s="119"/>
+      <c r="V13" s="113"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -3423,10 +3426,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="118" t="s">
+      <c r="AA13" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB13" s="119"/>
+      <c r="AB13" s="113"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -3467,9 +3470,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="128"/>
-      <c r="I14" s="129"/>
-      <c r="J14" s="130"/>
+      <c r="H14" s="140"/>
+      <c r="I14" s="141"/>
+      <c r="J14" s="142"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -3477,11 +3480,11 @@
       <c r="M14" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N14" s="93" t="s">
+      <c r="N14" s="116" t="s">
         <v>60</v>
       </c>
-      <c r="O14" s="94"/>
-      <c r="P14" s="95"/>
+      <c r="O14" s="117"/>
+      <c r="P14" s="118"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -3491,10 +3494,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="118" t="s">
+      <c r="U14" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V14" s="119"/>
+      <c r="V14" s="113"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -3507,10 +3510,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="118" t="s">
+      <c r="AA14" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB14" s="119"/>
+      <c r="AB14" s="113"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -3551,9 +3554,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="128"/>
-      <c r="I15" s="129"/>
-      <c r="J15" s="130"/>
+      <c r="H15" s="140"/>
+      <c r="I15" s="141"/>
+      <c r="J15" s="142"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -3561,11 +3564,11 @@
       <c r="M15" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N15" s="93" t="s">
+      <c r="N15" s="116" t="s">
         <v>61</v>
       </c>
-      <c r="O15" s="94"/>
-      <c r="P15" s="95"/>
+      <c r="O15" s="117"/>
+      <c r="P15" s="118"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -3575,10 +3578,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="118" t="s">
+      <c r="U15" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V15" s="119"/>
+      <c r="V15" s="113"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -3591,10 +3594,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="118" t="s">
+      <c r="AA15" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB15" s="119"/>
+      <c r="AB15" s="113"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -3629,21 +3632,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="128"/>
-      <c r="G16" s="129"/>
-      <c r="H16" s="129"/>
-      <c r="I16" s="129"/>
-      <c r="J16" s="130"/>
+      <c r="F16" s="140"/>
+      <c r="G16" s="141"/>
+      <c r="H16" s="141"/>
+      <c r="I16" s="141"/>
+      <c r="J16" s="142"/>
       <c r="K16" s="40" t="s">
         <v>50</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="93" t="s">
+      <c r="N16" s="116" t="s">
         <v>51</v>
       </c>
-      <c r="O16" s="94"/>
-      <c r="P16" s="95"/>
+      <c r="O16" s="117"/>
+      <c r="P16" s="118"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -3653,10 +3656,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="118" t="s">
+      <c r="U16" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V16" s="119"/>
+      <c r="V16" s="113"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -3669,10 +3672,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="118" t="s">
+      <c r="AA16" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB16" s="119"/>
+      <c r="AB16" s="113"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -3708,22 +3711,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="131" t="s">
+      <c r="G17" s="147" t="s">
         <v>77</v>
       </c>
-      <c r="H17" s="94"/>
-      <c r="I17" s="94"/>
-      <c r="J17" s="95"/>
+      <c r="H17" s="117"/>
+      <c r="I17" s="117"/>
+      <c r="J17" s="118"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="93" t="s">
+      <c r="N17" s="116" t="s">
         <v>65</v>
       </c>
-      <c r="O17" s="94"/>
-      <c r="P17" s="95"/>
+      <c r="O17" s="117"/>
+      <c r="P17" s="118"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -3733,10 +3736,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="118" t="s">
+      <c r="U17" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V17" s="119"/>
+      <c r="V17" s="113"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -3749,10 +3752,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="118" t="s">
+      <c r="AA17" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB17" s="119"/>
+      <c r="AB17" s="113"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -3788,12 +3791,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="131" t="s">
+      <c r="G18" s="147" t="s">
         <v>77</v>
       </c>
-      <c r="H18" s="94"/>
-      <c r="I18" s="94"/>
-      <c r="J18" s="95"/>
+      <c r="H18" s="117"/>
+      <c r="I18" s="117"/>
+      <c r="J18" s="118"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -3801,11 +3804,11 @@
       <c r="M18" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N18" s="93" t="s">
+      <c r="N18" s="116" t="s">
         <v>62</v>
       </c>
-      <c r="O18" s="94"/>
-      <c r="P18" s="95"/>
+      <c r="O18" s="117"/>
+      <c r="P18" s="118"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -3815,10 +3818,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="118" t="s">
+      <c r="U18" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V18" s="119"/>
+      <c r="V18" s="113"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -3831,10 +3834,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="118" t="s">
+      <c r="AA18" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB18" s="119"/>
+      <c r="AB18" s="113"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -3872,20 +3875,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="128"/>
-      <c r="H19" s="129"/>
-      <c r="I19" s="129"/>
-      <c r="J19" s="130"/>
+      <c r="G19" s="140"/>
+      <c r="H19" s="141"/>
+      <c r="I19" s="141"/>
+      <c r="J19" s="142"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="93" t="s">
+      <c r="N19" s="116" t="s">
         <v>94</v>
       </c>
-      <c r="O19" s="94"/>
-      <c r="P19" s="95"/>
+      <c r="O19" s="117"/>
+      <c r="P19" s="118"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -3895,10 +3898,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="118" t="s">
+      <c r="U19" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V19" s="119"/>
+      <c r="V19" s="113"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -3911,10 +3914,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="118" t="s">
+      <c r="AA19" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB19" s="119"/>
+      <c r="AB19" s="113"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -3954,20 +3957,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="128"/>
-      <c r="H20" s="129"/>
-      <c r="I20" s="129"/>
-      <c r="J20" s="130"/>
+      <c r="G20" s="140"/>
+      <c r="H20" s="141"/>
+      <c r="I20" s="141"/>
+      <c r="J20" s="142"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="93" t="s">
+      <c r="N20" s="116" t="s">
         <v>95</v>
       </c>
-      <c r="O20" s="94"/>
-      <c r="P20" s="95"/>
+      <c r="O20" s="117"/>
+      <c r="P20" s="118"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -3977,10 +3980,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="118" t="s">
+      <c r="U20" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V20" s="119"/>
+      <c r="V20" s="113"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -3993,10 +3996,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="118" t="s">
+      <c r="AA20" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB20" s="119"/>
+      <c r="AB20" s="113"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -4034,20 +4037,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="128"/>
-      <c r="H21" s="129"/>
-      <c r="I21" s="129"/>
-      <c r="J21" s="130"/>
+      <c r="G21" s="140"/>
+      <c r="H21" s="141"/>
+      <c r="I21" s="141"/>
+      <c r="J21" s="142"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="93" t="s">
+      <c r="N21" s="116" t="s">
         <v>63</v>
       </c>
-      <c r="O21" s="94"/>
-      <c r="P21" s="95"/>
+      <c r="O21" s="117"/>
+      <c r="P21" s="118"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -4057,10 +4060,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="118" t="s">
+      <c r="U21" s="112" t="s">
         <v>97</v>
       </c>
-      <c r="V21" s="119"/>
+      <c r="V21" s="113"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -4073,10 +4076,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="118" t="s">
+      <c r="AA21" s="112" t="s">
         <v>99</v>
       </c>
-      <c r="AB21" s="119"/>
+      <c r="AB21" s="113"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -4110,22 +4113,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="132"/>
-      <c r="F22" s="129"/>
-      <c r="G22" s="129"/>
-      <c r="H22" s="129"/>
-      <c r="I22" s="129"/>
-      <c r="J22" s="130"/>
+      <c r="E22" s="146"/>
+      <c r="F22" s="141"/>
+      <c r="G22" s="141"/>
+      <c r="H22" s="141"/>
+      <c r="I22" s="141"/>
+      <c r="J22" s="142"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="93" t="s">
+      <c r="N22" s="116" t="s">
         <v>64</v>
       </c>
-      <c r="O22" s="94"/>
-      <c r="P22" s="95"/>
+      <c r="O22" s="117"/>
+      <c r="P22" s="118"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -4135,10 +4138,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="118" t="s">
+      <c r="U22" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V22" s="119"/>
+      <c r="V22" s="113"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -4151,10 +4154,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="118" t="s">
+      <c r="AA22" s="112" t="s">
         <v>97</v>
       </c>
-      <c r="AB22" s="119"/>
+      <c r="AB22" s="113"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -4194,22 +4197,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="131" t="s">
+      <c r="G23" s="147" t="s">
         <v>78</v>
       </c>
-      <c r="H23" s="94"/>
-      <c r="I23" s="94"/>
-      <c r="J23" s="95"/>
+      <c r="H23" s="117"/>
+      <c r="I23" s="117"/>
+      <c r="J23" s="118"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="93" t="s">
+      <c r="N23" s="116" t="s">
         <v>83</v>
       </c>
-      <c r="O23" s="94"/>
-      <c r="P23" s="95"/>
+      <c r="O23" s="117"/>
+      <c r="P23" s="118"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -4219,10 +4222,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="118" t="s">
+      <c r="U23" s="112" t="s">
         <v>98</v>
       </c>
-      <c r="V23" s="119"/>
+      <c r="V23" s="113"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -4235,10 +4238,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="118" t="s">
+      <c r="AA23" s="112" t="s">
         <v>97</v>
       </c>
-      <c r="AB23" s="119"/>
+      <c r="AB23" s="113"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -4278,22 +4281,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="131" t="s">
+      <c r="G24" s="147" t="s">
         <v>78</v>
       </c>
-      <c r="H24" s="94"/>
-      <c r="I24" s="94"/>
-      <c r="J24" s="95"/>
+      <c r="H24" s="117"/>
+      <c r="I24" s="117"/>
+      <c r="J24" s="118"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="93" t="s">
+      <c r="N24" s="116" t="s">
         <v>82</v>
       </c>
-      <c r="O24" s="94"/>
-      <c r="P24" s="95"/>
+      <c r="O24" s="117"/>
+      <c r="P24" s="118"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -4303,10 +4306,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="118" t="s">
+      <c r="U24" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V24" s="119"/>
+      <c r="V24" s="113"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -4319,10 +4322,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="118" t="s">
+      <c r="AA24" s="112" t="s">
         <v>99</v>
       </c>
-      <c r="AB24" s="119"/>
+      <c r="AB24" s="113"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -4360,10 +4363,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="128"/>
-      <c r="H25" s="129"/>
-      <c r="I25" s="129"/>
-      <c r="J25" s="130"/>
+      <c r="G25" s="140"/>
+      <c r="H25" s="141"/>
+      <c r="I25" s="141"/>
+      <c r="J25" s="142"/>
       <c r="K25" s="49" t="s">
         <v>40</v>
       </c>
@@ -4371,11 +4374,11 @@
         <v>156</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="93" t="s">
+      <c r="N25" s="116" t="s">
         <v>42</v>
       </c>
-      <c r="O25" s="94"/>
-      <c r="P25" s="95"/>
+      <c r="O25" s="117"/>
+      <c r="P25" s="118"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -4385,10 +4388,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="118" t="s">
+      <c r="U25" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V25" s="119"/>
+      <c r="V25" s="113"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -4401,10 +4404,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="118" t="s">
+      <c r="AA25" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB25" s="119"/>
+      <c r="AB25" s="113"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -4442,10 +4445,10 @@
       <c r="F26" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="G26" s="128"/>
-      <c r="H26" s="129"/>
-      <c r="I26" s="129"/>
-      <c r="J26" s="130"/>
+      <c r="G26" s="140"/>
+      <c r="H26" s="141"/>
+      <c r="I26" s="141"/>
+      <c r="J26" s="142"/>
       <c r="K26" s="31" t="s">
         <v>41</v>
       </c>
@@ -4453,11 +4456,11 @@
         <v>156</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="93" t="s">
+      <c r="N26" s="116" t="s">
         <v>43</v>
       </c>
-      <c r="O26" s="94"/>
-      <c r="P26" s="95"/>
+      <c r="O26" s="117"/>
+      <c r="P26" s="118"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -4467,10 +4470,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="118" t="s">
+      <c r="U26" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V26" s="119"/>
+      <c r="V26" s="113"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -4483,10 +4486,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="118" t="s">
+      <c r="AA26" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB26" s="119"/>
+      <c r="AB26" s="113"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -4518,22 +4521,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="132"/>
-      <c r="F27" s="129"/>
-      <c r="G27" s="129"/>
-      <c r="H27" s="129"/>
-      <c r="I27" s="129"/>
-      <c r="J27" s="130"/>
+      <c r="E27" s="146"/>
+      <c r="F27" s="141"/>
+      <c r="G27" s="141"/>
+      <c r="H27" s="141"/>
+      <c r="I27" s="141"/>
+      <c r="J27" s="142"/>
       <c r="K27" s="25" t="s">
         <v>45</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="93" t="s">
+      <c r="N27" s="116" t="s">
         <v>47</v>
       </c>
-      <c r="O27" s="94"/>
-      <c r="P27" s="95"/>
+      <c r="O27" s="117"/>
+      <c r="P27" s="118"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -4543,10 +4546,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="118" t="s">
+      <c r="U27" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="V27" s="119"/>
+      <c r="V27" s="113"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -4559,10 +4562,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="118" t="s">
+      <c r="AA27" s="112" t="s">
         <v>74</v>
       </c>
-      <c r="AB27" s="119"/>
+      <c r="AB27" s="113"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -4594,12 +4597,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="136"/>
-      <c r="F28" s="137"/>
-      <c r="G28" s="137"/>
-      <c r="H28" s="137"/>
-      <c r="I28" s="137"/>
-      <c r="J28" s="138"/>
+      <c r="E28" s="143"/>
+      <c r="F28" s="144"/>
+      <c r="G28" s="144"/>
+      <c r="H28" s="144"/>
+      <c r="I28" s="144"/>
+      <c r="J28" s="145"/>
       <c r="K28" s="52" t="s">
         <v>46</v>
       </c>
@@ -4607,11 +4610,11 @@
         <v>156</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="110" t="s">
+      <c r="N28" s="137" t="s">
         <v>93</v>
       </c>
-      <c r="O28" s="111"/>
-      <c r="P28" s="112"/>
+      <c r="O28" s="138"/>
+      <c r="P28" s="139"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -4621,10 +4624,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="168" t="s">
+      <c r="U28" s="114" t="s">
         <v>74</v>
       </c>
-      <c r="V28" s="169"/>
+      <c r="V28" s="115"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -4637,10 +4640,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="168" t="s">
+      <c r="AA28" s="114" t="s">
         <v>74</v>
       </c>
-      <c r="AB28" s="169"/>
+      <c r="AB28" s="115"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -4717,18 +4720,18 @@
       <c r="S30" s="75" t="s">
         <v>157</v>
       </c>
-      <c r="T30" s="88" t="s">
+      <c r="T30" s="159" t="s">
         <v>158</v>
       </c>
-      <c r="U30" s="88"/>
-      <c r="V30" s="88"/>
-      <c r="W30" s="88"/>
-      <c r="X30" s="88"/>
-      <c r="Y30" s="88"/>
-      <c r="Z30" s="88"/>
-      <c r="AA30" s="88"/>
-      <c r="AB30" s="88"/>
-      <c r="AC30" s="89"/>
+      <c r="U30" s="159"/>
+      <c r="V30" s="159"/>
+      <c r="W30" s="159"/>
+      <c r="X30" s="159"/>
+      <c r="Y30" s="159"/>
+      <c r="Z30" s="159"/>
+      <c r="AA30" s="159"/>
+      <c r="AB30" s="159"/>
+      <c r="AC30" s="127"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="67" t="s">
@@ -4769,18 +4772,18 @@
       <c r="S31" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="T31" s="90" t="s">
+      <c r="T31" s="99" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="91"/>
-      <c r="V31" s="91"/>
-      <c r="W31" s="91"/>
-      <c r="X31" s="91"/>
-      <c r="Y31" s="91"/>
-      <c r="Z31" s="91"/>
-      <c r="AA31" s="91"/>
-      <c r="AB31" s="91"/>
-      <c r="AC31" s="92"/>
+      <c r="U31" s="133"/>
+      <c r="V31" s="133"/>
+      <c r="W31" s="133"/>
+      <c r="X31" s="133"/>
+      <c r="Y31" s="133"/>
+      <c r="Z31" s="133"/>
+      <c r="AA31" s="133"/>
+      <c r="AB31" s="133"/>
+      <c r="AC31" s="100"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="4" t="s">
@@ -4804,18 +4807,18 @@
       <c r="S32" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="T32" s="93" t="s">
+      <c r="T32" s="116" t="s">
         <v>164</v>
       </c>
-      <c r="U32" s="94"/>
-      <c r="V32" s="94"/>
-      <c r="W32" s="94"/>
-      <c r="X32" s="94"/>
-      <c r="Y32" s="94"/>
-      <c r="Z32" s="94"/>
-      <c r="AA32" s="94"/>
-      <c r="AB32" s="94"/>
-      <c r="AC32" s="95"/>
+      <c r="U32" s="117"/>
+      <c r="V32" s="117"/>
+      <c r="W32" s="117"/>
+      <c r="X32" s="117"/>
+      <c r="Y32" s="117"/>
+      <c r="Z32" s="117"/>
+      <c r="AA32" s="117"/>
+      <c r="AB32" s="117"/>
+      <c r="AC32" s="118"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H33" s="84" t="s">
@@ -4851,31 +4854,31 @@
       <c r="S33" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T33" s="93" t="s">
+      <c r="T33" s="116" t="s">
         <v>165</v>
       </c>
-      <c r="U33" s="94"/>
-      <c r="V33" s="94"/>
-      <c r="W33" s="94"/>
-      <c r="X33" s="94"/>
-      <c r="Y33" s="94"/>
-      <c r="Z33" s="94"/>
-      <c r="AA33" s="94"/>
-      <c r="AB33" s="94"/>
-      <c r="AC33" s="95"/>
+      <c r="U33" s="117"/>
+      <c r="V33" s="117"/>
+      <c r="W33" s="117"/>
+      <c r="X33" s="117"/>
+      <c r="Y33" s="117"/>
+      <c r="Z33" s="117"/>
+      <c r="AA33" s="117"/>
+      <c r="AB33" s="117"/>
+      <c r="AC33" s="118"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="165" t="s">
+      <c r="B34" s="107" t="s">
         <v>109</v>
       </c>
-      <c r="C34" s="139" t="s">
+      <c r="C34" s="105" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="141"/>
-      <c r="E34" s="139" t="s">
+      <c r="D34" s="106"/>
+      <c r="E34" s="105" t="s">
         <v>116</v>
       </c>
-      <c r="F34" s="141"/>
+      <c r="F34" s="106"/>
       <c r="H34" s="77" t="s">
         <v>66</v>
       </c>
@@ -4901,21 +4904,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="93" t="s">
+      <c r="T34" s="116" t="s">
         <v>166</v>
       </c>
-      <c r="U34" s="94"/>
-      <c r="V34" s="94"/>
-      <c r="W34" s="94"/>
-      <c r="X34" s="94"/>
-      <c r="Y34" s="94"/>
-      <c r="Z34" s="94"/>
-      <c r="AA34" s="94"/>
-      <c r="AB34" s="94"/>
-      <c r="AC34" s="95"/>
+      <c r="U34" s="117"/>
+      <c r="V34" s="117"/>
+      <c r="W34" s="117"/>
+      <c r="X34" s="117"/>
+      <c r="Y34" s="117"/>
+      <c r="Z34" s="117"/>
+      <c r="AA34" s="117"/>
+      <c r="AB34" s="117"/>
+      <c r="AC34" s="118"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="166"/>
+      <c r="B35" s="108"/>
       <c r="C35" s="64" t="s">
         <v>100</v>
       </c>
@@ -4934,18 +4937,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="93" t="s">
+      <c r="T35" s="116" t="s">
         <v>167</v>
       </c>
-      <c r="U35" s="94"/>
-      <c r="V35" s="94"/>
-      <c r="W35" s="94"/>
-      <c r="X35" s="94"/>
-      <c r="Y35" s="94"/>
-      <c r="Z35" s="94"/>
-      <c r="AA35" s="94"/>
-      <c r="AB35" s="94"/>
-      <c r="AC35" s="95"/>
+      <c r="U35" s="117"/>
+      <c r="V35" s="117"/>
+      <c r="W35" s="117"/>
+      <c r="X35" s="117"/>
+      <c r="Y35" s="117"/>
+      <c r="Z35" s="117"/>
+      <c r="AA35" s="117"/>
+      <c r="AB35" s="117"/>
+      <c r="AC35" s="118"/>
     </row>
     <row r="36" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B36" s="1">
@@ -4969,18 +4972,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="93" t="s">
+      <c r="T36" s="116" t="s">
         <v>168</v>
       </c>
-      <c r="U36" s="94"/>
-      <c r="V36" s="94"/>
-      <c r="W36" s="94"/>
-      <c r="X36" s="94"/>
-      <c r="Y36" s="94"/>
-      <c r="Z36" s="94"/>
-      <c r="AA36" s="94"/>
-      <c r="AB36" s="94"/>
-      <c r="AC36" s="95"/>
+      <c r="U36" s="117"/>
+      <c r="V36" s="117"/>
+      <c r="W36" s="117"/>
+      <c r="X36" s="117"/>
+      <c r="Y36" s="117"/>
+      <c r="Z36" s="117"/>
+      <c r="AA36" s="117"/>
+      <c r="AB36" s="117"/>
+      <c r="AC36" s="118"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="2">
@@ -5005,18 +5008,18 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="93" t="s">
+      <c r="T37" s="116" t="s">
         <v>195</v>
       </c>
-      <c r="U37" s="94"/>
-      <c r="V37" s="94"/>
-      <c r="W37" s="94"/>
-      <c r="X37" s="94"/>
-      <c r="Y37" s="94"/>
-      <c r="Z37" s="94"/>
-      <c r="AA37" s="94"/>
-      <c r="AB37" s="94"/>
-      <c r="AC37" s="95"/>
+      <c r="U37" s="117"/>
+      <c r="V37" s="117"/>
+      <c r="W37" s="117"/>
+      <c r="X37" s="117"/>
+      <c r="Y37" s="117"/>
+      <c r="Z37" s="117"/>
+      <c r="AA37" s="117"/>
+      <c r="AB37" s="117"/>
+      <c r="AC37" s="118"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="2">
@@ -5037,21 +5040,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="102" t="s">
+      <c r="S38" s="164" t="s">
         <v>73</v>
       </c>
-      <c r="T38" s="104" t="s">
+      <c r="T38" s="166" t="s">
         <v>169</v>
       </c>
-      <c r="U38" s="105"/>
-      <c r="V38" s="105"/>
-      <c r="W38" s="105"/>
-      <c r="X38" s="105"/>
-      <c r="Y38" s="105"/>
-      <c r="Z38" s="105"/>
-      <c r="AA38" s="105"/>
-      <c r="AB38" s="105"/>
-      <c r="AC38" s="106"/>
+      <c r="U38" s="167"/>
+      <c r="V38" s="167"/>
+      <c r="W38" s="167"/>
+      <c r="X38" s="167"/>
+      <c r="Y38" s="167"/>
+      <c r="Z38" s="167"/>
+      <c r="AA38" s="167"/>
+      <c r="AB38" s="167"/>
+      <c r="AC38" s="168"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="2">
@@ -5069,26 +5072,26 @@
       <c r="F39" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G39" s="113" t="s">
+      <c r="G39" s="172" t="s">
         <v>182</v>
       </c>
-      <c r="H39" s="96"/>
-      <c r="I39" s="96"/>
-      <c r="J39" s="97"/>
+      <c r="H39" s="160"/>
+      <c r="I39" s="160"/>
+      <c r="J39" s="161"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="103"/>
-      <c r="T39" s="107"/>
-      <c r="U39" s="108"/>
-      <c r="V39" s="108"/>
-      <c r="W39" s="108"/>
-      <c r="X39" s="108"/>
-      <c r="Y39" s="108"/>
-      <c r="Z39" s="108"/>
-      <c r="AA39" s="108"/>
-      <c r="AB39" s="108"/>
-      <c r="AC39" s="109"/>
+      <c r="S39" s="165"/>
+      <c r="T39" s="169"/>
+      <c r="U39" s="170"/>
+      <c r="V39" s="170"/>
+      <c r="W39" s="170"/>
+      <c r="X39" s="170"/>
+      <c r="Y39" s="170"/>
+      <c r="Z39" s="170"/>
+      <c r="AA39" s="170"/>
+      <c r="AB39" s="170"/>
+      <c r="AC39" s="171"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="2">
@@ -5106,28 +5109,28 @@
       <c r="F40" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G40" s="115"/>
-      <c r="H40" s="116"/>
-      <c r="I40" s="116"/>
-      <c r="J40" s="117"/>
+      <c r="G40" s="174"/>
+      <c r="H40" s="175"/>
+      <c r="I40" s="175"/>
+      <c r="J40" s="176"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="93" t="s">
+      <c r="T40" s="116" t="s">
         <v>170</v>
       </c>
-      <c r="U40" s="94"/>
-      <c r="V40" s="94"/>
-      <c r="W40" s="94"/>
-      <c r="X40" s="94"/>
-      <c r="Y40" s="94"/>
-      <c r="Z40" s="94"/>
-      <c r="AA40" s="94"/>
-      <c r="AB40" s="94"/>
-      <c r="AC40" s="95"/>
+      <c r="U40" s="117"/>
+      <c r="V40" s="117"/>
+      <c r="W40" s="117"/>
+      <c r="X40" s="117"/>
+      <c r="Y40" s="117"/>
+      <c r="Z40" s="117"/>
+      <c r="AA40" s="117"/>
+      <c r="AB40" s="117"/>
+      <c r="AC40" s="118"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="2">
@@ -5145,28 +5148,28 @@
       <c r="F41" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="G41" s="115"/>
-      <c r="H41" s="116"/>
-      <c r="I41" s="116"/>
-      <c r="J41" s="117"/>
+      <c r="G41" s="174"/>
+      <c r="H41" s="175"/>
+      <c r="I41" s="175"/>
+      <c r="J41" s="176"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="93" t="s">
+      <c r="T41" s="116" t="s">
         <v>171</v>
       </c>
-      <c r="U41" s="94"/>
-      <c r="V41" s="94"/>
-      <c r="W41" s="94"/>
-      <c r="X41" s="94"/>
-      <c r="Y41" s="94"/>
-      <c r="Z41" s="94"/>
-      <c r="AA41" s="94"/>
-      <c r="AB41" s="94"/>
-      <c r="AC41" s="95"/>
+      <c r="U41" s="117"/>
+      <c r="V41" s="117"/>
+      <c r="W41" s="117"/>
+      <c r="X41" s="117"/>
+      <c r="Y41" s="117"/>
+      <c r="Z41" s="117"/>
+      <c r="AA41" s="117"/>
+      <c r="AB41" s="117"/>
+      <c r="AC41" s="118"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="2">
@@ -5184,28 +5187,28 @@
       <c r="F42" s="76" t="s">
         <v>176</v>
       </c>
-      <c r="G42" s="114"/>
-      <c r="H42" s="98"/>
-      <c r="I42" s="98"/>
-      <c r="J42" s="99"/>
+      <c r="G42" s="173"/>
+      <c r="H42" s="162"/>
+      <c r="I42" s="162"/>
+      <c r="J42" s="163"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="T42" s="93" t="s">
+      <c r="T42" s="116" t="s">
         <v>172</v>
       </c>
-      <c r="U42" s="94"/>
-      <c r="V42" s="94"/>
-      <c r="W42" s="94"/>
-      <c r="X42" s="94"/>
-      <c r="Y42" s="94"/>
-      <c r="Z42" s="94"/>
-      <c r="AA42" s="94"/>
-      <c r="AB42" s="94"/>
-      <c r="AC42" s="95"/>
+      <c r="U42" s="117"/>
+      <c r="V42" s="117"/>
+      <c r="W42" s="117"/>
+      <c r="X42" s="117"/>
+      <c r="Y42" s="117"/>
+      <c r="Z42" s="117"/>
+      <c r="AA42" s="117"/>
+      <c r="AB42" s="117"/>
+      <c r="AC42" s="118"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="2">
@@ -5223,30 +5226,30 @@
       <c r="F43" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="G43" s="172" t="s">
+      <c r="G43" s="92" t="s">
         <v>192</v>
       </c>
-      <c r="H43" s="100"/>
-      <c r="I43" s="100"/>
-      <c r="J43" s="101"/>
+      <c r="H43" s="93"/>
+      <c r="I43" s="93"/>
+      <c r="J43" s="94"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="T43" s="93" t="s">
+      <c r="T43" s="116" t="s">
         <v>173</v>
       </c>
-      <c r="U43" s="94"/>
-      <c r="V43" s="94"/>
-      <c r="W43" s="94"/>
-      <c r="X43" s="94"/>
-      <c r="Y43" s="94"/>
-      <c r="Z43" s="94"/>
-      <c r="AA43" s="94"/>
-      <c r="AB43" s="94"/>
-      <c r="AC43" s="95"/>
+      <c r="U43" s="117"/>
+      <c r="V43" s="117"/>
+      <c r="W43" s="117"/>
+      <c r="X43" s="117"/>
+      <c r="Y43" s="117"/>
+      <c r="Z43" s="117"/>
+      <c r="AA43" s="117"/>
+      <c r="AB43" s="117"/>
+      <c r="AC43" s="118"/>
     </row>
     <row r="44" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="2">
@@ -5267,21 +5270,21 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="102" t="s">
+      <c r="S44" s="164" t="s">
         <v>76</v>
       </c>
-      <c r="T44" s="104" t="s">
+      <c r="T44" s="166" t="s">
         <v>174</v>
       </c>
-      <c r="U44" s="105"/>
-      <c r="V44" s="105"/>
-      <c r="W44" s="105"/>
-      <c r="X44" s="105"/>
-      <c r="Y44" s="105"/>
-      <c r="Z44" s="105"/>
-      <c r="AA44" s="105"/>
-      <c r="AB44" s="105"/>
-      <c r="AC44" s="106"/>
+      <c r="U44" s="167"/>
+      <c r="V44" s="167"/>
+      <c r="W44" s="167"/>
+      <c r="X44" s="167"/>
+      <c r="Y44" s="167"/>
+      <c r="Z44" s="167"/>
+      <c r="AA44" s="167"/>
+      <c r="AB44" s="167"/>
+      <c r="AC44" s="168"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="2">
@@ -5299,26 +5302,26 @@
       <c r="F45" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="G45" s="113" t="s">
+      <c r="G45" s="172" t="s">
         <v>181</v>
       </c>
-      <c r="H45" s="96"/>
-      <c r="I45" s="96"/>
-      <c r="J45" s="97"/>
+      <c r="H45" s="160"/>
+      <c r="I45" s="160"/>
+      <c r="J45" s="161"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="103"/>
-      <c r="T45" s="107"/>
-      <c r="U45" s="108"/>
-      <c r="V45" s="108"/>
-      <c r="W45" s="108"/>
-      <c r="X45" s="108"/>
-      <c r="Y45" s="108"/>
-      <c r="Z45" s="108"/>
-      <c r="AA45" s="108"/>
-      <c r="AB45" s="108"/>
-      <c r="AC45" s="109"/>
+      <c r="S45" s="165"/>
+      <c r="T45" s="169"/>
+      <c r="U45" s="170"/>
+      <c r="V45" s="170"/>
+      <c r="W45" s="170"/>
+      <c r="X45" s="170"/>
+      <c r="Y45" s="170"/>
+      <c r="Z45" s="170"/>
+      <c r="AA45" s="170"/>
+      <c r="AB45" s="170"/>
+      <c r="AC45" s="171"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B46" s="2">
@@ -5336,28 +5339,28 @@
       <c r="F46" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G46" s="114"/>
-      <c r="H46" s="98"/>
-      <c r="I46" s="98"/>
-      <c r="J46" s="99"/>
+      <c r="G46" s="173"/>
+      <c r="H46" s="162"/>
+      <c r="I46" s="162"/>
+      <c r="J46" s="163"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="T46" s="110" t="s">
+      <c r="T46" s="137" t="s">
         <v>175</v>
       </c>
-      <c r="U46" s="111"/>
-      <c r="V46" s="111"/>
-      <c r="W46" s="111"/>
-      <c r="X46" s="111"/>
-      <c r="Y46" s="111"/>
-      <c r="Z46" s="111"/>
-      <c r="AA46" s="111"/>
-      <c r="AB46" s="111"/>
-      <c r="AC46" s="112"/>
+      <c r="U46" s="138"/>
+      <c r="V46" s="138"/>
+      <c r="W46" s="138"/>
+      <c r="X46" s="138"/>
+      <c r="Y46" s="138"/>
+      <c r="Z46" s="138"/>
+      <c r="AA46" s="138"/>
+      <c r="AB46" s="138"/>
+      <c r="AC46" s="139"/>
     </row>
     <row r="47" spans="2:29" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="2">
@@ -5375,14 +5378,14 @@
       <c r="F47" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="G47" s="100" t="s">
+      <c r="G47" s="93" t="s">
         <v>152</v>
       </c>
-      <c r="H47" s="100"/>
-      <c r="I47" s="100"/>
-      <c r="J47" s="101"/>
-    </row>
-    <row r="48" spans="2:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="H47" s="93"/>
+      <c r="I47" s="93"/>
+      <c r="J47" s="94"/>
+    </row>
+    <row r="48" spans="2:29" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B48" s="2">
         <v>12</v>
       </c>
@@ -5399,7 +5402,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="49" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="2">
         <v>13</v>
       </c>
@@ -5407,14 +5410,20 @@
         <v>138</v>
       </c>
       <c r="D49" s="35" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>130</v>
       </c>
       <c r="F49" s="35" t="s">
-        <v>141</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="G49" s="172" t="s">
+        <v>155</v>
+      </c>
+      <c r="H49" s="160"/>
+      <c r="I49" s="160"/>
+      <c r="J49" s="161"/>
     </row>
     <row r="50" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="2">
@@ -5432,12 +5441,10 @@
       <c r="F50" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="G50" s="96" t="s">
-        <v>155</v>
-      </c>
-      <c r="H50" s="96"/>
-      <c r="I50" s="96"/>
-      <c r="J50" s="97"/>
+      <c r="G50" s="174"/>
+      <c r="H50" s="177"/>
+      <c r="I50" s="177"/>
+      <c r="J50" s="176"/>
     </row>
     <row r="51" spans="2:10" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" s="4">
@@ -5455,38 +5462,38 @@
       <c r="F51" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="G51" s="98"/>
-      <c r="H51" s="98"/>
-      <c r="I51" s="98"/>
-      <c r="J51" s="99"/>
+      <c r="G51" s="173"/>
+      <c r="H51" s="162"/>
+      <c r="I51" s="162"/>
+      <c r="J51" s="163"/>
     </row>
     <row r="52" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="167" t="s">
+      <c r="B52" s="109" t="s">
         <v>142</v>
       </c>
-      <c r="C52" s="148"/>
-      <c r="D52" s="148"/>
-      <c r="E52" s="148"/>
-      <c r="F52" s="149"/>
+      <c r="C52" s="110"/>
+      <c r="D52" s="110"/>
+      <c r="E52" s="110"/>
+      <c r="F52" s="111"/>
     </row>
     <row r="54" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B55" s="161" t="s">
+      <c r="B55" s="103" t="s">
         <v>183</v>
       </c>
-      <c r="C55" s="159" t="s">
+      <c r="C55" s="101" t="s">
         <v>185</v>
       </c>
-      <c r="D55" s="173" t="s">
+      <c r="D55" s="95" t="s">
         <v>184</v>
       </c>
-      <c r="E55" s="174"/>
+      <c r="E55" s="96"/>
     </row>
     <row r="56" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="162"/>
-      <c r="C56" s="160"/>
-      <c r="D56" s="175"/>
-      <c r="E56" s="176"/>
+      <c r="B56" s="104"/>
+      <c r="C56" s="102"/>
+      <c r="D56" s="97"/>
+      <c r="E56" s="98"/>
     </row>
     <row r="57" spans="2:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="81">
@@ -5495,10 +5502,10 @@
       <c r="C57" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D57" s="90" t="s">
+      <c r="D57" s="99" t="s">
         <v>207</v>
       </c>
-      <c r="E57" s="92"/>
+      <c r="E57" s="100"/>
     </row>
     <row r="58" spans="2:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="82">
@@ -5507,10 +5514,10 @@
       <c r="C58" s="86" t="s">
         <v>203</v>
       </c>
-      <c r="D58" s="163" t="s">
+      <c r="D58" s="88" t="s">
         <v>206</v>
       </c>
-      <c r="E58" s="164"/>
+      <c r="E58" s="89"/>
     </row>
     <row r="59" spans="2:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="82">
@@ -5519,10 +5526,10 @@
       <c r="C59" s="38" t="s">
         <v>204</v>
       </c>
-      <c r="D59" s="163" t="s">
+      <c r="D59" s="88" t="s">
         <v>205</v>
       </c>
-      <c r="E59" s="164"/>
+      <c r="E59" s="89"/>
     </row>
     <row r="60" spans="2:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="82">
@@ -5531,10 +5538,10 @@
       <c r="C60" s="86" t="s">
         <v>186</v>
       </c>
-      <c r="D60" s="163" t="s">
+      <c r="D60" s="88" t="s">
         <v>189</v>
       </c>
-      <c r="E60" s="164"/>
+      <c r="E60" s="89"/>
     </row>
     <row r="61" spans="2:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="82">
@@ -5543,10 +5550,10 @@
       <c r="C61" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="D61" s="163" t="s">
+      <c r="D61" s="88" t="s">
         <v>190</v>
       </c>
-      <c r="E61" s="164"/>
+      <c r="E61" s="89"/>
     </row>
     <row r="62" spans="2:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="82">
@@ -5555,10 +5562,10 @@
       <c r="C62" s="38" t="s">
         <v>188</v>
       </c>
-      <c r="D62" s="163" t="s">
+      <c r="D62" s="88" t="s">
         <v>191</v>
       </c>
-      <c r="E62" s="164"/>
+      <c r="E62" s="89"/>
     </row>
     <row r="63" spans="2:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="82">
@@ -5567,102 +5574,201 @@
       <c r="C63" s="86" t="s">
         <v>196</v>
       </c>
-      <c r="D63" s="163" t="s">
+      <c r="D63" s="88" t="s">
         <v>197</v>
       </c>
-      <c r="E63" s="164"/>
+      <c r="E63" s="89"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B64" s="82">
         <v>7</v>
       </c>
       <c r="C64" s="86"/>
-      <c r="D64" s="163"/>
-      <c r="E64" s="164"/>
+      <c r="D64" s="88"/>
+      <c r="E64" s="89"/>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="82">
         <v>8</v>
       </c>
       <c r="C65" s="86"/>
-      <c r="D65" s="163"/>
-      <c r="E65" s="164"/>
+      <c r="D65" s="88"/>
+      <c r="E65" s="89"/>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" s="82">
         <v>9</v>
       </c>
       <c r="C66" s="86"/>
-      <c r="D66" s="163"/>
-      <c r="E66" s="164"/>
+      <c r="D66" s="88"/>
+      <c r="E66" s="89"/>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" s="82">
         <v>10</v>
       </c>
       <c r="C67" s="86"/>
-      <c r="D67" s="163"/>
-      <c r="E67" s="164"/>
+      <c r="D67" s="88"/>
+      <c r="E67" s="89"/>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" s="82">
         <v>11</v>
       </c>
       <c r="C68" s="86"/>
-      <c r="D68" s="163"/>
-      <c r="E68" s="164"/>
+      <c r="D68" s="88"/>
+      <c r="E68" s="89"/>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69" s="82">
         <v>12</v>
       </c>
       <c r="C69" s="86"/>
-      <c r="D69" s="163"/>
-      <c r="E69" s="164"/>
+      <c r="D69" s="88"/>
+      <c r="E69" s="89"/>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B70" s="82">
         <v>13</v>
       </c>
       <c r="C70" s="86"/>
-      <c r="D70" s="163"/>
-      <c r="E70" s="164"/>
+      <c r="D70" s="88"/>
+      <c r="E70" s="89"/>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B71" s="82">
         <v>14</v>
       </c>
       <c r="C71" s="86"/>
-      <c r="D71" s="163"/>
-      <c r="E71" s="164"/>
+      <c r="D71" s="88"/>
+      <c r="E71" s="89"/>
     </row>
     <row r="72" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B72" s="83">
         <v>15</v>
       </c>
       <c r="C72" s="87"/>
-      <c r="D72" s="170"/>
-      <c r="E72" s="171"/>
+      <c r="D72" s="90"/>
+      <c r="E72" s="91"/>
     </row>
   </sheetData>
   <mergeCells count="158">
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D55:E56"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="T30:AC30"/>
+    <mergeCell ref="T31:AC31"/>
+    <mergeCell ref="T32:AC32"/>
+    <mergeCell ref="T33:AC33"/>
+    <mergeCell ref="T34:AC34"/>
+    <mergeCell ref="T35:AC35"/>
+    <mergeCell ref="T36:AC36"/>
+    <mergeCell ref="T37:AC37"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="S38:S39"/>
+    <mergeCell ref="T38:AC39"/>
+    <mergeCell ref="S44:S45"/>
+    <mergeCell ref="T44:AC45"/>
+    <mergeCell ref="T40:AC40"/>
+    <mergeCell ref="T41:AC41"/>
+    <mergeCell ref="T42:AC42"/>
+    <mergeCell ref="T43:AC43"/>
+    <mergeCell ref="T46:AC46"/>
+    <mergeCell ref="G45:J46"/>
+    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="AA20:AB20"/>
+    <mergeCell ref="AA21:AB21"/>
+    <mergeCell ref="AA22:AB22"/>
+    <mergeCell ref="AA15:AB15"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="U4:V4"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="U22:V22"/>
+    <mergeCell ref="U21:V21"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V6"/>
+    <mergeCell ref="U7:V7"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="U9:V9"/>
+    <mergeCell ref="U20:V20"/>
+    <mergeCell ref="U15:V15"/>
+    <mergeCell ref="U16:V16"/>
+    <mergeCell ref="U17:V17"/>
+    <mergeCell ref="U18:V18"/>
+    <mergeCell ref="U19:V19"/>
+    <mergeCell ref="U10:V10"/>
+    <mergeCell ref="U11:V11"/>
+    <mergeCell ref="AA23:AB23"/>
+    <mergeCell ref="AA6:AB6"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AA17:AB17"/>
+    <mergeCell ref="AA18:AB18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="N13:P13"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="N24:P24"/>
+    <mergeCell ref="E27:J27"/>
+    <mergeCell ref="E22:J22"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K2:P2"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="N26:P26"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AA11:AB11"/>
     <mergeCell ref="C55:C56"/>
     <mergeCell ref="B55:B56"/>
     <mergeCell ref="D58:E58"/>
@@ -5687,123 +5793,24 @@
     <mergeCell ref="N20:P20"/>
     <mergeCell ref="N21:P21"/>
     <mergeCell ref="N23:P23"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AA11:AB11"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="N27:P27"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="E28:J28"/>
-    <mergeCell ref="N24:P24"/>
-    <mergeCell ref="E27:J27"/>
-    <mergeCell ref="E22:J22"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K2:P2"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AA17:AB17"/>
-    <mergeCell ref="AA18:AB18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="AA19:AB19"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="AA20:AB20"/>
-    <mergeCell ref="AA21:AB21"/>
-    <mergeCell ref="AA22:AB22"/>
-    <mergeCell ref="AA15:AB15"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="U4:V4"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="U22:V22"/>
-    <mergeCell ref="U21:V21"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V6"/>
-    <mergeCell ref="U7:V7"/>
-    <mergeCell ref="U8:V8"/>
-    <mergeCell ref="U9:V9"/>
-    <mergeCell ref="U20:V20"/>
-    <mergeCell ref="U15:V15"/>
-    <mergeCell ref="U16:V16"/>
-    <mergeCell ref="U17:V17"/>
-    <mergeCell ref="U18:V18"/>
-    <mergeCell ref="U19:V19"/>
-    <mergeCell ref="U10:V10"/>
-    <mergeCell ref="U11:V11"/>
-    <mergeCell ref="AA23:AB23"/>
-    <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="T30:AC30"/>
-    <mergeCell ref="T31:AC31"/>
-    <mergeCell ref="T32:AC32"/>
-    <mergeCell ref="T33:AC33"/>
-    <mergeCell ref="T34:AC34"/>
-    <mergeCell ref="T35:AC35"/>
-    <mergeCell ref="T36:AC36"/>
-    <mergeCell ref="T37:AC37"/>
-    <mergeCell ref="G50:J51"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="S38:S39"/>
-    <mergeCell ref="T38:AC39"/>
-    <mergeCell ref="S44:S45"/>
-    <mergeCell ref="T44:AC45"/>
-    <mergeCell ref="T40:AC40"/>
-    <mergeCell ref="T41:AC41"/>
-    <mergeCell ref="T42:AC42"/>
-    <mergeCell ref="T43:AC43"/>
-    <mergeCell ref="T46:AC46"/>
-    <mergeCell ref="G45:J46"/>
-    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D55:E56"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="G49:J51"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Se creo el sistema ECAM, tanto tipo 1 como tipo 0. Tambien se documento las posiciones de datos dentro del ECAM
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BA19C1-875F-463A-86B6-57AFA879B049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{859BADAC-C186-402D-8BA3-9977ED71BF21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="233">
   <si>
     <t>OpCode</t>
   </si>
@@ -660,13 +660,88 @@
   </si>
   <si>
     <t xml:space="preserve">No Excepción </t>
+  </si>
+  <si>
+    <t>Dispositivo</t>
+  </si>
+  <si>
+    <t>Bus Lógico</t>
+  </si>
+  <si>
+    <t>Dispositivo (ID)</t>
+  </si>
+  <si>
+    <t>Función</t>
+  </si>
+  <si>
+    <t>Offset ECAM (Hex)</t>
+  </si>
+  <si>
+    <t>Dirección Base ECAM + (Bus &lt;&lt; 20) + (Device_X &lt;&lt; 15) + (Function_0 &lt;&lt; 12)</t>
+  </si>
+  <si>
+    <t>ECAM</t>
+  </si>
+  <si>
+    <t>Bus</t>
+  </si>
+  <si>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>E0000000</t>
+  </si>
+  <si>
+    <t>Res Max</t>
+  </si>
+  <si>
+    <t>fff</t>
+  </si>
+  <si>
+    <t>Extensión 1</t>
+  </si>
+  <si>
+    <t>Extensión 2</t>
+  </si>
+  <si>
+    <t>Extensión 3</t>
+  </si>
+  <si>
+    <t>Extensión 4</t>
+  </si>
+  <si>
+    <t>Extensión 5</t>
+  </si>
+  <si>
+    <t>Extensión 6</t>
+  </si>
+  <si>
+    <t>Extensión 7</t>
+  </si>
+  <si>
+    <t>Extensión 8</t>
+  </si>
+  <si>
+    <t>Extesión Rápida 1</t>
+  </si>
+  <si>
+    <t>Extesión Rápida 2</t>
+  </si>
+  <si>
+    <t>LVC Switch</t>
+  </si>
+  <si>
+    <t>MMIO Controller</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -694,6 +769,25 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Google Sans Text"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1660,7 +1754,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="204">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1923,6 +2017,123 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1956,11 +2167,23 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2007,15 +2230,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2058,9 +2272,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2070,15 +2281,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2139,18 +2341,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2174,24 +2364,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2473,8 +2645,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:AI72"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:AI71"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="15"/>
     <col min="2" max="3" width="19.85546875" style="15" customWidth="1"/>
@@ -2487,75 +2659,74 @@
     <col min="14" max="14" width="22.28515625" style="15" customWidth="1"/>
     <col min="15" max="15" width="18.7109375" style="15" customWidth="1"/>
     <col min="16" max="16" width="20" style="15" customWidth="1"/>
-    <col min="17" max="18" width="9.140625" style="15"/>
-    <col min="19" max="19" width="12.140625" style="15" customWidth="1"/>
-    <col min="20" max="20" width="10.7109375" style="15" customWidth="1"/>
-    <col min="21" max="21" width="6.85546875" style="15" customWidth="1"/>
-    <col min="22" max="22" width="6.42578125" style="15" customWidth="1"/>
+    <col min="17" max="17" width="9.140625" style="15" customWidth="1"/>
+    <col min="18" max="20" width="22.28515625" style="15" customWidth="1"/>
+    <col min="21" max="21" width="11.140625" style="15" customWidth="1"/>
+    <col min="22" max="22" width="16" style="15" customWidth="1"/>
     <col min="23" max="26" width="10.7109375" style="15" customWidth="1"/>
     <col min="27" max="28" width="6" style="15" customWidth="1"/>
     <col min="29" max="35" width="10.7109375" style="15" customWidth="1"/>
     <col min="36" max="16384" width="9.140625" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="134" t="s">
+    <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
+    <row r="2" spans="2:35" ht="15.75" thickBot="1">
+      <c r="B2" s="173" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="149" t="s">
+      <c r="C2" s="185" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="150"/>
-      <c r="E2" s="151" t="s">
+      <c r="D2" s="186"/>
+      <c r="E2" s="187" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="151"/>
-      <c r="G2" s="152" t="s">
+      <c r="F2" s="187"/>
+      <c r="G2" s="188" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="151"/>
-      <c r="I2" s="151" t="s">
+      <c r="H2" s="187"/>
+      <c r="I2" s="187" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="151"/>
-      <c r="K2" s="153" t="s">
+      <c r="J2" s="187"/>
+      <c r="K2" s="189" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="151"/>
-      <c r="M2" s="151"/>
-      <c r="N2" s="151"/>
-      <c r="O2" s="151"/>
-      <c r="P2" s="154"/>
-      <c r="R2" s="130" t="s">
+      <c r="L2" s="187"/>
+      <c r="M2" s="187"/>
+      <c r="N2" s="187"/>
+      <c r="O2" s="187"/>
+      <c r="P2" s="190"/>
+      <c r="R2" s="170" t="s">
         <v>66</v>
       </c>
-      <c r="S2" s="127" t="s">
+      <c r="S2" s="167" t="s">
         <v>67</v>
       </c>
-      <c r="T2" s="120" t="s">
+      <c r="T2" s="160" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="121"/>
-      <c r="V2" s="121"/>
-      <c r="W2" s="121"/>
-      <c r="X2" s="121"/>
-      <c r="Y2" s="121"/>
-      <c r="Z2" s="121"/>
-      <c r="AA2" s="121"/>
-      <c r="AB2" s="121" t="s">
+      <c r="U2" s="161"/>
+      <c r="V2" s="161"/>
+      <c r="W2" s="161"/>
+      <c r="X2" s="161"/>
+      <c r="Y2" s="161"/>
+      <c r="Z2" s="161"/>
+      <c r="AA2" s="161"/>
+      <c r="AB2" s="161" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="121"/>
-      <c r="AD2" s="121"/>
-      <c r="AE2" s="121"/>
-      <c r="AF2" s="121"/>
-      <c r="AG2" s="121"/>
-      <c r="AH2" s="121"/>
-      <c r="AI2" s="122"/>
-    </row>
-    <row r="3" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="135"/>
+      <c r="AC2" s="161"/>
+      <c r="AD2" s="161"/>
+      <c r="AE2" s="161"/>
+      <c r="AF2" s="161"/>
+      <c r="AG2" s="161"/>
+      <c r="AH2" s="161"/>
+      <c r="AI2" s="162"/>
+    </row>
+    <row r="3" spans="2:35" ht="15.75" thickBot="1">
+      <c r="B3" s="174"/>
       <c r="C3" s="16" t="s">
         <v>80</v>
       </c>
@@ -2580,21 +2751,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="105"/>
-      <c r="L3" s="148"/>
-      <c r="M3" s="148"/>
-      <c r="N3" s="148"/>
-      <c r="O3" s="148"/>
-      <c r="P3" s="106"/>
-      <c r="R3" s="131"/>
-      <c r="S3" s="128"/>
+      <c r="K3" s="148"/>
+      <c r="L3" s="184"/>
+      <c r="M3" s="184"/>
+      <c r="N3" s="184"/>
+      <c r="O3" s="184"/>
+      <c r="P3" s="149"/>
+      <c r="R3" s="171"/>
+      <c r="S3" s="168"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="158" t="s">
+      <c r="U3" s="194" t="s">
         <v>84</v>
       </c>
-      <c r="V3" s="158"/>
+      <c r="V3" s="194"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -2607,10 +2778,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="119" t="s">
+      <c r="AA3" s="159" t="s">
         <v>75</v>
       </c>
-      <c r="AB3" s="119"/>
+      <c r="AB3" s="159"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -2633,22 +2804,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="136"/>
+    <row r="4" spans="2:35" ht="15.75" thickBot="1">
+      <c r="B4" s="175"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="123" t="s">
+      <c r="E4" s="163" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
-      <c r="H4" s="110"/>
-      <c r="I4" s="110"/>
-      <c r="J4" s="111"/>
+      <c r="F4" s="153"/>
+      <c r="G4" s="153"/>
+      <c r="H4" s="153"/>
+      <c r="I4" s="153"/>
+      <c r="J4" s="154"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -2658,20 +2829,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="123" t="s">
+      <c r="N4" s="163" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="110"/>
-      <c r="P4" s="111"/>
-      <c r="R4" s="132"/>
-      <c r="S4" s="129"/>
+      <c r="O4" s="153"/>
+      <c r="P4" s="154"/>
+      <c r="R4" s="172"/>
+      <c r="S4" s="169"/>
       <c r="T4" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="U4" s="123" t="s">
+      <c r="U4" s="163" t="s">
         <v>76</v>
       </c>
-      <c r="V4" s="124"/>
+      <c r="V4" s="164"/>
       <c r="W4" s="7" t="s">
         <v>72</v>
       </c>
@@ -2684,10 +2855,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="123" t="s">
+      <c r="AA4" s="163" t="s">
         <v>73</v>
       </c>
-      <c r="AB4" s="124"/>
+      <c r="AB4" s="164"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -2710,7 +2881,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:35" ht="15.75" thickBot="1">
       <c r="B5" s="1">
         <v>0</v>
       </c>
@@ -2719,22 +2890,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="155"/>
-      <c r="F5" s="156"/>
-      <c r="G5" s="156"/>
-      <c r="H5" s="156"/>
-      <c r="I5" s="156"/>
-      <c r="J5" s="157"/>
+      <c r="E5" s="191"/>
+      <c r="F5" s="192"/>
+      <c r="G5" s="192"/>
+      <c r="H5" s="192"/>
+      <c r="I5" s="192"/>
+      <c r="J5" s="193"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="99" t="s">
+      <c r="N5" s="121" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="133"/>
-      <c r="P5" s="100"/>
+      <c r="O5" s="122"/>
+      <c r="P5" s="123"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -2744,10 +2915,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="125" t="s">
+      <c r="U5" s="165" t="s">
         <v>74</v>
       </c>
-      <c r="V5" s="126"/>
+      <c r="V5" s="166"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -2760,10 +2931,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="125" t="s">
+      <c r="AA5" s="165" t="s">
         <v>74</v>
       </c>
-      <c r="AB5" s="126"/>
+      <c r="AB5" s="166"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -2786,7 +2957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:35" ht="15.75" thickBot="1">
       <c r="B6" s="2">
         <v>1</v>
       </c>
@@ -2795,12 +2966,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="146"/>
-      <c r="F6" s="141"/>
-      <c r="G6" s="141"/>
-      <c r="H6" s="141"/>
-      <c r="I6" s="141"/>
-      <c r="J6" s="142"/>
+      <c r="E6" s="182"/>
+      <c r="F6" s="177"/>
+      <c r="G6" s="177"/>
+      <c r="H6" s="177"/>
+      <c r="I6" s="177"/>
+      <c r="J6" s="178"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -2808,11 +2979,11 @@
         <v>156</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="116" t="s">
+      <c r="N6" s="118" t="s">
         <v>96</v>
       </c>
-      <c r="O6" s="117"/>
-      <c r="P6" s="118"/>
+      <c r="O6" s="119"/>
+      <c r="P6" s="120"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -2822,10 +2993,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="112" t="s">
+      <c r="U6" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V6" s="113"/>
+      <c r="V6" s="156"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -2838,10 +3009,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="112" t="s">
+      <c r="AA6" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB6" s="113"/>
+      <c r="AB6" s="156"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -2864,7 +3035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:35" ht="15.75" thickBot="1">
       <c r="B7" s="2">
         <v>2</v>
       </c>
@@ -2882,9 +3053,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="140"/>
-      <c r="I7" s="141"/>
-      <c r="J7" s="142"/>
+      <c r="H7" s="176"/>
+      <c r="I7" s="177"/>
+      <c r="J7" s="178"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -2892,11 +3063,11 @@
       <c r="M7" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N7" s="116" t="s">
+      <c r="N7" s="118" t="s">
         <v>53</v>
       </c>
-      <c r="O7" s="117"/>
-      <c r="P7" s="118"/>
+      <c r="O7" s="119"/>
+      <c r="P7" s="120"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -2906,10 +3077,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="112" t="s">
+      <c r="U7" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V7" s="113"/>
+      <c r="V7" s="156"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -2922,10 +3093,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="112" t="s">
+      <c r="AA7" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB7" s="113"/>
+      <c r="AB7" s="156"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -2948,7 +3119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:35" ht="15.75" thickBot="1">
       <c r="B8" s="2">
         <v>3</v>
       </c>
@@ -2966,9 +3137,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="140"/>
-      <c r="I8" s="141"/>
-      <c r="J8" s="142"/>
+      <c r="H8" s="176"/>
+      <c r="I8" s="177"/>
+      <c r="J8" s="178"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -2976,11 +3147,11 @@
       <c r="M8" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N8" s="116" t="s">
+      <c r="N8" s="118" t="s">
         <v>54</v>
       </c>
-      <c r="O8" s="117"/>
-      <c r="P8" s="118"/>
+      <c r="O8" s="119"/>
+      <c r="P8" s="120"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -2990,10 +3161,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="112" t="s">
+      <c r="U8" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V8" s="113"/>
+      <c r="V8" s="156"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -3006,10 +3177,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="112" t="s">
+      <c r="AA8" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB8" s="113"/>
+      <c r="AB8" s="156"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -3032,7 +3203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:35" ht="15.75" thickBot="1">
       <c r="B9" s="1">
         <v>4</v>
       </c>
@@ -3050,9 +3221,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="140"/>
-      <c r="I9" s="141"/>
-      <c r="J9" s="142"/>
+      <c r="H9" s="176"/>
+      <c r="I9" s="177"/>
+      <c r="J9" s="178"/>
       <c r="K9" s="37" t="s">
         <v>48</v>
       </c>
@@ -3060,11 +3231,11 @@
       <c r="M9" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N9" s="116" t="s">
+      <c r="N9" s="118" t="s">
         <v>55</v>
       </c>
-      <c r="O9" s="117"/>
-      <c r="P9" s="118"/>
+      <c r="O9" s="119"/>
+      <c r="P9" s="120"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -3074,10 +3245,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="112" t="s">
+      <c r="U9" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V9" s="113"/>
+      <c r="V9" s="156"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -3090,10 +3261,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="112" t="s">
+      <c r="AA9" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB9" s="113"/>
+      <c r="AB9" s="156"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -3116,7 +3287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:35" ht="15.75" thickBot="1">
       <c r="B10" s="2">
         <v>5</v>
       </c>
@@ -3134,9 +3305,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="140"/>
-      <c r="I10" s="141"/>
-      <c r="J10" s="142"/>
+      <c r="H10" s="176"/>
+      <c r="I10" s="177"/>
+      <c r="J10" s="178"/>
       <c r="K10" s="37" t="s">
         <v>49</v>
       </c>
@@ -3144,11 +3315,11 @@
       <c r="M10" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N10" s="116" t="s">
+      <c r="N10" s="118" t="s">
         <v>56</v>
       </c>
-      <c r="O10" s="117"/>
-      <c r="P10" s="118"/>
+      <c r="O10" s="119"/>
+      <c r="P10" s="120"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -3158,10 +3329,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="112" t="s">
+      <c r="U10" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V10" s="113"/>
+      <c r="V10" s="156"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -3174,10 +3345,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="112" t="s">
+      <c r="AA10" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB10" s="113"/>
+      <c r="AB10" s="156"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -3200,7 +3371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:35" ht="15.75" thickBot="1">
       <c r="B11" s="2">
         <v>6</v>
       </c>
@@ -3218,9 +3389,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="140"/>
-      <c r="I11" s="141"/>
-      <c r="J11" s="142"/>
+      <c r="H11" s="176"/>
+      <c r="I11" s="177"/>
+      <c r="J11" s="178"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -3228,11 +3399,11 @@
       <c r="M11" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N11" s="116" t="s">
+      <c r="N11" s="118" t="s">
         <v>57</v>
       </c>
-      <c r="O11" s="117"/>
-      <c r="P11" s="118"/>
+      <c r="O11" s="119"/>
+      <c r="P11" s="120"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -3242,10 +3413,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="112" t="s">
+      <c r="U11" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V11" s="113"/>
+      <c r="V11" s="156"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -3258,10 +3429,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="112" t="s">
+      <c r="AA11" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB11" s="113"/>
+      <c r="AB11" s="156"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -3284,7 +3455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:35" ht="15.75" thickBot="1">
       <c r="B12" s="2">
         <v>7</v>
       </c>
@@ -3302,9 +3473,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="140"/>
-      <c r="I12" s="141"/>
-      <c r="J12" s="142"/>
+      <c r="H12" s="176"/>
+      <c r="I12" s="177"/>
+      <c r="J12" s="178"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -3312,11 +3483,11 @@
       <c r="M12" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N12" s="116" t="s">
+      <c r="N12" s="118" t="s">
         <v>58</v>
       </c>
-      <c r="O12" s="117"/>
-      <c r="P12" s="118"/>
+      <c r="O12" s="119"/>
+      <c r="P12" s="120"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -3326,10 +3497,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="112" t="s">
+      <c r="U12" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V12" s="113"/>
+      <c r="V12" s="156"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -3342,10 +3513,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="112" t="s">
+      <c r="AA12" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB12" s="113"/>
+      <c r="AB12" s="156"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -3368,7 +3539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:35" ht="15.75" thickBot="1">
       <c r="B13" s="1">
         <v>8</v>
       </c>
@@ -3386,9 +3557,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="140"/>
-      <c r="I13" s="141"/>
-      <c r="J13" s="142"/>
+      <c r="H13" s="176"/>
+      <c r="I13" s="177"/>
+      <c r="J13" s="178"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -3396,11 +3567,11 @@
       <c r="M13" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N13" s="116" t="s">
+      <c r="N13" s="118" t="s">
         <v>59</v>
       </c>
-      <c r="O13" s="117"/>
-      <c r="P13" s="118"/>
+      <c r="O13" s="119"/>
+      <c r="P13" s="120"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -3410,10 +3581,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="112" t="s">
+      <c r="U13" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V13" s="113"/>
+      <c r="V13" s="156"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -3426,10 +3597,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="112" t="s">
+      <c r="AA13" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB13" s="113"/>
+      <c r="AB13" s="156"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -3452,7 +3623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:35" ht="15.75" thickBot="1">
       <c r="B14" s="2">
         <v>9</v>
       </c>
@@ -3470,9 +3641,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="140"/>
-      <c r="I14" s="141"/>
-      <c r="J14" s="142"/>
+      <c r="H14" s="176"/>
+      <c r="I14" s="177"/>
+      <c r="J14" s="178"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -3480,11 +3651,11 @@
       <c r="M14" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N14" s="116" t="s">
+      <c r="N14" s="118" t="s">
         <v>60</v>
       </c>
-      <c r="O14" s="117"/>
-      <c r="P14" s="118"/>
+      <c r="O14" s="119"/>
+      <c r="P14" s="120"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -3494,10 +3665,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="112" t="s">
+      <c r="U14" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V14" s="113"/>
+      <c r="V14" s="156"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -3510,10 +3681,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="112" t="s">
+      <c r="AA14" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB14" s="113"/>
+      <c r="AB14" s="156"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -3536,7 +3707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:35" ht="15.75" thickBot="1">
       <c r="B15" s="2">
         <v>10</v>
       </c>
@@ -3554,9 +3725,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="140"/>
-      <c r="I15" s="141"/>
-      <c r="J15" s="142"/>
+      <c r="H15" s="176"/>
+      <c r="I15" s="177"/>
+      <c r="J15" s="178"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -3564,11 +3735,11 @@
       <c r="M15" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N15" s="116" t="s">
+      <c r="N15" s="118" t="s">
         <v>61</v>
       </c>
-      <c r="O15" s="117"/>
-      <c r="P15" s="118"/>
+      <c r="O15" s="119"/>
+      <c r="P15" s="120"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -3578,10 +3749,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="112" t="s">
+      <c r="U15" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V15" s="113"/>
+      <c r="V15" s="156"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -3594,10 +3765,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="112" t="s">
+      <c r="AA15" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB15" s="113"/>
+      <c r="AB15" s="156"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -3620,7 +3791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:35" ht="15.75" thickBot="1">
       <c r="B16" s="2">
         <v>11</v>
       </c>
@@ -3632,21 +3803,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="140"/>
-      <c r="G16" s="141"/>
-      <c r="H16" s="141"/>
-      <c r="I16" s="141"/>
-      <c r="J16" s="142"/>
+      <c r="F16" s="176"/>
+      <c r="G16" s="177"/>
+      <c r="H16" s="177"/>
+      <c r="I16" s="177"/>
+      <c r="J16" s="178"/>
       <c r="K16" s="40" t="s">
         <v>50</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="116" t="s">
+      <c r="N16" s="118" t="s">
         <v>51</v>
       </c>
-      <c r="O16" s="117"/>
-      <c r="P16" s="118"/>
+      <c r="O16" s="119"/>
+      <c r="P16" s="120"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -3656,10 +3827,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="112" t="s">
+      <c r="U16" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V16" s="113"/>
+      <c r="V16" s="156"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -3672,10 +3843,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="112" t="s">
+      <c r="AA16" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB16" s="113"/>
+      <c r="AB16" s="156"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -3698,7 +3869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:35" ht="15.75" thickBot="1">
       <c r="B17" s="2">
         <v>12</v>
       </c>
@@ -3711,22 +3882,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="147" t="s">
+      <c r="G17" s="183" t="s">
         <v>77</v>
       </c>
-      <c r="H17" s="117"/>
-      <c r="I17" s="117"/>
-      <c r="J17" s="118"/>
+      <c r="H17" s="119"/>
+      <c r="I17" s="119"/>
+      <c r="J17" s="120"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="116" t="s">
+      <c r="N17" s="118" t="s">
         <v>65</v>
       </c>
-      <c r="O17" s="117"/>
-      <c r="P17" s="118"/>
+      <c r="O17" s="119"/>
+      <c r="P17" s="120"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -3736,10 +3907,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="112" t="s">
+      <c r="U17" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V17" s="113"/>
+      <c r="V17" s="156"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -3752,10 +3923,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="112" t="s">
+      <c r="AA17" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB17" s="113"/>
+      <c r="AB17" s="156"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -3778,7 +3949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:35" ht="15.75" thickBot="1">
       <c r="B18" s="2">
         <v>13</v>
       </c>
@@ -3791,12 +3962,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="147" t="s">
+      <c r="G18" s="183" t="s">
         <v>77</v>
       </c>
-      <c r="H18" s="117"/>
-      <c r="I18" s="117"/>
-      <c r="J18" s="118"/>
+      <c r="H18" s="119"/>
+      <c r="I18" s="119"/>
+      <c r="J18" s="120"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -3804,11 +3975,11 @@
       <c r="M18" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N18" s="116" t="s">
+      <c r="N18" s="118" t="s">
         <v>62</v>
       </c>
-      <c r="O18" s="117"/>
-      <c r="P18" s="118"/>
+      <c r="O18" s="119"/>
+      <c r="P18" s="120"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -3818,10 +3989,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="112" t="s">
+      <c r="U18" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V18" s="113"/>
+      <c r="V18" s="156"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -3834,10 +4005,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="112" t="s">
+      <c r="AA18" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB18" s="113"/>
+      <c r="AB18" s="156"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -3860,7 +4031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:35" ht="15.75" thickBot="1">
       <c r="B19" s="2">
         <v>14</v>
       </c>
@@ -3875,20 +4046,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="140"/>
-      <c r="H19" s="141"/>
-      <c r="I19" s="141"/>
-      <c r="J19" s="142"/>
+      <c r="G19" s="176"/>
+      <c r="H19" s="177"/>
+      <c r="I19" s="177"/>
+      <c r="J19" s="178"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="116" t="s">
+      <c r="N19" s="118" t="s">
         <v>94</v>
       </c>
-      <c r="O19" s="117"/>
-      <c r="P19" s="118"/>
+      <c r="O19" s="119"/>
+      <c r="P19" s="120"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -3898,10 +4069,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="112" t="s">
+      <c r="U19" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V19" s="113"/>
+      <c r="V19" s="156"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -3914,10 +4085,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="112" t="s">
+      <c r="AA19" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB19" s="113"/>
+      <c r="AB19" s="156"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -3940,7 +4111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:35" ht="15.75" thickBot="1">
       <c r="B20" s="2">
         <v>15</v>
       </c>
@@ -3957,20 +4128,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="140"/>
-      <c r="H20" s="141"/>
-      <c r="I20" s="141"/>
-      <c r="J20" s="142"/>
+      <c r="G20" s="176"/>
+      <c r="H20" s="177"/>
+      <c r="I20" s="177"/>
+      <c r="J20" s="178"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="116" t="s">
+      <c r="N20" s="118" t="s">
         <v>95</v>
       </c>
-      <c r="O20" s="117"/>
-      <c r="P20" s="118"/>
+      <c r="O20" s="119"/>
+      <c r="P20" s="120"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -3980,10 +4151,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="112" t="s">
+      <c r="U20" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V20" s="113"/>
+      <c r="V20" s="156"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -3996,10 +4167,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="112" t="s">
+      <c r="AA20" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB20" s="113"/>
+      <c r="AB20" s="156"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -4022,7 +4193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:35" ht="15.75" thickBot="1">
       <c r="B21" s="2">
         <v>16</v>
       </c>
@@ -4037,20 +4208,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="140"/>
-      <c r="H21" s="141"/>
-      <c r="I21" s="141"/>
-      <c r="J21" s="142"/>
+      <c r="G21" s="176"/>
+      <c r="H21" s="177"/>
+      <c r="I21" s="177"/>
+      <c r="J21" s="178"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="116" t="s">
+      <c r="N21" s="118" t="s">
         <v>63</v>
       </c>
-      <c r="O21" s="117"/>
-      <c r="P21" s="118"/>
+      <c r="O21" s="119"/>
+      <c r="P21" s="120"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -4060,10 +4231,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="112" t="s">
+      <c r="U21" s="155" t="s">
         <v>97</v>
       </c>
-      <c r="V21" s="113"/>
+      <c r="V21" s="156"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -4076,10 +4247,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="112" t="s">
+      <c r="AA21" s="155" t="s">
         <v>99</v>
       </c>
-      <c r="AB21" s="113"/>
+      <c r="AB21" s="156"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -4102,7 +4273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:35" ht="15.75" thickBot="1">
       <c r="B22" s="2">
         <v>17</v>
       </c>
@@ -4113,22 +4284,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="146"/>
-      <c r="F22" s="141"/>
-      <c r="G22" s="141"/>
-      <c r="H22" s="141"/>
-      <c r="I22" s="141"/>
-      <c r="J22" s="142"/>
+      <c r="E22" s="182"/>
+      <c r="F22" s="177"/>
+      <c r="G22" s="177"/>
+      <c r="H22" s="177"/>
+      <c r="I22" s="177"/>
+      <c r="J22" s="178"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="116" t="s">
+      <c r="N22" s="118" t="s">
         <v>64</v>
       </c>
-      <c r="O22" s="117"/>
-      <c r="P22" s="118"/>
+      <c r="O22" s="119"/>
+      <c r="P22" s="120"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -4138,10 +4309,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="112" t="s">
+      <c r="U22" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V22" s="113"/>
+      <c r="V22" s="156"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -4154,10 +4325,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="112" t="s">
+      <c r="AA22" s="155" t="s">
         <v>97</v>
       </c>
-      <c r="AB22" s="113"/>
+      <c r="AB22" s="156"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -4180,7 +4351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:35" ht="15.75" thickBot="1">
       <c r="B23" s="2">
         <v>18</v>
       </c>
@@ -4197,22 +4368,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="147" t="s">
+      <c r="G23" s="183" t="s">
         <v>78</v>
       </c>
-      <c r="H23" s="117"/>
-      <c r="I23" s="117"/>
-      <c r="J23" s="118"/>
+      <c r="H23" s="119"/>
+      <c r="I23" s="119"/>
+      <c r="J23" s="120"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="116" t="s">
+      <c r="N23" s="118" t="s">
         <v>83</v>
       </c>
-      <c r="O23" s="117"/>
-      <c r="P23" s="118"/>
+      <c r="O23" s="119"/>
+      <c r="P23" s="120"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -4222,10 +4393,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="112" t="s">
+      <c r="U23" s="155" t="s">
         <v>98</v>
       </c>
-      <c r="V23" s="113"/>
+      <c r="V23" s="156"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -4238,10 +4409,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="112" t="s">
+      <c r="AA23" s="155" t="s">
         <v>97</v>
       </c>
-      <c r="AB23" s="113"/>
+      <c r="AB23" s="156"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -4264,7 +4435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:35" ht="15.75" thickBot="1">
       <c r="B24" s="2">
         <v>19</v>
       </c>
@@ -4281,22 +4452,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="147" t="s">
+      <c r="G24" s="183" t="s">
         <v>78</v>
       </c>
-      <c r="H24" s="117"/>
-      <c r="I24" s="117"/>
-      <c r="J24" s="118"/>
+      <c r="H24" s="119"/>
+      <c r="I24" s="119"/>
+      <c r="J24" s="120"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="116" t="s">
+      <c r="N24" s="118" t="s">
         <v>82</v>
       </c>
-      <c r="O24" s="117"/>
-      <c r="P24" s="118"/>
+      <c r="O24" s="119"/>
+      <c r="P24" s="120"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -4306,10 +4477,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="112" t="s">
+      <c r="U24" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V24" s="113"/>
+      <c r="V24" s="156"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -4322,10 +4493,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="112" t="s">
+      <c r="AA24" s="155" t="s">
         <v>99</v>
       </c>
-      <c r="AB24" s="113"/>
+      <c r="AB24" s="156"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -4348,7 +4519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:35" ht="15.75" thickBot="1">
       <c r="B25" s="2">
         <v>20</v>
       </c>
@@ -4363,10 +4534,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="140"/>
-      <c r="H25" s="141"/>
-      <c r="I25" s="141"/>
-      <c r="J25" s="142"/>
+      <c r="G25" s="176"/>
+      <c r="H25" s="177"/>
+      <c r="I25" s="177"/>
+      <c r="J25" s="178"/>
       <c r="K25" s="49" t="s">
         <v>40</v>
       </c>
@@ -4374,11 +4545,11 @@
         <v>156</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="116" t="s">
+      <c r="N25" s="118" t="s">
         <v>42</v>
       </c>
-      <c r="O25" s="117"/>
-      <c r="P25" s="118"/>
+      <c r="O25" s="119"/>
+      <c r="P25" s="120"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -4388,10 +4559,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="112" t="s">
+      <c r="U25" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V25" s="113"/>
+      <c r="V25" s="156"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -4404,10 +4575,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="112" t="s">
+      <c r="AA25" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB25" s="113"/>
+      <c r="AB25" s="156"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -4430,7 +4601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:35" ht="15.75" thickBot="1">
       <c r="B26" s="2">
         <v>21</v>
       </c>
@@ -4445,10 +4616,10 @@
       <c r="F26" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="G26" s="140"/>
-      <c r="H26" s="141"/>
-      <c r="I26" s="141"/>
-      <c r="J26" s="142"/>
+      <c r="G26" s="176"/>
+      <c r="H26" s="177"/>
+      <c r="I26" s="177"/>
+      <c r="J26" s="178"/>
       <c r="K26" s="31" t="s">
         <v>41</v>
       </c>
@@ -4456,11 +4627,11 @@
         <v>156</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="116" t="s">
+      <c r="N26" s="118" t="s">
         <v>43</v>
       </c>
-      <c r="O26" s="117"/>
-      <c r="P26" s="118"/>
+      <c r="O26" s="119"/>
+      <c r="P26" s="120"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -4470,10 +4641,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="112" t="s">
+      <c r="U26" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V26" s="113"/>
+      <c r="V26" s="156"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -4486,10 +4657,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="112" t="s">
+      <c r="AA26" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB26" s="113"/>
+      <c r="AB26" s="156"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -4512,7 +4683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:35" ht="15.75" thickBot="1">
       <c r="B27" s="3">
         <v>22</v>
       </c>
@@ -4521,22 +4692,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="146"/>
-      <c r="F27" s="141"/>
-      <c r="G27" s="141"/>
-      <c r="H27" s="141"/>
-      <c r="I27" s="141"/>
-      <c r="J27" s="142"/>
+      <c r="E27" s="182"/>
+      <c r="F27" s="177"/>
+      <c r="G27" s="177"/>
+      <c r="H27" s="177"/>
+      <c r="I27" s="177"/>
+      <c r="J27" s="178"/>
       <c r="K27" s="25" t="s">
         <v>45</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="116" t="s">
+      <c r="N27" s="118" t="s">
         <v>47</v>
       </c>
-      <c r="O27" s="117"/>
-      <c r="P27" s="118"/>
+      <c r="O27" s="119"/>
+      <c r="P27" s="120"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -4546,10 +4717,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="112" t="s">
+      <c r="U27" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="V27" s="113"/>
+      <c r="V27" s="156"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -4562,10 +4733,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="112" t="s">
+      <c r="AA27" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="AB27" s="113"/>
+      <c r="AB27" s="156"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -4588,7 +4759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:35" ht="15.75" thickBot="1">
       <c r="B28" s="4">
         <v>23</v>
       </c>
@@ -4597,12 +4768,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="143"/>
-      <c r="F28" s="144"/>
-      <c r="G28" s="144"/>
-      <c r="H28" s="144"/>
-      <c r="I28" s="144"/>
-      <c r="J28" s="145"/>
+      <c r="E28" s="179"/>
+      <c r="F28" s="180"/>
+      <c r="G28" s="180"/>
+      <c r="H28" s="180"/>
+      <c r="I28" s="180"/>
+      <c r="J28" s="181"/>
       <c r="K28" s="52" t="s">
         <v>46</v>
       </c>
@@ -4610,11 +4781,11 @@
         <v>156</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="137" t="s">
+      <c r="N28" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="O28" s="138"/>
-      <c r="P28" s="139"/>
+      <c r="O28" s="116"/>
+      <c r="P28" s="117"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -4624,10 +4795,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="114" t="s">
+      <c r="U28" s="157" t="s">
         <v>74</v>
       </c>
-      <c r="V28" s="115"/>
+      <c r="V28" s="158"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -4640,10 +4811,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="114" t="s">
+      <c r="AA28" s="157" t="s">
         <v>74</v>
       </c>
-      <c r="AB28" s="115"/>
+      <c r="AB28" s="158"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -4666,8 +4837,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="2:35" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:35" ht="15.75" thickBot="1"/>
+    <row r="30" spans="2:35" ht="21.75" customHeight="1" thickBot="1">
       <c r="B30" s="66" t="s">
         <v>85</v>
       </c>
@@ -4720,20 +4891,20 @@
       <c r="S30" s="75" t="s">
         <v>157</v>
       </c>
-      <c r="T30" s="159" t="s">
+      <c r="T30" s="195" t="s">
         <v>158</v>
       </c>
-      <c r="U30" s="159"/>
-      <c r="V30" s="159"/>
-      <c r="W30" s="159"/>
-      <c r="X30" s="159"/>
-      <c r="Y30" s="159"/>
-      <c r="Z30" s="159"/>
-      <c r="AA30" s="159"/>
-      <c r="AB30" s="159"/>
-      <c r="AC30" s="127"/>
-    </row>
-    <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U30" s="195"/>
+      <c r="V30" s="195"/>
+      <c r="W30" s="195"/>
+      <c r="X30" s="195"/>
+      <c r="Y30" s="195"/>
+      <c r="Z30" s="195"/>
+      <c r="AA30" s="195"/>
+      <c r="AB30" s="195"/>
+      <c r="AC30" s="167"/>
+    </row>
+    <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B31" s="67" t="s">
         <v>73</v>
       </c>
@@ -4772,20 +4943,20 @@
       <c r="S31" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="T31" s="99" t="s">
+      <c r="T31" s="121" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="133"/>
-      <c r="V31" s="133"/>
-      <c r="W31" s="133"/>
-      <c r="X31" s="133"/>
-      <c r="Y31" s="133"/>
-      <c r="Z31" s="133"/>
-      <c r="AA31" s="133"/>
-      <c r="AB31" s="133"/>
-      <c r="AC31" s="100"/>
-    </row>
-    <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U31" s="122"/>
+      <c r="V31" s="122"/>
+      <c r="W31" s="122"/>
+      <c r="X31" s="122"/>
+      <c r="Y31" s="122"/>
+      <c r="Z31" s="122"/>
+      <c r="AA31" s="122"/>
+      <c r="AB31" s="122"/>
+      <c r="AC31" s="123"/>
+    </row>
+    <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B32" s="4" t="s">
         <v>76</v>
       </c>
@@ -4807,20 +4978,20 @@
       <c r="S32" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="T32" s="116" t="s">
+      <c r="T32" s="118" t="s">
         <v>164</v>
       </c>
-      <c r="U32" s="117"/>
-      <c r="V32" s="117"/>
-      <c r="W32" s="117"/>
-      <c r="X32" s="117"/>
-      <c r="Y32" s="117"/>
-      <c r="Z32" s="117"/>
-      <c r="AA32" s="117"/>
-      <c r="AB32" s="117"/>
-      <c r="AC32" s="118"/>
-    </row>
-    <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U32" s="119"/>
+      <c r="V32" s="119"/>
+      <c r="W32" s="119"/>
+      <c r="X32" s="119"/>
+      <c r="Y32" s="119"/>
+      <c r="Z32" s="119"/>
+      <c r="AA32" s="119"/>
+      <c r="AB32" s="119"/>
+      <c r="AC32" s="120"/>
+    </row>
+    <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
       <c r="H33" s="84" t="s">
         <v>198</v>
       </c>
@@ -4854,31 +5025,31 @@
       <c r="S33" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T33" s="116" t="s">
+      <c r="T33" s="118" t="s">
         <v>165</v>
       </c>
-      <c r="U33" s="117"/>
-      <c r="V33" s="117"/>
-      <c r="W33" s="117"/>
-      <c r="X33" s="117"/>
-      <c r="Y33" s="117"/>
-      <c r="Z33" s="117"/>
-      <c r="AA33" s="117"/>
-      <c r="AB33" s="117"/>
-      <c r="AC33" s="118"/>
-    </row>
-    <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="107" t="s">
+      <c r="U33" s="119"/>
+      <c r="V33" s="119"/>
+      <c r="W33" s="119"/>
+      <c r="X33" s="119"/>
+      <c r="Y33" s="119"/>
+      <c r="Z33" s="119"/>
+      <c r="AA33" s="119"/>
+      <c r="AB33" s="119"/>
+      <c r="AC33" s="120"/>
+    </row>
+    <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
+      <c r="B34" s="150" t="s">
         <v>109</v>
       </c>
-      <c r="C34" s="105" t="s">
+      <c r="C34" s="148" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="106"/>
-      <c r="E34" s="105" t="s">
+      <c r="D34" s="149"/>
+      <c r="E34" s="148" t="s">
         <v>116</v>
       </c>
-      <c r="F34" s="106"/>
+      <c r="F34" s="149"/>
       <c r="H34" s="77" t="s">
         <v>66</v>
       </c>
@@ -4904,21 +5075,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="116" t="s">
+      <c r="T34" s="118" t="s">
         <v>166</v>
       </c>
-      <c r="U34" s="117"/>
-      <c r="V34" s="117"/>
-      <c r="W34" s="117"/>
-      <c r="X34" s="117"/>
-      <c r="Y34" s="117"/>
-      <c r="Z34" s="117"/>
-      <c r="AA34" s="117"/>
-      <c r="AB34" s="117"/>
-      <c r="AC34" s="118"/>
-    </row>
-    <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="108"/>
+      <c r="U34" s="119"/>
+      <c r="V34" s="119"/>
+      <c r="W34" s="119"/>
+      <c r="X34" s="119"/>
+      <c r="Y34" s="119"/>
+      <c r="Z34" s="119"/>
+      <c r="AA34" s="119"/>
+      <c r="AB34" s="119"/>
+      <c r="AC34" s="120"/>
+    </row>
+    <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
+      <c r="B35" s="151"/>
       <c r="C35" s="64" t="s">
         <v>100</v>
       </c>
@@ -4937,20 +5108,20 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="116" t="s">
+      <c r="T35" s="118" t="s">
         <v>167</v>
       </c>
-      <c r="U35" s="117"/>
-      <c r="V35" s="117"/>
-      <c r="W35" s="117"/>
-      <c r="X35" s="117"/>
-      <c r="Y35" s="117"/>
-      <c r="Z35" s="117"/>
-      <c r="AA35" s="117"/>
-      <c r="AB35" s="117"/>
-      <c r="AC35" s="118"/>
-    </row>
-    <row r="36" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="U35" s="119"/>
+      <c r="V35" s="119"/>
+      <c r="W35" s="119"/>
+      <c r="X35" s="119"/>
+      <c r="Y35" s="119"/>
+      <c r="Z35" s="119"/>
+      <c r="AA35" s="119"/>
+      <c r="AB35" s="119"/>
+      <c r="AC35" s="120"/>
+    </row>
+    <row r="36" spans="2:29">
       <c r="B36" s="1">
         <v>0</v>
       </c>
@@ -4972,20 +5143,20 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="116" t="s">
+      <c r="T36" s="118" t="s">
         <v>168</v>
       </c>
-      <c r="U36" s="117"/>
-      <c r="V36" s="117"/>
-      <c r="W36" s="117"/>
-      <c r="X36" s="117"/>
-      <c r="Y36" s="117"/>
-      <c r="Z36" s="117"/>
-      <c r="AA36" s="117"/>
-      <c r="AB36" s="117"/>
-      <c r="AC36" s="118"/>
-    </row>
-    <row r="37" spans="2:29" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U36" s="119"/>
+      <c r="V36" s="119"/>
+      <c r="W36" s="119"/>
+      <c r="X36" s="119"/>
+      <c r="Y36" s="119"/>
+      <c r="Z36" s="119"/>
+      <c r="AA36" s="119"/>
+      <c r="AB36" s="119"/>
+      <c r="AC36" s="120"/>
+    </row>
+    <row r="37" spans="2:29" ht="36.75" customHeight="1">
       <c r="B37" s="2">
         <v>1</v>
       </c>
@@ -5008,20 +5179,20 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="116" t="s">
+      <c r="T37" s="118" t="s">
         <v>195</v>
       </c>
-      <c r="U37" s="117"/>
-      <c r="V37" s="117"/>
-      <c r="W37" s="117"/>
-      <c r="X37" s="117"/>
-      <c r="Y37" s="117"/>
-      <c r="Z37" s="117"/>
-      <c r="AA37" s="117"/>
-      <c r="AB37" s="117"/>
-      <c r="AC37" s="118"/>
-    </row>
-    <row r="38" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U37" s="119"/>
+      <c r="V37" s="119"/>
+      <c r="W37" s="119"/>
+      <c r="X37" s="119"/>
+      <c r="Y37" s="119"/>
+      <c r="Z37" s="119"/>
+      <c r="AA37" s="119"/>
+      <c r="AB37" s="119"/>
+      <c r="AC37" s="120"/>
+    </row>
+    <row r="38" spans="2:29" ht="15.75" thickBot="1">
       <c r="B38" s="2">
         <v>2</v>
       </c>
@@ -5040,23 +5211,23 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="164" t="s">
+      <c r="S38" s="196" t="s">
         <v>73</v>
       </c>
-      <c r="T38" s="166" t="s">
+      <c r="T38" s="198" t="s">
         <v>169</v>
       </c>
-      <c r="U38" s="167"/>
-      <c r="V38" s="167"/>
-      <c r="W38" s="167"/>
-      <c r="X38" s="167"/>
-      <c r="Y38" s="167"/>
-      <c r="Z38" s="167"/>
-      <c r="AA38" s="167"/>
-      <c r="AB38" s="167"/>
-      <c r="AC38" s="168"/>
-    </row>
-    <row r="39" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U38" s="199"/>
+      <c r="V38" s="199"/>
+      <c r="W38" s="199"/>
+      <c r="X38" s="199"/>
+      <c r="Y38" s="199"/>
+      <c r="Z38" s="199"/>
+      <c r="AA38" s="199"/>
+      <c r="AB38" s="199"/>
+      <c r="AC38" s="200"/>
+    </row>
+    <row r="39" spans="2:29" ht="15" customHeight="1">
       <c r="B39" s="2">
         <v>3</v>
       </c>
@@ -5072,28 +5243,28 @@
       <c r="F39" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G39" s="172" t="s">
+      <c r="G39" s="112" t="s">
         <v>182</v>
       </c>
-      <c r="H39" s="160"/>
-      <c r="I39" s="160"/>
-      <c r="J39" s="161"/>
+      <c r="H39" s="113"/>
+      <c r="I39" s="113"/>
+      <c r="J39" s="114"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="165"/>
-      <c r="T39" s="169"/>
-      <c r="U39" s="170"/>
-      <c r="V39" s="170"/>
-      <c r="W39" s="170"/>
-      <c r="X39" s="170"/>
-      <c r="Y39" s="170"/>
-      <c r="Z39" s="170"/>
-      <c r="AA39" s="170"/>
-      <c r="AB39" s="170"/>
-      <c r="AC39" s="171"/>
-    </row>
-    <row r="40" spans="2:29" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S39" s="197"/>
+      <c r="T39" s="201"/>
+      <c r="U39" s="202"/>
+      <c r="V39" s="202"/>
+      <c r="W39" s="202"/>
+      <c r="X39" s="202"/>
+      <c r="Y39" s="202"/>
+      <c r="Z39" s="202"/>
+      <c r="AA39" s="202"/>
+      <c r="AB39" s="202"/>
+      <c r="AC39" s="203"/>
+    </row>
+    <row r="40" spans="2:29" ht="37.5" customHeight="1">
       <c r="B40" s="2">
         <v>4</v>
       </c>
@@ -5109,30 +5280,30 @@
       <c r="F40" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G40" s="174"/>
-      <c r="H40" s="175"/>
-      <c r="I40" s="175"/>
-      <c r="J40" s="176"/>
+      <c r="G40" s="138"/>
+      <c r="H40" s="139"/>
+      <c r="I40" s="139"/>
+      <c r="J40" s="140"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="116" t="s">
+      <c r="T40" s="118" t="s">
         <v>170</v>
       </c>
-      <c r="U40" s="117"/>
-      <c r="V40" s="117"/>
-      <c r="W40" s="117"/>
-      <c r="X40" s="117"/>
-      <c r="Y40" s="117"/>
-      <c r="Z40" s="117"/>
-      <c r="AA40" s="117"/>
-      <c r="AB40" s="117"/>
-      <c r="AC40" s="118"/>
-    </row>
-    <row r="41" spans="2:29" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U40" s="119"/>
+      <c r="V40" s="119"/>
+      <c r="W40" s="119"/>
+      <c r="X40" s="119"/>
+      <c r="Y40" s="119"/>
+      <c r="Z40" s="119"/>
+      <c r="AA40" s="119"/>
+      <c r="AB40" s="119"/>
+      <c r="AC40" s="120"/>
+    </row>
+    <row r="41" spans="2:29" ht="30" customHeight="1">
       <c r="B41" s="2">
         <v>5</v>
       </c>
@@ -5148,30 +5319,30 @@
       <c r="F41" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="G41" s="174"/>
-      <c r="H41" s="175"/>
-      <c r="I41" s="175"/>
-      <c r="J41" s="176"/>
+      <c r="G41" s="138"/>
+      <c r="H41" s="139"/>
+      <c r="I41" s="139"/>
+      <c r="J41" s="140"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="116" t="s">
+      <c r="T41" s="118" t="s">
         <v>171</v>
       </c>
-      <c r="U41" s="117"/>
-      <c r="V41" s="117"/>
-      <c r="W41" s="117"/>
-      <c r="X41" s="117"/>
-      <c r="Y41" s="117"/>
-      <c r="Z41" s="117"/>
-      <c r="AA41" s="117"/>
-      <c r="AB41" s="117"/>
-      <c r="AC41" s="118"/>
-    </row>
-    <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U41" s="119"/>
+      <c r="V41" s="119"/>
+      <c r="W41" s="119"/>
+      <c r="X41" s="119"/>
+      <c r="Y41" s="119"/>
+      <c r="Z41" s="119"/>
+      <c r="AA41" s="119"/>
+      <c r="AB41" s="119"/>
+      <c r="AC41" s="120"/>
+    </row>
+    <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
       <c r="B42" s="2">
         <v>6</v>
       </c>
@@ -5187,30 +5358,30 @@
       <c r="F42" s="76" t="s">
         <v>176</v>
       </c>
-      <c r="G42" s="173"/>
-      <c r="H42" s="162"/>
-      <c r="I42" s="162"/>
-      <c r="J42" s="163"/>
+      <c r="G42" s="141"/>
+      <c r="H42" s="142"/>
+      <c r="I42" s="142"/>
+      <c r="J42" s="143"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="T42" s="116" t="s">
+      <c r="T42" s="118" t="s">
         <v>172</v>
       </c>
-      <c r="U42" s="117"/>
-      <c r="V42" s="117"/>
-      <c r="W42" s="117"/>
-      <c r="X42" s="117"/>
-      <c r="Y42" s="117"/>
-      <c r="Z42" s="117"/>
-      <c r="AA42" s="117"/>
-      <c r="AB42" s="117"/>
-      <c r="AC42" s="118"/>
-    </row>
-    <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U42" s="119"/>
+      <c r="V42" s="119"/>
+      <c r="W42" s="119"/>
+      <c r="X42" s="119"/>
+      <c r="Y42" s="119"/>
+      <c r="Z42" s="119"/>
+      <c r="AA42" s="119"/>
+      <c r="AB42" s="119"/>
+      <c r="AC42" s="120"/>
+    </row>
+    <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
       <c r="B43" s="2">
         <v>7</v>
       </c>
@@ -5226,32 +5397,32 @@
       <c r="F43" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="G43" s="92" t="s">
+      <c r="G43" s="131" t="s">
         <v>192</v>
       </c>
-      <c r="H43" s="93"/>
-      <c r="I43" s="93"/>
-      <c r="J43" s="94"/>
+      <c r="H43" s="132"/>
+      <c r="I43" s="132"/>
+      <c r="J43" s="133"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="T43" s="116" t="s">
+      <c r="T43" s="118" t="s">
         <v>173</v>
       </c>
-      <c r="U43" s="117"/>
-      <c r="V43" s="117"/>
-      <c r="W43" s="117"/>
-      <c r="X43" s="117"/>
-      <c r="Y43" s="117"/>
-      <c r="Z43" s="117"/>
-      <c r="AA43" s="117"/>
-      <c r="AB43" s="117"/>
-      <c r="AC43" s="118"/>
-    </row>
-    <row r="44" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U43" s="119"/>
+      <c r="V43" s="119"/>
+      <c r="W43" s="119"/>
+      <c r="X43" s="119"/>
+      <c r="Y43" s="119"/>
+      <c r="Z43" s="119"/>
+      <c r="AA43" s="119"/>
+      <c r="AB43" s="119"/>
+      <c r="AC43" s="120"/>
+    </row>
+    <row r="44" spans="2:29" ht="15.75" thickBot="1">
       <c r="B44" s="2">
         <v>8</v>
       </c>
@@ -5270,23 +5441,23 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="164" t="s">
+      <c r="S44" s="196" t="s">
         <v>76</v>
       </c>
-      <c r="T44" s="166" t="s">
+      <c r="T44" s="198" t="s">
         <v>174</v>
       </c>
-      <c r="U44" s="167"/>
-      <c r="V44" s="167"/>
-      <c r="W44" s="167"/>
-      <c r="X44" s="167"/>
-      <c r="Y44" s="167"/>
-      <c r="Z44" s="167"/>
-      <c r="AA44" s="167"/>
-      <c r="AB44" s="167"/>
-      <c r="AC44" s="168"/>
-    </row>
-    <row r="45" spans="2:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U44" s="199"/>
+      <c r="V44" s="199"/>
+      <c r="W44" s="199"/>
+      <c r="X44" s="199"/>
+      <c r="Y44" s="199"/>
+      <c r="Z44" s="199"/>
+      <c r="AA44" s="199"/>
+      <c r="AB44" s="199"/>
+      <c r="AC44" s="200"/>
+    </row>
+    <row r="45" spans="2:29" ht="30.75" customHeight="1">
       <c r="B45" s="2">
         <v>9</v>
       </c>
@@ -5302,28 +5473,28 @@
       <c r="F45" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="G45" s="172" t="s">
+      <c r="G45" s="112" t="s">
         <v>181</v>
       </c>
-      <c r="H45" s="160"/>
-      <c r="I45" s="160"/>
-      <c r="J45" s="161"/>
+      <c r="H45" s="113"/>
+      <c r="I45" s="113"/>
+      <c r="J45" s="114"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="165"/>
-      <c r="T45" s="169"/>
-      <c r="U45" s="170"/>
-      <c r="V45" s="170"/>
-      <c r="W45" s="170"/>
-      <c r="X45" s="170"/>
-      <c r="Y45" s="170"/>
-      <c r="Z45" s="170"/>
-      <c r="AA45" s="170"/>
-      <c r="AB45" s="170"/>
-      <c r="AC45" s="171"/>
-    </row>
-    <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S45" s="197"/>
+      <c r="T45" s="201"/>
+      <c r="U45" s="202"/>
+      <c r="V45" s="202"/>
+      <c r="W45" s="202"/>
+      <c r="X45" s="202"/>
+      <c r="Y45" s="202"/>
+      <c r="Z45" s="202"/>
+      <c r="AA45" s="202"/>
+      <c r="AB45" s="202"/>
+      <c r="AC45" s="203"/>
+    </row>
+    <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
       <c r="B46" s="2">
         <v>10</v>
       </c>
@@ -5339,30 +5510,30 @@
       <c r="F46" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G46" s="173"/>
-      <c r="H46" s="162"/>
-      <c r="I46" s="162"/>
-      <c r="J46" s="163"/>
+      <c r="G46" s="141"/>
+      <c r="H46" s="142"/>
+      <c r="I46" s="142"/>
+      <c r="J46" s="143"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="T46" s="137" t="s">
+      <c r="T46" s="115" t="s">
         <v>175</v>
       </c>
-      <c r="U46" s="138"/>
-      <c r="V46" s="138"/>
-      <c r="W46" s="138"/>
-      <c r="X46" s="138"/>
-      <c r="Y46" s="138"/>
-      <c r="Z46" s="138"/>
-      <c r="AA46" s="138"/>
-      <c r="AB46" s="138"/>
-      <c r="AC46" s="139"/>
-    </row>
-    <row r="47" spans="2:29" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U46" s="116"/>
+      <c r="V46" s="116"/>
+      <c r="W46" s="116"/>
+      <c r="X46" s="116"/>
+      <c r="Y46" s="116"/>
+      <c r="Z46" s="116"/>
+      <c r="AA46" s="116"/>
+      <c r="AB46" s="116"/>
+      <c r="AC46" s="117"/>
+    </row>
+    <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
       <c r="B47" s="2">
         <v>11</v>
       </c>
@@ -5378,14 +5549,14 @@
       <c r="F47" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="G47" s="93" t="s">
+      <c r="G47" s="132" t="s">
         <v>152</v>
       </c>
-      <c r="H47" s="93"/>
-      <c r="I47" s="93"/>
-      <c r="J47" s="94"/>
-    </row>
-    <row r="48" spans="2:29" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H47" s="132"/>
+      <c r="I47" s="132"/>
+      <c r="J47" s="133"/>
+    </row>
+    <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
       <c r="B48" s="2">
         <v>12</v>
       </c>
@@ -5401,8 +5572,32 @@
       <c r="F48" s="35" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="49" spans="2:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R48" s="89" t="s">
+        <v>208</v>
+      </c>
+      <c r="S48" s="104" t="s">
+        <v>209</v>
+      </c>
+      <c r="T48" s="104" t="s">
+        <v>210</v>
+      </c>
+      <c r="U48" s="104" t="s">
+        <v>211</v>
+      </c>
+      <c r="V48" s="103" t="s">
+        <v>212</v>
+      </c>
+      <c r="W48" s="112" t="s">
+        <v>213</v>
+      </c>
+      <c r="X48" s="113"/>
+      <c r="Y48" s="113"/>
+      <c r="Z48" s="114"/>
+      <c r="AA48" s="107" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="49" spans="2:26" ht="33.75" customHeight="1">
       <c r="B49" s="2">
         <v>13</v>
       </c>
@@ -5418,14 +5613,38 @@
       <c r="F49" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="G49" s="172" t="s">
+      <c r="G49" s="112" t="s">
         <v>155</v>
       </c>
-      <c r="H49" s="160"/>
-      <c r="I49" s="160"/>
-      <c r="J49" s="161"/>
-    </row>
-    <row r="50" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H49" s="113"/>
+      <c r="I49" s="113"/>
+      <c r="J49" s="114"/>
+      <c r="R49" s="90" t="s">
+        <v>232</v>
+      </c>
+      <c r="S49" s="96">
+        <v>0</v>
+      </c>
+      <c r="T49" s="97">
+        <v>0</v>
+      </c>
+      <c r="U49" s="97">
+        <v>0</v>
+      </c>
+      <c r="V49" s="98" t="str">
+        <f>DEC2HEX(HEX2DEC($X$49)+_xlfn.BITLSHIFT(S49,20)+_xlfn.BITLSHIFT(T49,15)+_xlfn.BITLSHIFT(U49,12))</f>
+        <v>E0000000</v>
+      </c>
+      <c r="W49" s="93" t="s">
+        <v>214</v>
+      </c>
+      <c r="X49" s="121" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y49" s="122"/>
+      <c r="Z49" s="123"/>
+    </row>
+    <row r="50" spans="2:26" ht="30" customHeight="1">
       <c r="B50" s="2">
         <v>14</v>
       </c>
@@ -5441,12 +5660,36 @@
       <c r="F50" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="G50" s="174"/>
-      <c r="H50" s="177"/>
-      <c r="I50" s="177"/>
-      <c r="J50" s="176"/>
-    </row>
-    <row r="51" spans="2:10" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G50" s="138"/>
+      <c r="H50" s="139"/>
+      <c r="I50" s="139"/>
+      <c r="J50" s="140"/>
+      <c r="R50" s="91" t="s">
+        <v>229</v>
+      </c>
+      <c r="S50" s="99">
+        <v>0</v>
+      </c>
+      <c r="T50" s="100">
+        <v>1</v>
+      </c>
+      <c r="U50" s="100">
+        <v>0</v>
+      </c>
+      <c r="V50" s="105" t="str">
+        <f t="shared" ref="V50:V60" si="1">DEC2HEX(HEX2DEC($X$49)+_xlfn.BITLSHIFT(S50,20)+_xlfn.BITLSHIFT(T50,15)+_xlfn.BITLSHIFT(U50,12))</f>
+        <v>E0008000</v>
+      </c>
+      <c r="W50" s="94" t="s">
+        <v>215</v>
+      </c>
+      <c r="X50" s="118">
+        <v>1</v>
+      </c>
+      <c r="Y50" s="119"/>
+      <c r="Z50" s="120"/>
+    </row>
+    <row r="51" spans="2:26" ht="32.25" customHeight="1" thickBot="1">
       <c r="B51" s="4">
         <v>15</v>
       </c>
@@ -5462,197 +5705,383 @@
       <c r="F51" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="G51" s="173"/>
-      <c r="H51" s="162"/>
-      <c r="I51" s="162"/>
-      <c r="J51" s="163"/>
-    </row>
-    <row r="52" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="109" t="s">
+      <c r="G51" s="141"/>
+      <c r="H51" s="142"/>
+      <c r="I51" s="142"/>
+      <c r="J51" s="143"/>
+      <c r="R51" s="91" t="s">
+        <v>230</v>
+      </c>
+      <c r="S51" s="99">
+        <v>0</v>
+      </c>
+      <c r="T51" s="100">
+        <v>2</v>
+      </c>
+      <c r="U51" s="100">
+        <v>0</v>
+      </c>
+      <c r="V51" s="105" t="str">
+        <f t="shared" si="1"/>
+        <v>E0010000</v>
+      </c>
+      <c r="W51" s="94" t="s">
+        <v>216</v>
+      </c>
+      <c r="X51" s="118">
+        <v>5</v>
+      </c>
+      <c r="Y51" s="119"/>
+      <c r="Z51" s="120"/>
+    </row>
+    <row r="52" spans="2:26" ht="30.75" customHeight="1" thickBot="1">
+      <c r="B52" s="152" t="s">
         <v>142</v>
       </c>
-      <c r="C52" s="110"/>
-      <c r="D52" s="110"/>
-      <c r="E52" s="110"/>
-      <c r="F52" s="111"/>
-    </row>
-    <row r="54" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B55" s="103" t="s">
+      <c r="C52" s="153"/>
+      <c r="D52" s="153"/>
+      <c r="E52" s="153"/>
+      <c r="F52" s="154"/>
+      <c r="R52" s="108" t="s">
+        <v>231</v>
+      </c>
+      <c r="S52" s="109">
+        <v>0</v>
+      </c>
+      <c r="T52" s="110">
+        <v>3</v>
+      </c>
+      <c r="U52" s="110">
+        <v>0</v>
+      </c>
+      <c r="V52" s="111" t="str">
+        <f t="shared" si="1"/>
+        <v>E0018000</v>
+      </c>
+      <c r="W52" s="95" t="s">
+        <v>217</v>
+      </c>
+      <c r="X52" s="115">
+        <v>0</v>
+      </c>
+      <c r="Y52" s="116"/>
+      <c r="Z52" s="117"/>
+    </row>
+    <row r="53" spans="2:26" ht="31.5" customHeight="1" thickBot="1">
+      <c r="R53" s="90" t="s">
+        <v>221</v>
+      </c>
+      <c r="S53" s="96">
+        <v>1</v>
+      </c>
+      <c r="T53" s="97">
+        <v>0</v>
+      </c>
+      <c r="U53" s="97">
+        <v>0</v>
+      </c>
+      <c r="V53" s="98" t="str">
+        <f t="shared" si="1"/>
+        <v>E0100000</v>
+      </c>
+      <c r="W53" s="88" t="s">
+        <v>219</v>
+      </c>
+      <c r="X53" s="124" t="str">
+        <f>DEC2HEX(HEX2DEC($X$49)+_xlfn.BITLSHIFT(X50,20)+_xlfn.BITLSHIFT(X51,15)+_xlfn.BITLSHIFT(X52,12)+4095)</f>
+        <v>E0128FFF</v>
+      </c>
+      <c r="Y53" s="125"/>
+      <c r="Z53" s="126"/>
+    </row>
+    <row r="54" spans="2:26" ht="24.75" customHeight="1">
+      <c r="B54" s="146" t="s">
         <v>183</v>
       </c>
-      <c r="C55" s="101" t="s">
+      <c r="C54" s="144" t="s">
         <v>185</v>
       </c>
-      <c r="D55" s="95" t="s">
+      <c r="D54" s="134" t="s">
         <v>184</v>
       </c>
-      <c r="E55" s="96"/>
-    </row>
-    <row r="56" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="104"/>
-      <c r="C56" s="102"/>
-      <c r="D56" s="97"/>
-      <c r="E56" s="98"/>
-    </row>
-    <row r="57" spans="2:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="81">
-        <v>0</v>
-      </c>
-      <c r="C57" s="23" t="s">
+      <c r="E54" s="135"/>
+      <c r="R54" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="S54" s="99">
+        <v>1</v>
+      </c>
+      <c r="T54" s="100">
+        <v>1</v>
+      </c>
+      <c r="U54" s="100">
+        <v>0</v>
+      </c>
+      <c r="V54" s="105" t="str">
+        <f t="shared" si="1"/>
+        <v>E0108000</v>
+      </c>
+    </row>
+    <row r="55" spans="2:26" ht="24" customHeight="1" thickBot="1">
+      <c r="B55" s="147"/>
+      <c r="C55" s="145"/>
+      <c r="D55" s="136"/>
+      <c r="E55" s="137"/>
+      <c r="R55" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="S55" s="99">
+        <v>1</v>
+      </c>
+      <c r="T55" s="100">
+        <v>2</v>
+      </c>
+      <c r="U55" s="100">
+        <v>0</v>
+      </c>
+      <c r="V55" s="105" t="str">
+        <f t="shared" si="1"/>
+        <v>E0110000</v>
+      </c>
+    </row>
+    <row r="56" spans="2:26" ht="41.25" customHeight="1">
+      <c r="B56" s="81">
+        <v>0</v>
+      </c>
+      <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D57" s="99" t="s">
+      <c r="D56" s="121" t="s">
         <v>207</v>
       </c>
-      <c r="E57" s="100"/>
-    </row>
-    <row r="58" spans="2:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E56" s="123"/>
+      <c r="R56" s="91" t="s">
+        <v>224</v>
+      </c>
+      <c r="S56" s="99">
+        <v>1</v>
+      </c>
+      <c r="T56" s="100">
+        <v>3</v>
+      </c>
+      <c r="U56" s="100">
+        <v>0</v>
+      </c>
+      <c r="V56" s="105" t="str">
+        <f t="shared" si="1"/>
+        <v>E0118000</v>
+      </c>
+    </row>
+    <row r="57" spans="2:26" ht="31.5" customHeight="1">
+      <c r="B57" s="82">
+        <v>1</v>
+      </c>
+      <c r="C57" s="86" t="s">
+        <v>203</v>
+      </c>
+      <c r="D57" s="127" t="s">
+        <v>206</v>
+      </c>
+      <c r="E57" s="128"/>
+      <c r="R57" s="91" t="s">
+        <v>225</v>
+      </c>
+      <c r="S57" s="99">
+        <v>1</v>
+      </c>
+      <c r="T57" s="100">
+        <v>4</v>
+      </c>
+      <c r="U57" s="100">
+        <v>0</v>
+      </c>
+      <c r="V57" s="105" t="str">
+        <f t="shared" si="1"/>
+        <v>E0120000</v>
+      </c>
+    </row>
+    <row r="58" spans="2:26" ht="30.75" customHeight="1">
       <c r="B58" s="82">
+        <v>2</v>
+      </c>
+      <c r="C58" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="D58" s="127" t="s">
+        <v>205</v>
+      </c>
+      <c r="E58" s="128"/>
+      <c r="R58" s="91" t="s">
+        <v>226</v>
+      </c>
+      <c r="S58" s="99">
         <v>1</v>
       </c>
-      <c r="C58" s="86" t="s">
-        <v>203</v>
-      </c>
-      <c r="D58" s="88" t="s">
-        <v>206</v>
-      </c>
-      <c r="E58" s="89"/>
-    </row>
-    <row r="59" spans="2:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="T58" s="100">
+        <v>5</v>
+      </c>
+      <c r="U58" s="100">
+        <v>0</v>
+      </c>
+      <c r="V58" s="105" t="str">
+        <f t="shared" si="1"/>
+        <v>E0128000</v>
+      </c>
+    </row>
+    <row r="59" spans="2:26" ht="33.75" customHeight="1">
       <c r="B59" s="82">
-        <v>2</v>
-      </c>
-      <c r="C59" s="38" t="s">
-        <v>204</v>
-      </c>
-      <c r="D59" s="88" t="s">
-        <v>205</v>
-      </c>
-      <c r="E59" s="89"/>
-    </row>
-    <row r="60" spans="2:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="C59" s="86" t="s">
+        <v>186</v>
+      </c>
+      <c r="D59" s="127" t="s">
+        <v>189</v>
+      </c>
+      <c r="E59" s="128"/>
+      <c r="R59" s="91" t="s">
+        <v>227</v>
+      </c>
+      <c r="S59" s="99">
+        <v>1</v>
+      </c>
+      <c r="T59" s="100">
+        <v>6</v>
+      </c>
+      <c r="U59" s="100">
+        <v>0</v>
+      </c>
+      <c r="V59" s="105" t="str">
+        <f t="shared" si="1"/>
+        <v>E0130000</v>
+      </c>
+    </row>
+    <row r="60" spans="2:26" ht="28.5" customHeight="1" thickBot="1">
       <c r="B60" s="82">
-        <v>3</v>
-      </c>
-      <c r="C60" s="86" t="s">
-        <v>186</v>
-      </c>
-      <c r="D60" s="88" t="s">
-        <v>189</v>
-      </c>
-      <c r="E60" s="89"/>
-    </row>
-    <row r="61" spans="2:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="C60" s="38" t="s">
+        <v>187</v>
+      </c>
+      <c r="D60" s="127" t="s">
+        <v>190</v>
+      </c>
+      <c r="E60" s="128"/>
+      <c r="R60" s="92" t="s">
+        <v>228</v>
+      </c>
+      <c r="S60" s="101">
+        <v>1</v>
+      </c>
+      <c r="T60" s="102">
+        <v>7</v>
+      </c>
+      <c r="U60" s="102">
+        <v>0</v>
+      </c>
+      <c r="V60" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v>E0138000</v>
+      </c>
+    </row>
+    <row r="61" spans="2:26" ht="40.5" customHeight="1">
       <c r="B61" s="82">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C61" s="38" t="s">
-        <v>187</v>
-      </c>
-      <c r="D61" s="88" t="s">
-        <v>190</v>
-      </c>
-      <c r="E61" s="89"/>
-    </row>
-    <row r="62" spans="2:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+      <c r="D61" s="127" t="s">
+        <v>191</v>
+      </c>
+      <c r="E61" s="128"/>
+    </row>
+    <row r="62" spans="2:26" ht="36" customHeight="1">
       <c r="B62" s="82">
-        <v>5</v>
-      </c>
-      <c r="C62" s="38" t="s">
-        <v>188</v>
-      </c>
-      <c r="D62" s="88" t="s">
-        <v>191</v>
-      </c>
-      <c r="E62" s="89"/>
-    </row>
-    <row r="63" spans="2:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="C62" s="86" t="s">
+        <v>196</v>
+      </c>
+      <c r="D62" s="127" t="s">
+        <v>197</v>
+      </c>
+      <c r="E62" s="128"/>
+    </row>
+    <row r="63" spans="2:26">
       <c r="B63" s="82">
-        <v>6</v>
-      </c>
-      <c r="C63" s="86" t="s">
-        <v>196</v>
-      </c>
-      <c r="D63" s="88" t="s">
-        <v>197</v>
-      </c>
-      <c r="E63" s="89"/>
-    </row>
-    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="C63" s="86"/>
+      <c r="D63" s="127"/>
+      <c r="E63" s="128"/>
+    </row>
+    <row r="64" spans="2:26">
       <c r="B64" s="82">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C64" s="86"/>
-      <c r="D64" s="88"/>
-      <c r="E64" s="89"/>
-    </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D64" s="127"/>
+      <c r="E64" s="128"/>
+    </row>
+    <row r="65" spans="2:5">
       <c r="B65" s="82">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C65" s="86"/>
-      <c r="D65" s="88"/>
-      <c r="E65" s="89"/>
-    </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D65" s="127"/>
+      <c r="E65" s="128"/>
+    </row>
+    <row r="66" spans="2:5">
       <c r="B66" s="82">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C66" s="86"/>
-      <c r="D66" s="88"/>
-      <c r="E66" s="89"/>
-    </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D66" s="127"/>
+      <c r="E66" s="128"/>
+    </row>
+    <row r="67" spans="2:5">
       <c r="B67" s="82">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C67" s="86"/>
-      <c r="D67" s="88"/>
-      <c r="E67" s="89"/>
-    </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D67" s="127"/>
+      <c r="E67" s="128"/>
+    </row>
+    <row r="68" spans="2:5">
       <c r="B68" s="82">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C68" s="86"/>
-      <c r="D68" s="88"/>
-      <c r="E68" s="89"/>
-    </row>
-    <row r="69" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D68" s="127"/>
+      <c r="E68" s="128"/>
+    </row>
+    <row r="69" spans="2:5">
       <c r="B69" s="82">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C69" s="86"/>
-      <c r="D69" s="88"/>
-      <c r="E69" s="89"/>
-    </row>
-    <row r="70" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D69" s="127"/>
+      <c r="E69" s="128"/>
+    </row>
+    <row r="70" spans="2:5">
       <c r="B70" s="82">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C70" s="86"/>
-      <c r="D70" s="88"/>
-      <c r="E70" s="89"/>
-    </row>
-    <row r="71" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B71" s="82">
-        <v>14</v>
-      </c>
-      <c r="C71" s="86"/>
-      <c r="D71" s="88"/>
-      <c r="E71" s="89"/>
-    </row>
-    <row r="72" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="83">
+      <c r="D70" s="127"/>
+      <c r="E70" s="128"/>
+    </row>
+    <row r="71" spans="2:5" ht="15.75" thickBot="1">
+      <c r="B71" s="83">
         <v>15</v>
       </c>
-      <c r="C72" s="87"/>
-      <c r="D72" s="90"/>
-      <c r="E72" s="91"/>
+      <c r="C71" s="87"/>
+      <c r="D71" s="129"/>
+      <c r="E71" s="130"/>
     </row>
   </sheetData>
-  <mergeCells count="158">
+  <mergeCells count="164">
     <mergeCell ref="T30:AC30"/>
     <mergeCell ref="T31:AC31"/>
     <mergeCell ref="T32:AC32"/>
@@ -5769,9 +6198,9 @@
     <mergeCell ref="AA9:AB9"/>
     <mergeCell ref="AA10:AB10"/>
     <mergeCell ref="AA11:AB11"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D57:E57"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="B34:B35"/>
@@ -5793,9 +6222,16 @@
     <mergeCell ref="N20:P20"/>
     <mergeCell ref="N21:P21"/>
     <mergeCell ref="N23:P23"/>
+    <mergeCell ref="W48:Z48"/>
+    <mergeCell ref="X52:Z52"/>
+    <mergeCell ref="X51:Z51"/>
+    <mergeCell ref="X50:Z50"/>
+    <mergeCell ref="X49:Z49"/>
+    <mergeCell ref="X53:Z53"/>
+    <mergeCell ref="D70:E70"/>
     <mergeCell ref="D71:E71"/>
-    <mergeCell ref="D72:E72"/>
     <mergeCell ref="G43:J43"/>
+    <mergeCell ref="D61:E61"/>
     <mergeCell ref="D62:E62"/>
     <mergeCell ref="D63:E63"/>
     <mergeCell ref="D64:E64"/>
@@ -5804,12 +6240,11 @@
     <mergeCell ref="D67:E67"/>
     <mergeCell ref="D68:E68"/>
     <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D55:E56"/>
+    <mergeCell ref="D54:E55"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D58:E58"/>
     <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="D56:E56"/>
     <mergeCell ref="G49:J51"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Re estructuración y creación de root complex.md
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{859BADAC-C186-402D-8BA3-9977ED71BF21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C581456E-547A-4067-B3CA-868092A674CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="278">
   <si>
     <t>OpCode</t>
   </si>
@@ -735,6 +735,243 @@
   </si>
   <si>
     <t>MMIO Controller</t>
+  </si>
+  <si>
+    <t>Base Class (Hex)</t>
+  </si>
+  <si>
+    <t>Familia Principal</t>
+  </si>
+  <si>
+    <t>Sub-Class (Hex)</t>
+  </si>
+  <si>
+    <t>Dispositivo Específico</t>
+  </si>
+  <si>
+    <t>Prog IF de ejemplo (Hex)</t>
+  </si>
+  <si>
+    <t>0x01</t>
+  </si>
+  <si>
+    <t>Controladores de Almacenamiento</t>
+  </si>
+  <si>
+    <t>IDE Controller</t>
+  </si>
+  <si>
+    <r>
+      <t>0x8A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Bus Master)</t>
+    </r>
+  </si>
+  <si>
+    <t>0x06</t>
+  </si>
+  <si>
+    <t>SATA Controller</t>
+  </si>
+  <si>
+    <r>
+      <t>0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (AHCI)</t>
+    </r>
+  </si>
+  <si>
+    <t>0x08</t>
+  </si>
+  <si>
+    <t>NVMe (Memoria No Volátil)</t>
+  </si>
+  <si>
+    <r>
+      <t>0x02</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (NVM Express)</t>
+    </r>
+  </si>
+  <si>
+    <t>0x02</t>
+  </si>
+  <si>
+    <t>Controladores de Red</t>
+  </si>
+  <si>
+    <t>0x00</t>
+  </si>
+  <si>
+    <t>Ethernet Controller</t>
+  </si>
+  <si>
+    <t>0x80</t>
+  </si>
+  <si>
+    <t>Network Controller (Otros/Wi-Fi)</t>
+  </si>
+  <si>
+    <t>0x03</t>
+  </si>
+  <si>
+    <t>Controladores de Pantalla</t>
+  </si>
+  <si>
+    <t>VGA Compatible (Tu GPU)</t>
+  </si>
+  <si>
+    <r>
+      <t>0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (VGA estándar)</t>
+    </r>
+  </si>
+  <si>
+    <t>Controlador 3D (No VGA)</t>
+  </si>
+  <si>
+    <t>0x04</t>
+  </si>
+  <si>
+    <t>Controladores Multimedia</t>
+  </si>
+  <si>
+    <t>Audio Device</t>
+  </si>
+  <si>
+    <t>Dispositivo de Audio HD (Intel HDA)</t>
+  </si>
+  <si>
+    <t>0x05</t>
+  </si>
+  <si>
+    <t>Controladores de Memoria</t>
+  </si>
+  <si>
+    <t>RAM</t>
+  </si>
+  <si>
+    <t>Puentes (Bridges)</t>
+  </si>
+  <si>
+    <t>Host Bridge (El Root Complex real)</t>
+  </si>
+  <si>
+    <t>PCI-to-PCI Bridge (Tu Switch)</t>
+  </si>
+  <si>
+    <r>
+      <t>0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Modo normal) o </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Sustractivo)</t>
+    </r>
+  </si>
+  <si>
+    <t>0x0C</t>
+  </si>
+  <si>
+    <t>Buses Serie</t>
+  </si>
+  <si>
+    <t>USB Controller</t>
+  </si>
+  <si>
+    <r>
+      <t>0x20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (EHCI/USB 2.0) o </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (xHCI/USB 3.0)</t>
+    </r>
+  </si>
+  <si>
+    <t>SMBus (Sensores de placa base)</t>
+  </si>
+  <si>
+    <t>Revision ID &amp; Class Code</t>
+  </si>
+  <si>
+    <t>Base-Sub-Prog IF-Revision</t>
+  </si>
+  <si>
+    <t>00-00-00-00</t>
   </si>
 </sst>
 </file>
@@ -840,7 +1077,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="73">
+  <borders count="74">
     <border>
       <left/>
       <right/>
@@ -1750,11 +1987,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="204">
+  <cellXfs count="234">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2089,6 +2341,69 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2098,40 +2413,157 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2140,6 +2572,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2149,12 +2605,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2167,202 +2617,94 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2645,7 +2987,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:AI71"/>
+  <dimension ref="B1:AI76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="15"/>
@@ -2660,73 +3002,79 @@
     <col min="15" max="15" width="18.7109375" style="15" customWidth="1"/>
     <col min="16" max="16" width="20" style="15" customWidth="1"/>
     <col min="17" max="17" width="9.140625" style="15" customWidth="1"/>
-    <col min="18" max="20" width="22.28515625" style="15" customWidth="1"/>
-    <col min="21" max="21" width="11.140625" style="15" customWidth="1"/>
-    <col min="22" max="22" width="16" style="15" customWidth="1"/>
+    <col min="18" max="19" width="22.28515625" style="15" customWidth="1"/>
+    <col min="20" max="20" width="16.42578125" style="15" customWidth="1"/>
+    <col min="21" max="21" width="16" style="15" customWidth="1"/>
+    <col min="22" max="22" width="14.28515625" style="15" customWidth="1"/>
     <col min="23" max="26" width="10.7109375" style="15" customWidth="1"/>
     <col min="27" max="28" width="6" style="15" customWidth="1"/>
-    <col min="29" max="35" width="10.7109375" style="15" customWidth="1"/>
+    <col min="29" max="29" width="15.140625" style="15" customWidth="1"/>
+    <col min="30" max="30" width="13.28515625" style="15" customWidth="1"/>
+    <col min="31" max="31" width="14.140625" style="15" customWidth="1"/>
+    <col min="32" max="32" width="14.7109375" style="15" customWidth="1"/>
+    <col min="33" max="33" width="17.28515625" style="15" customWidth="1"/>
+    <col min="34" max="35" width="10.7109375" style="15" customWidth="1"/>
     <col min="36" max="16384" width="9.140625" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B2" s="173" t="s">
+      <c r="B2" s="157" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="185" t="s">
+      <c r="C2" s="166" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="186"/>
-      <c r="E2" s="187" t="s">
+      <c r="D2" s="167"/>
+      <c r="E2" s="168" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="187"/>
-      <c r="G2" s="188" t="s">
+      <c r="F2" s="168"/>
+      <c r="G2" s="169" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="187"/>
-      <c r="I2" s="187" t="s">
+      <c r="H2" s="168"/>
+      <c r="I2" s="168" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="187"/>
-      <c r="K2" s="189" t="s">
+      <c r="J2" s="168"/>
+      <c r="K2" s="170" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="187"/>
-      <c r="M2" s="187"/>
-      <c r="N2" s="187"/>
-      <c r="O2" s="187"/>
-      <c r="P2" s="190"/>
-      <c r="R2" s="170" t="s">
+      <c r="L2" s="168"/>
+      <c r="M2" s="168"/>
+      <c r="N2" s="168"/>
+      <c r="O2" s="168"/>
+      <c r="P2" s="171"/>
+      <c r="R2" s="176" t="s">
         <v>66</v>
       </c>
-      <c r="S2" s="167" t="s">
+      <c r="S2" s="113" t="s">
         <v>67</v>
       </c>
-      <c r="T2" s="160" t="s">
+      <c r="T2" s="180" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="161"/>
-      <c r="V2" s="161"/>
-      <c r="W2" s="161"/>
-      <c r="X2" s="161"/>
-      <c r="Y2" s="161"/>
-      <c r="Z2" s="161"/>
-      <c r="AA2" s="161"/>
-      <c r="AB2" s="161" t="s">
+      <c r="U2" s="181"/>
+      <c r="V2" s="181"/>
+      <c r="W2" s="181"/>
+      <c r="X2" s="181"/>
+      <c r="Y2" s="181"/>
+      <c r="Z2" s="181"/>
+      <c r="AA2" s="181"/>
+      <c r="AB2" s="181" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="161"/>
-      <c r="AD2" s="161"/>
-      <c r="AE2" s="161"/>
-      <c r="AF2" s="161"/>
-      <c r="AG2" s="161"/>
-      <c r="AH2" s="161"/>
-      <c r="AI2" s="162"/>
+      <c r="AC2" s="181"/>
+      <c r="AD2" s="181"/>
+      <c r="AE2" s="181"/>
+      <c r="AF2" s="181"/>
+      <c r="AG2" s="181"/>
+      <c r="AH2" s="181"/>
+      <c r="AI2" s="182"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B3" s="174"/>
+      <c r="B3" s="158"/>
       <c r="C3" s="16" t="s">
         <v>80</v>
       </c>
@@ -2751,21 +3099,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="148"/>
-      <c r="L3" s="184"/>
-      <c r="M3" s="184"/>
-      <c r="N3" s="184"/>
-      <c r="O3" s="184"/>
-      <c r="P3" s="149"/>
-      <c r="R3" s="171"/>
-      <c r="S3" s="168"/>
+      <c r="K3" s="163"/>
+      <c r="L3" s="164"/>
+      <c r="M3" s="164"/>
+      <c r="N3" s="164"/>
+      <c r="O3" s="164"/>
+      <c r="P3" s="165"/>
+      <c r="R3" s="177"/>
+      <c r="S3" s="174"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="194" t="s">
+      <c r="U3" s="144" t="s">
         <v>84</v>
       </c>
-      <c r="V3" s="194"/>
+      <c r="V3" s="144"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -2778,10 +3126,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="159" t="s">
+      <c r="AA3" s="179" t="s">
         <v>75</v>
       </c>
-      <c r="AB3" s="159"/>
+      <c r="AB3" s="179"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -2805,21 +3153,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B4" s="175"/>
+      <c r="B4" s="159"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="163" t="s">
+      <c r="E4" s="145" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="153"/>
-      <c r="G4" s="153"/>
-      <c r="H4" s="153"/>
-      <c r="I4" s="153"/>
-      <c r="J4" s="154"/>
+      <c r="F4" s="172"/>
+      <c r="G4" s="172"/>
+      <c r="H4" s="172"/>
+      <c r="I4" s="172"/>
+      <c r="J4" s="173"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -2829,20 +3177,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="163" t="s">
+      <c r="N4" s="145" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="153"/>
-      <c r="P4" s="154"/>
-      <c r="R4" s="172"/>
-      <c r="S4" s="169"/>
+      <c r="O4" s="172"/>
+      <c r="P4" s="173"/>
+      <c r="R4" s="178"/>
+      <c r="S4" s="175"/>
       <c r="T4" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="U4" s="163" t="s">
+      <c r="U4" s="145" t="s">
         <v>76</v>
       </c>
-      <c r="V4" s="164"/>
+      <c r="V4" s="146"/>
       <c r="W4" s="7" t="s">
         <v>72</v>
       </c>
@@ -2855,10 +3203,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="163" t="s">
+      <c r="AA4" s="145" t="s">
         <v>73</v>
       </c>
-      <c r="AB4" s="164"/>
+      <c r="AB4" s="146"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -2890,22 +3238,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="191"/>
-      <c r="F5" s="192"/>
-      <c r="G5" s="192"/>
-      <c r="H5" s="192"/>
-      <c r="I5" s="192"/>
-      <c r="J5" s="193"/>
+      <c r="E5" s="149"/>
+      <c r="F5" s="150"/>
+      <c r="G5" s="150"/>
+      <c r="H5" s="150"/>
+      <c r="I5" s="150"/>
+      <c r="J5" s="151"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="121" t="s">
+      <c r="N5" s="114" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="122"/>
-      <c r="P5" s="123"/>
+      <c r="O5" s="115"/>
+      <c r="P5" s="116"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -2915,10 +3263,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="165" t="s">
+      <c r="U5" s="147" t="s">
         <v>74</v>
       </c>
-      <c r="V5" s="166"/>
+      <c r="V5" s="148"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -2931,10 +3279,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="165" t="s">
+      <c r="AA5" s="147" t="s">
         <v>74</v>
       </c>
-      <c r="AB5" s="166"/>
+      <c r="AB5" s="148"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -2966,12 +3314,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="182"/>
-      <c r="F6" s="177"/>
-      <c r="G6" s="177"/>
-      <c r="H6" s="177"/>
-      <c r="I6" s="177"/>
-      <c r="J6" s="178"/>
+      <c r="E6" s="156"/>
+      <c r="F6" s="153"/>
+      <c r="G6" s="153"/>
+      <c r="H6" s="153"/>
+      <c r="I6" s="153"/>
+      <c r="J6" s="154"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -2979,11 +3327,11 @@
         <v>156</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="118" t="s">
+      <c r="N6" s="117" t="s">
         <v>96</v>
       </c>
-      <c r="O6" s="119"/>
-      <c r="P6" s="120"/>
+      <c r="O6" s="118"/>
+      <c r="P6" s="119"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -2993,10 +3341,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="155" t="s">
+      <c r="U6" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V6" s="156"/>
+      <c r="V6" s="143"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -3009,10 +3357,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="155" t="s">
+      <c r="AA6" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB6" s="156"/>
+      <c r="AB6" s="143"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -3053,9 +3401,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="176"/>
-      <c r="I7" s="177"/>
-      <c r="J7" s="178"/>
+      <c r="H7" s="152"/>
+      <c r="I7" s="153"/>
+      <c r="J7" s="154"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -3063,11 +3411,11 @@
       <c r="M7" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N7" s="118" t="s">
+      <c r="N7" s="117" t="s">
         <v>53</v>
       </c>
-      <c r="O7" s="119"/>
-      <c r="P7" s="120"/>
+      <c r="O7" s="118"/>
+      <c r="P7" s="119"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -3077,10 +3425,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="155" t="s">
+      <c r="U7" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V7" s="156"/>
+      <c r="V7" s="143"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -3093,10 +3441,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="155" t="s">
+      <c r="AA7" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB7" s="156"/>
+      <c r="AB7" s="143"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -3137,9 +3485,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="176"/>
-      <c r="I8" s="177"/>
-      <c r="J8" s="178"/>
+      <c r="H8" s="152"/>
+      <c r="I8" s="153"/>
+      <c r="J8" s="154"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -3147,11 +3495,11 @@
       <c r="M8" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N8" s="118" t="s">
+      <c r="N8" s="117" t="s">
         <v>54</v>
       </c>
-      <c r="O8" s="119"/>
-      <c r="P8" s="120"/>
+      <c r="O8" s="118"/>
+      <c r="P8" s="119"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -3161,10 +3509,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="155" t="s">
+      <c r="U8" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V8" s="156"/>
+      <c r="V8" s="143"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -3177,10 +3525,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="155" t="s">
+      <c r="AA8" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB8" s="156"/>
+      <c r="AB8" s="143"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -3221,9 +3569,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="176"/>
-      <c r="I9" s="177"/>
-      <c r="J9" s="178"/>
+      <c r="H9" s="152"/>
+      <c r="I9" s="153"/>
+      <c r="J9" s="154"/>
       <c r="K9" s="37" t="s">
         <v>48</v>
       </c>
@@ -3231,11 +3579,11 @@
       <c r="M9" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N9" s="118" t="s">
+      <c r="N9" s="117" t="s">
         <v>55</v>
       </c>
-      <c r="O9" s="119"/>
-      <c r="P9" s="120"/>
+      <c r="O9" s="118"/>
+      <c r="P9" s="119"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -3245,10 +3593,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="155" t="s">
+      <c r="U9" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V9" s="156"/>
+      <c r="V9" s="143"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -3261,10 +3609,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="155" t="s">
+      <c r="AA9" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB9" s="156"/>
+      <c r="AB9" s="143"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -3305,9 +3653,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="176"/>
-      <c r="I10" s="177"/>
-      <c r="J10" s="178"/>
+      <c r="H10" s="152"/>
+      <c r="I10" s="153"/>
+      <c r="J10" s="154"/>
       <c r="K10" s="37" t="s">
         <v>49</v>
       </c>
@@ -3315,11 +3663,11 @@
       <c r="M10" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N10" s="118" t="s">
+      <c r="N10" s="117" t="s">
         <v>56</v>
       </c>
-      <c r="O10" s="119"/>
-      <c r="P10" s="120"/>
+      <c r="O10" s="118"/>
+      <c r="P10" s="119"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -3329,10 +3677,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="155" t="s">
+      <c r="U10" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V10" s="156"/>
+      <c r="V10" s="143"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -3345,10 +3693,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="155" t="s">
+      <c r="AA10" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB10" s="156"/>
+      <c r="AB10" s="143"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -3389,9 +3737,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="176"/>
-      <c r="I11" s="177"/>
-      <c r="J11" s="178"/>
+      <c r="H11" s="152"/>
+      <c r="I11" s="153"/>
+      <c r="J11" s="154"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -3399,11 +3747,11 @@
       <c r="M11" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N11" s="118" t="s">
+      <c r="N11" s="117" t="s">
         <v>57</v>
       </c>
-      <c r="O11" s="119"/>
-      <c r="P11" s="120"/>
+      <c r="O11" s="118"/>
+      <c r="P11" s="119"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -3413,10 +3761,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="155" t="s">
+      <c r="U11" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V11" s="156"/>
+      <c r="V11" s="143"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -3429,10 +3777,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="155" t="s">
+      <c r="AA11" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB11" s="156"/>
+      <c r="AB11" s="143"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -3473,9 +3821,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="176"/>
-      <c r="I12" s="177"/>
-      <c r="J12" s="178"/>
+      <c r="H12" s="152"/>
+      <c r="I12" s="153"/>
+      <c r="J12" s="154"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -3483,11 +3831,11 @@
       <c r="M12" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N12" s="118" t="s">
+      <c r="N12" s="117" t="s">
         <v>58</v>
       </c>
-      <c r="O12" s="119"/>
-      <c r="P12" s="120"/>
+      <c r="O12" s="118"/>
+      <c r="P12" s="119"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -3497,10 +3845,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="155" t="s">
+      <c r="U12" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V12" s="156"/>
+      <c r="V12" s="143"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -3513,10 +3861,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="155" t="s">
+      <c r="AA12" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB12" s="156"/>
+      <c r="AB12" s="143"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -3557,9 +3905,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="176"/>
-      <c r="I13" s="177"/>
-      <c r="J13" s="178"/>
+      <c r="H13" s="152"/>
+      <c r="I13" s="153"/>
+      <c r="J13" s="154"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -3567,11 +3915,11 @@
       <c r="M13" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N13" s="118" t="s">
+      <c r="N13" s="117" t="s">
         <v>59</v>
       </c>
-      <c r="O13" s="119"/>
-      <c r="P13" s="120"/>
+      <c r="O13" s="118"/>
+      <c r="P13" s="119"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -3581,10 +3929,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="155" t="s">
+      <c r="U13" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V13" s="156"/>
+      <c r="V13" s="143"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -3597,10 +3945,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="155" t="s">
+      <c r="AA13" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB13" s="156"/>
+      <c r="AB13" s="143"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -3641,9 +3989,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="176"/>
-      <c r="I14" s="177"/>
-      <c r="J14" s="178"/>
+      <c r="H14" s="152"/>
+      <c r="I14" s="153"/>
+      <c r="J14" s="154"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -3651,11 +3999,11 @@
       <c r="M14" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N14" s="118" t="s">
+      <c r="N14" s="117" t="s">
         <v>60</v>
       </c>
-      <c r="O14" s="119"/>
-      <c r="P14" s="120"/>
+      <c r="O14" s="118"/>
+      <c r="P14" s="119"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -3665,10 +4013,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="155" t="s">
+      <c r="U14" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V14" s="156"/>
+      <c r="V14" s="143"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -3681,10 +4029,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="155" t="s">
+      <c r="AA14" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB14" s="156"/>
+      <c r="AB14" s="143"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -3725,9 +4073,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="176"/>
-      <c r="I15" s="177"/>
-      <c r="J15" s="178"/>
+      <c r="H15" s="152"/>
+      <c r="I15" s="153"/>
+      <c r="J15" s="154"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -3735,11 +4083,11 @@
       <c r="M15" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N15" s="118" t="s">
+      <c r="N15" s="117" t="s">
         <v>61</v>
       </c>
-      <c r="O15" s="119"/>
-      <c r="P15" s="120"/>
+      <c r="O15" s="118"/>
+      <c r="P15" s="119"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -3749,10 +4097,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="155" t="s">
+      <c r="U15" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V15" s="156"/>
+      <c r="V15" s="143"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -3765,10 +4113,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="155" t="s">
+      <c r="AA15" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB15" s="156"/>
+      <c r="AB15" s="143"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -3803,21 +4151,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="176"/>
-      <c r="G16" s="177"/>
-      <c r="H16" s="177"/>
-      <c r="I16" s="177"/>
-      <c r="J16" s="178"/>
+      <c r="F16" s="152"/>
+      <c r="G16" s="153"/>
+      <c r="H16" s="153"/>
+      <c r="I16" s="153"/>
+      <c r="J16" s="154"/>
       <c r="K16" s="40" t="s">
         <v>50</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="118" t="s">
+      <c r="N16" s="117" t="s">
         <v>51</v>
       </c>
-      <c r="O16" s="119"/>
-      <c r="P16" s="120"/>
+      <c r="O16" s="118"/>
+      <c r="P16" s="119"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -3827,10 +4175,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="155" t="s">
+      <c r="U16" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V16" s="156"/>
+      <c r="V16" s="143"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -3843,10 +4191,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="155" t="s">
+      <c r="AA16" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB16" s="156"/>
+      <c r="AB16" s="143"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -3882,22 +4230,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="183" t="s">
+      <c r="G17" s="155" t="s">
         <v>77</v>
       </c>
-      <c r="H17" s="119"/>
-      <c r="I17" s="119"/>
-      <c r="J17" s="120"/>
+      <c r="H17" s="118"/>
+      <c r="I17" s="118"/>
+      <c r="J17" s="119"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="118" t="s">
+      <c r="N17" s="117" t="s">
         <v>65</v>
       </c>
-      <c r="O17" s="119"/>
-      <c r="P17" s="120"/>
+      <c r="O17" s="118"/>
+      <c r="P17" s="119"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -3907,10 +4255,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="155" t="s">
+      <c r="U17" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V17" s="156"/>
+      <c r="V17" s="143"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -3923,10 +4271,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="155" t="s">
+      <c r="AA17" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB17" s="156"/>
+      <c r="AB17" s="143"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -3962,12 +4310,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="183" t="s">
+      <c r="G18" s="155" t="s">
         <v>77</v>
       </c>
-      <c r="H18" s="119"/>
-      <c r="I18" s="119"/>
-      <c r="J18" s="120"/>
+      <c r="H18" s="118"/>
+      <c r="I18" s="118"/>
+      <c r="J18" s="119"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -3975,11 +4323,11 @@
       <c r="M18" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="N18" s="118" t="s">
+      <c r="N18" s="117" t="s">
         <v>62</v>
       </c>
-      <c r="O18" s="119"/>
-      <c r="P18" s="120"/>
+      <c r="O18" s="118"/>
+      <c r="P18" s="119"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -3989,10 +4337,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="155" t="s">
+      <c r="U18" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V18" s="156"/>
+      <c r="V18" s="143"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -4005,10 +4353,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="155" t="s">
+      <c r="AA18" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB18" s="156"/>
+      <c r="AB18" s="143"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -4046,20 +4394,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="176"/>
-      <c r="H19" s="177"/>
-      <c r="I19" s="177"/>
-      <c r="J19" s="178"/>
+      <c r="G19" s="152"/>
+      <c r="H19" s="153"/>
+      <c r="I19" s="153"/>
+      <c r="J19" s="154"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="118" t="s">
+      <c r="N19" s="117" t="s">
         <v>94</v>
       </c>
-      <c r="O19" s="119"/>
-      <c r="P19" s="120"/>
+      <c r="O19" s="118"/>
+      <c r="P19" s="119"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -4069,10 +4417,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="155" t="s">
+      <c r="U19" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V19" s="156"/>
+      <c r="V19" s="143"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -4085,10 +4433,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="155" t="s">
+      <c r="AA19" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB19" s="156"/>
+      <c r="AB19" s="143"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -4128,20 +4476,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="176"/>
-      <c r="H20" s="177"/>
-      <c r="I20" s="177"/>
-      <c r="J20" s="178"/>
+      <c r="G20" s="152"/>
+      <c r="H20" s="153"/>
+      <c r="I20" s="153"/>
+      <c r="J20" s="154"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="118" t="s">
+      <c r="N20" s="117" t="s">
         <v>95</v>
       </c>
-      <c r="O20" s="119"/>
-      <c r="P20" s="120"/>
+      <c r="O20" s="118"/>
+      <c r="P20" s="119"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -4151,10 +4499,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="155" t="s">
+      <c r="U20" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V20" s="156"/>
+      <c r="V20" s="143"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -4167,10 +4515,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="155" t="s">
+      <c r="AA20" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB20" s="156"/>
+      <c r="AB20" s="143"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -4208,20 +4556,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="176"/>
-      <c r="H21" s="177"/>
-      <c r="I21" s="177"/>
-      <c r="J21" s="178"/>
+      <c r="G21" s="152"/>
+      <c r="H21" s="153"/>
+      <c r="I21" s="153"/>
+      <c r="J21" s="154"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="118" t="s">
+      <c r="N21" s="117" t="s">
         <v>63</v>
       </c>
-      <c r="O21" s="119"/>
-      <c r="P21" s="120"/>
+      <c r="O21" s="118"/>
+      <c r="P21" s="119"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -4231,10 +4579,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="155" t="s">
+      <c r="U21" s="142" t="s">
         <v>97</v>
       </c>
-      <c r="V21" s="156"/>
+      <c r="V21" s="143"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -4247,10 +4595,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="155" t="s">
+      <c r="AA21" s="142" t="s">
         <v>99</v>
       </c>
-      <c r="AB21" s="156"/>
+      <c r="AB21" s="143"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -4284,22 +4632,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="182"/>
-      <c r="F22" s="177"/>
-      <c r="G22" s="177"/>
-      <c r="H22" s="177"/>
-      <c r="I22" s="177"/>
-      <c r="J22" s="178"/>
+      <c r="E22" s="156"/>
+      <c r="F22" s="153"/>
+      <c r="G22" s="153"/>
+      <c r="H22" s="153"/>
+      <c r="I22" s="153"/>
+      <c r="J22" s="154"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="118" t="s">
+      <c r="N22" s="117" t="s">
         <v>64</v>
       </c>
-      <c r="O22" s="119"/>
-      <c r="P22" s="120"/>
+      <c r="O22" s="118"/>
+      <c r="P22" s="119"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -4309,10 +4657,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="155" t="s">
+      <c r="U22" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V22" s="156"/>
+      <c r="V22" s="143"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -4325,10 +4673,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="155" t="s">
+      <c r="AA22" s="142" t="s">
         <v>97</v>
       </c>
-      <c r="AB22" s="156"/>
+      <c r="AB22" s="143"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -4368,22 +4716,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="183" t="s">
+      <c r="G23" s="155" t="s">
         <v>78</v>
       </c>
-      <c r="H23" s="119"/>
-      <c r="I23" s="119"/>
-      <c r="J23" s="120"/>
+      <c r="H23" s="118"/>
+      <c r="I23" s="118"/>
+      <c r="J23" s="119"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="118" t="s">
+      <c r="N23" s="117" t="s">
         <v>83</v>
       </c>
-      <c r="O23" s="119"/>
-      <c r="P23" s="120"/>
+      <c r="O23" s="118"/>
+      <c r="P23" s="119"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -4393,10 +4741,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="155" t="s">
+      <c r="U23" s="142" t="s">
         <v>98</v>
       </c>
-      <c r="V23" s="156"/>
+      <c r="V23" s="143"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -4409,10 +4757,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="155" t="s">
+      <c r="AA23" s="142" t="s">
         <v>97</v>
       </c>
-      <c r="AB23" s="156"/>
+      <c r="AB23" s="143"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -4452,22 +4800,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="183" t="s">
+      <c r="G24" s="155" t="s">
         <v>78</v>
       </c>
-      <c r="H24" s="119"/>
-      <c r="I24" s="119"/>
-      <c r="J24" s="120"/>
+      <c r="H24" s="118"/>
+      <c r="I24" s="118"/>
+      <c r="J24" s="119"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="118" t="s">
+      <c r="N24" s="117" t="s">
         <v>82</v>
       </c>
-      <c r="O24" s="119"/>
-      <c r="P24" s="120"/>
+      <c r="O24" s="118"/>
+      <c r="P24" s="119"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -4477,10 +4825,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="155" t="s">
+      <c r="U24" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V24" s="156"/>
+      <c r="V24" s="143"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -4493,10 +4841,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="155" t="s">
+      <c r="AA24" s="142" t="s">
         <v>99</v>
       </c>
-      <c r="AB24" s="156"/>
+      <c r="AB24" s="143"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -4534,10 +4882,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="176"/>
-      <c r="H25" s="177"/>
-      <c r="I25" s="177"/>
-      <c r="J25" s="178"/>
+      <c r="G25" s="152"/>
+      <c r="H25" s="153"/>
+      <c r="I25" s="153"/>
+      <c r="J25" s="154"/>
       <c r="K25" s="49" t="s">
         <v>40</v>
       </c>
@@ -4545,11 +4893,11 @@
         <v>156</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="118" t="s">
+      <c r="N25" s="117" t="s">
         <v>42</v>
       </c>
-      <c r="O25" s="119"/>
-      <c r="P25" s="120"/>
+      <c r="O25" s="118"/>
+      <c r="P25" s="119"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -4559,10 +4907,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="155" t="s">
+      <c r="U25" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V25" s="156"/>
+      <c r="V25" s="143"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -4575,10 +4923,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="155" t="s">
+      <c r="AA25" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB25" s="156"/>
+      <c r="AB25" s="143"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -4616,10 +4964,10 @@
       <c r="F26" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="G26" s="176"/>
-      <c r="H26" s="177"/>
-      <c r="I26" s="177"/>
-      <c r="J26" s="178"/>
+      <c r="G26" s="152"/>
+      <c r="H26" s="153"/>
+      <c r="I26" s="153"/>
+      <c r="J26" s="154"/>
       <c r="K26" s="31" t="s">
         <v>41</v>
       </c>
@@ -4627,11 +4975,11 @@
         <v>156</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="118" t="s">
+      <c r="N26" s="117" t="s">
         <v>43</v>
       </c>
-      <c r="O26" s="119"/>
-      <c r="P26" s="120"/>
+      <c r="O26" s="118"/>
+      <c r="P26" s="119"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -4641,10 +4989,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="155" t="s">
+      <c r="U26" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V26" s="156"/>
+      <c r="V26" s="143"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -4657,10 +5005,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="155" t="s">
+      <c r="AA26" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB26" s="156"/>
+      <c r="AB26" s="143"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -4692,22 +5040,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="182"/>
-      <c r="F27" s="177"/>
-      <c r="G27" s="177"/>
-      <c r="H27" s="177"/>
-      <c r="I27" s="177"/>
-      <c r="J27" s="178"/>
+      <c r="E27" s="156"/>
+      <c r="F27" s="153"/>
+      <c r="G27" s="153"/>
+      <c r="H27" s="153"/>
+      <c r="I27" s="153"/>
+      <c r="J27" s="154"/>
       <c r="K27" s="25" t="s">
         <v>45</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="118" t="s">
+      <c r="N27" s="117" t="s">
         <v>47</v>
       </c>
-      <c r="O27" s="119"/>
-      <c r="P27" s="120"/>
+      <c r="O27" s="118"/>
+      <c r="P27" s="119"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -4717,10 +5065,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="155" t="s">
+      <c r="U27" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="V27" s="156"/>
+      <c r="V27" s="143"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -4733,10 +5081,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="155" t="s">
+      <c r="AA27" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="AB27" s="156"/>
+      <c r="AB27" s="143"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -4768,12 +5116,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="179"/>
-      <c r="F28" s="180"/>
-      <c r="G28" s="180"/>
-      <c r="H28" s="180"/>
-      <c r="I28" s="180"/>
-      <c r="J28" s="181"/>
+      <c r="E28" s="160"/>
+      <c r="F28" s="161"/>
+      <c r="G28" s="161"/>
+      <c r="H28" s="161"/>
+      <c r="I28" s="161"/>
+      <c r="J28" s="162"/>
       <c r="K28" s="52" t="s">
         <v>46</v>
       </c>
@@ -4781,11 +5129,11 @@
         <v>156</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="115" t="s">
+      <c r="N28" s="130" t="s">
         <v>93</v>
       </c>
-      <c r="O28" s="116"/>
-      <c r="P28" s="117"/>
+      <c r="O28" s="131"/>
+      <c r="P28" s="132"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -4795,10 +5143,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="157" t="s">
+      <c r="U28" s="192" t="s">
         <v>74</v>
       </c>
-      <c r="V28" s="158"/>
+      <c r="V28" s="193"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -4811,10 +5159,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="157" t="s">
+      <c r="AA28" s="192" t="s">
         <v>74</v>
       </c>
-      <c r="AB28" s="158"/>
+      <c r="AB28" s="193"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -4891,18 +5239,18 @@
       <c r="S30" s="75" t="s">
         <v>157</v>
       </c>
-      <c r="T30" s="195" t="s">
+      <c r="T30" s="112" t="s">
         <v>158</v>
       </c>
-      <c r="U30" s="195"/>
-      <c r="V30" s="195"/>
-      <c r="W30" s="195"/>
-      <c r="X30" s="195"/>
-      <c r="Y30" s="195"/>
-      <c r="Z30" s="195"/>
-      <c r="AA30" s="195"/>
-      <c r="AB30" s="195"/>
-      <c r="AC30" s="167"/>
+      <c r="U30" s="112"/>
+      <c r="V30" s="112"/>
+      <c r="W30" s="112"/>
+      <c r="X30" s="112"/>
+      <c r="Y30" s="112"/>
+      <c r="Z30" s="112"/>
+      <c r="AA30" s="112"/>
+      <c r="AB30" s="112"/>
+      <c r="AC30" s="113"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B31" s="67" t="s">
@@ -4943,18 +5291,18 @@
       <c r="S31" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="T31" s="121" t="s">
+      <c r="T31" s="114" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="122"/>
-      <c r="V31" s="122"/>
-      <c r="W31" s="122"/>
-      <c r="X31" s="122"/>
-      <c r="Y31" s="122"/>
-      <c r="Z31" s="122"/>
-      <c r="AA31" s="122"/>
-      <c r="AB31" s="122"/>
-      <c r="AC31" s="123"/>
+      <c r="U31" s="115"/>
+      <c r="V31" s="115"/>
+      <c r="W31" s="115"/>
+      <c r="X31" s="115"/>
+      <c r="Y31" s="115"/>
+      <c r="Z31" s="115"/>
+      <c r="AA31" s="115"/>
+      <c r="AB31" s="115"/>
+      <c r="AC31" s="116"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B32" s="4" t="s">
@@ -4978,18 +5326,18 @@
       <c r="S32" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="T32" s="118" t="s">
+      <c r="T32" s="117" t="s">
         <v>164</v>
       </c>
-      <c r="U32" s="119"/>
-      <c r="V32" s="119"/>
-      <c r="W32" s="119"/>
-      <c r="X32" s="119"/>
-      <c r="Y32" s="119"/>
-      <c r="Z32" s="119"/>
-      <c r="AA32" s="119"/>
-      <c r="AB32" s="119"/>
-      <c r="AC32" s="120"/>
+      <c r="U32" s="118"/>
+      <c r="V32" s="118"/>
+      <c r="W32" s="118"/>
+      <c r="X32" s="118"/>
+      <c r="Y32" s="118"/>
+      <c r="Z32" s="118"/>
+      <c r="AA32" s="118"/>
+      <c r="AB32" s="118"/>
+      <c r="AC32" s="119"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
       <c r="H33" s="84" t="s">
@@ -5025,31 +5373,31 @@
       <c r="S33" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T33" s="118" t="s">
+      <c r="T33" s="117" t="s">
         <v>165</v>
       </c>
-      <c r="U33" s="119"/>
-      <c r="V33" s="119"/>
-      <c r="W33" s="119"/>
-      <c r="X33" s="119"/>
-      <c r="Y33" s="119"/>
-      <c r="Z33" s="119"/>
-      <c r="AA33" s="119"/>
-      <c r="AB33" s="119"/>
-      <c r="AC33" s="120"/>
+      <c r="U33" s="118"/>
+      <c r="V33" s="118"/>
+      <c r="W33" s="118"/>
+      <c r="X33" s="118"/>
+      <c r="Y33" s="118"/>
+      <c r="Z33" s="118"/>
+      <c r="AA33" s="118"/>
+      <c r="AB33" s="118"/>
+      <c r="AC33" s="119"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B34" s="150" t="s">
+      <c r="B34" s="189" t="s">
         <v>109</v>
       </c>
-      <c r="C34" s="148" t="s">
+      <c r="C34" s="163" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="149"/>
-      <c r="E34" s="148" t="s">
+      <c r="D34" s="165"/>
+      <c r="E34" s="163" t="s">
         <v>116</v>
       </c>
-      <c r="F34" s="149"/>
+      <c r="F34" s="165"/>
       <c r="H34" s="77" t="s">
         <v>66</v>
       </c>
@@ -5075,21 +5423,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="118" t="s">
+      <c r="T34" s="117" t="s">
         <v>166</v>
       </c>
-      <c r="U34" s="119"/>
-      <c r="V34" s="119"/>
-      <c r="W34" s="119"/>
-      <c r="X34" s="119"/>
-      <c r="Y34" s="119"/>
-      <c r="Z34" s="119"/>
-      <c r="AA34" s="119"/>
-      <c r="AB34" s="119"/>
-      <c r="AC34" s="120"/>
+      <c r="U34" s="118"/>
+      <c r="V34" s="118"/>
+      <c r="W34" s="118"/>
+      <c r="X34" s="118"/>
+      <c r="Y34" s="118"/>
+      <c r="Z34" s="118"/>
+      <c r="AA34" s="118"/>
+      <c r="AB34" s="118"/>
+      <c r="AC34" s="119"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B35" s="151"/>
+      <c r="B35" s="190"/>
       <c r="C35" s="64" t="s">
         <v>100</v>
       </c>
@@ -5108,18 +5456,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="118" t="s">
+      <c r="T35" s="117" t="s">
         <v>167</v>
       </c>
-      <c r="U35" s="119"/>
-      <c r="V35" s="119"/>
-      <c r="W35" s="119"/>
-      <c r="X35" s="119"/>
-      <c r="Y35" s="119"/>
-      <c r="Z35" s="119"/>
-      <c r="AA35" s="119"/>
-      <c r="AB35" s="119"/>
-      <c r="AC35" s="120"/>
+      <c r="U35" s="118"/>
+      <c r="V35" s="118"/>
+      <c r="W35" s="118"/>
+      <c r="X35" s="118"/>
+      <c r="Y35" s="118"/>
+      <c r="Z35" s="118"/>
+      <c r="AA35" s="118"/>
+      <c r="AB35" s="118"/>
+      <c r="AC35" s="119"/>
     </row>
     <row r="36" spans="2:29">
       <c r="B36" s="1">
@@ -5143,18 +5491,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="118" t="s">
+      <c r="T36" s="117" t="s">
         <v>168</v>
       </c>
-      <c r="U36" s="119"/>
-      <c r="V36" s="119"/>
-      <c r="W36" s="119"/>
-      <c r="X36" s="119"/>
-      <c r="Y36" s="119"/>
-      <c r="Z36" s="119"/>
-      <c r="AA36" s="119"/>
-      <c r="AB36" s="119"/>
-      <c r="AC36" s="120"/>
+      <c r="U36" s="118"/>
+      <c r="V36" s="118"/>
+      <c r="W36" s="118"/>
+      <c r="X36" s="118"/>
+      <c r="Y36" s="118"/>
+      <c r="Z36" s="118"/>
+      <c r="AA36" s="118"/>
+      <c r="AB36" s="118"/>
+      <c r="AC36" s="119"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1">
       <c r="B37" s="2">
@@ -5179,18 +5527,18 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="118" t="s">
+      <c r="T37" s="117" t="s">
         <v>195</v>
       </c>
-      <c r="U37" s="119"/>
-      <c r="V37" s="119"/>
-      <c r="W37" s="119"/>
-      <c r="X37" s="119"/>
-      <c r="Y37" s="119"/>
-      <c r="Z37" s="119"/>
-      <c r="AA37" s="119"/>
-      <c r="AB37" s="119"/>
-      <c r="AC37" s="120"/>
+      <c r="U37" s="118"/>
+      <c r="V37" s="118"/>
+      <c r="W37" s="118"/>
+      <c r="X37" s="118"/>
+      <c r="Y37" s="118"/>
+      <c r="Z37" s="118"/>
+      <c r="AA37" s="118"/>
+      <c r="AB37" s="118"/>
+      <c r="AC37" s="119"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1">
       <c r="B38" s="2">
@@ -5211,21 +5559,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="196" t="s">
+      <c r="S38" s="122" t="s">
         <v>73</v>
       </c>
-      <c r="T38" s="198" t="s">
+      <c r="T38" s="124" t="s">
         <v>169</v>
       </c>
-      <c r="U38" s="199"/>
-      <c r="V38" s="199"/>
-      <c r="W38" s="199"/>
-      <c r="X38" s="199"/>
-      <c r="Y38" s="199"/>
-      <c r="Z38" s="199"/>
-      <c r="AA38" s="199"/>
-      <c r="AB38" s="199"/>
-      <c r="AC38" s="200"/>
+      <c r="U38" s="125"/>
+      <c r="V38" s="125"/>
+      <c r="W38" s="125"/>
+      <c r="X38" s="125"/>
+      <c r="Y38" s="125"/>
+      <c r="Z38" s="125"/>
+      <c r="AA38" s="125"/>
+      <c r="AB38" s="125"/>
+      <c r="AC38" s="126"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1">
       <c r="B39" s="2">
@@ -5243,26 +5591,26 @@
       <c r="F39" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G39" s="112" t="s">
+      <c r="G39" s="133" t="s">
         <v>182</v>
       </c>
-      <c r="H39" s="113"/>
-      <c r="I39" s="113"/>
-      <c r="J39" s="114"/>
+      <c r="H39" s="134"/>
+      <c r="I39" s="134"/>
+      <c r="J39" s="135"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="197"/>
-      <c r="T39" s="201"/>
-      <c r="U39" s="202"/>
-      <c r="V39" s="202"/>
-      <c r="W39" s="202"/>
-      <c r="X39" s="202"/>
-      <c r="Y39" s="202"/>
-      <c r="Z39" s="202"/>
-      <c r="AA39" s="202"/>
-      <c r="AB39" s="202"/>
-      <c r="AC39" s="203"/>
+      <c r="S39" s="123"/>
+      <c r="T39" s="127"/>
+      <c r="U39" s="128"/>
+      <c r="V39" s="128"/>
+      <c r="W39" s="128"/>
+      <c r="X39" s="128"/>
+      <c r="Y39" s="128"/>
+      <c r="Z39" s="128"/>
+      <c r="AA39" s="128"/>
+      <c r="AB39" s="128"/>
+      <c r="AC39" s="129"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1">
       <c r="B40" s="2">
@@ -5280,28 +5628,28 @@
       <c r="F40" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G40" s="138"/>
-      <c r="H40" s="139"/>
-      <c r="I40" s="139"/>
-      <c r="J40" s="140"/>
+      <c r="G40" s="139"/>
+      <c r="H40" s="140"/>
+      <c r="I40" s="140"/>
+      <c r="J40" s="141"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="118" t="s">
+      <c r="T40" s="117" t="s">
         <v>170</v>
       </c>
-      <c r="U40" s="119"/>
-      <c r="V40" s="119"/>
-      <c r="W40" s="119"/>
-      <c r="X40" s="119"/>
-      <c r="Y40" s="119"/>
-      <c r="Z40" s="119"/>
-      <c r="AA40" s="119"/>
-      <c r="AB40" s="119"/>
-      <c r="AC40" s="120"/>
+      <c r="U40" s="118"/>
+      <c r="V40" s="118"/>
+      <c r="W40" s="118"/>
+      <c r="X40" s="118"/>
+      <c r="Y40" s="118"/>
+      <c r="Z40" s="118"/>
+      <c r="AA40" s="118"/>
+      <c r="AB40" s="118"/>
+      <c r="AC40" s="119"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1">
       <c r="B41" s="2">
@@ -5319,28 +5667,28 @@
       <c r="F41" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="G41" s="138"/>
-      <c r="H41" s="139"/>
-      <c r="I41" s="139"/>
-      <c r="J41" s="140"/>
+      <c r="G41" s="139"/>
+      <c r="H41" s="140"/>
+      <c r="I41" s="140"/>
+      <c r="J41" s="141"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="118" t="s">
+      <c r="T41" s="117" t="s">
         <v>171</v>
       </c>
-      <c r="U41" s="119"/>
-      <c r="V41" s="119"/>
-      <c r="W41" s="119"/>
-      <c r="X41" s="119"/>
-      <c r="Y41" s="119"/>
-      <c r="Z41" s="119"/>
-      <c r="AA41" s="119"/>
-      <c r="AB41" s="119"/>
-      <c r="AC41" s="120"/>
+      <c r="U41" s="118"/>
+      <c r="V41" s="118"/>
+      <c r="W41" s="118"/>
+      <c r="X41" s="118"/>
+      <c r="Y41" s="118"/>
+      <c r="Z41" s="118"/>
+      <c r="AA41" s="118"/>
+      <c r="AB41" s="118"/>
+      <c r="AC41" s="119"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
       <c r="B42" s="2">
@@ -5358,28 +5706,28 @@
       <c r="F42" s="76" t="s">
         <v>176</v>
       </c>
-      <c r="G42" s="141"/>
-      <c r="H42" s="142"/>
-      <c r="I42" s="142"/>
-      <c r="J42" s="143"/>
+      <c r="G42" s="136"/>
+      <c r="H42" s="137"/>
+      <c r="I42" s="137"/>
+      <c r="J42" s="138"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="T42" s="118" t="s">
+      <c r="T42" s="117" t="s">
         <v>172</v>
       </c>
-      <c r="U42" s="119"/>
-      <c r="V42" s="119"/>
-      <c r="W42" s="119"/>
-      <c r="X42" s="119"/>
-      <c r="Y42" s="119"/>
-      <c r="Z42" s="119"/>
-      <c r="AA42" s="119"/>
-      <c r="AB42" s="119"/>
-      <c r="AC42" s="120"/>
+      <c r="U42" s="118"/>
+      <c r="V42" s="118"/>
+      <c r="W42" s="118"/>
+      <c r="X42" s="118"/>
+      <c r="Y42" s="118"/>
+      <c r="Z42" s="118"/>
+      <c r="AA42" s="118"/>
+      <c r="AB42" s="118"/>
+      <c r="AC42" s="119"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
       <c r="B43" s="2">
@@ -5397,30 +5745,30 @@
       <c r="F43" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="G43" s="131" t="s">
+      <c r="G43" s="199" t="s">
         <v>192</v>
       </c>
-      <c r="H43" s="132"/>
-      <c r="I43" s="132"/>
-      <c r="J43" s="133"/>
+      <c r="H43" s="120"/>
+      <c r="I43" s="120"/>
+      <c r="J43" s="121"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="T43" s="118" t="s">
+      <c r="T43" s="117" t="s">
         <v>173</v>
       </c>
-      <c r="U43" s="119"/>
-      <c r="V43" s="119"/>
-      <c r="W43" s="119"/>
-      <c r="X43" s="119"/>
-      <c r="Y43" s="119"/>
-      <c r="Z43" s="119"/>
-      <c r="AA43" s="119"/>
-      <c r="AB43" s="119"/>
-      <c r="AC43" s="120"/>
+      <c r="U43" s="118"/>
+      <c r="V43" s="118"/>
+      <c r="W43" s="118"/>
+      <c r="X43" s="118"/>
+      <c r="Y43" s="118"/>
+      <c r="Z43" s="118"/>
+      <c r="AA43" s="118"/>
+      <c r="AB43" s="118"/>
+      <c r="AC43" s="119"/>
     </row>
     <row r="44" spans="2:29" ht="15.75" thickBot="1">
       <c r="B44" s="2">
@@ -5441,21 +5789,21 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="196" t="s">
+      <c r="S44" s="122" t="s">
         <v>76</v>
       </c>
-      <c r="T44" s="198" t="s">
+      <c r="T44" s="124" t="s">
         <v>174</v>
       </c>
-      <c r="U44" s="199"/>
-      <c r="V44" s="199"/>
-      <c r="W44" s="199"/>
-      <c r="X44" s="199"/>
-      <c r="Y44" s="199"/>
-      <c r="Z44" s="199"/>
-      <c r="AA44" s="199"/>
-      <c r="AB44" s="199"/>
-      <c r="AC44" s="200"/>
+      <c r="U44" s="125"/>
+      <c r="V44" s="125"/>
+      <c r="W44" s="125"/>
+      <c r="X44" s="125"/>
+      <c r="Y44" s="125"/>
+      <c r="Z44" s="125"/>
+      <c r="AA44" s="125"/>
+      <c r="AB44" s="125"/>
+      <c r="AC44" s="126"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1">
       <c r="B45" s="2">
@@ -5473,26 +5821,26 @@
       <c r="F45" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="G45" s="112" t="s">
+      <c r="G45" s="133" t="s">
         <v>181</v>
       </c>
-      <c r="H45" s="113"/>
-      <c r="I45" s="113"/>
-      <c r="J45" s="114"/>
+      <c r="H45" s="134"/>
+      <c r="I45" s="134"/>
+      <c r="J45" s="135"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="197"/>
-      <c r="T45" s="201"/>
-      <c r="U45" s="202"/>
-      <c r="V45" s="202"/>
-      <c r="W45" s="202"/>
-      <c r="X45" s="202"/>
-      <c r="Y45" s="202"/>
-      <c r="Z45" s="202"/>
-      <c r="AA45" s="202"/>
-      <c r="AB45" s="202"/>
-      <c r="AC45" s="203"/>
+      <c r="S45" s="123"/>
+      <c r="T45" s="127"/>
+      <c r="U45" s="128"/>
+      <c r="V45" s="128"/>
+      <c r="W45" s="128"/>
+      <c r="X45" s="128"/>
+      <c r="Y45" s="128"/>
+      <c r="Z45" s="128"/>
+      <c r="AA45" s="128"/>
+      <c r="AB45" s="128"/>
+      <c r="AC45" s="129"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
       <c r="B46" s="2">
@@ -5510,28 +5858,28 @@
       <c r="F46" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G46" s="141"/>
-      <c r="H46" s="142"/>
-      <c r="I46" s="142"/>
-      <c r="J46" s="143"/>
+      <c r="G46" s="136"/>
+      <c r="H46" s="137"/>
+      <c r="I46" s="137"/>
+      <c r="J46" s="138"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="T46" s="115" t="s">
+      <c r="T46" s="130" t="s">
         <v>175</v>
       </c>
-      <c r="U46" s="116"/>
-      <c r="V46" s="116"/>
-      <c r="W46" s="116"/>
-      <c r="X46" s="116"/>
-      <c r="Y46" s="116"/>
-      <c r="Z46" s="116"/>
-      <c r="AA46" s="116"/>
-      <c r="AB46" s="116"/>
-      <c r="AC46" s="117"/>
+      <c r="U46" s="131"/>
+      <c r="V46" s="131"/>
+      <c r="W46" s="131"/>
+      <c r="X46" s="131"/>
+      <c r="Y46" s="131"/>
+      <c r="Z46" s="131"/>
+      <c r="AA46" s="131"/>
+      <c r="AB46" s="131"/>
+      <c r="AC46" s="132"/>
     </row>
     <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
       <c r="B47" s="2">
@@ -5549,12 +5897,12 @@
       <c r="F47" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="G47" s="132" t="s">
+      <c r="G47" s="120" t="s">
         <v>152</v>
       </c>
-      <c r="H47" s="132"/>
-      <c r="I47" s="132"/>
-      <c r="J47" s="133"/>
+      <c r="H47" s="120"/>
+      <c r="I47" s="120"/>
+      <c r="J47" s="121"/>
     </row>
     <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
       <c r="B48" s="2">
@@ -5581,23 +5929,23 @@
       <c r="T48" s="104" t="s">
         <v>210</v>
       </c>
-      <c r="U48" s="104" t="s">
+      <c r="U48" s="212" t="s">
         <v>211</v>
       </c>
       <c r="V48" s="103" t="s">
         <v>212</v>
       </c>
-      <c r="W48" s="112" t="s">
+      <c r="W48" s="133" t="s">
         <v>213</v>
       </c>
-      <c r="X48" s="113"/>
-      <c r="Y48" s="113"/>
-      <c r="Z48" s="114"/>
+      <c r="X48" s="134"/>
+      <c r="Y48" s="134"/>
+      <c r="Z48" s="135"/>
       <c r="AA48" s="107" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="49" spans="2:26" ht="33.75" customHeight="1">
+    <row r="49" spans="2:26" ht="35.25" customHeight="1">
       <c r="B49" s="2">
         <v>13</v>
       </c>
@@ -5613,12 +5961,12 @@
       <c r="F49" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="G49" s="112" t="s">
+      <c r="G49" s="133" t="s">
         <v>155</v>
       </c>
-      <c r="H49" s="113"/>
-      <c r="I49" s="113"/>
-      <c r="J49" s="114"/>
+      <c r="H49" s="134"/>
+      <c r="I49" s="134"/>
+      <c r="J49" s="135"/>
       <c r="R49" s="90" t="s">
         <v>232</v>
       </c>
@@ -5638,11 +5986,11 @@
       <c r="W49" s="93" t="s">
         <v>214</v>
       </c>
-      <c r="X49" s="121" t="s">
+      <c r="X49" s="114" t="s">
         <v>218</v>
       </c>
-      <c r="Y49" s="122"/>
-      <c r="Z49" s="123"/>
+      <c r="Y49" s="115"/>
+      <c r="Z49" s="116"/>
     </row>
     <row r="50" spans="2:26" ht="30" customHeight="1">
       <c r="B50" s="2">
@@ -5660,10 +6008,10 @@
       <c r="F50" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="G50" s="138"/>
-      <c r="H50" s="139"/>
-      <c r="I50" s="139"/>
-      <c r="J50" s="140"/>
+      <c r="G50" s="139"/>
+      <c r="H50" s="140"/>
+      <c r="I50" s="140"/>
+      <c r="J50" s="141"/>
       <c r="R50" s="91" t="s">
         <v>229</v>
       </c>
@@ -5683,11 +6031,11 @@
       <c r="W50" s="94" t="s">
         <v>215</v>
       </c>
-      <c r="X50" s="118">
+      <c r="X50" s="117">
         <v>1</v>
       </c>
-      <c r="Y50" s="119"/>
-      <c r="Z50" s="120"/>
+      <c r="Y50" s="118"/>
+      <c r="Z50" s="119"/>
     </row>
     <row r="51" spans="2:26" ht="32.25" customHeight="1" thickBot="1">
       <c r="B51" s="4">
@@ -5705,10 +6053,10 @@
       <c r="F51" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="G51" s="141"/>
-      <c r="H51" s="142"/>
-      <c r="I51" s="142"/>
-      <c r="J51" s="143"/>
+      <c r="G51" s="136"/>
+      <c r="H51" s="137"/>
+      <c r="I51" s="137"/>
+      <c r="J51" s="138"/>
       <c r="R51" s="91" t="s">
         <v>230</v>
       </c>
@@ -5728,20 +6076,20 @@
       <c r="W51" s="94" t="s">
         <v>216</v>
       </c>
-      <c r="X51" s="118">
+      <c r="X51" s="117">
         <v>5</v>
       </c>
-      <c r="Y51" s="119"/>
-      <c r="Z51" s="120"/>
+      <c r="Y51" s="118"/>
+      <c r="Z51" s="119"/>
     </row>
     <row r="52" spans="2:26" ht="30.75" customHeight="1" thickBot="1">
-      <c r="B52" s="152" t="s">
+      <c r="B52" s="191" t="s">
         <v>142</v>
       </c>
-      <c r="C52" s="153"/>
-      <c r="D52" s="153"/>
-      <c r="E52" s="153"/>
-      <c r="F52" s="154"/>
+      <c r="C52" s="172"/>
+      <c r="D52" s="172"/>
+      <c r="E52" s="172"/>
+      <c r="F52" s="173"/>
       <c r="R52" s="108" t="s">
         <v>231</v>
       </c>
@@ -5761,11 +6109,11 @@
       <c r="W52" s="95" t="s">
         <v>217</v>
       </c>
-      <c r="X52" s="115">
-        <v>0</v>
-      </c>
-      <c r="Y52" s="116"/>
-      <c r="Z52" s="117"/>
+      <c r="X52" s="130">
+        <v>0</v>
+      </c>
+      <c r="Y52" s="131"/>
+      <c r="Z52" s="132"/>
     </row>
     <row r="53" spans="2:26" ht="31.5" customHeight="1" thickBot="1">
       <c r="R53" s="90" t="s">
@@ -5787,24 +6135,24 @@
       <c r="W53" s="88" t="s">
         <v>219</v>
       </c>
-      <c r="X53" s="124" t="str">
+      <c r="X53" s="194" t="str">
         <f>DEC2HEX(HEX2DEC($X$49)+_xlfn.BITLSHIFT(X50,20)+_xlfn.BITLSHIFT(X51,15)+_xlfn.BITLSHIFT(X52,12)+4095)</f>
         <v>E0128FFF</v>
       </c>
-      <c r="Y53" s="125"/>
-      <c r="Z53" s="126"/>
+      <c r="Y53" s="195"/>
+      <c r="Z53" s="196"/>
     </row>
     <row r="54" spans="2:26" ht="24.75" customHeight="1">
-      <c r="B54" s="146" t="s">
+      <c r="B54" s="185" t="s">
         <v>183</v>
       </c>
-      <c r="C54" s="144" t="s">
+      <c r="C54" s="183" t="s">
         <v>185</v>
       </c>
-      <c r="D54" s="134" t="s">
+      <c r="D54" s="200" t="s">
         <v>184</v>
       </c>
-      <c r="E54" s="135"/>
+      <c r="E54" s="201"/>
       <c r="R54" s="91" t="s">
         <v>222</v>
       </c>
@@ -5823,10 +6171,10 @@
       </c>
     </row>
     <row r="55" spans="2:26" ht="24" customHeight="1" thickBot="1">
-      <c r="B55" s="147"/>
-      <c r="C55" s="145"/>
-      <c r="D55" s="136"/>
-      <c r="E55" s="137"/>
+      <c r="B55" s="186"/>
+      <c r="C55" s="184"/>
+      <c r="D55" s="202"/>
+      <c r="E55" s="203"/>
       <c r="R55" s="91" t="s">
         <v>223</v>
       </c>
@@ -5851,10 +6199,10 @@
       <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D56" s="121" t="s">
+      <c r="D56" s="114" t="s">
         <v>207</v>
       </c>
-      <c r="E56" s="123"/>
+      <c r="E56" s="116"/>
       <c r="R56" s="91" t="s">
         <v>224</v>
       </c>
@@ -5879,10 +6227,10 @@
       <c r="C57" s="86" t="s">
         <v>203</v>
       </c>
-      <c r="D57" s="127" t="s">
+      <c r="D57" s="187" t="s">
         <v>206</v>
       </c>
-      <c r="E57" s="128"/>
+      <c r="E57" s="188"/>
       <c r="R57" s="91" t="s">
         <v>225</v>
       </c>
@@ -5907,10 +6255,10 @@
       <c r="C58" s="38" t="s">
         <v>204</v>
       </c>
-      <c r="D58" s="127" t="s">
+      <c r="D58" s="187" t="s">
         <v>205</v>
       </c>
-      <c r="E58" s="128"/>
+      <c r="E58" s="188"/>
       <c r="R58" s="91" t="s">
         <v>226</v>
       </c>
@@ -5935,10 +6283,10 @@
       <c r="C59" s="86" t="s">
         <v>186</v>
       </c>
-      <c r="D59" s="127" t="s">
+      <c r="D59" s="187" t="s">
         <v>189</v>
       </c>
-      <c r="E59" s="128"/>
+      <c r="E59" s="188"/>
       <c r="R59" s="91" t="s">
         <v>227</v>
       </c>
@@ -5963,10 +6311,10 @@
       <c r="C60" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="D60" s="127" t="s">
+      <c r="D60" s="187" t="s">
         <v>190</v>
       </c>
-      <c r="E60" s="128"/>
+      <c r="E60" s="188"/>
       <c r="R60" s="92" t="s">
         <v>228</v>
       </c>
@@ -5984,124 +6332,464 @@
         <v>E0138000</v>
       </c>
     </row>
-    <row r="61" spans="2:26" ht="40.5" customHeight="1">
+    <row r="61" spans="2:26" ht="40.5" customHeight="1" thickBot="1">
       <c r="B61" s="82">
         <v>5</v>
       </c>
       <c r="C61" s="38" t="s">
         <v>188</v>
       </c>
-      <c r="D61" s="127" t="s">
+      <c r="D61" s="187" t="s">
         <v>191</v>
       </c>
-      <c r="E61" s="128"/>
-    </row>
-    <row r="62" spans="2:26" ht="36" customHeight="1">
+      <c r="E61" s="188"/>
+    </row>
+    <row r="62" spans="2:26" ht="53.25" customHeight="1" thickBot="1">
       <c r="B62" s="82">
         <v>6</v>
       </c>
       <c r="C62" s="86" t="s">
         <v>196</v>
       </c>
-      <c r="D62" s="127" t="s">
+      <c r="D62" s="187" t="s">
         <v>197</v>
       </c>
-      <c r="E62" s="128"/>
-    </row>
-    <row r="63" spans="2:26">
+      <c r="E62" s="188"/>
+      <c r="R62" s="213" t="s">
+        <v>233</v>
+      </c>
+      <c r="S62" s="214" t="s">
+        <v>234</v>
+      </c>
+      <c r="T62" s="215" t="s">
+        <v>235</v>
+      </c>
+      <c r="U62" s="215" t="s">
+        <v>236</v>
+      </c>
+      <c r="V62" s="216" t="s">
+        <v>237</v>
+      </c>
+      <c r="W62" s="191" t="s">
+        <v>275</v>
+      </c>
+      <c r="X62" s="172"/>
+      <c r="Y62" s="172"/>
+      <c r="Z62" s="173"/>
+    </row>
+    <row r="63" spans="2:26" ht="36" customHeight="1" thickBot="1">
       <c r="B63" s="82">
         <v>7</v>
       </c>
       <c r="C63" s="86"/>
-      <c r="D63" s="127"/>
-      <c r="E63" s="128"/>
-    </row>
-    <row r="64" spans="2:26">
+      <c r="D63" s="187"/>
+      <c r="E63" s="188"/>
+      <c r="R63" s="224" t="s">
+        <v>238</v>
+      </c>
+      <c r="S63" s="227" t="s">
+        <v>239</v>
+      </c>
+      <c r="T63" s="217" t="s">
+        <v>238</v>
+      </c>
+      <c r="U63" s="218" t="s">
+        <v>240</v>
+      </c>
+      <c r="V63" s="219" t="s">
+        <v>241</v>
+      </c>
+      <c r="W63" s="231" t="s">
+        <v>276</v>
+      </c>
+      <c r="X63" s="232"/>
+      <c r="Y63" s="232"/>
+      <c r="Z63" s="233"/>
+    </row>
+    <row r="64" spans="2:26" ht="40.5" customHeight="1" thickBot="1">
       <c r="B64" s="82">
         <v>8</v>
       </c>
       <c r="C64" s="86"/>
-      <c r="D64" s="127"/>
-      <c r="E64" s="128"/>
-    </row>
-    <row r="65" spans="2:5">
+      <c r="D64" s="187"/>
+      <c r="E64" s="188"/>
+      <c r="R64" s="225"/>
+      <c r="S64" s="228"/>
+      <c r="T64" s="204" t="s">
+        <v>242</v>
+      </c>
+      <c r="U64" s="205" t="s">
+        <v>243</v>
+      </c>
+      <c r="V64" s="207" t="s">
+        <v>244</v>
+      </c>
+      <c r="W64" s="194" t="s">
+        <v>277</v>
+      </c>
+      <c r="X64" s="195"/>
+      <c r="Y64" s="195"/>
+      <c r="Z64" s="196"/>
+    </row>
+    <row r="65" spans="2:22" ht="45.75" thickBot="1">
       <c r="B65" s="82">
         <v>9</v>
       </c>
       <c r="C65" s="86"/>
-      <c r="D65" s="127"/>
-      <c r="E65" s="128"/>
-    </row>
-    <row r="66" spans="2:5">
+      <c r="D65" s="187"/>
+      <c r="E65" s="188"/>
+      <c r="R65" s="226"/>
+      <c r="S65" s="229"/>
+      <c r="T65" s="209" t="s">
+        <v>245</v>
+      </c>
+      <c r="U65" s="220" t="s">
+        <v>246</v>
+      </c>
+      <c r="V65" s="210" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="66" spans="2:22" ht="30" customHeight="1">
       <c r="B66" s="82">
         <v>10</v>
       </c>
       <c r="C66" s="86"/>
-      <c r="D66" s="127"/>
-      <c r="E66" s="128"/>
-    </row>
-    <row r="67" spans="2:5">
+      <c r="D66" s="187"/>
+      <c r="E66" s="188"/>
+      <c r="R66" s="224" t="s">
+        <v>248</v>
+      </c>
+      <c r="S66" s="227" t="s">
+        <v>249</v>
+      </c>
+      <c r="T66" s="217" t="s">
+        <v>250</v>
+      </c>
+      <c r="U66" s="218" t="s">
+        <v>251</v>
+      </c>
+      <c r="V66" s="219" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="67" spans="2:22" ht="43.5" thickBot="1">
       <c r="B67" s="82">
         <v>11</v>
       </c>
       <c r="C67" s="86"/>
-      <c r="D67" s="127"/>
-      <c r="E67" s="128"/>
-    </row>
-    <row r="68" spans="2:5">
+      <c r="D67" s="187"/>
+      <c r="E67" s="188"/>
+      <c r="R67" s="226"/>
+      <c r="S67" s="229"/>
+      <c r="T67" s="209" t="s">
+        <v>252</v>
+      </c>
+      <c r="U67" s="208" t="s">
+        <v>253</v>
+      </c>
+      <c r="V67" s="210" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="68" spans="2:22" ht="45">
       <c r="B68" s="82">
         <v>12</v>
       </c>
       <c r="C68" s="86"/>
-      <c r="D68" s="127"/>
-      <c r="E68" s="128"/>
-    </row>
-    <row r="69" spans="2:5">
+      <c r="D68" s="187"/>
+      <c r="E68" s="188"/>
+      <c r="R68" s="224" t="s">
+        <v>254</v>
+      </c>
+      <c r="S68" s="227" t="s">
+        <v>255</v>
+      </c>
+      <c r="T68" s="217" t="s">
+        <v>250</v>
+      </c>
+      <c r="U68" s="206" t="s">
+        <v>256</v>
+      </c>
+      <c r="V68" s="219" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="69" spans="2:22" ht="29.25" thickBot="1">
       <c r="B69" s="82">
         <v>13</v>
       </c>
       <c r="C69" s="86"/>
-      <c r="D69" s="127"/>
-      <c r="E69" s="128"/>
-    </row>
-    <row r="70" spans="2:5">
+      <c r="D69" s="187"/>
+      <c r="E69" s="188"/>
+      <c r="R69" s="226"/>
+      <c r="S69" s="229"/>
+      <c r="T69" s="209" t="s">
+        <v>248</v>
+      </c>
+      <c r="U69" s="208" t="s">
+        <v>258</v>
+      </c>
+      <c r="V69" s="210" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="70" spans="2:22" ht="30" customHeight="1">
       <c r="B70" s="82">
         <v>14</v>
       </c>
       <c r="C70" s="86"/>
-      <c r="D70" s="127"/>
-      <c r="E70" s="128"/>
-    </row>
-    <row r="71" spans="2:5" ht="15.75" thickBot="1">
+      <c r="D70" s="187"/>
+      <c r="E70" s="188"/>
+      <c r="R70" s="224" t="s">
+        <v>259</v>
+      </c>
+      <c r="S70" s="227" t="s">
+        <v>260</v>
+      </c>
+      <c r="T70" s="217" t="s">
+        <v>238</v>
+      </c>
+      <c r="U70" s="218" t="s">
+        <v>261</v>
+      </c>
+      <c r="V70" s="219" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="71" spans="2:22" ht="43.5" thickBot="1">
       <c r="B71" s="83">
         <v>15</v>
       </c>
       <c r="C71" s="87"/>
-      <c r="D71" s="129"/>
-      <c r="E71" s="130"/>
+      <c r="D71" s="197"/>
+      <c r="E71" s="198"/>
+      <c r="R71" s="226"/>
+      <c r="S71" s="229"/>
+      <c r="T71" s="209" t="s">
+        <v>254</v>
+      </c>
+      <c r="U71" s="208" t="s">
+        <v>262</v>
+      </c>
+      <c r="V71" s="210" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="72" spans="2:22" ht="30.75" thickBot="1">
+      <c r="R72" s="230" t="s">
+        <v>263</v>
+      </c>
+      <c r="S72" s="211" t="s">
+        <v>264</v>
+      </c>
+      <c r="T72" s="221" t="s">
+        <v>250</v>
+      </c>
+      <c r="U72" s="222" t="s">
+        <v>265</v>
+      </c>
+      <c r="V72" s="223" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="73" spans="2:22" ht="42.75">
+      <c r="R73" s="224" t="s">
+        <v>242</v>
+      </c>
+      <c r="S73" s="227" t="s">
+        <v>266</v>
+      </c>
+      <c r="T73" s="217" t="s">
+        <v>250</v>
+      </c>
+      <c r="U73" s="218" t="s">
+        <v>267</v>
+      </c>
+      <c r="V73" s="219" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="74" spans="2:22" ht="57.75" thickBot="1">
+      <c r="R74" s="226"/>
+      <c r="S74" s="229"/>
+      <c r="T74" s="209" t="s">
+        <v>259</v>
+      </c>
+      <c r="U74" s="220" t="s">
+        <v>268</v>
+      </c>
+      <c r="V74" s="210" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="75" spans="2:22" ht="72" customHeight="1">
+      <c r="R75" s="224" t="s">
+        <v>270</v>
+      </c>
+      <c r="S75" s="227" t="s">
+        <v>271</v>
+      </c>
+      <c r="T75" s="217" t="s">
+        <v>254</v>
+      </c>
+      <c r="U75" s="206" t="s">
+        <v>272</v>
+      </c>
+      <c r="V75" s="219" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="76" spans="2:22" ht="43.5" thickBot="1">
+      <c r="R76" s="226"/>
+      <c r="S76" s="229"/>
+      <c r="T76" s="209" t="s">
+        <v>263</v>
+      </c>
+      <c r="U76" s="208" t="s">
+        <v>274</v>
+      </c>
+      <c r="V76" s="210" t="s">
+        <v>250</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="164">
-    <mergeCell ref="T30:AC30"/>
-    <mergeCell ref="T31:AC31"/>
-    <mergeCell ref="T32:AC32"/>
-    <mergeCell ref="T33:AC33"/>
-    <mergeCell ref="T34:AC34"/>
-    <mergeCell ref="T35:AC35"/>
-    <mergeCell ref="T36:AC36"/>
-    <mergeCell ref="T37:AC37"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="S38:S39"/>
-    <mergeCell ref="T38:AC39"/>
-    <mergeCell ref="S44:S45"/>
-    <mergeCell ref="T44:AC45"/>
-    <mergeCell ref="T40:AC40"/>
-    <mergeCell ref="T41:AC41"/>
-    <mergeCell ref="T42:AC42"/>
-    <mergeCell ref="T43:AC43"/>
-    <mergeCell ref="T46:AC46"/>
-    <mergeCell ref="G45:J46"/>
-    <mergeCell ref="G39:J42"/>
+  <mergeCells count="179">
+    <mergeCell ref="S73:S74"/>
+    <mergeCell ref="R73:R74"/>
+    <mergeCell ref="S75:S76"/>
+    <mergeCell ref="R75:R76"/>
+    <mergeCell ref="W62:Z62"/>
+    <mergeCell ref="W63:Z63"/>
+    <mergeCell ref="W64:Z64"/>
+    <mergeCell ref="R63:R65"/>
+    <mergeCell ref="R66:R67"/>
+    <mergeCell ref="S63:S65"/>
+    <mergeCell ref="S66:S67"/>
+    <mergeCell ref="S68:S69"/>
+    <mergeCell ref="R68:R69"/>
+    <mergeCell ref="R70:R71"/>
+    <mergeCell ref="S70:S71"/>
+    <mergeCell ref="W48:Z48"/>
+    <mergeCell ref="X52:Z52"/>
+    <mergeCell ref="X51:Z51"/>
+    <mergeCell ref="X50:Z50"/>
+    <mergeCell ref="X49:Z49"/>
+    <mergeCell ref="X53:Z53"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D54:E55"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="AA7:AB7"/>
+    <mergeCell ref="AA28:AB28"/>
+    <mergeCell ref="AA12:AB12"/>
+    <mergeCell ref="AA13:AB13"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AA25:AB25"/>
+    <mergeCell ref="AA26:AB26"/>
+    <mergeCell ref="U27:V27"/>
+    <mergeCell ref="AA27:AB27"/>
+    <mergeCell ref="U12:V12"/>
+    <mergeCell ref="AA14:AB14"/>
+    <mergeCell ref="U28:V28"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="N20:P20"/>
+    <mergeCell ref="N21:P21"/>
+    <mergeCell ref="N23:P23"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AA11:AB11"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="N26:P26"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="N24:P24"/>
+    <mergeCell ref="E27:J27"/>
+    <mergeCell ref="E22:J22"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K2:P2"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AA17:AB17"/>
+    <mergeCell ref="AA18:AB18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="N13:P13"/>
     <mergeCell ref="AA20:AB20"/>
     <mergeCell ref="AA21:AB21"/>
     <mergeCell ref="AA22:AB22"/>
@@ -6126,126 +6814,26 @@
     <mergeCell ref="U11:V11"/>
     <mergeCell ref="AA23:AB23"/>
     <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AA17:AB17"/>
-    <mergeCell ref="AA18:AB18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="AA19:AB19"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="N27:P27"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="E28:J28"/>
-    <mergeCell ref="N24:P24"/>
-    <mergeCell ref="E27:J27"/>
-    <mergeCell ref="E22:J22"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K2:P2"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AA11:AB11"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B52:F52"/>
-    <mergeCell ref="AA7:AB7"/>
-    <mergeCell ref="AA28:AB28"/>
-    <mergeCell ref="AA12:AB12"/>
-    <mergeCell ref="AA13:AB13"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AA25:AB25"/>
-    <mergeCell ref="AA26:AB26"/>
-    <mergeCell ref="U27:V27"/>
-    <mergeCell ref="AA27:AB27"/>
-    <mergeCell ref="U12:V12"/>
-    <mergeCell ref="AA14:AB14"/>
-    <mergeCell ref="U28:V28"/>
-    <mergeCell ref="N17:P17"/>
-    <mergeCell ref="N19:P19"/>
-    <mergeCell ref="N20:P20"/>
-    <mergeCell ref="N21:P21"/>
-    <mergeCell ref="N23:P23"/>
-    <mergeCell ref="W48:Z48"/>
-    <mergeCell ref="X52:Z52"/>
-    <mergeCell ref="X51:Z51"/>
-    <mergeCell ref="X50:Z50"/>
-    <mergeCell ref="X49:Z49"/>
-    <mergeCell ref="X53:Z53"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D54:E55"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="T30:AC30"/>
+    <mergeCell ref="T31:AC31"/>
+    <mergeCell ref="T32:AC32"/>
+    <mergeCell ref="T33:AC33"/>
+    <mergeCell ref="T34:AC34"/>
+    <mergeCell ref="T35:AC35"/>
+    <mergeCell ref="T36:AC36"/>
+    <mergeCell ref="T37:AC37"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="S38:S39"/>
+    <mergeCell ref="T38:AC39"/>
+    <mergeCell ref="S44:S45"/>
+    <mergeCell ref="T44:AC45"/>
+    <mergeCell ref="T40:AC40"/>
+    <mergeCell ref="T41:AC41"/>
+    <mergeCell ref="T42:AC42"/>
+    <mergeCell ref="T43:AC43"/>
+    <mergeCell ref="T46:AC46"/>
+    <mergeCell ref="G45:J46"/>
+    <mergeCell ref="G39:J42"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Se cambiaron las banderas de estados a un modelo mas realista, ademas se actualizo todo el Instr Fecher y el PC, se creo un nuevo estilo de LDI y las instrucciones silenciosas. finalmente el CPU paso la pruueba de Fibonacci
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF659EDA-1E1F-4E7C-A31D-3963FAB1A1A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A228B2A4-A3F3-4C34-BE5A-7A2D2332094A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="339">
   <si>
     <t>OpCode</t>
   </si>
@@ -1351,6 +1351,12 @@
   </si>
   <si>
     <t>int 32 / short 16 / char 8</t>
+  </si>
+  <si>
+    <t>Bit 31 = Silent Instr</t>
+  </si>
+  <si>
+    <t>Bit 31 = Alta/Baja</t>
   </si>
 </sst>
 </file>
@@ -1419,7 +1425,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1468,6 +1474,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="74">
     <border>
@@ -2398,7 +2410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="300">
+  <cellXfs count="301">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2931,6 +2943,276 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3006,42 +3288,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3051,24 +3297,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3083,219 +3311,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3609,62 +3624,62 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B2" s="269" t="s">
+      <c r="B2" s="234" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="281" t="s">
+      <c r="C2" s="249" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="282"/>
-      <c r="E2" s="283" t="s">
+      <c r="D2" s="250"/>
+      <c r="E2" s="251" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="283"/>
-      <c r="G2" s="284" t="s">
+      <c r="F2" s="251"/>
+      <c r="G2" s="252" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="283"/>
-      <c r="I2" s="283" t="s">
+      <c r="H2" s="251"/>
+      <c r="I2" s="251" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="283"/>
-      <c r="K2" s="285" t="s">
+      <c r="J2" s="251"/>
+      <c r="K2" s="253" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="283"/>
-      <c r="M2" s="283"/>
-      <c r="N2" s="283"/>
-      <c r="O2" s="283"/>
-      <c r="P2" s="286"/>
-      <c r="R2" s="266" t="s">
+      <c r="L2" s="251"/>
+      <c r="M2" s="251"/>
+      <c r="N2" s="251"/>
+      <c r="O2" s="251"/>
+      <c r="P2" s="254"/>
+      <c r="R2" s="230" t="s">
         <v>65</v>
       </c>
-      <c r="S2" s="263" t="s">
+      <c r="S2" s="227" t="s">
         <v>66</v>
       </c>
-      <c r="T2" s="256" t="s">
+      <c r="T2" s="220" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="257"/>
-      <c r="V2" s="257"/>
-      <c r="W2" s="257"/>
-      <c r="X2" s="257"/>
-      <c r="Y2" s="257"/>
-      <c r="Z2" s="257"/>
-      <c r="AA2" s="257"/>
-      <c r="AB2" s="257" t="s">
+      <c r="U2" s="221"/>
+      <c r="V2" s="221"/>
+      <c r="W2" s="221"/>
+      <c r="X2" s="221"/>
+      <c r="Y2" s="221"/>
+      <c r="Z2" s="221"/>
+      <c r="AA2" s="221"/>
+      <c r="AB2" s="221" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="257"/>
-      <c r="AD2" s="257"/>
-      <c r="AE2" s="257"/>
-      <c r="AF2" s="257"/>
-      <c r="AG2" s="257"/>
-      <c r="AH2" s="257"/>
-      <c r="AI2" s="258"/>
+      <c r="AC2" s="221"/>
+      <c r="AD2" s="221"/>
+      <c r="AE2" s="221"/>
+      <c r="AF2" s="221"/>
+      <c r="AG2" s="221"/>
+      <c r="AH2" s="221"/>
+      <c r="AI2" s="222"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B3" s="270"/>
+      <c r="B3" s="235"/>
       <c r="C3" s="16" t="s">
         <v>79</v>
       </c>
@@ -3689,21 +3704,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="247"/>
-      <c r="L3" s="280"/>
-      <c r="M3" s="280"/>
-      <c r="N3" s="280"/>
-      <c r="O3" s="280"/>
-      <c r="P3" s="248"/>
-      <c r="R3" s="267"/>
-      <c r="S3" s="264"/>
+      <c r="K3" s="205"/>
+      <c r="L3" s="248"/>
+      <c r="M3" s="248"/>
+      <c r="N3" s="248"/>
+      <c r="O3" s="248"/>
+      <c r="P3" s="206"/>
+      <c r="R3" s="231"/>
+      <c r="S3" s="228"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="290" t="s">
+      <c r="U3" s="258" t="s">
         <v>83</v>
       </c>
-      <c r="V3" s="290"/>
+      <c r="V3" s="258"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -3716,10 +3731,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="255" t="s">
+      <c r="AA3" s="219" t="s">
         <v>74</v>
       </c>
-      <c r="AB3" s="255"/>
+      <c r="AB3" s="219"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -3743,21 +3758,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B4" s="271"/>
+      <c r="B4" s="236"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="259" t="s">
+      <c r="E4" s="223" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="222"/>
-      <c r="G4" s="222"/>
-      <c r="H4" s="222"/>
-      <c r="I4" s="222"/>
-      <c r="J4" s="223"/>
+      <c r="F4" s="210"/>
+      <c r="G4" s="210"/>
+      <c r="H4" s="210"/>
+      <c r="I4" s="210"/>
+      <c r="J4" s="211"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -3767,20 +3782,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="259" t="s">
+      <c r="N4" s="223" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="222"/>
-      <c r="P4" s="223"/>
-      <c r="R4" s="268"/>
-      <c r="S4" s="265"/>
+      <c r="O4" s="210"/>
+      <c r="P4" s="211"/>
+      <c r="R4" s="232"/>
+      <c r="S4" s="229"/>
       <c r="T4" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="U4" s="259" t="s">
+      <c r="U4" s="223" t="s">
         <v>75</v>
       </c>
-      <c r="V4" s="260"/>
+      <c r="V4" s="224"/>
       <c r="W4" s="7" t="s">
         <v>71</v>
       </c>
@@ -3793,10 +3808,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="259" t="s">
+      <c r="AA4" s="223" t="s">
         <v>72</v>
       </c>
-      <c r="AB4" s="260"/>
+      <c r="AB4" s="224"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -3828,22 +3843,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="287"/>
-      <c r="F5" s="288"/>
-      <c r="G5" s="288"/>
-      <c r="H5" s="288"/>
-      <c r="I5" s="288"/>
-      <c r="J5" s="289"/>
+      <c r="E5" s="255"/>
+      <c r="F5" s="256"/>
+      <c r="G5" s="256"/>
+      <c r="H5" s="256"/>
+      <c r="I5" s="256"/>
+      <c r="J5" s="257"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="212" t="s">
+      <c r="N5" s="190" t="s">
         <v>51</v>
       </c>
-      <c r="O5" s="213"/>
-      <c r="P5" s="214"/>
+      <c r="O5" s="233"/>
+      <c r="P5" s="191"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -3853,10 +3868,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="261" t="s">
+      <c r="U5" s="225" t="s">
         <v>73</v>
       </c>
-      <c r="V5" s="262"/>
+      <c r="V5" s="226"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -3869,10 +3884,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="261" t="s">
+      <c r="AA5" s="225" t="s">
         <v>73</v>
       </c>
-      <c r="AB5" s="262"/>
+      <c r="AB5" s="226"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -3904,12 +3919,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="278"/>
-      <c r="F6" s="273"/>
-      <c r="G6" s="273"/>
-      <c r="H6" s="273"/>
-      <c r="I6" s="273"/>
-      <c r="J6" s="274"/>
+      <c r="E6" s="246"/>
+      <c r="F6" s="241"/>
+      <c r="G6" s="241"/>
+      <c r="H6" s="241"/>
+      <c r="I6" s="241"/>
+      <c r="J6" s="242"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -3917,11 +3932,11 @@
         <v>155</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="209" t="s">
+      <c r="N6" s="216" t="s">
         <v>95</v>
       </c>
-      <c r="O6" s="210"/>
-      <c r="P6" s="211"/>
+      <c r="O6" s="217"/>
+      <c r="P6" s="218"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -3931,10 +3946,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="251" t="s">
+      <c r="U6" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V6" s="252"/>
+      <c r="V6" s="213"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -3947,10 +3962,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="251" t="s">
+      <c r="AA6" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB6" s="252"/>
+      <c r="AB6" s="213"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -3977,7 +3992,9 @@
       <c r="B7" s="2">
         <v>2</v>
       </c>
-      <c r="C7" s="30"/>
+      <c r="C7" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D7" s="23" t="str">
         <f t="shared" si="0"/>
         <v>00010</v>
@@ -3991,9 +4008,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="272"/>
-      <c r="I7" s="273"/>
-      <c r="J7" s="274"/>
+      <c r="H7" s="240"/>
+      <c r="I7" s="241"/>
+      <c r="J7" s="242"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -4001,11 +4018,11 @@
       <c r="M7" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N7" s="209" t="s">
+      <c r="N7" s="216" t="s">
         <v>52</v>
       </c>
-      <c r="O7" s="210"/>
-      <c r="P7" s="211"/>
+      <c r="O7" s="217"/>
+      <c r="P7" s="218"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -4015,10 +4032,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="251" t="s">
+      <c r="U7" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V7" s="252"/>
+      <c r="V7" s="213"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -4031,10 +4048,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="251" t="s">
+      <c r="AA7" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB7" s="252"/>
+      <c r="AB7" s="213"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -4061,7 +4078,9 @@
       <c r="B8" s="2">
         <v>3</v>
       </c>
-      <c r="C8" s="30"/>
+      <c r="C8" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D8" s="23" t="str">
         <f t="shared" si="0"/>
         <v>00011</v>
@@ -4075,9 +4094,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="272"/>
-      <c r="I8" s="273"/>
-      <c r="J8" s="274"/>
+      <c r="H8" s="240"/>
+      <c r="I8" s="241"/>
+      <c r="J8" s="242"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -4085,11 +4104,11 @@
       <c r="M8" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N8" s="209" t="s">
+      <c r="N8" s="216" t="s">
         <v>53</v>
       </c>
-      <c r="O8" s="210"/>
-      <c r="P8" s="211"/>
+      <c r="O8" s="217"/>
+      <c r="P8" s="218"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -4099,10 +4118,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="251" t="s">
+      <c r="U8" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V8" s="252"/>
+      <c r="V8" s="213"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -4115,10 +4134,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="251" t="s">
+      <c r="AA8" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB8" s="252"/>
+      <c r="AB8" s="213"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -4145,7 +4164,9 @@
       <c r="B9" s="1">
         <v>4</v>
       </c>
-      <c r="C9" s="30"/>
+      <c r="C9" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D9" s="23" t="str">
         <f t="shared" si="0"/>
         <v>00100</v>
@@ -4159,9 +4180,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="272"/>
-      <c r="I9" s="273"/>
-      <c r="J9" s="274"/>
+      <c r="H9" s="240"/>
+      <c r="I9" s="241"/>
+      <c r="J9" s="242"/>
       <c r="K9" s="37" t="s">
         <v>47</v>
       </c>
@@ -4169,11 +4190,11 @@
       <c r="M9" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N9" s="209" t="s">
+      <c r="N9" s="216" t="s">
         <v>54</v>
       </c>
-      <c r="O9" s="210"/>
-      <c r="P9" s="211"/>
+      <c r="O9" s="217"/>
+      <c r="P9" s="218"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -4183,10 +4204,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="251" t="s">
+      <c r="U9" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V9" s="252"/>
+      <c r="V9" s="213"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -4199,10 +4220,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="251" t="s">
+      <c r="AA9" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB9" s="252"/>
+      <c r="AB9" s="213"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -4229,7 +4250,9 @@
       <c r="B10" s="2">
         <v>5</v>
       </c>
-      <c r="C10" s="30"/>
+      <c r="C10" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D10" s="23" t="str">
         <f t="shared" si="0"/>
         <v>00101</v>
@@ -4243,9 +4266,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="272"/>
-      <c r="I10" s="273"/>
-      <c r="J10" s="274"/>
+      <c r="H10" s="240"/>
+      <c r="I10" s="241"/>
+      <c r="J10" s="242"/>
       <c r="K10" s="37" t="s">
         <v>48</v>
       </c>
@@ -4253,11 +4276,11 @@
       <c r="M10" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N10" s="209" t="s">
+      <c r="N10" s="216" t="s">
         <v>55</v>
       </c>
-      <c r="O10" s="210"/>
-      <c r="P10" s="211"/>
+      <c r="O10" s="217"/>
+      <c r="P10" s="218"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -4267,10 +4290,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="251" t="s">
+      <c r="U10" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V10" s="252"/>
+      <c r="V10" s="213"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -4283,10 +4306,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="251" t="s">
+      <c r="AA10" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB10" s="252"/>
+      <c r="AB10" s="213"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -4313,7 +4336,9 @@
       <c r="B11" s="2">
         <v>6</v>
       </c>
-      <c r="C11" s="30"/>
+      <c r="C11" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D11" s="23" t="str">
         <f t="shared" si="0"/>
         <v>00110</v>
@@ -4327,9 +4352,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="272"/>
-      <c r="I11" s="273"/>
-      <c r="J11" s="274"/>
+      <c r="H11" s="240"/>
+      <c r="I11" s="241"/>
+      <c r="J11" s="242"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -4337,11 +4362,11 @@
       <c r="M11" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N11" s="209" t="s">
+      <c r="N11" s="216" t="s">
         <v>56</v>
       </c>
-      <c r="O11" s="210"/>
-      <c r="P11" s="211"/>
+      <c r="O11" s="217"/>
+      <c r="P11" s="218"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -4351,10 +4376,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="251" t="s">
+      <c r="U11" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V11" s="252"/>
+      <c r="V11" s="213"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -4367,10 +4392,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="251" t="s">
+      <c r="AA11" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB11" s="252"/>
+      <c r="AB11" s="213"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -4397,7 +4422,9 @@
       <c r="B12" s="2">
         <v>7</v>
       </c>
-      <c r="C12" s="30"/>
+      <c r="C12" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D12" s="23" t="str">
         <f t="shared" si="0"/>
         <v>00111</v>
@@ -4411,9 +4438,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="272"/>
-      <c r="I12" s="273"/>
-      <c r="J12" s="274"/>
+      <c r="H12" s="240"/>
+      <c r="I12" s="241"/>
+      <c r="J12" s="242"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -4421,11 +4448,11 @@
       <c r="M12" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N12" s="209" t="s">
+      <c r="N12" s="216" t="s">
         <v>57</v>
       </c>
-      <c r="O12" s="210"/>
-      <c r="P12" s="211"/>
+      <c r="O12" s="217"/>
+      <c r="P12" s="218"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -4435,10 +4462,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="251" t="s">
+      <c r="U12" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V12" s="252"/>
+      <c r="V12" s="213"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -4451,10 +4478,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="251" t="s">
+      <c r="AA12" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB12" s="252"/>
+      <c r="AB12" s="213"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -4481,7 +4508,9 @@
       <c r="B13" s="1">
         <v>8</v>
       </c>
-      <c r="C13" s="30"/>
+      <c r="C13" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D13" s="23" t="str">
         <f t="shared" si="0"/>
         <v>01000</v>
@@ -4495,9 +4524,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="272"/>
-      <c r="I13" s="273"/>
-      <c r="J13" s="274"/>
+      <c r="H13" s="240"/>
+      <c r="I13" s="241"/>
+      <c r="J13" s="242"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -4505,11 +4534,11 @@
       <c r="M13" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N13" s="209" t="s">
+      <c r="N13" s="216" t="s">
         <v>58</v>
       </c>
-      <c r="O13" s="210"/>
-      <c r="P13" s="211"/>
+      <c r="O13" s="217"/>
+      <c r="P13" s="218"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -4519,10 +4548,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="251" t="s">
+      <c r="U13" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V13" s="252"/>
+      <c r="V13" s="213"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -4535,10 +4564,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="251" t="s">
+      <c r="AA13" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB13" s="252"/>
+      <c r="AB13" s="213"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -4565,7 +4594,9 @@
       <c r="B14" s="2">
         <v>9</v>
       </c>
-      <c r="C14" s="30"/>
+      <c r="C14" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D14" s="23" t="str">
         <f t="shared" si="0"/>
         <v>01001</v>
@@ -4579,9 +4610,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="272"/>
-      <c r="I14" s="273"/>
-      <c r="J14" s="274"/>
+      <c r="H14" s="240"/>
+      <c r="I14" s="241"/>
+      <c r="J14" s="242"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -4589,11 +4620,11 @@
       <c r="M14" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N14" s="209" t="s">
+      <c r="N14" s="216" t="s">
         <v>59</v>
       </c>
-      <c r="O14" s="210"/>
-      <c r="P14" s="211"/>
+      <c r="O14" s="217"/>
+      <c r="P14" s="218"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -4603,10 +4634,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="251" t="s">
+      <c r="U14" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V14" s="252"/>
+      <c r="V14" s="213"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -4619,10 +4650,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="251" t="s">
+      <c r="AA14" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB14" s="252"/>
+      <c r="AB14" s="213"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -4649,7 +4680,9 @@
       <c r="B15" s="2">
         <v>10</v>
       </c>
-      <c r="C15" s="30"/>
+      <c r="C15" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D15" s="23" t="str">
         <f t="shared" si="0"/>
         <v>01010</v>
@@ -4663,9 +4696,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="272"/>
-      <c r="I15" s="273"/>
-      <c r="J15" s="274"/>
+      <c r="H15" s="240"/>
+      <c r="I15" s="241"/>
+      <c r="J15" s="242"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -4673,11 +4706,11 @@
       <c r="M15" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N15" s="209" t="s">
+      <c r="N15" s="216" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="210"/>
-      <c r="P15" s="211"/>
+      <c r="O15" s="217"/>
+      <c r="P15" s="218"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -4687,10 +4720,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="251" t="s">
+      <c r="U15" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V15" s="252"/>
+      <c r="V15" s="213"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -4703,10 +4736,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="251" t="s">
+      <c r="AA15" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB15" s="252"/>
+      <c r="AB15" s="213"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -4733,7 +4766,9 @@
       <c r="B16" s="2">
         <v>11</v>
       </c>
-      <c r="C16" s="30"/>
+      <c r="C16" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D16" s="23" t="str">
         <f t="shared" si="0"/>
         <v>01011</v>
@@ -4741,21 +4776,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="272"/>
-      <c r="G16" s="273"/>
-      <c r="H16" s="273"/>
-      <c r="I16" s="273"/>
-      <c r="J16" s="274"/>
+      <c r="F16" s="240"/>
+      <c r="G16" s="241"/>
+      <c r="H16" s="241"/>
+      <c r="I16" s="241"/>
+      <c r="J16" s="242"/>
       <c r="K16" s="40" t="s">
         <v>49</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="209" t="s">
+      <c r="N16" s="216" t="s">
         <v>50</v>
       </c>
-      <c r="O16" s="210"/>
-      <c r="P16" s="211"/>
+      <c r="O16" s="217"/>
+      <c r="P16" s="218"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -4765,10 +4800,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="251" t="s">
+      <c r="U16" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V16" s="252"/>
+      <c r="V16" s="213"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -4781,10 +4816,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="251" t="s">
+      <c r="AA16" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB16" s="252"/>
+      <c r="AB16" s="213"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -4811,7 +4846,9 @@
       <c r="B17" s="2">
         <v>12</v>
       </c>
-      <c r="C17" s="30"/>
+      <c r="C17" s="178" t="s">
+        <v>338</v>
+      </c>
       <c r="D17" s="23" t="str">
         <f t="shared" si="0"/>
         <v>01100</v>
@@ -4820,22 +4857,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="279" t="s">
+      <c r="G17" s="247" t="s">
         <v>76</v>
       </c>
-      <c r="H17" s="210"/>
-      <c r="I17" s="210"/>
-      <c r="J17" s="211"/>
+      <c r="H17" s="217"/>
+      <c r="I17" s="217"/>
+      <c r="J17" s="218"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="209" t="s">
+      <c r="N17" s="216" t="s">
         <v>64</v>
       </c>
-      <c r="O17" s="210"/>
-      <c r="P17" s="211"/>
+      <c r="O17" s="217"/>
+      <c r="P17" s="218"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -4845,10 +4882,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="251" t="s">
+      <c r="U17" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V17" s="252"/>
+      <c r="V17" s="213"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -4861,10 +4898,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="251" t="s">
+      <c r="AA17" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB17" s="252"/>
+      <c r="AB17" s="213"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -4891,7 +4928,9 @@
       <c r="B18" s="2">
         <v>13</v>
       </c>
-      <c r="C18" s="30"/>
+      <c r="C18" s="178" t="s">
+        <v>337</v>
+      </c>
       <c r="D18" s="23" t="str">
         <f t="shared" si="0"/>
         <v>01101</v>
@@ -4900,12 +4939,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="279" t="s">
+      <c r="G18" s="247" t="s">
         <v>76</v>
       </c>
-      <c r="H18" s="210"/>
-      <c r="I18" s="210"/>
-      <c r="J18" s="211"/>
+      <c r="H18" s="217"/>
+      <c r="I18" s="217"/>
+      <c r="J18" s="218"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -4913,11 +4952,11 @@
       <c r="M18" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N18" s="209" t="s">
+      <c r="N18" s="216" t="s">
         <v>61</v>
       </c>
-      <c r="O18" s="210"/>
-      <c r="P18" s="211"/>
+      <c r="O18" s="217"/>
+      <c r="P18" s="218"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -4927,10 +4966,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="251" t="s">
+      <c r="U18" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V18" s="252"/>
+      <c r="V18" s="213"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -4943,10 +4982,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="251" t="s">
+      <c r="AA18" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB18" s="252"/>
+      <c r="AB18" s="213"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -4984,20 +5023,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="272"/>
-      <c r="H19" s="273"/>
-      <c r="I19" s="273"/>
-      <c r="J19" s="274"/>
+      <c r="G19" s="240"/>
+      <c r="H19" s="241"/>
+      <c r="I19" s="241"/>
+      <c r="J19" s="242"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="209" t="s">
+      <c r="N19" s="216" t="s">
         <v>93</v>
       </c>
-      <c r="O19" s="210"/>
-      <c r="P19" s="211"/>
+      <c r="O19" s="217"/>
+      <c r="P19" s="218"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -5007,10 +5046,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="251" t="s">
+      <c r="U19" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V19" s="252"/>
+      <c r="V19" s="213"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -5023,10 +5062,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="251" t="s">
+      <c r="AA19" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB19" s="252"/>
+      <c r="AB19" s="213"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -5066,20 +5105,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="272"/>
-      <c r="H20" s="273"/>
-      <c r="I20" s="273"/>
-      <c r="J20" s="274"/>
+      <c r="G20" s="240"/>
+      <c r="H20" s="241"/>
+      <c r="I20" s="241"/>
+      <c r="J20" s="242"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="209" t="s">
+      <c r="N20" s="216" t="s">
         <v>94</v>
       </c>
-      <c r="O20" s="210"/>
-      <c r="P20" s="211"/>
+      <c r="O20" s="217"/>
+      <c r="P20" s="218"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -5089,10 +5128,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="251" t="s">
+      <c r="U20" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V20" s="252"/>
+      <c r="V20" s="213"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -5105,10 +5144,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="251" t="s">
+      <c r="AA20" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB20" s="252"/>
+      <c r="AB20" s="213"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -5146,20 +5185,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="272"/>
-      <c r="H21" s="273"/>
-      <c r="I21" s="273"/>
-      <c r="J21" s="274"/>
+      <c r="G21" s="240"/>
+      <c r="H21" s="241"/>
+      <c r="I21" s="241"/>
+      <c r="J21" s="242"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="209" t="s">
+      <c r="N21" s="216" t="s">
         <v>62</v>
       </c>
-      <c r="O21" s="210"/>
-      <c r="P21" s="211"/>
+      <c r="O21" s="217"/>
+      <c r="P21" s="218"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -5169,10 +5208,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="251" t="s">
+      <c r="U21" s="212" t="s">
         <v>96</v>
       </c>
-      <c r="V21" s="252"/>
+      <c r="V21" s="213"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -5185,10 +5224,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="251" t="s">
+      <c r="AA21" s="212" t="s">
         <v>98</v>
       </c>
-      <c r="AB21" s="252"/>
+      <c r="AB21" s="213"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -5222,22 +5261,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="278"/>
-      <c r="F22" s="273"/>
-      <c r="G22" s="273"/>
-      <c r="H22" s="273"/>
-      <c r="I22" s="273"/>
-      <c r="J22" s="274"/>
+      <c r="E22" s="246"/>
+      <c r="F22" s="241"/>
+      <c r="G22" s="241"/>
+      <c r="H22" s="241"/>
+      <c r="I22" s="241"/>
+      <c r="J22" s="242"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="209" t="s">
+      <c r="N22" s="216" t="s">
         <v>63</v>
       </c>
-      <c r="O22" s="210"/>
-      <c r="P22" s="211"/>
+      <c r="O22" s="217"/>
+      <c r="P22" s="218"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -5247,10 +5286,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="251" t="s">
+      <c r="U22" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V22" s="252"/>
+      <c r="V22" s="213"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -5263,10 +5302,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="251" t="s">
+      <c r="AA22" s="212" t="s">
         <v>96</v>
       </c>
-      <c r="AB22" s="252"/>
+      <c r="AB22" s="213"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -5306,22 +5345,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="279" t="s">
+      <c r="G23" s="247" t="s">
         <v>77</v>
       </c>
-      <c r="H23" s="210"/>
-      <c r="I23" s="210"/>
-      <c r="J23" s="211"/>
+      <c r="H23" s="217"/>
+      <c r="I23" s="217"/>
+      <c r="J23" s="218"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="209" t="s">
+      <c r="N23" s="216" t="s">
         <v>82</v>
       </c>
-      <c r="O23" s="210"/>
-      <c r="P23" s="211"/>
+      <c r="O23" s="217"/>
+      <c r="P23" s="218"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -5331,10 +5370,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="251" t="s">
+      <c r="U23" s="212" t="s">
         <v>97</v>
       </c>
-      <c r="V23" s="252"/>
+      <c r="V23" s="213"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -5347,10 +5386,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="251" t="s">
+      <c r="AA23" s="212" t="s">
         <v>96</v>
       </c>
-      <c r="AB23" s="252"/>
+      <c r="AB23" s="213"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -5390,22 +5429,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="279" t="s">
+      <c r="G24" s="247" t="s">
         <v>77</v>
       </c>
-      <c r="H24" s="210"/>
-      <c r="I24" s="210"/>
-      <c r="J24" s="211"/>
+      <c r="H24" s="217"/>
+      <c r="I24" s="217"/>
+      <c r="J24" s="218"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="209" t="s">
+      <c r="N24" s="216" t="s">
         <v>81</v>
       </c>
-      <c r="O24" s="210"/>
-      <c r="P24" s="211"/>
+      <c r="O24" s="217"/>
+      <c r="P24" s="218"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -5415,10 +5454,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="251" t="s">
+      <c r="U24" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V24" s="252"/>
+      <c r="V24" s="213"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -5431,10 +5470,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="251" t="s">
+      <c r="AA24" s="212" t="s">
         <v>98</v>
       </c>
-      <c r="AB24" s="252"/>
+      <c r="AB24" s="213"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -5472,10 +5511,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="272"/>
-      <c r="H25" s="273"/>
-      <c r="I25" s="273"/>
-      <c r="J25" s="274"/>
+      <c r="G25" s="240"/>
+      <c r="H25" s="241"/>
+      <c r="I25" s="241"/>
+      <c r="J25" s="242"/>
       <c r="K25" s="49" t="s">
         <v>39</v>
       </c>
@@ -5483,11 +5522,11 @@
         <v>155</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="209" t="s">
+      <c r="N25" s="216" t="s">
         <v>41</v>
       </c>
-      <c r="O25" s="210"/>
-      <c r="P25" s="211"/>
+      <c r="O25" s="217"/>
+      <c r="P25" s="218"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -5497,10 +5536,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="251" t="s">
+      <c r="U25" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V25" s="252"/>
+      <c r="V25" s="213"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -5513,10 +5552,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="251" t="s">
+      <c r="AA25" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB25" s="252"/>
+      <c r="AB25" s="213"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -5554,10 +5593,10 @@
       <c r="F26" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="G26" s="272"/>
-      <c r="H26" s="273"/>
-      <c r="I26" s="273"/>
-      <c r="J26" s="274"/>
+      <c r="G26" s="240"/>
+      <c r="H26" s="241"/>
+      <c r="I26" s="241"/>
+      <c r="J26" s="242"/>
       <c r="K26" s="31" t="s">
         <v>40</v>
       </c>
@@ -5565,11 +5604,11 @@
         <v>155</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="209" t="s">
+      <c r="N26" s="216" t="s">
         <v>42</v>
       </c>
-      <c r="O26" s="210"/>
-      <c r="P26" s="211"/>
+      <c r="O26" s="217"/>
+      <c r="P26" s="218"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -5579,10 +5618,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="251" t="s">
+      <c r="U26" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V26" s="252"/>
+      <c r="V26" s="213"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -5595,10 +5634,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="251" t="s">
+      <c r="AA26" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB26" s="252"/>
+      <c r="AB26" s="213"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -5630,22 +5669,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="278"/>
-      <c r="F27" s="273"/>
-      <c r="G27" s="273"/>
-      <c r="H27" s="273"/>
-      <c r="I27" s="273"/>
-      <c r="J27" s="274"/>
+      <c r="E27" s="246"/>
+      <c r="F27" s="241"/>
+      <c r="G27" s="241"/>
+      <c r="H27" s="241"/>
+      <c r="I27" s="241"/>
+      <c r="J27" s="242"/>
       <c r="K27" s="25" t="s">
         <v>44</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="209" t="s">
+      <c r="N27" s="216" t="s">
         <v>46</v>
       </c>
-      <c r="O27" s="210"/>
-      <c r="P27" s="211"/>
+      <c r="O27" s="217"/>
+      <c r="P27" s="218"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -5655,10 +5694,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="251" t="s">
+      <c r="U27" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V27" s="252"/>
+      <c r="V27" s="213"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -5671,10 +5710,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="251" t="s">
+      <c r="AA27" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB27" s="252"/>
+      <c r="AB27" s="213"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -5706,12 +5745,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="275"/>
-      <c r="F28" s="276"/>
-      <c r="G28" s="276"/>
-      <c r="H28" s="276"/>
-      <c r="I28" s="276"/>
-      <c r="J28" s="277"/>
+      <c r="E28" s="243"/>
+      <c r="F28" s="244"/>
+      <c r="G28" s="244"/>
+      <c r="H28" s="244"/>
+      <c r="I28" s="244"/>
+      <c r="J28" s="245"/>
       <c r="K28" s="52" t="s">
         <v>45</v>
       </c>
@@ -5719,11 +5758,11 @@
         <v>155</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="206" t="s">
+      <c r="N28" s="237" t="s">
         <v>92</v>
       </c>
-      <c r="O28" s="207"/>
-      <c r="P28" s="208"/>
+      <c r="O28" s="238"/>
+      <c r="P28" s="239"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -5733,10 +5772,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="253" t="s">
+      <c r="U28" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="V28" s="254"/>
+      <c r="V28" s="215"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -5749,10 +5788,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="253" t="s">
+      <c r="AA28" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="AB28" s="254"/>
+      <c r="AB28" s="215"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -5829,18 +5868,18 @@
       <c r="S30" s="75" t="s">
         <v>156</v>
       </c>
-      <c r="T30" s="291" t="s">
+      <c r="T30" s="259" t="s">
         <v>157</v>
       </c>
-      <c r="U30" s="291"/>
-      <c r="V30" s="291"/>
-      <c r="W30" s="291"/>
-      <c r="X30" s="291"/>
-      <c r="Y30" s="291"/>
-      <c r="Z30" s="291"/>
-      <c r="AA30" s="291"/>
-      <c r="AB30" s="291"/>
-      <c r="AC30" s="263"/>
+      <c r="U30" s="259"/>
+      <c r="V30" s="259"/>
+      <c r="W30" s="259"/>
+      <c r="X30" s="259"/>
+      <c r="Y30" s="259"/>
+      <c r="Z30" s="259"/>
+      <c r="AA30" s="259"/>
+      <c r="AB30" s="259"/>
+      <c r="AC30" s="227"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B31" s="67" t="s">
@@ -5881,18 +5920,18 @@
       <c r="S31" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="T31" s="212" t="s">
+      <c r="T31" s="190" t="s">
         <v>162</v>
       </c>
-      <c r="U31" s="213"/>
-      <c r="V31" s="213"/>
-      <c r="W31" s="213"/>
-      <c r="X31" s="213"/>
-      <c r="Y31" s="213"/>
-      <c r="Z31" s="213"/>
-      <c r="AA31" s="213"/>
-      <c r="AB31" s="213"/>
-      <c r="AC31" s="214"/>
+      <c r="U31" s="233"/>
+      <c r="V31" s="233"/>
+      <c r="W31" s="233"/>
+      <c r="X31" s="233"/>
+      <c r="Y31" s="233"/>
+      <c r="Z31" s="233"/>
+      <c r="AA31" s="233"/>
+      <c r="AB31" s="233"/>
+      <c r="AC31" s="191"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B32" s="4" t="s">
@@ -5916,18 +5955,18 @@
       <c r="S32" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="T32" s="209" t="s">
+      <c r="T32" s="216" t="s">
         <v>163</v>
       </c>
-      <c r="U32" s="210"/>
-      <c r="V32" s="210"/>
-      <c r="W32" s="210"/>
-      <c r="X32" s="210"/>
-      <c r="Y32" s="210"/>
-      <c r="Z32" s="210"/>
-      <c r="AA32" s="210"/>
-      <c r="AB32" s="210"/>
-      <c r="AC32" s="211"/>
+      <c r="U32" s="217"/>
+      <c r="V32" s="217"/>
+      <c r="W32" s="217"/>
+      <c r="X32" s="217"/>
+      <c r="Y32" s="217"/>
+      <c r="Z32" s="217"/>
+      <c r="AA32" s="217"/>
+      <c r="AB32" s="217"/>
+      <c r="AC32" s="218"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
       <c r="H33" s="84" t="s">
@@ -5963,31 +6002,31 @@
       <c r="S33" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="T33" s="209" t="s">
+      <c r="T33" s="216" t="s">
         <v>164</v>
       </c>
-      <c r="U33" s="210"/>
-      <c r="V33" s="210"/>
-      <c r="W33" s="210"/>
-      <c r="X33" s="210"/>
-      <c r="Y33" s="210"/>
-      <c r="Z33" s="210"/>
-      <c r="AA33" s="210"/>
-      <c r="AB33" s="210"/>
-      <c r="AC33" s="211"/>
+      <c r="U33" s="217"/>
+      <c r="V33" s="217"/>
+      <c r="W33" s="217"/>
+      <c r="X33" s="217"/>
+      <c r="Y33" s="217"/>
+      <c r="Z33" s="217"/>
+      <c r="AA33" s="217"/>
+      <c r="AB33" s="217"/>
+      <c r="AC33" s="218"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B34" s="249" t="s">
+      <c r="B34" s="207" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="247" t="s">
+      <c r="C34" s="205" t="s">
         <v>114</v>
       </c>
-      <c r="D34" s="248"/>
-      <c r="E34" s="247" t="s">
+      <c r="D34" s="206"/>
+      <c r="E34" s="205" t="s">
         <v>115</v>
       </c>
-      <c r="F34" s="248"/>
+      <c r="F34" s="206"/>
       <c r="H34" s="77" t="s">
         <v>65</v>
       </c>
@@ -6013,21 +6052,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="209" t="s">
+      <c r="T34" s="216" t="s">
         <v>165</v>
       </c>
-      <c r="U34" s="210"/>
-      <c r="V34" s="210"/>
-      <c r="W34" s="210"/>
-      <c r="X34" s="210"/>
-      <c r="Y34" s="210"/>
-      <c r="Z34" s="210"/>
-      <c r="AA34" s="210"/>
-      <c r="AB34" s="210"/>
-      <c r="AC34" s="211"/>
+      <c r="U34" s="217"/>
+      <c r="V34" s="217"/>
+      <c r="W34" s="217"/>
+      <c r="X34" s="217"/>
+      <c r="Y34" s="217"/>
+      <c r="Z34" s="217"/>
+      <c r="AA34" s="217"/>
+      <c r="AB34" s="217"/>
+      <c r="AC34" s="218"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B35" s="250"/>
+      <c r="B35" s="208"/>
       <c r="C35" s="64" t="s">
         <v>99</v>
       </c>
@@ -6046,18 +6085,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="209" t="s">
+      <c r="T35" s="216" t="s">
         <v>166</v>
       </c>
-      <c r="U35" s="210"/>
-      <c r="V35" s="210"/>
-      <c r="W35" s="210"/>
-      <c r="X35" s="210"/>
-      <c r="Y35" s="210"/>
-      <c r="Z35" s="210"/>
-      <c r="AA35" s="210"/>
-      <c r="AB35" s="210"/>
-      <c r="AC35" s="211"/>
+      <c r="U35" s="217"/>
+      <c r="V35" s="217"/>
+      <c r="W35" s="217"/>
+      <c r="X35" s="217"/>
+      <c r="Y35" s="217"/>
+      <c r="Z35" s="217"/>
+      <c r="AA35" s="217"/>
+      <c r="AB35" s="217"/>
+      <c r="AC35" s="218"/>
     </row>
     <row r="36" spans="2:29">
       <c r="B36" s="1">
@@ -6081,18 +6120,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="209" t="s">
+      <c r="T36" s="216" t="s">
         <v>167</v>
       </c>
-      <c r="U36" s="210"/>
-      <c r="V36" s="210"/>
-      <c r="W36" s="210"/>
-      <c r="X36" s="210"/>
-      <c r="Y36" s="210"/>
-      <c r="Z36" s="210"/>
-      <c r="AA36" s="210"/>
-      <c r="AB36" s="210"/>
-      <c r="AC36" s="211"/>
+      <c r="U36" s="217"/>
+      <c r="V36" s="217"/>
+      <c r="W36" s="217"/>
+      <c r="X36" s="217"/>
+      <c r="Y36" s="217"/>
+      <c r="Z36" s="217"/>
+      <c r="AA36" s="217"/>
+      <c r="AB36" s="217"/>
+      <c r="AC36" s="218"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1">
       <c r="B37" s="2">
@@ -6117,18 +6156,18 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="209" t="s">
+      <c r="T37" s="216" t="s">
         <v>194</v>
       </c>
-      <c r="U37" s="210"/>
-      <c r="V37" s="210"/>
-      <c r="W37" s="210"/>
-      <c r="X37" s="210"/>
-      <c r="Y37" s="210"/>
-      <c r="Z37" s="210"/>
-      <c r="AA37" s="210"/>
-      <c r="AB37" s="210"/>
-      <c r="AC37" s="211"/>
+      <c r="U37" s="217"/>
+      <c r="V37" s="217"/>
+      <c r="W37" s="217"/>
+      <c r="X37" s="217"/>
+      <c r="Y37" s="217"/>
+      <c r="Z37" s="217"/>
+      <c r="AA37" s="217"/>
+      <c r="AB37" s="217"/>
+      <c r="AC37" s="218"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1">
       <c r="B38" s="2">
@@ -6149,21 +6188,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="292" t="s">
+      <c r="S38" s="260" t="s">
         <v>72</v>
       </c>
-      <c r="T38" s="294" t="s">
+      <c r="T38" s="262" t="s">
         <v>168</v>
       </c>
-      <c r="U38" s="295"/>
-      <c r="V38" s="295"/>
-      <c r="W38" s="295"/>
-      <c r="X38" s="295"/>
-      <c r="Y38" s="295"/>
-      <c r="Z38" s="295"/>
-      <c r="AA38" s="295"/>
-      <c r="AB38" s="295"/>
-      <c r="AC38" s="296"/>
+      <c r="U38" s="263"/>
+      <c r="V38" s="263"/>
+      <c r="W38" s="263"/>
+      <c r="X38" s="263"/>
+      <c r="Y38" s="263"/>
+      <c r="Z38" s="263"/>
+      <c r="AA38" s="263"/>
+      <c r="AB38" s="263"/>
+      <c r="AC38" s="264"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1">
       <c r="B39" s="2">
@@ -6181,26 +6220,26 @@
       <c r="F39" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G39" s="203" t="s">
+      <c r="G39" s="192" t="s">
         <v>181</v>
       </c>
-      <c r="H39" s="204"/>
-      <c r="I39" s="204"/>
-      <c r="J39" s="205"/>
+      <c r="H39" s="193"/>
+      <c r="I39" s="193"/>
+      <c r="J39" s="194"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="293"/>
-      <c r="T39" s="297"/>
-      <c r="U39" s="298"/>
-      <c r="V39" s="298"/>
-      <c r="W39" s="298"/>
-      <c r="X39" s="298"/>
-      <c r="Y39" s="298"/>
-      <c r="Z39" s="298"/>
-      <c r="AA39" s="298"/>
-      <c r="AB39" s="298"/>
-      <c r="AC39" s="299"/>
+      <c r="S39" s="261"/>
+      <c r="T39" s="265"/>
+      <c r="U39" s="266"/>
+      <c r="V39" s="266"/>
+      <c r="W39" s="266"/>
+      <c r="X39" s="266"/>
+      <c r="Y39" s="266"/>
+      <c r="Z39" s="266"/>
+      <c r="AA39" s="266"/>
+      <c r="AB39" s="266"/>
+      <c r="AC39" s="267"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1">
       <c r="B40" s="2">
@@ -6218,28 +6257,28 @@
       <c r="F40" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G40" s="237"/>
-      <c r="H40" s="238"/>
-      <c r="I40" s="238"/>
-      <c r="J40" s="239"/>
+      <c r="G40" s="195"/>
+      <c r="H40" s="196"/>
+      <c r="I40" s="196"/>
+      <c r="J40" s="197"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="209" t="s">
+      <c r="T40" s="216" t="s">
         <v>169</v>
       </c>
-      <c r="U40" s="210"/>
-      <c r="V40" s="210"/>
-      <c r="W40" s="210"/>
-      <c r="X40" s="210"/>
-      <c r="Y40" s="210"/>
-      <c r="Z40" s="210"/>
-      <c r="AA40" s="210"/>
-      <c r="AB40" s="210"/>
-      <c r="AC40" s="211"/>
+      <c r="U40" s="217"/>
+      <c r="V40" s="217"/>
+      <c r="W40" s="217"/>
+      <c r="X40" s="217"/>
+      <c r="Y40" s="217"/>
+      <c r="Z40" s="217"/>
+      <c r="AA40" s="217"/>
+      <c r="AB40" s="217"/>
+      <c r="AC40" s="218"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1">
       <c r="B41" s="2">
@@ -6257,28 +6296,28 @@
       <c r="F41" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G41" s="237"/>
-      <c r="H41" s="238"/>
-      <c r="I41" s="238"/>
-      <c r="J41" s="239"/>
+      <c r="G41" s="195"/>
+      <c r="H41" s="196"/>
+      <c r="I41" s="196"/>
+      <c r="J41" s="197"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="209" t="s">
+      <c r="T41" s="216" t="s">
         <v>170</v>
       </c>
-      <c r="U41" s="210"/>
-      <c r="V41" s="210"/>
-      <c r="W41" s="210"/>
-      <c r="X41" s="210"/>
-      <c r="Y41" s="210"/>
-      <c r="Z41" s="210"/>
-      <c r="AA41" s="210"/>
-      <c r="AB41" s="210"/>
-      <c r="AC41" s="211"/>
+      <c r="U41" s="217"/>
+      <c r="V41" s="217"/>
+      <c r="W41" s="217"/>
+      <c r="X41" s="217"/>
+      <c r="Y41" s="217"/>
+      <c r="Z41" s="217"/>
+      <c r="AA41" s="217"/>
+      <c r="AB41" s="217"/>
+      <c r="AC41" s="218"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
       <c r="B42" s="2">
@@ -6296,28 +6335,28 @@
       <c r="F42" s="76" t="s">
         <v>175</v>
       </c>
-      <c r="G42" s="240"/>
-      <c r="H42" s="241"/>
-      <c r="I42" s="241"/>
-      <c r="J42" s="242"/>
+      <c r="G42" s="198"/>
+      <c r="H42" s="199"/>
+      <c r="I42" s="199"/>
+      <c r="J42" s="200"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T42" s="209" t="s">
+      <c r="T42" s="216" t="s">
         <v>171</v>
       </c>
-      <c r="U42" s="210"/>
-      <c r="V42" s="210"/>
-      <c r="W42" s="210"/>
-      <c r="X42" s="210"/>
-      <c r="Y42" s="210"/>
-      <c r="Z42" s="210"/>
-      <c r="AA42" s="210"/>
-      <c r="AB42" s="210"/>
-      <c r="AC42" s="211"/>
+      <c r="U42" s="217"/>
+      <c r="V42" s="217"/>
+      <c r="W42" s="217"/>
+      <c r="X42" s="217"/>
+      <c r="Y42" s="217"/>
+      <c r="Z42" s="217"/>
+      <c r="AA42" s="217"/>
+      <c r="AB42" s="217"/>
+      <c r="AC42" s="218"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
       <c r="B43" s="2">
@@ -6335,30 +6374,30 @@
       <c r="F43" s="35" t="s">
         <v>146</v>
       </c>
-      <c r="G43" s="218" t="s">
+      <c r="G43" s="183" t="s">
         <v>191</v>
       </c>
-      <c r="H43" s="219"/>
-      <c r="I43" s="219"/>
-      <c r="J43" s="220"/>
+      <c r="H43" s="184"/>
+      <c r="I43" s="184"/>
+      <c r="J43" s="185"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="T43" s="209" t="s">
+      <c r="T43" s="216" t="s">
         <v>172</v>
       </c>
-      <c r="U43" s="210"/>
-      <c r="V43" s="210"/>
-      <c r="W43" s="210"/>
-      <c r="X43" s="210"/>
-      <c r="Y43" s="210"/>
-      <c r="Z43" s="210"/>
-      <c r="AA43" s="210"/>
-      <c r="AB43" s="210"/>
-      <c r="AC43" s="211"/>
+      <c r="U43" s="217"/>
+      <c r="V43" s="217"/>
+      <c r="W43" s="217"/>
+      <c r="X43" s="217"/>
+      <c r="Y43" s="217"/>
+      <c r="Z43" s="217"/>
+      <c r="AA43" s="217"/>
+      <c r="AB43" s="217"/>
+      <c r="AC43" s="218"/>
     </row>
     <row r="44" spans="2:29" ht="15.75" thickBot="1">
       <c r="B44" s="2">
@@ -6379,21 +6418,21 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="292" t="s">
+      <c r="S44" s="260" t="s">
         <v>75</v>
       </c>
-      <c r="T44" s="294" t="s">
+      <c r="T44" s="262" t="s">
         <v>173</v>
       </c>
-      <c r="U44" s="295"/>
-      <c r="V44" s="295"/>
-      <c r="W44" s="295"/>
-      <c r="X44" s="295"/>
-      <c r="Y44" s="295"/>
-      <c r="Z44" s="295"/>
-      <c r="AA44" s="295"/>
-      <c r="AB44" s="295"/>
-      <c r="AC44" s="296"/>
+      <c r="U44" s="263"/>
+      <c r="V44" s="263"/>
+      <c r="W44" s="263"/>
+      <c r="X44" s="263"/>
+      <c r="Y44" s="263"/>
+      <c r="Z44" s="263"/>
+      <c r="AA44" s="263"/>
+      <c r="AB44" s="263"/>
+      <c r="AC44" s="264"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1">
       <c r="B45" s="2">
@@ -6411,26 +6450,26 @@
       <c r="F45" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="G45" s="203" t="s">
+      <c r="G45" s="192" t="s">
         <v>180</v>
       </c>
-      <c r="H45" s="204"/>
-      <c r="I45" s="204"/>
-      <c r="J45" s="205"/>
+      <c r="H45" s="193"/>
+      <c r="I45" s="193"/>
+      <c r="J45" s="194"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="293"/>
-      <c r="T45" s="297"/>
-      <c r="U45" s="298"/>
-      <c r="V45" s="298"/>
-      <c r="W45" s="298"/>
-      <c r="X45" s="298"/>
-      <c r="Y45" s="298"/>
-      <c r="Z45" s="298"/>
-      <c r="AA45" s="298"/>
-      <c r="AB45" s="298"/>
-      <c r="AC45" s="299"/>
+      <c r="S45" s="261"/>
+      <c r="T45" s="265"/>
+      <c r="U45" s="266"/>
+      <c r="V45" s="266"/>
+      <c r="W45" s="266"/>
+      <c r="X45" s="266"/>
+      <c r="Y45" s="266"/>
+      <c r="Z45" s="266"/>
+      <c r="AA45" s="266"/>
+      <c r="AB45" s="266"/>
+      <c r="AC45" s="267"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
       <c r="B46" s="2">
@@ -6448,28 +6487,28 @@
       <c r="F46" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="G46" s="240"/>
-      <c r="H46" s="241"/>
-      <c r="I46" s="241"/>
-      <c r="J46" s="242"/>
+      <c r="G46" s="198"/>
+      <c r="H46" s="199"/>
+      <c r="I46" s="199"/>
+      <c r="J46" s="200"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="T46" s="206" t="s">
+      <c r="T46" s="237" t="s">
         <v>174</v>
       </c>
-      <c r="U46" s="207"/>
-      <c r="V46" s="207"/>
-      <c r="W46" s="207"/>
-      <c r="X46" s="207"/>
-      <c r="Y46" s="207"/>
-      <c r="Z46" s="207"/>
-      <c r="AA46" s="207"/>
-      <c r="AB46" s="207"/>
-      <c r="AC46" s="208"/>
+      <c r="U46" s="238"/>
+      <c r="V46" s="238"/>
+      <c r="W46" s="238"/>
+      <c r="X46" s="238"/>
+      <c r="Y46" s="238"/>
+      <c r="Z46" s="238"/>
+      <c r="AA46" s="238"/>
+      <c r="AB46" s="238"/>
+      <c r="AC46" s="239"/>
     </row>
     <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
       <c r="B47" s="2">
@@ -6487,12 +6526,12 @@
       <c r="F47" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="G47" s="219" t="s">
+      <c r="G47" s="184" t="s">
         <v>151</v>
       </c>
-      <c r="H47" s="219"/>
-      <c r="I47" s="219"/>
-      <c r="J47" s="220"/>
+      <c r="H47" s="184"/>
+      <c r="I47" s="184"/>
+      <c r="J47" s="185"/>
     </row>
     <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
       <c r="B48" s="2">
@@ -6530,12 +6569,12 @@
       <c r="F49" s="35" t="s">
         <v>152</v>
       </c>
-      <c r="G49" s="203" t="s">
+      <c r="G49" s="192" t="s">
         <v>154</v>
       </c>
-      <c r="H49" s="204"/>
-      <c r="I49" s="204"/>
-      <c r="J49" s="205"/>
+      <c r="H49" s="193"/>
+      <c r="I49" s="193"/>
+      <c r="J49" s="194"/>
     </row>
     <row r="50" spans="2:10" ht="30" customHeight="1">
       <c r="B50" s="2">
@@ -6553,10 +6592,10 @@
       <c r="F50" s="35" t="s">
         <v>152</v>
       </c>
-      <c r="G50" s="237"/>
-      <c r="H50" s="238"/>
-      <c r="I50" s="238"/>
-      <c r="J50" s="239"/>
+      <c r="G50" s="195"/>
+      <c r="H50" s="196"/>
+      <c r="I50" s="196"/>
+      <c r="J50" s="197"/>
     </row>
     <row r="51" spans="2:10" ht="32.25" customHeight="1" thickBot="1">
       <c r="B51" s="4">
@@ -6574,38 +6613,38 @@
       <c r="F51" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="G51" s="240"/>
-      <c r="H51" s="241"/>
-      <c r="I51" s="241"/>
-      <c r="J51" s="242"/>
+      <c r="G51" s="198"/>
+      <c r="H51" s="199"/>
+      <c r="I51" s="199"/>
+      <c r="J51" s="200"/>
     </row>
     <row r="52" spans="2:10" ht="30.75" customHeight="1" thickBot="1">
-      <c r="B52" s="221" t="s">
+      <c r="B52" s="209" t="s">
         <v>141</v>
       </c>
-      <c r="C52" s="222"/>
-      <c r="D52" s="222"/>
-      <c r="E52" s="222"/>
-      <c r="F52" s="223"/>
+      <c r="C52" s="210"/>
+      <c r="D52" s="210"/>
+      <c r="E52" s="210"/>
+      <c r="F52" s="211"/>
     </row>
     <row r="53" spans="2:10" ht="31.5" customHeight="1" thickBot="1"/>
     <row r="54" spans="2:10" ht="24.75" customHeight="1">
-      <c r="B54" s="245" t="s">
+      <c r="B54" s="203" t="s">
         <v>182</v>
       </c>
-      <c r="C54" s="243" t="s">
+      <c r="C54" s="201" t="s">
         <v>184</v>
       </c>
-      <c r="D54" s="233" t="s">
+      <c r="D54" s="186" t="s">
         <v>183</v>
       </c>
-      <c r="E54" s="234"/>
+      <c r="E54" s="187"/>
     </row>
     <row r="55" spans="2:10" ht="24" customHeight="1" thickBot="1">
-      <c r="B55" s="246"/>
-      <c r="C55" s="244"/>
-      <c r="D55" s="235"/>
-      <c r="E55" s="236"/>
+      <c r="B55" s="204"/>
+      <c r="C55" s="202"/>
+      <c r="D55" s="188"/>
+      <c r="E55" s="189"/>
     </row>
     <row r="56" spans="2:10" ht="41.25" customHeight="1">
       <c r="B56" s="81">
@@ -6614,10 +6653,10 @@
       <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D56" s="212" t="s">
+      <c r="D56" s="190" t="s">
         <v>206</v>
       </c>
-      <c r="E56" s="214"/>
+      <c r="E56" s="191"/>
     </row>
     <row r="57" spans="2:10" ht="31.5" customHeight="1">
       <c r="B57" s="82">
@@ -6626,10 +6665,10 @@
       <c r="C57" s="86" t="s">
         <v>202</v>
       </c>
-      <c r="D57" s="229" t="s">
+      <c r="D57" s="179" t="s">
         <v>205</v>
       </c>
-      <c r="E57" s="230"/>
+      <c r="E57" s="180"/>
     </row>
     <row r="58" spans="2:10" ht="30.75" customHeight="1">
       <c r="B58" s="82">
@@ -6638,10 +6677,10 @@
       <c r="C58" s="38" t="s">
         <v>203</v>
       </c>
-      <c r="D58" s="229" t="s">
+      <c r="D58" s="179" t="s">
         <v>204</v>
       </c>
-      <c r="E58" s="230"/>
+      <c r="E58" s="180"/>
     </row>
     <row r="59" spans="2:10" ht="33.75" customHeight="1">
       <c r="B59" s="82">
@@ -6650,10 +6689,10 @@
       <c r="C59" s="86" t="s">
         <v>185</v>
       </c>
-      <c r="D59" s="229" t="s">
+      <c r="D59" s="179" t="s">
         <v>188</v>
       </c>
-      <c r="E59" s="230"/>
+      <c r="E59" s="180"/>
     </row>
     <row r="60" spans="2:10" ht="28.5" customHeight="1">
       <c r="B60" s="82">
@@ -6662,10 +6701,10 @@
       <c r="C60" s="38" t="s">
         <v>186</v>
       </c>
-      <c r="D60" s="229" t="s">
+      <c r="D60" s="179" t="s">
         <v>189</v>
       </c>
-      <c r="E60" s="230"/>
+      <c r="E60" s="180"/>
     </row>
     <row r="61" spans="2:10" ht="40.5" customHeight="1">
       <c r="B61" s="82">
@@ -6674,10 +6713,10 @@
       <c r="C61" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="D61" s="229" t="s">
+      <c r="D61" s="179" t="s">
         <v>190</v>
       </c>
-      <c r="E61" s="230"/>
+      <c r="E61" s="180"/>
     </row>
     <row r="62" spans="2:10" ht="53.25" customHeight="1">
       <c r="B62" s="82">
@@ -6686,82 +6725,82 @@
       <c r="C62" s="86" t="s">
         <v>195</v>
       </c>
-      <c r="D62" s="229" t="s">
+      <c r="D62" s="179" t="s">
         <v>196</v>
       </c>
-      <c r="E62" s="230"/>
+      <c r="E62" s="180"/>
     </row>
     <row r="63" spans="2:10" ht="36" customHeight="1">
       <c r="B63" s="82">
         <v>7</v>
       </c>
       <c r="C63" s="86"/>
-      <c r="D63" s="229"/>
-      <c r="E63" s="230"/>
+      <c r="D63" s="179"/>
+      <c r="E63" s="180"/>
     </row>
     <row r="64" spans="2:10" ht="40.5" customHeight="1">
       <c r="B64" s="82">
         <v>8</v>
       </c>
       <c r="C64" s="86"/>
-      <c r="D64" s="229"/>
-      <c r="E64" s="230"/>
+      <c r="D64" s="179"/>
+      <c r="E64" s="180"/>
     </row>
     <row r="65" spans="2:5">
       <c r="B65" s="82">
         <v>9</v>
       </c>
       <c r="C65" s="86"/>
-      <c r="D65" s="229"/>
-      <c r="E65" s="230"/>
+      <c r="D65" s="179"/>
+      <c r="E65" s="180"/>
     </row>
     <row r="66" spans="2:5" ht="30" customHeight="1">
       <c r="B66" s="82">
         <v>10</v>
       </c>
       <c r="C66" s="86"/>
-      <c r="D66" s="229"/>
-      <c r="E66" s="230"/>
+      <c r="D66" s="179"/>
+      <c r="E66" s="180"/>
     </row>
     <row r="67" spans="2:5">
       <c r="B67" s="82">
         <v>11</v>
       </c>
       <c r="C67" s="86"/>
-      <c r="D67" s="229"/>
-      <c r="E67" s="230"/>
+      <c r="D67" s="179"/>
+      <c r="E67" s="180"/>
     </row>
     <row r="68" spans="2:5">
       <c r="B68" s="82">
         <v>12</v>
       </c>
       <c r="C68" s="86"/>
-      <c r="D68" s="229"/>
-      <c r="E68" s="230"/>
+      <c r="D68" s="179"/>
+      <c r="E68" s="180"/>
     </row>
     <row r="69" spans="2:5">
       <c r="B69" s="82">
         <v>13</v>
       </c>
       <c r="C69" s="86"/>
-      <c r="D69" s="229"/>
-      <c r="E69" s="230"/>
+      <c r="D69" s="179"/>
+      <c r="E69" s="180"/>
     </row>
     <row r="70" spans="2:5" ht="30" customHeight="1">
       <c r="B70" s="82">
         <v>14</v>
       </c>
       <c r="C70" s="86"/>
-      <c r="D70" s="229"/>
-      <c r="E70" s="230"/>
+      <c r="D70" s="179"/>
+      <c r="E70" s="180"/>
     </row>
     <row r="71" spans="2:5" ht="15.75" thickBot="1">
       <c r="B71" s="83">
         <v>15</v>
       </c>
       <c r="C71" s="87"/>
-      <c r="D71" s="231"/>
-      <c r="E71" s="232"/>
+      <c r="D71" s="181"/>
+      <c r="E71" s="182"/>
     </row>
     <row r="75" spans="2:5" ht="72" customHeight="1"/>
   </sheetData>
@@ -6977,35 +7016,35 @@
       <c r="F2" s="103" t="s">
         <v>211</v>
       </c>
-      <c r="G2" s="203" t="s">
+      <c r="G2" s="192" t="s">
         <v>212</v>
       </c>
-      <c r="H2" s="204"/>
-      <c r="I2" s="204"/>
-      <c r="J2" s="205"/>
-      <c r="L2" s="194" t="s">
+      <c r="H2" s="193"/>
+      <c r="I2" s="193"/>
+      <c r="J2" s="194"/>
+      <c r="L2" s="284" t="s">
         <v>331</v>
       </c>
-      <c r="M2" s="195"/>
-      <c r="N2" s="195"/>
-      <c r="O2" s="196"/>
+      <c r="M2" s="285"/>
+      <c r="N2" s="285"/>
+      <c r="O2" s="286"/>
       <c r="P2" s="133"/>
-      <c r="Q2" s="197" t="s">
+      <c r="Q2" s="287" t="s">
         <v>291</v>
       </c>
-      <c r="R2" s="198"/>
-      <c r="S2" s="198"/>
-      <c r="T2" s="199"/>
+      <c r="R2" s="288"/>
+      <c r="S2" s="288"/>
+      <c r="T2" s="289"/>
       <c r="U2" s="133"/>
-      <c r="V2" s="187" t="s">
+      <c r="V2" s="277" t="s">
         <v>314</v>
       </c>
-      <c r="W2" s="188"/>
-      <c r="X2" s="188"/>
-      <c r="Y2" s="188"/>
-      <c r="Z2" s="188"/>
-      <c r="AA2" s="188"/>
-      <c r="AB2" s="189"/>
+      <c r="W2" s="278"/>
+      <c r="X2" s="278"/>
+      <c r="Y2" s="278"/>
+      <c r="Z2" s="278"/>
+      <c r="AA2" s="278"/>
+      <c r="AB2" s="279"/>
     </row>
     <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B3" s="90" t="s">
@@ -7027,11 +7066,11 @@
       <c r="G3" s="93" t="s">
         <v>213</v>
       </c>
-      <c r="H3" s="212" t="s">
+      <c r="H3" s="190" t="s">
         <v>217</v>
       </c>
-      <c r="I3" s="213"/>
-      <c r="J3" s="214"/>
+      <c r="I3" s="233"/>
+      <c r="J3" s="191"/>
       <c r="L3" s="145" t="s">
         <v>277</v>
       </c>
@@ -7070,11 +7109,11 @@
       <c r="Y3" s="171" t="s">
         <v>280</v>
       </c>
-      <c r="Z3" s="178" t="s">
+      <c r="Z3" s="268" t="s">
         <v>319</v>
       </c>
-      <c r="AA3" s="179"/>
-      <c r="AB3" s="180"/>
+      <c r="AA3" s="269"/>
+      <c r="AB3" s="270"/>
     </row>
     <row r="4" spans="2:28" ht="53.25" customHeight="1">
       <c r="B4" s="91" t="s">
@@ -7096,11 +7135,11 @@
       <c r="G4" s="94" t="s">
         <v>214</v>
       </c>
-      <c r="H4" s="209">
+      <c r="H4" s="216">
         <v>63</v>
       </c>
-      <c r="I4" s="210"/>
-      <c r="J4" s="211"/>
+      <c r="I4" s="217"/>
+      <c r="J4" s="218"/>
       <c r="L4" s="151" t="s">
         <v>246</v>
       </c>
@@ -7139,11 +7178,11 @@
       <c r="Y4" s="138" t="s">
         <v>317</v>
       </c>
-      <c r="Z4" s="181" t="s">
+      <c r="Z4" s="271" t="s">
         <v>320</v>
       </c>
-      <c r="AA4" s="182"/>
-      <c r="AB4" s="183"/>
+      <c r="AA4" s="272"/>
+      <c r="AB4" s="273"/>
     </row>
     <row r="5" spans="2:28" ht="47.25" customHeight="1">
       <c r="B5" s="91" t="s">
@@ -7165,11 +7204,11 @@
       <c r="G5" s="94" t="s">
         <v>215</v>
       </c>
-      <c r="H5" s="209">
+      <c r="H5" s="216">
         <v>31</v>
       </c>
-      <c r="I5" s="210"/>
-      <c r="J5" s="211"/>
+      <c r="I5" s="217"/>
+      <c r="J5" s="218"/>
       <c r="L5" s="149" t="s">
         <v>255</v>
       </c>
@@ -7208,9 +7247,9 @@
       <c r="Y5" s="135" t="s">
         <v>294</v>
       </c>
-      <c r="Z5" s="181"/>
-      <c r="AA5" s="182"/>
-      <c r="AB5" s="183"/>
+      <c r="Z5" s="271"/>
+      <c r="AA5" s="272"/>
+      <c r="AB5" s="273"/>
     </row>
     <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B6" s="108" t="s">
@@ -7232,11 +7271,11 @@
       <c r="G6" s="95" t="s">
         <v>216</v>
       </c>
-      <c r="H6" s="206">
+      <c r="H6" s="237">
         <v>7</v>
       </c>
-      <c r="I6" s="207"/>
-      <c r="J6" s="208"/>
+      <c r="I6" s="238"/>
+      <c r="J6" s="239"/>
       <c r="L6" s="152" t="s">
         <v>241</v>
       </c>
@@ -7275,9 +7314,9 @@
       <c r="Y6" s="144" t="s">
         <v>316</v>
       </c>
-      <c r="Z6" s="184"/>
-      <c r="AA6" s="185"/>
-      <c r="AB6" s="186"/>
+      <c r="Z6" s="274"/>
+      <c r="AA6" s="275"/>
+      <c r="AB6" s="276"/>
     </row>
     <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1">
       <c r="B7" s="90" t="s">
@@ -7299,12 +7338,12 @@
       <c r="G7" s="88" t="s">
         <v>274</v>
       </c>
-      <c r="H7" s="200" t="str">
+      <c r="H7" s="290" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12))</f>
         <v>E3FFF000</v>
       </c>
-      <c r="I7" s="201"/>
-      <c r="J7" s="202"/>
+      <c r="I7" s="291"/>
+      <c r="J7" s="292"/>
       <c r="L7" s="150" t="s">
         <v>266</v>
       </c>
@@ -7352,18 +7391,18 @@
       <c r="G8" s="88" t="s">
         <v>218</v>
       </c>
-      <c r="H8" s="200" t="str">
+      <c r="H8" s="290" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12)+4095)</f>
         <v>E3FFFFFF</v>
       </c>
-      <c r="I8" s="201"/>
-      <c r="J8" s="202"/>
-      <c r="L8" s="218" t="s">
+      <c r="I8" s="291"/>
+      <c r="J8" s="292"/>
+      <c r="L8" s="183" t="s">
         <v>333</v>
       </c>
-      <c r="M8" s="219"/>
-      <c r="N8" s="219"/>
-      <c r="O8" s="220"/>
+      <c r="M8" s="184"/>
+      <c r="N8" s="184"/>
+      <c r="O8" s="185"/>
       <c r="P8" s="133"/>
       <c r="Q8" s="164" t="s">
         <v>286</v>
@@ -7472,12 +7511,12 @@
       <c r="N11" s="133"/>
       <c r="O11" s="133"/>
       <c r="P11" s="133"/>
-      <c r="Q11" s="215" t="s">
+      <c r="Q11" s="293" t="s">
         <v>313</v>
       </c>
-      <c r="R11" s="216"/>
-      <c r="S11" s="216"/>
-      <c r="T11" s="217"/>
+      <c r="R11" s="294"/>
+      <c r="S11" s="294"/>
+      <c r="T11" s="295"/>
       <c r="U11" s="133"/>
     </row>
     <row r="12" spans="2:28" ht="44.25" customHeight="1" thickBot="1">
@@ -7629,12 +7668,12 @@
       <c r="F16" s="124" t="s">
         <v>233</v>
       </c>
-      <c r="G16" s="221" t="s">
+      <c r="G16" s="209" t="s">
         <v>271</v>
       </c>
-      <c r="H16" s="222"/>
-      <c r="I16" s="222"/>
-      <c r="J16" s="223"/>
+      <c r="H16" s="210"/>
+      <c r="I16" s="210"/>
+      <c r="J16" s="211"/>
       <c r="Q16" s="167" t="s">
         <v>307</v>
       </c>
@@ -7649,10 +7688,10 @@
       </c>
     </row>
     <row r="17" spans="2:20" ht="60.75" customHeight="1" thickBot="1">
-      <c r="B17" s="192" t="s">
+      <c r="B17" s="282" t="s">
         <v>234</v>
       </c>
-      <c r="C17" s="190" t="s">
+      <c r="C17" s="280" t="s">
         <v>235</v>
       </c>
       <c r="D17" s="125" t="s">
@@ -7664,12 +7703,12 @@
       <c r="F17" s="127" t="s">
         <v>237</v>
       </c>
-      <c r="G17" s="224" t="s">
+      <c r="G17" s="296" t="s">
         <v>272</v>
       </c>
-      <c r="H17" s="225"/>
-      <c r="I17" s="225"/>
-      <c r="J17" s="226"/>
+      <c r="H17" s="297"/>
+      <c r="I17" s="297"/>
+      <c r="J17" s="298"/>
       <c r="Q17" s="168" t="s">
         <v>310</v>
       </c>
@@ -7684,8 +7723,8 @@
       </c>
     </row>
     <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B18" s="227"/>
-      <c r="C18" s="228"/>
+      <c r="B18" s="299"/>
+      <c r="C18" s="300"/>
       <c r="D18" s="112" t="s">
         <v>238</v>
       </c>
@@ -7695,16 +7734,16 @@
       <c r="F18" s="115" t="s">
         <v>240</v>
       </c>
-      <c r="G18" s="200" t="s">
+      <c r="G18" s="290" t="s">
         <v>273</v>
       </c>
-      <c r="H18" s="201"/>
-      <c r="I18" s="201"/>
-      <c r="J18" s="202"/>
+      <c r="H18" s="291"/>
+      <c r="I18" s="291"/>
+      <c r="J18" s="292"/>
     </row>
     <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B19" s="193"/>
-      <c r="C19" s="191"/>
+      <c r="B19" s="283"/>
+      <c r="C19" s="281"/>
       <c r="D19" s="117" t="s">
         <v>241</v>
       </c>
@@ -7720,10 +7759,10 @@
       <c r="J19" s="15"/>
     </row>
     <row r="20" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B20" s="192" t="s">
+      <c r="B20" s="282" t="s">
         <v>244</v>
       </c>
-      <c r="C20" s="190" t="s">
+      <c r="C20" s="280" t="s">
         <v>245</v>
       </c>
       <c r="D20" s="125" t="s">
@@ -7741,8 +7780,8 @@
       <c r="J20" s="15"/>
     </row>
     <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B21" s="193"/>
-      <c r="C21" s="191"/>
+      <c r="B21" s="283"/>
+      <c r="C21" s="281"/>
       <c r="D21" s="117" t="s">
         <v>248</v>
       </c>
@@ -7758,10 +7797,10 @@
       <c r="J21" s="15"/>
     </row>
     <row r="22" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B22" s="192" t="s">
+      <c r="B22" s="282" t="s">
         <v>250</v>
       </c>
-      <c r="C22" s="190" t="s">
+      <c r="C22" s="280" t="s">
         <v>251</v>
       </c>
       <c r="D22" s="125" t="s">
@@ -7779,8 +7818,8 @@
       <c r="J22" s="15"/>
     </row>
     <row r="23" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B23" s="193"/>
-      <c r="C23" s="191"/>
+      <c r="B23" s="283"/>
+      <c r="C23" s="281"/>
       <c r="D23" s="117" t="s">
         <v>244</v>
       </c>
@@ -7796,10 +7835,10 @@
       <c r="J23" s="15"/>
     </row>
     <row r="24" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B24" s="192" t="s">
+      <c r="B24" s="282" t="s">
         <v>255</v>
       </c>
-      <c r="C24" s="190" t="s">
+      <c r="C24" s="280" t="s">
         <v>256</v>
       </c>
       <c r="D24" s="125" t="s">
@@ -7817,8 +7856,8 @@
       <c r="J24" s="15"/>
     </row>
     <row r="25" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B25" s="193"/>
-      <c r="C25" s="191"/>
+      <c r="B25" s="283"/>
+      <c r="C25" s="281"/>
       <c r="D25" s="117" t="s">
         <v>250</v>
       </c>
@@ -7855,10 +7894,10 @@
       <c r="J26" s="15"/>
     </row>
     <row r="27" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B27" s="192" t="s">
+      <c r="B27" s="282" t="s">
         <v>238</v>
       </c>
-      <c r="C27" s="190" t="s">
+      <c r="C27" s="280" t="s">
         <v>262</v>
       </c>
       <c r="D27" s="125" t="s">
@@ -7876,8 +7915,8 @@
       <c r="J27" s="15"/>
     </row>
     <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B28" s="193"/>
-      <c r="C28" s="191"/>
+      <c r="B28" s="283"/>
+      <c r="C28" s="281"/>
       <c r="D28" s="117" t="s">
         <v>255</v>
       </c>
@@ -7893,10 +7932,10 @@
       <c r="J28" s="15"/>
     </row>
     <row r="29" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B29" s="192" t="s">
+      <c r="B29" s="282" t="s">
         <v>266</v>
       </c>
-      <c r="C29" s="190" t="s">
+      <c r="C29" s="280" t="s">
         <v>267</v>
       </c>
       <c r="D29" s="125" t="s">
@@ -7914,8 +7953,8 @@
       <c r="J29" s="15"/>
     </row>
     <row r="30" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B30" s="193"/>
-      <c r="C30" s="191"/>
+      <c r="B30" s="283"/>
+      <c r="C30" s="281"/>
       <c r="D30" s="117" t="s">
         <v>259</v>
       </c>

</xml_diff>

<commit_message>
Se corrigio un bug que hacia que STR guarde datos
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A228B2A4-A3F3-4C34-BE5A-7A2D2332094A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B41B6A3-20E6-4C62-B18F-6B7CADE52CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2946,12 +2946,252 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2961,12 +3201,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2979,239 +3213,41 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3249,18 +3285,6 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3279,15 +3303,6 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3296,21 +3311,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3624,62 +3624,62 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B2" s="234" t="s">
+      <c r="B2" s="224" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="249" t="s">
+      <c r="C2" s="233" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="250"/>
-      <c r="E2" s="251" t="s">
+      <c r="D2" s="234"/>
+      <c r="E2" s="235" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="251"/>
-      <c r="G2" s="252" t="s">
+      <c r="F2" s="235"/>
+      <c r="G2" s="236" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="251"/>
-      <c r="I2" s="251" t="s">
+      <c r="H2" s="235"/>
+      <c r="I2" s="235" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="251"/>
-      <c r="K2" s="253" t="s">
+      <c r="J2" s="235"/>
+      <c r="K2" s="237" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="251"/>
-      <c r="M2" s="251"/>
-      <c r="N2" s="251"/>
-      <c r="O2" s="251"/>
-      <c r="P2" s="254"/>
-      <c r="R2" s="230" t="s">
+      <c r="L2" s="235"/>
+      <c r="M2" s="235"/>
+      <c r="N2" s="235"/>
+      <c r="O2" s="235"/>
+      <c r="P2" s="238"/>
+      <c r="R2" s="243" t="s">
         <v>65</v>
       </c>
-      <c r="S2" s="227" t="s">
+      <c r="S2" s="180" t="s">
         <v>66</v>
       </c>
-      <c r="T2" s="220" t="s">
+      <c r="T2" s="247" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="221"/>
-      <c r="V2" s="221"/>
-      <c r="W2" s="221"/>
-      <c r="X2" s="221"/>
-      <c r="Y2" s="221"/>
-      <c r="Z2" s="221"/>
-      <c r="AA2" s="221"/>
-      <c r="AB2" s="221" t="s">
+      <c r="U2" s="248"/>
+      <c r="V2" s="248"/>
+      <c r="W2" s="248"/>
+      <c r="X2" s="248"/>
+      <c r="Y2" s="248"/>
+      <c r="Z2" s="248"/>
+      <c r="AA2" s="248"/>
+      <c r="AB2" s="248" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="221"/>
-      <c r="AD2" s="221"/>
-      <c r="AE2" s="221"/>
-      <c r="AF2" s="221"/>
-      <c r="AG2" s="221"/>
-      <c r="AH2" s="221"/>
-      <c r="AI2" s="222"/>
+      <c r="AC2" s="248"/>
+      <c r="AD2" s="248"/>
+      <c r="AE2" s="248"/>
+      <c r="AF2" s="248"/>
+      <c r="AG2" s="248"/>
+      <c r="AH2" s="248"/>
+      <c r="AI2" s="249"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B3" s="235"/>
+      <c r="B3" s="225"/>
       <c r="C3" s="16" t="s">
         <v>79</v>
       </c>
@@ -3704,21 +3704,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="205"/>
-      <c r="L3" s="248"/>
-      <c r="M3" s="248"/>
-      <c r="N3" s="248"/>
-      <c r="O3" s="248"/>
-      <c r="P3" s="206"/>
-      <c r="R3" s="231"/>
-      <c r="S3" s="228"/>
+      <c r="K3" s="230"/>
+      <c r="L3" s="231"/>
+      <c r="M3" s="231"/>
+      <c r="N3" s="231"/>
+      <c r="O3" s="231"/>
+      <c r="P3" s="232"/>
+      <c r="R3" s="244"/>
+      <c r="S3" s="241"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="258" t="s">
+      <c r="U3" s="211" t="s">
         <v>83</v>
       </c>
-      <c r="V3" s="258"/>
+      <c r="V3" s="211"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -3731,10 +3731,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="219" t="s">
+      <c r="AA3" s="246" t="s">
         <v>74</v>
       </c>
-      <c r="AB3" s="219"/>
+      <c r="AB3" s="246"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -3758,21 +3758,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B4" s="236"/>
+      <c r="B4" s="226"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="223" t="s">
+      <c r="E4" s="212" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="210"/>
-      <c r="G4" s="210"/>
-      <c r="H4" s="210"/>
-      <c r="I4" s="210"/>
-      <c r="J4" s="211"/>
+      <c r="F4" s="239"/>
+      <c r="G4" s="239"/>
+      <c r="H4" s="239"/>
+      <c r="I4" s="239"/>
+      <c r="J4" s="240"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -3782,20 +3782,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="223" t="s">
+      <c r="N4" s="212" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="210"/>
-      <c r="P4" s="211"/>
-      <c r="R4" s="232"/>
-      <c r="S4" s="229"/>
+      <c r="O4" s="239"/>
+      <c r="P4" s="240"/>
+      <c r="R4" s="245"/>
+      <c r="S4" s="242"/>
       <c r="T4" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="U4" s="223" t="s">
+      <c r="U4" s="212" t="s">
         <v>75</v>
       </c>
-      <c r="V4" s="224"/>
+      <c r="V4" s="213"/>
       <c r="W4" s="7" t="s">
         <v>71</v>
       </c>
@@ -3808,10 +3808,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="223" t="s">
+      <c r="AA4" s="212" t="s">
         <v>72</v>
       </c>
-      <c r="AB4" s="224"/>
+      <c r="AB4" s="213"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -3843,22 +3843,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="255"/>
-      <c r="F5" s="256"/>
-      <c r="G5" s="256"/>
-      <c r="H5" s="256"/>
-      <c r="I5" s="256"/>
-      <c r="J5" s="257"/>
+      <c r="E5" s="216"/>
+      <c r="F5" s="217"/>
+      <c r="G5" s="217"/>
+      <c r="H5" s="217"/>
+      <c r="I5" s="217"/>
+      <c r="J5" s="218"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="190" t="s">
+      <c r="N5" s="181" t="s">
         <v>51</v>
       </c>
-      <c r="O5" s="233"/>
-      <c r="P5" s="191"/>
+      <c r="O5" s="182"/>
+      <c r="P5" s="183"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -3868,10 +3868,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="225" t="s">
+      <c r="U5" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="V5" s="226"/>
+      <c r="V5" s="215"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -3884,10 +3884,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="225" t="s">
+      <c r="AA5" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="AB5" s="226"/>
+      <c r="AB5" s="215"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -3919,12 +3919,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="246"/>
-      <c r="F6" s="241"/>
-      <c r="G6" s="241"/>
-      <c r="H6" s="241"/>
-      <c r="I6" s="241"/>
-      <c r="J6" s="242"/>
+      <c r="E6" s="223"/>
+      <c r="F6" s="220"/>
+      <c r="G6" s="220"/>
+      <c r="H6" s="220"/>
+      <c r="I6" s="220"/>
+      <c r="J6" s="221"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -3932,11 +3932,11 @@
         <v>155</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="216" t="s">
+      <c r="N6" s="184" t="s">
         <v>95</v>
       </c>
-      <c r="O6" s="217"/>
-      <c r="P6" s="218"/>
+      <c r="O6" s="185"/>
+      <c r="P6" s="186"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -3946,10 +3946,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="212" t="s">
+      <c r="U6" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V6" s="213"/>
+      <c r="V6" s="210"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -3962,10 +3962,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="212" t="s">
+      <c r="AA6" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB6" s="213"/>
+      <c r="AB6" s="210"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -4008,9 +4008,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="240"/>
-      <c r="I7" s="241"/>
-      <c r="J7" s="242"/>
+      <c r="H7" s="219"/>
+      <c r="I7" s="220"/>
+      <c r="J7" s="221"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -4018,11 +4018,11 @@
       <c r="M7" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N7" s="216" t="s">
+      <c r="N7" s="184" t="s">
         <v>52</v>
       </c>
-      <c r="O7" s="217"/>
-      <c r="P7" s="218"/>
+      <c r="O7" s="185"/>
+      <c r="P7" s="186"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -4032,10 +4032,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="212" t="s">
+      <c r="U7" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V7" s="213"/>
+      <c r="V7" s="210"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -4048,10 +4048,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="212" t="s">
+      <c r="AA7" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB7" s="213"/>
+      <c r="AB7" s="210"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -4094,9 +4094,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="240"/>
-      <c r="I8" s="241"/>
-      <c r="J8" s="242"/>
+      <c r="H8" s="219"/>
+      <c r="I8" s="220"/>
+      <c r="J8" s="221"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -4104,11 +4104,11 @@
       <c r="M8" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N8" s="216" t="s">
+      <c r="N8" s="184" t="s">
         <v>53</v>
       </c>
-      <c r="O8" s="217"/>
-      <c r="P8" s="218"/>
+      <c r="O8" s="185"/>
+      <c r="P8" s="186"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -4118,10 +4118,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="212" t="s">
+      <c r="U8" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V8" s="213"/>
+      <c r="V8" s="210"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -4134,10 +4134,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="212" t="s">
+      <c r="AA8" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB8" s="213"/>
+      <c r="AB8" s="210"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -4180,9 +4180,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="240"/>
-      <c r="I9" s="241"/>
-      <c r="J9" s="242"/>
+      <c r="H9" s="219"/>
+      <c r="I9" s="220"/>
+      <c r="J9" s="221"/>
       <c r="K9" s="37" t="s">
         <v>47</v>
       </c>
@@ -4190,11 +4190,11 @@
       <c r="M9" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N9" s="216" t="s">
+      <c r="N9" s="184" t="s">
         <v>54</v>
       </c>
-      <c r="O9" s="217"/>
-      <c r="P9" s="218"/>
+      <c r="O9" s="185"/>
+      <c r="P9" s="186"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -4204,10 +4204,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="212" t="s">
+      <c r="U9" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V9" s="213"/>
+      <c r="V9" s="210"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -4220,10 +4220,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="212" t="s">
+      <c r="AA9" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB9" s="213"/>
+      <c r="AB9" s="210"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -4266,9 +4266,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="240"/>
-      <c r="I10" s="241"/>
-      <c r="J10" s="242"/>
+      <c r="H10" s="219"/>
+      <c r="I10" s="220"/>
+      <c r="J10" s="221"/>
       <c r="K10" s="37" t="s">
         <v>48</v>
       </c>
@@ -4276,11 +4276,11 @@
       <c r="M10" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N10" s="216" t="s">
+      <c r="N10" s="184" t="s">
         <v>55</v>
       </c>
-      <c r="O10" s="217"/>
-      <c r="P10" s="218"/>
+      <c r="O10" s="185"/>
+      <c r="P10" s="186"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -4290,10 +4290,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="212" t="s">
+      <c r="U10" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V10" s="213"/>
+      <c r="V10" s="210"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -4306,10 +4306,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="212" t="s">
+      <c r="AA10" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB10" s="213"/>
+      <c r="AB10" s="210"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -4352,9 +4352,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="240"/>
-      <c r="I11" s="241"/>
-      <c r="J11" s="242"/>
+      <c r="H11" s="219"/>
+      <c r="I11" s="220"/>
+      <c r="J11" s="221"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -4362,11 +4362,11 @@
       <c r="M11" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N11" s="216" t="s">
+      <c r="N11" s="184" t="s">
         <v>56</v>
       </c>
-      <c r="O11" s="217"/>
-      <c r="P11" s="218"/>
+      <c r="O11" s="185"/>
+      <c r="P11" s="186"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -4376,10 +4376,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="212" t="s">
+      <c r="U11" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V11" s="213"/>
+      <c r="V11" s="210"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -4392,10 +4392,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="212" t="s">
+      <c r="AA11" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB11" s="213"/>
+      <c r="AB11" s="210"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -4438,9 +4438,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="240"/>
-      <c r="I12" s="241"/>
-      <c r="J12" s="242"/>
+      <c r="H12" s="219"/>
+      <c r="I12" s="220"/>
+      <c r="J12" s="221"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -4448,11 +4448,11 @@
       <c r="M12" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N12" s="216" t="s">
+      <c r="N12" s="184" t="s">
         <v>57</v>
       </c>
-      <c r="O12" s="217"/>
-      <c r="P12" s="218"/>
+      <c r="O12" s="185"/>
+      <c r="P12" s="186"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -4462,10 +4462,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="212" t="s">
+      <c r="U12" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V12" s="213"/>
+      <c r="V12" s="210"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -4478,10 +4478,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="212" t="s">
+      <c r="AA12" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB12" s="213"/>
+      <c r="AB12" s="210"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -4524,9 +4524,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="240"/>
-      <c r="I13" s="241"/>
-      <c r="J13" s="242"/>
+      <c r="H13" s="219"/>
+      <c r="I13" s="220"/>
+      <c r="J13" s="221"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -4534,11 +4534,11 @@
       <c r="M13" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N13" s="216" t="s">
+      <c r="N13" s="184" t="s">
         <v>58</v>
       </c>
-      <c r="O13" s="217"/>
-      <c r="P13" s="218"/>
+      <c r="O13" s="185"/>
+      <c r="P13" s="186"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -4548,10 +4548,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="212" t="s">
+      <c r="U13" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V13" s="213"/>
+      <c r="V13" s="210"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -4564,10 +4564,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="212" t="s">
+      <c r="AA13" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB13" s="213"/>
+      <c r="AB13" s="210"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -4610,9 +4610,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="240"/>
-      <c r="I14" s="241"/>
-      <c r="J14" s="242"/>
+      <c r="H14" s="219"/>
+      <c r="I14" s="220"/>
+      <c r="J14" s="221"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -4620,11 +4620,11 @@
       <c r="M14" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N14" s="216" t="s">
+      <c r="N14" s="184" t="s">
         <v>59</v>
       </c>
-      <c r="O14" s="217"/>
-      <c r="P14" s="218"/>
+      <c r="O14" s="185"/>
+      <c r="P14" s="186"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -4634,10 +4634,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="212" t="s">
+      <c r="U14" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V14" s="213"/>
+      <c r="V14" s="210"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -4650,10 +4650,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="212" t="s">
+      <c r="AA14" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB14" s="213"/>
+      <c r="AB14" s="210"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -4696,9 +4696,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="240"/>
-      <c r="I15" s="241"/>
-      <c r="J15" s="242"/>
+      <c r="H15" s="219"/>
+      <c r="I15" s="220"/>
+      <c r="J15" s="221"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -4706,11 +4706,11 @@
       <c r="M15" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N15" s="216" t="s">
+      <c r="N15" s="184" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="217"/>
-      <c r="P15" s="218"/>
+      <c r="O15" s="185"/>
+      <c r="P15" s="186"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -4720,10 +4720,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="212" t="s">
+      <c r="U15" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V15" s="213"/>
+      <c r="V15" s="210"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -4736,10 +4736,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="212" t="s">
+      <c r="AA15" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB15" s="213"/>
+      <c r="AB15" s="210"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -4776,21 +4776,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="240"/>
-      <c r="G16" s="241"/>
-      <c r="H16" s="241"/>
-      <c r="I16" s="241"/>
-      <c r="J16" s="242"/>
+      <c r="F16" s="219"/>
+      <c r="G16" s="220"/>
+      <c r="H16" s="220"/>
+      <c r="I16" s="220"/>
+      <c r="J16" s="221"/>
       <c r="K16" s="40" t="s">
         <v>49</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="216" t="s">
+      <c r="N16" s="184" t="s">
         <v>50</v>
       </c>
-      <c r="O16" s="217"/>
-      <c r="P16" s="218"/>
+      <c r="O16" s="185"/>
+      <c r="P16" s="186"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -4800,10 +4800,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="212" t="s">
+      <c r="U16" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V16" s="213"/>
+      <c r="V16" s="210"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -4816,10 +4816,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="212" t="s">
+      <c r="AA16" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB16" s="213"/>
+      <c r="AB16" s="210"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -4857,22 +4857,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="247" t="s">
+      <c r="G17" s="222" t="s">
         <v>76</v>
       </c>
-      <c r="H17" s="217"/>
-      <c r="I17" s="217"/>
-      <c r="J17" s="218"/>
+      <c r="H17" s="185"/>
+      <c r="I17" s="185"/>
+      <c r="J17" s="186"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="216" t="s">
+      <c r="N17" s="184" t="s">
         <v>64</v>
       </c>
-      <c r="O17" s="217"/>
-      <c r="P17" s="218"/>
+      <c r="O17" s="185"/>
+      <c r="P17" s="186"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -4882,10 +4882,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="212" t="s">
+      <c r="U17" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V17" s="213"/>
+      <c r="V17" s="210"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -4898,10 +4898,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="212" t="s">
+      <c r="AA17" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB17" s="213"/>
+      <c r="AB17" s="210"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -4939,12 +4939,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="247" t="s">
+      <c r="G18" s="222" t="s">
         <v>76</v>
       </c>
-      <c r="H18" s="217"/>
-      <c r="I18" s="217"/>
-      <c r="J18" s="218"/>
+      <c r="H18" s="185"/>
+      <c r="I18" s="185"/>
+      <c r="J18" s="186"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -4952,11 +4952,11 @@
       <c r="M18" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N18" s="216" t="s">
+      <c r="N18" s="184" t="s">
         <v>61</v>
       </c>
-      <c r="O18" s="217"/>
-      <c r="P18" s="218"/>
+      <c r="O18" s="185"/>
+      <c r="P18" s="186"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -4966,10 +4966,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="212" t="s">
+      <c r="U18" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V18" s="213"/>
+      <c r="V18" s="210"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -4982,10 +4982,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="212" t="s">
+      <c r="AA18" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB18" s="213"/>
+      <c r="AB18" s="210"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -5023,20 +5023,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="240"/>
-      <c r="H19" s="241"/>
-      <c r="I19" s="241"/>
-      <c r="J19" s="242"/>
+      <c r="G19" s="219"/>
+      <c r="H19" s="220"/>
+      <c r="I19" s="220"/>
+      <c r="J19" s="221"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="216" t="s">
+      <c r="N19" s="184" t="s">
         <v>93</v>
       </c>
-      <c r="O19" s="217"/>
-      <c r="P19" s="218"/>
+      <c r="O19" s="185"/>
+      <c r="P19" s="186"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -5046,10 +5046,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="212" t="s">
+      <c r="U19" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V19" s="213"/>
+      <c r="V19" s="210"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -5062,10 +5062,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="212" t="s">
+      <c r="AA19" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB19" s="213"/>
+      <c r="AB19" s="210"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -5105,20 +5105,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="240"/>
-      <c r="H20" s="241"/>
-      <c r="I20" s="241"/>
-      <c r="J20" s="242"/>
+      <c r="G20" s="219"/>
+      <c r="H20" s="220"/>
+      <c r="I20" s="220"/>
+      <c r="J20" s="221"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="216" t="s">
+      <c r="N20" s="184" t="s">
         <v>94</v>
       </c>
-      <c r="O20" s="217"/>
-      <c r="P20" s="218"/>
+      <c r="O20" s="185"/>
+      <c r="P20" s="186"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -5128,10 +5128,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="212" t="s">
+      <c r="U20" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V20" s="213"/>
+      <c r="V20" s="210"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -5144,10 +5144,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="212" t="s">
+      <c r="AA20" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB20" s="213"/>
+      <c r="AB20" s="210"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -5185,20 +5185,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="240"/>
-      <c r="H21" s="241"/>
-      <c r="I21" s="241"/>
-      <c r="J21" s="242"/>
+      <c r="G21" s="219"/>
+      <c r="H21" s="220"/>
+      <c r="I21" s="220"/>
+      <c r="J21" s="221"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="216" t="s">
+      <c r="N21" s="184" t="s">
         <v>62</v>
       </c>
-      <c r="O21" s="217"/>
-      <c r="P21" s="218"/>
+      <c r="O21" s="185"/>
+      <c r="P21" s="186"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -5208,10 +5208,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="212" t="s">
+      <c r="U21" s="209" t="s">
         <v>96</v>
       </c>
-      <c r="V21" s="213"/>
+      <c r="V21" s="210"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -5224,10 +5224,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="212" t="s">
+      <c r="AA21" s="209" t="s">
         <v>98</v>
       </c>
-      <c r="AB21" s="213"/>
+      <c r="AB21" s="210"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -5261,22 +5261,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="246"/>
-      <c r="F22" s="241"/>
-      <c r="G22" s="241"/>
-      <c r="H22" s="241"/>
-      <c r="I22" s="241"/>
-      <c r="J22" s="242"/>
+      <c r="E22" s="223"/>
+      <c r="F22" s="220"/>
+      <c r="G22" s="220"/>
+      <c r="H22" s="220"/>
+      <c r="I22" s="220"/>
+      <c r="J22" s="221"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="216" t="s">
+      <c r="N22" s="184" t="s">
         <v>63</v>
       </c>
-      <c r="O22" s="217"/>
-      <c r="P22" s="218"/>
+      <c r="O22" s="185"/>
+      <c r="P22" s="186"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -5286,10 +5286,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="212" t="s">
+      <c r="U22" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V22" s="213"/>
+      <c r="V22" s="210"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -5302,10 +5302,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="212" t="s">
+      <c r="AA22" s="209" t="s">
         <v>96</v>
       </c>
-      <c r="AB22" s="213"/>
+      <c r="AB22" s="210"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -5345,22 +5345,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="247" t="s">
+      <c r="G23" s="222" t="s">
         <v>77</v>
       </c>
-      <c r="H23" s="217"/>
-      <c r="I23" s="217"/>
-      <c r="J23" s="218"/>
+      <c r="H23" s="185"/>
+      <c r="I23" s="185"/>
+      <c r="J23" s="186"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="216" t="s">
+      <c r="N23" s="184" t="s">
         <v>82</v>
       </c>
-      <c r="O23" s="217"/>
-      <c r="P23" s="218"/>
+      <c r="O23" s="185"/>
+      <c r="P23" s="186"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -5370,10 +5370,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="212" t="s">
+      <c r="U23" s="209" t="s">
         <v>97</v>
       </c>
-      <c r="V23" s="213"/>
+      <c r="V23" s="210"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -5386,10 +5386,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="212" t="s">
+      <c r="AA23" s="209" t="s">
         <v>96</v>
       </c>
-      <c r="AB23" s="213"/>
+      <c r="AB23" s="210"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -5429,22 +5429,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="247" t="s">
+      <c r="G24" s="222" t="s">
         <v>77</v>
       </c>
-      <c r="H24" s="217"/>
-      <c r="I24" s="217"/>
-      <c r="J24" s="218"/>
+      <c r="H24" s="185"/>
+      <c r="I24" s="185"/>
+      <c r="J24" s="186"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="216" t="s">
+      <c r="N24" s="184" t="s">
         <v>81</v>
       </c>
-      <c r="O24" s="217"/>
-      <c r="P24" s="218"/>
+      <c r="O24" s="185"/>
+      <c r="P24" s="186"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -5454,15 +5454,15 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="212" t="s">
+      <c r="U24" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V24" s="213"/>
+      <c r="V24" s="210"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
       <c r="X24" s="34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y24" s="34">
         <v>0</v>
@@ -5470,10 +5470,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="212" t="s">
+      <c r="AA24" s="209" t="s">
         <v>98</v>
       </c>
-      <c r="AB24" s="213"/>
+      <c r="AB24" s="210"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -5511,10 +5511,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="240"/>
-      <c r="H25" s="241"/>
-      <c r="I25" s="241"/>
-      <c r="J25" s="242"/>
+      <c r="G25" s="219"/>
+      <c r="H25" s="220"/>
+      <c r="I25" s="220"/>
+      <c r="J25" s="221"/>
       <c r="K25" s="49" t="s">
         <v>39</v>
       </c>
@@ -5522,11 +5522,11 @@
         <v>155</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="216" t="s">
+      <c r="N25" s="184" t="s">
         <v>41</v>
       </c>
-      <c r="O25" s="217"/>
-      <c r="P25" s="218"/>
+      <c r="O25" s="185"/>
+      <c r="P25" s="186"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -5536,10 +5536,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="212" t="s">
+      <c r="U25" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V25" s="213"/>
+      <c r="V25" s="210"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -5552,10 +5552,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="212" t="s">
+      <c r="AA25" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB25" s="213"/>
+      <c r="AB25" s="210"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -5593,10 +5593,10 @@
       <c r="F26" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="G26" s="240"/>
-      <c r="H26" s="241"/>
-      <c r="I26" s="241"/>
-      <c r="J26" s="242"/>
+      <c r="G26" s="219"/>
+      <c r="H26" s="220"/>
+      <c r="I26" s="220"/>
+      <c r="J26" s="221"/>
       <c r="K26" s="31" t="s">
         <v>40</v>
       </c>
@@ -5604,11 +5604,11 @@
         <v>155</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="216" t="s">
+      <c r="N26" s="184" t="s">
         <v>42</v>
       </c>
-      <c r="O26" s="217"/>
-      <c r="P26" s="218"/>
+      <c r="O26" s="185"/>
+      <c r="P26" s="186"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -5618,10 +5618,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="212" t="s">
+      <c r="U26" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V26" s="213"/>
+      <c r="V26" s="210"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -5634,10 +5634,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="212" t="s">
+      <c r="AA26" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB26" s="213"/>
+      <c r="AB26" s="210"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -5669,22 +5669,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="246"/>
-      <c r="F27" s="241"/>
-      <c r="G27" s="241"/>
-      <c r="H27" s="241"/>
-      <c r="I27" s="241"/>
-      <c r="J27" s="242"/>
+      <c r="E27" s="223"/>
+      <c r="F27" s="220"/>
+      <c r="G27" s="220"/>
+      <c r="H27" s="220"/>
+      <c r="I27" s="220"/>
+      <c r="J27" s="221"/>
       <c r="K27" s="25" t="s">
         <v>44</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="216" t="s">
+      <c r="N27" s="184" t="s">
         <v>46</v>
       </c>
-      <c r="O27" s="217"/>
-      <c r="P27" s="218"/>
+      <c r="O27" s="185"/>
+      <c r="P27" s="186"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -5694,10 +5694,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="212" t="s">
+      <c r="U27" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V27" s="213"/>
+      <c r="V27" s="210"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -5710,10 +5710,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="212" t="s">
+      <c r="AA27" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB27" s="213"/>
+      <c r="AB27" s="210"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -5745,12 +5745,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="243"/>
-      <c r="F28" s="244"/>
-      <c r="G28" s="244"/>
-      <c r="H28" s="244"/>
-      <c r="I28" s="244"/>
-      <c r="J28" s="245"/>
+      <c r="E28" s="227"/>
+      <c r="F28" s="228"/>
+      <c r="G28" s="228"/>
+      <c r="H28" s="228"/>
+      <c r="I28" s="228"/>
+      <c r="J28" s="229"/>
       <c r="K28" s="52" t="s">
         <v>45</v>
       </c>
@@ -5758,11 +5758,11 @@
         <v>155</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="237" t="s">
+      <c r="N28" s="197" t="s">
         <v>92</v>
       </c>
-      <c r="O28" s="238"/>
-      <c r="P28" s="239"/>
+      <c r="O28" s="198"/>
+      <c r="P28" s="199"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -5772,10 +5772,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="214" t="s">
+      <c r="U28" s="259" t="s">
         <v>73</v>
       </c>
-      <c r="V28" s="215"/>
+      <c r="V28" s="260"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -5788,10 +5788,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="214" t="s">
+      <c r="AA28" s="259" t="s">
         <v>73</v>
       </c>
-      <c r="AB28" s="215"/>
+      <c r="AB28" s="260"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -5868,18 +5868,18 @@
       <c r="S30" s="75" t="s">
         <v>156</v>
       </c>
-      <c r="T30" s="259" t="s">
+      <c r="T30" s="179" t="s">
         <v>157</v>
       </c>
-      <c r="U30" s="259"/>
-      <c r="V30" s="259"/>
-      <c r="W30" s="259"/>
-      <c r="X30" s="259"/>
-      <c r="Y30" s="259"/>
-      <c r="Z30" s="259"/>
-      <c r="AA30" s="259"/>
-      <c r="AB30" s="259"/>
-      <c r="AC30" s="227"/>
+      <c r="U30" s="179"/>
+      <c r="V30" s="179"/>
+      <c r="W30" s="179"/>
+      <c r="X30" s="179"/>
+      <c r="Y30" s="179"/>
+      <c r="Z30" s="179"/>
+      <c r="AA30" s="179"/>
+      <c r="AB30" s="179"/>
+      <c r="AC30" s="180"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B31" s="67" t="s">
@@ -5920,18 +5920,18 @@
       <c r="S31" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="T31" s="190" t="s">
+      <c r="T31" s="181" t="s">
         <v>162</v>
       </c>
-      <c r="U31" s="233"/>
-      <c r="V31" s="233"/>
-      <c r="W31" s="233"/>
-      <c r="X31" s="233"/>
-      <c r="Y31" s="233"/>
-      <c r="Z31" s="233"/>
-      <c r="AA31" s="233"/>
-      <c r="AB31" s="233"/>
-      <c r="AC31" s="191"/>
+      <c r="U31" s="182"/>
+      <c r="V31" s="182"/>
+      <c r="W31" s="182"/>
+      <c r="X31" s="182"/>
+      <c r="Y31" s="182"/>
+      <c r="Z31" s="182"/>
+      <c r="AA31" s="182"/>
+      <c r="AB31" s="182"/>
+      <c r="AC31" s="183"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B32" s="4" t="s">
@@ -5955,18 +5955,18 @@
       <c r="S32" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="T32" s="216" t="s">
+      <c r="T32" s="184" t="s">
         <v>163</v>
       </c>
-      <c r="U32" s="217"/>
-      <c r="V32" s="217"/>
-      <c r="W32" s="217"/>
-      <c r="X32" s="217"/>
-      <c r="Y32" s="217"/>
-      <c r="Z32" s="217"/>
-      <c r="AA32" s="217"/>
-      <c r="AB32" s="217"/>
-      <c r="AC32" s="218"/>
+      <c r="U32" s="185"/>
+      <c r="V32" s="185"/>
+      <c r="W32" s="185"/>
+      <c r="X32" s="185"/>
+      <c r="Y32" s="185"/>
+      <c r="Z32" s="185"/>
+      <c r="AA32" s="185"/>
+      <c r="AB32" s="185"/>
+      <c r="AC32" s="186"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
       <c r="H33" s="84" t="s">
@@ -6002,31 +6002,31 @@
       <c r="S33" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="T33" s="216" t="s">
+      <c r="T33" s="184" t="s">
         <v>164</v>
       </c>
-      <c r="U33" s="217"/>
-      <c r="V33" s="217"/>
-      <c r="W33" s="217"/>
-      <c r="X33" s="217"/>
-      <c r="Y33" s="217"/>
-      <c r="Z33" s="217"/>
-      <c r="AA33" s="217"/>
-      <c r="AB33" s="217"/>
-      <c r="AC33" s="218"/>
+      <c r="U33" s="185"/>
+      <c r="V33" s="185"/>
+      <c r="W33" s="185"/>
+      <c r="X33" s="185"/>
+      <c r="Y33" s="185"/>
+      <c r="Z33" s="185"/>
+      <c r="AA33" s="185"/>
+      <c r="AB33" s="185"/>
+      <c r="AC33" s="186"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B34" s="207" t="s">
+      <c r="B34" s="256" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="205" t="s">
+      <c r="C34" s="230" t="s">
         <v>114</v>
       </c>
-      <c r="D34" s="206"/>
-      <c r="E34" s="205" t="s">
+      <c r="D34" s="232"/>
+      <c r="E34" s="230" t="s">
         <v>115</v>
       </c>
-      <c r="F34" s="206"/>
+      <c r="F34" s="232"/>
       <c r="H34" s="77" t="s">
         <v>65</v>
       </c>
@@ -6052,21 +6052,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="216" t="s">
+      <c r="T34" s="184" t="s">
         <v>165</v>
       </c>
-      <c r="U34" s="217"/>
-      <c r="V34" s="217"/>
-      <c r="W34" s="217"/>
-      <c r="X34" s="217"/>
-      <c r="Y34" s="217"/>
-      <c r="Z34" s="217"/>
-      <c r="AA34" s="217"/>
-      <c r="AB34" s="217"/>
-      <c r="AC34" s="218"/>
+      <c r="U34" s="185"/>
+      <c r="V34" s="185"/>
+      <c r="W34" s="185"/>
+      <c r="X34" s="185"/>
+      <c r="Y34" s="185"/>
+      <c r="Z34" s="185"/>
+      <c r="AA34" s="185"/>
+      <c r="AB34" s="185"/>
+      <c r="AC34" s="186"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B35" s="208"/>
+      <c r="B35" s="257"/>
       <c r="C35" s="64" t="s">
         <v>99</v>
       </c>
@@ -6085,18 +6085,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="216" t="s">
+      <c r="T35" s="184" t="s">
         <v>166</v>
       </c>
-      <c r="U35" s="217"/>
-      <c r="V35" s="217"/>
-      <c r="W35" s="217"/>
-      <c r="X35" s="217"/>
-      <c r="Y35" s="217"/>
-      <c r="Z35" s="217"/>
-      <c r="AA35" s="217"/>
-      <c r="AB35" s="217"/>
-      <c r="AC35" s="218"/>
+      <c r="U35" s="185"/>
+      <c r="V35" s="185"/>
+      <c r="W35" s="185"/>
+      <c r="X35" s="185"/>
+      <c r="Y35" s="185"/>
+      <c r="Z35" s="185"/>
+      <c r="AA35" s="185"/>
+      <c r="AB35" s="185"/>
+      <c r="AC35" s="186"/>
     </row>
     <row r="36" spans="2:29">
       <c r="B36" s="1">
@@ -6120,18 +6120,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="216" t="s">
+      <c r="T36" s="184" t="s">
         <v>167</v>
       </c>
-      <c r="U36" s="217"/>
-      <c r="V36" s="217"/>
-      <c r="W36" s="217"/>
-      <c r="X36" s="217"/>
-      <c r="Y36" s="217"/>
-      <c r="Z36" s="217"/>
-      <c r="AA36" s="217"/>
-      <c r="AB36" s="217"/>
-      <c r="AC36" s="218"/>
+      <c r="U36" s="185"/>
+      <c r="V36" s="185"/>
+      <c r="W36" s="185"/>
+      <c r="X36" s="185"/>
+      <c r="Y36" s="185"/>
+      <c r="Z36" s="185"/>
+      <c r="AA36" s="185"/>
+      <c r="AB36" s="185"/>
+      <c r="AC36" s="186"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1">
       <c r="B37" s="2">
@@ -6156,18 +6156,18 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="216" t="s">
+      <c r="T37" s="184" t="s">
         <v>194</v>
       </c>
-      <c r="U37" s="217"/>
-      <c r="V37" s="217"/>
-      <c r="W37" s="217"/>
-      <c r="X37" s="217"/>
-      <c r="Y37" s="217"/>
-      <c r="Z37" s="217"/>
-      <c r="AA37" s="217"/>
-      <c r="AB37" s="217"/>
-      <c r="AC37" s="218"/>
+      <c r="U37" s="185"/>
+      <c r="V37" s="185"/>
+      <c r="W37" s="185"/>
+      <c r="X37" s="185"/>
+      <c r="Y37" s="185"/>
+      <c r="Z37" s="185"/>
+      <c r="AA37" s="185"/>
+      <c r="AB37" s="185"/>
+      <c r="AC37" s="186"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1">
       <c r="B38" s="2">
@@ -6188,21 +6188,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="260" t="s">
+      <c r="S38" s="189" t="s">
         <v>72</v>
       </c>
-      <c r="T38" s="262" t="s">
+      <c r="T38" s="191" t="s">
         <v>168</v>
       </c>
-      <c r="U38" s="263"/>
-      <c r="V38" s="263"/>
-      <c r="W38" s="263"/>
-      <c r="X38" s="263"/>
-      <c r="Y38" s="263"/>
-      <c r="Z38" s="263"/>
-      <c r="AA38" s="263"/>
-      <c r="AB38" s="263"/>
-      <c r="AC38" s="264"/>
+      <c r="U38" s="192"/>
+      <c r="V38" s="192"/>
+      <c r="W38" s="192"/>
+      <c r="X38" s="192"/>
+      <c r="Y38" s="192"/>
+      <c r="Z38" s="192"/>
+      <c r="AA38" s="192"/>
+      <c r="AB38" s="192"/>
+      <c r="AC38" s="193"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1">
       <c r="B39" s="2">
@@ -6220,26 +6220,26 @@
       <c r="F39" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G39" s="192" t="s">
+      <c r="G39" s="200" t="s">
         <v>181</v>
       </c>
-      <c r="H39" s="193"/>
-      <c r="I39" s="193"/>
-      <c r="J39" s="194"/>
+      <c r="H39" s="201"/>
+      <c r="I39" s="201"/>
+      <c r="J39" s="202"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="261"/>
-      <c r="T39" s="265"/>
-      <c r="U39" s="266"/>
-      <c r="V39" s="266"/>
-      <c r="W39" s="266"/>
-      <c r="X39" s="266"/>
-      <c r="Y39" s="266"/>
-      <c r="Z39" s="266"/>
-      <c r="AA39" s="266"/>
-      <c r="AB39" s="266"/>
-      <c r="AC39" s="267"/>
+      <c r="S39" s="190"/>
+      <c r="T39" s="194"/>
+      <c r="U39" s="195"/>
+      <c r="V39" s="195"/>
+      <c r="W39" s="195"/>
+      <c r="X39" s="195"/>
+      <c r="Y39" s="195"/>
+      <c r="Z39" s="195"/>
+      <c r="AA39" s="195"/>
+      <c r="AB39" s="195"/>
+      <c r="AC39" s="196"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1">
       <c r="B40" s="2">
@@ -6257,28 +6257,28 @@
       <c r="F40" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G40" s="195"/>
-      <c r="H40" s="196"/>
-      <c r="I40" s="196"/>
-      <c r="J40" s="197"/>
+      <c r="G40" s="206"/>
+      <c r="H40" s="207"/>
+      <c r="I40" s="207"/>
+      <c r="J40" s="208"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="216" t="s">
+      <c r="T40" s="184" t="s">
         <v>169</v>
       </c>
-      <c r="U40" s="217"/>
-      <c r="V40" s="217"/>
-      <c r="W40" s="217"/>
-      <c r="X40" s="217"/>
-      <c r="Y40" s="217"/>
-      <c r="Z40" s="217"/>
-      <c r="AA40" s="217"/>
-      <c r="AB40" s="217"/>
-      <c r="AC40" s="218"/>
+      <c r="U40" s="185"/>
+      <c r="V40" s="185"/>
+      <c r="W40" s="185"/>
+      <c r="X40" s="185"/>
+      <c r="Y40" s="185"/>
+      <c r="Z40" s="185"/>
+      <c r="AA40" s="185"/>
+      <c r="AB40" s="185"/>
+      <c r="AC40" s="186"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1">
       <c r="B41" s="2">
@@ -6296,28 +6296,28 @@
       <c r="F41" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G41" s="195"/>
-      <c r="H41" s="196"/>
-      <c r="I41" s="196"/>
-      <c r="J41" s="197"/>
+      <c r="G41" s="206"/>
+      <c r="H41" s="207"/>
+      <c r="I41" s="207"/>
+      <c r="J41" s="208"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="216" t="s">
+      <c r="T41" s="184" t="s">
         <v>170</v>
       </c>
-      <c r="U41" s="217"/>
-      <c r="V41" s="217"/>
-      <c r="W41" s="217"/>
-      <c r="X41" s="217"/>
-      <c r="Y41" s="217"/>
-      <c r="Z41" s="217"/>
-      <c r="AA41" s="217"/>
-      <c r="AB41" s="217"/>
-      <c r="AC41" s="218"/>
+      <c r="U41" s="185"/>
+      <c r="V41" s="185"/>
+      <c r="W41" s="185"/>
+      <c r="X41" s="185"/>
+      <c r="Y41" s="185"/>
+      <c r="Z41" s="185"/>
+      <c r="AA41" s="185"/>
+      <c r="AB41" s="185"/>
+      <c r="AC41" s="186"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
       <c r="B42" s="2">
@@ -6335,28 +6335,28 @@
       <c r="F42" s="76" t="s">
         <v>175</v>
       </c>
-      <c r="G42" s="198"/>
-      <c r="H42" s="199"/>
-      <c r="I42" s="199"/>
-      <c r="J42" s="200"/>
+      <c r="G42" s="203"/>
+      <c r="H42" s="204"/>
+      <c r="I42" s="204"/>
+      <c r="J42" s="205"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T42" s="216" t="s">
+      <c r="T42" s="184" t="s">
         <v>171</v>
       </c>
-      <c r="U42" s="217"/>
-      <c r="V42" s="217"/>
-      <c r="W42" s="217"/>
-      <c r="X42" s="217"/>
-      <c r="Y42" s="217"/>
-      <c r="Z42" s="217"/>
-      <c r="AA42" s="217"/>
-      <c r="AB42" s="217"/>
-      <c r="AC42" s="218"/>
+      <c r="U42" s="185"/>
+      <c r="V42" s="185"/>
+      <c r="W42" s="185"/>
+      <c r="X42" s="185"/>
+      <c r="Y42" s="185"/>
+      <c r="Z42" s="185"/>
+      <c r="AA42" s="185"/>
+      <c r="AB42" s="185"/>
+      <c r="AC42" s="186"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
       <c r="B43" s="2">
@@ -6374,30 +6374,30 @@
       <c r="F43" s="35" t="s">
         <v>146</v>
       </c>
-      <c r="G43" s="183" t="s">
+      <c r="G43" s="263" t="s">
         <v>191</v>
       </c>
-      <c r="H43" s="184"/>
-      <c r="I43" s="184"/>
-      <c r="J43" s="185"/>
+      <c r="H43" s="187"/>
+      <c r="I43" s="187"/>
+      <c r="J43" s="188"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="T43" s="216" t="s">
+      <c r="T43" s="184" t="s">
         <v>172</v>
       </c>
-      <c r="U43" s="217"/>
-      <c r="V43" s="217"/>
-      <c r="W43" s="217"/>
-      <c r="X43" s="217"/>
-      <c r="Y43" s="217"/>
-      <c r="Z43" s="217"/>
-      <c r="AA43" s="217"/>
-      <c r="AB43" s="217"/>
-      <c r="AC43" s="218"/>
+      <c r="U43" s="185"/>
+      <c r="V43" s="185"/>
+      <c r="W43" s="185"/>
+      <c r="X43" s="185"/>
+      <c r="Y43" s="185"/>
+      <c r="Z43" s="185"/>
+      <c r="AA43" s="185"/>
+      <c r="AB43" s="185"/>
+      <c r="AC43" s="186"/>
     </row>
     <row r="44" spans="2:29" ht="15.75" thickBot="1">
       <c r="B44" s="2">
@@ -6418,21 +6418,21 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="260" t="s">
+      <c r="S44" s="189" t="s">
         <v>75</v>
       </c>
-      <c r="T44" s="262" t="s">
+      <c r="T44" s="191" t="s">
         <v>173</v>
       </c>
-      <c r="U44" s="263"/>
-      <c r="V44" s="263"/>
-      <c r="W44" s="263"/>
-      <c r="X44" s="263"/>
-      <c r="Y44" s="263"/>
-      <c r="Z44" s="263"/>
-      <c r="AA44" s="263"/>
-      <c r="AB44" s="263"/>
-      <c r="AC44" s="264"/>
+      <c r="U44" s="192"/>
+      <c r="V44" s="192"/>
+      <c r="W44" s="192"/>
+      <c r="X44" s="192"/>
+      <c r="Y44" s="192"/>
+      <c r="Z44" s="192"/>
+      <c r="AA44" s="192"/>
+      <c r="AB44" s="192"/>
+      <c r="AC44" s="193"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1">
       <c r="B45" s="2">
@@ -6450,26 +6450,26 @@
       <c r="F45" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="G45" s="192" t="s">
+      <c r="G45" s="200" t="s">
         <v>180</v>
       </c>
-      <c r="H45" s="193"/>
-      <c r="I45" s="193"/>
-      <c r="J45" s="194"/>
+      <c r="H45" s="201"/>
+      <c r="I45" s="201"/>
+      <c r="J45" s="202"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="261"/>
-      <c r="T45" s="265"/>
-      <c r="U45" s="266"/>
-      <c r="V45" s="266"/>
-      <c r="W45" s="266"/>
-      <c r="X45" s="266"/>
-      <c r="Y45" s="266"/>
-      <c r="Z45" s="266"/>
-      <c r="AA45" s="266"/>
-      <c r="AB45" s="266"/>
-      <c r="AC45" s="267"/>
+      <c r="S45" s="190"/>
+      <c r="T45" s="194"/>
+      <c r="U45" s="195"/>
+      <c r="V45" s="195"/>
+      <c r="W45" s="195"/>
+      <c r="X45" s="195"/>
+      <c r="Y45" s="195"/>
+      <c r="Z45" s="195"/>
+      <c r="AA45" s="195"/>
+      <c r="AB45" s="195"/>
+      <c r="AC45" s="196"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
       <c r="B46" s="2">
@@ -6487,28 +6487,28 @@
       <c r="F46" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="G46" s="198"/>
-      <c r="H46" s="199"/>
-      <c r="I46" s="199"/>
-      <c r="J46" s="200"/>
+      <c r="G46" s="203"/>
+      <c r="H46" s="204"/>
+      <c r="I46" s="204"/>
+      <c r="J46" s="205"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="T46" s="237" t="s">
+      <c r="T46" s="197" t="s">
         <v>174</v>
       </c>
-      <c r="U46" s="238"/>
-      <c r="V46" s="238"/>
-      <c r="W46" s="238"/>
-      <c r="X46" s="238"/>
-      <c r="Y46" s="238"/>
-      <c r="Z46" s="238"/>
-      <c r="AA46" s="238"/>
-      <c r="AB46" s="238"/>
-      <c r="AC46" s="239"/>
+      <c r="U46" s="198"/>
+      <c r="V46" s="198"/>
+      <c r="W46" s="198"/>
+      <c r="X46" s="198"/>
+      <c r="Y46" s="198"/>
+      <c r="Z46" s="198"/>
+      <c r="AA46" s="198"/>
+      <c r="AB46" s="198"/>
+      <c r="AC46" s="199"/>
     </row>
     <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
       <c r="B47" s="2">
@@ -6526,12 +6526,12 @@
       <c r="F47" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="G47" s="184" t="s">
+      <c r="G47" s="187" t="s">
         <v>151</v>
       </c>
-      <c r="H47" s="184"/>
-      <c r="I47" s="184"/>
-      <c r="J47" s="185"/>
+      <c r="H47" s="187"/>
+      <c r="I47" s="187"/>
+      <c r="J47" s="188"/>
     </row>
     <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
       <c r="B48" s="2">
@@ -6569,12 +6569,12 @@
       <c r="F49" s="35" t="s">
         <v>152</v>
       </c>
-      <c r="G49" s="192" t="s">
+      <c r="G49" s="200" t="s">
         <v>154</v>
       </c>
-      <c r="H49" s="193"/>
-      <c r="I49" s="193"/>
-      <c r="J49" s="194"/>
+      <c r="H49" s="201"/>
+      <c r="I49" s="201"/>
+      <c r="J49" s="202"/>
     </row>
     <row r="50" spans="2:10" ht="30" customHeight="1">
       <c r="B50" s="2">
@@ -6592,10 +6592,10 @@
       <c r="F50" s="35" t="s">
         <v>152</v>
       </c>
-      <c r="G50" s="195"/>
-      <c r="H50" s="196"/>
-      <c r="I50" s="196"/>
-      <c r="J50" s="197"/>
+      <c r="G50" s="206"/>
+      <c r="H50" s="207"/>
+      <c r="I50" s="207"/>
+      <c r="J50" s="208"/>
     </row>
     <row r="51" spans="2:10" ht="32.25" customHeight="1" thickBot="1">
       <c r="B51" s="4">
@@ -6613,38 +6613,38 @@
       <c r="F51" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="G51" s="198"/>
-      <c r="H51" s="199"/>
-      <c r="I51" s="199"/>
-      <c r="J51" s="200"/>
+      <c r="G51" s="203"/>
+      <c r="H51" s="204"/>
+      <c r="I51" s="204"/>
+      <c r="J51" s="205"/>
     </row>
     <row r="52" spans="2:10" ht="30.75" customHeight="1" thickBot="1">
-      <c r="B52" s="209" t="s">
+      <c r="B52" s="258" t="s">
         <v>141</v>
       </c>
-      <c r="C52" s="210"/>
-      <c r="D52" s="210"/>
-      <c r="E52" s="210"/>
-      <c r="F52" s="211"/>
+      <c r="C52" s="239"/>
+      <c r="D52" s="239"/>
+      <c r="E52" s="239"/>
+      <c r="F52" s="240"/>
     </row>
     <row r="53" spans="2:10" ht="31.5" customHeight="1" thickBot="1"/>
     <row r="54" spans="2:10" ht="24.75" customHeight="1">
-      <c r="B54" s="203" t="s">
+      <c r="B54" s="252" t="s">
         <v>182</v>
       </c>
-      <c r="C54" s="201" t="s">
+      <c r="C54" s="250" t="s">
         <v>184</v>
       </c>
-      <c r="D54" s="186" t="s">
+      <c r="D54" s="264" t="s">
         <v>183</v>
       </c>
-      <c r="E54" s="187"/>
+      <c r="E54" s="265"/>
     </row>
     <row r="55" spans="2:10" ht="24" customHeight="1" thickBot="1">
-      <c r="B55" s="204"/>
-      <c r="C55" s="202"/>
-      <c r="D55" s="188"/>
-      <c r="E55" s="189"/>
+      <c r="B55" s="253"/>
+      <c r="C55" s="251"/>
+      <c r="D55" s="266"/>
+      <c r="E55" s="267"/>
     </row>
     <row r="56" spans="2:10" ht="41.25" customHeight="1">
       <c r="B56" s="81">
@@ -6653,10 +6653,10 @@
       <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D56" s="190" t="s">
+      <c r="D56" s="181" t="s">
         <v>206</v>
       </c>
-      <c r="E56" s="191"/>
+      <c r="E56" s="183"/>
     </row>
     <row r="57" spans="2:10" ht="31.5" customHeight="1">
       <c r="B57" s="82">
@@ -6665,10 +6665,10 @@
       <c r="C57" s="86" t="s">
         <v>202</v>
       </c>
-      <c r="D57" s="179" t="s">
+      <c r="D57" s="254" t="s">
         <v>205</v>
       </c>
-      <c r="E57" s="180"/>
+      <c r="E57" s="255"/>
     </row>
     <row r="58" spans="2:10" ht="30.75" customHeight="1">
       <c r="B58" s="82">
@@ -6677,10 +6677,10 @@
       <c r="C58" s="38" t="s">
         <v>203</v>
       </c>
-      <c r="D58" s="179" t="s">
+      <c r="D58" s="254" t="s">
         <v>204</v>
       </c>
-      <c r="E58" s="180"/>
+      <c r="E58" s="255"/>
     </row>
     <row r="59" spans="2:10" ht="33.75" customHeight="1">
       <c r="B59" s="82">
@@ -6689,10 +6689,10 @@
       <c r="C59" s="86" t="s">
         <v>185</v>
       </c>
-      <c r="D59" s="179" t="s">
+      <c r="D59" s="254" t="s">
         <v>188</v>
       </c>
-      <c r="E59" s="180"/>
+      <c r="E59" s="255"/>
     </row>
     <row r="60" spans="2:10" ht="28.5" customHeight="1">
       <c r="B60" s="82">
@@ -6701,10 +6701,10 @@
       <c r="C60" s="38" t="s">
         <v>186</v>
       </c>
-      <c r="D60" s="179" t="s">
+      <c r="D60" s="254" t="s">
         <v>189</v>
       </c>
-      <c r="E60" s="180"/>
+      <c r="E60" s="255"/>
     </row>
     <row r="61" spans="2:10" ht="40.5" customHeight="1">
       <c r="B61" s="82">
@@ -6713,10 +6713,10 @@
       <c r="C61" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="D61" s="179" t="s">
+      <c r="D61" s="254" t="s">
         <v>190</v>
       </c>
-      <c r="E61" s="180"/>
+      <c r="E61" s="255"/>
     </row>
     <row r="62" spans="2:10" ht="53.25" customHeight="1">
       <c r="B62" s="82">
@@ -6725,106 +6725,200 @@
       <c r="C62" s="86" t="s">
         <v>195</v>
       </c>
-      <c r="D62" s="179" t="s">
+      <c r="D62" s="254" t="s">
         <v>196</v>
       </c>
-      <c r="E62" s="180"/>
+      <c r="E62" s="255"/>
     </row>
     <row r="63" spans="2:10" ht="36" customHeight="1">
       <c r="B63" s="82">
         <v>7</v>
       </c>
       <c r="C63" s="86"/>
-      <c r="D63" s="179"/>
-      <c r="E63" s="180"/>
+      <c r="D63" s="254"/>
+      <c r="E63" s="255"/>
     </row>
     <row r="64" spans="2:10" ht="40.5" customHeight="1">
       <c r="B64" s="82">
         <v>8</v>
       </c>
       <c r="C64" s="86"/>
-      <c r="D64" s="179"/>
-      <c r="E64" s="180"/>
+      <c r="D64" s="254"/>
+      <c r="E64" s="255"/>
     </row>
     <row r="65" spans="2:5">
       <c r="B65" s="82">
         <v>9</v>
       </c>
       <c r="C65" s="86"/>
-      <c r="D65" s="179"/>
-      <c r="E65" s="180"/>
+      <c r="D65" s="254"/>
+      <c r="E65" s="255"/>
     </row>
     <row r="66" spans="2:5" ht="30" customHeight="1">
       <c r="B66" s="82">
         <v>10</v>
       </c>
       <c r="C66" s="86"/>
-      <c r="D66" s="179"/>
-      <c r="E66" s="180"/>
+      <c r="D66" s="254"/>
+      <c r="E66" s="255"/>
     </row>
     <row r="67" spans="2:5">
       <c r="B67" s="82">
         <v>11</v>
       </c>
       <c r="C67" s="86"/>
-      <c r="D67" s="179"/>
-      <c r="E67" s="180"/>
+      <c r="D67" s="254"/>
+      <c r="E67" s="255"/>
     </row>
     <row r="68" spans="2:5">
       <c r="B68" s="82">
         <v>12</v>
       </c>
       <c r="C68" s="86"/>
-      <c r="D68" s="179"/>
-      <c r="E68" s="180"/>
+      <c r="D68" s="254"/>
+      <c r="E68" s="255"/>
     </row>
     <row r="69" spans="2:5">
       <c r="B69" s="82">
         <v>13</v>
       </c>
       <c r="C69" s="86"/>
-      <c r="D69" s="179"/>
-      <c r="E69" s="180"/>
+      <c r="D69" s="254"/>
+      <c r="E69" s="255"/>
     </row>
     <row r="70" spans="2:5" ht="30" customHeight="1">
       <c r="B70" s="82">
         <v>14</v>
       </c>
       <c r="C70" s="86"/>
-      <c r="D70" s="179"/>
-      <c r="E70" s="180"/>
+      <c r="D70" s="254"/>
+      <c r="E70" s="255"/>
     </row>
     <row r="71" spans="2:5" ht="15.75" thickBot="1">
       <c r="B71" s="83">
         <v>15</v>
       </c>
       <c r="C71" s="87"/>
-      <c r="D71" s="181"/>
-      <c r="E71" s="182"/>
+      <c r="D71" s="261"/>
+      <c r="E71" s="262"/>
     </row>
     <row r="75" spans="2:5" ht="72" customHeight="1"/>
   </sheetData>
   <mergeCells count="158">
-    <mergeCell ref="T30:AC30"/>
-    <mergeCell ref="T31:AC31"/>
-    <mergeCell ref="T32:AC32"/>
-    <mergeCell ref="T33:AC33"/>
-    <mergeCell ref="T34:AC34"/>
-    <mergeCell ref="T35:AC35"/>
-    <mergeCell ref="T36:AC36"/>
-    <mergeCell ref="T37:AC37"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="S38:S39"/>
-    <mergeCell ref="T38:AC39"/>
-    <mergeCell ref="S44:S45"/>
-    <mergeCell ref="T44:AC45"/>
-    <mergeCell ref="T40:AC40"/>
-    <mergeCell ref="T41:AC41"/>
-    <mergeCell ref="T42:AC42"/>
-    <mergeCell ref="T43:AC43"/>
-    <mergeCell ref="T46:AC46"/>
-    <mergeCell ref="G45:J46"/>
-    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D54:E55"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="AA7:AB7"/>
+    <mergeCell ref="AA28:AB28"/>
+    <mergeCell ref="AA12:AB12"/>
+    <mergeCell ref="AA13:AB13"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AA25:AB25"/>
+    <mergeCell ref="AA26:AB26"/>
+    <mergeCell ref="U27:V27"/>
+    <mergeCell ref="AA27:AB27"/>
+    <mergeCell ref="U12:V12"/>
+    <mergeCell ref="AA14:AB14"/>
+    <mergeCell ref="U28:V28"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="N20:P20"/>
+    <mergeCell ref="N21:P21"/>
+    <mergeCell ref="N23:P23"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AA11:AB11"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="N26:P26"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="N24:P24"/>
+    <mergeCell ref="E27:J27"/>
+    <mergeCell ref="E22:J22"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K2:P2"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AA17:AB17"/>
+    <mergeCell ref="AA18:AB18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="N13:P13"/>
     <mergeCell ref="AA20:AB20"/>
     <mergeCell ref="AA21:AB21"/>
     <mergeCell ref="AA22:AB22"/>
@@ -6849,120 +6943,26 @@
     <mergeCell ref="U11:V11"/>
     <mergeCell ref="AA23:AB23"/>
     <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AA17:AB17"/>
-    <mergeCell ref="AA18:AB18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="AA19:AB19"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="N27:P27"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="E28:J28"/>
-    <mergeCell ref="N24:P24"/>
-    <mergeCell ref="E27:J27"/>
-    <mergeCell ref="E22:J22"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K2:P2"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AA11:AB11"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B52:F52"/>
-    <mergeCell ref="AA7:AB7"/>
-    <mergeCell ref="AA28:AB28"/>
-    <mergeCell ref="AA12:AB12"/>
-    <mergeCell ref="AA13:AB13"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AA25:AB25"/>
-    <mergeCell ref="AA26:AB26"/>
-    <mergeCell ref="U27:V27"/>
-    <mergeCell ref="AA27:AB27"/>
-    <mergeCell ref="U12:V12"/>
-    <mergeCell ref="AA14:AB14"/>
-    <mergeCell ref="U28:V28"/>
-    <mergeCell ref="N17:P17"/>
-    <mergeCell ref="N19:P19"/>
-    <mergeCell ref="N20:P20"/>
-    <mergeCell ref="N21:P21"/>
-    <mergeCell ref="N23:P23"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D54:E55"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="T30:AC30"/>
+    <mergeCell ref="T31:AC31"/>
+    <mergeCell ref="T32:AC32"/>
+    <mergeCell ref="T33:AC33"/>
+    <mergeCell ref="T34:AC34"/>
+    <mergeCell ref="T35:AC35"/>
+    <mergeCell ref="T36:AC36"/>
+    <mergeCell ref="T37:AC37"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="S38:S39"/>
+    <mergeCell ref="T38:AC39"/>
+    <mergeCell ref="S44:S45"/>
+    <mergeCell ref="T44:AC45"/>
+    <mergeCell ref="T40:AC40"/>
+    <mergeCell ref="T41:AC41"/>
+    <mergeCell ref="T42:AC42"/>
+    <mergeCell ref="T43:AC43"/>
+    <mergeCell ref="T46:AC46"/>
+    <mergeCell ref="G45:J46"/>
+    <mergeCell ref="G39:J42"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7016,35 +7016,35 @@
       <c r="F2" s="103" t="s">
         <v>211</v>
       </c>
-      <c r="G2" s="192" t="s">
+      <c r="G2" s="200" t="s">
         <v>212</v>
       </c>
-      <c r="H2" s="193"/>
-      <c r="I2" s="193"/>
-      <c r="J2" s="194"/>
-      <c r="L2" s="284" t="s">
+      <c r="H2" s="201"/>
+      <c r="I2" s="201"/>
+      <c r="J2" s="202"/>
+      <c r="L2" s="292" t="s">
         <v>331</v>
       </c>
-      <c r="M2" s="285"/>
-      <c r="N2" s="285"/>
-      <c r="O2" s="286"/>
+      <c r="M2" s="293"/>
+      <c r="N2" s="293"/>
+      <c r="O2" s="294"/>
       <c r="P2" s="133"/>
-      <c r="Q2" s="287" t="s">
+      <c r="Q2" s="295" t="s">
         <v>291</v>
       </c>
-      <c r="R2" s="288"/>
-      <c r="S2" s="288"/>
-      <c r="T2" s="289"/>
+      <c r="R2" s="296"/>
+      <c r="S2" s="296"/>
+      <c r="T2" s="297"/>
       <c r="U2" s="133"/>
-      <c r="V2" s="277" t="s">
+      <c r="V2" s="289" t="s">
         <v>314</v>
       </c>
-      <c r="W2" s="278"/>
-      <c r="X2" s="278"/>
-      <c r="Y2" s="278"/>
-      <c r="Z2" s="278"/>
-      <c r="AA2" s="278"/>
-      <c r="AB2" s="279"/>
+      <c r="W2" s="290"/>
+      <c r="X2" s="290"/>
+      <c r="Y2" s="290"/>
+      <c r="Z2" s="290"/>
+      <c r="AA2" s="290"/>
+      <c r="AB2" s="291"/>
     </row>
     <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B3" s="90" t="s">
@@ -7066,11 +7066,11 @@
       <c r="G3" s="93" t="s">
         <v>213</v>
       </c>
-      <c r="H3" s="190" t="s">
+      <c r="H3" s="181" t="s">
         <v>217</v>
       </c>
-      <c r="I3" s="233"/>
-      <c r="J3" s="191"/>
+      <c r="I3" s="182"/>
+      <c r="J3" s="183"/>
       <c r="L3" s="145" t="s">
         <v>277</v>
       </c>
@@ -7109,11 +7109,11 @@
       <c r="Y3" s="171" t="s">
         <v>280</v>
       </c>
-      <c r="Z3" s="268" t="s">
+      <c r="Z3" s="280" t="s">
         <v>319</v>
       </c>
-      <c r="AA3" s="269"/>
-      <c r="AB3" s="270"/>
+      <c r="AA3" s="281"/>
+      <c r="AB3" s="282"/>
     </row>
     <row r="4" spans="2:28" ht="53.25" customHeight="1">
       <c r="B4" s="91" t="s">
@@ -7135,11 +7135,11 @@
       <c r="G4" s="94" t="s">
         <v>214</v>
       </c>
-      <c r="H4" s="216">
+      <c r="H4" s="184">
         <v>63</v>
       </c>
-      <c r="I4" s="217"/>
-      <c r="J4" s="218"/>
+      <c r="I4" s="185"/>
+      <c r="J4" s="186"/>
       <c r="L4" s="151" t="s">
         <v>246</v>
       </c>
@@ -7178,11 +7178,11 @@
       <c r="Y4" s="138" t="s">
         <v>317</v>
       </c>
-      <c r="Z4" s="271" t="s">
+      <c r="Z4" s="283" t="s">
         <v>320</v>
       </c>
-      <c r="AA4" s="272"/>
-      <c r="AB4" s="273"/>
+      <c r="AA4" s="284"/>
+      <c r="AB4" s="285"/>
     </row>
     <row r="5" spans="2:28" ht="47.25" customHeight="1">
       <c r="B5" s="91" t="s">
@@ -7204,11 +7204,11 @@
       <c r="G5" s="94" t="s">
         <v>215</v>
       </c>
-      <c r="H5" s="216">
+      <c r="H5" s="184">
         <v>31</v>
       </c>
-      <c r="I5" s="217"/>
-      <c r="J5" s="218"/>
+      <c r="I5" s="185"/>
+      <c r="J5" s="186"/>
       <c r="L5" s="149" t="s">
         <v>255</v>
       </c>
@@ -7247,9 +7247,9 @@
       <c r="Y5" s="135" t="s">
         <v>294</v>
       </c>
-      <c r="Z5" s="271"/>
-      <c r="AA5" s="272"/>
-      <c r="AB5" s="273"/>
+      <c r="Z5" s="283"/>
+      <c r="AA5" s="284"/>
+      <c r="AB5" s="285"/>
     </row>
     <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B6" s="108" t="s">
@@ -7271,11 +7271,11 @@
       <c r="G6" s="95" t="s">
         <v>216</v>
       </c>
-      <c r="H6" s="237">
+      <c r="H6" s="197">
         <v>7</v>
       </c>
-      <c r="I6" s="238"/>
-      <c r="J6" s="239"/>
+      <c r="I6" s="198"/>
+      <c r="J6" s="199"/>
       <c r="L6" s="152" t="s">
         <v>241</v>
       </c>
@@ -7314,9 +7314,9 @@
       <c r="Y6" s="144" t="s">
         <v>316</v>
       </c>
-      <c r="Z6" s="274"/>
-      <c r="AA6" s="275"/>
-      <c r="AB6" s="276"/>
+      <c r="Z6" s="286"/>
+      <c r="AA6" s="287"/>
+      <c r="AB6" s="288"/>
     </row>
     <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1">
       <c r="B7" s="90" t="s">
@@ -7338,12 +7338,12 @@
       <c r="G7" s="88" t="s">
         <v>274</v>
       </c>
-      <c r="H7" s="290" t="str">
+      <c r="H7" s="275" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12))</f>
         <v>E3FFF000</v>
       </c>
-      <c r="I7" s="291"/>
-      <c r="J7" s="292"/>
+      <c r="I7" s="276"/>
+      <c r="J7" s="277"/>
       <c r="L7" s="150" t="s">
         <v>266</v>
       </c>
@@ -7391,18 +7391,18 @@
       <c r="G8" s="88" t="s">
         <v>218</v>
       </c>
-      <c r="H8" s="290" t="str">
+      <c r="H8" s="275" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12)+4095)</f>
         <v>E3FFFFFF</v>
       </c>
-      <c r="I8" s="291"/>
-      <c r="J8" s="292"/>
-      <c r="L8" s="183" t="s">
+      <c r="I8" s="276"/>
+      <c r="J8" s="277"/>
+      <c r="L8" s="263" t="s">
         <v>333</v>
       </c>
-      <c r="M8" s="184"/>
-      <c r="N8" s="184"/>
-      <c r="O8" s="185"/>
+      <c r="M8" s="187"/>
+      <c r="N8" s="187"/>
+      <c r="O8" s="188"/>
       <c r="P8" s="133"/>
       <c r="Q8" s="164" t="s">
         <v>286</v>
@@ -7511,12 +7511,12 @@
       <c r="N11" s="133"/>
       <c r="O11" s="133"/>
       <c r="P11" s="133"/>
-      <c r="Q11" s="293" t="s">
+      <c r="Q11" s="298" t="s">
         <v>313</v>
       </c>
-      <c r="R11" s="294"/>
-      <c r="S11" s="294"/>
-      <c r="T11" s="295"/>
+      <c r="R11" s="299"/>
+      <c r="S11" s="299"/>
+      <c r="T11" s="300"/>
       <c r="U11" s="133"/>
     </row>
     <row r="12" spans="2:28" ht="44.25" customHeight="1" thickBot="1">
@@ -7668,12 +7668,12 @@
       <c r="F16" s="124" t="s">
         <v>233</v>
       </c>
-      <c r="G16" s="209" t="s">
+      <c r="G16" s="258" t="s">
         <v>271</v>
       </c>
-      <c r="H16" s="210"/>
-      <c r="I16" s="210"/>
-      <c r="J16" s="211"/>
+      <c r="H16" s="239"/>
+      <c r="I16" s="239"/>
+      <c r="J16" s="240"/>
       <c r="Q16" s="167" t="s">
         <v>307</v>
       </c>
@@ -7688,10 +7688,10 @@
       </c>
     </row>
     <row r="17" spans="2:20" ht="60.75" customHeight="1" thickBot="1">
-      <c r="B17" s="282" t="s">
+      <c r="B17" s="270" t="s">
         <v>234</v>
       </c>
-      <c r="C17" s="280" t="s">
+      <c r="C17" s="268" t="s">
         <v>235</v>
       </c>
       <c r="D17" s="125" t="s">
@@ -7703,12 +7703,12 @@
       <c r="F17" s="127" t="s">
         <v>237</v>
       </c>
-      <c r="G17" s="296" t="s">
+      <c r="G17" s="272" t="s">
         <v>272</v>
       </c>
-      <c r="H17" s="297"/>
-      <c r="I17" s="297"/>
-      <c r="J17" s="298"/>
+      <c r="H17" s="273"/>
+      <c r="I17" s="273"/>
+      <c r="J17" s="274"/>
       <c r="Q17" s="168" t="s">
         <v>310</v>
       </c>
@@ -7723,8 +7723,8 @@
       </c>
     </row>
     <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B18" s="299"/>
-      <c r="C18" s="300"/>
+      <c r="B18" s="278"/>
+      <c r="C18" s="279"/>
       <c r="D18" s="112" t="s">
         <v>238</v>
       </c>
@@ -7734,16 +7734,16 @@
       <c r="F18" s="115" t="s">
         <v>240</v>
       </c>
-      <c r="G18" s="290" t="s">
+      <c r="G18" s="275" t="s">
         <v>273</v>
       </c>
-      <c r="H18" s="291"/>
-      <c r="I18" s="291"/>
-      <c r="J18" s="292"/>
+      <c r="H18" s="276"/>
+      <c r="I18" s="276"/>
+      <c r="J18" s="277"/>
     </row>
     <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B19" s="283"/>
-      <c r="C19" s="281"/>
+      <c r="B19" s="271"/>
+      <c r="C19" s="269"/>
       <c r="D19" s="117" t="s">
         <v>241</v>
       </c>
@@ -7759,10 +7759,10 @@
       <c r="J19" s="15"/>
     </row>
     <row r="20" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B20" s="282" t="s">
+      <c r="B20" s="270" t="s">
         <v>244</v>
       </c>
-      <c r="C20" s="280" t="s">
+      <c r="C20" s="268" t="s">
         <v>245</v>
       </c>
       <c r="D20" s="125" t="s">
@@ -7780,8 +7780,8 @@
       <c r="J20" s="15"/>
     </row>
     <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B21" s="283"/>
-      <c r="C21" s="281"/>
+      <c r="B21" s="271"/>
+      <c r="C21" s="269"/>
       <c r="D21" s="117" t="s">
         <v>248</v>
       </c>
@@ -7797,10 +7797,10 @@
       <c r="J21" s="15"/>
     </row>
     <row r="22" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B22" s="282" t="s">
+      <c r="B22" s="270" t="s">
         <v>250</v>
       </c>
-      <c r="C22" s="280" t="s">
+      <c r="C22" s="268" t="s">
         <v>251</v>
       </c>
       <c r="D22" s="125" t="s">
@@ -7818,8 +7818,8 @@
       <c r="J22" s="15"/>
     </row>
     <row r="23" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B23" s="283"/>
-      <c r="C23" s="281"/>
+      <c r="B23" s="271"/>
+      <c r="C23" s="269"/>
       <c r="D23" s="117" t="s">
         <v>244</v>
       </c>
@@ -7835,10 +7835,10 @@
       <c r="J23" s="15"/>
     </row>
     <row r="24" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B24" s="282" t="s">
+      <c r="B24" s="270" t="s">
         <v>255</v>
       </c>
-      <c r="C24" s="280" t="s">
+      <c r="C24" s="268" t="s">
         <v>256</v>
       </c>
       <c r="D24" s="125" t="s">
@@ -7856,8 +7856,8 @@
       <c r="J24" s="15"/>
     </row>
     <row r="25" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B25" s="283"/>
-      <c r="C25" s="281"/>
+      <c r="B25" s="271"/>
+      <c r="C25" s="269"/>
       <c r="D25" s="117" t="s">
         <v>250</v>
       </c>
@@ -7894,10 +7894,10 @@
       <c r="J26" s="15"/>
     </row>
     <row r="27" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B27" s="282" t="s">
+      <c r="B27" s="270" t="s">
         <v>238</v>
       </c>
-      <c r="C27" s="280" t="s">
+      <c r="C27" s="268" t="s">
         <v>262</v>
       </c>
       <c r="D27" s="125" t="s">
@@ -7915,8 +7915,8 @@
       <c r="J27" s="15"/>
     </row>
     <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B28" s="283"/>
-      <c r="C28" s="281"/>
+      <c r="B28" s="271"/>
+      <c r="C28" s="269"/>
       <c r="D28" s="117" t="s">
         <v>255</v>
       </c>
@@ -7932,10 +7932,10 @@
       <c r="J28" s="15"/>
     </row>
     <row r="29" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B29" s="282" t="s">
+      <c r="B29" s="270" t="s">
         <v>266</v>
       </c>
-      <c r="C29" s="280" t="s">
+      <c r="C29" s="268" t="s">
         <v>267</v>
       </c>
       <c r="D29" s="125" t="s">
@@ -7953,8 +7953,8 @@
       <c r="J29" s="15"/>
     </row>
     <row r="30" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B30" s="283"/>
-      <c r="C30" s="281"/>
+      <c r="B30" s="271"/>
+      <c r="C30" s="269"/>
       <c r="D30" s="117" t="s">
         <v>259</v>
       </c>
@@ -7971,19 +7971,6 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C17:C19"/>
     <mergeCell ref="Z3:AB3"/>
     <mergeCell ref="Z4:AB6"/>
     <mergeCell ref="V2:AB2"/>
@@ -8000,6 +7987,19 @@
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="Q11:T11"/>
     <mergeCell ref="L8:O8"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="C17:C19"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Paso la prueba de subrutinas
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B41B6A3-20E6-4C62-B18F-6B7CADE52CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314EFB9C-60A5-4278-915E-6C5313FF5BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="339">
   <si>
     <t>OpCode</t>
   </si>
@@ -1347,9 +1347,6 @@
     </r>
   </si>
   <si>
-    <t>Intr 64</t>
-  </si>
-  <si>
     <t>int 32 / short 16 / char 8</t>
   </si>
   <si>
@@ -1357,6 +1354,9 @@
   </si>
   <si>
     <t>Bit 31 = Alta/Baja</t>
+  </si>
+  <si>
+    <t>PC 32</t>
   </si>
 </sst>
 </file>
@@ -2410,7 +2410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="301">
+  <cellXfs count="302">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2946,29 +2946,20 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2976,37 +2967,22 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3018,6 +2994,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3027,155 +3012,23 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3186,32 +3039,215 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -3225,6 +3261,42 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3232,15 +3304,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3249,68 +3312,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3624,62 +3627,62 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B2" s="224" t="s">
+      <c r="B2" s="234" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="233" t="s">
+      <c r="C2" s="249" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="234"/>
-      <c r="E2" s="235" t="s">
+      <c r="D2" s="250"/>
+      <c r="E2" s="251" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="235"/>
-      <c r="G2" s="236" t="s">
+      <c r="F2" s="251"/>
+      <c r="G2" s="252" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="235"/>
-      <c r="I2" s="235" t="s">
+      <c r="H2" s="251"/>
+      <c r="I2" s="251" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="235"/>
-      <c r="K2" s="237" t="s">
+      <c r="J2" s="251"/>
+      <c r="K2" s="253" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="235"/>
-      <c r="M2" s="235"/>
-      <c r="N2" s="235"/>
-      <c r="O2" s="235"/>
-      <c r="P2" s="238"/>
-      <c r="R2" s="243" t="s">
+      <c r="L2" s="251"/>
+      <c r="M2" s="251"/>
+      <c r="N2" s="251"/>
+      <c r="O2" s="251"/>
+      <c r="P2" s="254"/>
+      <c r="R2" s="230" t="s">
         <v>65</v>
       </c>
-      <c r="S2" s="180" t="s">
+      <c r="S2" s="227" t="s">
         <v>66</v>
       </c>
-      <c r="T2" s="247" t="s">
+      <c r="T2" s="220" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="248"/>
-      <c r="V2" s="248"/>
-      <c r="W2" s="248"/>
-      <c r="X2" s="248"/>
-      <c r="Y2" s="248"/>
-      <c r="Z2" s="248"/>
-      <c r="AA2" s="248"/>
-      <c r="AB2" s="248" t="s">
+      <c r="U2" s="221"/>
+      <c r="V2" s="221"/>
+      <c r="W2" s="221"/>
+      <c r="X2" s="221"/>
+      <c r="Y2" s="221"/>
+      <c r="Z2" s="221"/>
+      <c r="AA2" s="221"/>
+      <c r="AB2" s="221" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="248"/>
-      <c r="AD2" s="248"/>
-      <c r="AE2" s="248"/>
-      <c r="AF2" s="248"/>
-      <c r="AG2" s="248"/>
-      <c r="AH2" s="248"/>
-      <c r="AI2" s="249"/>
+      <c r="AC2" s="221"/>
+      <c r="AD2" s="221"/>
+      <c r="AE2" s="221"/>
+      <c r="AF2" s="221"/>
+      <c r="AG2" s="221"/>
+      <c r="AH2" s="221"/>
+      <c r="AI2" s="222"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B3" s="225"/>
+      <c r="B3" s="235"/>
       <c r="C3" s="16" t="s">
         <v>79</v>
       </c>
@@ -3704,21 +3707,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="230"/>
-      <c r="L3" s="231"/>
-      <c r="M3" s="231"/>
-      <c r="N3" s="231"/>
-      <c r="O3" s="231"/>
-      <c r="P3" s="232"/>
-      <c r="R3" s="244"/>
-      <c r="S3" s="241"/>
+      <c r="K3" s="205"/>
+      <c r="L3" s="248"/>
+      <c r="M3" s="248"/>
+      <c r="N3" s="248"/>
+      <c r="O3" s="248"/>
+      <c r="P3" s="206"/>
+      <c r="R3" s="231"/>
+      <c r="S3" s="228"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="211" t="s">
+      <c r="U3" s="258" t="s">
         <v>83</v>
       </c>
-      <c r="V3" s="211"/>
+      <c r="V3" s="258"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -3731,10 +3734,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="246" t="s">
+      <c r="AA3" s="219" t="s">
         <v>74</v>
       </c>
-      <c r="AB3" s="246"/>
+      <c r="AB3" s="219"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -3758,21 +3761,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B4" s="226"/>
+      <c r="B4" s="236"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="212" t="s">
+      <c r="E4" s="223" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="239"/>
-      <c r="G4" s="239"/>
-      <c r="H4" s="239"/>
-      <c r="I4" s="239"/>
-      <c r="J4" s="240"/>
+      <c r="F4" s="210"/>
+      <c r="G4" s="210"/>
+      <c r="H4" s="210"/>
+      <c r="I4" s="210"/>
+      <c r="J4" s="211"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -3782,20 +3785,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="212" t="s">
+      <c r="N4" s="223" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="239"/>
-      <c r="P4" s="240"/>
-      <c r="R4" s="245"/>
-      <c r="S4" s="242"/>
+      <c r="O4" s="210"/>
+      <c r="P4" s="211"/>
+      <c r="R4" s="232"/>
+      <c r="S4" s="229"/>
       <c r="T4" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="U4" s="212" t="s">
+      <c r="U4" s="223" t="s">
         <v>75</v>
       </c>
-      <c r="V4" s="213"/>
+      <c r="V4" s="224"/>
       <c r="W4" s="7" t="s">
         <v>71</v>
       </c>
@@ -3808,10 +3811,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="212" t="s">
+      <c r="AA4" s="223" t="s">
         <v>72</v>
       </c>
-      <c r="AB4" s="213"/>
+      <c r="AB4" s="224"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -3843,22 +3846,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="216"/>
-      <c r="F5" s="217"/>
-      <c r="G5" s="217"/>
-      <c r="H5" s="217"/>
-      <c r="I5" s="217"/>
-      <c r="J5" s="218"/>
+      <c r="E5" s="255"/>
+      <c r="F5" s="256"/>
+      <c r="G5" s="256"/>
+      <c r="H5" s="256"/>
+      <c r="I5" s="256"/>
+      <c r="J5" s="257"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="181" t="s">
+      <c r="N5" s="190" t="s">
         <v>51</v>
       </c>
-      <c r="O5" s="182"/>
-      <c r="P5" s="183"/>
+      <c r="O5" s="233"/>
+      <c r="P5" s="191"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -3868,10 +3871,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="214" t="s">
+      <c r="U5" s="225" t="s">
         <v>73</v>
       </c>
-      <c r="V5" s="215"/>
+      <c r="V5" s="226"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -3884,10 +3887,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="214" t="s">
+      <c r="AA5" s="225" t="s">
         <v>73</v>
       </c>
-      <c r="AB5" s="215"/>
+      <c r="AB5" s="226"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -3919,12 +3922,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="223"/>
-      <c r="F6" s="220"/>
-      <c r="G6" s="220"/>
-      <c r="H6" s="220"/>
-      <c r="I6" s="220"/>
-      <c r="J6" s="221"/>
+      <c r="E6" s="246"/>
+      <c r="F6" s="241"/>
+      <c r="G6" s="241"/>
+      <c r="H6" s="241"/>
+      <c r="I6" s="241"/>
+      <c r="J6" s="242"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -3932,11 +3935,11 @@
         <v>155</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="184" t="s">
+      <c r="N6" s="216" t="s">
         <v>95</v>
       </c>
-      <c r="O6" s="185"/>
-      <c r="P6" s="186"/>
+      <c r="O6" s="217"/>
+      <c r="P6" s="218"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -3946,10 +3949,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="209" t="s">
+      <c r="U6" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V6" s="210"/>
+      <c r="V6" s="213"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -3962,10 +3965,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="209" t="s">
+      <c r="AA6" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB6" s="210"/>
+      <c r="AB6" s="213"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -3993,7 +3996,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D7" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4008,9 +4011,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="219"/>
-      <c r="I7" s="220"/>
-      <c r="J7" s="221"/>
+      <c r="H7" s="240"/>
+      <c r="I7" s="241"/>
+      <c r="J7" s="242"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -4018,11 +4021,11 @@
       <c r="M7" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N7" s="184" t="s">
+      <c r="N7" s="216" t="s">
         <v>52</v>
       </c>
-      <c r="O7" s="185"/>
-      <c r="P7" s="186"/>
+      <c r="O7" s="217"/>
+      <c r="P7" s="218"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -4032,10 +4035,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="209" t="s">
+      <c r="U7" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V7" s="210"/>
+      <c r="V7" s="213"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -4048,10 +4051,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="209" t="s">
+      <c r="AA7" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB7" s="210"/>
+      <c r="AB7" s="213"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -4079,7 +4082,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D8" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4094,9 +4097,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="219"/>
-      <c r="I8" s="220"/>
-      <c r="J8" s="221"/>
+      <c r="H8" s="240"/>
+      <c r="I8" s="241"/>
+      <c r="J8" s="242"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -4104,11 +4107,11 @@
       <c r="M8" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N8" s="184" t="s">
+      <c r="N8" s="216" t="s">
         <v>53</v>
       </c>
-      <c r="O8" s="185"/>
-      <c r="P8" s="186"/>
+      <c r="O8" s="217"/>
+      <c r="P8" s="218"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -4118,10 +4121,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="209" t="s">
+      <c r="U8" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V8" s="210"/>
+      <c r="V8" s="213"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -4134,10 +4137,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="209" t="s">
+      <c r="AA8" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB8" s="210"/>
+      <c r="AB8" s="213"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -4165,7 +4168,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D9" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4180,9 +4183,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="219"/>
-      <c r="I9" s="220"/>
-      <c r="J9" s="221"/>
+      <c r="H9" s="240"/>
+      <c r="I9" s="241"/>
+      <c r="J9" s="242"/>
       <c r="K9" s="37" t="s">
         <v>47</v>
       </c>
@@ -4190,11 +4193,11 @@
       <c r="M9" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N9" s="184" t="s">
+      <c r="N9" s="216" t="s">
         <v>54</v>
       </c>
-      <c r="O9" s="185"/>
-      <c r="P9" s="186"/>
+      <c r="O9" s="217"/>
+      <c r="P9" s="218"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -4204,10 +4207,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="209" t="s">
+      <c r="U9" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V9" s="210"/>
+      <c r="V9" s="213"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -4220,10 +4223,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="209" t="s">
+      <c r="AA9" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB9" s="210"/>
+      <c r="AB9" s="213"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -4251,7 +4254,7 @@
         <v>5</v>
       </c>
       <c r="C10" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D10" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4266,9 +4269,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="219"/>
-      <c r="I10" s="220"/>
-      <c r="J10" s="221"/>
+      <c r="H10" s="240"/>
+      <c r="I10" s="241"/>
+      <c r="J10" s="242"/>
       <c r="K10" s="37" t="s">
         <v>48</v>
       </c>
@@ -4276,11 +4279,11 @@
       <c r="M10" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N10" s="184" t="s">
+      <c r="N10" s="216" t="s">
         <v>55</v>
       </c>
-      <c r="O10" s="185"/>
-      <c r="P10" s="186"/>
+      <c r="O10" s="217"/>
+      <c r="P10" s="218"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -4290,10 +4293,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="209" t="s">
+      <c r="U10" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V10" s="210"/>
+      <c r="V10" s="213"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -4306,10 +4309,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="209" t="s">
+      <c r="AA10" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB10" s="210"/>
+      <c r="AB10" s="213"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -4337,7 +4340,7 @@
         <v>6</v>
       </c>
       <c r="C11" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D11" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4352,9 +4355,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="219"/>
-      <c r="I11" s="220"/>
-      <c r="J11" s="221"/>
+      <c r="H11" s="240"/>
+      <c r="I11" s="241"/>
+      <c r="J11" s="242"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -4362,11 +4365,11 @@
       <c r="M11" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N11" s="184" t="s">
+      <c r="N11" s="216" t="s">
         <v>56</v>
       </c>
-      <c r="O11" s="185"/>
-      <c r="P11" s="186"/>
+      <c r="O11" s="217"/>
+      <c r="P11" s="218"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -4376,10 +4379,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="209" t="s">
+      <c r="U11" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V11" s="210"/>
+      <c r="V11" s="213"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -4392,10 +4395,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="209" t="s">
+      <c r="AA11" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB11" s="210"/>
+      <c r="AB11" s="213"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -4423,7 +4426,7 @@
         <v>7</v>
       </c>
       <c r="C12" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D12" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4438,9 +4441,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="219"/>
-      <c r="I12" s="220"/>
-      <c r="J12" s="221"/>
+      <c r="H12" s="240"/>
+      <c r="I12" s="241"/>
+      <c r="J12" s="242"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -4448,11 +4451,11 @@
       <c r="M12" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N12" s="184" t="s">
+      <c r="N12" s="216" t="s">
         <v>57</v>
       </c>
-      <c r="O12" s="185"/>
-      <c r="P12" s="186"/>
+      <c r="O12" s="217"/>
+      <c r="P12" s="218"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -4462,10 +4465,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="209" t="s">
+      <c r="U12" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V12" s="210"/>
+      <c r="V12" s="213"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -4478,10 +4481,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="209" t="s">
+      <c r="AA12" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB12" s="210"/>
+      <c r="AB12" s="213"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -4509,7 +4512,7 @@
         <v>8</v>
       </c>
       <c r="C13" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D13" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4524,9 +4527,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="219"/>
-      <c r="I13" s="220"/>
-      <c r="J13" s="221"/>
+      <c r="H13" s="240"/>
+      <c r="I13" s="241"/>
+      <c r="J13" s="242"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -4534,11 +4537,11 @@
       <c r="M13" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N13" s="184" t="s">
+      <c r="N13" s="216" t="s">
         <v>58</v>
       </c>
-      <c r="O13" s="185"/>
-      <c r="P13" s="186"/>
+      <c r="O13" s="217"/>
+      <c r="P13" s="218"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -4548,10 +4551,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="209" t="s">
+      <c r="U13" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V13" s="210"/>
+      <c r="V13" s="213"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -4564,10 +4567,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="209" t="s">
+      <c r="AA13" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB13" s="210"/>
+      <c r="AB13" s="213"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -4595,7 +4598,7 @@
         <v>9</v>
       </c>
       <c r="C14" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D14" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4610,9 +4613,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="219"/>
-      <c r="I14" s="220"/>
-      <c r="J14" s="221"/>
+      <c r="H14" s="240"/>
+      <c r="I14" s="241"/>
+      <c r="J14" s="242"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -4620,11 +4623,11 @@
       <c r="M14" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N14" s="184" t="s">
+      <c r="N14" s="216" t="s">
         <v>59</v>
       </c>
-      <c r="O14" s="185"/>
-      <c r="P14" s="186"/>
+      <c r="O14" s="217"/>
+      <c r="P14" s="218"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -4634,10 +4637,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="209" t="s">
+      <c r="U14" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V14" s="210"/>
+      <c r="V14" s="213"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -4650,10 +4653,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="209" t="s">
+      <c r="AA14" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB14" s="210"/>
+      <c r="AB14" s="213"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -4681,7 +4684,7 @@
         <v>10</v>
       </c>
       <c r="C15" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D15" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4696,9 +4699,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="219"/>
-      <c r="I15" s="220"/>
-      <c r="J15" s="221"/>
+      <c r="H15" s="240"/>
+      <c r="I15" s="241"/>
+      <c r="J15" s="242"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -4706,11 +4709,11 @@
       <c r="M15" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N15" s="184" t="s">
+      <c r="N15" s="216" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="185"/>
-      <c r="P15" s="186"/>
+      <c r="O15" s="217"/>
+      <c r="P15" s="218"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -4720,10 +4723,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="209" t="s">
+      <c r="U15" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V15" s="210"/>
+      <c r="V15" s="213"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -4736,10 +4739,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="209" t="s">
+      <c r="AA15" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB15" s="210"/>
+      <c r="AB15" s="213"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -4767,7 +4770,7 @@
         <v>11</v>
       </c>
       <c r="C16" s="178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D16" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4776,21 +4779,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="219"/>
-      <c r="G16" s="220"/>
-      <c r="H16" s="220"/>
-      <c r="I16" s="220"/>
-      <c r="J16" s="221"/>
+      <c r="F16" s="240"/>
+      <c r="G16" s="241"/>
+      <c r="H16" s="241"/>
+      <c r="I16" s="241"/>
+      <c r="J16" s="242"/>
       <c r="K16" s="40" t="s">
         <v>49</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="184" t="s">
+      <c r="N16" s="216" t="s">
         <v>50</v>
       </c>
-      <c r="O16" s="185"/>
-      <c r="P16" s="186"/>
+      <c r="O16" s="217"/>
+      <c r="P16" s="218"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -4800,10 +4803,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="209" t="s">
+      <c r="U16" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V16" s="210"/>
+      <c r="V16" s="213"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -4816,10 +4819,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="209" t="s">
+      <c r="AA16" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB16" s="210"/>
+      <c r="AB16" s="213"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -4847,7 +4850,7 @@
         <v>12</v>
       </c>
       <c r="C17" s="178" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D17" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4857,22 +4860,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="222" t="s">
+      <c r="G17" s="247" t="s">
         <v>76</v>
       </c>
-      <c r="H17" s="185"/>
-      <c r="I17" s="185"/>
-      <c r="J17" s="186"/>
+      <c r="H17" s="217"/>
+      <c r="I17" s="217"/>
+      <c r="J17" s="218"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="184" t="s">
+      <c r="N17" s="216" t="s">
         <v>64</v>
       </c>
-      <c r="O17" s="185"/>
-      <c r="P17" s="186"/>
+      <c r="O17" s="217"/>
+      <c r="P17" s="218"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -4882,10 +4885,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="209" t="s">
+      <c r="U17" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V17" s="210"/>
+      <c r="V17" s="213"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -4898,10 +4901,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="209" t="s">
+      <c r="AA17" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB17" s="210"/>
+      <c r="AB17" s="213"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -4929,9 +4932,9 @@
         <v>13</v>
       </c>
       <c r="C18" s="178" t="s">
-        <v>337</v>
-      </c>
-      <c r="D18" s="23" t="str">
+        <v>336</v>
+      </c>
+      <c r="D18" s="301" t="str">
         <f t="shared" si="0"/>
         <v>01101</v>
       </c>
@@ -4939,12 +4942,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="222" t="s">
+      <c r="G18" s="247" t="s">
         <v>76</v>
       </c>
-      <c r="H18" s="185"/>
-      <c r="I18" s="185"/>
-      <c r="J18" s="186"/>
+      <c r="H18" s="217"/>
+      <c r="I18" s="217"/>
+      <c r="J18" s="218"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -4952,11 +4955,11 @@
       <c r="M18" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="N18" s="184" t="s">
+      <c r="N18" s="216" t="s">
         <v>61</v>
       </c>
-      <c r="O18" s="185"/>
-      <c r="P18" s="186"/>
+      <c r="O18" s="217"/>
+      <c r="P18" s="218"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -4966,10 +4969,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="209" t="s">
+      <c r="U18" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V18" s="210"/>
+      <c r="V18" s="213"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -4982,10 +4985,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="209" t="s">
+      <c r="AA18" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB18" s="210"/>
+      <c r="AB18" s="213"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -5012,9 +5015,7 @@
       <c r="B19" s="2">
         <v>14</v>
       </c>
-      <c r="C19" s="38" t="s">
-        <v>335</v>
-      </c>
+      <c r="C19" s="48"/>
       <c r="D19" s="23" t="str">
         <f t="shared" si="0"/>
         <v>01110</v>
@@ -5023,20 +5024,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="219"/>
-      <c r="H19" s="220"/>
-      <c r="I19" s="220"/>
-      <c r="J19" s="221"/>
+      <c r="G19" s="240"/>
+      <c r="H19" s="241"/>
+      <c r="I19" s="241"/>
+      <c r="J19" s="242"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="184" t="s">
+      <c r="N19" s="216" t="s">
         <v>93</v>
       </c>
-      <c r="O19" s="185"/>
-      <c r="P19" s="186"/>
+      <c r="O19" s="217"/>
+      <c r="P19" s="218"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -5046,10 +5047,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="209" t="s">
+      <c r="U19" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V19" s="210"/>
+      <c r="V19" s="213"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -5062,10 +5063,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="209" t="s">
+      <c r="AA19" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB19" s="210"/>
+      <c r="AB19" s="213"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -5092,9 +5093,7 @@
       <c r="B20" s="2">
         <v>15</v>
       </c>
-      <c r="C20" s="38" t="s">
-        <v>335</v>
-      </c>
+      <c r="C20" s="48"/>
       <c r="D20" s="23" t="str">
         <f t="shared" si="0"/>
         <v>01111</v>
@@ -5105,20 +5104,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="219"/>
-      <c r="H20" s="220"/>
-      <c r="I20" s="220"/>
-      <c r="J20" s="221"/>
+      <c r="G20" s="240"/>
+      <c r="H20" s="241"/>
+      <c r="I20" s="241"/>
+      <c r="J20" s="242"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="184" t="s">
+      <c r="N20" s="216" t="s">
         <v>94</v>
       </c>
-      <c r="O20" s="185"/>
-      <c r="P20" s="186"/>
+      <c r="O20" s="217"/>
+      <c r="P20" s="218"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -5128,10 +5127,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="209" t="s">
+      <c r="U20" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V20" s="210"/>
+      <c r="V20" s="213"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -5144,10 +5143,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="209" t="s">
+      <c r="AA20" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB20" s="210"/>
+      <c r="AB20" s="213"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -5175,7 +5174,7 @@
         <v>16</v>
       </c>
       <c r="C21" s="38" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D21" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5185,20 +5184,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="219"/>
-      <c r="H21" s="220"/>
-      <c r="I21" s="220"/>
-      <c r="J21" s="221"/>
+      <c r="G21" s="240"/>
+      <c r="H21" s="241"/>
+      <c r="I21" s="241"/>
+      <c r="J21" s="242"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="184" t="s">
+      <c r="N21" s="216" t="s">
         <v>62</v>
       </c>
-      <c r="O21" s="185"/>
-      <c r="P21" s="186"/>
+      <c r="O21" s="217"/>
+      <c r="P21" s="218"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -5208,10 +5207,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="209" t="s">
+      <c r="U21" s="212" t="s">
         <v>96</v>
       </c>
-      <c r="V21" s="210"/>
+      <c r="V21" s="213"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -5224,10 +5223,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="209" t="s">
+      <c r="AA21" s="212" t="s">
         <v>98</v>
       </c>
-      <c r="AB21" s="210"/>
+      <c r="AB21" s="213"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -5255,28 +5254,28 @@
         <v>17</v>
       </c>
       <c r="C22" s="38" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D22" s="23" t="str">
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="223"/>
-      <c r="F22" s="220"/>
-      <c r="G22" s="220"/>
-      <c r="H22" s="220"/>
-      <c r="I22" s="220"/>
-      <c r="J22" s="221"/>
+      <c r="E22" s="246"/>
+      <c r="F22" s="241"/>
+      <c r="G22" s="241"/>
+      <c r="H22" s="241"/>
+      <c r="I22" s="241"/>
+      <c r="J22" s="242"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="184" t="s">
+      <c r="N22" s="216" t="s">
         <v>63</v>
       </c>
-      <c r="O22" s="185"/>
-      <c r="P22" s="186"/>
+      <c r="O22" s="217"/>
+      <c r="P22" s="218"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -5286,10 +5285,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="209" t="s">
+      <c r="U22" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V22" s="210"/>
+      <c r="V22" s="213"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -5302,10 +5301,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="209" t="s">
+      <c r="AA22" s="212" t="s">
         <v>96</v>
       </c>
-      <c r="AB22" s="210"/>
+      <c r="AB22" s="213"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -5333,7 +5332,7 @@
         <v>18</v>
       </c>
       <c r="C23" s="38" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D23" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5345,22 +5344,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="222" t="s">
+      <c r="G23" s="247" t="s">
         <v>77</v>
       </c>
-      <c r="H23" s="185"/>
-      <c r="I23" s="185"/>
-      <c r="J23" s="186"/>
+      <c r="H23" s="217"/>
+      <c r="I23" s="217"/>
+      <c r="J23" s="218"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="184" t="s">
+      <c r="N23" s="216" t="s">
         <v>82</v>
       </c>
-      <c r="O23" s="185"/>
-      <c r="P23" s="186"/>
+      <c r="O23" s="217"/>
+      <c r="P23" s="218"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -5370,10 +5369,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="209" t="s">
+      <c r="U23" s="212" t="s">
         <v>97</v>
       </c>
-      <c r="V23" s="210"/>
+      <c r="V23" s="213"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -5386,10 +5385,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="209" t="s">
+      <c r="AA23" s="212" t="s">
         <v>96</v>
       </c>
-      <c r="AB23" s="210"/>
+      <c r="AB23" s="213"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -5417,7 +5416,7 @@
         <v>19</v>
       </c>
       <c r="C24" s="38" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D24" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5429,22 +5428,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="222" t="s">
+      <c r="G24" s="247" t="s">
         <v>77</v>
       </c>
-      <c r="H24" s="185"/>
-      <c r="I24" s="185"/>
-      <c r="J24" s="186"/>
+      <c r="H24" s="217"/>
+      <c r="I24" s="217"/>
+      <c r="J24" s="218"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="184" t="s">
+      <c r="N24" s="216" t="s">
         <v>81</v>
       </c>
-      <c r="O24" s="185"/>
-      <c r="P24" s="186"/>
+      <c r="O24" s="217"/>
+      <c r="P24" s="218"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -5454,10 +5453,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="209" t="s">
+      <c r="U24" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V24" s="210"/>
+      <c r="V24" s="213"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -5470,10 +5469,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="209" t="s">
+      <c r="AA24" s="212" t="s">
         <v>98</v>
       </c>
-      <c r="AB24" s="210"/>
+      <c r="AB24" s="213"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -5511,10 +5510,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="219"/>
-      <c r="H25" s="220"/>
-      <c r="I25" s="220"/>
-      <c r="J25" s="221"/>
+      <c r="G25" s="240"/>
+      <c r="H25" s="241"/>
+      <c r="I25" s="241"/>
+      <c r="J25" s="242"/>
       <c r="K25" s="49" t="s">
         <v>39</v>
       </c>
@@ -5522,11 +5521,11 @@
         <v>155</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="184" t="s">
+      <c r="N25" s="216" t="s">
         <v>41</v>
       </c>
-      <c r="O25" s="185"/>
-      <c r="P25" s="186"/>
+      <c r="O25" s="217"/>
+      <c r="P25" s="218"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -5536,10 +5535,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="209" t="s">
+      <c r="U25" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V25" s="210"/>
+      <c r="V25" s="213"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -5552,10 +5551,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="209" t="s">
+      <c r="AA25" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB25" s="210"/>
+      <c r="AB25" s="213"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -5593,10 +5592,10 @@
       <c r="F26" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="G26" s="219"/>
-      <c r="H26" s="220"/>
-      <c r="I26" s="220"/>
-      <c r="J26" s="221"/>
+      <c r="G26" s="240"/>
+      <c r="H26" s="241"/>
+      <c r="I26" s="241"/>
+      <c r="J26" s="242"/>
       <c r="K26" s="31" t="s">
         <v>40</v>
       </c>
@@ -5604,11 +5603,11 @@
         <v>155</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="184" t="s">
+      <c r="N26" s="216" t="s">
         <v>42</v>
       </c>
-      <c r="O26" s="185"/>
-      <c r="P26" s="186"/>
+      <c r="O26" s="217"/>
+      <c r="P26" s="218"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -5618,10 +5617,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="209" t="s">
+      <c r="U26" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V26" s="210"/>
+      <c r="V26" s="213"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -5634,10 +5633,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="209" t="s">
+      <c r="AA26" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB26" s="210"/>
+      <c r="AB26" s="213"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -5669,22 +5668,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="223"/>
-      <c r="F27" s="220"/>
-      <c r="G27" s="220"/>
-      <c r="H27" s="220"/>
-      <c r="I27" s="220"/>
-      <c r="J27" s="221"/>
+      <c r="E27" s="246"/>
+      <c r="F27" s="241"/>
+      <c r="G27" s="241"/>
+      <c r="H27" s="241"/>
+      <c r="I27" s="241"/>
+      <c r="J27" s="242"/>
       <c r="K27" s="25" t="s">
         <v>44</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="184" t="s">
+      <c r="N27" s="216" t="s">
         <v>46</v>
       </c>
-      <c r="O27" s="185"/>
-      <c r="P27" s="186"/>
+      <c r="O27" s="217"/>
+      <c r="P27" s="218"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -5694,10 +5693,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="209" t="s">
+      <c r="U27" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V27" s="210"/>
+      <c r="V27" s="213"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -5710,10 +5709,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="209" t="s">
+      <c r="AA27" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB27" s="210"/>
+      <c r="AB27" s="213"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -5745,12 +5744,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="227"/>
-      <c r="F28" s="228"/>
-      <c r="G28" s="228"/>
-      <c r="H28" s="228"/>
-      <c r="I28" s="228"/>
-      <c r="J28" s="229"/>
+      <c r="E28" s="243"/>
+      <c r="F28" s="244"/>
+      <c r="G28" s="244"/>
+      <c r="H28" s="244"/>
+      <c r="I28" s="244"/>
+      <c r="J28" s="245"/>
       <c r="K28" s="52" t="s">
         <v>45</v>
       </c>
@@ -5758,11 +5757,11 @@
         <v>155</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="197" t="s">
+      <c r="N28" s="237" t="s">
         <v>92</v>
       </c>
-      <c r="O28" s="198"/>
-      <c r="P28" s="199"/>
+      <c r="O28" s="238"/>
+      <c r="P28" s="239"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -5772,10 +5771,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="259" t="s">
+      <c r="U28" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="V28" s="260"/>
+      <c r="V28" s="215"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -5788,10 +5787,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="259" t="s">
+      <c r="AA28" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="AB28" s="260"/>
+      <c r="AB28" s="215"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -5868,18 +5867,18 @@
       <c r="S30" s="75" t="s">
         <v>156</v>
       </c>
-      <c r="T30" s="179" t="s">
+      <c r="T30" s="259" t="s">
         <v>157</v>
       </c>
-      <c r="U30" s="179"/>
-      <c r="V30" s="179"/>
-      <c r="W30" s="179"/>
-      <c r="X30" s="179"/>
-      <c r="Y30" s="179"/>
-      <c r="Z30" s="179"/>
-      <c r="AA30" s="179"/>
-      <c r="AB30" s="179"/>
-      <c r="AC30" s="180"/>
+      <c r="U30" s="259"/>
+      <c r="V30" s="259"/>
+      <c r="W30" s="259"/>
+      <c r="X30" s="259"/>
+      <c r="Y30" s="259"/>
+      <c r="Z30" s="259"/>
+      <c r="AA30" s="259"/>
+      <c r="AB30" s="259"/>
+      <c r="AC30" s="227"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B31" s="67" t="s">
@@ -5920,18 +5919,18 @@
       <c r="S31" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="T31" s="181" t="s">
+      <c r="T31" s="190" t="s">
         <v>162</v>
       </c>
-      <c r="U31" s="182"/>
-      <c r="V31" s="182"/>
-      <c r="W31" s="182"/>
-      <c r="X31" s="182"/>
-      <c r="Y31" s="182"/>
-      <c r="Z31" s="182"/>
-      <c r="AA31" s="182"/>
-      <c r="AB31" s="182"/>
-      <c r="AC31" s="183"/>
+      <c r="U31" s="233"/>
+      <c r="V31" s="233"/>
+      <c r="W31" s="233"/>
+      <c r="X31" s="233"/>
+      <c r="Y31" s="233"/>
+      <c r="Z31" s="233"/>
+      <c r="AA31" s="233"/>
+      <c r="AB31" s="233"/>
+      <c r="AC31" s="191"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B32" s="4" t="s">
@@ -5955,18 +5954,18 @@
       <c r="S32" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="T32" s="184" t="s">
+      <c r="T32" s="216" t="s">
         <v>163</v>
       </c>
-      <c r="U32" s="185"/>
-      <c r="V32" s="185"/>
-      <c r="W32" s="185"/>
-      <c r="X32" s="185"/>
-      <c r="Y32" s="185"/>
-      <c r="Z32" s="185"/>
-      <c r="AA32" s="185"/>
-      <c r="AB32" s="185"/>
-      <c r="AC32" s="186"/>
+      <c r="U32" s="217"/>
+      <c r="V32" s="217"/>
+      <c r="W32" s="217"/>
+      <c r="X32" s="217"/>
+      <c r="Y32" s="217"/>
+      <c r="Z32" s="217"/>
+      <c r="AA32" s="217"/>
+      <c r="AB32" s="217"/>
+      <c r="AC32" s="218"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
       <c r="H33" s="84" t="s">
@@ -6002,31 +6001,31 @@
       <c r="S33" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="T33" s="184" t="s">
+      <c r="T33" s="216" t="s">
         <v>164</v>
       </c>
-      <c r="U33" s="185"/>
-      <c r="V33" s="185"/>
-      <c r="W33" s="185"/>
-      <c r="X33" s="185"/>
-      <c r="Y33" s="185"/>
-      <c r="Z33" s="185"/>
-      <c r="AA33" s="185"/>
-      <c r="AB33" s="185"/>
-      <c r="AC33" s="186"/>
+      <c r="U33" s="217"/>
+      <c r="V33" s="217"/>
+      <c r="W33" s="217"/>
+      <c r="X33" s="217"/>
+      <c r="Y33" s="217"/>
+      <c r="Z33" s="217"/>
+      <c r="AA33" s="217"/>
+      <c r="AB33" s="217"/>
+      <c r="AC33" s="218"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B34" s="256" t="s">
+      <c r="B34" s="207" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="230" t="s">
+      <c r="C34" s="205" t="s">
         <v>114</v>
       </c>
-      <c r="D34" s="232"/>
-      <c r="E34" s="230" t="s">
+      <c r="D34" s="206"/>
+      <c r="E34" s="205" t="s">
         <v>115</v>
       </c>
-      <c r="F34" s="232"/>
+      <c r="F34" s="206"/>
       <c r="H34" s="77" t="s">
         <v>65</v>
       </c>
@@ -6052,21 +6051,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="184" t="s">
+      <c r="T34" s="216" t="s">
         <v>165</v>
       </c>
-      <c r="U34" s="185"/>
-      <c r="V34" s="185"/>
-      <c r="W34" s="185"/>
-      <c r="X34" s="185"/>
-      <c r="Y34" s="185"/>
-      <c r="Z34" s="185"/>
-      <c r="AA34" s="185"/>
-      <c r="AB34" s="185"/>
-      <c r="AC34" s="186"/>
+      <c r="U34" s="217"/>
+      <c r="V34" s="217"/>
+      <c r="W34" s="217"/>
+      <c r="X34" s="217"/>
+      <c r="Y34" s="217"/>
+      <c r="Z34" s="217"/>
+      <c r="AA34" s="217"/>
+      <c r="AB34" s="217"/>
+      <c r="AC34" s="218"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B35" s="257"/>
+      <c r="B35" s="208"/>
       <c r="C35" s="64" t="s">
         <v>99</v>
       </c>
@@ -6085,18 +6084,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="184" t="s">
+      <c r="T35" s="216" t="s">
         <v>166</v>
       </c>
-      <c r="U35" s="185"/>
-      <c r="V35" s="185"/>
-      <c r="W35" s="185"/>
-      <c r="X35" s="185"/>
-      <c r="Y35" s="185"/>
-      <c r="Z35" s="185"/>
-      <c r="AA35" s="185"/>
-      <c r="AB35" s="185"/>
-      <c r="AC35" s="186"/>
+      <c r="U35" s="217"/>
+      <c r="V35" s="217"/>
+      <c r="W35" s="217"/>
+      <c r="X35" s="217"/>
+      <c r="Y35" s="217"/>
+      <c r="Z35" s="217"/>
+      <c r="AA35" s="217"/>
+      <c r="AB35" s="217"/>
+      <c r="AC35" s="218"/>
     </row>
     <row r="36" spans="2:29">
       <c r="B36" s="1">
@@ -6120,18 +6119,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="184" t="s">
+      <c r="T36" s="216" t="s">
         <v>167</v>
       </c>
-      <c r="U36" s="185"/>
-      <c r="V36" s="185"/>
-      <c r="W36" s="185"/>
-      <c r="X36" s="185"/>
-      <c r="Y36" s="185"/>
-      <c r="Z36" s="185"/>
-      <c r="AA36" s="185"/>
-      <c r="AB36" s="185"/>
-      <c r="AC36" s="186"/>
+      <c r="U36" s="217"/>
+      <c r="V36" s="217"/>
+      <c r="W36" s="217"/>
+      <c r="X36" s="217"/>
+      <c r="Y36" s="217"/>
+      <c r="Z36" s="217"/>
+      <c r="AA36" s="217"/>
+      <c r="AB36" s="217"/>
+      <c r="AC36" s="218"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1">
       <c r="B37" s="2">
@@ -6156,18 +6155,18 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="184" t="s">
+      <c r="T37" s="216" t="s">
         <v>194</v>
       </c>
-      <c r="U37" s="185"/>
-      <c r="V37" s="185"/>
-      <c r="W37" s="185"/>
-      <c r="X37" s="185"/>
-      <c r="Y37" s="185"/>
-      <c r="Z37" s="185"/>
-      <c r="AA37" s="185"/>
-      <c r="AB37" s="185"/>
-      <c r="AC37" s="186"/>
+      <c r="U37" s="217"/>
+      <c r="V37" s="217"/>
+      <c r="W37" s="217"/>
+      <c r="X37" s="217"/>
+      <c r="Y37" s="217"/>
+      <c r="Z37" s="217"/>
+      <c r="AA37" s="217"/>
+      <c r="AB37" s="217"/>
+      <c r="AC37" s="218"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1">
       <c r="B38" s="2">
@@ -6188,21 +6187,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="189" t="s">
+      <c r="S38" s="260" t="s">
         <v>72</v>
       </c>
-      <c r="T38" s="191" t="s">
+      <c r="T38" s="262" t="s">
         <v>168</v>
       </c>
-      <c r="U38" s="192"/>
-      <c r="V38" s="192"/>
-      <c r="W38" s="192"/>
-      <c r="X38" s="192"/>
-      <c r="Y38" s="192"/>
-      <c r="Z38" s="192"/>
-      <c r="AA38" s="192"/>
-      <c r="AB38" s="192"/>
-      <c r="AC38" s="193"/>
+      <c r="U38" s="263"/>
+      <c r="V38" s="263"/>
+      <c r="W38" s="263"/>
+      <c r="X38" s="263"/>
+      <c r="Y38" s="263"/>
+      <c r="Z38" s="263"/>
+      <c r="AA38" s="263"/>
+      <c r="AB38" s="263"/>
+      <c r="AC38" s="264"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1">
       <c r="B39" s="2">
@@ -6220,26 +6219,26 @@
       <c r="F39" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G39" s="200" t="s">
+      <c r="G39" s="192" t="s">
         <v>181</v>
       </c>
-      <c r="H39" s="201"/>
-      <c r="I39" s="201"/>
-      <c r="J39" s="202"/>
+      <c r="H39" s="193"/>
+      <c r="I39" s="193"/>
+      <c r="J39" s="194"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="190"/>
-      <c r="T39" s="194"/>
-      <c r="U39" s="195"/>
-      <c r="V39" s="195"/>
-      <c r="W39" s="195"/>
-      <c r="X39" s="195"/>
-      <c r="Y39" s="195"/>
-      <c r="Z39" s="195"/>
-      <c r="AA39" s="195"/>
-      <c r="AB39" s="195"/>
-      <c r="AC39" s="196"/>
+      <c r="S39" s="261"/>
+      <c r="T39" s="265"/>
+      <c r="U39" s="266"/>
+      <c r="V39" s="266"/>
+      <c r="W39" s="266"/>
+      <c r="X39" s="266"/>
+      <c r="Y39" s="266"/>
+      <c r="Z39" s="266"/>
+      <c r="AA39" s="266"/>
+      <c r="AB39" s="266"/>
+      <c r="AC39" s="267"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1">
       <c r="B40" s="2">
@@ -6257,28 +6256,28 @@
       <c r="F40" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G40" s="206"/>
-      <c r="H40" s="207"/>
-      <c r="I40" s="207"/>
-      <c r="J40" s="208"/>
+      <c r="G40" s="195"/>
+      <c r="H40" s="196"/>
+      <c r="I40" s="196"/>
+      <c r="J40" s="197"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="184" t="s">
+      <c r="T40" s="216" t="s">
         <v>169</v>
       </c>
-      <c r="U40" s="185"/>
-      <c r="V40" s="185"/>
-      <c r="W40" s="185"/>
-      <c r="X40" s="185"/>
-      <c r="Y40" s="185"/>
-      <c r="Z40" s="185"/>
-      <c r="AA40" s="185"/>
-      <c r="AB40" s="185"/>
-      <c r="AC40" s="186"/>
+      <c r="U40" s="217"/>
+      <c r="V40" s="217"/>
+      <c r="W40" s="217"/>
+      <c r="X40" s="217"/>
+      <c r="Y40" s="217"/>
+      <c r="Z40" s="217"/>
+      <c r="AA40" s="217"/>
+      <c r="AB40" s="217"/>
+      <c r="AC40" s="218"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1">
       <c r="B41" s="2">
@@ -6296,28 +6295,28 @@
       <c r="F41" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G41" s="206"/>
-      <c r="H41" s="207"/>
-      <c r="I41" s="207"/>
-      <c r="J41" s="208"/>
+      <c r="G41" s="195"/>
+      <c r="H41" s="196"/>
+      <c r="I41" s="196"/>
+      <c r="J41" s="197"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="184" t="s">
+      <c r="T41" s="216" t="s">
         <v>170</v>
       </c>
-      <c r="U41" s="185"/>
-      <c r="V41" s="185"/>
-      <c r="W41" s="185"/>
-      <c r="X41" s="185"/>
-      <c r="Y41" s="185"/>
-      <c r="Z41" s="185"/>
-      <c r="AA41" s="185"/>
-      <c r="AB41" s="185"/>
-      <c r="AC41" s="186"/>
+      <c r="U41" s="217"/>
+      <c r="V41" s="217"/>
+      <c r="W41" s="217"/>
+      <c r="X41" s="217"/>
+      <c r="Y41" s="217"/>
+      <c r="Z41" s="217"/>
+      <c r="AA41" s="217"/>
+      <c r="AB41" s="217"/>
+      <c r="AC41" s="218"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
       <c r="B42" s="2">
@@ -6335,28 +6334,28 @@
       <c r="F42" s="76" t="s">
         <v>175</v>
       </c>
-      <c r="G42" s="203"/>
-      <c r="H42" s="204"/>
-      <c r="I42" s="204"/>
-      <c r="J42" s="205"/>
+      <c r="G42" s="198"/>
+      <c r="H42" s="199"/>
+      <c r="I42" s="199"/>
+      <c r="J42" s="200"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T42" s="184" t="s">
+      <c r="T42" s="216" t="s">
         <v>171</v>
       </c>
-      <c r="U42" s="185"/>
-      <c r="V42" s="185"/>
-      <c r="W42" s="185"/>
-      <c r="X42" s="185"/>
-      <c r="Y42" s="185"/>
-      <c r="Z42" s="185"/>
-      <c r="AA42" s="185"/>
-      <c r="AB42" s="185"/>
-      <c r="AC42" s="186"/>
+      <c r="U42" s="217"/>
+      <c r="V42" s="217"/>
+      <c r="W42" s="217"/>
+      <c r="X42" s="217"/>
+      <c r="Y42" s="217"/>
+      <c r="Z42" s="217"/>
+      <c r="AA42" s="217"/>
+      <c r="AB42" s="217"/>
+      <c r="AC42" s="218"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
       <c r="B43" s="2">
@@ -6374,30 +6373,30 @@
       <c r="F43" s="35" t="s">
         <v>146</v>
       </c>
-      <c r="G43" s="263" t="s">
+      <c r="G43" s="183" t="s">
         <v>191</v>
       </c>
-      <c r="H43" s="187"/>
-      <c r="I43" s="187"/>
-      <c r="J43" s="188"/>
+      <c r="H43" s="184"/>
+      <c r="I43" s="184"/>
+      <c r="J43" s="185"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="T43" s="184" t="s">
+      <c r="T43" s="216" t="s">
         <v>172</v>
       </c>
-      <c r="U43" s="185"/>
-      <c r="V43" s="185"/>
-      <c r="W43" s="185"/>
-      <c r="X43" s="185"/>
-      <c r="Y43" s="185"/>
-      <c r="Z43" s="185"/>
-      <c r="AA43" s="185"/>
-      <c r="AB43" s="185"/>
-      <c r="AC43" s="186"/>
+      <c r="U43" s="217"/>
+      <c r="V43" s="217"/>
+      <c r="W43" s="217"/>
+      <c r="X43" s="217"/>
+      <c r="Y43" s="217"/>
+      <c r="Z43" s="217"/>
+      <c r="AA43" s="217"/>
+      <c r="AB43" s="217"/>
+      <c r="AC43" s="218"/>
     </row>
     <row r="44" spans="2:29" ht="15.75" thickBot="1">
       <c r="B44" s="2">
@@ -6418,21 +6417,21 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="189" t="s">
+      <c r="S44" s="260" t="s">
         <v>75</v>
       </c>
-      <c r="T44" s="191" t="s">
+      <c r="T44" s="262" t="s">
         <v>173</v>
       </c>
-      <c r="U44" s="192"/>
-      <c r="V44" s="192"/>
-      <c r="W44" s="192"/>
-      <c r="X44" s="192"/>
-      <c r="Y44" s="192"/>
-      <c r="Z44" s="192"/>
-      <c r="AA44" s="192"/>
-      <c r="AB44" s="192"/>
-      <c r="AC44" s="193"/>
+      <c r="U44" s="263"/>
+      <c r="V44" s="263"/>
+      <c r="W44" s="263"/>
+      <c r="X44" s="263"/>
+      <c r="Y44" s="263"/>
+      <c r="Z44" s="263"/>
+      <c r="AA44" s="263"/>
+      <c r="AB44" s="263"/>
+      <c r="AC44" s="264"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1">
       <c r="B45" s="2">
@@ -6450,26 +6449,26 @@
       <c r="F45" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="G45" s="200" t="s">
+      <c r="G45" s="192" t="s">
         <v>180</v>
       </c>
-      <c r="H45" s="201"/>
-      <c r="I45" s="201"/>
-      <c r="J45" s="202"/>
+      <c r="H45" s="193"/>
+      <c r="I45" s="193"/>
+      <c r="J45" s="194"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="190"/>
-      <c r="T45" s="194"/>
-      <c r="U45" s="195"/>
-      <c r="V45" s="195"/>
-      <c r="W45" s="195"/>
-      <c r="X45" s="195"/>
-      <c r="Y45" s="195"/>
-      <c r="Z45" s="195"/>
-      <c r="AA45" s="195"/>
-      <c r="AB45" s="195"/>
-      <c r="AC45" s="196"/>
+      <c r="S45" s="261"/>
+      <c r="T45" s="265"/>
+      <c r="U45" s="266"/>
+      <c r="V45" s="266"/>
+      <c r="W45" s="266"/>
+      <c r="X45" s="266"/>
+      <c r="Y45" s="266"/>
+      <c r="Z45" s="266"/>
+      <c r="AA45" s="266"/>
+      <c r="AB45" s="266"/>
+      <c r="AC45" s="267"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
       <c r="B46" s="2">
@@ -6487,28 +6486,28 @@
       <c r="F46" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="G46" s="203"/>
-      <c r="H46" s="204"/>
-      <c r="I46" s="204"/>
-      <c r="J46" s="205"/>
+      <c r="G46" s="198"/>
+      <c r="H46" s="199"/>
+      <c r="I46" s="199"/>
+      <c r="J46" s="200"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="T46" s="197" t="s">
+      <c r="T46" s="237" t="s">
         <v>174</v>
       </c>
-      <c r="U46" s="198"/>
-      <c r="V46" s="198"/>
-      <c r="W46" s="198"/>
-      <c r="X46" s="198"/>
-      <c r="Y46" s="198"/>
-      <c r="Z46" s="198"/>
-      <c r="AA46" s="198"/>
-      <c r="AB46" s="198"/>
-      <c r="AC46" s="199"/>
+      <c r="U46" s="238"/>
+      <c r="V46" s="238"/>
+      <c r="W46" s="238"/>
+      <c r="X46" s="238"/>
+      <c r="Y46" s="238"/>
+      <c r="Z46" s="238"/>
+      <c r="AA46" s="238"/>
+      <c r="AB46" s="238"/>
+      <c r="AC46" s="239"/>
     </row>
     <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
       <c r="B47" s="2">
@@ -6526,12 +6525,12 @@
       <c r="F47" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="G47" s="187" t="s">
+      <c r="G47" s="184" t="s">
         <v>151</v>
       </c>
-      <c r="H47" s="187"/>
-      <c r="I47" s="187"/>
-      <c r="J47" s="188"/>
+      <c r="H47" s="184"/>
+      <c r="I47" s="184"/>
+      <c r="J47" s="185"/>
     </row>
     <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
       <c r="B48" s="2">
@@ -6569,12 +6568,12 @@
       <c r="F49" s="35" t="s">
         <v>152</v>
       </c>
-      <c r="G49" s="200" t="s">
+      <c r="G49" s="192" t="s">
         <v>154</v>
       </c>
-      <c r="H49" s="201"/>
-      <c r="I49" s="201"/>
-      <c r="J49" s="202"/>
+      <c r="H49" s="193"/>
+      <c r="I49" s="193"/>
+      <c r="J49" s="194"/>
     </row>
     <row r="50" spans="2:10" ht="30" customHeight="1">
       <c r="B50" s="2">
@@ -6592,10 +6591,10 @@
       <c r="F50" s="35" t="s">
         <v>152</v>
       </c>
-      <c r="G50" s="206"/>
-      <c r="H50" s="207"/>
-      <c r="I50" s="207"/>
-      <c r="J50" s="208"/>
+      <c r="G50" s="195"/>
+      <c r="H50" s="196"/>
+      <c r="I50" s="196"/>
+      <c r="J50" s="197"/>
     </row>
     <row r="51" spans="2:10" ht="32.25" customHeight="1" thickBot="1">
       <c r="B51" s="4">
@@ -6613,38 +6612,38 @@
       <c r="F51" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="G51" s="203"/>
-      <c r="H51" s="204"/>
-      <c r="I51" s="204"/>
-      <c r="J51" s="205"/>
+      <c r="G51" s="198"/>
+      <c r="H51" s="199"/>
+      <c r="I51" s="199"/>
+      <c r="J51" s="200"/>
     </row>
     <row r="52" spans="2:10" ht="30.75" customHeight="1" thickBot="1">
-      <c r="B52" s="258" t="s">
+      <c r="B52" s="209" t="s">
         <v>141</v>
       </c>
-      <c r="C52" s="239"/>
-      <c r="D52" s="239"/>
-      <c r="E52" s="239"/>
-      <c r="F52" s="240"/>
+      <c r="C52" s="210"/>
+      <c r="D52" s="210"/>
+      <c r="E52" s="210"/>
+      <c r="F52" s="211"/>
     </row>
     <row r="53" spans="2:10" ht="31.5" customHeight="1" thickBot="1"/>
     <row r="54" spans="2:10" ht="24.75" customHeight="1">
-      <c r="B54" s="252" t="s">
+      <c r="B54" s="203" t="s">
         <v>182</v>
       </c>
-      <c r="C54" s="250" t="s">
+      <c r="C54" s="201" t="s">
         <v>184</v>
       </c>
-      <c r="D54" s="264" t="s">
+      <c r="D54" s="186" t="s">
         <v>183</v>
       </c>
-      <c r="E54" s="265"/>
+      <c r="E54" s="187"/>
     </row>
     <row r="55" spans="2:10" ht="24" customHeight="1" thickBot="1">
-      <c r="B55" s="253"/>
-      <c r="C55" s="251"/>
-      <c r="D55" s="266"/>
-      <c r="E55" s="267"/>
+      <c r="B55" s="204"/>
+      <c r="C55" s="202"/>
+      <c r="D55" s="188"/>
+      <c r="E55" s="189"/>
     </row>
     <row r="56" spans="2:10" ht="41.25" customHeight="1">
       <c r="B56" s="81">
@@ -6653,10 +6652,10 @@
       <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D56" s="181" t="s">
+      <c r="D56" s="190" t="s">
         <v>206</v>
       </c>
-      <c r="E56" s="183"/>
+      <c r="E56" s="191"/>
     </row>
     <row r="57" spans="2:10" ht="31.5" customHeight="1">
       <c r="B57" s="82">
@@ -6665,10 +6664,10 @@
       <c r="C57" s="86" t="s">
         <v>202</v>
       </c>
-      <c r="D57" s="254" t="s">
+      <c r="D57" s="179" t="s">
         <v>205</v>
       </c>
-      <c r="E57" s="255"/>
+      <c r="E57" s="180"/>
     </row>
     <row r="58" spans="2:10" ht="30.75" customHeight="1">
       <c r="B58" s="82">
@@ -6677,10 +6676,10 @@
       <c r="C58" s="38" t="s">
         <v>203</v>
       </c>
-      <c r="D58" s="254" t="s">
+      <c r="D58" s="179" t="s">
         <v>204</v>
       </c>
-      <c r="E58" s="255"/>
+      <c r="E58" s="180"/>
     </row>
     <row r="59" spans="2:10" ht="33.75" customHeight="1">
       <c r="B59" s="82">
@@ -6689,10 +6688,10 @@
       <c r="C59" s="86" t="s">
         <v>185</v>
       </c>
-      <c r="D59" s="254" t="s">
+      <c r="D59" s="179" t="s">
         <v>188</v>
       </c>
-      <c r="E59" s="255"/>
+      <c r="E59" s="180"/>
     </row>
     <row r="60" spans="2:10" ht="28.5" customHeight="1">
       <c r="B60" s="82">
@@ -6701,10 +6700,10 @@
       <c r="C60" s="38" t="s">
         <v>186</v>
       </c>
-      <c r="D60" s="254" t="s">
+      <c r="D60" s="179" t="s">
         <v>189</v>
       </c>
-      <c r="E60" s="255"/>
+      <c r="E60" s="180"/>
     </row>
     <row r="61" spans="2:10" ht="40.5" customHeight="1">
       <c r="B61" s="82">
@@ -6713,10 +6712,10 @@
       <c r="C61" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="D61" s="254" t="s">
+      <c r="D61" s="179" t="s">
         <v>190</v>
       </c>
-      <c r="E61" s="255"/>
+      <c r="E61" s="180"/>
     </row>
     <row r="62" spans="2:10" ht="53.25" customHeight="1">
       <c r="B62" s="82">
@@ -6725,104 +6724,202 @@
       <c r="C62" s="86" t="s">
         <v>195</v>
       </c>
-      <c r="D62" s="254" t="s">
+      <c r="D62" s="179" t="s">
         <v>196</v>
       </c>
-      <c r="E62" s="255"/>
+      <c r="E62" s="180"/>
     </row>
     <row r="63" spans="2:10" ht="36" customHeight="1">
       <c r="B63" s="82">
         <v>7</v>
       </c>
       <c r="C63" s="86"/>
-      <c r="D63" s="254"/>
-      <c r="E63" s="255"/>
+      <c r="D63" s="179"/>
+      <c r="E63" s="180"/>
     </row>
     <row r="64" spans="2:10" ht="40.5" customHeight="1">
       <c r="B64" s="82">
         <v>8</v>
       </c>
       <c r="C64" s="86"/>
-      <c r="D64" s="254"/>
-      <c r="E64" s="255"/>
+      <c r="D64" s="179"/>
+      <c r="E64" s="180"/>
     </row>
     <row r="65" spans="2:5">
       <c r="B65" s="82">
         <v>9</v>
       </c>
       <c r="C65" s="86"/>
-      <c r="D65" s="254"/>
-      <c r="E65" s="255"/>
+      <c r="D65" s="179"/>
+      <c r="E65" s="180"/>
     </row>
     <row r="66" spans="2:5" ht="30" customHeight="1">
       <c r="B66" s="82">
         <v>10</v>
       </c>
       <c r="C66" s="86"/>
-      <c r="D66" s="254"/>
-      <c r="E66" s="255"/>
+      <c r="D66" s="179"/>
+      <c r="E66" s="180"/>
     </row>
     <row r="67" spans="2:5">
       <c r="B67" s="82">
         <v>11</v>
       </c>
       <c r="C67" s="86"/>
-      <c r="D67" s="254"/>
-      <c r="E67" s="255"/>
+      <c r="D67" s="179"/>
+      <c r="E67" s="180"/>
     </row>
     <row r="68" spans="2:5">
       <c r="B68" s="82">
         <v>12</v>
       </c>
       <c r="C68" s="86"/>
-      <c r="D68" s="254"/>
-      <c r="E68" s="255"/>
+      <c r="D68" s="179"/>
+      <c r="E68" s="180"/>
     </row>
     <row r="69" spans="2:5">
       <c r="B69" s="82">
         <v>13</v>
       </c>
       <c r="C69" s="86"/>
-      <c r="D69" s="254"/>
-      <c r="E69" s="255"/>
+      <c r="D69" s="179"/>
+      <c r="E69" s="180"/>
     </row>
     <row r="70" spans="2:5" ht="30" customHeight="1">
       <c r="B70" s="82">
         <v>14</v>
       </c>
       <c r="C70" s="86"/>
-      <c r="D70" s="254"/>
-      <c r="E70" s="255"/>
+      <c r="D70" s="179"/>
+      <c r="E70" s="180"/>
     </row>
     <row r="71" spans="2:5" ht="15.75" thickBot="1">
       <c r="B71" s="83">
         <v>15</v>
       </c>
       <c r="C71" s="87"/>
-      <c r="D71" s="261"/>
-      <c r="E71" s="262"/>
+      <c r="D71" s="181"/>
+      <c r="E71" s="182"/>
     </row>
     <row r="75" spans="2:5" ht="72" customHeight="1"/>
   </sheetData>
   <mergeCells count="158">
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D54:E55"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="T30:AC30"/>
+    <mergeCell ref="T31:AC31"/>
+    <mergeCell ref="T32:AC32"/>
+    <mergeCell ref="T33:AC33"/>
+    <mergeCell ref="T34:AC34"/>
+    <mergeCell ref="T35:AC35"/>
+    <mergeCell ref="T36:AC36"/>
+    <mergeCell ref="T37:AC37"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="S38:S39"/>
+    <mergeCell ref="T38:AC39"/>
+    <mergeCell ref="S44:S45"/>
+    <mergeCell ref="T44:AC45"/>
+    <mergeCell ref="T40:AC40"/>
+    <mergeCell ref="T41:AC41"/>
+    <mergeCell ref="T42:AC42"/>
+    <mergeCell ref="T43:AC43"/>
+    <mergeCell ref="T46:AC46"/>
+    <mergeCell ref="G45:J46"/>
+    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="AA20:AB20"/>
+    <mergeCell ref="AA21:AB21"/>
+    <mergeCell ref="AA22:AB22"/>
+    <mergeCell ref="AA15:AB15"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="U4:V4"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="U22:V22"/>
+    <mergeCell ref="U21:V21"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V6"/>
+    <mergeCell ref="U7:V7"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="U9:V9"/>
+    <mergeCell ref="U20:V20"/>
+    <mergeCell ref="U15:V15"/>
+    <mergeCell ref="U16:V16"/>
+    <mergeCell ref="U17:V17"/>
+    <mergeCell ref="U18:V18"/>
+    <mergeCell ref="U19:V19"/>
+    <mergeCell ref="U10:V10"/>
+    <mergeCell ref="U11:V11"/>
+    <mergeCell ref="AA23:AB23"/>
+    <mergeCell ref="AA6:AB6"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AA17:AB17"/>
+    <mergeCell ref="AA18:AB18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="N13:P13"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="N24:P24"/>
+    <mergeCell ref="E27:J27"/>
+    <mergeCell ref="E22:J22"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K2:P2"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="N26:P26"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AA11:AB11"/>
     <mergeCell ref="C54:C55"/>
     <mergeCell ref="B54:B55"/>
     <mergeCell ref="D57:E57"/>
@@ -6847,122 +6944,24 @@
     <mergeCell ref="N20:P20"/>
     <mergeCell ref="N21:P21"/>
     <mergeCell ref="N23:P23"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AA11:AB11"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="N27:P27"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="E28:J28"/>
-    <mergeCell ref="N24:P24"/>
-    <mergeCell ref="E27:J27"/>
-    <mergeCell ref="E22:J22"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K2:P2"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AA17:AB17"/>
-    <mergeCell ref="AA18:AB18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="AA19:AB19"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="AA20:AB20"/>
-    <mergeCell ref="AA21:AB21"/>
-    <mergeCell ref="AA22:AB22"/>
-    <mergeCell ref="AA15:AB15"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="U4:V4"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="U22:V22"/>
-    <mergeCell ref="U21:V21"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V6"/>
-    <mergeCell ref="U7:V7"/>
-    <mergeCell ref="U8:V8"/>
-    <mergeCell ref="U9:V9"/>
-    <mergeCell ref="U20:V20"/>
-    <mergeCell ref="U15:V15"/>
-    <mergeCell ref="U16:V16"/>
-    <mergeCell ref="U17:V17"/>
-    <mergeCell ref="U18:V18"/>
-    <mergeCell ref="U19:V19"/>
-    <mergeCell ref="U10:V10"/>
-    <mergeCell ref="U11:V11"/>
-    <mergeCell ref="AA23:AB23"/>
-    <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="T30:AC30"/>
-    <mergeCell ref="T31:AC31"/>
-    <mergeCell ref="T32:AC32"/>
-    <mergeCell ref="T33:AC33"/>
-    <mergeCell ref="T34:AC34"/>
-    <mergeCell ref="T35:AC35"/>
-    <mergeCell ref="T36:AC36"/>
-    <mergeCell ref="T37:AC37"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="S38:S39"/>
-    <mergeCell ref="T38:AC39"/>
-    <mergeCell ref="S44:S45"/>
-    <mergeCell ref="T44:AC45"/>
-    <mergeCell ref="T40:AC40"/>
-    <mergeCell ref="T41:AC41"/>
-    <mergeCell ref="T42:AC42"/>
-    <mergeCell ref="T43:AC43"/>
-    <mergeCell ref="T46:AC46"/>
-    <mergeCell ref="G45:J46"/>
-    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D54:E55"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="G49:J51"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7016,35 +7015,35 @@
       <c r="F2" s="103" t="s">
         <v>211</v>
       </c>
-      <c r="G2" s="200" t="s">
+      <c r="G2" s="192" t="s">
         <v>212</v>
       </c>
-      <c r="H2" s="201"/>
-      <c r="I2" s="201"/>
-      <c r="J2" s="202"/>
-      <c r="L2" s="292" t="s">
+      <c r="H2" s="193"/>
+      <c r="I2" s="193"/>
+      <c r="J2" s="194"/>
+      <c r="L2" s="284" t="s">
         <v>331</v>
       </c>
-      <c r="M2" s="293"/>
-      <c r="N2" s="293"/>
-      <c r="O2" s="294"/>
+      <c r="M2" s="285"/>
+      <c r="N2" s="285"/>
+      <c r="O2" s="286"/>
       <c r="P2" s="133"/>
-      <c r="Q2" s="295" t="s">
+      <c r="Q2" s="287" t="s">
         <v>291</v>
       </c>
-      <c r="R2" s="296"/>
-      <c r="S2" s="296"/>
-      <c r="T2" s="297"/>
+      <c r="R2" s="288"/>
+      <c r="S2" s="288"/>
+      <c r="T2" s="289"/>
       <c r="U2" s="133"/>
-      <c r="V2" s="289" t="s">
+      <c r="V2" s="277" t="s">
         <v>314</v>
       </c>
-      <c r="W2" s="290"/>
-      <c r="X2" s="290"/>
-      <c r="Y2" s="290"/>
-      <c r="Z2" s="290"/>
-      <c r="AA2" s="290"/>
-      <c r="AB2" s="291"/>
+      <c r="W2" s="278"/>
+      <c r="X2" s="278"/>
+      <c r="Y2" s="278"/>
+      <c r="Z2" s="278"/>
+      <c r="AA2" s="278"/>
+      <c r="AB2" s="279"/>
     </row>
     <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B3" s="90" t="s">
@@ -7066,11 +7065,11 @@
       <c r="G3" s="93" t="s">
         <v>213</v>
       </c>
-      <c r="H3" s="181" t="s">
+      <c r="H3" s="190" t="s">
         <v>217</v>
       </c>
-      <c r="I3" s="182"/>
-      <c r="J3" s="183"/>
+      <c r="I3" s="233"/>
+      <c r="J3" s="191"/>
       <c r="L3" s="145" t="s">
         <v>277</v>
       </c>
@@ -7109,11 +7108,11 @@
       <c r="Y3" s="171" t="s">
         <v>280</v>
       </c>
-      <c r="Z3" s="280" t="s">
+      <c r="Z3" s="268" t="s">
         <v>319</v>
       </c>
-      <c r="AA3" s="281"/>
-      <c r="AB3" s="282"/>
+      <c r="AA3" s="269"/>
+      <c r="AB3" s="270"/>
     </row>
     <row r="4" spans="2:28" ht="53.25" customHeight="1">
       <c r="B4" s="91" t="s">
@@ -7135,11 +7134,11 @@
       <c r="G4" s="94" t="s">
         <v>214</v>
       </c>
-      <c r="H4" s="184">
+      <c r="H4" s="216">
         <v>63</v>
       </c>
-      <c r="I4" s="185"/>
-      <c r="J4" s="186"/>
+      <c r="I4" s="217"/>
+      <c r="J4" s="218"/>
       <c r="L4" s="151" t="s">
         <v>246</v>
       </c>
@@ -7178,11 +7177,11 @@
       <c r="Y4" s="138" t="s">
         <v>317</v>
       </c>
-      <c r="Z4" s="283" t="s">
+      <c r="Z4" s="271" t="s">
         <v>320</v>
       </c>
-      <c r="AA4" s="284"/>
-      <c r="AB4" s="285"/>
+      <c r="AA4" s="272"/>
+      <c r="AB4" s="273"/>
     </row>
     <row r="5" spans="2:28" ht="47.25" customHeight="1">
       <c r="B5" s="91" t="s">
@@ -7204,11 +7203,11 @@
       <c r="G5" s="94" t="s">
         <v>215</v>
       </c>
-      <c r="H5" s="184">
+      <c r="H5" s="216">
         <v>31</v>
       </c>
-      <c r="I5" s="185"/>
-      <c r="J5" s="186"/>
+      <c r="I5" s="217"/>
+      <c r="J5" s="218"/>
       <c r="L5" s="149" t="s">
         <v>255</v>
       </c>
@@ -7247,9 +7246,9 @@
       <c r="Y5" s="135" t="s">
         <v>294</v>
       </c>
-      <c r="Z5" s="283"/>
-      <c r="AA5" s="284"/>
-      <c r="AB5" s="285"/>
+      <c r="Z5" s="271"/>
+      <c r="AA5" s="272"/>
+      <c r="AB5" s="273"/>
     </row>
     <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B6" s="108" t="s">
@@ -7271,11 +7270,11 @@
       <c r="G6" s="95" t="s">
         <v>216</v>
       </c>
-      <c r="H6" s="197">
+      <c r="H6" s="237">
         <v>7</v>
       </c>
-      <c r="I6" s="198"/>
-      <c r="J6" s="199"/>
+      <c r="I6" s="238"/>
+      <c r="J6" s="239"/>
       <c r="L6" s="152" t="s">
         <v>241</v>
       </c>
@@ -7314,9 +7313,9 @@
       <c r="Y6" s="144" t="s">
         <v>316</v>
       </c>
-      <c r="Z6" s="286"/>
-      <c r="AA6" s="287"/>
-      <c r="AB6" s="288"/>
+      <c r="Z6" s="274"/>
+      <c r="AA6" s="275"/>
+      <c r="AB6" s="276"/>
     </row>
     <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1">
       <c r="B7" s="90" t="s">
@@ -7338,12 +7337,12 @@
       <c r="G7" s="88" t="s">
         <v>274</v>
       </c>
-      <c r="H7" s="275" t="str">
+      <c r="H7" s="290" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12))</f>
         <v>E3FFF000</v>
       </c>
-      <c r="I7" s="276"/>
-      <c r="J7" s="277"/>
+      <c r="I7" s="291"/>
+      <c r="J7" s="292"/>
       <c r="L7" s="150" t="s">
         <v>266</v>
       </c>
@@ -7391,18 +7390,18 @@
       <c r="G8" s="88" t="s">
         <v>218</v>
       </c>
-      <c r="H8" s="275" t="str">
+      <c r="H8" s="290" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12)+4095)</f>
         <v>E3FFFFFF</v>
       </c>
-      <c r="I8" s="276"/>
-      <c r="J8" s="277"/>
-      <c r="L8" s="263" t="s">
+      <c r="I8" s="291"/>
+      <c r="J8" s="292"/>
+      <c r="L8" s="183" t="s">
         <v>333</v>
       </c>
-      <c r="M8" s="187"/>
-      <c r="N8" s="187"/>
-      <c r="O8" s="188"/>
+      <c r="M8" s="184"/>
+      <c r="N8" s="184"/>
+      <c r="O8" s="185"/>
       <c r="P8" s="133"/>
       <c r="Q8" s="164" t="s">
         <v>286</v>
@@ -7511,12 +7510,12 @@
       <c r="N11" s="133"/>
       <c r="O11" s="133"/>
       <c r="P11" s="133"/>
-      <c r="Q11" s="298" t="s">
+      <c r="Q11" s="293" t="s">
         <v>313</v>
       </c>
-      <c r="R11" s="299"/>
-      <c r="S11" s="299"/>
-      <c r="T11" s="300"/>
+      <c r="R11" s="294"/>
+      <c r="S11" s="294"/>
+      <c r="T11" s="295"/>
       <c r="U11" s="133"/>
     </row>
     <row r="12" spans="2:28" ht="44.25" customHeight="1" thickBot="1">
@@ -7668,12 +7667,12 @@
       <c r="F16" s="124" t="s">
         <v>233</v>
       </c>
-      <c r="G16" s="258" t="s">
+      <c r="G16" s="209" t="s">
         <v>271</v>
       </c>
-      <c r="H16" s="239"/>
-      <c r="I16" s="239"/>
-      <c r="J16" s="240"/>
+      <c r="H16" s="210"/>
+      <c r="I16" s="210"/>
+      <c r="J16" s="211"/>
       <c r="Q16" s="167" t="s">
         <v>307</v>
       </c>
@@ -7688,10 +7687,10 @@
       </c>
     </row>
     <row r="17" spans="2:20" ht="60.75" customHeight="1" thickBot="1">
-      <c r="B17" s="270" t="s">
+      <c r="B17" s="282" t="s">
         <v>234</v>
       </c>
-      <c r="C17" s="268" t="s">
+      <c r="C17" s="280" t="s">
         <v>235</v>
       </c>
       <c r="D17" s="125" t="s">
@@ -7703,12 +7702,12 @@
       <c r="F17" s="127" t="s">
         <v>237</v>
       </c>
-      <c r="G17" s="272" t="s">
+      <c r="G17" s="296" t="s">
         <v>272</v>
       </c>
-      <c r="H17" s="273"/>
-      <c r="I17" s="273"/>
-      <c r="J17" s="274"/>
+      <c r="H17" s="297"/>
+      <c r="I17" s="297"/>
+      <c r="J17" s="298"/>
       <c r="Q17" s="168" t="s">
         <v>310</v>
       </c>
@@ -7723,8 +7722,8 @@
       </c>
     </row>
     <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B18" s="278"/>
-      <c r="C18" s="279"/>
+      <c r="B18" s="299"/>
+      <c r="C18" s="300"/>
       <c r="D18" s="112" t="s">
         <v>238</v>
       </c>
@@ -7734,16 +7733,16 @@
       <c r="F18" s="115" t="s">
         <v>240</v>
       </c>
-      <c r="G18" s="275" t="s">
+      <c r="G18" s="290" t="s">
         <v>273</v>
       </c>
-      <c r="H18" s="276"/>
-      <c r="I18" s="276"/>
-      <c r="J18" s="277"/>
+      <c r="H18" s="291"/>
+      <c r="I18" s="291"/>
+      <c r="J18" s="292"/>
     </row>
     <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B19" s="271"/>
-      <c r="C19" s="269"/>
+      <c r="B19" s="283"/>
+      <c r="C19" s="281"/>
       <c r="D19" s="117" t="s">
         <v>241</v>
       </c>
@@ -7759,10 +7758,10 @@
       <c r="J19" s="15"/>
     </row>
     <row r="20" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B20" s="270" t="s">
+      <c r="B20" s="282" t="s">
         <v>244</v>
       </c>
-      <c r="C20" s="268" t="s">
+      <c r="C20" s="280" t="s">
         <v>245</v>
       </c>
       <c r="D20" s="125" t="s">
@@ -7780,8 +7779,8 @@
       <c r="J20" s="15"/>
     </row>
     <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B21" s="271"/>
-      <c r="C21" s="269"/>
+      <c r="B21" s="283"/>
+      <c r="C21" s="281"/>
       <c r="D21" s="117" t="s">
         <v>248</v>
       </c>
@@ -7797,10 +7796,10 @@
       <c r="J21" s="15"/>
     </row>
     <row r="22" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B22" s="270" t="s">
+      <c r="B22" s="282" t="s">
         <v>250</v>
       </c>
-      <c r="C22" s="268" t="s">
+      <c r="C22" s="280" t="s">
         <v>251</v>
       </c>
       <c r="D22" s="125" t="s">
@@ -7818,8 +7817,8 @@
       <c r="J22" s="15"/>
     </row>
     <row r="23" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B23" s="271"/>
-      <c r="C23" s="269"/>
+      <c r="B23" s="283"/>
+      <c r="C23" s="281"/>
       <c r="D23" s="117" t="s">
         <v>244</v>
       </c>
@@ -7835,10 +7834,10 @@
       <c r="J23" s="15"/>
     </row>
     <row r="24" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B24" s="270" t="s">
+      <c r="B24" s="282" t="s">
         <v>255</v>
       </c>
-      <c r="C24" s="268" t="s">
+      <c r="C24" s="280" t="s">
         <v>256</v>
       </c>
       <c r="D24" s="125" t="s">
@@ -7856,8 +7855,8 @@
       <c r="J24" s="15"/>
     </row>
     <row r="25" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B25" s="271"/>
-      <c r="C25" s="269"/>
+      <c r="B25" s="283"/>
+      <c r="C25" s="281"/>
       <c r="D25" s="117" t="s">
         <v>250</v>
       </c>
@@ -7894,10 +7893,10 @@
       <c r="J26" s="15"/>
     </row>
     <row r="27" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B27" s="270" t="s">
+      <c r="B27" s="282" t="s">
         <v>238</v>
       </c>
-      <c r="C27" s="268" t="s">
+      <c r="C27" s="280" t="s">
         <v>262</v>
       </c>
       <c r="D27" s="125" t="s">
@@ -7915,8 +7914,8 @@
       <c r="J27" s="15"/>
     </row>
     <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B28" s="271"/>
-      <c r="C28" s="269"/>
+      <c r="B28" s="283"/>
+      <c r="C28" s="281"/>
       <c r="D28" s="117" t="s">
         <v>255</v>
       </c>
@@ -7932,10 +7931,10 @@
       <c r="J28" s="15"/>
     </row>
     <row r="29" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B29" s="270" t="s">
+      <c r="B29" s="282" t="s">
         <v>266</v>
       </c>
-      <c r="C29" s="268" t="s">
+      <c r="C29" s="280" t="s">
         <v>267</v>
       </c>
       <c r="D29" s="125" t="s">
@@ -7953,8 +7952,8 @@
       <c r="J29" s="15"/>
     </row>
     <row r="30" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B30" s="271"/>
-      <c r="C30" s="269"/>
+      <c r="B30" s="283"/>
+      <c r="C30" s="281"/>
       <c r="D30" s="117" t="s">
         <v>259</v>
       </c>
@@ -7971,6 +7970,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="C17:C19"/>
     <mergeCell ref="Z3:AB3"/>
     <mergeCell ref="Z4:AB6"/>
     <mergeCell ref="V2:AB2"/>
@@ -7987,19 +7999,6 @@
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="Q11:T11"/>
     <mergeCell ref="L8:O8"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C17:C19"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Se corrigieron errores menores de la MMU y de la unidad de bypass, y se logro llegar hasta el caso 7
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C2CE748-57F5-4596-8899-81787E9821BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C68A95A-94BF-46F8-8B68-D866329A350D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="345">
   <si>
     <t>OpCode</t>
   </si>
@@ -1372,6 +1372,9 @@
   </si>
   <si>
     <t>Previous En_INTs</t>
+  </si>
+  <si>
+    <t>Nota: Estas excepciones son propias de la MMU, incluyen (Not Present, Kernel Only y Read Only). El kernel debe leer las direcciones y demas para entender de que error se trata</t>
   </si>
 </sst>
 </file>
@@ -2950,6 +2953,312 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2986,18 +3295,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3016,51 +3313,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3068,255 +3320,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3631,62 +3634,62 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B2" s="269" t="s">
+      <c r="B2" s="224" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="281" t="s">
+      <c r="C2" s="233" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="282"/>
-      <c r="E2" s="283" t="s">
+      <c r="D2" s="234"/>
+      <c r="E2" s="235" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="283"/>
-      <c r="G2" s="284" t="s">
+      <c r="F2" s="235"/>
+      <c r="G2" s="236" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="283"/>
-      <c r="I2" s="283" t="s">
+      <c r="H2" s="235"/>
+      <c r="I2" s="235" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="283"/>
-      <c r="K2" s="285" t="s">
+      <c r="J2" s="235"/>
+      <c r="K2" s="237" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="283"/>
-      <c r="M2" s="283"/>
-      <c r="N2" s="283"/>
-      <c r="O2" s="283"/>
-      <c r="P2" s="286"/>
-      <c r="R2" s="266" t="s">
+      <c r="L2" s="235"/>
+      <c r="M2" s="235"/>
+      <c r="N2" s="235"/>
+      <c r="O2" s="235"/>
+      <c r="P2" s="238"/>
+      <c r="R2" s="243" t="s">
         <v>65</v>
       </c>
-      <c r="S2" s="263" t="s">
+      <c r="S2" s="180" t="s">
         <v>66</v>
       </c>
-      <c r="T2" s="256" t="s">
+      <c r="T2" s="247" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="257"/>
-      <c r="V2" s="257"/>
-      <c r="W2" s="257"/>
-      <c r="X2" s="257"/>
-      <c r="Y2" s="257"/>
-      <c r="Z2" s="257"/>
-      <c r="AA2" s="257"/>
-      <c r="AB2" s="257" t="s">
+      <c r="U2" s="248"/>
+      <c r="V2" s="248"/>
+      <c r="W2" s="248"/>
+      <c r="X2" s="248"/>
+      <c r="Y2" s="248"/>
+      <c r="Z2" s="248"/>
+      <c r="AA2" s="248"/>
+      <c r="AB2" s="248" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="257"/>
-      <c r="AD2" s="257"/>
-      <c r="AE2" s="257"/>
-      <c r="AF2" s="257"/>
-      <c r="AG2" s="257"/>
-      <c r="AH2" s="257"/>
-      <c r="AI2" s="258"/>
+      <c r="AC2" s="248"/>
+      <c r="AD2" s="248"/>
+      <c r="AE2" s="248"/>
+      <c r="AF2" s="248"/>
+      <c r="AG2" s="248"/>
+      <c r="AH2" s="248"/>
+      <c r="AI2" s="249"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B3" s="270"/>
+      <c r="B3" s="225"/>
       <c r="C3" s="16" t="s">
         <v>79</v>
       </c>
@@ -3711,21 +3714,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="247"/>
-      <c r="L3" s="280"/>
-      <c r="M3" s="280"/>
-      <c r="N3" s="280"/>
-      <c r="O3" s="280"/>
-      <c r="P3" s="248"/>
-      <c r="R3" s="267"/>
-      <c r="S3" s="264"/>
+      <c r="K3" s="230"/>
+      <c r="L3" s="231"/>
+      <c r="M3" s="231"/>
+      <c r="N3" s="231"/>
+      <c r="O3" s="231"/>
+      <c r="P3" s="232"/>
+      <c r="R3" s="244"/>
+      <c r="S3" s="241"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="290" t="s">
+      <c r="U3" s="211" t="s">
         <v>83</v>
       </c>
-      <c r="V3" s="290"/>
+      <c r="V3" s="211"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -3738,10 +3741,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="255" t="s">
+      <c r="AA3" s="246" t="s">
         <v>74</v>
       </c>
-      <c r="AB3" s="255"/>
+      <c r="AB3" s="246"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -3765,21 +3768,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B4" s="271"/>
+      <c r="B4" s="226"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="259" t="s">
+      <c r="E4" s="212" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="222"/>
-      <c r="G4" s="222"/>
-      <c r="H4" s="222"/>
-      <c r="I4" s="222"/>
-      <c r="J4" s="223"/>
+      <c r="F4" s="239"/>
+      <c r="G4" s="239"/>
+      <c r="H4" s="239"/>
+      <c r="I4" s="239"/>
+      <c r="J4" s="240"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -3789,20 +3792,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="259" t="s">
+      <c r="N4" s="212" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="222"/>
-      <c r="P4" s="223"/>
-      <c r="R4" s="268"/>
-      <c r="S4" s="265"/>
+      <c r="O4" s="239"/>
+      <c r="P4" s="240"/>
+      <c r="R4" s="245"/>
+      <c r="S4" s="242"/>
       <c r="T4" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="U4" s="259" t="s">
+      <c r="U4" s="212" t="s">
         <v>75</v>
       </c>
-      <c r="V4" s="260"/>
+      <c r="V4" s="213"/>
       <c r="W4" s="7" t="s">
         <v>71</v>
       </c>
@@ -3815,10 +3818,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="259" t="s">
+      <c r="AA4" s="212" t="s">
         <v>72</v>
       </c>
-      <c r="AB4" s="260"/>
+      <c r="AB4" s="213"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -3850,22 +3853,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="287"/>
-      <c r="F5" s="288"/>
-      <c r="G5" s="288"/>
-      <c r="H5" s="288"/>
-      <c r="I5" s="288"/>
-      <c r="J5" s="289"/>
+      <c r="E5" s="216"/>
+      <c r="F5" s="217"/>
+      <c r="G5" s="217"/>
+      <c r="H5" s="217"/>
+      <c r="I5" s="217"/>
+      <c r="J5" s="218"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="212" t="s">
+      <c r="N5" s="181" t="s">
         <v>51</v>
       </c>
-      <c r="O5" s="213"/>
-      <c r="P5" s="214"/>
+      <c r="O5" s="182"/>
+      <c r="P5" s="183"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -3875,10 +3878,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="261" t="s">
+      <c r="U5" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="V5" s="262"/>
+      <c r="V5" s="215"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -3891,10 +3894,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="261" t="s">
+      <c r="AA5" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="AB5" s="262"/>
+      <c r="AB5" s="215"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -3926,12 +3929,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="278"/>
-      <c r="F6" s="273"/>
-      <c r="G6" s="273"/>
-      <c r="H6" s="273"/>
-      <c r="I6" s="273"/>
-      <c r="J6" s="274"/>
+      <c r="E6" s="223"/>
+      <c r="F6" s="220"/>
+      <c r="G6" s="220"/>
+      <c r="H6" s="220"/>
+      <c r="I6" s="220"/>
+      <c r="J6" s="221"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -3939,11 +3942,11 @@
         <v>154</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="209" t="s">
+      <c r="N6" s="184" t="s">
         <v>95</v>
       </c>
-      <c r="O6" s="210"/>
-      <c r="P6" s="211"/>
+      <c r="O6" s="185"/>
+      <c r="P6" s="186"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -3953,10 +3956,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="251" t="s">
+      <c r="U6" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V6" s="252"/>
+      <c r="V6" s="210"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -3969,10 +3972,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="251" t="s">
+      <c r="AA6" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB6" s="252"/>
+      <c r="AB6" s="210"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -4015,9 +4018,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="272"/>
-      <c r="I7" s="273"/>
-      <c r="J7" s="274"/>
+      <c r="H7" s="219"/>
+      <c r="I7" s="220"/>
+      <c r="J7" s="221"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -4025,11 +4028,11 @@
       <c r="M7" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N7" s="209" t="s">
+      <c r="N7" s="184" t="s">
         <v>52</v>
       </c>
-      <c r="O7" s="210"/>
-      <c r="P7" s="211"/>
+      <c r="O7" s="185"/>
+      <c r="P7" s="186"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -4039,10 +4042,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="251" t="s">
+      <c r="U7" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V7" s="252"/>
+      <c r="V7" s="210"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -4055,10 +4058,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="251" t="s">
+      <c r="AA7" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB7" s="252"/>
+      <c r="AB7" s="210"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -4101,9 +4104,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="272"/>
-      <c r="I8" s="273"/>
-      <c r="J8" s="274"/>
+      <c r="H8" s="219"/>
+      <c r="I8" s="220"/>
+      <c r="J8" s="221"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -4111,11 +4114,11 @@
       <c r="M8" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N8" s="209" t="s">
+      <c r="N8" s="184" t="s">
         <v>53</v>
       </c>
-      <c r="O8" s="210"/>
-      <c r="P8" s="211"/>
+      <c r="O8" s="185"/>
+      <c r="P8" s="186"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -4125,10 +4128,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="251" t="s">
+      <c r="U8" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V8" s="252"/>
+      <c r="V8" s="210"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -4141,10 +4144,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="251" t="s">
+      <c r="AA8" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB8" s="252"/>
+      <c r="AB8" s="210"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -4187,9 +4190,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="272"/>
-      <c r="I9" s="273"/>
-      <c r="J9" s="274"/>
+      <c r="H9" s="219"/>
+      <c r="I9" s="220"/>
+      <c r="J9" s="221"/>
       <c r="K9" s="37" t="s">
         <v>47</v>
       </c>
@@ -4197,11 +4200,11 @@
       <c r="M9" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N9" s="209" t="s">
+      <c r="N9" s="184" t="s">
         <v>54</v>
       </c>
-      <c r="O9" s="210"/>
-      <c r="P9" s="211"/>
+      <c r="O9" s="185"/>
+      <c r="P9" s="186"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -4211,10 +4214,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="251" t="s">
+      <c r="U9" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V9" s="252"/>
+      <c r="V9" s="210"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -4227,10 +4230,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="251" t="s">
+      <c r="AA9" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB9" s="252"/>
+      <c r="AB9" s="210"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -4273,9 +4276,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="272"/>
-      <c r="I10" s="273"/>
-      <c r="J10" s="274"/>
+      <c r="H10" s="219"/>
+      <c r="I10" s="220"/>
+      <c r="J10" s="221"/>
       <c r="K10" s="37" t="s">
         <v>48</v>
       </c>
@@ -4283,11 +4286,11 @@
       <c r="M10" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N10" s="209" t="s">
+      <c r="N10" s="184" t="s">
         <v>55</v>
       </c>
-      <c r="O10" s="210"/>
-      <c r="P10" s="211"/>
+      <c r="O10" s="185"/>
+      <c r="P10" s="186"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -4297,10 +4300,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="251" t="s">
+      <c r="U10" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V10" s="252"/>
+      <c r="V10" s="210"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -4313,10 +4316,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="251" t="s">
+      <c r="AA10" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB10" s="252"/>
+      <c r="AB10" s="210"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -4359,9 +4362,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="272"/>
-      <c r="I11" s="273"/>
-      <c r="J11" s="274"/>
+      <c r="H11" s="219"/>
+      <c r="I11" s="220"/>
+      <c r="J11" s="221"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -4369,11 +4372,11 @@
       <c r="M11" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N11" s="209" t="s">
+      <c r="N11" s="184" t="s">
         <v>56</v>
       </c>
-      <c r="O11" s="210"/>
-      <c r="P11" s="211"/>
+      <c r="O11" s="185"/>
+      <c r="P11" s="186"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -4383,10 +4386,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="251" t="s">
+      <c r="U11" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V11" s="252"/>
+      <c r="V11" s="210"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -4399,10 +4402,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="251" t="s">
+      <c r="AA11" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB11" s="252"/>
+      <c r="AB11" s="210"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -4445,9 +4448,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="272"/>
-      <c r="I12" s="273"/>
-      <c r="J12" s="274"/>
+      <c r="H12" s="219"/>
+      <c r="I12" s="220"/>
+      <c r="J12" s="221"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -4455,11 +4458,11 @@
       <c r="M12" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N12" s="209" t="s">
+      <c r="N12" s="184" t="s">
         <v>57</v>
       </c>
-      <c r="O12" s="210"/>
-      <c r="P12" s="211"/>
+      <c r="O12" s="185"/>
+      <c r="P12" s="186"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -4469,10 +4472,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="251" t="s">
+      <c r="U12" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V12" s="252"/>
+      <c r="V12" s="210"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -4485,10 +4488,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="251" t="s">
+      <c r="AA12" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB12" s="252"/>
+      <c r="AB12" s="210"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -4531,9 +4534,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="272"/>
-      <c r="I13" s="273"/>
-      <c r="J13" s="274"/>
+      <c r="H13" s="219"/>
+      <c r="I13" s="220"/>
+      <c r="J13" s="221"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -4541,11 +4544,11 @@
       <c r="M13" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N13" s="209" t="s">
+      <c r="N13" s="184" t="s">
         <v>58</v>
       </c>
-      <c r="O13" s="210"/>
-      <c r="P13" s="211"/>
+      <c r="O13" s="185"/>
+      <c r="P13" s="186"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -4555,10 +4558,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="251" t="s">
+      <c r="U13" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V13" s="252"/>
+      <c r="V13" s="210"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -4571,10 +4574,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="251" t="s">
+      <c r="AA13" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB13" s="252"/>
+      <c r="AB13" s="210"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -4617,9 +4620,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="272"/>
-      <c r="I14" s="273"/>
-      <c r="J14" s="274"/>
+      <c r="H14" s="219"/>
+      <c r="I14" s="220"/>
+      <c r="J14" s="221"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -4627,11 +4630,11 @@
       <c r="M14" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N14" s="209" t="s">
+      <c r="N14" s="184" t="s">
         <v>59</v>
       </c>
-      <c r="O14" s="210"/>
-      <c r="P14" s="211"/>
+      <c r="O14" s="185"/>
+      <c r="P14" s="186"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -4641,10 +4644,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="251" t="s">
+      <c r="U14" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V14" s="252"/>
+      <c r="V14" s="210"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -4657,10 +4660,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="251" t="s">
+      <c r="AA14" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB14" s="252"/>
+      <c r="AB14" s="210"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -4703,9 +4706,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="272"/>
-      <c r="I15" s="273"/>
-      <c r="J15" s="274"/>
+      <c r="H15" s="219"/>
+      <c r="I15" s="220"/>
+      <c r="J15" s="221"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -4713,11 +4716,11 @@
       <c r="M15" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N15" s="209" t="s">
+      <c r="N15" s="184" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="210"/>
-      <c r="P15" s="211"/>
+      <c r="O15" s="185"/>
+      <c r="P15" s="186"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -4727,10 +4730,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="251" t="s">
+      <c r="U15" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V15" s="252"/>
+      <c r="V15" s="210"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -4743,10 +4746,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="251" t="s">
+      <c r="AA15" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB15" s="252"/>
+      <c r="AB15" s="210"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -4783,21 +4786,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="272"/>
-      <c r="G16" s="273"/>
-      <c r="H16" s="273"/>
-      <c r="I16" s="273"/>
-      <c r="J16" s="274"/>
+      <c r="F16" s="219"/>
+      <c r="G16" s="220"/>
+      <c r="H16" s="220"/>
+      <c r="I16" s="220"/>
+      <c r="J16" s="221"/>
       <c r="K16" s="40" t="s">
         <v>49</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="209" t="s">
+      <c r="N16" s="184" t="s">
         <v>50</v>
       </c>
-      <c r="O16" s="210"/>
-      <c r="P16" s="211"/>
+      <c r="O16" s="185"/>
+      <c r="P16" s="186"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -4807,10 +4810,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="251" t="s">
+      <c r="U16" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V16" s="252"/>
+      <c r="V16" s="210"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -4823,10 +4826,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="251" t="s">
+      <c r="AA16" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB16" s="252"/>
+      <c r="AB16" s="210"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -4864,22 +4867,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="279" t="s">
+      <c r="G17" s="222" t="s">
         <v>76</v>
       </c>
-      <c r="H17" s="210"/>
-      <c r="I17" s="210"/>
-      <c r="J17" s="211"/>
+      <c r="H17" s="185"/>
+      <c r="I17" s="185"/>
+      <c r="J17" s="186"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="209" t="s">
+      <c r="N17" s="184" t="s">
         <v>64</v>
       </c>
-      <c r="O17" s="210"/>
-      <c r="P17" s="211"/>
+      <c r="O17" s="185"/>
+      <c r="P17" s="186"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -4889,10 +4892,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="251" t="s">
+      <c r="U17" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V17" s="252"/>
+      <c r="V17" s="210"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -4905,10 +4908,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="251" t="s">
+      <c r="AA17" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB17" s="252"/>
+      <c r="AB17" s="210"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -4946,12 +4949,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="279" t="s">
+      <c r="G18" s="222" t="s">
         <v>76</v>
       </c>
-      <c r="H18" s="210"/>
-      <c r="I18" s="210"/>
-      <c r="J18" s="211"/>
+      <c r="H18" s="185"/>
+      <c r="I18" s="185"/>
+      <c r="J18" s="186"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -4959,11 +4962,11 @@
       <c r="M18" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N18" s="209" t="s">
+      <c r="N18" s="184" t="s">
         <v>61</v>
       </c>
-      <c r="O18" s="210"/>
-      <c r="P18" s="211"/>
+      <c r="O18" s="185"/>
+      <c r="P18" s="186"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -4973,10 +4976,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="251" t="s">
+      <c r="U18" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V18" s="252"/>
+      <c r="V18" s="210"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -4989,10 +4992,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="251" t="s">
+      <c r="AA18" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB18" s="252"/>
+      <c r="AB18" s="210"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -5028,20 +5031,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="272"/>
-      <c r="H19" s="273"/>
-      <c r="I19" s="273"/>
-      <c r="J19" s="274"/>
+      <c r="G19" s="219"/>
+      <c r="H19" s="220"/>
+      <c r="I19" s="220"/>
+      <c r="J19" s="221"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="209" t="s">
+      <c r="N19" s="184" t="s">
         <v>93</v>
       </c>
-      <c r="O19" s="210"/>
-      <c r="P19" s="211"/>
+      <c r="O19" s="185"/>
+      <c r="P19" s="186"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -5051,10 +5054,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="251" t="s">
+      <c r="U19" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V19" s="252"/>
+      <c r="V19" s="210"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -5067,10 +5070,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="251" t="s">
+      <c r="AA19" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB19" s="252"/>
+      <c r="AB19" s="210"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -5108,20 +5111,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="272"/>
-      <c r="H20" s="273"/>
-      <c r="I20" s="273"/>
-      <c r="J20" s="274"/>
+      <c r="G20" s="219"/>
+      <c r="H20" s="220"/>
+      <c r="I20" s="220"/>
+      <c r="J20" s="221"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="209" t="s">
+      <c r="N20" s="184" t="s">
         <v>94</v>
       </c>
-      <c r="O20" s="210"/>
-      <c r="P20" s="211"/>
+      <c r="O20" s="185"/>
+      <c r="P20" s="186"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -5131,10 +5134,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="251" t="s">
+      <c r="U20" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V20" s="252"/>
+      <c r="V20" s="210"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -5147,10 +5150,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="251" t="s">
+      <c r="AA20" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB20" s="252"/>
+      <c r="AB20" s="210"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -5188,20 +5191,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="272"/>
-      <c r="H21" s="273"/>
-      <c r="I21" s="273"/>
-      <c r="J21" s="274"/>
+      <c r="G21" s="219"/>
+      <c r="H21" s="220"/>
+      <c r="I21" s="220"/>
+      <c r="J21" s="221"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="209" t="s">
+      <c r="N21" s="184" t="s">
         <v>62</v>
       </c>
-      <c r="O21" s="210"/>
-      <c r="P21" s="211"/>
+      <c r="O21" s="185"/>
+      <c r="P21" s="186"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -5211,10 +5214,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="251" t="s">
+      <c r="U21" s="209" t="s">
         <v>96</v>
       </c>
-      <c r="V21" s="252"/>
+      <c r="V21" s="210"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -5227,10 +5230,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="251" t="s">
+      <c r="AA21" s="209" t="s">
         <v>98</v>
       </c>
-      <c r="AB21" s="252"/>
+      <c r="AB21" s="210"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -5264,22 +5267,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="278"/>
-      <c r="F22" s="273"/>
-      <c r="G22" s="273"/>
-      <c r="H22" s="273"/>
-      <c r="I22" s="273"/>
-      <c r="J22" s="274"/>
+      <c r="E22" s="223"/>
+      <c r="F22" s="220"/>
+      <c r="G22" s="220"/>
+      <c r="H22" s="220"/>
+      <c r="I22" s="220"/>
+      <c r="J22" s="221"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="209" t="s">
+      <c r="N22" s="184" t="s">
         <v>63</v>
       </c>
-      <c r="O22" s="210"/>
-      <c r="P22" s="211"/>
+      <c r="O22" s="185"/>
+      <c r="P22" s="186"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -5289,10 +5292,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="251" t="s">
+      <c r="U22" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V22" s="252"/>
+      <c r="V22" s="210"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -5305,10 +5308,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="251" t="s">
+      <c r="AA22" s="209" t="s">
         <v>96</v>
       </c>
-      <c r="AB22" s="252"/>
+      <c r="AB22" s="210"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -5348,22 +5351,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="279" t="s">
+      <c r="G23" s="222" t="s">
         <v>77</v>
       </c>
-      <c r="H23" s="210"/>
-      <c r="I23" s="210"/>
-      <c r="J23" s="211"/>
+      <c r="H23" s="185"/>
+      <c r="I23" s="185"/>
+      <c r="J23" s="186"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="209" t="s">
+      <c r="N23" s="184" t="s">
         <v>82</v>
       </c>
-      <c r="O23" s="210"/>
-      <c r="P23" s="211"/>
+      <c r="O23" s="185"/>
+      <c r="P23" s="186"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -5373,10 +5376,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="251" t="s">
+      <c r="U23" s="209" t="s">
         <v>97</v>
       </c>
-      <c r="V23" s="252"/>
+      <c r="V23" s="210"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -5389,10 +5392,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="251" t="s">
+      <c r="AA23" s="209" t="s">
         <v>96</v>
       </c>
-      <c r="AB23" s="252"/>
+      <c r="AB23" s="210"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -5432,22 +5435,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="279" t="s">
+      <c r="G24" s="222" t="s">
         <v>77</v>
       </c>
-      <c r="H24" s="210"/>
-      <c r="I24" s="210"/>
-      <c r="J24" s="211"/>
+      <c r="H24" s="185"/>
+      <c r="I24" s="185"/>
+      <c r="J24" s="186"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="209" t="s">
+      <c r="N24" s="184" t="s">
         <v>81</v>
       </c>
-      <c r="O24" s="210"/>
-      <c r="P24" s="211"/>
+      <c r="O24" s="185"/>
+      <c r="P24" s="186"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -5457,10 +5460,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="251" t="s">
+      <c r="U24" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V24" s="252"/>
+      <c r="V24" s="210"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -5473,10 +5476,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="251" t="s">
+      <c r="AA24" s="209" t="s">
         <v>98</v>
       </c>
-      <c r="AB24" s="252"/>
+      <c r="AB24" s="210"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -5514,10 +5517,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="272"/>
-      <c r="H25" s="273"/>
-      <c r="I25" s="273"/>
-      <c r="J25" s="274"/>
+      <c r="G25" s="219"/>
+      <c r="H25" s="220"/>
+      <c r="I25" s="220"/>
+      <c r="J25" s="221"/>
       <c r="K25" s="49" t="s">
         <v>39</v>
       </c>
@@ -5525,11 +5528,11 @@
         <v>154</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="209" t="s">
+      <c r="N25" s="184" t="s">
         <v>41</v>
       </c>
-      <c r="O25" s="210"/>
-      <c r="P25" s="211"/>
+      <c r="O25" s="185"/>
+      <c r="P25" s="186"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -5539,10 +5542,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="251" t="s">
+      <c r="U25" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V25" s="252"/>
+      <c r="V25" s="210"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -5555,10 +5558,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="251" t="s">
+      <c r="AA25" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB25" s="252"/>
+      <c r="AB25" s="210"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -5596,10 +5599,10 @@
       <c r="F26" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="G26" s="272"/>
-      <c r="H26" s="273"/>
-      <c r="I26" s="273"/>
-      <c r="J26" s="274"/>
+      <c r="G26" s="219"/>
+      <c r="H26" s="220"/>
+      <c r="I26" s="220"/>
+      <c r="J26" s="221"/>
       <c r="K26" s="31" t="s">
         <v>40</v>
       </c>
@@ -5607,11 +5610,11 @@
         <v>154</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="209" t="s">
+      <c r="N26" s="184" t="s">
         <v>42</v>
       </c>
-      <c r="O26" s="210"/>
-      <c r="P26" s="211"/>
+      <c r="O26" s="185"/>
+      <c r="P26" s="186"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -5621,10 +5624,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="251" t="s">
+      <c r="U26" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V26" s="252"/>
+      <c r="V26" s="210"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -5637,10 +5640,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="251" t="s">
+      <c r="AA26" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB26" s="252"/>
+      <c r="AB26" s="210"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -5672,22 +5675,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="278"/>
-      <c r="F27" s="273"/>
-      <c r="G27" s="273"/>
-      <c r="H27" s="273"/>
-      <c r="I27" s="273"/>
-      <c r="J27" s="274"/>
+      <c r="E27" s="223"/>
+      <c r="F27" s="220"/>
+      <c r="G27" s="220"/>
+      <c r="H27" s="220"/>
+      <c r="I27" s="220"/>
+      <c r="J27" s="221"/>
       <c r="K27" s="25" t="s">
         <v>44</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="209" t="s">
+      <c r="N27" s="184" t="s">
         <v>46</v>
       </c>
-      <c r="O27" s="210"/>
-      <c r="P27" s="211"/>
+      <c r="O27" s="185"/>
+      <c r="P27" s="186"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -5697,10 +5700,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="251" t="s">
+      <c r="U27" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="V27" s="252"/>
+      <c r="V27" s="210"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -5713,10 +5716,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="251" t="s">
+      <c r="AA27" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="AB27" s="252"/>
+      <c r="AB27" s="210"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -5748,12 +5751,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="275"/>
-      <c r="F28" s="276"/>
-      <c r="G28" s="276"/>
-      <c r="H28" s="276"/>
-      <c r="I28" s="276"/>
-      <c r="J28" s="277"/>
+      <c r="E28" s="227"/>
+      <c r="F28" s="228"/>
+      <c r="G28" s="228"/>
+      <c r="H28" s="228"/>
+      <c r="I28" s="228"/>
+      <c r="J28" s="229"/>
       <c r="K28" s="52" t="s">
         <v>45</v>
       </c>
@@ -5761,11 +5764,11 @@
         <v>154</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="206" t="s">
+      <c r="N28" s="197" t="s">
         <v>92</v>
       </c>
-      <c r="O28" s="207"/>
-      <c r="P28" s="208"/>
+      <c r="O28" s="198"/>
+      <c r="P28" s="199"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -5775,10 +5778,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="253" t="s">
+      <c r="U28" s="259" t="s">
         <v>73</v>
       </c>
-      <c r="V28" s="254"/>
+      <c r="V28" s="260"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -5791,10 +5794,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="253" t="s">
+      <c r="AA28" s="259" t="s">
         <v>73</v>
       </c>
-      <c r="AB28" s="254"/>
+      <c r="AB28" s="260"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -5871,18 +5874,18 @@
       <c r="S30" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="T30" s="291" t="s">
+      <c r="T30" s="179" t="s">
         <v>156</v>
       </c>
-      <c r="U30" s="291"/>
-      <c r="V30" s="291"/>
-      <c r="W30" s="291"/>
-      <c r="X30" s="291"/>
-      <c r="Y30" s="291"/>
-      <c r="Z30" s="291"/>
-      <c r="AA30" s="291"/>
-      <c r="AB30" s="291"/>
-      <c r="AC30" s="263"/>
+      <c r="U30" s="179"/>
+      <c r="V30" s="179"/>
+      <c r="W30" s="179"/>
+      <c r="X30" s="179"/>
+      <c r="Y30" s="179"/>
+      <c r="Z30" s="179"/>
+      <c r="AA30" s="179"/>
+      <c r="AB30" s="179"/>
+      <c r="AC30" s="180"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B31" s="67" t="s">
@@ -5923,18 +5926,18 @@
       <c r="S31" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="T31" s="212" t="s">
+      <c r="T31" s="181" t="s">
         <v>161</v>
       </c>
-      <c r="U31" s="213"/>
-      <c r="V31" s="213"/>
-      <c r="W31" s="213"/>
-      <c r="X31" s="213"/>
-      <c r="Y31" s="213"/>
-      <c r="Z31" s="213"/>
-      <c r="AA31" s="213"/>
-      <c r="AB31" s="213"/>
-      <c r="AC31" s="214"/>
+      <c r="U31" s="182"/>
+      <c r="V31" s="182"/>
+      <c r="W31" s="182"/>
+      <c r="X31" s="182"/>
+      <c r="Y31" s="182"/>
+      <c r="Z31" s="182"/>
+      <c r="AA31" s="182"/>
+      <c r="AB31" s="182"/>
+      <c r="AC31" s="183"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B32" s="4" t="s">
@@ -5958,18 +5961,18 @@
       <c r="S32" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="T32" s="209" t="s">
+      <c r="T32" s="184" t="s">
         <v>162</v>
       </c>
-      <c r="U32" s="210"/>
-      <c r="V32" s="210"/>
-      <c r="W32" s="210"/>
-      <c r="X32" s="210"/>
-      <c r="Y32" s="210"/>
-      <c r="Z32" s="210"/>
-      <c r="AA32" s="210"/>
-      <c r="AB32" s="210"/>
-      <c r="AC32" s="211"/>
+      <c r="U32" s="185"/>
+      <c r="V32" s="185"/>
+      <c r="W32" s="185"/>
+      <c r="X32" s="185"/>
+      <c r="Y32" s="185"/>
+      <c r="Z32" s="185"/>
+      <c r="AA32" s="185"/>
+      <c r="AB32" s="185"/>
+      <c r="AC32" s="186"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
       <c r="H33" s="84" t="s">
@@ -6005,31 +6008,31 @@
       <c r="S33" s="37" t="s">
         <v>158</v>
       </c>
-      <c r="T33" s="209" t="s">
+      <c r="T33" s="184" t="s">
         <v>163</v>
       </c>
-      <c r="U33" s="210"/>
-      <c r="V33" s="210"/>
-      <c r="W33" s="210"/>
-      <c r="X33" s="210"/>
-      <c r="Y33" s="210"/>
-      <c r="Z33" s="210"/>
-      <c r="AA33" s="210"/>
-      <c r="AB33" s="210"/>
-      <c r="AC33" s="211"/>
+      <c r="U33" s="185"/>
+      <c r="V33" s="185"/>
+      <c r="W33" s="185"/>
+      <c r="X33" s="185"/>
+      <c r="Y33" s="185"/>
+      <c r="Z33" s="185"/>
+      <c r="AA33" s="185"/>
+      <c r="AB33" s="185"/>
+      <c r="AC33" s="186"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B34" s="249" t="s">
+      <c r="B34" s="256" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="247" t="s">
+      <c r="C34" s="230" t="s">
         <v>114</v>
       </c>
-      <c r="D34" s="248"/>
-      <c r="E34" s="247" t="s">
+      <c r="D34" s="232"/>
+      <c r="E34" s="230" t="s">
         <v>115</v>
       </c>
-      <c r="F34" s="248"/>
+      <c r="F34" s="232"/>
       <c r="H34" s="77" t="s">
         <v>65</v>
       </c>
@@ -6055,21 +6058,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="209" t="s">
+      <c r="T34" s="184" t="s">
         <v>164</v>
       </c>
-      <c r="U34" s="210"/>
-      <c r="V34" s="210"/>
-      <c r="W34" s="210"/>
-      <c r="X34" s="210"/>
-      <c r="Y34" s="210"/>
-      <c r="Z34" s="210"/>
-      <c r="AA34" s="210"/>
-      <c r="AB34" s="210"/>
-      <c r="AC34" s="211"/>
+      <c r="U34" s="185"/>
+      <c r="V34" s="185"/>
+      <c r="W34" s="185"/>
+      <c r="X34" s="185"/>
+      <c r="Y34" s="185"/>
+      <c r="Z34" s="185"/>
+      <c r="AA34" s="185"/>
+      <c r="AB34" s="185"/>
+      <c r="AC34" s="186"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B35" s="250"/>
+      <c r="B35" s="257"/>
       <c r="C35" s="64" t="s">
         <v>99</v>
       </c>
@@ -6088,18 +6091,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="209" t="s">
+      <c r="T35" s="184" t="s">
         <v>165</v>
       </c>
-      <c r="U35" s="210"/>
-      <c r="V35" s="210"/>
-      <c r="W35" s="210"/>
-      <c r="X35" s="210"/>
-      <c r="Y35" s="210"/>
-      <c r="Z35" s="210"/>
-      <c r="AA35" s="210"/>
-      <c r="AB35" s="210"/>
-      <c r="AC35" s="211"/>
+      <c r="U35" s="185"/>
+      <c r="V35" s="185"/>
+      <c r="W35" s="185"/>
+      <c r="X35" s="185"/>
+      <c r="Y35" s="185"/>
+      <c r="Z35" s="185"/>
+      <c r="AA35" s="185"/>
+      <c r="AB35" s="185"/>
+      <c r="AC35" s="186"/>
     </row>
     <row r="36" spans="2:29" ht="36" customHeight="1" thickBot="1">
       <c r="B36" s="1">
@@ -6150,18 +6153,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="209" t="s">
+      <c r="T36" s="184" t="s">
         <v>166</v>
       </c>
-      <c r="U36" s="210"/>
-      <c r="V36" s="210"/>
-      <c r="W36" s="210"/>
-      <c r="X36" s="210"/>
-      <c r="Y36" s="210"/>
-      <c r="Z36" s="210"/>
-      <c r="AA36" s="210"/>
-      <c r="AB36" s="210"/>
-      <c r="AC36" s="211"/>
+      <c r="U36" s="185"/>
+      <c r="V36" s="185"/>
+      <c r="W36" s="185"/>
+      <c r="X36" s="185"/>
+      <c r="Y36" s="185"/>
+      <c r="Z36" s="185"/>
+      <c r="AA36" s="185"/>
+      <c r="AB36" s="185"/>
+      <c r="AC36" s="186"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1" thickBot="1">
       <c r="B37" s="2">
@@ -6186,7 +6189,7 @@
       <c r="J37" s="79"/>
       <c r="K37" s="79"/>
       <c r="L37" s="79"/>
-      <c r="M37" s="300" t="s">
+      <c r="M37" s="178" t="s">
         <v>343</v>
       </c>
       <c r="N37" s="79" t="s">
@@ -6204,18 +6207,18 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="209" t="s">
+      <c r="T37" s="184" t="s">
         <v>193</v>
       </c>
-      <c r="U37" s="210"/>
-      <c r="V37" s="210"/>
-      <c r="W37" s="210"/>
-      <c r="X37" s="210"/>
-      <c r="Y37" s="210"/>
-      <c r="Z37" s="210"/>
-      <c r="AA37" s="210"/>
-      <c r="AB37" s="210"/>
-      <c r="AC37" s="211"/>
+      <c r="U37" s="185"/>
+      <c r="V37" s="185"/>
+      <c r="W37" s="185"/>
+      <c r="X37" s="185"/>
+      <c r="Y37" s="185"/>
+      <c r="Z37" s="185"/>
+      <c r="AA37" s="185"/>
+      <c r="AB37" s="185"/>
+      <c r="AC37" s="186"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1">
       <c r="B38" s="2">
@@ -6236,21 +6239,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="292" t="s">
+      <c r="S38" s="189" t="s">
         <v>72</v>
       </c>
-      <c r="T38" s="294" t="s">
+      <c r="T38" s="191" t="s">
         <v>167</v>
       </c>
-      <c r="U38" s="295"/>
-      <c r="V38" s="295"/>
-      <c r="W38" s="295"/>
-      <c r="X38" s="295"/>
-      <c r="Y38" s="295"/>
-      <c r="Z38" s="295"/>
-      <c r="AA38" s="295"/>
-      <c r="AB38" s="295"/>
-      <c r="AC38" s="296"/>
+      <c r="U38" s="192"/>
+      <c r="V38" s="192"/>
+      <c r="W38" s="192"/>
+      <c r="X38" s="192"/>
+      <c r="Y38" s="192"/>
+      <c r="Z38" s="192"/>
+      <c r="AA38" s="192"/>
+      <c r="AB38" s="192"/>
+      <c r="AC38" s="193"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1">
       <c r="B39" s="2">
@@ -6268,26 +6271,26 @@
       <c r="F39" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G39" s="203" t="s">
+      <c r="G39" s="200" t="s">
         <v>180</v>
       </c>
-      <c r="H39" s="204"/>
-      <c r="I39" s="204"/>
-      <c r="J39" s="205"/>
+      <c r="H39" s="201"/>
+      <c r="I39" s="201"/>
+      <c r="J39" s="202"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="293"/>
-      <c r="T39" s="297"/>
-      <c r="U39" s="298"/>
-      <c r="V39" s="298"/>
-      <c r="W39" s="298"/>
-      <c r="X39" s="298"/>
-      <c r="Y39" s="298"/>
-      <c r="Z39" s="298"/>
-      <c r="AA39" s="298"/>
-      <c r="AB39" s="298"/>
-      <c r="AC39" s="299"/>
+      <c r="S39" s="190"/>
+      <c r="T39" s="194"/>
+      <c r="U39" s="195"/>
+      <c r="V39" s="195"/>
+      <c r="W39" s="195"/>
+      <c r="X39" s="195"/>
+      <c r="Y39" s="195"/>
+      <c r="Z39" s="195"/>
+      <c r="AA39" s="195"/>
+      <c r="AB39" s="195"/>
+      <c r="AC39" s="196"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1">
       <c r="B40" s="2">
@@ -6305,28 +6308,28 @@
       <c r="F40" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G40" s="237"/>
-      <c r="H40" s="238"/>
-      <c r="I40" s="238"/>
-      <c r="J40" s="239"/>
+      <c r="G40" s="206"/>
+      <c r="H40" s="207"/>
+      <c r="I40" s="207"/>
+      <c r="J40" s="208"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="209" t="s">
+      <c r="T40" s="184" t="s">
         <v>168</v>
       </c>
-      <c r="U40" s="210"/>
-      <c r="V40" s="210"/>
-      <c r="W40" s="210"/>
-      <c r="X40" s="210"/>
-      <c r="Y40" s="210"/>
-      <c r="Z40" s="210"/>
-      <c r="AA40" s="210"/>
-      <c r="AB40" s="210"/>
-      <c r="AC40" s="211"/>
+      <c r="U40" s="185"/>
+      <c r="V40" s="185"/>
+      <c r="W40" s="185"/>
+      <c r="X40" s="185"/>
+      <c r="Y40" s="185"/>
+      <c r="Z40" s="185"/>
+      <c r="AA40" s="185"/>
+      <c r="AB40" s="185"/>
+      <c r="AC40" s="186"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1">
       <c r="B41" s="2">
@@ -6344,28 +6347,28 @@
       <c r="F41" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G41" s="237"/>
-      <c r="H41" s="238"/>
-      <c r="I41" s="238"/>
-      <c r="J41" s="239"/>
+      <c r="G41" s="206"/>
+      <c r="H41" s="207"/>
+      <c r="I41" s="207"/>
+      <c r="J41" s="208"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="209" t="s">
+      <c r="T41" s="184" t="s">
         <v>169</v>
       </c>
-      <c r="U41" s="210"/>
-      <c r="V41" s="210"/>
-      <c r="W41" s="210"/>
-      <c r="X41" s="210"/>
-      <c r="Y41" s="210"/>
-      <c r="Z41" s="210"/>
-      <c r="AA41" s="210"/>
-      <c r="AB41" s="210"/>
-      <c r="AC41" s="211"/>
+      <c r="U41" s="185"/>
+      <c r="V41" s="185"/>
+      <c r="W41" s="185"/>
+      <c r="X41" s="185"/>
+      <c r="Y41" s="185"/>
+      <c r="Z41" s="185"/>
+      <c r="AA41" s="185"/>
+      <c r="AB41" s="185"/>
+      <c r="AC41" s="186"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
       <c r="B42" s="2">
@@ -6383,28 +6386,28 @@
       <c r="F42" s="76" t="s">
         <v>174</v>
       </c>
-      <c r="G42" s="240"/>
-      <c r="H42" s="241"/>
-      <c r="I42" s="241"/>
-      <c r="J42" s="242"/>
+      <c r="G42" s="203"/>
+      <c r="H42" s="204"/>
+      <c r="I42" s="204"/>
+      <c r="J42" s="205"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="T42" s="209" t="s">
+      <c r="T42" s="184" t="s">
         <v>170</v>
       </c>
-      <c r="U42" s="210"/>
-      <c r="V42" s="210"/>
-      <c r="W42" s="210"/>
-      <c r="X42" s="210"/>
-      <c r="Y42" s="210"/>
-      <c r="Z42" s="210"/>
-      <c r="AA42" s="210"/>
-      <c r="AB42" s="210"/>
-      <c r="AC42" s="211"/>
+      <c r="U42" s="185"/>
+      <c r="V42" s="185"/>
+      <c r="W42" s="185"/>
+      <c r="X42" s="185"/>
+      <c r="Y42" s="185"/>
+      <c r="Z42" s="185"/>
+      <c r="AA42" s="185"/>
+      <c r="AB42" s="185"/>
+      <c r="AC42" s="186"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
       <c r="B43" s="2">
@@ -6422,30 +6425,30 @@
       <c r="F43" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G43" s="218" t="s">
+      <c r="G43" s="263" t="s">
         <v>190</v>
       </c>
-      <c r="H43" s="219"/>
-      <c r="I43" s="219"/>
-      <c r="J43" s="220"/>
+      <c r="H43" s="187"/>
+      <c r="I43" s="187"/>
+      <c r="J43" s="188"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T43" s="209" t="s">
+      <c r="T43" s="184" t="s">
         <v>171</v>
       </c>
-      <c r="U43" s="210"/>
-      <c r="V43" s="210"/>
-      <c r="W43" s="210"/>
-      <c r="X43" s="210"/>
-      <c r="Y43" s="210"/>
-      <c r="Z43" s="210"/>
-      <c r="AA43" s="210"/>
-      <c r="AB43" s="210"/>
-      <c r="AC43" s="211"/>
+      <c r="U43" s="185"/>
+      <c r="V43" s="185"/>
+      <c r="W43" s="185"/>
+      <c r="X43" s="185"/>
+      <c r="Y43" s="185"/>
+      <c r="Z43" s="185"/>
+      <c r="AA43" s="185"/>
+      <c r="AB43" s="185"/>
+      <c r="AC43" s="186"/>
     </row>
     <row r="44" spans="2:29" ht="45.75" thickBot="1">
       <c r="B44" s="2">
@@ -6466,21 +6469,21 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="292" t="s">
+      <c r="S44" s="189" t="s">
         <v>75</v>
       </c>
-      <c r="T44" s="294" t="s">
+      <c r="T44" s="191" t="s">
         <v>172</v>
       </c>
-      <c r="U44" s="295"/>
-      <c r="V44" s="295"/>
-      <c r="W44" s="295"/>
-      <c r="X44" s="295"/>
-      <c r="Y44" s="295"/>
-      <c r="Z44" s="295"/>
-      <c r="AA44" s="295"/>
-      <c r="AB44" s="295"/>
-      <c r="AC44" s="296"/>
+      <c r="U44" s="192"/>
+      <c r="V44" s="192"/>
+      <c r="W44" s="192"/>
+      <c r="X44" s="192"/>
+      <c r="Y44" s="192"/>
+      <c r="Z44" s="192"/>
+      <c r="AA44" s="192"/>
+      <c r="AB44" s="192"/>
+      <c r="AC44" s="193"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1">
       <c r="B45" s="2">
@@ -6498,26 +6501,26 @@
       <c r="F45" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="G45" s="203" t="s">
+      <c r="G45" s="200" t="s">
         <v>179</v>
       </c>
-      <c r="H45" s="204"/>
-      <c r="I45" s="204"/>
-      <c r="J45" s="205"/>
+      <c r="H45" s="201"/>
+      <c r="I45" s="201"/>
+      <c r="J45" s="202"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="293"/>
-      <c r="T45" s="297"/>
-      <c r="U45" s="298"/>
-      <c r="V45" s="298"/>
-      <c r="W45" s="298"/>
-      <c r="X45" s="298"/>
-      <c r="Y45" s="298"/>
-      <c r="Z45" s="298"/>
-      <c r="AA45" s="298"/>
-      <c r="AB45" s="298"/>
-      <c r="AC45" s="299"/>
+      <c r="S45" s="190"/>
+      <c r="T45" s="194"/>
+      <c r="U45" s="195"/>
+      <c r="V45" s="195"/>
+      <c r="W45" s="195"/>
+      <c r="X45" s="195"/>
+      <c r="Y45" s="195"/>
+      <c r="Z45" s="195"/>
+      <c r="AA45" s="195"/>
+      <c r="AB45" s="195"/>
+      <c r="AC45" s="196"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
       <c r="B46" s="2">
@@ -6535,28 +6538,28 @@
       <c r="F46" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="G46" s="240"/>
-      <c r="H46" s="241"/>
-      <c r="I46" s="241"/>
-      <c r="J46" s="242"/>
+      <c r="G46" s="203"/>
+      <c r="H46" s="204"/>
+      <c r="I46" s="204"/>
+      <c r="J46" s="205"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="T46" s="206" t="s">
+      <c r="T46" s="197" t="s">
         <v>173</v>
       </c>
-      <c r="U46" s="207"/>
-      <c r="V46" s="207"/>
-      <c r="W46" s="207"/>
-      <c r="X46" s="207"/>
-      <c r="Y46" s="207"/>
-      <c r="Z46" s="207"/>
-      <c r="AA46" s="207"/>
-      <c r="AB46" s="207"/>
-      <c r="AC46" s="208"/>
+      <c r="U46" s="198"/>
+      <c r="V46" s="198"/>
+      <c r="W46" s="198"/>
+      <c r="X46" s="198"/>
+      <c r="Y46" s="198"/>
+      <c r="Z46" s="198"/>
+      <c r="AA46" s="198"/>
+      <c r="AB46" s="198"/>
+      <c r="AC46" s="199"/>
     </row>
     <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
       <c r="B47" s="2">
@@ -6574,12 +6577,12 @@
       <c r="F47" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="G47" s="219" t="s">
+      <c r="G47" s="187" t="s">
         <v>150</v>
       </c>
-      <c r="H47" s="219"/>
-      <c r="I47" s="219"/>
-      <c r="J47" s="220"/>
+      <c r="H47" s="187"/>
+      <c r="I47" s="187"/>
+      <c r="J47" s="188"/>
     </row>
     <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
       <c r="B48" s="2">
@@ -6617,12 +6620,12 @@
       <c r="F49" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="G49" s="203" t="s">
+      <c r="G49" s="200" t="s">
         <v>153</v>
       </c>
-      <c r="H49" s="204"/>
-      <c r="I49" s="204"/>
-      <c r="J49" s="205"/>
+      <c r="H49" s="201"/>
+      <c r="I49" s="201"/>
+      <c r="J49" s="202"/>
     </row>
     <row r="50" spans="2:10" ht="30" customHeight="1">
       <c r="B50" s="2">
@@ -6640,10 +6643,10 @@
       <c r="F50" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="G50" s="237"/>
-      <c r="H50" s="238"/>
-      <c r="I50" s="238"/>
-      <c r="J50" s="239"/>
+      <c r="G50" s="206"/>
+      <c r="H50" s="207"/>
+      <c r="I50" s="207"/>
+      <c r="J50" s="208"/>
     </row>
     <row r="51" spans="2:10" ht="32.25" customHeight="1" thickBot="1">
       <c r="B51" s="4">
@@ -6661,50 +6664,50 @@
       <c r="F51" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="G51" s="240"/>
-      <c r="H51" s="241"/>
-      <c r="I51" s="241"/>
-      <c r="J51" s="242"/>
+      <c r="G51" s="203"/>
+      <c r="H51" s="204"/>
+      <c r="I51" s="204"/>
+      <c r="J51" s="205"/>
     </row>
     <row r="52" spans="2:10" ht="30.75" customHeight="1" thickBot="1">
-      <c r="B52" s="221" t="s">
+      <c r="B52" s="258" t="s">
         <v>140</v>
       </c>
-      <c r="C52" s="222"/>
-      <c r="D52" s="222"/>
-      <c r="E52" s="222"/>
-      <c r="F52" s="223"/>
+      <c r="C52" s="239"/>
+      <c r="D52" s="239"/>
+      <c r="E52" s="239"/>
+      <c r="F52" s="240"/>
     </row>
     <row r="53" spans="2:10" ht="31.5" customHeight="1" thickBot="1"/>
     <row r="54" spans="2:10" ht="24.75" customHeight="1">
-      <c r="B54" s="245" t="s">
+      <c r="B54" s="252" t="s">
         <v>181</v>
       </c>
-      <c r="C54" s="243" t="s">
+      <c r="C54" s="250" t="s">
         <v>183</v>
       </c>
-      <c r="D54" s="233" t="s">
+      <c r="D54" s="264" t="s">
         <v>182</v>
       </c>
-      <c r="E54" s="234"/>
+      <c r="E54" s="265"/>
     </row>
     <row r="55" spans="2:10" ht="24" customHeight="1" thickBot="1">
-      <c r="B55" s="246"/>
-      <c r="C55" s="244"/>
-      <c r="D55" s="235"/>
-      <c r="E55" s="236"/>
-    </row>
-    <row r="56" spans="2:10" ht="41.25" customHeight="1">
+      <c r="B55" s="253"/>
+      <c r="C55" s="251"/>
+      <c r="D55" s="266"/>
+      <c r="E55" s="267"/>
+    </row>
+    <row r="56" spans="2:10" ht="41.25" customHeight="1" thickBot="1">
       <c r="B56" s="81">
         <v>0</v>
       </c>
       <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D56" s="212" t="s">
+      <c r="D56" s="181" t="s">
         <v>205</v>
       </c>
-      <c r="E56" s="214"/>
+      <c r="E56" s="183"/>
     </row>
     <row r="57" spans="2:10" ht="31.5" customHeight="1">
       <c r="B57" s="82">
@@ -6713,22 +6716,32 @@
       <c r="C57" s="85" t="s">
         <v>201</v>
       </c>
-      <c r="D57" s="229" t="s">
+      <c r="D57" s="254" t="s">
         <v>204</v>
       </c>
-      <c r="E57" s="230"/>
-    </row>
-    <row r="58" spans="2:10" ht="30.75" customHeight="1">
+      <c r="E57" s="255"/>
+      <c r="F57" s="200" t="s">
+        <v>344</v>
+      </c>
+      <c r="G57" s="201"/>
+      <c r="H57" s="201"/>
+      <c r="I57" s="202"/>
+    </row>
+    <row r="58" spans="2:10" ht="30.75" customHeight="1" thickBot="1">
       <c r="B58" s="82">
         <v>2</v>
       </c>
       <c r="C58" s="38" t="s">
         <v>202</v>
       </c>
-      <c r="D58" s="229" t="s">
+      <c r="D58" s="254" t="s">
         <v>203</v>
       </c>
-      <c r="E58" s="230"/>
+      <c r="E58" s="255"/>
+      <c r="F58" s="203"/>
+      <c r="G58" s="204"/>
+      <c r="H58" s="204"/>
+      <c r="I58" s="205"/>
     </row>
     <row r="59" spans="2:10" ht="33.75" customHeight="1">
       <c r="B59" s="82">
@@ -6737,10 +6750,10 @@
       <c r="C59" s="85" t="s">
         <v>184</v>
       </c>
-      <c r="D59" s="229" t="s">
+      <c r="D59" s="254" t="s">
         <v>187</v>
       </c>
-      <c r="E59" s="230"/>
+      <c r="E59" s="255"/>
     </row>
     <row r="60" spans="2:10" ht="28.5" customHeight="1">
       <c r="B60" s="82">
@@ -6749,10 +6762,10 @@
       <c r="C60" s="38" t="s">
         <v>185</v>
       </c>
-      <c r="D60" s="229" t="s">
+      <c r="D60" s="254" t="s">
         <v>188</v>
       </c>
-      <c r="E60" s="230"/>
+      <c r="E60" s="255"/>
     </row>
     <row r="61" spans="2:10" ht="40.5" customHeight="1">
       <c r="B61" s="82">
@@ -6761,10 +6774,10 @@
       <c r="C61" s="38" t="s">
         <v>186</v>
       </c>
-      <c r="D61" s="229" t="s">
+      <c r="D61" s="254" t="s">
         <v>189</v>
       </c>
-      <c r="E61" s="230"/>
+      <c r="E61" s="255"/>
     </row>
     <row r="62" spans="2:10" ht="53.25" customHeight="1">
       <c r="B62" s="82">
@@ -6773,106 +6786,201 @@
       <c r="C62" s="85" t="s">
         <v>194</v>
       </c>
-      <c r="D62" s="229" t="s">
+      <c r="D62" s="254" t="s">
         <v>195</v>
       </c>
-      <c r="E62" s="230"/>
+      <c r="E62" s="255"/>
     </row>
     <row r="63" spans="2:10" ht="36" customHeight="1">
       <c r="B63" s="82">
         <v>7</v>
       </c>
       <c r="C63" s="85"/>
-      <c r="D63" s="229"/>
-      <c r="E63" s="230"/>
+      <c r="D63" s="254"/>
+      <c r="E63" s="255"/>
     </row>
     <row r="64" spans="2:10" ht="40.5" customHeight="1">
       <c r="B64" s="82">
         <v>8</v>
       </c>
       <c r="C64" s="85"/>
-      <c r="D64" s="229"/>
-      <c r="E64" s="230"/>
+      <c r="D64" s="254"/>
+      <c r="E64" s="255"/>
     </row>
     <row r="65" spans="2:5">
       <c r="B65" s="82">
         <v>9</v>
       </c>
       <c r="C65" s="85"/>
-      <c r="D65" s="229"/>
-      <c r="E65" s="230"/>
+      <c r="D65" s="254"/>
+      <c r="E65" s="255"/>
     </row>
     <row r="66" spans="2:5" ht="30" customHeight="1">
       <c r="B66" s="82">
         <v>10</v>
       </c>
       <c r="C66" s="85"/>
-      <c r="D66" s="229"/>
-      <c r="E66" s="230"/>
+      <c r="D66" s="254"/>
+      <c r="E66" s="255"/>
     </row>
     <row r="67" spans="2:5">
       <c r="B67" s="82">
         <v>11</v>
       </c>
       <c r="C67" s="85"/>
-      <c r="D67" s="229"/>
-      <c r="E67" s="230"/>
+      <c r="D67" s="254"/>
+      <c r="E67" s="255"/>
     </row>
     <row r="68" spans="2:5">
       <c r="B68" s="82">
         <v>12</v>
       </c>
       <c r="C68" s="85"/>
-      <c r="D68" s="229"/>
-      <c r="E68" s="230"/>
+      <c r="D68" s="254"/>
+      <c r="E68" s="255"/>
     </row>
     <row r="69" spans="2:5">
       <c r="B69" s="82">
         <v>13</v>
       </c>
       <c r="C69" s="85"/>
-      <c r="D69" s="229"/>
-      <c r="E69" s="230"/>
+      <c r="D69" s="254"/>
+      <c r="E69" s="255"/>
     </row>
     <row r="70" spans="2:5" ht="30" customHeight="1">
       <c r="B70" s="82">
         <v>14</v>
       </c>
       <c r="C70" s="85"/>
-      <c r="D70" s="229"/>
-      <c r="E70" s="230"/>
+      <c r="D70" s="254"/>
+      <c r="E70" s="255"/>
     </row>
     <row r="71" spans="2:5" ht="15.75" thickBot="1">
       <c r="B71" s="83">
         <v>15</v>
       </c>
       <c r="C71" s="86"/>
-      <c r="D71" s="231"/>
-      <c r="E71" s="232"/>
+      <c r="D71" s="261"/>
+      <c r="E71" s="262"/>
     </row>
     <row r="75" spans="2:5" ht="72" customHeight="1"/>
   </sheetData>
-  <mergeCells count="158">
-    <mergeCell ref="T30:AC30"/>
-    <mergeCell ref="T31:AC31"/>
-    <mergeCell ref="T32:AC32"/>
-    <mergeCell ref="T33:AC33"/>
-    <mergeCell ref="T34:AC34"/>
-    <mergeCell ref="T35:AC35"/>
-    <mergeCell ref="T36:AC36"/>
-    <mergeCell ref="T37:AC37"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="S38:S39"/>
-    <mergeCell ref="T38:AC39"/>
-    <mergeCell ref="S44:S45"/>
-    <mergeCell ref="T44:AC45"/>
-    <mergeCell ref="T40:AC40"/>
-    <mergeCell ref="T41:AC41"/>
-    <mergeCell ref="T42:AC42"/>
-    <mergeCell ref="T43:AC43"/>
-    <mergeCell ref="T46:AC46"/>
-    <mergeCell ref="G45:J46"/>
-    <mergeCell ref="G39:J42"/>
+  <mergeCells count="159">
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D54:E55"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="F57:I58"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="AA7:AB7"/>
+    <mergeCell ref="AA28:AB28"/>
+    <mergeCell ref="AA12:AB12"/>
+    <mergeCell ref="AA13:AB13"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AA25:AB25"/>
+    <mergeCell ref="AA26:AB26"/>
+    <mergeCell ref="U27:V27"/>
+    <mergeCell ref="AA27:AB27"/>
+    <mergeCell ref="U12:V12"/>
+    <mergeCell ref="AA14:AB14"/>
+    <mergeCell ref="U28:V28"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="N20:P20"/>
+    <mergeCell ref="N21:P21"/>
+    <mergeCell ref="N23:P23"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AA11:AB11"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="N26:P26"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="N24:P24"/>
+    <mergeCell ref="E27:J27"/>
+    <mergeCell ref="E22:J22"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K2:P2"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AA17:AB17"/>
+    <mergeCell ref="AA18:AB18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="N13:P13"/>
     <mergeCell ref="AA20:AB20"/>
     <mergeCell ref="AA21:AB21"/>
     <mergeCell ref="AA22:AB22"/>
@@ -6897,120 +7005,26 @@
     <mergeCell ref="U11:V11"/>
     <mergeCell ref="AA23:AB23"/>
     <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AA17:AB17"/>
-    <mergeCell ref="AA18:AB18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="AA19:AB19"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="N27:P27"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="E28:J28"/>
-    <mergeCell ref="N24:P24"/>
-    <mergeCell ref="E27:J27"/>
-    <mergeCell ref="E22:J22"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K2:P2"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AA11:AB11"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B52:F52"/>
-    <mergeCell ref="AA7:AB7"/>
-    <mergeCell ref="AA28:AB28"/>
-    <mergeCell ref="AA12:AB12"/>
-    <mergeCell ref="AA13:AB13"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AA25:AB25"/>
-    <mergeCell ref="AA26:AB26"/>
-    <mergeCell ref="U27:V27"/>
-    <mergeCell ref="AA27:AB27"/>
-    <mergeCell ref="U12:V12"/>
-    <mergeCell ref="AA14:AB14"/>
-    <mergeCell ref="U28:V28"/>
-    <mergeCell ref="N17:P17"/>
-    <mergeCell ref="N19:P19"/>
-    <mergeCell ref="N20:P20"/>
-    <mergeCell ref="N21:P21"/>
-    <mergeCell ref="N23:P23"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D54:E55"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="T30:AC30"/>
+    <mergeCell ref="T31:AC31"/>
+    <mergeCell ref="T32:AC32"/>
+    <mergeCell ref="T33:AC33"/>
+    <mergeCell ref="T34:AC34"/>
+    <mergeCell ref="T35:AC35"/>
+    <mergeCell ref="T36:AC36"/>
+    <mergeCell ref="T37:AC37"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="S38:S39"/>
+    <mergeCell ref="T38:AC39"/>
+    <mergeCell ref="S44:S45"/>
+    <mergeCell ref="T44:AC45"/>
+    <mergeCell ref="T40:AC40"/>
+    <mergeCell ref="T41:AC41"/>
+    <mergeCell ref="T42:AC42"/>
+    <mergeCell ref="T43:AC43"/>
+    <mergeCell ref="T46:AC46"/>
+    <mergeCell ref="G45:J46"/>
+    <mergeCell ref="G39:J42"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7064,35 +7078,35 @@
       <c r="F2" s="102" t="s">
         <v>210</v>
       </c>
-      <c r="G2" s="203" t="s">
+      <c r="G2" s="200" t="s">
         <v>211</v>
       </c>
-      <c r="H2" s="204"/>
-      <c r="I2" s="204"/>
-      <c r="J2" s="205"/>
-      <c r="L2" s="194" t="s">
+      <c r="H2" s="201"/>
+      <c r="I2" s="201"/>
+      <c r="J2" s="202"/>
+      <c r="L2" s="292" t="s">
         <v>330</v>
       </c>
-      <c r="M2" s="195"/>
-      <c r="N2" s="195"/>
-      <c r="O2" s="196"/>
+      <c r="M2" s="293"/>
+      <c r="N2" s="293"/>
+      <c r="O2" s="294"/>
       <c r="P2" s="132"/>
-      <c r="Q2" s="197" t="s">
+      <c r="Q2" s="295" t="s">
         <v>290</v>
       </c>
-      <c r="R2" s="198"/>
-      <c r="S2" s="198"/>
-      <c r="T2" s="199"/>
+      <c r="R2" s="296"/>
+      <c r="S2" s="296"/>
+      <c r="T2" s="297"/>
       <c r="U2" s="132"/>
-      <c r="V2" s="187" t="s">
+      <c r="V2" s="289" t="s">
         <v>313</v>
       </c>
-      <c r="W2" s="188"/>
-      <c r="X2" s="188"/>
-      <c r="Y2" s="188"/>
-      <c r="Z2" s="188"/>
-      <c r="AA2" s="188"/>
-      <c r="AB2" s="189"/>
+      <c r="W2" s="290"/>
+      <c r="X2" s="290"/>
+      <c r="Y2" s="290"/>
+      <c r="Z2" s="290"/>
+      <c r="AA2" s="290"/>
+      <c r="AB2" s="291"/>
     </row>
     <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B3" s="89" t="s">
@@ -7114,11 +7128,11 @@
       <c r="G3" s="92" t="s">
         <v>212</v>
       </c>
-      <c r="H3" s="212" t="s">
+      <c r="H3" s="181" t="s">
         <v>216</v>
       </c>
-      <c r="I3" s="213"/>
-      <c r="J3" s="214"/>
+      <c r="I3" s="182"/>
+      <c r="J3" s="183"/>
       <c r="L3" s="144" t="s">
         <v>276</v>
       </c>
@@ -7157,11 +7171,11 @@
       <c r="Y3" s="170" t="s">
         <v>279</v>
       </c>
-      <c r="Z3" s="178" t="s">
+      <c r="Z3" s="280" t="s">
         <v>318</v>
       </c>
-      <c r="AA3" s="179"/>
-      <c r="AB3" s="180"/>
+      <c r="AA3" s="281"/>
+      <c r="AB3" s="282"/>
     </row>
     <row r="4" spans="2:28" ht="53.25" customHeight="1">
       <c r="B4" s="90" t="s">
@@ -7183,11 +7197,11 @@
       <c r="G4" s="93" t="s">
         <v>213</v>
       </c>
-      <c r="H4" s="209">
+      <c r="H4" s="184">
         <v>63</v>
       </c>
-      <c r="I4" s="210"/>
-      <c r="J4" s="211"/>
+      <c r="I4" s="185"/>
+      <c r="J4" s="186"/>
       <c r="L4" s="150" t="s">
         <v>245</v>
       </c>
@@ -7226,11 +7240,11 @@
       <c r="Y4" s="137" t="s">
         <v>316</v>
       </c>
-      <c r="Z4" s="181" t="s">
+      <c r="Z4" s="283" t="s">
         <v>319</v>
       </c>
-      <c r="AA4" s="182"/>
-      <c r="AB4" s="183"/>
+      <c r="AA4" s="284"/>
+      <c r="AB4" s="285"/>
     </row>
     <row r="5" spans="2:28" ht="47.25" customHeight="1">
       <c r="B5" s="90" t="s">
@@ -7252,11 +7266,11 @@
       <c r="G5" s="93" t="s">
         <v>214</v>
       </c>
-      <c r="H5" s="209">
+      <c r="H5" s="184">
         <v>31</v>
       </c>
-      <c r="I5" s="210"/>
-      <c r="J5" s="211"/>
+      <c r="I5" s="185"/>
+      <c r="J5" s="186"/>
       <c r="L5" s="148" t="s">
         <v>254</v>
       </c>
@@ -7295,9 +7309,9 @@
       <c r="Y5" s="134" t="s">
         <v>293</v>
       </c>
-      <c r="Z5" s="181"/>
-      <c r="AA5" s="182"/>
-      <c r="AB5" s="183"/>
+      <c r="Z5" s="283"/>
+      <c r="AA5" s="284"/>
+      <c r="AB5" s="285"/>
     </row>
     <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B6" s="107" t="s">
@@ -7319,11 +7333,11 @@
       <c r="G6" s="94" t="s">
         <v>215</v>
       </c>
-      <c r="H6" s="206">
+      <c r="H6" s="197">
         <v>7</v>
       </c>
-      <c r="I6" s="207"/>
-      <c r="J6" s="208"/>
+      <c r="I6" s="198"/>
+      <c r="J6" s="199"/>
       <c r="L6" s="151" t="s">
         <v>240</v>
       </c>
@@ -7362,9 +7376,9 @@
       <c r="Y6" s="143" t="s">
         <v>315</v>
       </c>
-      <c r="Z6" s="184"/>
-      <c r="AA6" s="185"/>
-      <c r="AB6" s="186"/>
+      <c r="Z6" s="286"/>
+      <c r="AA6" s="287"/>
+      <c r="AB6" s="288"/>
     </row>
     <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1">
       <c r="B7" s="89" t="s">
@@ -7386,12 +7400,12 @@
       <c r="G7" s="87" t="s">
         <v>273</v>
       </c>
-      <c r="H7" s="200" t="str">
+      <c r="H7" s="275" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12))</f>
         <v>E3FFF000</v>
       </c>
-      <c r="I7" s="201"/>
-      <c r="J7" s="202"/>
+      <c r="I7" s="276"/>
+      <c r="J7" s="277"/>
       <c r="L7" s="149" t="s">
         <v>265</v>
       </c>
@@ -7439,18 +7453,18 @@
       <c r="G8" s="87" t="s">
         <v>217</v>
       </c>
-      <c r="H8" s="200" t="str">
+      <c r="H8" s="275" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12)+4095)</f>
         <v>E3FFFFFF</v>
       </c>
-      <c r="I8" s="201"/>
-      <c r="J8" s="202"/>
-      <c r="L8" s="218" t="s">
+      <c r="I8" s="276"/>
+      <c r="J8" s="277"/>
+      <c r="L8" s="263" t="s">
         <v>332</v>
       </c>
-      <c r="M8" s="219"/>
-      <c r="N8" s="219"/>
-      <c r="O8" s="220"/>
+      <c r="M8" s="187"/>
+      <c r="N8" s="187"/>
+      <c r="O8" s="188"/>
       <c r="P8" s="132"/>
       <c r="Q8" s="163" t="s">
         <v>285</v>
@@ -7559,12 +7573,12 @@
       <c r="N11" s="132"/>
       <c r="O11" s="132"/>
       <c r="P11" s="132"/>
-      <c r="Q11" s="215" t="s">
+      <c r="Q11" s="298" t="s">
         <v>312</v>
       </c>
-      <c r="R11" s="216"/>
-      <c r="S11" s="216"/>
-      <c r="T11" s="217"/>
+      <c r="R11" s="299"/>
+      <c r="S11" s="299"/>
+      <c r="T11" s="300"/>
       <c r="U11" s="132"/>
     </row>
     <row r="12" spans="2:28" ht="44.25" customHeight="1" thickBot="1">
@@ -7716,12 +7730,12 @@
       <c r="F16" s="123" t="s">
         <v>232</v>
       </c>
-      <c r="G16" s="221" t="s">
+      <c r="G16" s="258" t="s">
         <v>270</v>
       </c>
-      <c r="H16" s="222"/>
-      <c r="I16" s="222"/>
-      <c r="J16" s="223"/>
+      <c r="H16" s="239"/>
+      <c r="I16" s="239"/>
+      <c r="J16" s="240"/>
       <c r="Q16" s="166" t="s">
         <v>306</v>
       </c>
@@ -7736,10 +7750,10 @@
       </c>
     </row>
     <row r="17" spans="2:20" ht="60.75" customHeight="1" thickBot="1">
-      <c r="B17" s="192" t="s">
+      <c r="B17" s="270" t="s">
         <v>233</v>
       </c>
-      <c r="C17" s="190" t="s">
+      <c r="C17" s="268" t="s">
         <v>234</v>
       </c>
       <c r="D17" s="124" t="s">
@@ -7751,12 +7765,12 @@
       <c r="F17" s="126" t="s">
         <v>236</v>
       </c>
-      <c r="G17" s="224" t="s">
+      <c r="G17" s="272" t="s">
         <v>271</v>
       </c>
-      <c r="H17" s="225"/>
-      <c r="I17" s="225"/>
-      <c r="J17" s="226"/>
+      <c r="H17" s="273"/>
+      <c r="I17" s="273"/>
+      <c r="J17" s="274"/>
       <c r="Q17" s="167" t="s">
         <v>309</v>
       </c>
@@ -7771,8 +7785,8 @@
       </c>
     </row>
     <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B18" s="227"/>
-      <c r="C18" s="228"/>
+      <c r="B18" s="278"/>
+      <c r="C18" s="279"/>
       <c r="D18" s="111" t="s">
         <v>237</v>
       </c>
@@ -7782,16 +7796,16 @@
       <c r="F18" s="114" t="s">
         <v>239</v>
       </c>
-      <c r="G18" s="200" t="s">
+      <c r="G18" s="275" t="s">
         <v>272</v>
       </c>
-      <c r="H18" s="201"/>
-      <c r="I18" s="201"/>
-      <c r="J18" s="202"/>
+      <c r="H18" s="276"/>
+      <c r="I18" s="276"/>
+      <c r="J18" s="277"/>
     </row>
     <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B19" s="193"/>
-      <c r="C19" s="191"/>
+      <c r="B19" s="271"/>
+      <c r="C19" s="269"/>
       <c r="D19" s="116" t="s">
         <v>240</v>
       </c>
@@ -7807,10 +7821,10 @@
       <c r="J19" s="15"/>
     </row>
     <row r="20" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B20" s="192" t="s">
+      <c r="B20" s="270" t="s">
         <v>243</v>
       </c>
-      <c r="C20" s="190" t="s">
+      <c r="C20" s="268" t="s">
         <v>244</v>
       </c>
       <c r="D20" s="124" t="s">
@@ -7828,8 +7842,8 @@
       <c r="J20" s="15"/>
     </row>
     <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B21" s="193"/>
-      <c r="C21" s="191"/>
+      <c r="B21" s="271"/>
+      <c r="C21" s="269"/>
       <c r="D21" s="116" t="s">
         <v>247</v>
       </c>
@@ -7845,10 +7859,10 @@
       <c r="J21" s="15"/>
     </row>
     <row r="22" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B22" s="192" t="s">
+      <c r="B22" s="270" t="s">
         <v>249</v>
       </c>
-      <c r="C22" s="190" t="s">
+      <c r="C22" s="268" t="s">
         <v>250</v>
       </c>
       <c r="D22" s="124" t="s">
@@ -7866,8 +7880,8 @@
       <c r="J22" s="15"/>
     </row>
     <row r="23" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B23" s="193"/>
-      <c r="C23" s="191"/>
+      <c r="B23" s="271"/>
+      <c r="C23" s="269"/>
       <c r="D23" s="116" t="s">
         <v>243</v>
       </c>
@@ -7883,10 +7897,10 @@
       <c r="J23" s="15"/>
     </row>
     <row r="24" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B24" s="192" t="s">
+      <c r="B24" s="270" t="s">
         <v>254</v>
       </c>
-      <c r="C24" s="190" t="s">
+      <c r="C24" s="268" t="s">
         <v>255</v>
       </c>
       <c r="D24" s="124" t="s">
@@ -7904,8 +7918,8 @@
       <c r="J24" s="15"/>
     </row>
     <row r="25" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B25" s="193"/>
-      <c r="C25" s="191"/>
+      <c r="B25" s="271"/>
+      <c r="C25" s="269"/>
       <c r="D25" s="116" t="s">
         <v>249</v>
       </c>
@@ -7942,10 +7956,10 @@
       <c r="J26" s="15"/>
     </row>
     <row r="27" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B27" s="192" t="s">
+      <c r="B27" s="270" t="s">
         <v>237</v>
       </c>
-      <c r="C27" s="190" t="s">
+      <c r="C27" s="268" t="s">
         <v>261</v>
       </c>
       <c r="D27" s="124" t="s">
@@ -7963,8 +7977,8 @@
       <c r="J27" s="15"/>
     </row>
     <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B28" s="193"/>
-      <c r="C28" s="191"/>
+      <c r="B28" s="271"/>
+      <c r="C28" s="269"/>
       <c r="D28" s="116" t="s">
         <v>254</v>
       </c>
@@ -7980,10 +7994,10 @@
       <c r="J28" s="15"/>
     </row>
     <row r="29" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B29" s="192" t="s">
+      <c r="B29" s="270" t="s">
         <v>265</v>
       </c>
-      <c r="C29" s="190" t="s">
+      <c r="C29" s="268" t="s">
         <v>266</v>
       </c>
       <c r="D29" s="124" t="s">
@@ -8001,8 +8015,8 @@
       <c r="J29" s="15"/>
     </row>
     <row r="30" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B30" s="193"/>
-      <c r="C30" s="191"/>
+      <c r="B30" s="271"/>
+      <c r="C30" s="269"/>
       <c r="D30" s="116" t="s">
         <v>258</v>
       </c>
@@ -8019,19 +8033,6 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C17:C19"/>
     <mergeCell ref="Z3:AB3"/>
     <mergeCell ref="Z4:AB6"/>
     <mergeCell ref="V2:AB2"/>
@@ -8048,6 +8049,19 @@
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="Q11:T11"/>
     <mergeCell ref="L8:O8"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="C17:C19"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fallo la prueba 8, se requiere re hacer la MMU. Luego hay que re probar los casos
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C68A95A-94BF-46F8-8B68-D866329A350D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE3E799-9A91-48EA-9637-D3E5CB207745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="344">
   <si>
     <t>OpCode</t>
   </si>
@@ -571,9 +571,6 @@
   </si>
   <si>
     <t>En_TLB</t>
-  </si>
-  <si>
-    <t>En_Interrup</t>
   </si>
   <si>
     <t>Nota: Dentro de ALU/Branch Unit</t>
@@ -2956,29 +2953,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2986,37 +2974,22 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3028,6 +3001,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3037,155 +3019,23 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3196,32 +3046,215 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -3235,6 +3268,42 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3242,15 +3311,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3258,69 +3318,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3634,62 +3631,62 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B2" s="224" t="s">
+      <c r="B2" s="234" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="233" t="s">
+      <c r="C2" s="249" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="234"/>
-      <c r="E2" s="235" t="s">
+      <c r="D2" s="250"/>
+      <c r="E2" s="251" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="235"/>
-      <c r="G2" s="236" t="s">
+      <c r="F2" s="251"/>
+      <c r="G2" s="252" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="235"/>
-      <c r="I2" s="235" t="s">
+      <c r="H2" s="251"/>
+      <c r="I2" s="251" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="235"/>
-      <c r="K2" s="237" t="s">
+      <c r="J2" s="251"/>
+      <c r="K2" s="253" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="235"/>
-      <c r="M2" s="235"/>
-      <c r="N2" s="235"/>
-      <c r="O2" s="235"/>
-      <c r="P2" s="238"/>
-      <c r="R2" s="243" t="s">
+      <c r="L2" s="251"/>
+      <c r="M2" s="251"/>
+      <c r="N2" s="251"/>
+      <c r="O2" s="251"/>
+      <c r="P2" s="254"/>
+      <c r="R2" s="230" t="s">
         <v>65</v>
       </c>
-      <c r="S2" s="180" t="s">
+      <c r="S2" s="227" t="s">
         <v>66</v>
       </c>
-      <c r="T2" s="247" t="s">
+      <c r="T2" s="220" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="248"/>
-      <c r="V2" s="248"/>
-      <c r="W2" s="248"/>
-      <c r="X2" s="248"/>
-      <c r="Y2" s="248"/>
-      <c r="Z2" s="248"/>
-      <c r="AA2" s="248"/>
-      <c r="AB2" s="248" t="s">
+      <c r="U2" s="221"/>
+      <c r="V2" s="221"/>
+      <c r="W2" s="221"/>
+      <c r="X2" s="221"/>
+      <c r="Y2" s="221"/>
+      <c r="Z2" s="221"/>
+      <c r="AA2" s="221"/>
+      <c r="AB2" s="221" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="248"/>
-      <c r="AD2" s="248"/>
-      <c r="AE2" s="248"/>
-      <c r="AF2" s="248"/>
-      <c r="AG2" s="248"/>
-      <c r="AH2" s="248"/>
-      <c r="AI2" s="249"/>
+      <c r="AC2" s="221"/>
+      <c r="AD2" s="221"/>
+      <c r="AE2" s="221"/>
+      <c r="AF2" s="221"/>
+      <c r="AG2" s="221"/>
+      <c r="AH2" s="221"/>
+      <c r="AI2" s="222"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B3" s="225"/>
+      <c r="B3" s="235"/>
       <c r="C3" s="16" t="s">
         <v>79</v>
       </c>
@@ -3714,21 +3711,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="230"/>
-      <c r="L3" s="231"/>
-      <c r="M3" s="231"/>
-      <c r="N3" s="231"/>
-      <c r="O3" s="231"/>
-      <c r="P3" s="232"/>
-      <c r="R3" s="244"/>
-      <c r="S3" s="241"/>
+      <c r="K3" s="205"/>
+      <c r="L3" s="248"/>
+      <c r="M3" s="248"/>
+      <c r="N3" s="248"/>
+      <c r="O3" s="248"/>
+      <c r="P3" s="206"/>
+      <c r="R3" s="231"/>
+      <c r="S3" s="228"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="211" t="s">
+      <c r="U3" s="258" t="s">
         <v>83</v>
       </c>
-      <c r="V3" s="211"/>
+      <c r="V3" s="258"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -3741,10 +3738,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="246" t="s">
+      <c r="AA3" s="219" t="s">
         <v>74</v>
       </c>
-      <c r="AB3" s="246"/>
+      <c r="AB3" s="219"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -3768,21 +3765,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B4" s="226"/>
+      <c r="B4" s="236"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="212" t="s">
+      <c r="E4" s="223" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="239"/>
-      <c r="G4" s="239"/>
-      <c r="H4" s="239"/>
-      <c r="I4" s="239"/>
-      <c r="J4" s="240"/>
+      <c r="F4" s="210"/>
+      <c r="G4" s="210"/>
+      <c r="H4" s="210"/>
+      <c r="I4" s="210"/>
+      <c r="J4" s="211"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -3792,20 +3789,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="212" t="s">
+      <c r="N4" s="223" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="239"/>
-      <c r="P4" s="240"/>
-      <c r="R4" s="245"/>
-      <c r="S4" s="242"/>
+      <c r="O4" s="210"/>
+      <c r="P4" s="211"/>
+      <c r="R4" s="232"/>
+      <c r="S4" s="229"/>
       <c r="T4" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="U4" s="212" t="s">
+      <c r="U4" s="223" t="s">
         <v>75</v>
       </c>
-      <c r="V4" s="213"/>
+      <c r="V4" s="224"/>
       <c r="W4" s="7" t="s">
         <v>71</v>
       </c>
@@ -3818,10 +3815,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="212" t="s">
+      <c r="AA4" s="223" t="s">
         <v>72</v>
       </c>
-      <c r="AB4" s="213"/>
+      <c r="AB4" s="224"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -3853,22 +3850,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="216"/>
-      <c r="F5" s="217"/>
-      <c r="G5" s="217"/>
-      <c r="H5" s="217"/>
-      <c r="I5" s="217"/>
-      <c r="J5" s="218"/>
+      <c r="E5" s="255"/>
+      <c r="F5" s="256"/>
+      <c r="G5" s="256"/>
+      <c r="H5" s="256"/>
+      <c r="I5" s="256"/>
+      <c r="J5" s="257"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="181" t="s">
+      <c r="N5" s="190" t="s">
         <v>51</v>
       </c>
-      <c r="O5" s="182"/>
-      <c r="P5" s="183"/>
+      <c r="O5" s="233"/>
+      <c r="P5" s="191"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -3878,10 +3875,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="214" t="s">
+      <c r="U5" s="225" t="s">
         <v>73</v>
       </c>
-      <c r="V5" s="215"/>
+      <c r="V5" s="226"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -3894,10 +3891,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="214" t="s">
+      <c r="AA5" s="225" t="s">
         <v>73</v>
       </c>
-      <c r="AB5" s="215"/>
+      <c r="AB5" s="226"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -3929,12 +3926,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="223"/>
-      <c r="F6" s="220"/>
-      <c r="G6" s="220"/>
-      <c r="H6" s="220"/>
-      <c r="I6" s="220"/>
-      <c r="J6" s="221"/>
+      <c r="E6" s="246"/>
+      <c r="F6" s="241"/>
+      <c r="G6" s="241"/>
+      <c r="H6" s="241"/>
+      <c r="I6" s="241"/>
+      <c r="J6" s="242"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -3942,11 +3939,11 @@
         <v>154</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="184" t="s">
+      <c r="N6" s="216" t="s">
         <v>95</v>
       </c>
-      <c r="O6" s="185"/>
-      <c r="P6" s="186"/>
+      <c r="O6" s="217"/>
+      <c r="P6" s="218"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -3956,10 +3953,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="209" t="s">
+      <c r="U6" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V6" s="210"/>
+      <c r="V6" s="213"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -3972,10 +3969,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="209" t="s">
+      <c r="AA6" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB6" s="210"/>
+      <c r="AB6" s="213"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -4003,7 +4000,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D7" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4018,9 +4015,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="219"/>
-      <c r="I7" s="220"/>
-      <c r="J7" s="221"/>
+      <c r="H7" s="240"/>
+      <c r="I7" s="241"/>
+      <c r="J7" s="242"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -4028,11 +4025,11 @@
       <c r="M7" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N7" s="184" t="s">
+      <c r="N7" s="216" t="s">
         <v>52</v>
       </c>
-      <c r="O7" s="185"/>
-      <c r="P7" s="186"/>
+      <c r="O7" s="217"/>
+      <c r="P7" s="218"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -4042,10 +4039,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="209" t="s">
+      <c r="U7" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V7" s="210"/>
+      <c r="V7" s="213"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -4058,10 +4055,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="209" t="s">
+      <c r="AA7" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB7" s="210"/>
+      <c r="AB7" s="213"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -4089,7 +4086,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D8" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4104,9 +4101,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="219"/>
-      <c r="I8" s="220"/>
-      <c r="J8" s="221"/>
+      <c r="H8" s="240"/>
+      <c r="I8" s="241"/>
+      <c r="J8" s="242"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -4114,11 +4111,11 @@
       <c r="M8" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N8" s="184" t="s">
+      <c r="N8" s="216" t="s">
         <v>53</v>
       </c>
-      <c r="O8" s="185"/>
-      <c r="P8" s="186"/>
+      <c r="O8" s="217"/>
+      <c r="P8" s="218"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -4128,10 +4125,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="209" t="s">
+      <c r="U8" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V8" s="210"/>
+      <c r="V8" s="213"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -4144,10 +4141,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="209" t="s">
+      <c r="AA8" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB8" s="210"/>
+      <c r="AB8" s="213"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -4175,7 +4172,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D9" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4190,9 +4187,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="219"/>
-      <c r="I9" s="220"/>
-      <c r="J9" s="221"/>
+      <c r="H9" s="240"/>
+      <c r="I9" s="241"/>
+      <c r="J9" s="242"/>
       <c r="K9" s="37" t="s">
         <v>47</v>
       </c>
@@ -4200,11 +4197,11 @@
       <c r="M9" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N9" s="184" t="s">
+      <c r="N9" s="216" t="s">
         <v>54</v>
       </c>
-      <c r="O9" s="185"/>
-      <c r="P9" s="186"/>
+      <c r="O9" s="217"/>
+      <c r="P9" s="218"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -4214,10 +4211,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="209" t="s">
+      <c r="U9" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V9" s="210"/>
+      <c r="V9" s="213"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -4230,10 +4227,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="209" t="s">
+      <c r="AA9" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB9" s="210"/>
+      <c r="AB9" s="213"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -4261,7 +4258,7 @@
         <v>5</v>
       </c>
       <c r="C10" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D10" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4276,9 +4273,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="219"/>
-      <c r="I10" s="220"/>
-      <c r="J10" s="221"/>
+      <c r="H10" s="240"/>
+      <c r="I10" s="241"/>
+      <c r="J10" s="242"/>
       <c r="K10" s="37" t="s">
         <v>48</v>
       </c>
@@ -4286,11 +4283,11 @@
       <c r="M10" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N10" s="184" t="s">
+      <c r="N10" s="216" t="s">
         <v>55</v>
       </c>
-      <c r="O10" s="185"/>
-      <c r="P10" s="186"/>
+      <c r="O10" s="217"/>
+      <c r="P10" s="218"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -4300,10 +4297,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="209" t="s">
+      <c r="U10" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V10" s="210"/>
+      <c r="V10" s="213"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -4316,10 +4313,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="209" t="s">
+      <c r="AA10" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB10" s="210"/>
+      <c r="AB10" s="213"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -4347,7 +4344,7 @@
         <v>6</v>
       </c>
       <c r="C11" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D11" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4362,9 +4359,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="219"/>
-      <c r="I11" s="220"/>
-      <c r="J11" s="221"/>
+      <c r="H11" s="240"/>
+      <c r="I11" s="241"/>
+      <c r="J11" s="242"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -4372,11 +4369,11 @@
       <c r="M11" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N11" s="184" t="s">
+      <c r="N11" s="216" t="s">
         <v>56</v>
       </c>
-      <c r="O11" s="185"/>
-      <c r="P11" s="186"/>
+      <c r="O11" s="217"/>
+      <c r="P11" s="218"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -4386,10 +4383,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="209" t="s">
+      <c r="U11" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V11" s="210"/>
+      <c r="V11" s="213"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -4402,10 +4399,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="209" t="s">
+      <c r="AA11" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB11" s="210"/>
+      <c r="AB11" s="213"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -4433,7 +4430,7 @@
         <v>7</v>
       </c>
       <c r="C12" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D12" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4448,9 +4445,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="219"/>
-      <c r="I12" s="220"/>
-      <c r="J12" s="221"/>
+      <c r="H12" s="240"/>
+      <c r="I12" s="241"/>
+      <c r="J12" s="242"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -4458,11 +4455,11 @@
       <c r="M12" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N12" s="184" t="s">
+      <c r="N12" s="216" t="s">
         <v>57</v>
       </c>
-      <c r="O12" s="185"/>
-      <c r="P12" s="186"/>
+      <c r="O12" s="217"/>
+      <c r="P12" s="218"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -4472,10 +4469,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="209" t="s">
+      <c r="U12" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V12" s="210"/>
+      <c r="V12" s="213"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -4488,10 +4485,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="209" t="s">
+      <c r="AA12" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB12" s="210"/>
+      <c r="AB12" s="213"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -4519,7 +4516,7 @@
         <v>8</v>
       </c>
       <c r="C13" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D13" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4534,9 +4531,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="219"/>
-      <c r="I13" s="220"/>
-      <c r="J13" s="221"/>
+      <c r="H13" s="240"/>
+      <c r="I13" s="241"/>
+      <c r="J13" s="242"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -4544,11 +4541,11 @@
       <c r="M13" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N13" s="184" t="s">
+      <c r="N13" s="216" t="s">
         <v>58</v>
       </c>
-      <c r="O13" s="185"/>
-      <c r="P13" s="186"/>
+      <c r="O13" s="217"/>
+      <c r="P13" s="218"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -4558,10 +4555,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="209" t="s">
+      <c r="U13" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V13" s="210"/>
+      <c r="V13" s="213"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -4574,10 +4571,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="209" t="s">
+      <c r="AA13" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB13" s="210"/>
+      <c r="AB13" s="213"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -4605,7 +4602,7 @@
         <v>9</v>
       </c>
       <c r="C14" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D14" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4620,9 +4617,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="219"/>
-      <c r="I14" s="220"/>
-      <c r="J14" s="221"/>
+      <c r="H14" s="240"/>
+      <c r="I14" s="241"/>
+      <c r="J14" s="242"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -4630,11 +4627,11 @@
       <c r="M14" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N14" s="184" t="s">
+      <c r="N14" s="216" t="s">
         <v>59</v>
       </c>
-      <c r="O14" s="185"/>
-      <c r="P14" s="186"/>
+      <c r="O14" s="217"/>
+      <c r="P14" s="218"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -4644,10 +4641,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="209" t="s">
+      <c r="U14" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V14" s="210"/>
+      <c r="V14" s="213"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -4660,10 +4657,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="209" t="s">
+      <c r="AA14" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB14" s="210"/>
+      <c r="AB14" s="213"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -4691,7 +4688,7 @@
         <v>10</v>
       </c>
       <c r="C15" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D15" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4706,9 +4703,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="219"/>
-      <c r="I15" s="220"/>
-      <c r="J15" s="221"/>
+      <c r="H15" s="240"/>
+      <c r="I15" s="241"/>
+      <c r="J15" s="242"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -4716,11 +4713,11 @@
       <c r="M15" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N15" s="184" t="s">
+      <c r="N15" s="216" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="185"/>
-      <c r="P15" s="186"/>
+      <c r="O15" s="217"/>
+      <c r="P15" s="218"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -4730,10 +4727,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="209" t="s">
+      <c r="U15" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V15" s="210"/>
+      <c r="V15" s="213"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -4746,10 +4743,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="209" t="s">
+      <c r="AA15" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB15" s="210"/>
+      <c r="AB15" s="213"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -4777,7 +4774,7 @@
         <v>11</v>
       </c>
       <c r="C16" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D16" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4786,21 +4783,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="219"/>
-      <c r="G16" s="220"/>
-      <c r="H16" s="220"/>
-      <c r="I16" s="220"/>
-      <c r="J16" s="221"/>
+      <c r="F16" s="240"/>
+      <c r="G16" s="241"/>
+      <c r="H16" s="241"/>
+      <c r="I16" s="241"/>
+      <c r="J16" s="242"/>
       <c r="K16" s="40" t="s">
         <v>49</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="184" t="s">
+      <c r="N16" s="216" t="s">
         <v>50</v>
       </c>
-      <c r="O16" s="185"/>
-      <c r="P16" s="186"/>
+      <c r="O16" s="217"/>
+      <c r="P16" s="218"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -4810,10 +4807,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="209" t="s">
+      <c r="U16" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V16" s="210"/>
+      <c r="V16" s="213"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -4826,10 +4823,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="209" t="s">
+      <c r="AA16" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB16" s="210"/>
+      <c r="AB16" s="213"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -4857,7 +4854,7 @@
         <v>12</v>
       </c>
       <c r="C17" s="177" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D17" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4867,22 +4864,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="222" t="s">
+      <c r="G17" s="247" t="s">
         <v>76</v>
       </c>
-      <c r="H17" s="185"/>
-      <c r="I17" s="185"/>
-      <c r="J17" s="186"/>
+      <c r="H17" s="217"/>
+      <c r="I17" s="217"/>
+      <c r="J17" s="218"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="184" t="s">
+      <c r="N17" s="216" t="s">
         <v>64</v>
       </c>
-      <c r="O17" s="185"/>
-      <c r="P17" s="186"/>
+      <c r="O17" s="217"/>
+      <c r="P17" s="218"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -4892,10 +4889,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="209" t="s">
+      <c r="U17" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V17" s="210"/>
+      <c r="V17" s="213"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -4908,10 +4905,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="209" t="s">
+      <c r="AA17" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB17" s="210"/>
+      <c r="AB17" s="213"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -4939,7 +4936,7 @@
         <v>13</v>
       </c>
       <c r="C18" s="177" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D18" s="23" t="str">
         <f t="shared" si="0"/>
@@ -4949,12 +4946,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="222" t="s">
+      <c r="G18" s="247" t="s">
         <v>76</v>
       </c>
-      <c r="H18" s="185"/>
-      <c r="I18" s="185"/>
-      <c r="J18" s="186"/>
+      <c r="H18" s="217"/>
+      <c r="I18" s="217"/>
+      <c r="J18" s="218"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -4962,11 +4959,11 @@
       <c r="M18" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N18" s="184" t="s">
+      <c r="N18" s="216" t="s">
         <v>61</v>
       </c>
-      <c r="O18" s="185"/>
-      <c r="P18" s="186"/>
+      <c r="O18" s="217"/>
+      <c r="P18" s="218"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -4976,10 +4973,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="209" t="s">
+      <c r="U18" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V18" s="210"/>
+      <c r="V18" s="213"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -4992,10 +4989,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="209" t="s">
+      <c r="AA18" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB18" s="210"/>
+      <c r="AB18" s="213"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -5031,20 +5028,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="219"/>
-      <c r="H19" s="220"/>
-      <c r="I19" s="220"/>
-      <c r="J19" s="221"/>
+      <c r="G19" s="240"/>
+      <c r="H19" s="241"/>
+      <c r="I19" s="241"/>
+      <c r="J19" s="242"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="184" t="s">
+      <c r="N19" s="216" t="s">
         <v>93</v>
       </c>
-      <c r="O19" s="185"/>
-      <c r="P19" s="186"/>
+      <c r="O19" s="217"/>
+      <c r="P19" s="218"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -5054,10 +5051,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="209" t="s">
+      <c r="U19" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V19" s="210"/>
+      <c r="V19" s="213"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -5070,10 +5067,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="209" t="s">
+      <c r="AA19" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB19" s="210"/>
+      <c r="AB19" s="213"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -5111,20 +5108,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="219"/>
-      <c r="H20" s="220"/>
-      <c r="I20" s="220"/>
-      <c r="J20" s="221"/>
+      <c r="G20" s="240"/>
+      <c r="H20" s="241"/>
+      <c r="I20" s="241"/>
+      <c r="J20" s="242"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="184" t="s">
+      <c r="N20" s="216" t="s">
         <v>94</v>
       </c>
-      <c r="O20" s="185"/>
-      <c r="P20" s="186"/>
+      <c r="O20" s="217"/>
+      <c r="P20" s="218"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -5134,10 +5131,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="209" t="s">
+      <c r="U20" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V20" s="210"/>
+      <c r="V20" s="213"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -5150,10 +5147,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="209" t="s">
+      <c r="AA20" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB20" s="210"/>
+      <c r="AB20" s="213"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -5181,7 +5178,7 @@
         <v>16</v>
       </c>
       <c r="C21" s="38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D21" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5191,20 +5188,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="219"/>
-      <c r="H21" s="220"/>
-      <c r="I21" s="220"/>
-      <c r="J21" s="221"/>
+      <c r="G21" s="240"/>
+      <c r="H21" s="241"/>
+      <c r="I21" s="241"/>
+      <c r="J21" s="242"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="184" t="s">
+      <c r="N21" s="216" t="s">
         <v>62</v>
       </c>
-      <c r="O21" s="185"/>
-      <c r="P21" s="186"/>
+      <c r="O21" s="217"/>
+      <c r="P21" s="218"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -5214,10 +5211,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="209" t="s">
+      <c r="U21" s="212" t="s">
         <v>96</v>
       </c>
-      <c r="V21" s="210"/>
+      <c r="V21" s="213"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -5230,10 +5227,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="209" t="s">
+      <c r="AA21" s="212" t="s">
         <v>98</v>
       </c>
-      <c r="AB21" s="210"/>
+      <c r="AB21" s="213"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -5261,28 +5258,28 @@
         <v>17</v>
       </c>
       <c r="C22" s="38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D22" s="23" t="str">
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="223"/>
-      <c r="F22" s="220"/>
-      <c r="G22" s="220"/>
-      <c r="H22" s="220"/>
-      <c r="I22" s="220"/>
-      <c r="J22" s="221"/>
+      <c r="E22" s="246"/>
+      <c r="F22" s="241"/>
+      <c r="G22" s="241"/>
+      <c r="H22" s="241"/>
+      <c r="I22" s="241"/>
+      <c r="J22" s="242"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="184" t="s">
+      <c r="N22" s="216" t="s">
         <v>63</v>
       </c>
-      <c r="O22" s="185"/>
-      <c r="P22" s="186"/>
+      <c r="O22" s="217"/>
+      <c r="P22" s="218"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -5292,10 +5289,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="209" t="s">
+      <c r="U22" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V22" s="210"/>
+      <c r="V22" s="213"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -5308,10 +5305,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="209" t="s">
+      <c r="AA22" s="212" t="s">
         <v>96</v>
       </c>
-      <c r="AB22" s="210"/>
+      <c r="AB22" s="213"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -5339,7 +5336,7 @@
         <v>18</v>
       </c>
       <c r="C23" s="38" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D23" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5351,22 +5348,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="222" t="s">
+      <c r="G23" s="247" t="s">
         <v>77</v>
       </c>
-      <c r="H23" s="185"/>
-      <c r="I23" s="185"/>
-      <c r="J23" s="186"/>
+      <c r="H23" s="217"/>
+      <c r="I23" s="217"/>
+      <c r="J23" s="218"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="184" t="s">
+      <c r="N23" s="216" t="s">
         <v>82</v>
       </c>
-      <c r="O23" s="185"/>
-      <c r="P23" s="186"/>
+      <c r="O23" s="217"/>
+      <c r="P23" s="218"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -5376,10 +5373,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="209" t="s">
+      <c r="U23" s="212" t="s">
         <v>97</v>
       </c>
-      <c r="V23" s="210"/>
+      <c r="V23" s="213"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -5392,10 +5389,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="209" t="s">
+      <c r="AA23" s="212" t="s">
         <v>96</v>
       </c>
-      <c r="AB23" s="210"/>
+      <c r="AB23" s="213"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -5423,7 +5420,7 @@
         <v>19</v>
       </c>
       <c r="C24" s="38" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D24" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5435,22 +5432,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="222" t="s">
+      <c r="G24" s="247" t="s">
         <v>77</v>
       </c>
-      <c r="H24" s="185"/>
-      <c r="I24" s="185"/>
-      <c r="J24" s="186"/>
+      <c r="H24" s="217"/>
+      <c r="I24" s="217"/>
+      <c r="J24" s="218"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="184" t="s">
+      <c r="N24" s="216" t="s">
         <v>81</v>
       </c>
-      <c r="O24" s="185"/>
-      <c r="P24" s="186"/>
+      <c r="O24" s="217"/>
+      <c r="P24" s="218"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -5460,10 +5457,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="209" t="s">
+      <c r="U24" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V24" s="210"/>
+      <c r="V24" s="213"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -5476,10 +5473,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="209" t="s">
+      <c r="AA24" s="212" t="s">
         <v>98</v>
       </c>
-      <c r="AB24" s="210"/>
+      <c r="AB24" s="213"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -5517,10 +5514,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="219"/>
-      <c r="H25" s="220"/>
-      <c r="I25" s="220"/>
-      <c r="J25" s="221"/>
+      <c r="G25" s="240"/>
+      <c r="H25" s="241"/>
+      <c r="I25" s="241"/>
+      <c r="J25" s="242"/>
       <c r="K25" s="49" t="s">
         <v>39</v>
       </c>
@@ -5528,11 +5525,11 @@
         <v>154</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="184" t="s">
+      <c r="N25" s="216" t="s">
         <v>41</v>
       </c>
-      <c r="O25" s="185"/>
-      <c r="P25" s="186"/>
+      <c r="O25" s="217"/>
+      <c r="P25" s="218"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -5542,10 +5539,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="209" t="s">
+      <c r="U25" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V25" s="210"/>
+      <c r="V25" s="213"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -5558,10 +5555,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="209" t="s">
+      <c r="AA25" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB25" s="210"/>
+      <c r="AB25" s="213"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -5599,10 +5596,10 @@
       <c r="F26" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="G26" s="219"/>
-      <c r="H26" s="220"/>
-      <c r="I26" s="220"/>
-      <c r="J26" s="221"/>
+      <c r="G26" s="240"/>
+      <c r="H26" s="241"/>
+      <c r="I26" s="241"/>
+      <c r="J26" s="242"/>
       <c r="K26" s="31" t="s">
         <v>40</v>
       </c>
@@ -5610,11 +5607,11 @@
         <v>154</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="184" t="s">
+      <c r="N26" s="216" t="s">
         <v>42</v>
       </c>
-      <c r="O26" s="185"/>
-      <c r="P26" s="186"/>
+      <c r="O26" s="217"/>
+      <c r="P26" s="218"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -5624,10 +5621,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="209" t="s">
+      <c r="U26" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V26" s="210"/>
+      <c r="V26" s="213"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -5640,10 +5637,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="209" t="s">
+      <c r="AA26" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB26" s="210"/>
+      <c r="AB26" s="213"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -5675,22 +5672,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="223"/>
-      <c r="F27" s="220"/>
-      <c r="G27" s="220"/>
-      <c r="H27" s="220"/>
-      <c r="I27" s="220"/>
-      <c r="J27" s="221"/>
+      <c r="E27" s="246"/>
+      <c r="F27" s="241"/>
+      <c r="G27" s="241"/>
+      <c r="H27" s="241"/>
+      <c r="I27" s="241"/>
+      <c r="J27" s="242"/>
       <c r="K27" s="25" t="s">
         <v>44</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="184" t="s">
+      <c r="N27" s="216" t="s">
         <v>46</v>
       </c>
-      <c r="O27" s="185"/>
-      <c r="P27" s="186"/>
+      <c r="O27" s="217"/>
+      <c r="P27" s="218"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -5700,10 +5697,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="209" t="s">
+      <c r="U27" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="V27" s="210"/>
+      <c r="V27" s="213"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -5716,10 +5713,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="209" t="s">
+      <c r="AA27" s="212" t="s">
         <v>73</v>
       </c>
-      <c r="AB27" s="210"/>
+      <c r="AB27" s="213"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -5751,12 +5748,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="227"/>
-      <c r="F28" s="228"/>
-      <c r="G28" s="228"/>
-      <c r="H28" s="228"/>
-      <c r="I28" s="228"/>
-      <c r="J28" s="229"/>
+      <c r="E28" s="243"/>
+      <c r="F28" s="244"/>
+      <c r="G28" s="244"/>
+      <c r="H28" s="244"/>
+      <c r="I28" s="244"/>
+      <c r="J28" s="245"/>
       <c r="K28" s="52" t="s">
         <v>45</v>
       </c>
@@ -5764,11 +5761,11 @@
         <v>154</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="197" t="s">
+      <c r="N28" s="237" t="s">
         <v>92</v>
       </c>
-      <c r="O28" s="198"/>
-      <c r="P28" s="199"/>
+      <c r="O28" s="238"/>
+      <c r="P28" s="239"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -5778,10 +5775,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="259" t="s">
+      <c r="U28" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="V28" s="260"/>
+      <c r="V28" s="215"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -5794,10 +5791,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="259" t="s">
+      <c r="AA28" s="214" t="s">
         <v>73</v>
       </c>
-      <c r="AB28" s="260"/>
+      <c r="AB28" s="215"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -5874,18 +5871,18 @@
       <c r="S30" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="T30" s="179" t="s">
+      <c r="T30" s="259" t="s">
         <v>156</v>
       </c>
-      <c r="U30" s="179"/>
-      <c r="V30" s="179"/>
-      <c r="W30" s="179"/>
-      <c r="X30" s="179"/>
-      <c r="Y30" s="179"/>
-      <c r="Z30" s="179"/>
-      <c r="AA30" s="179"/>
-      <c r="AB30" s="179"/>
-      <c r="AC30" s="180"/>
+      <c r="U30" s="259"/>
+      <c r="V30" s="259"/>
+      <c r="W30" s="259"/>
+      <c r="X30" s="259"/>
+      <c r="Y30" s="259"/>
+      <c r="Z30" s="259"/>
+      <c r="AA30" s="259"/>
+      <c r="AB30" s="259"/>
+      <c r="AC30" s="227"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B31" s="67" t="s">
@@ -5911,9 +5908,7 @@
       <c r="K31" s="79"/>
       <c r="L31" s="79"/>
       <c r="M31" s="79"/>
-      <c r="N31" s="79" t="s">
-        <v>178</v>
-      </c>
+      <c r="N31" s="79"/>
       <c r="O31" s="79" t="s">
         <v>177</v>
       </c>
@@ -5926,18 +5921,18 @@
       <c r="S31" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="T31" s="181" t="s">
+      <c r="T31" s="190" t="s">
         <v>161</v>
       </c>
-      <c r="U31" s="182"/>
-      <c r="V31" s="182"/>
-      <c r="W31" s="182"/>
-      <c r="X31" s="182"/>
-      <c r="Y31" s="182"/>
-      <c r="Z31" s="182"/>
-      <c r="AA31" s="182"/>
-      <c r="AB31" s="182"/>
-      <c r="AC31" s="183"/>
+      <c r="U31" s="233"/>
+      <c r="V31" s="233"/>
+      <c r="W31" s="233"/>
+      <c r="X31" s="233"/>
+      <c r="Y31" s="233"/>
+      <c r="Z31" s="233"/>
+      <c r="AA31" s="233"/>
+      <c r="AB31" s="233"/>
+      <c r="AC31" s="191"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B32" s="4" t="s">
@@ -5961,22 +5956,22 @@
       <c r="S32" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="T32" s="184" t="s">
+      <c r="T32" s="216" t="s">
         <v>162</v>
       </c>
-      <c r="U32" s="185"/>
-      <c r="V32" s="185"/>
-      <c r="W32" s="185"/>
-      <c r="X32" s="185"/>
-      <c r="Y32" s="185"/>
-      <c r="Z32" s="185"/>
-      <c r="AA32" s="185"/>
-      <c r="AB32" s="185"/>
-      <c r="AC32" s="186"/>
+      <c r="U32" s="217"/>
+      <c r="V32" s="217"/>
+      <c r="W32" s="217"/>
+      <c r="X32" s="217"/>
+      <c r="Y32" s="217"/>
+      <c r="Z32" s="217"/>
+      <c r="AA32" s="217"/>
+      <c r="AB32" s="217"/>
+      <c r="AC32" s="218"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
       <c r="H33" s="84" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I33" s="73">
         <v>7</v>
@@ -6008,31 +6003,31 @@
       <c r="S33" s="37" t="s">
         <v>158</v>
       </c>
-      <c r="T33" s="184" t="s">
+      <c r="T33" s="216" t="s">
         <v>163</v>
       </c>
-      <c r="U33" s="185"/>
-      <c r="V33" s="185"/>
-      <c r="W33" s="185"/>
-      <c r="X33" s="185"/>
-      <c r="Y33" s="185"/>
-      <c r="Z33" s="185"/>
-      <c r="AA33" s="185"/>
-      <c r="AB33" s="185"/>
-      <c r="AC33" s="186"/>
+      <c r="U33" s="217"/>
+      <c r="V33" s="217"/>
+      <c r="W33" s="217"/>
+      <c r="X33" s="217"/>
+      <c r="Y33" s="217"/>
+      <c r="Z33" s="217"/>
+      <c r="AA33" s="217"/>
+      <c r="AB33" s="217"/>
+      <c r="AC33" s="218"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B34" s="256" t="s">
+      <c r="B34" s="207" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="230" t="s">
+      <c r="C34" s="205" t="s">
         <v>114</v>
       </c>
-      <c r="D34" s="232"/>
-      <c r="E34" s="230" t="s">
+      <c r="D34" s="206"/>
+      <c r="E34" s="205" t="s">
         <v>115</v>
       </c>
-      <c r="F34" s="232"/>
+      <c r="F34" s="206"/>
       <c r="H34" s="77" t="s">
         <v>65</v>
       </c>
@@ -6041,16 +6036,16 @@
       <c r="K34" s="79"/>
       <c r="L34" s="79"/>
       <c r="M34" s="79" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="N34" s="79" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O34" s="79" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="P34" s="80" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="R34" s="2">
         <v>3</v>
@@ -6058,21 +6053,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="184" t="s">
+      <c r="T34" s="216" t="s">
         <v>164</v>
       </c>
-      <c r="U34" s="185"/>
-      <c r="V34" s="185"/>
-      <c r="W34" s="185"/>
-      <c r="X34" s="185"/>
-      <c r="Y34" s="185"/>
-      <c r="Z34" s="185"/>
-      <c r="AA34" s="185"/>
-      <c r="AB34" s="185"/>
-      <c r="AC34" s="186"/>
+      <c r="U34" s="217"/>
+      <c r="V34" s="217"/>
+      <c r="W34" s="217"/>
+      <c r="X34" s="217"/>
+      <c r="Y34" s="217"/>
+      <c r="Z34" s="217"/>
+      <c r="AA34" s="217"/>
+      <c r="AB34" s="217"/>
+      <c r="AC34" s="218"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B35" s="257"/>
+      <c r="B35" s="208"/>
       <c r="C35" s="64" t="s">
         <v>99</v>
       </c>
@@ -6091,18 +6086,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="184" t="s">
+      <c r="T35" s="216" t="s">
         <v>165</v>
       </c>
-      <c r="U35" s="185"/>
-      <c r="V35" s="185"/>
-      <c r="W35" s="185"/>
-      <c r="X35" s="185"/>
-      <c r="Y35" s="185"/>
-      <c r="Z35" s="185"/>
-      <c r="AA35" s="185"/>
-      <c r="AB35" s="185"/>
-      <c r="AC35" s="186"/>
+      <c r="U35" s="217"/>
+      <c r="V35" s="217"/>
+      <c r="W35" s="217"/>
+      <c r="X35" s="217"/>
+      <c r="Y35" s="217"/>
+      <c r="Z35" s="217"/>
+      <c r="AA35" s="217"/>
+      <c r="AB35" s="217"/>
+      <c r="AC35" s="218"/>
     </row>
     <row r="36" spans="2:29" ht="36" customHeight="1" thickBot="1">
       <c r="B36" s="1">
@@ -6121,7 +6116,7 @@
         <v>141</v>
       </c>
       <c r="H36" s="84" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="I36" s="73">
         <v>7</v>
@@ -6153,18 +6148,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="184" t="s">
+      <c r="T36" s="216" t="s">
         <v>166</v>
       </c>
-      <c r="U36" s="185"/>
-      <c r="V36" s="185"/>
-      <c r="W36" s="185"/>
-      <c r="X36" s="185"/>
-      <c r="Y36" s="185"/>
-      <c r="Z36" s="185"/>
-      <c r="AA36" s="185"/>
-      <c r="AB36" s="185"/>
-      <c r="AC36" s="186"/>
+      <c r="U36" s="217"/>
+      <c r="V36" s="217"/>
+      <c r="W36" s="217"/>
+      <c r="X36" s="217"/>
+      <c r="Y36" s="217"/>
+      <c r="Z36" s="217"/>
+      <c r="AA36" s="217"/>
+      <c r="AB36" s="217"/>
+      <c r="AC36" s="218"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1" thickBot="1">
       <c r="B37" s="2">
@@ -6190,16 +6185,16 @@
       <c r="K37" s="79"/>
       <c r="L37" s="79"/>
       <c r="M37" s="178" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="N37" s="79" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="O37" s="79" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="P37" s="80" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="R37" s="2">
         <v>6</v>
@@ -6207,18 +6202,18 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="184" t="s">
-        <v>193</v>
-      </c>
-      <c r="U37" s="185"/>
-      <c r="V37" s="185"/>
-      <c r="W37" s="185"/>
-      <c r="X37" s="185"/>
-      <c r="Y37" s="185"/>
-      <c r="Z37" s="185"/>
-      <c r="AA37" s="185"/>
-      <c r="AB37" s="185"/>
-      <c r="AC37" s="186"/>
+      <c r="T37" s="216" t="s">
+        <v>192</v>
+      </c>
+      <c r="U37" s="217"/>
+      <c r="V37" s="217"/>
+      <c r="W37" s="217"/>
+      <c r="X37" s="217"/>
+      <c r="Y37" s="217"/>
+      <c r="Z37" s="217"/>
+      <c r="AA37" s="217"/>
+      <c r="AB37" s="217"/>
+      <c r="AC37" s="218"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1">
       <c r="B38" s="2">
@@ -6239,21 +6234,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="189" t="s">
+      <c r="S38" s="260" t="s">
         <v>72</v>
       </c>
-      <c r="T38" s="191" t="s">
+      <c r="T38" s="262" t="s">
         <v>167</v>
       </c>
-      <c r="U38" s="192"/>
-      <c r="V38" s="192"/>
-      <c r="W38" s="192"/>
-      <c r="X38" s="192"/>
-      <c r="Y38" s="192"/>
-      <c r="Z38" s="192"/>
-      <c r="AA38" s="192"/>
-      <c r="AB38" s="192"/>
-      <c r="AC38" s="193"/>
+      <c r="U38" s="263"/>
+      <c r="V38" s="263"/>
+      <c r="W38" s="263"/>
+      <c r="X38" s="263"/>
+      <c r="Y38" s="263"/>
+      <c r="Z38" s="263"/>
+      <c r="AA38" s="263"/>
+      <c r="AB38" s="263"/>
+      <c r="AC38" s="264"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1">
       <c r="B39" s="2">
@@ -6271,26 +6266,26 @@
       <c r="F39" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G39" s="200" t="s">
-        <v>180</v>
-      </c>
-      <c r="H39" s="201"/>
-      <c r="I39" s="201"/>
-      <c r="J39" s="202"/>
+      <c r="G39" s="192" t="s">
+        <v>179</v>
+      </c>
+      <c r="H39" s="193"/>
+      <c r="I39" s="193"/>
+      <c r="J39" s="194"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="190"/>
-      <c r="T39" s="194"/>
-      <c r="U39" s="195"/>
-      <c r="V39" s="195"/>
-      <c r="W39" s="195"/>
-      <c r="X39" s="195"/>
-      <c r="Y39" s="195"/>
-      <c r="Z39" s="195"/>
-      <c r="AA39" s="195"/>
-      <c r="AB39" s="195"/>
-      <c r="AC39" s="196"/>
+      <c r="S39" s="261"/>
+      <c r="T39" s="265"/>
+      <c r="U39" s="266"/>
+      <c r="V39" s="266"/>
+      <c r="W39" s="266"/>
+      <c r="X39" s="266"/>
+      <c r="Y39" s="266"/>
+      <c r="Z39" s="266"/>
+      <c r="AA39" s="266"/>
+      <c r="AB39" s="266"/>
+      <c r="AC39" s="267"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1">
       <c r="B40" s="2">
@@ -6308,28 +6303,28 @@
       <c r="F40" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G40" s="206"/>
-      <c r="H40" s="207"/>
-      <c r="I40" s="207"/>
-      <c r="J40" s="208"/>
+      <c r="G40" s="195"/>
+      <c r="H40" s="196"/>
+      <c r="I40" s="196"/>
+      <c r="J40" s="197"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="184" t="s">
+      <c r="T40" s="216" t="s">
         <v>168</v>
       </c>
-      <c r="U40" s="185"/>
-      <c r="V40" s="185"/>
-      <c r="W40" s="185"/>
-      <c r="X40" s="185"/>
-      <c r="Y40" s="185"/>
-      <c r="Z40" s="185"/>
-      <c r="AA40" s="185"/>
-      <c r="AB40" s="185"/>
-      <c r="AC40" s="186"/>
+      <c r="U40" s="217"/>
+      <c r="V40" s="217"/>
+      <c r="W40" s="217"/>
+      <c r="X40" s="217"/>
+      <c r="Y40" s="217"/>
+      <c r="Z40" s="217"/>
+      <c r="AA40" s="217"/>
+      <c r="AB40" s="217"/>
+      <c r="AC40" s="218"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1">
       <c r="B41" s="2">
@@ -6347,28 +6342,28 @@
       <c r="F41" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G41" s="206"/>
-      <c r="H41" s="207"/>
-      <c r="I41" s="207"/>
-      <c r="J41" s="208"/>
+      <c r="G41" s="195"/>
+      <c r="H41" s="196"/>
+      <c r="I41" s="196"/>
+      <c r="J41" s="197"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="184" t="s">
+      <c r="T41" s="216" t="s">
         <v>169</v>
       </c>
-      <c r="U41" s="185"/>
-      <c r="V41" s="185"/>
-      <c r="W41" s="185"/>
-      <c r="X41" s="185"/>
-      <c r="Y41" s="185"/>
-      <c r="Z41" s="185"/>
-      <c r="AA41" s="185"/>
-      <c r="AB41" s="185"/>
-      <c r="AC41" s="186"/>
+      <c r="U41" s="217"/>
+      <c r="V41" s="217"/>
+      <c r="W41" s="217"/>
+      <c r="X41" s="217"/>
+      <c r="Y41" s="217"/>
+      <c r="Z41" s="217"/>
+      <c r="AA41" s="217"/>
+      <c r="AB41" s="217"/>
+      <c r="AC41" s="218"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
       <c r="B42" s="2">
@@ -6386,28 +6381,28 @@
       <c r="F42" s="76" t="s">
         <v>174</v>
       </c>
-      <c r="G42" s="203"/>
-      <c r="H42" s="204"/>
-      <c r="I42" s="204"/>
-      <c r="J42" s="205"/>
+      <c r="G42" s="198"/>
+      <c r="H42" s="199"/>
+      <c r="I42" s="199"/>
+      <c r="J42" s="200"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="T42" s="184" t="s">
+      <c r="T42" s="216" t="s">
         <v>170</v>
       </c>
-      <c r="U42" s="185"/>
-      <c r="V42" s="185"/>
-      <c r="W42" s="185"/>
-      <c r="X42" s="185"/>
-      <c r="Y42" s="185"/>
-      <c r="Z42" s="185"/>
-      <c r="AA42" s="185"/>
-      <c r="AB42" s="185"/>
-      <c r="AC42" s="186"/>
+      <c r="U42" s="217"/>
+      <c r="V42" s="217"/>
+      <c r="W42" s="217"/>
+      <c r="X42" s="217"/>
+      <c r="Y42" s="217"/>
+      <c r="Z42" s="217"/>
+      <c r="AA42" s="217"/>
+      <c r="AB42" s="217"/>
+      <c r="AC42" s="218"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
       <c r="B43" s="2">
@@ -6425,30 +6420,30 @@
       <c r="F43" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G43" s="263" t="s">
-        <v>190</v>
-      </c>
-      <c r="H43" s="187"/>
-      <c r="I43" s="187"/>
-      <c r="J43" s="188"/>
+      <c r="G43" s="183" t="s">
+        <v>189</v>
+      </c>
+      <c r="H43" s="184"/>
+      <c r="I43" s="184"/>
+      <c r="J43" s="185"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T43" s="184" t="s">
+      <c r="T43" s="216" t="s">
         <v>171</v>
       </c>
-      <c r="U43" s="185"/>
-      <c r="V43" s="185"/>
-      <c r="W43" s="185"/>
-      <c r="X43" s="185"/>
-      <c r="Y43" s="185"/>
-      <c r="Z43" s="185"/>
-      <c r="AA43" s="185"/>
-      <c r="AB43" s="185"/>
-      <c r="AC43" s="186"/>
+      <c r="U43" s="217"/>
+      <c r="V43" s="217"/>
+      <c r="W43" s="217"/>
+      <c r="X43" s="217"/>
+      <c r="Y43" s="217"/>
+      <c r="Z43" s="217"/>
+      <c r="AA43" s="217"/>
+      <c r="AB43" s="217"/>
+      <c r="AC43" s="218"/>
     </row>
     <row r="44" spans="2:29" ht="45.75" thickBot="1">
       <c r="B44" s="2">
@@ -6458,32 +6453,32 @@
         <v>137</v>
       </c>
       <c r="D44" s="69" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E44" s="9" t="s">
         <v>124</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="189" t="s">
+      <c r="S44" s="260" t="s">
         <v>75</v>
       </c>
-      <c r="T44" s="191" t="s">
+      <c r="T44" s="262" t="s">
         <v>172</v>
       </c>
-      <c r="U44" s="192"/>
-      <c r="V44" s="192"/>
-      <c r="W44" s="192"/>
-      <c r="X44" s="192"/>
-      <c r="Y44" s="192"/>
-      <c r="Z44" s="192"/>
-      <c r="AA44" s="192"/>
-      <c r="AB44" s="192"/>
-      <c r="AC44" s="193"/>
+      <c r="U44" s="263"/>
+      <c r="V44" s="263"/>
+      <c r="W44" s="263"/>
+      <c r="X44" s="263"/>
+      <c r="Y44" s="263"/>
+      <c r="Z44" s="263"/>
+      <c r="AA44" s="263"/>
+      <c r="AB44" s="263"/>
+      <c r="AC44" s="264"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1">
       <c r="B45" s="2">
@@ -6501,26 +6496,26 @@
       <c r="F45" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="G45" s="200" t="s">
-        <v>179</v>
-      </c>
-      <c r="H45" s="201"/>
-      <c r="I45" s="201"/>
-      <c r="J45" s="202"/>
+      <c r="G45" s="192" t="s">
+        <v>178</v>
+      </c>
+      <c r="H45" s="193"/>
+      <c r="I45" s="193"/>
+      <c r="J45" s="194"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="190"/>
-      <c r="T45" s="194"/>
-      <c r="U45" s="195"/>
-      <c r="V45" s="195"/>
-      <c r="W45" s="195"/>
-      <c r="X45" s="195"/>
-      <c r="Y45" s="195"/>
-      <c r="Z45" s="195"/>
-      <c r="AA45" s="195"/>
-      <c r="AB45" s="195"/>
-      <c r="AC45" s="196"/>
+      <c r="S45" s="261"/>
+      <c r="T45" s="265"/>
+      <c r="U45" s="266"/>
+      <c r="V45" s="266"/>
+      <c r="W45" s="266"/>
+      <c r="X45" s="266"/>
+      <c r="Y45" s="266"/>
+      <c r="Z45" s="266"/>
+      <c r="AA45" s="266"/>
+      <c r="AB45" s="266"/>
+      <c r="AC45" s="267"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
       <c r="B46" s="2">
@@ -6538,28 +6533,28 @@
       <c r="F46" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="G46" s="203"/>
-      <c r="H46" s="204"/>
-      <c r="I46" s="204"/>
-      <c r="J46" s="205"/>
+      <c r="G46" s="198"/>
+      <c r="H46" s="199"/>
+      <c r="I46" s="199"/>
+      <c r="J46" s="200"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="T46" s="197" t="s">
+      <c r="T46" s="237" t="s">
         <v>173</v>
       </c>
-      <c r="U46" s="198"/>
-      <c r="V46" s="198"/>
-      <c r="W46" s="198"/>
-      <c r="X46" s="198"/>
-      <c r="Y46" s="198"/>
-      <c r="Z46" s="198"/>
-      <c r="AA46" s="198"/>
-      <c r="AB46" s="198"/>
-      <c r="AC46" s="199"/>
+      <c r="U46" s="238"/>
+      <c r="V46" s="238"/>
+      <c r="W46" s="238"/>
+      <c r="X46" s="238"/>
+      <c r="Y46" s="238"/>
+      <c r="Z46" s="238"/>
+      <c r="AA46" s="238"/>
+      <c r="AB46" s="238"/>
+      <c r="AC46" s="239"/>
     </row>
     <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
       <c r="B47" s="2">
@@ -6577,12 +6572,12 @@
       <c r="F47" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="G47" s="187" t="s">
+      <c r="G47" s="184" t="s">
         <v>150</v>
       </c>
-      <c r="H47" s="187"/>
-      <c r="I47" s="187"/>
-      <c r="J47" s="188"/>
+      <c r="H47" s="184"/>
+      <c r="I47" s="184"/>
+      <c r="J47" s="185"/>
     </row>
     <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
       <c r="B48" s="2">
@@ -6592,16 +6587,16 @@
         <v>137</v>
       </c>
       <c r="D48" s="69" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E48" s="9" t="s">
         <v>128</v>
       </c>
       <c r="F48" s="35" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AA48" s="106" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="49" spans="2:10" ht="35.25" customHeight="1">
@@ -6620,12 +6615,12 @@
       <c r="F49" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="G49" s="200" t="s">
+      <c r="G49" s="192" t="s">
         <v>153</v>
       </c>
-      <c r="H49" s="201"/>
-      <c r="I49" s="201"/>
-      <c r="J49" s="202"/>
+      <c r="H49" s="193"/>
+      <c r="I49" s="193"/>
+      <c r="J49" s="194"/>
     </row>
     <row r="50" spans="2:10" ht="30" customHeight="1">
       <c r="B50" s="2">
@@ -6643,10 +6638,10 @@
       <c r="F50" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="G50" s="206"/>
-      <c r="H50" s="207"/>
-      <c r="I50" s="207"/>
-      <c r="J50" s="208"/>
+      <c r="G50" s="195"/>
+      <c r="H50" s="196"/>
+      <c r="I50" s="196"/>
+      <c r="J50" s="197"/>
     </row>
     <row r="51" spans="2:10" ht="32.25" customHeight="1" thickBot="1">
       <c r="B51" s="4">
@@ -6664,38 +6659,38 @@
       <c r="F51" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="G51" s="203"/>
-      <c r="H51" s="204"/>
-      <c r="I51" s="204"/>
-      <c r="J51" s="205"/>
+      <c r="G51" s="198"/>
+      <c r="H51" s="199"/>
+      <c r="I51" s="199"/>
+      <c r="J51" s="200"/>
     </row>
     <row r="52" spans="2:10" ht="30.75" customHeight="1" thickBot="1">
-      <c r="B52" s="258" t="s">
+      <c r="B52" s="209" t="s">
         <v>140</v>
       </c>
-      <c r="C52" s="239"/>
-      <c r="D52" s="239"/>
-      <c r="E52" s="239"/>
-      <c r="F52" s="240"/>
+      <c r="C52" s="210"/>
+      <c r="D52" s="210"/>
+      <c r="E52" s="210"/>
+      <c r="F52" s="211"/>
     </row>
     <row r="53" spans="2:10" ht="31.5" customHeight="1" thickBot="1"/>
     <row r="54" spans="2:10" ht="24.75" customHeight="1">
-      <c r="B54" s="252" t="s">
+      <c r="B54" s="203" t="s">
+        <v>180</v>
+      </c>
+      <c r="C54" s="201" t="s">
+        <v>182</v>
+      </c>
+      <c r="D54" s="186" t="s">
         <v>181</v>
       </c>
-      <c r="C54" s="250" t="s">
-        <v>183</v>
-      </c>
-      <c r="D54" s="264" t="s">
-        <v>182</v>
-      </c>
-      <c r="E54" s="265"/>
+      <c r="E54" s="187"/>
     </row>
     <row r="55" spans="2:10" ht="24" customHeight="1" thickBot="1">
-      <c r="B55" s="253"/>
-      <c r="C55" s="251"/>
-      <c r="D55" s="266"/>
-      <c r="E55" s="267"/>
+      <c r="B55" s="204"/>
+      <c r="C55" s="202"/>
+      <c r="D55" s="188"/>
+      <c r="E55" s="189"/>
     </row>
     <row r="56" spans="2:10" ht="41.25" customHeight="1" thickBot="1">
       <c r="B56" s="81">
@@ -6704,187 +6699,284 @@
       <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D56" s="181" t="s">
-        <v>205</v>
-      </c>
-      <c r="E56" s="183"/>
+      <c r="D56" s="190" t="s">
+        <v>204</v>
+      </c>
+      <c r="E56" s="191"/>
     </row>
     <row r="57" spans="2:10" ht="31.5" customHeight="1">
       <c r="B57" s="82">
         <v>1</v>
       </c>
       <c r="C57" s="85" t="s">
-        <v>201</v>
-      </c>
-      <c r="D57" s="254" t="s">
-        <v>204</v>
-      </c>
-      <c r="E57" s="255"/>
-      <c r="F57" s="200" t="s">
-        <v>344</v>
-      </c>
-      <c r="G57" s="201"/>
-      <c r="H57" s="201"/>
-      <c r="I57" s="202"/>
+        <v>200</v>
+      </c>
+      <c r="D57" s="179" t="s">
+        <v>203</v>
+      </c>
+      <c r="E57" s="180"/>
+      <c r="F57" s="192" t="s">
+        <v>343</v>
+      </c>
+      <c r="G57" s="193"/>
+      <c r="H57" s="193"/>
+      <c r="I57" s="194"/>
     </row>
     <row r="58" spans="2:10" ht="30.75" customHeight="1" thickBot="1">
       <c r="B58" s="82">
         <v>2</v>
       </c>
       <c r="C58" s="38" t="s">
+        <v>201</v>
+      </c>
+      <c r="D58" s="179" t="s">
         <v>202</v>
       </c>
-      <c r="D58" s="254" t="s">
-        <v>203</v>
-      </c>
-      <c r="E58" s="255"/>
-      <c r="F58" s="203"/>
-      <c r="G58" s="204"/>
-      <c r="H58" s="204"/>
-      <c r="I58" s="205"/>
+      <c r="E58" s="180"/>
+      <c r="F58" s="198"/>
+      <c r="G58" s="199"/>
+      <c r="H58" s="199"/>
+      <c r="I58" s="200"/>
     </row>
     <row r="59" spans="2:10" ht="33.75" customHeight="1">
       <c r="B59" s="82">
         <v>3</v>
       </c>
       <c r="C59" s="85" t="s">
-        <v>184</v>
-      </c>
-      <c r="D59" s="254" t="s">
-        <v>187</v>
-      </c>
-      <c r="E59" s="255"/>
+        <v>183</v>
+      </c>
+      <c r="D59" s="179" t="s">
+        <v>186</v>
+      </c>
+      <c r="E59" s="180"/>
     </row>
     <row r="60" spans="2:10" ht="28.5" customHeight="1">
       <c r="B60" s="82">
         <v>4</v>
       </c>
       <c r="C60" s="38" t="s">
-        <v>185</v>
-      </c>
-      <c r="D60" s="254" t="s">
-        <v>188</v>
-      </c>
-      <c r="E60" s="255"/>
+        <v>184</v>
+      </c>
+      <c r="D60" s="179" t="s">
+        <v>187</v>
+      </c>
+      <c r="E60" s="180"/>
     </row>
     <row r="61" spans="2:10" ht="40.5" customHeight="1">
       <c r="B61" s="82">
         <v>5</v>
       </c>
       <c r="C61" s="38" t="s">
-        <v>186</v>
-      </c>
-      <c r="D61" s="254" t="s">
-        <v>189</v>
-      </c>
-      <c r="E61" s="255"/>
+        <v>185</v>
+      </c>
+      <c r="D61" s="179" t="s">
+        <v>188</v>
+      </c>
+      <c r="E61" s="180"/>
     </row>
     <row r="62" spans="2:10" ht="53.25" customHeight="1">
       <c r="B62" s="82">
         <v>6</v>
       </c>
       <c r="C62" s="85" t="s">
+        <v>193</v>
+      </c>
+      <c r="D62" s="179" t="s">
         <v>194</v>
       </c>
-      <c r="D62" s="254" t="s">
-        <v>195</v>
-      </c>
-      <c r="E62" s="255"/>
+      <c r="E62" s="180"/>
     </row>
     <row r="63" spans="2:10" ht="36" customHeight="1">
       <c r="B63" s="82">
         <v>7</v>
       </c>
       <c r="C63" s="85"/>
-      <c r="D63" s="254"/>
-      <c r="E63" s="255"/>
+      <c r="D63" s="179"/>
+      <c r="E63" s="180"/>
     </row>
     <row r="64" spans="2:10" ht="40.5" customHeight="1">
       <c r="B64" s="82">
         <v>8</v>
       </c>
       <c r="C64" s="85"/>
-      <c r="D64" s="254"/>
-      <c r="E64" s="255"/>
+      <c r="D64" s="179"/>
+      <c r="E64" s="180"/>
     </row>
     <row r="65" spans="2:5">
       <c r="B65" s="82">
         <v>9</v>
       </c>
       <c r="C65" s="85"/>
-      <c r="D65" s="254"/>
-      <c r="E65" s="255"/>
+      <c r="D65" s="179"/>
+      <c r="E65" s="180"/>
     </row>
     <row r="66" spans="2:5" ht="30" customHeight="1">
       <c r="B66" s="82">
         <v>10</v>
       </c>
       <c r="C66" s="85"/>
-      <c r="D66" s="254"/>
-      <c r="E66" s="255"/>
+      <c r="D66" s="179"/>
+      <c r="E66" s="180"/>
     </row>
     <row r="67" spans="2:5">
       <c r="B67" s="82">
         <v>11</v>
       </c>
       <c r="C67" s="85"/>
-      <c r="D67" s="254"/>
-      <c r="E67" s="255"/>
+      <c r="D67" s="179"/>
+      <c r="E67" s="180"/>
     </row>
     <row r="68" spans="2:5">
       <c r="B68" s="82">
         <v>12</v>
       </c>
       <c r="C68" s="85"/>
-      <c r="D68" s="254"/>
-      <c r="E68" s="255"/>
+      <c r="D68" s="179"/>
+      <c r="E68" s="180"/>
     </row>
     <row r="69" spans="2:5">
       <c r="B69" s="82">
         <v>13</v>
       </c>
       <c r="C69" s="85"/>
-      <c r="D69" s="254"/>
-      <c r="E69" s="255"/>
+      <c r="D69" s="179"/>
+      <c r="E69" s="180"/>
     </row>
     <row r="70" spans="2:5" ht="30" customHeight="1">
       <c r="B70" s="82">
         <v>14</v>
       </c>
       <c r="C70" s="85"/>
-      <c r="D70" s="254"/>
-      <c r="E70" s="255"/>
+      <c r="D70" s="179"/>
+      <c r="E70" s="180"/>
     </row>
     <row r="71" spans="2:5" ht="15.75" thickBot="1">
       <c r="B71" s="83">
         <v>15</v>
       </c>
       <c r="C71" s="86"/>
-      <c r="D71" s="261"/>
-      <c r="E71" s="262"/>
+      <c r="D71" s="181"/>
+      <c r="E71" s="182"/>
     </row>
     <row r="75" spans="2:5" ht="72" customHeight="1"/>
   </sheetData>
   <mergeCells count="159">
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D54:E55"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="G49:J51"/>
-    <mergeCell ref="F57:I58"/>
+    <mergeCell ref="T30:AC30"/>
+    <mergeCell ref="T31:AC31"/>
+    <mergeCell ref="T32:AC32"/>
+    <mergeCell ref="T33:AC33"/>
+    <mergeCell ref="T34:AC34"/>
+    <mergeCell ref="T35:AC35"/>
+    <mergeCell ref="T36:AC36"/>
+    <mergeCell ref="T37:AC37"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="S38:S39"/>
+    <mergeCell ref="T38:AC39"/>
+    <mergeCell ref="S44:S45"/>
+    <mergeCell ref="T44:AC45"/>
+    <mergeCell ref="T40:AC40"/>
+    <mergeCell ref="T41:AC41"/>
+    <mergeCell ref="T42:AC42"/>
+    <mergeCell ref="T43:AC43"/>
+    <mergeCell ref="T46:AC46"/>
+    <mergeCell ref="G45:J46"/>
+    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="AA20:AB20"/>
+    <mergeCell ref="AA21:AB21"/>
+    <mergeCell ref="AA22:AB22"/>
+    <mergeCell ref="AA15:AB15"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="U4:V4"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="U22:V22"/>
+    <mergeCell ref="U21:V21"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V6"/>
+    <mergeCell ref="U7:V7"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="U9:V9"/>
+    <mergeCell ref="U20:V20"/>
+    <mergeCell ref="U15:V15"/>
+    <mergeCell ref="U16:V16"/>
+    <mergeCell ref="U17:V17"/>
+    <mergeCell ref="U18:V18"/>
+    <mergeCell ref="U19:V19"/>
+    <mergeCell ref="U10:V10"/>
+    <mergeCell ref="U11:V11"/>
+    <mergeCell ref="AA23:AB23"/>
+    <mergeCell ref="AA6:AB6"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AA17:AB17"/>
+    <mergeCell ref="AA18:AB18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="N13:P13"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="N24:P24"/>
+    <mergeCell ref="E27:J27"/>
+    <mergeCell ref="E22:J22"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K2:P2"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="N26:P26"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AA11:AB11"/>
     <mergeCell ref="C54:C55"/>
     <mergeCell ref="B54:B55"/>
     <mergeCell ref="D57:E57"/>
@@ -6909,122 +7001,25 @@
     <mergeCell ref="N20:P20"/>
     <mergeCell ref="N21:P21"/>
     <mergeCell ref="N23:P23"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AA11:AB11"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="N27:P27"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="E28:J28"/>
-    <mergeCell ref="N24:P24"/>
-    <mergeCell ref="E27:J27"/>
-    <mergeCell ref="E22:J22"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K2:P2"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AA17:AB17"/>
-    <mergeCell ref="AA18:AB18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="AA19:AB19"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="AA20:AB20"/>
-    <mergeCell ref="AA21:AB21"/>
-    <mergeCell ref="AA22:AB22"/>
-    <mergeCell ref="AA15:AB15"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="U4:V4"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="U22:V22"/>
-    <mergeCell ref="U21:V21"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V6"/>
-    <mergeCell ref="U7:V7"/>
-    <mergeCell ref="U8:V8"/>
-    <mergeCell ref="U9:V9"/>
-    <mergeCell ref="U20:V20"/>
-    <mergeCell ref="U15:V15"/>
-    <mergeCell ref="U16:V16"/>
-    <mergeCell ref="U17:V17"/>
-    <mergeCell ref="U18:V18"/>
-    <mergeCell ref="U19:V19"/>
-    <mergeCell ref="U10:V10"/>
-    <mergeCell ref="U11:V11"/>
-    <mergeCell ref="AA23:AB23"/>
-    <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="T30:AC30"/>
-    <mergeCell ref="T31:AC31"/>
-    <mergeCell ref="T32:AC32"/>
-    <mergeCell ref="T33:AC33"/>
-    <mergeCell ref="T34:AC34"/>
-    <mergeCell ref="T35:AC35"/>
-    <mergeCell ref="T36:AC36"/>
-    <mergeCell ref="T37:AC37"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="S38:S39"/>
-    <mergeCell ref="T38:AC39"/>
-    <mergeCell ref="S44:S45"/>
-    <mergeCell ref="T44:AC45"/>
-    <mergeCell ref="T40:AC40"/>
-    <mergeCell ref="T41:AC41"/>
-    <mergeCell ref="T42:AC42"/>
-    <mergeCell ref="T43:AC43"/>
-    <mergeCell ref="T46:AC46"/>
-    <mergeCell ref="G45:J46"/>
-    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D54:E55"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="F57:I58"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7064,53 +7059,53 @@
     <row r="1" spans="2:28" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:28" ht="31.5" customHeight="1" thickBot="1">
       <c r="B2" s="88" t="s">
+        <v>205</v>
+      </c>
+      <c r="C2" s="103" t="s">
         <v>206</v>
       </c>
-      <c r="C2" s="103" t="s">
+      <c r="D2" s="103" t="s">
         <v>207</v>
       </c>
-      <c r="D2" s="103" t="s">
+      <c r="E2" s="119" t="s">
         <v>208</v>
       </c>
-      <c r="E2" s="119" t="s">
+      <c r="F2" s="102" t="s">
         <v>209</v>
       </c>
-      <c r="F2" s="102" t="s">
+      <c r="G2" s="192" t="s">
         <v>210</v>
       </c>
-      <c r="G2" s="200" t="s">
-        <v>211</v>
-      </c>
-      <c r="H2" s="201"/>
-      <c r="I2" s="201"/>
-      <c r="J2" s="202"/>
-      <c r="L2" s="292" t="s">
-        <v>330</v>
-      </c>
-      <c r="M2" s="293"/>
-      <c r="N2" s="293"/>
-      <c r="O2" s="294"/>
+      <c r="H2" s="193"/>
+      <c r="I2" s="193"/>
+      <c r="J2" s="194"/>
+      <c r="L2" s="284" t="s">
+        <v>329</v>
+      </c>
+      <c r="M2" s="285"/>
+      <c r="N2" s="285"/>
+      <c r="O2" s="286"/>
       <c r="P2" s="132"/>
-      <c r="Q2" s="295" t="s">
-        <v>290</v>
-      </c>
-      <c r="R2" s="296"/>
-      <c r="S2" s="296"/>
-      <c r="T2" s="297"/>
+      <c r="Q2" s="287" t="s">
+        <v>289</v>
+      </c>
+      <c r="R2" s="288"/>
+      <c r="S2" s="288"/>
+      <c r="T2" s="289"/>
       <c r="U2" s="132"/>
-      <c r="V2" s="289" t="s">
-        <v>313</v>
-      </c>
-      <c r="W2" s="290"/>
-      <c r="X2" s="290"/>
-      <c r="Y2" s="290"/>
-      <c r="Z2" s="290"/>
-      <c r="AA2" s="290"/>
-      <c r="AB2" s="291"/>
+      <c r="V2" s="277" t="s">
+        <v>312</v>
+      </c>
+      <c r="W2" s="278"/>
+      <c r="X2" s="278"/>
+      <c r="Y2" s="278"/>
+      <c r="Z2" s="278"/>
+      <c r="AA2" s="278"/>
+      <c r="AB2" s="279"/>
     </row>
     <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B3" s="89" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C3" s="95">
         <v>0</v>
@@ -7126,60 +7121,60 @@
         <v>E0000000</v>
       </c>
       <c r="G3" s="92" t="s">
-        <v>212</v>
-      </c>
-      <c r="H3" s="181" t="s">
-        <v>216</v>
-      </c>
-      <c r="I3" s="182"/>
-      <c r="J3" s="183"/>
+        <v>211</v>
+      </c>
+      <c r="H3" s="190" t="s">
+        <v>215</v>
+      </c>
+      <c r="I3" s="233"/>
+      <c r="J3" s="191"/>
       <c r="L3" s="144" t="s">
+        <v>275</v>
+      </c>
+      <c r="M3" s="145" t="s">
         <v>276</v>
       </c>
-      <c r="M3" s="145" t="s">
+      <c r="N3" s="146" t="s">
         <v>277</v>
       </c>
-      <c r="N3" s="146" t="s">
+      <c r="O3" s="147" t="s">
         <v>278</v>
-      </c>
-      <c r="O3" s="147" t="s">
-        <v>279</v>
       </c>
       <c r="P3" s="132"/>
       <c r="Q3" s="168" t="s">
+        <v>275</v>
+      </c>
+      <c r="R3" s="169" t="s">
         <v>276</v>
       </c>
-      <c r="R3" s="169" t="s">
+      <c r="S3" s="169" t="s">
         <v>277</v>
       </c>
-      <c r="S3" s="169" t="s">
+      <c r="T3" s="170" t="s">
         <v>278</v>
-      </c>
-      <c r="T3" s="170" t="s">
-        <v>279</v>
       </c>
       <c r="U3" s="132"/>
       <c r="V3" s="168" t="s">
+        <v>275</v>
+      </c>
+      <c r="W3" s="171" t="s">
         <v>276</v>
       </c>
-      <c r="W3" s="171" t="s">
+      <c r="X3" s="169" t="s">
         <v>277</v>
       </c>
-      <c r="X3" s="169" t="s">
+      <c r="Y3" s="170" t="s">
         <v>278</v>
       </c>
-      <c r="Y3" s="170" t="s">
-        <v>279</v>
-      </c>
-      <c r="Z3" s="280" t="s">
-        <v>318</v>
-      </c>
-      <c r="AA3" s="281"/>
-      <c r="AB3" s="282"/>
+      <c r="Z3" s="268" t="s">
+        <v>317</v>
+      </c>
+      <c r="AA3" s="269"/>
+      <c r="AB3" s="270"/>
     </row>
     <row r="4" spans="2:28" ht="53.25" customHeight="1">
       <c r="B4" s="90" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C4" s="98">
         <v>0</v>
@@ -7195,60 +7190,60 @@
         <v>E0008000</v>
       </c>
       <c r="G4" s="93" t="s">
-        <v>213</v>
-      </c>
-      <c r="H4" s="184">
+        <v>212</v>
+      </c>
+      <c r="H4" s="216">
         <v>63</v>
       </c>
-      <c r="I4" s="185"/>
-      <c r="J4" s="186"/>
+      <c r="I4" s="217"/>
+      <c r="J4" s="218"/>
       <c r="L4" s="150" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="M4" s="176" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="N4" s="99" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="O4" s="134" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="P4" s="132"/>
       <c r="Q4" s="162" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="R4" s="138" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="S4" s="136" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="T4" s="137" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="U4" s="132"/>
       <c r="V4" s="162" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="W4" s="138" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="X4" s="136" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="Y4" s="137" t="s">
-        <v>316</v>
-      </c>
-      <c r="Z4" s="283" t="s">
-        <v>319</v>
-      </c>
-      <c r="AA4" s="284"/>
-      <c r="AB4" s="285"/>
+        <v>315</v>
+      </c>
+      <c r="Z4" s="271" t="s">
+        <v>318</v>
+      </c>
+      <c r="AA4" s="272"/>
+      <c r="AB4" s="273"/>
     </row>
     <row r="5" spans="2:28" ht="47.25" customHeight="1">
       <c r="B5" s="90" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C5" s="98">
         <v>0</v>
@@ -7264,58 +7259,58 @@
         <v>E0010000</v>
       </c>
       <c r="G5" s="93" t="s">
-        <v>214</v>
-      </c>
-      <c r="H5" s="184">
+        <v>213</v>
+      </c>
+      <c r="H5" s="216">
         <v>31</v>
       </c>
-      <c r="I5" s="185"/>
-      <c r="J5" s="186"/>
+      <c r="I5" s="217"/>
+      <c r="J5" s="218"/>
       <c r="L5" s="148" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="M5" s="98" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="N5" s="173" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="O5" s="134" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="P5" s="132"/>
       <c r="Q5" s="163" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="R5" s="139" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="S5" s="133" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="T5" s="134" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="U5" s="132"/>
       <c r="V5" s="163" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="W5" s="139" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="X5" s="133" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="Y5" s="134" t="s">
-        <v>293</v>
-      </c>
-      <c r="Z5" s="283"/>
-      <c r="AA5" s="284"/>
-      <c r="AB5" s="285"/>
+        <v>292</v>
+      </c>
+      <c r="Z5" s="271"/>
+      <c r="AA5" s="272"/>
+      <c r="AB5" s="273"/>
     </row>
     <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B6" s="107" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C6" s="108">
         <v>0</v>
@@ -7331,58 +7326,58 @@
         <v>E0018000</v>
       </c>
       <c r="G6" s="94" t="s">
-        <v>215</v>
-      </c>
-      <c r="H6" s="197">
+        <v>214</v>
+      </c>
+      <c r="H6" s="237">
         <v>7</v>
       </c>
-      <c r="I6" s="198"/>
-      <c r="J6" s="199"/>
+      <c r="I6" s="238"/>
+      <c r="J6" s="239"/>
       <c r="L6" s="151" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="M6" s="141" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="N6" s="99" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="O6" s="134" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="P6" s="132"/>
       <c r="Q6" s="163" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="R6" s="139" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="S6" s="133" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="T6" s="134" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="U6" s="132"/>
       <c r="V6" s="164" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="W6" s="140" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="X6" s="135" t="s">
+        <v>313</v>
+      </c>
+      <c r="Y6" s="143" t="s">
         <v>314</v>
       </c>
-      <c r="Y6" s="143" t="s">
-        <v>315</v>
-      </c>
-      <c r="Z6" s="286"/>
-      <c r="AA6" s="287"/>
-      <c r="AB6" s="288"/>
+      <c r="Z6" s="274"/>
+      <c r="AA6" s="275"/>
+      <c r="AB6" s="276"/>
     </row>
     <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1">
       <c r="B7" s="89" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C7" s="95">
         <v>1</v>
@@ -7398,44 +7393,44 @@
         <v>E0100000</v>
       </c>
       <c r="G7" s="87" t="s">
-        <v>273</v>
-      </c>
-      <c r="H7" s="275" t="str">
+        <v>272</v>
+      </c>
+      <c r="H7" s="290" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12))</f>
         <v>E3FFF000</v>
       </c>
-      <c r="I7" s="276"/>
-      <c r="J7" s="277"/>
+      <c r="I7" s="291"/>
+      <c r="J7" s="292"/>
       <c r="L7" s="149" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="M7" s="142" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="N7" s="101" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="O7" s="143" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P7" s="132"/>
       <c r="Q7" s="163" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="R7" s="139" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="S7" s="133" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="T7" s="134" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="U7" s="132"/>
     </row>
     <row r="8" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B8" s="90" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C8" s="98">
         <v>1</v>
@@ -7451,41 +7446,41 @@
         <v>E0108000</v>
       </c>
       <c r="G8" s="87" t="s">
-        <v>217</v>
-      </c>
-      <c r="H8" s="275" t="str">
+        <v>216</v>
+      </c>
+      <c r="H8" s="290" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12)+4095)</f>
         <v>E3FFFFFF</v>
       </c>
-      <c r="I8" s="276"/>
-      <c r="J8" s="277"/>
-      <c r="L8" s="263" t="s">
-        <v>332</v>
-      </c>
-      <c r="M8" s="187"/>
-      <c r="N8" s="187"/>
-      <c r="O8" s="188"/>
+      <c r="I8" s="291"/>
+      <c r="J8" s="292"/>
+      <c r="L8" s="183" t="s">
+        <v>331</v>
+      </c>
+      <c r="M8" s="184"/>
+      <c r="N8" s="184"/>
+      <c r="O8" s="185"/>
       <c r="P8" s="132"/>
       <c r="Q8" s="163" t="s">
+        <v>284</v>
+      </c>
+      <c r="R8" s="139" t="s">
+        <v>279</v>
+      </c>
+      <c r="S8" s="133" t="s">
         <v>285</v>
       </c>
-      <c r="R8" s="139" t="s">
-        <v>280</v>
-      </c>
-      <c r="S8" s="133" t="s">
-        <v>286</v>
-      </c>
       <c r="T8" s="134" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="U8" s="132"/>
       <c r="X8" s="172" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="9" spans="2:28" ht="65.25" customHeight="1" thickBot="1">
       <c r="B9" s="90" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C9" s="98">
         <v>1</v>
@@ -7506,22 +7501,22 @@
       <c r="J9" s="15"/>
       <c r="P9" s="132"/>
       <c r="Q9" s="164" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="R9" s="140" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="S9" s="135" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="T9" s="143" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="U9" s="132"/>
     </row>
     <row r="10" spans="2:28" ht="28.5" customHeight="1" thickBot="1">
       <c r="B10" s="90" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C10" s="98">
         <v>1</v>
@@ -7549,7 +7544,7 @@
     </row>
     <row r="11" spans="2:28" ht="36.75" customHeight="1" thickBot="1">
       <c r="B11" s="90" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C11" s="98">
         <v>1</v>
@@ -7573,17 +7568,17 @@
       <c r="N11" s="132"/>
       <c r="O11" s="132"/>
       <c r="P11" s="132"/>
-      <c r="Q11" s="298" t="s">
-        <v>312</v>
-      </c>
-      <c r="R11" s="299"/>
-      <c r="S11" s="299"/>
-      <c r="T11" s="300"/>
+      <c r="Q11" s="293" t="s">
+        <v>311</v>
+      </c>
+      <c r="R11" s="294"/>
+      <c r="S11" s="294"/>
+      <c r="T11" s="295"/>
       <c r="U11" s="132"/>
     </row>
     <row r="12" spans="2:28" ht="44.25" customHeight="1" thickBot="1">
       <c r="B12" s="90" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C12" s="98">
         <v>1</v>
@@ -7608,22 +7603,22 @@
       <c r="O12" s="132"/>
       <c r="P12" s="132"/>
       <c r="Q12" s="144" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="R12" s="174" t="s">
+        <v>276</v>
+      </c>
+      <c r="S12" s="174" t="s">
         <v>277</v>
       </c>
-      <c r="S12" s="174" t="s">
+      <c r="T12" s="175" t="s">
         <v>278</v>
-      </c>
-      <c r="T12" s="175" t="s">
-        <v>279</v>
       </c>
       <c r="U12" s="132"/>
     </row>
     <row r="13" spans="2:28" ht="51.75" customHeight="1" thickBot="1">
       <c r="B13" s="91" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C13" s="100">
         <v>1</v>
@@ -7648,16 +7643,16 @@
       <c r="O13" s="132"/>
       <c r="P13" s="132"/>
       <c r="Q13" s="165" t="s">
+        <v>294</v>
+      </c>
+      <c r="R13" s="159" t="s">
         <v>295</v>
       </c>
-      <c r="R13" s="159" t="s">
+      <c r="S13" s="160" t="s">
         <v>296</v>
       </c>
-      <c r="S13" s="160" t="s">
+      <c r="T13" s="161" t="s">
         <v>297</v>
-      </c>
-      <c r="T13" s="161" t="s">
-        <v>298</v>
       </c>
       <c r="U13" s="132"/>
     </row>
@@ -7672,16 +7667,16 @@
       <c r="O14" s="132"/>
       <c r="P14" s="132"/>
       <c r="Q14" s="166" t="s">
+        <v>298</v>
+      </c>
+      <c r="R14" s="157" t="s">
+        <v>295</v>
+      </c>
+      <c r="S14" s="152" t="s">
         <v>299</v>
       </c>
-      <c r="R14" s="157" t="s">
-        <v>296</v>
-      </c>
-      <c r="S14" s="152" t="s">
+      <c r="T14" s="153" t="s">
         <v>300</v>
-      </c>
-      <c r="T14" s="153" t="s">
-        <v>301</v>
       </c>
       <c r="U14" s="132"/>
     </row>
@@ -7701,119 +7696,119 @@
       <c r="O15" s="132"/>
       <c r="P15" s="132"/>
       <c r="Q15" s="166" t="s">
+        <v>301</v>
+      </c>
+      <c r="R15" s="157" t="s">
         <v>302</v>
       </c>
-      <c r="R15" s="157" t="s">
+      <c r="S15" s="152" t="s">
         <v>303</v>
       </c>
-      <c r="S15" s="152" t="s">
+      <c r="T15" s="153" t="s">
         <v>304</v>
-      </c>
-      <c r="T15" s="153" t="s">
-        <v>305</v>
       </c>
       <c r="U15" s="132"/>
     </row>
     <row r="16" spans="2:28" ht="68.25" customHeight="1" thickBot="1">
       <c r="B16" s="120" t="s">
+        <v>227</v>
+      </c>
+      <c r="C16" s="121" t="s">
         <v>228</v>
       </c>
-      <c r="C16" s="121" t="s">
+      <c r="D16" s="122" t="s">
         <v>229</v>
       </c>
-      <c r="D16" s="122" t="s">
+      <c r="E16" s="122" t="s">
         <v>230</v>
       </c>
-      <c r="E16" s="122" t="s">
+      <c r="F16" s="123" t="s">
         <v>231</v>
       </c>
-      <c r="F16" s="123" t="s">
+      <c r="G16" s="209" t="s">
+        <v>269</v>
+      </c>
+      <c r="H16" s="210"/>
+      <c r="I16" s="210"/>
+      <c r="J16" s="211"/>
+      <c r="Q16" s="166" t="s">
+        <v>305</v>
+      </c>
+      <c r="R16" s="157" t="s">
+        <v>279</v>
+      </c>
+      <c r="S16" s="152" t="s">
+        <v>306</v>
+      </c>
+      <c r="T16" s="154" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="17" spans="2:20" ht="60.75" customHeight="1" thickBot="1">
+      <c r="B17" s="282" t="s">
         <v>232</v>
       </c>
-      <c r="G16" s="258" t="s">
+      <c r="C17" s="280" t="s">
+        <v>233</v>
+      </c>
+      <c r="D17" s="124" t="s">
+        <v>232</v>
+      </c>
+      <c r="E17" s="125" t="s">
+        <v>234</v>
+      </c>
+      <c r="F17" s="126" t="s">
+        <v>235</v>
+      </c>
+      <c r="G17" s="296" t="s">
         <v>270</v>
       </c>
-      <c r="H16" s="239"/>
-      <c r="I16" s="239"/>
-      <c r="J16" s="240"/>
-      <c r="Q16" s="166" t="s">
-        <v>306</v>
-      </c>
-      <c r="R16" s="157" t="s">
-        <v>280</v>
-      </c>
-      <c r="S16" s="152" t="s">
-        <v>307</v>
-      </c>
-      <c r="T16" s="154" t="s">
+      <c r="H17" s="297"/>
+      <c r="I17" s="297"/>
+      <c r="J17" s="298"/>
+      <c r="Q17" s="167" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="17" spans="2:20" ht="60.75" customHeight="1" thickBot="1">
-      <c r="B17" s="270" t="s">
-        <v>233</v>
-      </c>
-      <c r="C17" s="268" t="s">
-        <v>234</v>
-      </c>
-      <c r="D17" s="124" t="s">
-        <v>233</v>
-      </c>
-      <c r="E17" s="125" t="s">
-        <v>235</v>
-      </c>
-      <c r="F17" s="126" t="s">
+      <c r="R17" s="158" t="s">
+        <v>302</v>
+      </c>
+      <c r="S17" s="155" t="s">
+        <v>309</v>
+      </c>
+      <c r="T17" s="156" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+      <c r="B18" s="299"/>
+      <c r="C18" s="300"/>
+      <c r="D18" s="111" t="s">
         <v>236</v>
       </c>
-      <c r="G17" s="272" t="s">
+      <c r="E18" s="112" t="s">
+        <v>237</v>
+      </c>
+      <c r="F18" s="114" t="s">
+        <v>238</v>
+      </c>
+      <c r="G18" s="290" t="s">
         <v>271</v>
       </c>
-      <c r="H17" s="273"/>
-      <c r="I17" s="273"/>
-      <c r="J17" s="274"/>
-      <c r="Q17" s="167" t="s">
-        <v>309</v>
-      </c>
-      <c r="R17" s="158" t="s">
-        <v>303</v>
-      </c>
-      <c r="S17" s="155" t="s">
-        <v>310</v>
-      </c>
-      <c r="T17" s="156" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B18" s="278"/>
-      <c r="C18" s="279"/>
-      <c r="D18" s="111" t="s">
-        <v>237</v>
-      </c>
-      <c r="E18" s="112" t="s">
-        <v>238</v>
-      </c>
-      <c r="F18" s="114" t="s">
+      <c r="H18" s="291"/>
+      <c r="I18" s="291"/>
+      <c r="J18" s="292"/>
+    </row>
+    <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+      <c r="B19" s="283"/>
+      <c r="C19" s="281"/>
+      <c r="D19" s="116" t="s">
         <v>239</v>
       </c>
-      <c r="G18" s="275" t="s">
-        <v>272</v>
-      </c>
-      <c r="H18" s="276"/>
-      <c r="I18" s="276"/>
-      <c r="J18" s="277"/>
-    </row>
-    <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B19" s="271"/>
-      <c r="C19" s="269"/>
-      <c r="D19" s="116" t="s">
+      <c r="E19" s="127" t="s">
         <v>240</v>
       </c>
-      <c r="E19" s="127" t="s">
+      <c r="F19" s="117" t="s">
         <v>241</v>
-      </c>
-      <c r="F19" s="117" t="s">
-        <v>242</v>
       </c>
       <c r="G19" s="15"/>
       <c r="H19" s="15"/>
@@ -7821,20 +7816,20 @@
       <c r="J19" s="15"/>
     </row>
     <row r="20" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B20" s="270" t="s">
+      <c r="B20" s="282" t="s">
+        <v>242</v>
+      </c>
+      <c r="C20" s="280" t="s">
         <v>243</v>
       </c>
-      <c r="C20" s="268" t="s">
+      <c r="D20" s="124" t="s">
         <v>244</v>
       </c>
-      <c r="D20" s="124" t="s">
+      <c r="E20" s="125" t="s">
         <v>245</v>
       </c>
-      <c r="E20" s="125" t="s">
-        <v>246</v>
-      </c>
       <c r="F20" s="126" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G20" s="15"/>
       <c r="H20" s="15"/>
@@ -7842,16 +7837,16 @@
       <c r="J20" s="15"/>
     </row>
     <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B21" s="271"/>
-      <c r="C21" s="269"/>
+      <c r="B21" s="283"/>
+      <c r="C21" s="281"/>
       <c r="D21" s="116" t="s">
+        <v>246</v>
+      </c>
+      <c r="E21" s="115" t="s">
         <v>247</v>
       </c>
-      <c r="E21" s="115" t="s">
-        <v>248</v>
-      </c>
       <c r="F21" s="117" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G21" s="15"/>
       <c r="H21" s="15"/>
@@ -7859,20 +7854,20 @@
       <c r="J21" s="15"/>
     </row>
     <row r="22" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B22" s="270" t="s">
+      <c r="B22" s="282" t="s">
+        <v>248</v>
+      </c>
+      <c r="C22" s="280" t="s">
         <v>249</v>
       </c>
-      <c r="C22" s="268" t="s">
+      <c r="D22" s="124" t="s">
+        <v>244</v>
+      </c>
+      <c r="E22" s="113" t="s">
         <v>250</v>
       </c>
-      <c r="D22" s="124" t="s">
-        <v>245</v>
-      </c>
-      <c r="E22" s="113" t="s">
+      <c r="F22" s="126" t="s">
         <v>251</v>
-      </c>
-      <c r="F22" s="126" t="s">
-        <v>252</v>
       </c>
       <c r="G22" s="15"/>
       <c r="H22" s="15"/>
@@ -7880,16 +7875,16 @@
       <c r="J22" s="15"/>
     </row>
     <row r="23" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B23" s="271"/>
-      <c r="C23" s="269"/>
+      <c r="B23" s="283"/>
+      <c r="C23" s="281"/>
       <c r="D23" s="116" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E23" s="115" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F23" s="117" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G23" s="15"/>
       <c r="H23" s="15"/>
@@ -7897,20 +7892,20 @@
       <c r="J23" s="15"/>
     </row>
     <row r="24" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B24" s="270" t="s">
+      <c r="B24" s="282" t="s">
+        <v>253</v>
+      </c>
+      <c r="C24" s="280" t="s">
         <v>254</v>
       </c>
-      <c r="C24" s="268" t="s">
+      <c r="D24" s="124" t="s">
+        <v>232</v>
+      </c>
+      <c r="E24" s="125" t="s">
         <v>255</v>
       </c>
-      <c r="D24" s="124" t="s">
-        <v>233</v>
-      </c>
-      <c r="E24" s="125" t="s">
-        <v>256</v>
-      </c>
       <c r="F24" s="126" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G24" s="15"/>
       <c r="H24" s="15"/>
@@ -7918,16 +7913,16 @@
       <c r="J24" s="15"/>
     </row>
     <row r="25" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B25" s="271"/>
-      <c r="C25" s="269"/>
+      <c r="B25" s="283"/>
+      <c r="C25" s="281"/>
       <c r="D25" s="116" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E25" s="115" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F25" s="117" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G25" s="15"/>
       <c r="H25" s="15"/>
@@ -7936,19 +7931,19 @@
     </row>
     <row r="26" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
       <c r="B26" s="131" t="s">
+        <v>257</v>
+      </c>
+      <c r="C26" s="118" t="s">
         <v>258</v>
       </c>
-      <c r="C26" s="118" t="s">
+      <c r="D26" s="128" t="s">
+        <v>244</v>
+      </c>
+      <c r="E26" s="129" t="s">
         <v>259</v>
       </c>
-      <c r="D26" s="128" t="s">
-        <v>245</v>
-      </c>
-      <c r="E26" s="129" t="s">
-        <v>260</v>
-      </c>
       <c r="F26" s="130" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G26" s="15"/>
       <c r="H26" s="15"/>
@@ -7956,20 +7951,20 @@
       <c r="J26" s="15"/>
     </row>
     <row r="27" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B27" s="270" t="s">
-        <v>237</v>
-      </c>
-      <c r="C27" s="268" t="s">
+      <c r="B27" s="282" t="s">
+        <v>236</v>
+      </c>
+      <c r="C27" s="280" t="s">
+        <v>260</v>
+      </c>
+      <c r="D27" s="124" t="s">
+        <v>244</v>
+      </c>
+      <c r="E27" s="125" t="s">
         <v>261</v>
       </c>
-      <c r="D27" s="124" t="s">
-        <v>245</v>
-      </c>
-      <c r="E27" s="125" t="s">
-        <v>262</v>
-      </c>
       <c r="F27" s="126" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G27" s="15"/>
       <c r="H27" s="15"/>
@@ -7977,16 +7972,16 @@
       <c r="J27" s="15"/>
     </row>
     <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B28" s="271"/>
-      <c r="C28" s="269"/>
+      <c r="B28" s="283"/>
+      <c r="C28" s="281"/>
       <c r="D28" s="116" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E28" s="127" t="s">
+        <v>262</v>
+      </c>
+      <c r="F28" s="117" t="s">
         <v>263</v>
-      </c>
-      <c r="F28" s="117" t="s">
-        <v>264</v>
       </c>
       <c r="G28" s="15"/>
       <c r="H28" s="15"/>
@@ -7994,20 +7989,20 @@
       <c r="J28" s="15"/>
     </row>
     <row r="29" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B29" s="270" t="s">
+      <c r="B29" s="282" t="s">
+        <v>264</v>
+      </c>
+      <c r="C29" s="280" t="s">
         <v>265</v>
       </c>
-      <c r="C29" s="268" t="s">
+      <c r="D29" s="124" t="s">
+        <v>248</v>
+      </c>
+      <c r="E29" s="113" t="s">
         <v>266</v>
       </c>
-      <c r="D29" s="124" t="s">
-        <v>249</v>
-      </c>
-      <c r="E29" s="113" t="s">
+      <c r="F29" s="126" t="s">
         <v>267</v>
-      </c>
-      <c r="F29" s="126" t="s">
-        <v>268</v>
       </c>
       <c r="G29" s="15"/>
       <c r="H29" s="15"/>
@@ -8015,16 +8010,16 @@
       <c r="J29" s="15"/>
     </row>
     <row r="30" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B30" s="271"/>
-      <c r="C30" s="269"/>
+      <c r="B30" s="283"/>
+      <c r="C30" s="281"/>
       <c r="D30" s="116" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E30" s="115" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F30" s="117" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G30" s="15"/>
       <c r="H30" s="15"/>
@@ -8033,6 +8028,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="C17:C19"/>
     <mergeCell ref="Z3:AB3"/>
     <mergeCell ref="Z4:AB6"/>
     <mergeCell ref="V2:AB2"/>
@@ -8049,19 +8057,6 @@
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="Q11:T11"/>
     <mergeCell ref="L8:O8"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C17:C19"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Se termino la nueva version de la MMU. Quedaria probar el sistema entero
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Escritorio\Procesador-32-bits\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1964A2DD-2D08-4306-B366-3BD95F5C1A1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF8803C-73B8-4A22-BF06-2C9428F2D4E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="356">
   <si>
     <t>OpCode</t>
   </si>
@@ -1405,6 +1405,9 @@
   </si>
   <si>
     <t>Codigo para intento de ejecutar zona no ejecutable</t>
+  </si>
+  <si>
+    <t>Flush TLBs</t>
   </si>
 </sst>
 </file>
@@ -2461,7 +2464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="315">
+  <cellXfs count="316">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2997,67 +3000,79 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="74" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3069,6 +3084,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3078,155 +3102,32 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3237,32 +3138,212 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -3276,6 +3357,42 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3283,15 +3400,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3300,110 +3408,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="74" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3720,62 +3726,62 @@
   <sheetData>
     <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B2" s="224" t="s">
+      <c r="B2" s="248" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="233" t="s">
+      <c r="C2" s="263" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="234"/>
-      <c r="E2" s="235" t="s">
+      <c r="D2" s="264"/>
+      <c r="E2" s="265" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="235"/>
-      <c r="G2" s="236" t="s">
+      <c r="F2" s="265"/>
+      <c r="G2" s="266" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="235"/>
-      <c r="I2" s="235" t="s">
+      <c r="H2" s="265"/>
+      <c r="I2" s="265" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="235"/>
-      <c r="K2" s="237" t="s">
+      <c r="J2" s="265"/>
+      <c r="K2" s="267" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="235"/>
-      <c r="M2" s="235"/>
-      <c r="N2" s="235"/>
-      <c r="O2" s="235"/>
-      <c r="P2" s="238"/>
-      <c r="R2" s="243" t="s">
+      <c r="L2" s="265"/>
+      <c r="M2" s="265"/>
+      <c r="N2" s="265"/>
+      <c r="O2" s="265"/>
+      <c r="P2" s="268"/>
+      <c r="R2" s="244" t="s">
         <v>65</v>
       </c>
-      <c r="S2" s="180" t="s">
+      <c r="S2" s="242" t="s">
         <v>66</v>
       </c>
-      <c r="T2" s="247" t="s">
+      <c r="T2" s="235" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="248"/>
-      <c r="V2" s="248"/>
-      <c r="W2" s="248"/>
-      <c r="X2" s="248"/>
-      <c r="Y2" s="248"/>
-      <c r="Z2" s="248"/>
-      <c r="AA2" s="248"/>
-      <c r="AB2" s="248" t="s">
+      <c r="U2" s="236"/>
+      <c r="V2" s="236"/>
+      <c r="W2" s="236"/>
+      <c r="X2" s="236"/>
+      <c r="Y2" s="236"/>
+      <c r="Z2" s="236"/>
+      <c r="AA2" s="236"/>
+      <c r="AB2" s="236" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="248"/>
-      <c r="AD2" s="248"/>
-      <c r="AE2" s="248"/>
-      <c r="AF2" s="248"/>
-      <c r="AG2" s="248"/>
-      <c r="AH2" s="248"/>
-      <c r="AI2" s="249"/>
+      <c r="AC2" s="236"/>
+      <c r="AD2" s="236"/>
+      <c r="AE2" s="236"/>
+      <c r="AF2" s="236"/>
+      <c r="AG2" s="236"/>
+      <c r="AH2" s="236"/>
+      <c r="AI2" s="237"/>
     </row>
     <row r="3" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B3" s="225"/>
+      <c r="B3" s="249"/>
       <c r="C3" s="16" t="s">
         <v>79</v>
       </c>
@@ -3800,21 +3806,21 @@
       <c r="J3" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="230"/>
-      <c r="L3" s="231"/>
-      <c r="M3" s="231"/>
-      <c r="N3" s="231"/>
-      <c r="O3" s="231"/>
-      <c r="P3" s="232"/>
-      <c r="R3" s="244"/>
-      <c r="S3" s="241"/>
+      <c r="K3" s="220"/>
+      <c r="L3" s="262"/>
+      <c r="M3" s="262"/>
+      <c r="N3" s="262"/>
+      <c r="O3" s="262"/>
+      <c r="P3" s="221"/>
+      <c r="R3" s="245"/>
+      <c r="S3" s="184"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="211" t="s">
+      <c r="U3" s="272" t="s">
         <v>83</v>
       </c>
-      <c r="V3" s="211"/>
+      <c r="V3" s="272"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -3827,10 +3833,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="246" t="s">
+      <c r="AA3" s="234" t="s">
         <v>74</v>
       </c>
-      <c r="AB3" s="246"/>
+      <c r="AB3" s="234"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -3854,21 +3860,21 @@
       </c>
     </row>
     <row r="4" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B4" s="226"/>
+      <c r="B4" s="250"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="212" t="s">
+      <c r="E4" s="238" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="239"/>
-      <c r="G4" s="239"/>
-      <c r="H4" s="239"/>
-      <c r="I4" s="239"/>
-      <c r="J4" s="240"/>
+      <c r="F4" s="225"/>
+      <c r="G4" s="225"/>
+      <c r="H4" s="225"/>
+      <c r="I4" s="225"/>
+      <c r="J4" s="226"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -3878,20 +3884,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="212" t="s">
+      <c r="N4" s="238" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="239"/>
-      <c r="P4" s="240"/>
-      <c r="R4" s="245"/>
-      <c r="S4" s="242"/>
+      <c r="O4" s="225"/>
+      <c r="P4" s="226"/>
+      <c r="R4" s="246"/>
+      <c r="S4" s="243"/>
       <c r="T4" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="U4" s="212" t="s">
+      <c r="U4" s="238" t="s">
         <v>75</v>
       </c>
-      <c r="V4" s="213"/>
+      <c r="V4" s="239"/>
       <c r="W4" s="7" t="s">
         <v>71</v>
       </c>
@@ -3904,10 +3910,10 @@
       <c r="Z4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA4" s="212" t="s">
+      <c r="AA4" s="238" t="s">
         <v>72</v>
       </c>
-      <c r="AB4" s="213"/>
+      <c r="AB4" s="239"/>
       <c r="AC4" s="7" t="s">
         <v>12</v>
       </c>
@@ -3939,22 +3945,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="216"/>
-      <c r="F5" s="217"/>
-      <c r="G5" s="217"/>
-      <c r="H5" s="217"/>
-      <c r="I5" s="217"/>
-      <c r="J5" s="218"/>
+      <c r="E5" s="269"/>
+      <c r="F5" s="270"/>
+      <c r="G5" s="270"/>
+      <c r="H5" s="270"/>
+      <c r="I5" s="270"/>
+      <c r="J5" s="271"/>
       <c r="K5" s="25" t="s">
         <v>10</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="181" t="s">
+      <c r="N5" s="202" t="s">
         <v>51</v>
       </c>
-      <c r="O5" s="182"/>
-      <c r="P5" s="183"/>
+      <c r="O5" s="247"/>
+      <c r="P5" s="203"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -3964,10 +3970,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="214" t="s">
+      <c r="U5" s="240" t="s">
         <v>73</v>
       </c>
-      <c r="V5" s="215"/>
+      <c r="V5" s="241"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -3980,10 +3986,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="214" t="s">
+      <c r="AA5" s="240" t="s">
         <v>73</v>
       </c>
-      <c r="AB5" s="215"/>
+      <c r="AB5" s="241"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -4015,12 +4021,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="223"/>
-      <c r="F6" s="220"/>
-      <c r="G6" s="220"/>
-      <c r="H6" s="220"/>
-      <c r="I6" s="220"/>
-      <c r="J6" s="221"/>
+      <c r="E6" s="260"/>
+      <c r="F6" s="255"/>
+      <c r="G6" s="255"/>
+      <c r="H6" s="255"/>
+      <c r="I6" s="255"/>
+      <c r="J6" s="256"/>
       <c r="K6" s="31" t="s">
         <v>11</v>
       </c>
@@ -4028,11 +4034,11 @@
         <v>154</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="184" t="s">
+      <c r="N6" s="231" t="s">
         <v>95</v>
       </c>
-      <c r="O6" s="185"/>
-      <c r="P6" s="186"/>
+      <c r="O6" s="232"/>
+      <c r="P6" s="233"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -4042,10 +4048,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="209" t="s">
+      <c r="U6" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V6" s="210"/>
+      <c r="V6" s="228"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -4058,10 +4064,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="209" t="s">
+      <c r="AA6" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB6" s="210"/>
+      <c r="AB6" s="228"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -4104,9 +4110,9 @@
       <c r="G7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="219"/>
-      <c r="I7" s="220"/>
-      <c r="J7" s="221"/>
+      <c r="H7" s="254"/>
+      <c r="I7" s="255"/>
+      <c r="J7" s="256"/>
       <c r="K7" s="25" t="s">
         <v>13</v>
       </c>
@@ -4114,11 +4120,11 @@
       <c r="M7" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N7" s="184" t="s">
+      <c r="N7" s="231" t="s">
         <v>52</v>
       </c>
-      <c r="O7" s="185"/>
-      <c r="P7" s="186"/>
+      <c r="O7" s="232"/>
+      <c r="P7" s="233"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -4128,10 +4134,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="209" t="s">
+      <c r="U7" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V7" s="210"/>
+      <c r="V7" s="228"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -4144,10 +4150,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="209" t="s">
+      <c r="AA7" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB7" s="210"/>
+      <c r="AB7" s="228"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -4190,9 +4196,9 @@
       <c r="G8" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="219"/>
-      <c r="I8" s="220"/>
-      <c r="J8" s="221"/>
+      <c r="H8" s="254"/>
+      <c r="I8" s="255"/>
+      <c r="J8" s="256"/>
       <c r="K8" s="37" t="s">
         <v>14</v>
       </c>
@@ -4200,11 +4206,11 @@
       <c r="M8" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N8" s="184" t="s">
+      <c r="N8" s="231" t="s">
         <v>53</v>
       </c>
-      <c r="O8" s="185"/>
-      <c r="P8" s="186"/>
+      <c r="O8" s="232"/>
+      <c r="P8" s="233"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -4214,10 +4220,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="209" t="s">
+      <c r="U8" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V8" s="210"/>
+      <c r="V8" s="228"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -4230,10 +4236,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="209" t="s">
+      <c r="AA8" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB8" s="210"/>
+      <c r="AB8" s="228"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -4276,9 +4282,9 @@
       <c r="G9" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="219"/>
-      <c r="I9" s="220"/>
-      <c r="J9" s="221"/>
+      <c r="H9" s="254"/>
+      <c r="I9" s="255"/>
+      <c r="J9" s="256"/>
       <c r="K9" s="37" t="s">
         <v>47</v>
       </c>
@@ -4286,11 +4292,11 @@
       <c r="M9" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N9" s="184" t="s">
+      <c r="N9" s="231" t="s">
         <v>54</v>
       </c>
-      <c r="O9" s="185"/>
-      <c r="P9" s="186"/>
+      <c r="O9" s="232"/>
+      <c r="P9" s="233"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -4300,10 +4306,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="209" t="s">
+      <c r="U9" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V9" s="210"/>
+      <c r="V9" s="228"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -4316,10 +4322,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="209" t="s">
+      <c r="AA9" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB9" s="210"/>
+      <c r="AB9" s="228"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -4362,9 +4368,9 @@
       <c r="G10" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="219"/>
-      <c r="I10" s="220"/>
-      <c r="J10" s="221"/>
+      <c r="H10" s="254"/>
+      <c r="I10" s="255"/>
+      <c r="J10" s="256"/>
       <c r="K10" s="37" t="s">
         <v>48</v>
       </c>
@@ -4372,11 +4378,11 @@
       <c r="M10" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N10" s="184" t="s">
+      <c r="N10" s="231" t="s">
         <v>55</v>
       </c>
-      <c r="O10" s="185"/>
-      <c r="P10" s="186"/>
+      <c r="O10" s="232"/>
+      <c r="P10" s="233"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -4386,10 +4392,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="209" t="s">
+      <c r="U10" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V10" s="210"/>
+      <c r="V10" s="228"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -4402,10 +4408,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="209" t="s">
+      <c r="AA10" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB10" s="210"/>
+      <c r="AB10" s="228"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -4448,9 +4454,9 @@
       <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="219"/>
-      <c r="I11" s="220"/>
-      <c r="J11" s="221"/>
+      <c r="H11" s="254"/>
+      <c r="I11" s="255"/>
+      <c r="J11" s="256"/>
       <c r="K11" s="37" t="s">
         <v>15</v>
       </c>
@@ -4458,11 +4464,11 @@
       <c r="M11" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N11" s="184" t="s">
+      <c r="N11" s="231" t="s">
         <v>56</v>
       </c>
-      <c r="O11" s="185"/>
-      <c r="P11" s="186"/>
+      <c r="O11" s="232"/>
+      <c r="P11" s="233"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -4472,10 +4478,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="209" t="s">
+      <c r="U11" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V11" s="210"/>
+      <c r="V11" s="228"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -4488,10 +4494,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="209" t="s">
+      <c r="AA11" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB11" s="210"/>
+      <c r="AB11" s="228"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -4534,9 +4540,9 @@
       <c r="G12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="219"/>
-      <c r="I12" s="220"/>
-      <c r="J12" s="221"/>
+      <c r="H12" s="254"/>
+      <c r="I12" s="255"/>
+      <c r="J12" s="256"/>
       <c r="K12" s="37" t="s">
         <v>16</v>
       </c>
@@ -4544,11 +4550,11 @@
       <c r="M12" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N12" s="184" t="s">
+      <c r="N12" s="231" t="s">
         <v>57</v>
       </c>
-      <c r="O12" s="185"/>
-      <c r="P12" s="186"/>
+      <c r="O12" s="232"/>
+      <c r="P12" s="233"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -4558,10 +4564,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="209" t="s">
+      <c r="U12" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V12" s="210"/>
+      <c r="V12" s="228"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -4574,10 +4580,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="209" t="s">
+      <c r="AA12" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB12" s="210"/>
+      <c r="AB12" s="228"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -4620,9 +4626,9 @@
       <c r="G13" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="219"/>
-      <c r="I13" s="220"/>
-      <c r="J13" s="221"/>
+      <c r="H13" s="254"/>
+      <c r="I13" s="255"/>
+      <c r="J13" s="256"/>
       <c r="K13" s="37" t="s">
         <v>17</v>
       </c>
@@ -4630,11 +4636,11 @@
       <c r="M13" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N13" s="184" t="s">
+      <c r="N13" s="231" t="s">
         <v>58</v>
       </c>
-      <c r="O13" s="185"/>
-      <c r="P13" s="186"/>
+      <c r="O13" s="232"/>
+      <c r="P13" s="233"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -4644,10 +4650,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="209" t="s">
+      <c r="U13" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V13" s="210"/>
+      <c r="V13" s="228"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -4660,10 +4666,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="209" t="s">
+      <c r="AA13" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB13" s="210"/>
+      <c r="AB13" s="228"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -4706,9 +4712,9 @@
       <c r="G14" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="219"/>
-      <c r="I14" s="220"/>
-      <c r="J14" s="221"/>
+      <c r="H14" s="254"/>
+      <c r="I14" s="255"/>
+      <c r="J14" s="256"/>
       <c r="K14" s="37" t="s">
         <v>18</v>
       </c>
@@ -4716,11 +4722,11 @@
       <c r="M14" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N14" s="184" t="s">
+      <c r="N14" s="231" t="s">
         <v>59</v>
       </c>
-      <c r="O14" s="185"/>
-      <c r="P14" s="186"/>
+      <c r="O14" s="232"/>
+      <c r="P14" s="233"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -4730,10 +4736,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="209" t="s">
+      <c r="U14" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V14" s="210"/>
+      <c r="V14" s="228"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -4746,10 +4752,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="209" t="s">
+      <c r="AA14" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB14" s="210"/>
+      <c r="AB14" s="228"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -4792,9 +4798,9 @@
       <c r="G15" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="219"/>
-      <c r="I15" s="220"/>
-      <c r="J15" s="221"/>
+      <c r="H15" s="254"/>
+      <c r="I15" s="255"/>
+      <c r="J15" s="256"/>
       <c r="K15" s="31" t="s">
         <v>19</v>
       </c>
@@ -4802,11 +4808,11 @@
       <c r="M15" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N15" s="184" t="s">
+      <c r="N15" s="231" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="185"/>
-      <c r="P15" s="186"/>
+      <c r="O15" s="232"/>
+      <c r="P15" s="233"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -4816,10 +4822,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="209" t="s">
+      <c r="U15" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V15" s="210"/>
+      <c r="V15" s="228"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -4832,10 +4838,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="209" t="s">
+      <c r="AA15" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB15" s="210"/>
+      <c r="AB15" s="228"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -4872,21 +4878,21 @@
       <c r="E16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="219"/>
-      <c r="G16" s="220"/>
-      <c r="H16" s="220"/>
-      <c r="I16" s="220"/>
-      <c r="J16" s="221"/>
+      <c r="F16" s="254"/>
+      <c r="G16" s="255"/>
+      <c r="H16" s="255"/>
+      <c r="I16" s="255"/>
+      <c r="J16" s="256"/>
       <c r="K16" s="40" t="s">
         <v>49</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="184" t="s">
+      <c r="N16" s="231" t="s">
         <v>50</v>
       </c>
-      <c r="O16" s="185"/>
-      <c r="P16" s="186"/>
+      <c r="O16" s="232"/>
+      <c r="P16" s="233"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -4896,10 +4902,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="209" t="s">
+      <c r="U16" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V16" s="210"/>
+      <c r="V16" s="228"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -4912,10 +4918,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="209" t="s">
+      <c r="AA16" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB16" s="210"/>
+      <c r="AB16" s="228"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -4953,22 +4959,22 @@
         <v>28</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="222" t="s">
+      <c r="G17" s="261" t="s">
         <v>76</v>
       </c>
-      <c r="H17" s="185"/>
-      <c r="I17" s="185"/>
-      <c r="J17" s="186"/>
+      <c r="H17" s="232"/>
+      <c r="I17" s="232"/>
+      <c r="J17" s="233"/>
       <c r="K17" s="25" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="184" t="s">
+      <c r="N17" s="231" t="s">
         <v>64</v>
       </c>
-      <c r="O17" s="185"/>
-      <c r="P17" s="186"/>
+      <c r="O17" s="232"/>
+      <c r="P17" s="233"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -4978,10 +4984,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="209" t="s">
+      <c r="U17" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V17" s="210"/>
+      <c r="V17" s="228"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -4994,10 +5000,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="209" t="s">
+      <c r="AA17" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB17" s="210"/>
+      <c r="AB17" s="228"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -5035,12 +5041,12 @@
         <v>28</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="222" t="s">
+      <c r="G18" s="261" t="s">
         <v>76</v>
       </c>
-      <c r="H18" s="185"/>
-      <c r="I18" s="185"/>
-      <c r="J18" s="186"/>
+      <c r="H18" s="232"/>
+      <c r="I18" s="232"/>
+      <c r="J18" s="233"/>
       <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
@@ -5048,11 +5054,11 @@
       <c r="M18" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="N18" s="184" t="s">
+      <c r="N18" s="231" t="s">
         <v>61</v>
       </c>
-      <c r="O18" s="185"/>
-      <c r="P18" s="186"/>
+      <c r="O18" s="232"/>
+      <c r="P18" s="233"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -5062,10 +5068,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="209" t="s">
+      <c r="U18" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V18" s="210"/>
+      <c r="V18" s="228"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -5078,10 +5084,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="209" t="s">
+      <c r="AA18" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB18" s="210"/>
+      <c r="AB18" s="228"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -5117,20 +5123,20 @@
       <c r="F19" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="219"/>
-      <c r="H19" s="220"/>
-      <c r="I19" s="220"/>
-      <c r="J19" s="221"/>
+      <c r="G19" s="254"/>
+      <c r="H19" s="255"/>
+      <c r="I19" s="255"/>
+      <c r="J19" s="256"/>
       <c r="K19" s="25" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="184" t="s">
+      <c r="N19" s="231" t="s">
         <v>93</v>
       </c>
-      <c r="O19" s="185"/>
-      <c r="P19" s="186"/>
+      <c r="O19" s="232"/>
+      <c r="P19" s="233"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -5140,10 +5146,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="209" t="s">
+      <c r="U19" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V19" s="210"/>
+      <c r="V19" s="228"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -5156,10 +5162,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="209" t="s">
+      <c r="AA19" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB19" s="210"/>
+      <c r="AB19" s="228"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -5197,20 +5203,20 @@
       <c r="F20" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="219"/>
-      <c r="H20" s="220"/>
-      <c r="I20" s="220"/>
-      <c r="J20" s="221"/>
+      <c r="G20" s="254"/>
+      <c r="H20" s="255"/>
+      <c r="I20" s="255"/>
+      <c r="J20" s="256"/>
       <c r="K20" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="184" t="s">
+      <c r="N20" s="231" t="s">
         <v>94</v>
       </c>
-      <c r="O20" s="185"/>
-      <c r="P20" s="186"/>
+      <c r="O20" s="232"/>
+      <c r="P20" s="233"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -5220,10 +5226,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="209" t="s">
+      <c r="U20" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V20" s="210"/>
+      <c r="V20" s="228"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -5236,10 +5242,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="209" t="s">
+      <c r="AA20" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB20" s="210"/>
+      <c r="AB20" s="228"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -5277,20 +5283,20 @@
       <c r="F21" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="219"/>
-      <c r="H21" s="220"/>
-      <c r="I21" s="220"/>
-      <c r="J21" s="221"/>
+      <c r="G21" s="254"/>
+      <c r="H21" s="255"/>
+      <c r="I21" s="255"/>
+      <c r="J21" s="256"/>
       <c r="K21" s="44" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="184" t="s">
+      <c r="N21" s="231" t="s">
         <v>62</v>
       </c>
-      <c r="O21" s="185"/>
-      <c r="P21" s="186"/>
+      <c r="O21" s="232"/>
+      <c r="P21" s="233"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -5300,10 +5306,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="209" t="s">
+      <c r="U21" s="227" t="s">
         <v>96</v>
       </c>
-      <c r="V21" s="210"/>
+      <c r="V21" s="228"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -5316,10 +5322,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="209" t="s">
+      <c r="AA21" s="227" t="s">
         <v>98</v>
       </c>
-      <c r="AB21" s="210"/>
+      <c r="AB21" s="228"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -5353,22 +5359,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="223"/>
-      <c r="F22" s="220"/>
-      <c r="G22" s="220"/>
-      <c r="H22" s="220"/>
-      <c r="I22" s="220"/>
-      <c r="J22" s="221"/>
+      <c r="E22" s="260"/>
+      <c r="F22" s="255"/>
+      <c r="G22" s="255"/>
+      <c r="H22" s="255"/>
+      <c r="I22" s="255"/>
+      <c r="J22" s="256"/>
       <c r="K22" s="40" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="184" t="s">
+      <c r="N22" s="231" t="s">
         <v>63</v>
       </c>
-      <c r="O22" s="185"/>
-      <c r="P22" s="186"/>
+      <c r="O22" s="232"/>
+      <c r="P22" s="233"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -5378,10 +5384,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="209" t="s">
+      <c r="U22" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V22" s="210"/>
+      <c r="V22" s="228"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -5394,10 +5400,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="209" t="s">
+      <c r="AA22" s="227" t="s">
         <v>96</v>
       </c>
-      <c r="AB22" s="210"/>
+      <c r="AB22" s="228"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -5437,22 +5443,22 @@
       <c r="F23" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="222" t="s">
+      <c r="G23" s="261" t="s">
         <v>77</v>
       </c>
-      <c r="H23" s="185"/>
-      <c r="I23" s="185"/>
-      <c r="J23" s="186"/>
+      <c r="H23" s="232"/>
+      <c r="I23" s="232"/>
+      <c r="J23" s="233"/>
       <c r="K23" s="44" t="s">
         <v>26</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="184" t="s">
+      <c r="N23" s="231" t="s">
         <v>82</v>
       </c>
-      <c r="O23" s="185"/>
-      <c r="P23" s="186"/>
+      <c r="O23" s="232"/>
+      <c r="P23" s="233"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -5462,10 +5468,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="209" t="s">
+      <c r="U23" s="227" t="s">
         <v>97</v>
       </c>
-      <c r="V23" s="210"/>
+      <c r="V23" s="228"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -5478,10 +5484,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="209" t="s">
+      <c r="AA23" s="227" t="s">
         <v>96</v>
       </c>
-      <c r="AB23" s="210"/>
+      <c r="AB23" s="228"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -5521,22 +5527,22 @@
       <c r="F24" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="222" t="s">
+      <c r="G24" s="261" t="s">
         <v>77</v>
       </c>
-      <c r="H24" s="185"/>
-      <c r="I24" s="185"/>
-      <c r="J24" s="186"/>
+      <c r="H24" s="232"/>
+      <c r="I24" s="232"/>
+      <c r="J24" s="233"/>
       <c r="K24" s="31" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="184" t="s">
+      <c r="N24" s="231" t="s">
         <v>81</v>
       </c>
-      <c r="O24" s="185"/>
-      <c r="P24" s="186"/>
+      <c r="O24" s="232"/>
+      <c r="P24" s="233"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -5546,10 +5552,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="209" t="s">
+      <c r="U24" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V24" s="210"/>
+      <c r="V24" s="228"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -5562,10 +5568,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="209" t="s">
+      <c r="AA24" s="227" t="s">
         <v>98</v>
       </c>
-      <c r="AB24" s="210"/>
+      <c r="AB24" s="228"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -5603,10 +5609,10 @@
       <c r="F25" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="219"/>
-      <c r="H25" s="220"/>
-      <c r="I25" s="220"/>
-      <c r="J25" s="221"/>
+      <c r="G25" s="254"/>
+      <c r="H25" s="255"/>
+      <c r="I25" s="255"/>
+      <c r="J25" s="256"/>
       <c r="K25" s="49" t="s">
         <v>39</v>
       </c>
@@ -5614,11 +5620,11 @@
         <v>154</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="184" t="s">
+      <c r="N25" s="231" t="s">
         <v>41</v>
       </c>
-      <c r="O25" s="185"/>
-      <c r="P25" s="186"/>
+      <c r="O25" s="232"/>
+      <c r="P25" s="233"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -5628,10 +5634,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="209" t="s">
+      <c r="U25" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V25" s="210"/>
+      <c r="V25" s="228"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -5644,10 +5650,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="209" t="s">
+      <c r="AA25" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB25" s="210"/>
+      <c r="AB25" s="228"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -5685,10 +5691,10 @@
       <c r="F26" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="G26" s="219"/>
-      <c r="H26" s="220"/>
-      <c r="I26" s="220"/>
-      <c r="J26" s="221"/>
+      <c r="G26" s="254"/>
+      <c r="H26" s="255"/>
+      <c r="I26" s="255"/>
+      <c r="J26" s="256"/>
       <c r="K26" s="31" t="s">
         <v>40</v>
       </c>
@@ -5696,11 +5702,11 @@
         <v>154</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="184" t="s">
+      <c r="N26" s="231" t="s">
         <v>42</v>
       </c>
-      <c r="O26" s="185"/>
-      <c r="P26" s="186"/>
+      <c r="O26" s="232"/>
+      <c r="P26" s="233"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -5710,10 +5716,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="209" t="s">
+      <c r="U26" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V26" s="210"/>
+      <c r="V26" s="228"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -5726,10 +5732,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="209" t="s">
+      <c r="AA26" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB26" s="210"/>
+      <c r="AB26" s="228"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -5761,22 +5767,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="223"/>
-      <c r="F27" s="220"/>
-      <c r="G27" s="220"/>
-      <c r="H27" s="220"/>
-      <c r="I27" s="220"/>
-      <c r="J27" s="221"/>
+      <c r="E27" s="260"/>
+      <c r="F27" s="255"/>
+      <c r="G27" s="255"/>
+      <c r="H27" s="255"/>
+      <c r="I27" s="255"/>
+      <c r="J27" s="256"/>
       <c r="K27" s="25" t="s">
         <v>44</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="184" t="s">
+      <c r="N27" s="231" t="s">
         <v>46</v>
       </c>
-      <c r="O27" s="185"/>
-      <c r="P27" s="186"/>
+      <c r="O27" s="232"/>
+      <c r="P27" s="233"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -5786,10 +5792,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="209" t="s">
+      <c r="U27" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="V27" s="210"/>
+      <c r="V27" s="228"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -5802,10 +5808,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="209" t="s">
+      <c r="AA27" s="227" t="s">
         <v>73</v>
       </c>
-      <c r="AB27" s="210"/>
+      <c r="AB27" s="228"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -5837,12 +5843,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="227"/>
-      <c r="F28" s="228"/>
-      <c r="G28" s="228"/>
-      <c r="H28" s="228"/>
-      <c r="I28" s="228"/>
-      <c r="J28" s="229"/>
+      <c r="E28" s="257"/>
+      <c r="F28" s="258"/>
+      <c r="G28" s="258"/>
+      <c r="H28" s="258"/>
+      <c r="I28" s="258"/>
+      <c r="J28" s="259"/>
       <c r="K28" s="52" t="s">
         <v>45</v>
       </c>
@@ -5850,11 +5856,11 @@
         <v>154</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="197" t="s">
+      <c r="N28" s="251" t="s">
         <v>92</v>
       </c>
-      <c r="O28" s="198"/>
-      <c r="P28" s="199"/>
+      <c r="O28" s="252"/>
+      <c r="P28" s="253"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -5864,10 +5870,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="259" t="s">
+      <c r="U28" s="229" t="s">
         <v>73</v>
       </c>
-      <c r="V28" s="260"/>
+      <c r="V28" s="230"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -5880,10 +5886,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="259" t="s">
+      <c r="AA28" s="229" t="s">
         <v>73</v>
       </c>
-      <c r="AB28" s="260"/>
+      <c r="AB28" s="230"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -5960,18 +5966,18 @@
       <c r="S30" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="T30" s="179" t="s">
+      <c r="T30" s="273" t="s">
         <v>156</v>
       </c>
-      <c r="U30" s="179"/>
-      <c r="V30" s="179"/>
-      <c r="W30" s="179"/>
-      <c r="X30" s="179"/>
-      <c r="Y30" s="179"/>
-      <c r="Z30" s="179"/>
-      <c r="AA30" s="179"/>
-      <c r="AB30" s="179"/>
-      <c r="AC30" s="180"/>
+      <c r="U30" s="273"/>
+      <c r="V30" s="273"/>
+      <c r="W30" s="273"/>
+      <c r="X30" s="273"/>
+      <c r="Y30" s="273"/>
+      <c r="Z30" s="273"/>
+      <c r="AA30" s="273"/>
+      <c r="AB30" s="273"/>
+      <c r="AC30" s="242"/>
     </row>
     <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B31" s="67" t="s">
@@ -5997,7 +6003,9 @@
       <c r="K31" s="79"/>
       <c r="L31" s="79"/>
       <c r="M31" s="79"/>
-      <c r="N31" s="79"/>
+      <c r="N31" s="79" t="s">
+        <v>355</v>
+      </c>
       <c r="O31" s="79" t="s">
         <v>177</v>
       </c>
@@ -6010,18 +6018,18 @@
       <c r="S31" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="T31" s="181" t="s">
+      <c r="T31" s="202" t="s">
         <v>161</v>
       </c>
-      <c r="U31" s="182"/>
-      <c r="V31" s="182"/>
-      <c r="W31" s="182"/>
-      <c r="X31" s="182"/>
-      <c r="Y31" s="182"/>
-      <c r="Z31" s="182"/>
-      <c r="AA31" s="182"/>
-      <c r="AB31" s="182"/>
-      <c r="AC31" s="183"/>
+      <c r="U31" s="247"/>
+      <c r="V31" s="247"/>
+      <c r="W31" s="247"/>
+      <c r="X31" s="247"/>
+      <c r="Y31" s="247"/>
+      <c r="Z31" s="247"/>
+      <c r="AA31" s="247"/>
+      <c r="AB31" s="247"/>
+      <c r="AC31" s="203"/>
     </row>
     <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
       <c r="B32" s="4" t="s">
@@ -6039,24 +6047,25 @@
       <c r="F32" s="14" t="s">
         <v>89</v>
       </c>
+      <c r="N32" s="315"/>
       <c r="R32" s="2">
         <v>1</v>
       </c>
       <c r="S32" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="T32" s="184" t="s">
+      <c r="T32" s="231" t="s">
         <v>162</v>
       </c>
-      <c r="U32" s="185"/>
-      <c r="V32" s="185"/>
-      <c r="W32" s="185"/>
-      <c r="X32" s="185"/>
-      <c r="Y32" s="185"/>
-      <c r="Z32" s="185"/>
-      <c r="AA32" s="185"/>
-      <c r="AB32" s="185"/>
-      <c r="AC32" s="186"/>
+      <c r="U32" s="232"/>
+      <c r="V32" s="232"/>
+      <c r="W32" s="232"/>
+      <c r="X32" s="232"/>
+      <c r="Y32" s="232"/>
+      <c r="Z32" s="232"/>
+      <c r="AA32" s="232"/>
+      <c r="AB32" s="232"/>
+      <c r="AC32" s="233"/>
     </row>
     <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
       <c r="H33" s="84" t="s">
@@ -6092,31 +6101,31 @@
       <c r="S33" s="37" t="s">
         <v>158</v>
       </c>
-      <c r="T33" s="184" t="s">
+      <c r="T33" s="231" t="s">
         <v>163</v>
       </c>
-      <c r="U33" s="185"/>
-      <c r="V33" s="185"/>
-      <c r="W33" s="185"/>
-      <c r="X33" s="185"/>
-      <c r="Y33" s="185"/>
-      <c r="Z33" s="185"/>
-      <c r="AA33" s="185"/>
-      <c r="AB33" s="185"/>
-      <c r="AC33" s="186"/>
+      <c r="U33" s="232"/>
+      <c r="V33" s="232"/>
+      <c r="W33" s="232"/>
+      <c r="X33" s="232"/>
+      <c r="Y33" s="232"/>
+      <c r="Z33" s="232"/>
+      <c r="AA33" s="232"/>
+      <c r="AB33" s="232"/>
+      <c r="AC33" s="233"/>
     </row>
     <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B34" s="256" t="s">
+      <c r="B34" s="222" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="230" t="s">
+      <c r="C34" s="220" t="s">
         <v>114</v>
       </c>
-      <c r="D34" s="232"/>
-      <c r="E34" s="230" t="s">
+      <c r="D34" s="221"/>
+      <c r="E34" s="220" t="s">
         <v>115</v>
       </c>
-      <c r="F34" s="232"/>
+      <c r="F34" s="221"/>
       <c r="H34" s="77" t="s">
         <v>65</v>
       </c>
@@ -6144,21 +6153,21 @@
       <c r="S34" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T34" s="184" t="s">
+      <c r="T34" s="231" t="s">
         <v>164</v>
       </c>
-      <c r="U34" s="185"/>
-      <c r="V34" s="185"/>
-      <c r="W34" s="185"/>
-      <c r="X34" s="185"/>
-      <c r="Y34" s="185"/>
-      <c r="Z34" s="185"/>
-      <c r="AA34" s="185"/>
-      <c r="AB34" s="185"/>
-      <c r="AC34" s="186"/>
+      <c r="U34" s="232"/>
+      <c r="V34" s="232"/>
+      <c r="W34" s="232"/>
+      <c r="X34" s="232"/>
+      <c r="Y34" s="232"/>
+      <c r="Z34" s="232"/>
+      <c r="AA34" s="232"/>
+      <c r="AB34" s="232"/>
+      <c r="AC34" s="233"/>
     </row>
     <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B35" s="257"/>
+      <c r="B35" s="223"/>
       <c r="C35" s="64" t="s">
         <v>99</v>
       </c>
@@ -6177,18 +6186,18 @@
       <c r="S35" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T35" s="184" t="s">
+      <c r="T35" s="231" t="s">
         <v>165</v>
       </c>
-      <c r="U35" s="185"/>
-      <c r="V35" s="185"/>
-      <c r="W35" s="185"/>
-      <c r="X35" s="185"/>
-      <c r="Y35" s="185"/>
-      <c r="Z35" s="185"/>
-      <c r="AA35" s="185"/>
-      <c r="AB35" s="185"/>
-      <c r="AC35" s="186"/>
+      <c r="U35" s="232"/>
+      <c r="V35" s="232"/>
+      <c r="W35" s="232"/>
+      <c r="X35" s="232"/>
+      <c r="Y35" s="232"/>
+      <c r="Z35" s="232"/>
+      <c r="AA35" s="232"/>
+      <c r="AB35" s="232"/>
+      <c r="AC35" s="233"/>
     </row>
     <row r="36" spans="2:29" ht="36" customHeight="1" thickBot="1">
       <c r="B36" s="1">
@@ -6239,18 +6248,18 @@
       <c r="S36" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T36" s="184" t="s">
+      <c r="T36" s="231" t="s">
         <v>166</v>
       </c>
-      <c r="U36" s="185"/>
-      <c r="V36" s="185"/>
-      <c r="W36" s="185"/>
-      <c r="X36" s="185"/>
-      <c r="Y36" s="185"/>
-      <c r="Z36" s="185"/>
-      <c r="AA36" s="185"/>
-      <c r="AB36" s="185"/>
-      <c r="AC36" s="186"/>
+      <c r="U36" s="232"/>
+      <c r="V36" s="232"/>
+      <c r="W36" s="232"/>
+      <c r="X36" s="232"/>
+      <c r="Y36" s="232"/>
+      <c r="Z36" s="232"/>
+      <c r="AA36" s="232"/>
+      <c r="AB36" s="232"/>
+      <c r="AC36" s="233"/>
     </row>
     <row r="37" spans="2:29" ht="36.75" customHeight="1" thickBot="1">
       <c r="B37" s="2">
@@ -6293,18 +6302,18 @@
       <c r="S37" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="T37" s="184" t="s">
+      <c r="T37" s="231" t="s">
         <v>192</v>
       </c>
-      <c r="U37" s="185"/>
-      <c r="V37" s="185"/>
-      <c r="W37" s="185"/>
-      <c r="X37" s="185"/>
-      <c r="Y37" s="185"/>
-      <c r="Z37" s="185"/>
-      <c r="AA37" s="185"/>
-      <c r="AB37" s="185"/>
-      <c r="AC37" s="186"/>
+      <c r="U37" s="232"/>
+      <c r="V37" s="232"/>
+      <c r="W37" s="232"/>
+      <c r="X37" s="232"/>
+      <c r="Y37" s="232"/>
+      <c r="Z37" s="232"/>
+      <c r="AA37" s="232"/>
+      <c r="AB37" s="232"/>
+      <c r="AC37" s="233"/>
     </row>
     <row r="38" spans="2:29" ht="15.75" thickBot="1">
       <c r="B38" s="2">
@@ -6325,21 +6334,21 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="189" t="s">
+      <c r="S38" s="274" t="s">
         <v>72</v>
       </c>
-      <c r="T38" s="191" t="s">
+      <c r="T38" s="276" t="s">
         <v>167</v>
       </c>
-      <c r="U38" s="192"/>
-      <c r="V38" s="192"/>
-      <c r="W38" s="192"/>
-      <c r="X38" s="192"/>
-      <c r="Y38" s="192"/>
-      <c r="Z38" s="192"/>
-      <c r="AA38" s="192"/>
-      <c r="AB38" s="192"/>
-      <c r="AC38" s="193"/>
+      <c r="U38" s="277"/>
+      <c r="V38" s="277"/>
+      <c r="W38" s="277"/>
+      <c r="X38" s="277"/>
+      <c r="Y38" s="277"/>
+      <c r="Z38" s="277"/>
+      <c r="AA38" s="277"/>
+      <c r="AB38" s="277"/>
+      <c r="AC38" s="278"/>
     </row>
     <row r="39" spans="2:29" ht="15" customHeight="1">
       <c r="B39" s="2">
@@ -6357,26 +6366,26 @@
       <c r="F39" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G39" s="200" t="s">
+      <c r="G39" s="204" t="s">
         <v>179</v>
       </c>
-      <c r="H39" s="201"/>
-      <c r="I39" s="201"/>
-      <c r="J39" s="202"/>
+      <c r="H39" s="205"/>
+      <c r="I39" s="205"/>
+      <c r="J39" s="206"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="190"/>
-      <c r="T39" s="194"/>
-      <c r="U39" s="195"/>
-      <c r="V39" s="195"/>
-      <c r="W39" s="195"/>
-      <c r="X39" s="195"/>
-      <c r="Y39" s="195"/>
-      <c r="Z39" s="195"/>
-      <c r="AA39" s="195"/>
-      <c r="AB39" s="195"/>
-      <c r="AC39" s="196"/>
+      <c r="S39" s="275"/>
+      <c r="T39" s="279"/>
+      <c r="U39" s="280"/>
+      <c r="V39" s="280"/>
+      <c r="W39" s="280"/>
+      <c r="X39" s="280"/>
+      <c r="Y39" s="280"/>
+      <c r="Z39" s="280"/>
+      <c r="AA39" s="280"/>
+      <c r="AB39" s="280"/>
+      <c r="AC39" s="281"/>
     </row>
     <row r="40" spans="2:29" ht="37.5" customHeight="1">
       <c r="B40" s="2">
@@ -6394,28 +6403,28 @@
       <c r="F40" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="G40" s="206"/>
-      <c r="H40" s="207"/>
-      <c r="I40" s="207"/>
-      <c r="J40" s="208"/>
+      <c r="G40" s="207"/>
+      <c r="H40" s="208"/>
+      <c r="I40" s="208"/>
+      <c r="J40" s="209"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="T40" s="184" t="s">
+      <c r="T40" s="231" t="s">
         <v>168</v>
       </c>
-      <c r="U40" s="185"/>
-      <c r="V40" s="185"/>
-      <c r="W40" s="185"/>
-      <c r="X40" s="185"/>
-      <c r="Y40" s="185"/>
-      <c r="Z40" s="185"/>
-      <c r="AA40" s="185"/>
-      <c r="AB40" s="185"/>
-      <c r="AC40" s="186"/>
+      <c r="U40" s="232"/>
+      <c r="V40" s="232"/>
+      <c r="W40" s="232"/>
+      <c r="X40" s="232"/>
+      <c r="Y40" s="232"/>
+      <c r="Z40" s="232"/>
+      <c r="AA40" s="232"/>
+      <c r="AB40" s="232"/>
+      <c r="AC40" s="233"/>
     </row>
     <row r="41" spans="2:29" ht="30" customHeight="1">
       <c r="B41" s="2">
@@ -6433,28 +6442,28 @@
       <c r="F41" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G41" s="206"/>
-      <c r="H41" s="207"/>
-      <c r="I41" s="207"/>
-      <c r="J41" s="208"/>
+      <c r="G41" s="207"/>
+      <c r="H41" s="208"/>
+      <c r="I41" s="208"/>
+      <c r="J41" s="209"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T41" s="184" t="s">
+      <c r="T41" s="231" t="s">
         <v>169</v>
       </c>
-      <c r="U41" s="185"/>
-      <c r="V41" s="185"/>
-      <c r="W41" s="185"/>
-      <c r="X41" s="185"/>
-      <c r="Y41" s="185"/>
-      <c r="Z41" s="185"/>
-      <c r="AA41" s="185"/>
-      <c r="AB41" s="185"/>
-      <c r="AC41" s="186"/>
+      <c r="U41" s="232"/>
+      <c r="V41" s="232"/>
+      <c r="W41" s="232"/>
+      <c r="X41" s="232"/>
+      <c r="Y41" s="232"/>
+      <c r="Z41" s="232"/>
+      <c r="AA41" s="232"/>
+      <c r="AB41" s="232"/>
+      <c r="AC41" s="233"/>
     </row>
     <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
       <c r="B42" s="2">
@@ -6472,28 +6481,28 @@
       <c r="F42" s="76" t="s">
         <v>174</v>
       </c>
-      <c r="G42" s="203"/>
-      <c r="H42" s="204"/>
-      <c r="I42" s="204"/>
-      <c r="J42" s="205"/>
+      <c r="G42" s="210"/>
+      <c r="H42" s="211"/>
+      <c r="I42" s="211"/>
+      <c r="J42" s="212"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="T42" s="184" t="s">
+      <c r="T42" s="231" t="s">
         <v>170</v>
       </c>
-      <c r="U42" s="185"/>
-      <c r="V42" s="185"/>
-      <c r="W42" s="185"/>
-      <c r="X42" s="185"/>
-      <c r="Y42" s="185"/>
-      <c r="Z42" s="185"/>
-      <c r="AA42" s="185"/>
-      <c r="AB42" s="185"/>
-      <c r="AC42" s="186"/>
+      <c r="U42" s="232"/>
+      <c r="V42" s="232"/>
+      <c r="W42" s="232"/>
+      <c r="X42" s="232"/>
+      <c r="Y42" s="232"/>
+      <c r="Z42" s="232"/>
+      <c r="AA42" s="232"/>
+      <c r="AB42" s="232"/>
+      <c r="AC42" s="233"/>
     </row>
     <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
       <c r="B43" s="2">
@@ -6511,30 +6520,30 @@
       <c r="F43" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="G43" s="263" t="s">
+      <c r="G43" s="179" t="s">
         <v>189</v>
       </c>
-      <c r="H43" s="187"/>
-      <c r="I43" s="187"/>
-      <c r="J43" s="188"/>
+      <c r="H43" s="197"/>
+      <c r="I43" s="197"/>
+      <c r="J43" s="180"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="T43" s="184" t="s">
+      <c r="T43" s="231" t="s">
         <v>171</v>
       </c>
-      <c r="U43" s="185"/>
-      <c r="V43" s="185"/>
-      <c r="W43" s="185"/>
-      <c r="X43" s="185"/>
-      <c r="Y43" s="185"/>
-      <c r="Z43" s="185"/>
-      <c r="AA43" s="185"/>
-      <c r="AB43" s="185"/>
-      <c r="AC43" s="186"/>
+      <c r="U43" s="232"/>
+      <c r="V43" s="232"/>
+      <c r="W43" s="232"/>
+      <c r="X43" s="232"/>
+      <c r="Y43" s="232"/>
+      <c r="Z43" s="232"/>
+      <c r="AA43" s="232"/>
+      <c r="AB43" s="232"/>
+      <c r="AC43" s="233"/>
     </row>
     <row r="44" spans="2:29" ht="45.75" thickBot="1">
       <c r="B44" s="2">
@@ -6555,21 +6564,21 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="189" t="s">
+      <c r="S44" s="274" t="s">
         <v>75</v>
       </c>
-      <c r="T44" s="191" t="s">
+      <c r="T44" s="276" t="s">
         <v>172</v>
       </c>
-      <c r="U44" s="192"/>
-      <c r="V44" s="192"/>
-      <c r="W44" s="192"/>
-      <c r="X44" s="192"/>
-      <c r="Y44" s="192"/>
-      <c r="Z44" s="192"/>
-      <c r="AA44" s="192"/>
-      <c r="AB44" s="192"/>
-      <c r="AC44" s="193"/>
+      <c r="U44" s="277"/>
+      <c r="V44" s="277"/>
+      <c r="W44" s="277"/>
+      <c r="X44" s="277"/>
+      <c r="Y44" s="277"/>
+      <c r="Z44" s="277"/>
+      <c r="AA44" s="277"/>
+      <c r="AB44" s="277"/>
+      <c r="AC44" s="278"/>
     </row>
     <row r="45" spans="2:29" ht="30.75" customHeight="1">
       <c r="B45" s="2">
@@ -6587,26 +6596,26 @@
       <c r="F45" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="G45" s="200" t="s">
+      <c r="G45" s="204" t="s">
         <v>178</v>
       </c>
-      <c r="H45" s="201"/>
-      <c r="I45" s="201"/>
-      <c r="J45" s="202"/>
+      <c r="H45" s="205"/>
+      <c r="I45" s="205"/>
+      <c r="J45" s="206"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="190"/>
-      <c r="T45" s="194"/>
-      <c r="U45" s="195"/>
-      <c r="V45" s="195"/>
-      <c r="W45" s="195"/>
-      <c r="X45" s="195"/>
-      <c r="Y45" s="195"/>
-      <c r="Z45" s="195"/>
-      <c r="AA45" s="195"/>
-      <c r="AB45" s="195"/>
-      <c r="AC45" s="196"/>
+      <c r="S45" s="275"/>
+      <c r="T45" s="279"/>
+      <c r="U45" s="280"/>
+      <c r="V45" s="280"/>
+      <c r="W45" s="280"/>
+      <c r="X45" s="280"/>
+      <c r="Y45" s="280"/>
+      <c r="Z45" s="280"/>
+      <c r="AA45" s="280"/>
+      <c r="AB45" s="280"/>
+      <c r="AC45" s="281"/>
     </row>
     <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
       <c r="B46" s="2">
@@ -6624,28 +6633,28 @@
       <c r="F46" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="G46" s="203"/>
-      <c r="H46" s="204"/>
-      <c r="I46" s="204"/>
-      <c r="J46" s="205"/>
+      <c r="G46" s="210"/>
+      <c r="H46" s="211"/>
+      <c r="I46" s="211"/>
+      <c r="J46" s="212"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="T46" s="197" t="s">
+      <c r="T46" s="251" t="s">
         <v>173</v>
       </c>
-      <c r="U46" s="198"/>
-      <c r="V46" s="198"/>
-      <c r="W46" s="198"/>
-      <c r="X46" s="198"/>
-      <c r="Y46" s="198"/>
-      <c r="Z46" s="198"/>
-      <c r="AA46" s="198"/>
-      <c r="AB46" s="198"/>
-      <c r="AC46" s="199"/>
+      <c r="U46" s="252"/>
+      <c r="V46" s="252"/>
+      <c r="W46" s="252"/>
+      <c r="X46" s="252"/>
+      <c r="Y46" s="252"/>
+      <c r="Z46" s="252"/>
+      <c r="AA46" s="252"/>
+      <c r="AB46" s="252"/>
+      <c r="AC46" s="253"/>
     </row>
     <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
       <c r="B47" s="2">
@@ -6663,12 +6672,12 @@
       <c r="F47" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="G47" s="187" t="s">
+      <c r="G47" s="197" t="s">
         <v>150</v>
       </c>
-      <c r="H47" s="187"/>
-      <c r="I47" s="187"/>
-      <c r="J47" s="188"/>
+      <c r="H47" s="197"/>
+      <c r="I47" s="197"/>
+      <c r="J47" s="180"/>
     </row>
     <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
       <c r="B48" s="2">
@@ -6706,12 +6715,12 @@
       <c r="F49" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="G49" s="200" t="s">
+      <c r="G49" s="204" t="s">
         <v>153</v>
       </c>
-      <c r="H49" s="201"/>
-      <c r="I49" s="201"/>
-      <c r="J49" s="202"/>
+      <c r="H49" s="205"/>
+      <c r="I49" s="205"/>
+      <c r="J49" s="206"/>
     </row>
     <row r="50" spans="2:14" ht="30" customHeight="1">
       <c r="B50" s="2">
@@ -6729,10 +6738,10 @@
       <c r="F50" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="G50" s="206"/>
-      <c r="H50" s="207"/>
-      <c r="I50" s="207"/>
-      <c r="J50" s="208"/>
+      <c r="G50" s="207"/>
+      <c r="H50" s="208"/>
+      <c r="I50" s="208"/>
+      <c r="J50" s="209"/>
     </row>
     <row r="51" spans="2:14" ht="32.25" customHeight="1" thickBot="1">
       <c r="B51" s="4">
@@ -6750,54 +6759,54 @@
       <c r="F51" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="G51" s="203"/>
-      <c r="H51" s="204"/>
-      <c r="I51" s="204"/>
-      <c r="J51" s="205"/>
+      <c r="G51" s="210"/>
+      <c r="H51" s="211"/>
+      <c r="I51" s="211"/>
+      <c r="J51" s="212"/>
     </row>
     <row r="52" spans="2:14" ht="30.75" customHeight="1" thickBot="1">
-      <c r="B52" s="258" t="s">
+      <c r="B52" s="224" t="s">
         <v>140</v>
       </c>
-      <c r="C52" s="239"/>
-      <c r="D52" s="239"/>
-      <c r="E52" s="239"/>
-      <c r="F52" s="240"/>
+      <c r="C52" s="225"/>
+      <c r="D52" s="225"/>
+      <c r="E52" s="225"/>
+      <c r="F52" s="226"/>
     </row>
     <row r="53" spans="2:14" ht="31.5" customHeight="1" thickBot="1"/>
     <row r="54" spans="2:14" ht="36.75" customHeight="1">
-      <c r="B54" s="252" t="s">
+      <c r="B54" s="218" t="s">
         <v>180</v>
       </c>
-      <c r="C54" s="250" t="s">
+      <c r="C54" s="215" t="s">
         <v>182</v>
       </c>
-      <c r="D54" s="264" t="s">
+      <c r="D54" s="198" t="s">
         <v>181</v>
       </c>
-      <c r="E54" s="265"/>
-      <c r="H54" s="301" t="s">
+      <c r="E54" s="199"/>
+      <c r="H54" s="213" t="s">
         <v>344</v>
       </c>
-      <c r="I54" s="250" t="s">
+      <c r="I54" s="215" t="s">
         <v>182</v>
       </c>
-      <c r="J54" s="304" t="s">
+      <c r="J54" s="181" t="s">
         <v>181</v>
       </c>
-      <c r="K54" s="305"/>
-      <c r="L54" s="306"/>
+      <c r="K54" s="182"/>
+      <c r="L54" s="183"/>
     </row>
     <row r="55" spans="2:14" ht="24" customHeight="1" thickBot="1">
-      <c r="B55" s="253"/>
-      <c r="C55" s="251"/>
-      <c r="D55" s="266"/>
-      <c r="E55" s="267"/>
-      <c r="H55" s="302"/>
-      <c r="I55" s="307"/>
-      <c r="J55" s="241"/>
-      <c r="K55" s="303"/>
-      <c r="L55" s="308"/>
+      <c r="B55" s="219"/>
+      <c r="C55" s="217"/>
+      <c r="D55" s="200"/>
+      <c r="E55" s="201"/>
+      <c r="H55" s="214"/>
+      <c r="I55" s="216"/>
+      <c r="J55" s="184"/>
+      <c r="K55" s="185"/>
+      <c r="L55" s="186"/>
     </row>
     <row r="56" spans="2:14" ht="49.5" customHeight="1" thickBot="1">
       <c r="B56" s="81">
@@ -6806,25 +6815,25 @@
       <c r="C56" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D56" s="181" t="s">
+      <c r="D56" s="202" t="s">
         <v>200</v>
       </c>
-      <c r="E56" s="183"/>
+      <c r="E56" s="203"/>
       <c r="H56" s="81" t="s">
         <v>347</v>
       </c>
       <c r="I56" s="45" t="s">
         <v>342</v>
       </c>
-      <c r="J56" s="312" t="s">
+      <c r="J56" s="187" t="s">
         <v>345</v>
       </c>
-      <c r="K56" s="313"/>
-      <c r="L56" s="314"/>
-      <c r="M56" s="263" t="s">
+      <c r="K56" s="188"/>
+      <c r="L56" s="189"/>
+      <c r="M56" s="179" t="s">
         <v>348</v>
       </c>
-      <c r="N56" s="188"/>
+      <c r="N56" s="180"/>
     </row>
     <row r="57" spans="2:14" ht="49.5" customHeight="1" thickBot="1">
       <c r="B57" s="82">
@@ -6833,25 +6842,25 @@
       <c r="C57" s="85" t="s">
         <v>339</v>
       </c>
-      <c r="D57" s="254" t="s">
+      <c r="D57" s="193" t="s">
         <v>340</v>
       </c>
-      <c r="E57" s="255"/>
-      <c r="F57" s="263" t="s">
+      <c r="E57" s="194"/>
+      <c r="F57" s="179" t="s">
         <v>341</v>
       </c>
-      <c r="G57" s="188"/>
+      <c r="G57" s="180"/>
       <c r="H57" s="82">
         <v>0</v>
       </c>
       <c r="I57" s="85" t="s">
         <v>346</v>
       </c>
-      <c r="J57" s="309" t="s">
+      <c r="J57" s="190" t="s">
         <v>351</v>
       </c>
-      <c r="K57" s="310"/>
-      <c r="L57" s="311"/>
+      <c r="K57" s="191"/>
+      <c r="L57" s="192"/>
     </row>
     <row r="58" spans="2:14" ht="30.75" customHeight="1">
       <c r="B58" s="82">
@@ -6860,21 +6869,21 @@
       <c r="C58" s="85" t="s">
         <v>193</v>
       </c>
-      <c r="D58" s="254" t="s">
+      <c r="D58" s="193" t="s">
         <v>194</v>
       </c>
-      <c r="E58" s="255"/>
+      <c r="E58" s="194"/>
       <c r="H58" s="82">
         <v>1</v>
       </c>
       <c r="I58" s="85" t="s">
         <v>349</v>
       </c>
-      <c r="J58" s="309" t="s">
+      <c r="J58" s="190" t="s">
         <v>352</v>
       </c>
-      <c r="K58" s="310"/>
-      <c r="L58" s="311"/>
+      <c r="K58" s="191"/>
+      <c r="L58" s="192"/>
     </row>
     <row r="59" spans="2:14" ht="33.75" customHeight="1">
       <c r="B59" s="82">
@@ -6883,21 +6892,21 @@
       <c r="C59" s="85" t="s">
         <v>183</v>
       </c>
-      <c r="D59" s="254" t="s">
+      <c r="D59" s="193" t="s">
         <v>186</v>
       </c>
-      <c r="E59" s="255"/>
+      <c r="E59" s="194"/>
       <c r="H59" s="82">
         <v>2</v>
       </c>
       <c r="I59" s="85" t="s">
         <v>343</v>
       </c>
-      <c r="J59" s="309" t="s">
+      <c r="J59" s="190" t="s">
         <v>353</v>
       </c>
-      <c r="K59" s="310"/>
-      <c r="L59" s="311"/>
+      <c r="K59" s="191"/>
+      <c r="L59" s="192"/>
     </row>
     <row r="60" spans="2:14" ht="28.5" customHeight="1">
       <c r="B60" s="82">
@@ -6906,21 +6915,21 @@
       <c r="C60" s="38" t="s">
         <v>184</v>
       </c>
-      <c r="D60" s="254" t="s">
+      <c r="D60" s="193" t="s">
         <v>187</v>
       </c>
-      <c r="E60" s="255"/>
+      <c r="E60" s="194"/>
       <c r="H60" s="82">
         <v>3</v>
       </c>
       <c r="I60" s="38" t="s">
         <v>350</v>
       </c>
-      <c r="J60" s="309" t="s">
+      <c r="J60" s="190" t="s">
         <v>354</v>
       </c>
-      <c r="K60" s="310"/>
-      <c r="L60" s="311"/>
+      <c r="K60" s="191"/>
+      <c r="L60" s="192"/>
     </row>
     <row r="61" spans="2:14" ht="40.5" customHeight="1">
       <c r="B61" s="82">
@@ -6929,146 +6938,231 @@
       <c r="C61" s="38" t="s">
         <v>185</v>
       </c>
-      <c r="D61" s="254" t="s">
+      <c r="D61" s="193" t="s">
         <v>188</v>
       </c>
-      <c r="E61" s="255"/>
+      <c r="E61" s="194"/>
       <c r="H61" s="82">
         <v>4</v>
       </c>
       <c r="I61" s="38"/>
-      <c r="J61" s="309"/>
-      <c r="K61" s="310"/>
-      <c r="L61" s="311"/>
+      <c r="J61" s="190"/>
+      <c r="K61" s="191"/>
+      <c r="L61" s="192"/>
     </row>
     <row r="62" spans="2:14" ht="53.25" customHeight="1">
       <c r="B62" s="82">
         <v>6</v>
       </c>
       <c r="C62" s="38"/>
-      <c r="D62" s="254"/>
-      <c r="E62" s="255"/>
+      <c r="D62" s="193"/>
+      <c r="E62" s="194"/>
       <c r="H62" s="82">
         <v>5</v>
       </c>
       <c r="I62" s="38"/>
-      <c r="J62" s="309"/>
-      <c r="K62" s="310"/>
-      <c r="L62" s="311"/>
+      <c r="J62" s="190"/>
+      <c r="K62" s="191"/>
+      <c r="L62" s="192"/>
     </row>
     <row r="63" spans="2:14" ht="36" customHeight="1">
       <c r="B63" s="82">
         <v>7</v>
       </c>
       <c r="C63" s="85"/>
-      <c r="D63" s="254"/>
-      <c r="E63" s="255"/>
+      <c r="D63" s="193"/>
+      <c r="E63" s="194"/>
       <c r="H63" s="82">
         <v>6</v>
       </c>
       <c r="I63" s="85"/>
-      <c r="J63" s="309"/>
-      <c r="K63" s="310"/>
-      <c r="L63" s="311"/>
+      <c r="J63" s="190"/>
+      <c r="K63" s="191"/>
+      <c r="L63" s="192"/>
     </row>
     <row r="64" spans="2:14" ht="40.5" customHeight="1">
       <c r="B64" s="82">
         <v>8</v>
       </c>
       <c r="C64" s="85"/>
-      <c r="D64" s="254"/>
-      <c r="E64" s="255"/>
+      <c r="D64" s="193"/>
+      <c r="E64" s="194"/>
     </row>
     <row r="65" spans="2:5">
       <c r="B65" s="82">
         <v>9</v>
       </c>
       <c r="C65" s="85"/>
-      <c r="D65" s="254"/>
-      <c r="E65" s="255"/>
+      <c r="D65" s="193"/>
+      <c r="E65" s="194"/>
     </row>
     <row r="66" spans="2:5" ht="30" customHeight="1">
       <c r="B66" s="82">
         <v>10</v>
       </c>
       <c r="C66" s="85"/>
-      <c r="D66" s="254"/>
-      <c r="E66" s="255"/>
+      <c r="D66" s="193"/>
+      <c r="E66" s="194"/>
     </row>
     <row r="67" spans="2:5">
       <c r="B67" s="82">
         <v>11</v>
       </c>
       <c r="C67" s="85"/>
-      <c r="D67" s="254"/>
-      <c r="E67" s="255"/>
+      <c r="D67" s="193"/>
+      <c r="E67" s="194"/>
     </row>
     <row r="68" spans="2:5">
       <c r="B68" s="82">
         <v>12</v>
       </c>
       <c r="C68" s="85"/>
-      <c r="D68" s="254"/>
-      <c r="E68" s="255"/>
+      <c r="D68" s="193"/>
+      <c r="E68" s="194"/>
     </row>
     <row r="69" spans="2:5">
       <c r="B69" s="82">
         <v>13</v>
       </c>
       <c r="C69" s="85"/>
-      <c r="D69" s="254"/>
-      <c r="E69" s="255"/>
+      <c r="D69" s="193"/>
+      <c r="E69" s="194"/>
     </row>
     <row r="70" spans="2:5" ht="30" customHeight="1">
       <c r="B70" s="82">
         <v>14</v>
       </c>
       <c r="C70" s="85"/>
-      <c r="D70" s="254"/>
-      <c r="E70" s="255"/>
+      <c r="D70" s="193"/>
+      <c r="E70" s="194"/>
     </row>
     <row r="71" spans="2:5" ht="15.75" thickBot="1">
       <c r="B71" s="83">
         <v>15</v>
       </c>
       <c r="C71" s="86"/>
-      <c r="D71" s="261"/>
-      <c r="E71" s="262"/>
+      <c r="D71" s="195"/>
+      <c r="E71" s="196"/>
     </row>
     <row r="75" spans="2:5" ht="72" customHeight="1"/>
   </sheetData>
   <mergeCells count="171">
-    <mergeCell ref="M56:N56"/>
-    <mergeCell ref="J54:L55"/>
-    <mergeCell ref="J56:L56"/>
-    <mergeCell ref="J57:L57"/>
-    <mergeCell ref="J58:L58"/>
-    <mergeCell ref="J59:L59"/>
-    <mergeCell ref="J60:L60"/>
-    <mergeCell ref="J61:L61"/>
-    <mergeCell ref="J62:L62"/>
-    <mergeCell ref="J63:L63"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D54:E55"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="G49:J51"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="F57:G57"/>
-    <mergeCell ref="H54:H55"/>
-    <mergeCell ref="I54:I55"/>
+    <mergeCell ref="T30:AC30"/>
+    <mergeCell ref="T31:AC31"/>
+    <mergeCell ref="T32:AC32"/>
+    <mergeCell ref="T33:AC33"/>
+    <mergeCell ref="T34:AC34"/>
+    <mergeCell ref="T35:AC35"/>
+    <mergeCell ref="T36:AC36"/>
+    <mergeCell ref="T37:AC37"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="S38:S39"/>
+    <mergeCell ref="T38:AC39"/>
+    <mergeCell ref="S44:S45"/>
+    <mergeCell ref="T44:AC45"/>
+    <mergeCell ref="T40:AC40"/>
+    <mergeCell ref="T41:AC41"/>
+    <mergeCell ref="T42:AC42"/>
+    <mergeCell ref="T43:AC43"/>
+    <mergeCell ref="T46:AC46"/>
+    <mergeCell ref="G45:J46"/>
+    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="AA20:AB20"/>
+    <mergeCell ref="AA21:AB21"/>
+    <mergeCell ref="AA22:AB22"/>
+    <mergeCell ref="AA15:AB15"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="U4:V4"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="U22:V22"/>
+    <mergeCell ref="U21:V21"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V6"/>
+    <mergeCell ref="U7:V7"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="U9:V9"/>
+    <mergeCell ref="U20:V20"/>
+    <mergeCell ref="U15:V15"/>
+    <mergeCell ref="U16:V16"/>
+    <mergeCell ref="U17:V17"/>
+    <mergeCell ref="U18:V18"/>
+    <mergeCell ref="U19:V19"/>
+    <mergeCell ref="U10:V10"/>
+    <mergeCell ref="U11:V11"/>
+    <mergeCell ref="AA23:AB23"/>
+    <mergeCell ref="AA6:AB6"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AA17:AB17"/>
+    <mergeCell ref="AA18:AB18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="N13:P13"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="N24:P24"/>
+    <mergeCell ref="E27:J27"/>
+    <mergeCell ref="E22:J22"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K2:P2"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="N26:P26"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AA11:AB11"/>
     <mergeCell ref="C54:C55"/>
     <mergeCell ref="B54:B55"/>
     <mergeCell ref="D57:E57"/>
@@ -7093,122 +7187,37 @@
     <mergeCell ref="N20:P20"/>
     <mergeCell ref="N21:P21"/>
     <mergeCell ref="N23:P23"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AA11:AB11"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="N27:P27"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="E28:J28"/>
-    <mergeCell ref="N24:P24"/>
-    <mergeCell ref="E27:J27"/>
-    <mergeCell ref="E22:J22"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K2:P2"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AA17:AB17"/>
-    <mergeCell ref="AA18:AB18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="AA19:AB19"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="AA20:AB20"/>
-    <mergeCell ref="AA21:AB21"/>
-    <mergeCell ref="AA22:AB22"/>
-    <mergeCell ref="AA15:AB15"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="U4:V4"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="U22:V22"/>
-    <mergeCell ref="U21:V21"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V6"/>
-    <mergeCell ref="U7:V7"/>
-    <mergeCell ref="U8:V8"/>
-    <mergeCell ref="U9:V9"/>
-    <mergeCell ref="U20:V20"/>
-    <mergeCell ref="U15:V15"/>
-    <mergeCell ref="U16:V16"/>
-    <mergeCell ref="U17:V17"/>
-    <mergeCell ref="U18:V18"/>
-    <mergeCell ref="U19:V19"/>
-    <mergeCell ref="U10:V10"/>
-    <mergeCell ref="U11:V11"/>
-    <mergeCell ref="AA23:AB23"/>
-    <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="T30:AC30"/>
-    <mergeCell ref="T31:AC31"/>
-    <mergeCell ref="T32:AC32"/>
-    <mergeCell ref="T33:AC33"/>
-    <mergeCell ref="T34:AC34"/>
-    <mergeCell ref="T35:AC35"/>
-    <mergeCell ref="T36:AC36"/>
-    <mergeCell ref="T37:AC37"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="S38:S39"/>
-    <mergeCell ref="T38:AC39"/>
-    <mergeCell ref="S44:S45"/>
-    <mergeCell ref="T44:AC45"/>
-    <mergeCell ref="T40:AC40"/>
-    <mergeCell ref="T41:AC41"/>
-    <mergeCell ref="T42:AC42"/>
-    <mergeCell ref="T43:AC43"/>
-    <mergeCell ref="T46:AC46"/>
-    <mergeCell ref="G45:J46"/>
-    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="J63:L63"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D54:E55"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="H54:H55"/>
+    <mergeCell ref="I54:I55"/>
+    <mergeCell ref="M56:N56"/>
+    <mergeCell ref="J54:L55"/>
+    <mergeCell ref="J56:L56"/>
+    <mergeCell ref="J57:L57"/>
+    <mergeCell ref="J58:L58"/>
+    <mergeCell ref="J59:L59"/>
+    <mergeCell ref="J60:L60"/>
+    <mergeCell ref="J61:L61"/>
+    <mergeCell ref="J62:L62"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7262,35 +7271,35 @@
       <c r="F2" s="102" t="s">
         <v>205</v>
       </c>
-      <c r="G2" s="200" t="s">
+      <c r="G2" s="204" t="s">
         <v>206</v>
       </c>
-      <c r="H2" s="201"/>
-      <c r="I2" s="201"/>
-      <c r="J2" s="202"/>
-      <c r="L2" s="292" t="s">
+      <c r="H2" s="205"/>
+      <c r="I2" s="205"/>
+      <c r="J2" s="206"/>
+      <c r="L2" s="298" t="s">
         <v>325</v>
       </c>
-      <c r="M2" s="293"/>
-      <c r="N2" s="293"/>
-      <c r="O2" s="294"/>
+      <c r="M2" s="299"/>
+      <c r="N2" s="299"/>
+      <c r="O2" s="300"/>
       <c r="P2" s="132"/>
-      <c r="Q2" s="295" t="s">
+      <c r="Q2" s="301" t="s">
         <v>285</v>
       </c>
-      <c r="R2" s="296"/>
-      <c r="S2" s="296"/>
-      <c r="T2" s="297"/>
+      <c r="R2" s="302"/>
+      <c r="S2" s="302"/>
+      <c r="T2" s="303"/>
       <c r="U2" s="132"/>
-      <c r="V2" s="289" t="s">
+      <c r="V2" s="291" t="s">
         <v>308</v>
       </c>
-      <c r="W2" s="290"/>
-      <c r="X2" s="290"/>
-      <c r="Y2" s="290"/>
-      <c r="Z2" s="290"/>
-      <c r="AA2" s="290"/>
-      <c r="AB2" s="291"/>
+      <c r="W2" s="292"/>
+      <c r="X2" s="292"/>
+      <c r="Y2" s="292"/>
+      <c r="Z2" s="292"/>
+      <c r="AA2" s="292"/>
+      <c r="AB2" s="293"/>
     </row>
     <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B3" s="89" t="s">
@@ -7312,11 +7321,11 @@
       <c r="G3" s="92" t="s">
         <v>207</v>
       </c>
-      <c r="H3" s="181" t="s">
+      <c r="H3" s="202" t="s">
         <v>211</v>
       </c>
-      <c r="I3" s="182"/>
-      <c r="J3" s="183"/>
+      <c r="I3" s="247"/>
+      <c r="J3" s="203"/>
       <c r="L3" s="144" t="s">
         <v>271</v>
       </c>
@@ -7355,11 +7364,11 @@
       <c r="Y3" s="170" t="s">
         <v>274</v>
       </c>
-      <c r="Z3" s="280" t="s">
+      <c r="Z3" s="282" t="s">
         <v>313</v>
       </c>
-      <c r="AA3" s="281"/>
-      <c r="AB3" s="282"/>
+      <c r="AA3" s="283"/>
+      <c r="AB3" s="284"/>
     </row>
     <row r="4" spans="2:28" ht="53.25" customHeight="1">
       <c r="B4" s="90" t="s">
@@ -7381,11 +7390,11 @@
       <c r="G4" s="93" t="s">
         <v>208</v>
       </c>
-      <c r="H4" s="184">
+      <c r="H4" s="231">
         <v>63</v>
       </c>
-      <c r="I4" s="185"/>
-      <c r="J4" s="186"/>
+      <c r="I4" s="232"/>
+      <c r="J4" s="233"/>
       <c r="L4" s="150" t="s">
         <v>240</v>
       </c>
@@ -7424,11 +7433,11 @@
       <c r="Y4" s="137" t="s">
         <v>311</v>
       </c>
-      <c r="Z4" s="283" t="s">
+      <c r="Z4" s="285" t="s">
         <v>314</v>
       </c>
-      <c r="AA4" s="284"/>
-      <c r="AB4" s="285"/>
+      <c r="AA4" s="286"/>
+      <c r="AB4" s="287"/>
     </row>
     <row r="5" spans="2:28" ht="47.25" customHeight="1">
       <c r="B5" s="90" t="s">
@@ -7450,11 +7459,11 @@
       <c r="G5" s="93" t="s">
         <v>209</v>
       </c>
-      <c r="H5" s="184">
+      <c r="H5" s="231">
         <v>31</v>
       </c>
-      <c r="I5" s="185"/>
-      <c r="J5" s="186"/>
+      <c r="I5" s="232"/>
+      <c r="J5" s="233"/>
       <c r="L5" s="148" t="s">
         <v>249</v>
       </c>
@@ -7493,9 +7502,9 @@
       <c r="Y5" s="134" t="s">
         <v>288</v>
       </c>
-      <c r="Z5" s="283"/>
-      <c r="AA5" s="284"/>
-      <c r="AB5" s="285"/>
+      <c r="Z5" s="285"/>
+      <c r="AA5" s="286"/>
+      <c r="AB5" s="287"/>
     </row>
     <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
       <c r="B6" s="107" t="s">
@@ -7517,11 +7526,11 @@
       <c r="G6" s="94" t="s">
         <v>210</v>
       </c>
-      <c r="H6" s="197">
+      <c r="H6" s="251">
         <v>7</v>
       </c>
-      <c r="I6" s="198"/>
-      <c r="J6" s="199"/>
+      <c r="I6" s="252"/>
+      <c r="J6" s="253"/>
       <c r="L6" s="151" t="s">
         <v>235</v>
       </c>
@@ -7560,9 +7569,9 @@
       <c r="Y6" s="143" t="s">
         <v>310</v>
       </c>
-      <c r="Z6" s="286"/>
-      <c r="AA6" s="287"/>
-      <c r="AB6" s="288"/>
+      <c r="Z6" s="288"/>
+      <c r="AA6" s="289"/>
+      <c r="AB6" s="290"/>
     </row>
     <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1">
       <c r="B7" s="89" t="s">
@@ -7584,12 +7593,12 @@
       <c r="G7" s="87" t="s">
         <v>268</v>
       </c>
-      <c r="H7" s="275" t="str">
+      <c r="H7" s="304" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12))</f>
         <v>E3FFF000</v>
       </c>
-      <c r="I7" s="276"/>
-      <c r="J7" s="277"/>
+      <c r="I7" s="305"/>
+      <c r="J7" s="306"/>
       <c r="L7" s="149" t="s">
         <v>260</v>
       </c>
@@ -7637,18 +7646,18 @@
       <c r="G8" s="87" t="s">
         <v>212</v>
       </c>
-      <c r="H8" s="275" t="str">
+      <c r="H8" s="304" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12)+4095)</f>
         <v>E3FFFFFF</v>
       </c>
-      <c r="I8" s="276"/>
-      <c r="J8" s="277"/>
-      <c r="L8" s="263" t="s">
+      <c r="I8" s="305"/>
+      <c r="J8" s="306"/>
+      <c r="L8" s="179" t="s">
         <v>327</v>
       </c>
-      <c r="M8" s="187"/>
-      <c r="N8" s="187"/>
-      <c r="O8" s="188"/>
+      <c r="M8" s="197"/>
+      <c r="N8" s="197"/>
+      <c r="O8" s="180"/>
       <c r="P8" s="132"/>
       <c r="Q8" s="163" t="s">
         <v>280</v>
@@ -7757,12 +7766,12 @@
       <c r="N11" s="132"/>
       <c r="O11" s="132"/>
       <c r="P11" s="132"/>
-      <c r="Q11" s="298" t="s">
+      <c r="Q11" s="307" t="s">
         <v>307</v>
       </c>
-      <c r="R11" s="299"/>
-      <c r="S11" s="299"/>
-      <c r="T11" s="300"/>
+      <c r="R11" s="308"/>
+      <c r="S11" s="308"/>
+      <c r="T11" s="309"/>
       <c r="U11" s="132"/>
     </row>
     <row r="12" spans="2:28" ht="44.25" customHeight="1" thickBot="1">
@@ -7914,12 +7923,12 @@
       <c r="F16" s="123" t="s">
         <v>227</v>
       </c>
-      <c r="G16" s="258" t="s">
+      <c r="G16" s="224" t="s">
         <v>265</v>
       </c>
-      <c r="H16" s="239"/>
-      <c r="I16" s="239"/>
-      <c r="J16" s="240"/>
+      <c r="H16" s="225"/>
+      <c r="I16" s="225"/>
+      <c r="J16" s="226"/>
       <c r="Q16" s="166" t="s">
         <v>301</v>
       </c>
@@ -7934,10 +7943,10 @@
       </c>
     </row>
     <row r="17" spans="2:20" ht="60.75" customHeight="1" thickBot="1">
-      <c r="B17" s="270" t="s">
+      <c r="B17" s="296" t="s">
         <v>228</v>
       </c>
-      <c r="C17" s="268" t="s">
+      <c r="C17" s="294" t="s">
         <v>229</v>
       </c>
       <c r="D17" s="124" t="s">
@@ -7949,12 +7958,12 @@
       <c r="F17" s="126" t="s">
         <v>231</v>
       </c>
-      <c r="G17" s="272" t="s">
+      <c r="G17" s="310" t="s">
         <v>266</v>
       </c>
-      <c r="H17" s="273"/>
-      <c r="I17" s="273"/>
-      <c r="J17" s="274"/>
+      <c r="H17" s="311"/>
+      <c r="I17" s="311"/>
+      <c r="J17" s="312"/>
       <c r="Q17" s="167" t="s">
         <v>304</v>
       </c>
@@ -7969,8 +7978,8 @@
       </c>
     </row>
     <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B18" s="278"/>
-      <c r="C18" s="279"/>
+      <c r="B18" s="313"/>
+      <c r="C18" s="314"/>
       <c r="D18" s="111" t="s">
         <v>232</v>
       </c>
@@ -7980,16 +7989,16 @@
       <c r="F18" s="114" t="s">
         <v>234</v>
       </c>
-      <c r="G18" s="275" t="s">
+      <c r="G18" s="304" t="s">
         <v>267</v>
       </c>
-      <c r="H18" s="276"/>
-      <c r="I18" s="276"/>
-      <c r="J18" s="277"/>
+      <c r="H18" s="305"/>
+      <c r="I18" s="305"/>
+      <c r="J18" s="306"/>
     </row>
     <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B19" s="271"/>
-      <c r="C19" s="269"/>
+      <c r="B19" s="297"/>
+      <c r="C19" s="295"/>
       <c r="D19" s="116" t="s">
         <v>235</v>
       </c>
@@ -8005,10 +8014,10 @@
       <c r="J19" s="15"/>
     </row>
     <row r="20" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B20" s="270" t="s">
+      <c r="B20" s="296" t="s">
         <v>238</v>
       </c>
-      <c r="C20" s="268" t="s">
+      <c r="C20" s="294" t="s">
         <v>239</v>
       </c>
       <c r="D20" s="124" t="s">
@@ -8026,8 +8035,8 @@
       <c r="J20" s="15"/>
     </row>
     <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B21" s="271"/>
-      <c r="C21" s="269"/>
+      <c r="B21" s="297"/>
+      <c r="C21" s="295"/>
       <c r="D21" s="116" t="s">
         <v>242</v>
       </c>
@@ -8043,10 +8052,10 @@
       <c r="J21" s="15"/>
     </row>
     <row r="22" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B22" s="270" t="s">
+      <c r="B22" s="296" t="s">
         <v>244</v>
       </c>
-      <c r="C22" s="268" t="s">
+      <c r="C22" s="294" t="s">
         <v>245</v>
       </c>
       <c r="D22" s="124" t="s">
@@ -8064,8 +8073,8 @@
       <c r="J22" s="15"/>
     </row>
     <row r="23" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B23" s="271"/>
-      <c r="C23" s="269"/>
+      <c r="B23" s="297"/>
+      <c r="C23" s="295"/>
       <c r="D23" s="116" t="s">
         <v>238</v>
       </c>
@@ -8081,10 +8090,10 @@
       <c r="J23" s="15"/>
     </row>
     <row r="24" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B24" s="270" t="s">
+      <c r="B24" s="296" t="s">
         <v>249</v>
       </c>
-      <c r="C24" s="268" t="s">
+      <c r="C24" s="294" t="s">
         <v>250</v>
       </c>
       <c r="D24" s="124" t="s">
@@ -8102,8 +8111,8 @@
       <c r="J24" s="15"/>
     </row>
     <row r="25" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B25" s="271"/>
-      <c r="C25" s="269"/>
+      <c r="B25" s="297"/>
+      <c r="C25" s="295"/>
       <c r="D25" s="116" t="s">
         <v>244</v>
       </c>
@@ -8140,10 +8149,10 @@
       <c r="J26" s="15"/>
     </row>
     <row r="27" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B27" s="270" t="s">
+      <c r="B27" s="296" t="s">
         <v>232</v>
       </c>
-      <c r="C27" s="268" t="s">
+      <c r="C27" s="294" t="s">
         <v>256</v>
       </c>
       <c r="D27" s="124" t="s">
@@ -8161,8 +8170,8 @@
       <c r="J27" s="15"/>
     </row>
     <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B28" s="271"/>
-      <c r="C28" s="269"/>
+      <c r="B28" s="297"/>
+      <c r="C28" s="295"/>
       <c r="D28" s="116" t="s">
         <v>249</v>
       </c>
@@ -8178,10 +8187,10 @@
       <c r="J28" s="15"/>
     </row>
     <row r="29" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B29" s="270" t="s">
+      <c r="B29" s="296" t="s">
         <v>260</v>
       </c>
-      <c r="C29" s="268" t="s">
+      <c r="C29" s="294" t="s">
         <v>261</v>
       </c>
       <c r="D29" s="124" t="s">
@@ -8199,8 +8208,8 @@
       <c r="J29" s="15"/>
     </row>
     <row r="30" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B30" s="271"/>
-      <c r="C30" s="269"/>
+      <c r="B30" s="297"/>
+      <c r="C30" s="295"/>
       <c r="D30" s="116" t="s">
         <v>253</v>
       </c>
@@ -8217,6 +8226,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="C17:C19"/>
     <mergeCell ref="Z3:AB3"/>
     <mergeCell ref="Z4:AB6"/>
     <mergeCell ref="V2:AB2"/>
@@ -8233,19 +8255,6 @@
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="Q11:T11"/>
     <mergeCell ref="L8:O8"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C17:C19"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Se probo el sistema de ECAMs basico. Escritura de registros y activación. Queda probarlo con un dispositivo y probar la lectura
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF109DF0-A31D-4D95-98E0-FCF8388255BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A46BD151-59A6-49BF-A562-8E457EA2DBFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CPU" sheetId="1" r:id="rId1"/>
@@ -1477,7 +1477,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3117,6 +3117,159 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3135,12 +3288,6 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="74" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3219,21 +3366,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3243,29 +3378,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3309,15 +3426,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3330,15 +3438,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3378,9 +3477,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3390,15 +3486,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3482,93 +3569,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3851,7 +3851,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:AI75"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="15"/>
     <col min="2" max="2" width="19.85546875" style="15" customWidth="1"/>
@@ -3887,64 +3887,64 @@
     <col min="36" max="16384" width="9.140625" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
-    <row r="2" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B2" s="273" t="s">
+    <row r="1" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="305" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="288" t="s">
+      <c r="C2" s="317" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="289"/>
-      <c r="E2" s="290" t="s">
+      <c r="D2" s="318"/>
+      <c r="E2" s="319" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="290"/>
-      <c r="G2" s="291" t="s">
+      <c r="F2" s="319"/>
+      <c r="G2" s="320" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="290"/>
-      <c r="I2" s="290" t="s">
+      <c r="H2" s="319"/>
+      <c r="I2" s="319" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="290"/>
-      <c r="K2" s="292" t="s">
+      <c r="J2" s="319"/>
+      <c r="K2" s="321" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="290"/>
-      <c r="M2" s="290"/>
-      <c r="N2" s="290"/>
-      <c r="O2" s="290"/>
-      <c r="P2" s="293"/>
-      <c r="R2" s="269" t="s">
+      <c r="L2" s="319"/>
+      <c r="M2" s="319"/>
+      <c r="N2" s="319"/>
+      <c r="O2" s="319"/>
+      <c r="P2" s="322"/>
+      <c r="R2" s="302" t="s">
         <v>61</v>
       </c>
-      <c r="S2" s="267" t="s">
+      <c r="S2" s="300" t="s">
         <v>62</v>
       </c>
-      <c r="T2" s="260" t="s">
+      <c r="T2" s="293" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="261"/>
-      <c r="V2" s="261"/>
-      <c r="W2" s="261"/>
-      <c r="X2" s="261"/>
-      <c r="Y2" s="261"/>
-      <c r="Z2" s="261"/>
-      <c r="AA2" s="261"/>
-      <c r="AB2" s="261" t="s">
+      <c r="U2" s="294"/>
+      <c r="V2" s="294"/>
+      <c r="W2" s="294"/>
+      <c r="X2" s="294"/>
+      <c r="Y2" s="294"/>
+      <c r="Z2" s="294"/>
+      <c r="AA2" s="294"/>
+      <c r="AB2" s="294" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="261"/>
-      <c r="AD2" s="261"/>
-      <c r="AE2" s="261"/>
-      <c r="AF2" s="261"/>
-      <c r="AG2" s="261"/>
-      <c r="AH2" s="261"/>
-      <c r="AI2" s="262"/>
-    </row>
-    <row r="3" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B3" s="274"/>
+      <c r="AC2" s="294"/>
+      <c r="AD2" s="294"/>
+      <c r="AE2" s="294"/>
+      <c r="AF2" s="294"/>
+      <c r="AG2" s="294"/>
+      <c r="AH2" s="294"/>
+      <c r="AI2" s="295"/>
+    </row>
+    <row r="3" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="306"/>
       <c r="C3" s="16" t="s">
         <v>75</v>
       </c>
@@ -3969,21 +3969,21 @@
       <c r="J3" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="245"/>
-      <c r="L3" s="287"/>
-      <c r="M3" s="287"/>
-      <c r="N3" s="287"/>
-      <c r="O3" s="287"/>
-      <c r="P3" s="246"/>
-      <c r="R3" s="270"/>
-      <c r="S3" s="196"/>
+      <c r="K3" s="284"/>
+      <c r="L3" s="316"/>
+      <c r="M3" s="316"/>
+      <c r="N3" s="316"/>
+      <c r="O3" s="316"/>
+      <c r="P3" s="285"/>
+      <c r="R3" s="303"/>
+      <c r="S3" s="245"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="297" t="s">
+      <c r="U3" s="326" t="s">
         <v>79</v>
       </c>
-      <c r="V3" s="297"/>
+      <c r="V3" s="326"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -3996,10 +3996,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="259" t="s">
+      <c r="AA3" s="292" t="s">
         <v>70</v>
       </c>
-      <c r="AB3" s="259"/>
+      <c r="AB3" s="292"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -4022,22 +4022,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B4" s="275"/>
+    <row r="4" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="307"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="263" t="s">
+      <c r="E4" s="296" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="250"/>
-      <c r="G4" s="250"/>
-      <c r="H4" s="250"/>
-      <c r="I4" s="250"/>
-      <c r="J4" s="251"/>
+      <c r="F4" s="229"/>
+      <c r="G4" s="229"/>
+      <c r="H4" s="229"/>
+      <c r="I4" s="229"/>
+      <c r="J4" s="230"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -4047,20 +4047,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="263" t="s">
+      <c r="N4" s="296" t="s">
         <v>333</v>
       </c>
-      <c r="O4" s="250"/>
-      <c r="P4" s="251"/>
-      <c r="R4" s="271"/>
-      <c r="S4" s="268"/>
+      <c r="O4" s="229"/>
+      <c r="P4" s="230"/>
+      <c r="R4" s="304"/>
+      <c r="S4" s="301"/>
       <c r="T4" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="U4" s="263" t="s">
+      <c r="U4" s="296" t="s">
         <v>71</v>
       </c>
-      <c r="V4" s="264"/>
+      <c r="V4" s="297"/>
       <c r="W4" s="7" t="s">
         <v>67</v>
       </c>
@@ -4073,10 +4073,10 @@
       <c r="Z4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AA4" s="263" t="s">
+      <c r="AA4" s="296" t="s">
         <v>68</v>
       </c>
-      <c r="AB4" s="264"/>
+      <c r="AB4" s="297"/>
       <c r="AC4" s="7" t="s">
         <v>11</v>
       </c>
@@ -4099,7 +4099,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="2:35" ht="15.75" thickBot="1">
+    <row r="5" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
         <v>0</v>
       </c>
@@ -4108,22 +4108,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="294"/>
-      <c r="F5" s="295"/>
-      <c r="G5" s="295"/>
-      <c r="H5" s="295"/>
-      <c r="I5" s="295"/>
-      <c r="J5" s="296"/>
+      <c r="E5" s="323"/>
+      <c r="F5" s="324"/>
+      <c r="G5" s="324"/>
+      <c r="H5" s="324"/>
+      <c r="I5" s="324"/>
+      <c r="J5" s="325"/>
       <c r="K5" s="25" t="s">
         <v>9</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="230" t="s">
+      <c r="N5" s="219" t="s">
         <v>49</v>
       </c>
-      <c r="O5" s="272"/>
-      <c r="P5" s="231"/>
+      <c r="O5" s="220"/>
+      <c r="P5" s="221"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -4133,10 +4133,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="265" t="s">
+      <c r="U5" s="298" t="s">
         <v>69</v>
       </c>
-      <c r="V5" s="266"/>
+      <c r="V5" s="299"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -4149,10 +4149,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="265" t="s">
+      <c r="AA5" s="298" t="s">
         <v>69</v>
       </c>
-      <c r="AB5" s="266"/>
+      <c r="AB5" s="299"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -4175,7 +4175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:35" ht="15.75" thickBot="1">
+    <row r="6" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2">
         <v>1</v>
       </c>
@@ -4184,12 +4184,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="285"/>
-      <c r="F6" s="280"/>
-      <c r="G6" s="280"/>
-      <c r="H6" s="280"/>
-      <c r="I6" s="280"/>
-      <c r="J6" s="281"/>
+      <c r="E6" s="314"/>
+      <c r="F6" s="309"/>
+      <c r="G6" s="309"/>
+      <c r="H6" s="309"/>
+      <c r="I6" s="309"/>
+      <c r="J6" s="310"/>
       <c r="K6" s="31" t="s">
         <v>10</v>
       </c>
@@ -4197,11 +4197,11 @@
         <v>133</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="256" t="s">
+      <c r="N6" s="216" t="s">
         <v>334</v>
       </c>
-      <c r="O6" s="257"/>
-      <c r="P6" s="258"/>
+      <c r="O6" s="217"/>
+      <c r="P6" s="218"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -4211,10 +4211,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="252" t="s">
+      <c r="U6" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V6" s="253"/>
+      <c r="V6" s="289"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -4227,10 +4227,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="252" t="s">
+      <c r="AA6" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB6" s="253"/>
+      <c r="AB6" s="289"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -4253,7 +4253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:35" ht="15.75" thickBot="1">
+    <row r="7" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2">
         <v>2</v>
       </c>
@@ -4273,9 +4273,9 @@
       <c r="G7" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="279"/>
-      <c r="I7" s="280"/>
-      <c r="J7" s="281"/>
+      <c r="H7" s="308"/>
+      <c r="I7" s="309"/>
+      <c r="J7" s="310"/>
       <c r="K7" s="25" t="s">
         <v>12</v>
       </c>
@@ -4283,11 +4283,11 @@
       <c r="M7" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N7" s="256" t="s">
+      <c r="N7" s="216" t="s">
         <v>50</v>
       </c>
-      <c r="O7" s="257"/>
-      <c r="P7" s="258"/>
+      <c r="O7" s="217"/>
+      <c r="P7" s="218"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -4297,10 +4297,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="252" t="s">
+      <c r="U7" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V7" s="253"/>
+      <c r="V7" s="289"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -4313,10 +4313,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="252" t="s">
+      <c r="AA7" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB7" s="253"/>
+      <c r="AB7" s="289"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -4339,7 +4339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:35" ht="15.75" thickBot="1">
+    <row r="8" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2">
         <v>3</v>
       </c>
@@ -4359,9 +4359,9 @@
       <c r="G8" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H8" s="279"/>
-      <c r="I8" s="280"/>
-      <c r="J8" s="281"/>
+      <c r="H8" s="308"/>
+      <c r="I8" s="309"/>
+      <c r="J8" s="310"/>
       <c r="K8" s="37" t="s">
         <v>13</v>
       </c>
@@ -4369,11 +4369,11 @@
       <c r="M8" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N8" s="256" t="s">
+      <c r="N8" s="216" t="s">
         <v>51</v>
       </c>
-      <c r="O8" s="257"/>
-      <c r="P8" s="258"/>
+      <c r="O8" s="217"/>
+      <c r="P8" s="218"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -4383,10 +4383,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="252" t="s">
+      <c r="U8" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V8" s="253"/>
+      <c r="V8" s="289"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -4399,10 +4399,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="252" t="s">
+      <c r="AA8" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB8" s="253"/>
+      <c r="AB8" s="289"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -4425,7 +4425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:35" ht="15.75" thickBot="1">
+    <row r="9" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
         <v>4</v>
       </c>
@@ -4445,9 +4445,9 @@
       <c r="G9" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H9" s="279"/>
-      <c r="I9" s="280"/>
-      <c r="J9" s="281"/>
+      <c r="H9" s="308"/>
+      <c r="I9" s="309"/>
+      <c r="J9" s="310"/>
       <c r="K9" s="37" t="s">
         <v>46</v>
       </c>
@@ -4455,11 +4455,11 @@
       <c r="M9" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N9" s="256" t="s">
+      <c r="N9" s="216" t="s">
         <v>52</v>
       </c>
-      <c r="O9" s="257"/>
-      <c r="P9" s="258"/>
+      <c r="O9" s="217"/>
+      <c r="P9" s="218"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -4469,10 +4469,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="252" t="s">
+      <c r="U9" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V9" s="253"/>
+      <c r="V9" s="289"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -4485,10 +4485,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="252" t="s">
+      <c r="AA9" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB9" s="253"/>
+      <c r="AB9" s="289"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -4511,7 +4511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:35" ht="15.75" thickBot="1">
+    <row r="10" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2">
         <v>5</v>
       </c>
@@ -4531,9 +4531,9 @@
       <c r="G10" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="279"/>
-      <c r="I10" s="280"/>
-      <c r="J10" s="281"/>
+      <c r="H10" s="308"/>
+      <c r="I10" s="309"/>
+      <c r="J10" s="310"/>
       <c r="K10" s="37" t="s">
         <v>47</v>
       </c>
@@ -4541,11 +4541,11 @@
       <c r="M10" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N10" s="256" t="s">
+      <c r="N10" s="216" t="s">
         <v>53</v>
       </c>
-      <c r="O10" s="257"/>
-      <c r="P10" s="258"/>
+      <c r="O10" s="217"/>
+      <c r="P10" s="218"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -4555,10 +4555,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="252" t="s">
+      <c r="U10" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V10" s="253"/>
+      <c r="V10" s="289"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -4571,10 +4571,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="252" t="s">
+      <c r="AA10" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB10" s="253"/>
+      <c r="AB10" s="289"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -4597,7 +4597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:35" ht="15.75" thickBot="1">
+    <row r="11" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2">
         <v>6</v>
       </c>
@@ -4617,9 +4617,9 @@
       <c r="G11" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H11" s="279"/>
-      <c r="I11" s="280"/>
-      <c r="J11" s="281"/>
+      <c r="H11" s="308"/>
+      <c r="I11" s="309"/>
+      <c r="J11" s="310"/>
       <c r="K11" s="37" t="s">
         <v>14</v>
       </c>
@@ -4627,11 +4627,11 @@
       <c r="M11" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N11" s="256" t="s">
+      <c r="N11" s="216" t="s">
         <v>54</v>
       </c>
-      <c r="O11" s="257"/>
-      <c r="P11" s="258"/>
+      <c r="O11" s="217"/>
+      <c r="P11" s="218"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -4641,10 +4641,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="252" t="s">
+      <c r="U11" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V11" s="253"/>
+      <c r="V11" s="289"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -4657,10 +4657,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="252" t="s">
+      <c r="AA11" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB11" s="253"/>
+      <c r="AB11" s="289"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -4683,7 +4683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:35" ht="15.75" thickBot="1">
+    <row r="12" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2">
         <v>7</v>
       </c>
@@ -4703,9 +4703,9 @@
       <c r="G12" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H12" s="279"/>
-      <c r="I12" s="280"/>
-      <c r="J12" s="281"/>
+      <c r="H12" s="308"/>
+      <c r="I12" s="309"/>
+      <c r="J12" s="310"/>
       <c r="K12" s="37" t="s">
         <v>15</v>
       </c>
@@ -4713,11 +4713,11 @@
       <c r="M12" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N12" s="256" t="s">
+      <c r="N12" s="216" t="s">
         <v>55</v>
       </c>
-      <c r="O12" s="257"/>
-      <c r="P12" s="258"/>
+      <c r="O12" s="217"/>
+      <c r="P12" s="218"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -4727,10 +4727,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="252" t="s">
+      <c r="U12" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V12" s="253"/>
+      <c r="V12" s="289"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -4743,10 +4743,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="252" t="s">
+      <c r="AA12" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB12" s="253"/>
+      <c r="AB12" s="289"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -4769,7 +4769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:35" ht="15.75" thickBot="1">
+    <row r="13" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="1">
         <v>8</v>
       </c>
@@ -4789,9 +4789,9 @@
       <c r="G13" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="279"/>
-      <c r="I13" s="280"/>
-      <c r="J13" s="281"/>
+      <c r="H13" s="308"/>
+      <c r="I13" s="309"/>
+      <c r="J13" s="310"/>
       <c r="K13" s="37" t="s">
         <v>16</v>
       </c>
@@ -4799,11 +4799,11 @@
       <c r="M13" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N13" s="256" t="s">
+      <c r="N13" s="216" t="s">
         <v>56</v>
       </c>
-      <c r="O13" s="257"/>
-      <c r="P13" s="258"/>
+      <c r="O13" s="217"/>
+      <c r="P13" s="218"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -4813,10 +4813,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="252" t="s">
+      <c r="U13" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V13" s="253"/>
+      <c r="V13" s="289"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -4829,10 +4829,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="252" t="s">
+      <c r="AA13" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB13" s="253"/>
+      <c r="AB13" s="289"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -4855,7 +4855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:35" ht="15.75" thickBot="1">
+    <row r="14" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2">
         <v>9</v>
       </c>
@@ -4875,9 +4875,9 @@
       <c r="G14" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H14" s="279"/>
-      <c r="I14" s="280"/>
-      <c r="J14" s="281"/>
+      <c r="H14" s="308"/>
+      <c r="I14" s="309"/>
+      <c r="J14" s="310"/>
       <c r="K14" s="37" t="s">
         <v>17</v>
       </c>
@@ -4885,11 +4885,11 @@
       <c r="M14" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N14" s="256" t="s">
+      <c r="N14" s="216" t="s">
         <v>335</v>
       </c>
-      <c r="O14" s="257"/>
-      <c r="P14" s="258"/>
+      <c r="O14" s="217"/>
+      <c r="P14" s="218"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -4899,10 +4899,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="252" t="s">
+      <c r="U14" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V14" s="253"/>
+      <c r="V14" s="289"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -4915,10 +4915,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="252" t="s">
+      <c r="AA14" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB14" s="253"/>
+      <c r="AB14" s="289"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -4941,7 +4941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:35" ht="15.75" thickBot="1">
+    <row r="15" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2">
         <v>10</v>
       </c>
@@ -4961,9 +4961,9 @@
       <c r="G15" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H15" s="279"/>
-      <c r="I15" s="280"/>
-      <c r="J15" s="281"/>
+      <c r="H15" s="308"/>
+      <c r="I15" s="309"/>
+      <c r="J15" s="310"/>
       <c r="K15" s="31" t="s">
         <v>18</v>
       </c>
@@ -4971,11 +4971,11 @@
       <c r="M15" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N15" s="256" t="s">
+      <c r="N15" s="216" t="s">
         <v>336</v>
       </c>
-      <c r="O15" s="257"/>
-      <c r="P15" s="258"/>
+      <c r="O15" s="217"/>
+      <c r="P15" s="218"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -4985,10 +4985,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="252" t="s">
+      <c r="U15" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V15" s="253"/>
+      <c r="V15" s="289"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -5001,10 +5001,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="252" t="s">
+      <c r="AA15" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB15" s="253"/>
+      <c r="AB15" s="289"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -5027,7 +5027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:35" ht="15.75" thickBot="1">
+    <row r="16" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="2">
         <v>11</v>
       </c>
@@ -5041,21 +5041,21 @@
       <c r="E16" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="F16" s="279"/>
-      <c r="G16" s="280"/>
-      <c r="H16" s="280"/>
-      <c r="I16" s="280"/>
-      <c r="J16" s="281"/>
+      <c r="F16" s="308"/>
+      <c r="G16" s="309"/>
+      <c r="H16" s="309"/>
+      <c r="I16" s="309"/>
+      <c r="J16" s="310"/>
       <c r="K16" s="40" t="s">
         <v>48</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="256" t="s">
+      <c r="N16" s="216" t="s">
         <v>337</v>
       </c>
-      <c r="O16" s="257"/>
-      <c r="P16" s="258"/>
+      <c r="O16" s="217"/>
+      <c r="P16" s="218"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -5065,10 +5065,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="252" t="s">
+      <c r="U16" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V16" s="253"/>
+      <c r="V16" s="289"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -5081,10 +5081,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="252" t="s">
+      <c r="AA16" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB16" s="253"/>
+      <c r="AB16" s="289"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -5107,7 +5107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:35" ht="15.75" thickBot="1">
+    <row r="17" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="2">
         <v>12</v>
       </c>
@@ -5122,22 +5122,22 @@
         <v>27</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="286" t="s">
+      <c r="G17" s="315" t="s">
         <v>72</v>
       </c>
-      <c r="H17" s="257"/>
-      <c r="I17" s="257"/>
-      <c r="J17" s="258"/>
+      <c r="H17" s="217"/>
+      <c r="I17" s="217"/>
+      <c r="J17" s="218"/>
       <c r="K17" s="25" t="s">
         <v>19</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="256" t="s">
+      <c r="N17" s="216" t="s">
         <v>60</v>
       </c>
-      <c r="O17" s="257"/>
-      <c r="P17" s="258"/>
+      <c r="O17" s="217"/>
+      <c r="P17" s="218"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -5147,10 +5147,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="252" t="s">
+      <c r="U17" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V17" s="253"/>
+      <c r="V17" s="289"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -5163,10 +5163,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="252" t="s">
+      <c r="AA17" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB17" s="253"/>
+      <c r="AB17" s="289"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -5189,7 +5189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:35" ht="15.75" thickBot="1">
+    <row r="18" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="2">
         <v>13</v>
       </c>
@@ -5204,12 +5204,12 @@
         <v>27</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="286" t="s">
+      <c r="G18" s="315" t="s">
         <v>72</v>
       </c>
-      <c r="H18" s="257"/>
-      <c r="I18" s="257"/>
-      <c r="J18" s="258"/>
+      <c r="H18" s="217"/>
+      <c r="I18" s="217"/>
+      <c r="J18" s="218"/>
       <c r="K18" s="40" t="s">
         <v>20</v>
       </c>
@@ -5217,11 +5217,11 @@
       <c r="M18" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="N18" s="256" t="s">
+      <c r="N18" s="216" t="s">
         <v>57</v>
       </c>
-      <c r="O18" s="257"/>
-      <c r="P18" s="258"/>
+      <c r="O18" s="217"/>
+      <c r="P18" s="218"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -5231,10 +5231,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="252" t="s">
+      <c r="U18" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V18" s="253"/>
+      <c r="V18" s="289"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -5247,10 +5247,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="252" t="s">
+      <c r="AA18" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB18" s="253"/>
+      <c r="AB18" s="289"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -5273,7 +5273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:35" ht="15.75" thickBot="1">
+    <row r="19" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="2">
         <v>14</v>
       </c>
@@ -5286,20 +5286,20 @@
       <c r="F19" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G19" s="279"/>
-      <c r="H19" s="280"/>
-      <c r="I19" s="280"/>
-      <c r="J19" s="281"/>
+      <c r="G19" s="308"/>
+      <c r="H19" s="309"/>
+      <c r="I19" s="309"/>
+      <c r="J19" s="310"/>
       <c r="K19" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="256" t="s">
+      <c r="N19" s="216" t="s">
         <v>338</v>
       </c>
-      <c r="O19" s="257"/>
-      <c r="P19" s="258"/>
+      <c r="O19" s="217"/>
+      <c r="P19" s="218"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -5309,10 +5309,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="252" t="s">
+      <c r="U19" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V19" s="253"/>
+      <c r="V19" s="289"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -5325,10 +5325,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="252" t="s">
+      <c r="AA19" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB19" s="253"/>
+      <c r="AB19" s="289"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -5351,7 +5351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:35" ht="15.75" thickBot="1">
+    <row r="20" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="2">
         <v>15</v>
       </c>
@@ -5366,20 +5366,20 @@
       <c r="F20" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G20" s="279"/>
-      <c r="H20" s="280"/>
-      <c r="I20" s="280"/>
-      <c r="J20" s="281"/>
+      <c r="G20" s="308"/>
+      <c r="H20" s="309"/>
+      <c r="I20" s="309"/>
+      <c r="J20" s="310"/>
       <c r="K20" s="37" t="s">
         <v>22</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="256" t="s">
+      <c r="N20" s="216" t="s">
         <v>339</v>
       </c>
-      <c r="O20" s="257"/>
-      <c r="P20" s="258"/>
+      <c r="O20" s="217"/>
+      <c r="P20" s="218"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -5389,10 +5389,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="252" t="s">
+      <c r="U20" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V20" s="253"/>
+      <c r="V20" s="289"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -5405,10 +5405,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="252" t="s">
+      <c r="AA20" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB20" s="253"/>
+      <c r="AB20" s="289"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -5431,7 +5431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:35" ht="15.75" thickBot="1">
+    <row r="21" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="2">
         <v>16</v>
       </c>
@@ -5446,20 +5446,20 @@
       <c r="F21" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G21" s="279"/>
-      <c r="H21" s="280"/>
-      <c r="I21" s="280"/>
-      <c r="J21" s="281"/>
+      <c r="G21" s="308"/>
+      <c r="H21" s="309"/>
+      <c r="I21" s="309"/>
+      <c r="J21" s="310"/>
       <c r="K21" s="44" t="s">
         <v>23</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="256" t="s">
+      <c r="N21" s="216" t="s">
         <v>58</v>
       </c>
-      <c r="O21" s="257"/>
-      <c r="P21" s="258"/>
+      <c r="O21" s="217"/>
+      <c r="P21" s="218"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -5469,10 +5469,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="252" t="s">
+      <c r="U21" s="288" t="s">
         <v>88</v>
       </c>
-      <c r="V21" s="253"/>
+      <c r="V21" s="289"/>
       <c r="W21" s="34">
         <v>1</v>
       </c>
@@ -5485,10 +5485,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="252" t="s">
+      <c r="AA21" s="288" t="s">
         <v>90</v>
       </c>
-      <c r="AB21" s="253"/>
+      <c r="AB21" s="289"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -5511,7 +5511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:35" ht="15.75" thickBot="1">
+    <row r="22" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="2">
         <v>17</v>
       </c>
@@ -5522,22 +5522,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="285"/>
-      <c r="F22" s="280"/>
-      <c r="G22" s="280"/>
-      <c r="H22" s="280"/>
-      <c r="I22" s="280"/>
-      <c r="J22" s="281"/>
+      <c r="E22" s="314"/>
+      <c r="F22" s="309"/>
+      <c r="G22" s="309"/>
+      <c r="H22" s="309"/>
+      <c r="I22" s="309"/>
+      <c r="J22" s="310"/>
       <c r="K22" s="40" t="s">
         <v>24</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="256" t="s">
+      <c r="N22" s="216" t="s">
         <v>59</v>
       </c>
-      <c r="O22" s="257"/>
-      <c r="P22" s="258"/>
+      <c r="O22" s="217"/>
+      <c r="P22" s="218"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -5547,10 +5547,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="252" t="s">
+      <c r="U22" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V22" s="253"/>
+      <c r="V22" s="289"/>
       <c r="W22" s="34">
         <v>1</v>
       </c>
@@ -5563,10 +5563,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="252" t="s">
+      <c r="AA22" s="288" t="s">
         <v>88</v>
       </c>
-      <c r="AB22" s="253"/>
+      <c r="AB22" s="289"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -5589,7 +5589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:35" ht="15.75" thickBot="1">
+    <row r="23" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="2">
         <v>18</v>
       </c>
@@ -5606,22 +5606,22 @@
       <c r="F23" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G23" s="286" t="s">
+      <c r="G23" s="315" t="s">
         <v>73</v>
       </c>
-      <c r="H23" s="257"/>
-      <c r="I23" s="257"/>
-      <c r="J23" s="258"/>
+      <c r="H23" s="217"/>
+      <c r="I23" s="217"/>
+      <c r="J23" s="218"/>
       <c r="K23" s="44" t="s">
         <v>25</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="256" t="s">
+      <c r="N23" s="216" t="s">
         <v>78</v>
       </c>
-      <c r="O23" s="257"/>
-      <c r="P23" s="258"/>
+      <c r="O23" s="217"/>
+      <c r="P23" s="218"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -5631,10 +5631,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="252" t="s">
+      <c r="U23" s="288" t="s">
         <v>89</v>
       </c>
-      <c r="V23" s="253"/>
+      <c r="V23" s="289"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -5647,10 +5647,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="252" t="s">
+      <c r="AA23" s="288" t="s">
         <v>88</v>
       </c>
-      <c r="AB23" s="253"/>
+      <c r="AB23" s="289"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -5673,7 +5673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:35" ht="15.75" thickBot="1">
+    <row r="24" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="2">
         <v>19</v>
       </c>
@@ -5690,22 +5690,22 @@
       <c r="F24" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G24" s="286" t="s">
+      <c r="G24" s="315" t="s">
         <v>73</v>
       </c>
-      <c r="H24" s="257"/>
-      <c r="I24" s="257"/>
-      <c r="J24" s="258"/>
+      <c r="H24" s="217"/>
+      <c r="I24" s="217"/>
+      <c r="J24" s="218"/>
       <c r="K24" s="31" t="s">
         <v>26</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="256" t="s">
+      <c r="N24" s="216" t="s">
         <v>77</v>
       </c>
-      <c r="O24" s="257"/>
-      <c r="P24" s="258"/>
+      <c r="O24" s="217"/>
+      <c r="P24" s="218"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -5715,10 +5715,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="252" t="s">
+      <c r="U24" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V24" s="253"/>
+      <c r="V24" s="289"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -5731,10 +5731,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="252" t="s">
+      <c r="AA24" s="288" t="s">
         <v>90</v>
       </c>
-      <c r="AB24" s="253"/>
+      <c r="AB24" s="289"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -5757,7 +5757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:35" ht="15.75" thickBot="1">
+    <row r="25" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="2">
         <v>20</v>
       </c>
@@ -5772,10 +5772,10 @@
       <c r="F25" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="G25" s="279"/>
-      <c r="H25" s="280"/>
-      <c r="I25" s="280"/>
-      <c r="J25" s="281"/>
+      <c r="G25" s="308"/>
+      <c r="H25" s="309"/>
+      <c r="I25" s="309"/>
+      <c r="J25" s="310"/>
       <c r="K25" s="49" t="s">
         <v>38</v>
       </c>
@@ -5783,11 +5783,11 @@
         <v>133</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="256" t="s">
+      <c r="N25" s="216" t="s">
         <v>40</v>
       </c>
-      <c r="O25" s="257"/>
-      <c r="P25" s="258"/>
+      <c r="O25" s="217"/>
+      <c r="P25" s="218"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -5797,10 +5797,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="252" t="s">
+      <c r="U25" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V25" s="253"/>
+      <c r="V25" s="289"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -5813,10 +5813,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="252" t="s">
+      <c r="AA25" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB25" s="253"/>
+      <c r="AB25" s="289"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -5839,7 +5839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:35" ht="15.75" thickBot="1">
+    <row r="26" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="2">
         <v>21</v>
       </c>
@@ -5854,10 +5854,10 @@
       <c r="F26" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="G26" s="279"/>
-      <c r="H26" s="280"/>
-      <c r="I26" s="280"/>
-      <c r="J26" s="281"/>
+      <c r="G26" s="308"/>
+      <c r="H26" s="309"/>
+      <c r="I26" s="309"/>
+      <c r="J26" s="310"/>
       <c r="K26" s="31" t="s">
         <v>39</v>
       </c>
@@ -5865,11 +5865,11 @@
         <v>133</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="256" t="s">
+      <c r="N26" s="216" t="s">
         <v>41</v>
       </c>
-      <c r="O26" s="257"/>
-      <c r="P26" s="258"/>
+      <c r="O26" s="217"/>
+      <c r="P26" s="218"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -5879,10 +5879,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="252" t="s">
+      <c r="U26" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V26" s="253"/>
+      <c r="V26" s="289"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -5895,10 +5895,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="252" t="s">
+      <c r="AA26" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB26" s="253"/>
+      <c r="AB26" s="289"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -5921,7 +5921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:35" ht="15.75" thickBot="1">
+    <row r="27" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="3">
         <v>22</v>
       </c>
@@ -5930,22 +5930,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="285"/>
-      <c r="F27" s="280"/>
-      <c r="G27" s="280"/>
-      <c r="H27" s="280"/>
-      <c r="I27" s="280"/>
-      <c r="J27" s="281"/>
+      <c r="E27" s="314"/>
+      <c r="F27" s="309"/>
+      <c r="G27" s="309"/>
+      <c r="H27" s="309"/>
+      <c r="I27" s="309"/>
+      <c r="J27" s="310"/>
       <c r="K27" s="25" t="s">
         <v>43</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="256" t="s">
+      <c r="N27" s="216" t="s">
         <v>45</v>
       </c>
-      <c r="O27" s="257"/>
-      <c r="P27" s="258"/>
+      <c r="O27" s="217"/>
+      <c r="P27" s="218"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -5955,10 +5955,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="252" t="s">
+      <c r="U27" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="V27" s="253"/>
+      <c r="V27" s="289"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -5971,10 +5971,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="252" t="s">
+      <c r="AA27" s="288" t="s">
         <v>69</v>
       </c>
-      <c r="AB27" s="253"/>
+      <c r="AB27" s="289"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -5997,7 +5997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:35" ht="15.75" thickBot="1">
+    <row r="28" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="4">
         <v>23</v>
       </c>
@@ -6006,12 +6006,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="282"/>
-      <c r="F28" s="283"/>
-      <c r="G28" s="283"/>
-      <c r="H28" s="283"/>
-      <c r="I28" s="283"/>
-      <c r="J28" s="284"/>
+      <c r="E28" s="311"/>
+      <c r="F28" s="312"/>
+      <c r="G28" s="312"/>
+      <c r="H28" s="312"/>
+      <c r="I28" s="312"/>
+      <c r="J28" s="313"/>
       <c r="K28" s="52" t="s">
         <v>44</v>
       </c>
@@ -6019,11 +6019,11 @@
         <v>133</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="276" t="s">
+      <c r="N28" s="213" t="s">
         <v>340</v>
       </c>
-      <c r="O28" s="277"/>
-      <c r="P28" s="278"/>
+      <c r="O28" s="214"/>
+      <c r="P28" s="215"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -6033,10 +6033,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="254" t="s">
+      <c r="U28" s="290" t="s">
         <v>69</v>
       </c>
-      <c r="V28" s="255"/>
+      <c r="V28" s="291"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -6049,10 +6049,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="254" t="s">
+      <c r="AA28" s="290" t="s">
         <v>69</v>
       </c>
-      <c r="AB28" s="255"/>
+      <c r="AB28" s="291"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -6075,8 +6075,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:35" ht="15.75" thickBot="1"/>
-    <row r="30" spans="2:35" ht="21.75" customHeight="1" thickBot="1">
+    <row r="29" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="2:35" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="66" t="s">
         <v>80</v>
       </c>
@@ -6129,20 +6129,20 @@
       <c r="S30" s="75" t="s">
         <v>134</v>
       </c>
-      <c r="T30" s="298" t="s">
+      <c r="T30" s="327" t="s">
         <v>135</v>
       </c>
-      <c r="U30" s="298"/>
-      <c r="V30" s="298"/>
-      <c r="W30" s="298"/>
-      <c r="X30" s="298"/>
-      <c r="Y30" s="298"/>
-      <c r="Z30" s="298"/>
-      <c r="AA30" s="298"/>
-      <c r="AB30" s="298"/>
-      <c r="AC30" s="267"/>
-    </row>
-    <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
+      <c r="U30" s="327"/>
+      <c r="V30" s="327"/>
+      <c r="W30" s="327"/>
+      <c r="X30" s="327"/>
+      <c r="Y30" s="327"/>
+      <c r="Z30" s="327"/>
+      <c r="AA30" s="327"/>
+      <c r="AB30" s="327"/>
+      <c r="AC30" s="300"/>
+    </row>
+    <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="67" t="s">
         <v>68</v>
       </c>
@@ -6181,20 +6181,20 @@
       <c r="S31" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="T31" s="230" t="s">
+      <c r="T31" s="219" t="s">
         <v>140</v>
       </c>
-      <c r="U31" s="272"/>
-      <c r="V31" s="272"/>
-      <c r="W31" s="272"/>
-      <c r="X31" s="272"/>
-      <c r="Y31" s="272"/>
-      <c r="Z31" s="272"/>
-      <c r="AA31" s="272"/>
-      <c r="AB31" s="272"/>
-      <c r="AC31" s="231"/>
-    </row>
-    <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
+      <c r="U31" s="220"/>
+      <c r="V31" s="220"/>
+      <c r="W31" s="220"/>
+      <c r="X31" s="220"/>
+      <c r="Y31" s="220"/>
+      <c r="Z31" s="220"/>
+      <c r="AA31" s="220"/>
+      <c r="AB31" s="220"/>
+      <c r="AC31" s="221"/>
+    </row>
+    <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="4" t="s">
         <v>71</v>
       </c>
@@ -6216,20 +6216,20 @@
       <c r="S32" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="T32" s="256" t="s">
+      <c r="T32" s="216" t="s">
         <v>141</v>
       </c>
-      <c r="U32" s="257"/>
-      <c r="V32" s="257"/>
-      <c r="W32" s="257"/>
-      <c r="X32" s="257"/>
-      <c r="Y32" s="257"/>
-      <c r="Z32" s="257"/>
-      <c r="AA32" s="257"/>
-      <c r="AB32" s="257"/>
-      <c r="AC32" s="258"/>
-    </row>
-    <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
+      <c r="U32" s="217"/>
+      <c r="V32" s="217"/>
+      <c r="W32" s="217"/>
+      <c r="X32" s="217"/>
+      <c r="Y32" s="217"/>
+      <c r="Z32" s="217"/>
+      <c r="AA32" s="217"/>
+      <c r="AB32" s="217"/>
+      <c r="AC32" s="218"/>
+    </row>
+    <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H33" s="84" t="s">
         <v>167</v>
       </c>
@@ -6263,31 +6263,31 @@
       <c r="S33" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="T33" s="256" t="s">
+      <c r="T33" s="216" t="s">
         <v>142</v>
       </c>
-      <c r="U33" s="257"/>
-      <c r="V33" s="257"/>
-      <c r="W33" s="257"/>
-      <c r="X33" s="257"/>
-      <c r="Y33" s="257"/>
-      <c r="Z33" s="257"/>
-      <c r="AA33" s="257"/>
-      <c r="AB33" s="257"/>
-      <c r="AC33" s="258"/>
-    </row>
-    <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B34" s="247" t="s">
+      <c r="U33" s="217"/>
+      <c r="V33" s="217"/>
+      <c r="W33" s="217"/>
+      <c r="X33" s="217"/>
+      <c r="Y33" s="217"/>
+      <c r="Z33" s="217"/>
+      <c r="AA33" s="217"/>
+      <c r="AB33" s="217"/>
+      <c r="AC33" s="218"/>
+    </row>
+    <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="286" t="s">
         <v>95</v>
       </c>
-      <c r="C34" s="245" t="s">
+      <c r="C34" s="284" t="s">
         <v>101</v>
       </c>
-      <c r="D34" s="246"/>
-      <c r="E34" s="245" t="s">
+      <c r="D34" s="285"/>
+      <c r="E34" s="284" t="s">
         <v>102</v>
       </c>
-      <c r="F34" s="246"/>
+      <c r="F34" s="285"/>
       <c r="H34" s="77" t="s">
         <v>61</v>
       </c>
@@ -6315,21 +6315,21 @@
       <c r="S34" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T34" s="256" t="s">
+      <c r="T34" s="216" t="s">
         <v>143</v>
       </c>
-      <c r="U34" s="257"/>
-      <c r="V34" s="257"/>
-      <c r="W34" s="257"/>
-      <c r="X34" s="257"/>
-      <c r="Y34" s="257"/>
-      <c r="Z34" s="257"/>
-      <c r="AA34" s="257"/>
-      <c r="AB34" s="257"/>
-      <c r="AC34" s="258"/>
-    </row>
-    <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B35" s="248"/>
+      <c r="U34" s="217"/>
+      <c r="V34" s="217"/>
+      <c r="W34" s="217"/>
+      <c r="X34" s="217"/>
+      <c r="Y34" s="217"/>
+      <c r="Z34" s="217"/>
+      <c r="AA34" s="217"/>
+      <c r="AB34" s="217"/>
+      <c r="AC34" s="218"/>
+    </row>
+    <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="287"/>
       <c r="C35" s="64" t="s">
         <v>91</v>
       </c>
@@ -6348,20 +6348,20 @@
       <c r="S35" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="T35" s="256" t="s">
+      <c r="T35" s="216" t="s">
         <v>144</v>
       </c>
-      <c r="U35" s="257"/>
-      <c r="V35" s="257"/>
-      <c r="W35" s="257"/>
-      <c r="X35" s="257"/>
-      <c r="Y35" s="257"/>
-      <c r="Z35" s="257"/>
-      <c r="AA35" s="257"/>
-      <c r="AB35" s="257"/>
-      <c r="AC35" s="258"/>
-    </row>
-    <row r="36" spans="2:29" ht="36" customHeight="1" thickBot="1">
+      <c r="U35" s="217"/>
+      <c r="V35" s="217"/>
+      <c r="W35" s="217"/>
+      <c r="X35" s="217"/>
+      <c r="Y35" s="217"/>
+      <c r="Z35" s="217"/>
+      <c r="AA35" s="217"/>
+      <c r="AB35" s="217"/>
+      <c r="AC35" s="218"/>
+    </row>
+    <row r="36" spans="2:29" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="1">
         <v>0</v>
       </c>
@@ -6410,20 +6410,20 @@
       <c r="S36" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T36" s="256" t="s">
+      <c r="T36" s="216" t="s">
         <v>145</v>
       </c>
-      <c r="U36" s="257"/>
-      <c r="V36" s="257"/>
-      <c r="W36" s="257"/>
-      <c r="X36" s="257"/>
-      <c r="Y36" s="257"/>
-      <c r="Z36" s="257"/>
-      <c r="AA36" s="257"/>
-      <c r="AB36" s="257"/>
-      <c r="AC36" s="258"/>
-    </row>
-    <row r="37" spans="2:29" ht="36.75" customHeight="1" thickBot="1">
+      <c r="U36" s="217"/>
+      <c r="V36" s="217"/>
+      <c r="W36" s="217"/>
+      <c r="X36" s="217"/>
+      <c r="Y36" s="217"/>
+      <c r="Z36" s="217"/>
+      <c r="AA36" s="217"/>
+      <c r="AB36" s="217"/>
+      <c r="AC36" s="218"/>
+    </row>
+    <row r="37" spans="2:29" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="2">
         <v>1</v>
       </c>
@@ -6464,20 +6464,20 @@
       <c r="S37" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T37" s="256" t="s">
+      <c r="T37" s="216" t="s">
         <v>165</v>
       </c>
-      <c r="U37" s="257"/>
-      <c r="V37" s="257"/>
-      <c r="W37" s="257"/>
-      <c r="X37" s="257"/>
-      <c r="Y37" s="257"/>
-      <c r="Z37" s="257"/>
-      <c r="AA37" s="257"/>
-      <c r="AB37" s="257"/>
-      <c r="AC37" s="258"/>
-    </row>
-    <row r="38" spans="2:29" ht="15.75" thickBot="1">
+      <c r="U37" s="217"/>
+      <c r="V37" s="217"/>
+      <c r="W37" s="217"/>
+      <c r="X37" s="217"/>
+      <c r="Y37" s="217"/>
+      <c r="Z37" s="217"/>
+      <c r="AA37" s="217"/>
+      <c r="AB37" s="217"/>
+      <c r="AC37" s="218"/>
+    </row>
+    <row r="38" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="2">
         <v>2</v>
       </c>
@@ -6496,23 +6496,23 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="299" t="s">
+      <c r="S38" s="328" t="s">
         <v>68</v>
       </c>
-      <c r="T38" s="301" t="s">
+      <c r="T38" s="330" t="s">
         <v>146</v>
       </c>
-      <c r="U38" s="302"/>
-      <c r="V38" s="302"/>
-      <c r="W38" s="302"/>
-      <c r="X38" s="302"/>
-      <c r="Y38" s="302"/>
-      <c r="Z38" s="302"/>
-      <c r="AA38" s="302"/>
-      <c r="AB38" s="302"/>
-      <c r="AC38" s="303"/>
-    </row>
-    <row r="39" spans="2:29" ht="15" customHeight="1">
+      <c r="U38" s="331"/>
+      <c r="V38" s="331"/>
+      <c r="W38" s="331"/>
+      <c r="X38" s="331"/>
+      <c r="Y38" s="331"/>
+      <c r="Z38" s="331"/>
+      <c r="AA38" s="331"/>
+      <c r="AB38" s="331"/>
+      <c r="AC38" s="332"/>
+    </row>
+    <row r="39" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="2">
         <v>3</v>
       </c>
@@ -6528,28 +6528,28 @@
       <c r="F39" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="G39" s="232" t="s">
+      <c r="G39" s="210" t="s">
         <v>155</v>
       </c>
-      <c r="H39" s="233"/>
-      <c r="I39" s="233"/>
-      <c r="J39" s="234"/>
+      <c r="H39" s="211"/>
+      <c r="I39" s="211"/>
+      <c r="J39" s="212"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="300"/>
-      <c r="T39" s="304"/>
-      <c r="U39" s="305"/>
-      <c r="V39" s="305"/>
-      <c r="W39" s="305"/>
-      <c r="X39" s="305"/>
-      <c r="Y39" s="305"/>
-      <c r="Z39" s="305"/>
-      <c r="AA39" s="305"/>
-      <c r="AB39" s="305"/>
-      <c r="AC39" s="306"/>
-    </row>
-    <row r="40" spans="2:29" ht="37.5" customHeight="1">
+      <c r="S39" s="329"/>
+      <c r="T39" s="333"/>
+      <c r="U39" s="334"/>
+      <c r="V39" s="334"/>
+      <c r="W39" s="334"/>
+      <c r="X39" s="334"/>
+      <c r="Y39" s="334"/>
+      <c r="Z39" s="334"/>
+      <c r="AA39" s="334"/>
+      <c r="AB39" s="334"/>
+      <c r="AC39" s="335"/>
+    </row>
+    <row r="40" spans="2:29" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="2">
         <v>4</v>
       </c>
@@ -6565,30 +6565,30 @@
       <c r="F40" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="G40" s="235"/>
-      <c r="H40" s="236"/>
-      <c r="I40" s="236"/>
-      <c r="J40" s="237"/>
+      <c r="G40" s="274"/>
+      <c r="H40" s="275"/>
+      <c r="I40" s="275"/>
+      <c r="J40" s="276"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T40" s="256" t="s">
+      <c r="T40" s="216" t="s">
         <v>344</v>
       </c>
-      <c r="U40" s="257"/>
-      <c r="V40" s="257"/>
-      <c r="W40" s="257"/>
-      <c r="X40" s="257"/>
-      <c r="Y40" s="257"/>
-      <c r="Z40" s="257"/>
-      <c r="AA40" s="257"/>
-      <c r="AB40" s="257"/>
-      <c r="AC40" s="258"/>
-    </row>
-    <row r="41" spans="2:29" ht="30" customHeight="1">
+      <c r="U40" s="217"/>
+      <c r="V40" s="217"/>
+      <c r="W40" s="217"/>
+      <c r="X40" s="217"/>
+      <c r="Y40" s="217"/>
+      <c r="Z40" s="217"/>
+      <c r="AA40" s="217"/>
+      <c r="AB40" s="217"/>
+      <c r="AC40" s="218"/>
+    </row>
+    <row r="41" spans="2:29" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="2">
         <v>5</v>
       </c>
@@ -6604,30 +6604,30 @@
       <c r="F41" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="G41" s="235"/>
-      <c r="H41" s="236"/>
-      <c r="I41" s="236"/>
-      <c r="J41" s="237"/>
+      <c r="G41" s="274"/>
+      <c r="H41" s="275"/>
+      <c r="I41" s="275"/>
+      <c r="J41" s="276"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="T41" s="256" t="s">
+      <c r="T41" s="216" t="s">
         <v>347</v>
       </c>
-      <c r="U41" s="257"/>
-      <c r="V41" s="257"/>
-      <c r="W41" s="257"/>
-      <c r="X41" s="257"/>
-      <c r="Y41" s="257"/>
-      <c r="Z41" s="257"/>
-      <c r="AA41" s="257"/>
-      <c r="AB41" s="257"/>
-      <c r="AC41" s="258"/>
-    </row>
-    <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
+      <c r="U41" s="217"/>
+      <c r="V41" s="217"/>
+      <c r="W41" s="217"/>
+      <c r="X41" s="217"/>
+      <c r="Y41" s="217"/>
+      <c r="Z41" s="217"/>
+      <c r="AA41" s="217"/>
+      <c r="AB41" s="217"/>
+      <c r="AC41" s="218"/>
+    </row>
+    <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="2">
         <v>6</v>
       </c>
@@ -6643,30 +6643,30 @@
       <c r="F42" s="76" t="s">
         <v>150</v>
       </c>
-      <c r="G42" s="238"/>
-      <c r="H42" s="239"/>
-      <c r="I42" s="239"/>
-      <c r="J42" s="240"/>
+      <c r="G42" s="277"/>
+      <c r="H42" s="278"/>
+      <c r="I42" s="278"/>
+      <c r="J42" s="279"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>138</v>
       </c>
-      <c r="T42" s="256" t="s">
+      <c r="T42" s="216" t="s">
         <v>147</v>
       </c>
-      <c r="U42" s="257"/>
-      <c r="V42" s="257"/>
-      <c r="W42" s="257"/>
-      <c r="X42" s="257"/>
-      <c r="Y42" s="257"/>
-      <c r="Z42" s="257"/>
-      <c r="AA42" s="257"/>
-      <c r="AB42" s="257"/>
-      <c r="AC42" s="258"/>
-    </row>
-    <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
+      <c r="U42" s="217"/>
+      <c r="V42" s="217"/>
+      <c r="W42" s="217"/>
+      <c r="X42" s="217"/>
+      <c r="Y42" s="217"/>
+      <c r="Z42" s="217"/>
+      <c r="AA42" s="217"/>
+      <c r="AB42" s="217"/>
+      <c r="AC42" s="218"/>
+    </row>
+    <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="2">
         <v>7</v>
       </c>
@@ -6682,32 +6682,32 @@
       <c r="F43" s="35" t="s">
         <v>350</v>
       </c>
-      <c r="G43" s="191" t="s">
+      <c r="G43" s="225" t="s">
         <v>351</v>
       </c>
-      <c r="H43" s="227"/>
-      <c r="I43" s="227"/>
-      <c r="J43" s="192"/>
+      <c r="H43" s="226"/>
+      <c r="I43" s="226"/>
+      <c r="J43" s="227"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>139</v>
       </c>
-      <c r="T43" s="256" t="s">
+      <c r="T43" s="216" t="s">
         <v>148</v>
       </c>
-      <c r="U43" s="257"/>
-      <c r="V43" s="257"/>
-      <c r="W43" s="257"/>
-      <c r="X43" s="257"/>
-      <c r="Y43" s="257"/>
-      <c r="Z43" s="257"/>
-      <c r="AA43" s="257"/>
-      <c r="AB43" s="257"/>
-      <c r="AC43" s="258"/>
-    </row>
-    <row r="44" spans="2:29" ht="45.75" thickBot="1">
+      <c r="U43" s="217"/>
+      <c r="V43" s="217"/>
+      <c r="W43" s="217"/>
+      <c r="X43" s="217"/>
+      <c r="Y43" s="217"/>
+      <c r="Z43" s="217"/>
+      <c r="AA43" s="217"/>
+      <c r="AB43" s="217"/>
+      <c r="AC43" s="218"/>
+    </row>
+    <row r="44" spans="2:29" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="2">
         <v>8</v>
       </c>
@@ -6726,23 +6726,23 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="299" t="s">
+      <c r="S44" s="328" t="s">
         <v>71</v>
       </c>
-      <c r="T44" s="301" t="s">
+      <c r="T44" s="330" t="s">
         <v>353</v>
       </c>
-      <c r="U44" s="302"/>
-      <c r="V44" s="302"/>
-      <c r="W44" s="302"/>
-      <c r="X44" s="302"/>
-      <c r="Y44" s="302"/>
-      <c r="Z44" s="302"/>
-      <c r="AA44" s="302"/>
-      <c r="AB44" s="302"/>
-      <c r="AC44" s="303"/>
-    </row>
-    <row r="45" spans="2:29" ht="30.75" customHeight="1">
+      <c r="U44" s="331"/>
+      <c r="V44" s="331"/>
+      <c r="W44" s="331"/>
+      <c r="X44" s="331"/>
+      <c r="Y44" s="331"/>
+      <c r="Z44" s="331"/>
+      <c r="AA44" s="331"/>
+      <c r="AB44" s="331"/>
+      <c r="AC44" s="332"/>
+    </row>
+    <row r="45" spans="2:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="2">
         <v>9</v>
       </c>
@@ -6758,28 +6758,28 @@
       <c r="F45" s="35" t="s">
         <v>125</v>
       </c>
-      <c r="G45" s="232" t="s">
+      <c r="G45" s="210" t="s">
         <v>154</v>
       </c>
-      <c r="H45" s="233"/>
-      <c r="I45" s="233"/>
-      <c r="J45" s="234"/>
+      <c r="H45" s="211"/>
+      <c r="I45" s="211"/>
+      <c r="J45" s="212"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="300"/>
-      <c r="T45" s="304"/>
-      <c r="U45" s="305"/>
-      <c r="V45" s="305"/>
-      <c r="W45" s="305"/>
-      <c r="X45" s="305"/>
-      <c r="Y45" s="305"/>
-      <c r="Z45" s="305"/>
-      <c r="AA45" s="305"/>
-      <c r="AB45" s="305"/>
-      <c r="AC45" s="306"/>
-    </row>
-    <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
+      <c r="S45" s="329"/>
+      <c r="T45" s="333"/>
+      <c r="U45" s="334"/>
+      <c r="V45" s="334"/>
+      <c r="W45" s="334"/>
+      <c r="X45" s="334"/>
+      <c r="Y45" s="334"/>
+      <c r="Z45" s="334"/>
+      <c r="AA45" s="334"/>
+      <c r="AB45" s="334"/>
+      <c r="AC45" s="335"/>
+    </row>
+    <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B46" s="2">
         <v>10</v>
       </c>
@@ -6795,30 +6795,30 @@
       <c r="F46" s="35" t="s">
         <v>128</v>
       </c>
-      <c r="G46" s="238"/>
-      <c r="H46" s="239"/>
-      <c r="I46" s="239"/>
-      <c r="J46" s="240"/>
+      <c r="G46" s="277"/>
+      <c r="H46" s="278"/>
+      <c r="I46" s="278"/>
+      <c r="J46" s="279"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>129</v>
       </c>
-      <c r="T46" s="276" t="s">
+      <c r="T46" s="213" t="s">
         <v>149</v>
       </c>
-      <c r="U46" s="277"/>
-      <c r="V46" s="277"/>
-      <c r="W46" s="277"/>
-      <c r="X46" s="277"/>
-      <c r="Y46" s="277"/>
-      <c r="Z46" s="277"/>
-      <c r="AA46" s="277"/>
-      <c r="AB46" s="277"/>
-      <c r="AC46" s="278"/>
-    </row>
-    <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
+      <c r="U46" s="214"/>
+      <c r="V46" s="214"/>
+      <c r="W46" s="214"/>
+      <c r="X46" s="214"/>
+      <c r="Y46" s="214"/>
+      <c r="Z46" s="214"/>
+      <c r="AA46" s="214"/>
+      <c r="AB46" s="214"/>
+      <c r="AC46" s="215"/>
+    </row>
+    <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="2">
         <v>11</v>
       </c>
@@ -6834,14 +6834,14 @@
       <c r="F47" s="35" t="s">
         <v>131</v>
       </c>
-      <c r="G47" s="227" t="s">
+      <c r="G47" s="226" t="s">
         <v>355</v>
       </c>
-      <c r="H47" s="227"/>
-      <c r="I47" s="227"/>
-      <c r="J47" s="192"/>
-    </row>
-    <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
+      <c r="H47" s="226"/>
+      <c r="I47" s="226"/>
+      <c r="J47" s="227"/>
+    </row>
+    <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B48" s="2">
         <v>12</v>
       </c>
@@ -6884,13 +6884,13 @@
       <c r="Z48" s="72">
         <v>0</v>
       </c>
-      <c r="AA48" s="185" t="s">
+      <c r="AA48" s="236" t="s">
         <v>357</v>
       </c>
-      <c r="AB48" s="186"/>
-      <c r="AC48" s="187"/>
-    </row>
-    <row r="49" spans="2:29" ht="35.25" customHeight="1" thickBot="1">
+      <c r="AB48" s="237"/>
+      <c r="AC48" s="238"/>
+    </row>
+    <row r="49" spans="2:29" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B49" s="2">
         <v>13</v>
       </c>
@@ -6906,12 +6906,12 @@
       <c r="F49" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="G49" s="232" t="s">
+      <c r="G49" s="210" t="s">
         <v>359</v>
       </c>
-      <c r="H49" s="233"/>
-      <c r="I49" s="233"/>
-      <c r="J49" s="234"/>
+      <c r="H49" s="211"/>
+      <c r="I49" s="211"/>
+      <c r="J49" s="212"/>
       <c r="R49" s="77" t="s">
         <v>61</v>
       </c>
@@ -6927,11 +6927,11 @@
       <c r="Z49" s="80" t="s">
         <v>319</v>
       </c>
-      <c r="AA49" s="188"/>
-      <c r="AB49" s="189"/>
-      <c r="AC49" s="190"/>
-    </row>
-    <row r="50" spans="2:29" ht="30" customHeight="1" thickBot="1">
+      <c r="AA49" s="239"/>
+      <c r="AB49" s="240"/>
+      <c r="AC49" s="241"/>
+    </row>
+    <row r="50" spans="2:29" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B50" s="2">
         <v>14</v>
       </c>
@@ -6947,12 +6947,12 @@
       <c r="F50" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="G50" s="235"/>
-      <c r="H50" s="236"/>
-      <c r="I50" s="236"/>
-      <c r="J50" s="237"/>
-    </row>
-    <row r="51" spans="2:29" ht="20.25" customHeight="1" thickBot="1">
+      <c r="G50" s="274"/>
+      <c r="H50" s="275"/>
+      <c r="I50" s="275"/>
+      <c r="J50" s="276"/>
+    </row>
+    <row r="51" spans="2:29" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" s="4">
         <v>15</v>
       </c>
@@ -6968,425 +6968,425 @@
       <c r="F51" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="G51" s="238"/>
-      <c r="H51" s="239"/>
-      <c r="I51" s="239"/>
-      <c r="J51" s="240"/>
-      <c r="R51" s="205" t="s">
+      <c r="G51" s="277"/>
+      <c r="H51" s="278"/>
+      <c r="I51" s="278"/>
+      <c r="J51" s="279"/>
+      <c r="R51" s="254" t="s">
         <v>322</v>
       </c>
-      <c r="S51" s="207" t="s">
+      <c r="S51" s="256" t="s">
         <v>158</v>
       </c>
-      <c r="T51" s="209" t="s">
+      <c r="T51" s="258" t="s">
         <v>157</v>
       </c>
-      <c r="U51" s="209"/>
-      <c r="V51" s="210"/>
-    </row>
-    <row r="52" spans="2:29" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B52" s="249" t="s">
+      <c r="U51" s="258"/>
+      <c r="V51" s="259"/>
+    </row>
+    <row r="52" spans="2:29" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="228" t="s">
         <v>360</v>
       </c>
-      <c r="C52" s="250"/>
-      <c r="D52" s="250"/>
-      <c r="E52" s="250"/>
-      <c r="F52" s="251"/>
-      <c r="R52" s="206"/>
-      <c r="S52" s="208"/>
-      <c r="T52" s="211"/>
-      <c r="U52" s="211"/>
-      <c r="V52" s="212"/>
-    </row>
-    <row r="53" spans="2:29" ht="48" customHeight="1" thickBot="1">
+      <c r="C52" s="229"/>
+      <c r="D52" s="229"/>
+      <c r="E52" s="229"/>
+      <c r="F52" s="230"/>
+      <c r="R52" s="255"/>
+      <c r="S52" s="257"/>
+      <c r="T52" s="260"/>
+      <c r="U52" s="260"/>
+      <c r="V52" s="261"/>
+    </row>
+    <row r="53" spans="2:29" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="R53" s="182" t="s">
         <v>211</v>
       </c>
       <c r="S53" s="183" t="s">
         <v>323</v>
       </c>
-      <c r="T53" s="200" t="s">
+      <c r="T53" s="249" t="s">
         <v>361</v>
       </c>
-      <c r="U53" s="200"/>
-      <c r="V53" s="201"/>
-    </row>
-    <row r="54" spans="2:29" ht="36.75" customHeight="1">
-      <c r="B54" s="243" t="s">
+      <c r="U53" s="249"/>
+      <c r="V53" s="250"/>
+    </row>
+    <row r="54" spans="2:29" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="282" t="s">
         <v>156</v>
       </c>
-      <c r="C54" s="207" t="s">
+      <c r="C54" s="256" t="s">
         <v>158</v>
       </c>
-      <c r="D54" s="209" t="s">
+      <c r="D54" s="258" t="s">
         <v>157</v>
       </c>
-      <c r="E54" s="210"/>
-      <c r="H54" s="205" t="s">
+      <c r="E54" s="259"/>
+      <c r="H54" s="254" t="s">
         <v>313</v>
       </c>
-      <c r="I54" s="207" t="s">
+      <c r="I54" s="256" t="s">
         <v>158</v>
       </c>
-      <c r="J54" s="193" t="s">
+      <c r="J54" s="242" t="s">
         <v>157</v>
       </c>
-      <c r="K54" s="194"/>
-      <c r="L54" s="195"/>
+      <c r="K54" s="243"/>
+      <c r="L54" s="244"/>
       <c r="R54" s="180" t="s">
         <v>220</v>
       </c>
       <c r="S54" s="178" t="s">
         <v>324</v>
       </c>
-      <c r="T54" s="213" t="s">
+      <c r="T54" s="262" t="s">
         <v>330</v>
       </c>
-      <c r="U54" s="213"/>
-      <c r="V54" s="214"/>
-    </row>
-    <row r="55" spans="2:29" ht="24" customHeight="1" thickBot="1">
-      <c r="B55" s="244"/>
-      <c r="C55" s="242"/>
-      <c r="D55" s="228"/>
-      <c r="E55" s="229"/>
-      <c r="H55" s="241"/>
-      <c r="I55" s="208"/>
-      <c r="J55" s="196"/>
-      <c r="K55" s="197"/>
-      <c r="L55" s="198"/>
+      <c r="U54" s="262"/>
+      <c r="V54" s="263"/>
+    </row>
+    <row r="55" spans="2:29" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B55" s="283"/>
+      <c r="C55" s="281"/>
+      <c r="D55" s="272"/>
+      <c r="E55" s="273"/>
+      <c r="H55" s="280"/>
+      <c r="I55" s="257"/>
+      <c r="J55" s="245"/>
+      <c r="K55" s="246"/>
+      <c r="L55" s="247"/>
       <c r="R55" s="180" t="s">
         <v>206</v>
       </c>
       <c r="S55" s="178" t="s">
         <v>325</v>
       </c>
-      <c r="T55" s="213" t="s">
+      <c r="T55" s="262" t="s">
         <v>362</v>
       </c>
-      <c r="U55" s="213"/>
-      <c r="V55" s="214"/>
-    </row>
-    <row r="56" spans="2:29" ht="60.75" customHeight="1" thickBot="1">
+      <c r="U55" s="262"/>
+      <c r="V55" s="263"/>
+    </row>
+    <row r="56" spans="2:29" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B56" s="81">
         <v>0</v>
       </c>
       <c r="C56" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="D56" s="230" t="s">
+      <c r="D56" s="219" t="s">
         <v>172</v>
       </c>
-      <c r="E56" s="231"/>
+      <c r="E56" s="221"/>
       <c r="H56" s="81" t="s">
         <v>316</v>
       </c>
       <c r="I56" s="45" t="s">
         <v>311</v>
       </c>
-      <c r="J56" s="199" t="s">
+      <c r="J56" s="248" t="s">
         <v>314</v>
       </c>
-      <c r="K56" s="200"/>
-      <c r="L56" s="201"/>
-      <c r="M56" s="191" t="s">
+      <c r="K56" s="249"/>
+      <c r="L56" s="250"/>
+      <c r="M56" s="225" t="s">
         <v>363</v>
       </c>
-      <c r="N56" s="192"/>
+      <c r="N56" s="227"/>
       <c r="R56" s="180" t="s">
         <v>231</v>
       </c>
       <c r="S56" s="178" t="s">
         <v>326</v>
       </c>
-      <c r="T56" s="213" t="s">
+      <c r="T56" s="262" t="s">
         <v>364</v>
       </c>
-      <c r="U56" s="213"/>
-      <c r="V56" s="214"/>
-    </row>
-    <row r="57" spans="2:29" ht="49.5" customHeight="1" thickBot="1">
+      <c r="U56" s="262"/>
+      <c r="V56" s="263"/>
+    </row>
+    <row r="57" spans="2:29" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B57" s="82">
         <v>1</v>
       </c>
       <c r="C57" s="85" t="s">
         <v>309</v>
       </c>
-      <c r="D57" s="224" t="s">
+      <c r="D57" s="269" t="s">
         <v>310</v>
       </c>
-      <c r="E57" s="214"/>
-      <c r="F57" s="191" t="s">
+      <c r="E57" s="263"/>
+      <c r="F57" s="225" t="s">
         <v>365</v>
       </c>
-      <c r="G57" s="192"/>
+      <c r="G57" s="227"/>
       <c r="H57" s="82">
         <v>0</v>
       </c>
       <c r="I57" s="85" t="s">
         <v>315</v>
       </c>
-      <c r="J57" s="202" t="s">
+      <c r="J57" s="251" t="s">
         <v>366</v>
       </c>
-      <c r="K57" s="203"/>
-      <c r="L57" s="204"/>
+      <c r="K57" s="252"/>
+      <c r="L57" s="253"/>
       <c r="R57" s="180" t="s">
         <v>247</v>
       </c>
       <c r="S57" s="36" t="s">
         <v>331</v>
       </c>
-      <c r="T57" s="213" t="s">
+      <c r="T57" s="262" t="s">
         <v>367</v>
       </c>
-      <c r="U57" s="213"/>
-      <c r="V57" s="214"/>
-    </row>
-    <row r="58" spans="2:29" ht="60" customHeight="1">
+      <c r="U57" s="262"/>
+      <c r="V57" s="263"/>
+    </row>
+    <row r="58" spans="2:29" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="82">
         <v>2</v>
       </c>
       <c r="C58" s="85" t="s">
         <v>166</v>
       </c>
-      <c r="D58" s="224" t="s">
+      <c r="D58" s="269" t="s">
         <v>368</v>
       </c>
-      <c r="E58" s="214"/>
+      <c r="E58" s="263"/>
       <c r="H58" s="82">
         <v>1</v>
       </c>
       <c r="I58" s="85" t="s">
         <v>369</v>
       </c>
-      <c r="J58" s="202" t="s">
+      <c r="J58" s="251" t="s">
         <v>370</v>
       </c>
-      <c r="K58" s="203"/>
-      <c r="L58" s="204"/>
+      <c r="K58" s="252"/>
+      <c r="L58" s="253"/>
       <c r="R58" s="180" t="s">
         <v>248</v>
       </c>
       <c r="S58" s="36" t="s">
         <v>327</v>
       </c>
-      <c r="T58" s="213" t="s">
+      <c r="T58" s="262" t="s">
         <v>371</v>
       </c>
-      <c r="U58" s="213"/>
-      <c r="V58" s="214"/>
-    </row>
-    <row r="59" spans="2:29" ht="61.5" customHeight="1">
+      <c r="U58" s="262"/>
+      <c r="V58" s="263"/>
+    </row>
+    <row r="59" spans="2:29" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="82">
         <v>3</v>
       </c>
       <c r="C59" s="85" t="s">
         <v>372</v>
       </c>
-      <c r="D59" s="224" t="s">
+      <c r="D59" s="269" t="s">
         <v>161</v>
       </c>
-      <c r="E59" s="214"/>
+      <c r="E59" s="263"/>
       <c r="H59" s="82">
         <v>2</v>
       </c>
       <c r="I59" s="85" t="s">
         <v>312</v>
       </c>
-      <c r="J59" s="202" t="s">
+      <c r="J59" s="251" t="s">
         <v>373</v>
       </c>
-      <c r="K59" s="203"/>
-      <c r="L59" s="204"/>
+      <c r="K59" s="252"/>
+      <c r="L59" s="253"/>
       <c r="R59" s="180" t="s">
         <v>249</v>
       </c>
       <c r="S59" s="36" t="s">
         <v>328</v>
       </c>
-      <c r="T59" s="213" t="s">
+      <c r="T59" s="262" t="s">
         <v>374</v>
       </c>
-      <c r="U59" s="213"/>
-      <c r="V59" s="214"/>
+      <c r="U59" s="262"/>
+      <c r="V59" s="263"/>
       <c r="X59" s="184"/>
     </row>
-    <row r="60" spans="2:29" ht="45.75" customHeight="1">
+    <row r="60" spans="2:29" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="82">
         <v>4</v>
       </c>
       <c r="C60" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="D60" s="224" t="s">
+      <c r="D60" s="269" t="s">
         <v>162</v>
       </c>
-      <c r="E60" s="214"/>
+      <c r="E60" s="263"/>
       <c r="H60" s="82">
         <v>3</v>
       </c>
       <c r="I60" s="38" t="s">
         <v>317</v>
       </c>
-      <c r="J60" s="202" t="s">
+      <c r="J60" s="251" t="s">
         <v>332</v>
       </c>
-      <c r="K60" s="203"/>
-      <c r="L60" s="204"/>
+      <c r="K60" s="252"/>
+      <c r="L60" s="253"/>
       <c r="R60" s="180" t="s">
         <v>250</v>
       </c>
       <c r="S60" s="178" t="s">
         <v>329</v>
       </c>
-      <c r="T60" s="215" t="s">
+      <c r="T60" s="264" t="s">
         <v>376</v>
       </c>
-      <c r="U60" s="216"/>
-      <c r="V60" s="217"/>
-    </row>
-    <row r="61" spans="2:29" ht="40.5" customHeight="1">
+      <c r="U60" s="265"/>
+      <c r="V60" s="266"/>
+    </row>
+    <row r="61" spans="2:29" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="82">
         <v>5</v>
       </c>
       <c r="C61" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="D61" s="224" t="s">
+      <c r="D61" s="269" t="s">
         <v>163</v>
       </c>
-      <c r="E61" s="214"/>
+      <c r="E61" s="263"/>
       <c r="H61" s="82">
         <v>4</v>
       </c>
       <c r="I61" s="38"/>
-      <c r="J61" s="202"/>
-      <c r="K61" s="203"/>
-      <c r="L61" s="204"/>
+      <c r="J61" s="251"/>
+      <c r="K61" s="252"/>
+      <c r="L61" s="253"/>
       <c r="R61" s="180" t="s">
         <v>251</v>
       </c>
       <c r="S61" s="178" t="s">
         <v>329</v>
       </c>
-      <c r="T61" s="218"/>
-      <c r="U61" s="219"/>
-      <c r="V61" s="220"/>
-    </row>
-    <row r="62" spans="2:29" ht="53.25" customHeight="1">
+      <c r="T61" s="267"/>
+      <c r="U61" s="189"/>
+      <c r="V61" s="190"/>
+    </row>
+    <row r="62" spans="2:29" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="82">
         <v>6</v>
       </c>
       <c r="C62" s="38"/>
-      <c r="D62" s="224"/>
-      <c r="E62" s="214"/>
+      <c r="D62" s="269"/>
+      <c r="E62" s="263"/>
       <c r="H62" s="82">
         <v>5</v>
       </c>
       <c r="I62" s="38"/>
-      <c r="J62" s="202"/>
-      <c r="K62" s="203"/>
-      <c r="L62" s="204"/>
+      <c r="J62" s="251"/>
+      <c r="K62" s="252"/>
+      <c r="L62" s="253"/>
       <c r="R62" s="180" t="s">
         <v>283</v>
       </c>
       <c r="S62" s="178" t="s">
         <v>329</v>
       </c>
-      <c r="T62" s="218"/>
-      <c r="U62" s="219"/>
-      <c r="V62" s="220"/>
-    </row>
-    <row r="63" spans="2:29" ht="36" customHeight="1" thickBot="1">
+      <c r="T62" s="267"/>
+      <c r="U62" s="189"/>
+      <c r="V62" s="190"/>
+    </row>
+    <row r="63" spans="2:29" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B63" s="82">
         <v>7</v>
       </c>
       <c r="C63" s="85"/>
-      <c r="D63" s="224"/>
-      <c r="E63" s="214"/>
+      <c r="D63" s="269"/>
+      <c r="E63" s="263"/>
       <c r="H63" s="82">
         <v>6</v>
       </c>
       <c r="I63" s="85"/>
-      <c r="J63" s="202"/>
-      <c r="K63" s="203"/>
-      <c r="L63" s="204"/>
+      <c r="J63" s="251"/>
+      <c r="K63" s="252"/>
+      <c r="L63" s="253"/>
       <c r="R63" s="181" t="s">
         <v>375</v>
       </c>
       <c r="S63" s="179" t="s">
         <v>329</v>
       </c>
-      <c r="T63" s="221"/>
-      <c r="U63" s="222"/>
-      <c r="V63" s="223"/>
-    </row>
-    <row r="64" spans="2:29" ht="40.5" customHeight="1">
+      <c r="T63" s="268"/>
+      <c r="U63" s="192"/>
+      <c r="V63" s="193"/>
+    </row>
+    <row r="64" spans="2:29" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="82">
         <v>8</v>
       </c>
       <c r="C64" s="85"/>
-      <c r="D64" s="224"/>
-      <c r="E64" s="214"/>
-    </row>
-    <row r="65" spans="2:5">
+      <c r="D64" s="269"/>
+      <c r="E64" s="263"/>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="82">
         <v>9</v>
       </c>
       <c r="C65" s="85"/>
-      <c r="D65" s="224"/>
-      <c r="E65" s="214"/>
-    </row>
-    <row r="66" spans="2:5" ht="30" customHeight="1">
+      <c r="D65" s="269"/>
+      <c r="E65" s="263"/>
+    </row>
+    <row r="66" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="82">
         <v>10</v>
       </c>
       <c r="C66" s="85"/>
-      <c r="D66" s="224"/>
-      <c r="E66" s="214"/>
-    </row>
-    <row r="67" spans="2:5">
+      <c r="D66" s="269"/>
+      <c r="E66" s="263"/>
+    </row>
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" s="82">
         <v>11</v>
       </c>
       <c r="C67" s="85"/>
-      <c r="D67" s="224"/>
-      <c r="E67" s="214"/>
-    </row>
-    <row r="68" spans="2:5">
+      <c r="D67" s="269"/>
+      <c r="E67" s="263"/>
+    </row>
+    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" s="82">
         <v>12</v>
       </c>
       <c r="C68" s="85"/>
-      <c r="D68" s="224"/>
-      <c r="E68" s="214"/>
-    </row>
-    <row r="69" spans="2:5">
+      <c r="D68" s="269"/>
+      <c r="E68" s="263"/>
+    </row>
+    <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69" s="82">
         <v>13</v>
       </c>
       <c r="C69" s="85"/>
-      <c r="D69" s="224"/>
-      <c r="E69" s="214"/>
-    </row>
-    <row r="70" spans="2:5" ht="30" customHeight="1">
+      <c r="D69" s="269"/>
+      <c r="E69" s="263"/>
+    </row>
+    <row r="70" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="82">
         <v>14</v>
       </c>
       <c r="C70" s="85"/>
-      <c r="D70" s="224"/>
-      <c r="E70" s="214"/>
-    </row>
-    <row r="71" spans="2:5" ht="15.75" thickBot="1">
+      <c r="D70" s="269"/>
+      <c r="E70" s="263"/>
+    </row>
+    <row r="71" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B71" s="83">
         <v>15</v>
       </c>
       <c r="C71" s="86"/>
-      <c r="D71" s="225"/>
-      <c r="E71" s="226"/>
-    </row>
-    <row r="75" spans="2:5" ht="72" customHeight="1"/>
+      <c r="D71" s="270"/>
+      <c r="E71" s="271"/>
+    </row>
+    <row r="75" spans="2:5" ht="72" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="183">
     <mergeCell ref="T30:AC30"/>
@@ -7586,13 +7586,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CBBBEA-E421-4197-9F44-CA2E8EC0215F}">
   <dimension ref="B1:AB30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="18.140625" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" customWidth="1"/>
     <col min="7" max="10" width="10.140625" customWidth="1"/>
     <col min="12" max="12" width="10.140625" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
@@ -7608,8 +7608,8 @@
     <col min="26" max="28" width="7.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" ht="15.75" thickBot="1"/>
-    <row r="2" spans="2:28" ht="31.5" customHeight="1" thickBot="1">
+    <row r="1" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:28" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="88" t="s">
         <v>173</v>
       </c>
@@ -7625,37 +7625,37 @@
       <c r="F2" s="102" t="s">
         <v>177</v>
       </c>
-      <c r="G2" s="232" t="s">
+      <c r="G2" s="210" t="s">
         <v>178</v>
       </c>
-      <c r="H2" s="233"/>
-      <c r="I2" s="233"/>
-      <c r="J2" s="234"/>
-      <c r="L2" s="319" t="s">
+      <c r="H2" s="211"/>
+      <c r="I2" s="211"/>
+      <c r="J2" s="212"/>
+      <c r="L2" s="201" t="s">
         <v>296</v>
       </c>
-      <c r="M2" s="320"/>
-      <c r="N2" s="320"/>
-      <c r="O2" s="321"/>
+      <c r="M2" s="202"/>
+      <c r="N2" s="202"/>
+      <c r="O2" s="203"/>
       <c r="P2" s="131"/>
-      <c r="Q2" s="322" t="s">
+      <c r="Q2" s="204" t="s">
         <v>256</v>
       </c>
-      <c r="R2" s="323"/>
-      <c r="S2" s="323"/>
-      <c r="T2" s="324"/>
+      <c r="R2" s="205"/>
+      <c r="S2" s="205"/>
+      <c r="T2" s="206"/>
       <c r="U2" s="131"/>
-      <c r="V2" s="312" t="s">
+      <c r="V2" s="194" t="s">
         <v>279</v>
       </c>
-      <c r="W2" s="313"/>
-      <c r="X2" s="313"/>
-      <c r="Y2" s="313"/>
-      <c r="Z2" s="313"/>
-      <c r="AA2" s="313"/>
-      <c r="AB2" s="314"/>
-    </row>
-    <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
+      <c r="W2" s="195"/>
+      <c r="X2" s="195"/>
+      <c r="Y2" s="195"/>
+      <c r="Z2" s="195"/>
+      <c r="AA2" s="195"/>
+      <c r="AB2" s="196"/>
+    </row>
+    <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="89" t="s">
         <v>240</v>
       </c>
@@ -7675,11 +7675,11 @@
       <c r="G3" s="92" t="s">
         <v>179</v>
       </c>
-      <c r="H3" s="230" t="s">
+      <c r="H3" s="219" t="s">
         <v>183</v>
       </c>
-      <c r="I3" s="272"/>
-      <c r="J3" s="231"/>
+      <c r="I3" s="220"/>
+      <c r="J3" s="221"/>
       <c r="L3" s="143" t="s">
         <v>242</v>
       </c>
@@ -7718,13 +7718,13 @@
       <c r="Y3" s="169" t="s">
         <v>245</v>
       </c>
-      <c r="Z3" s="307" t="s">
+      <c r="Z3" s="185" t="s">
         <v>284</v>
       </c>
-      <c r="AA3" s="308"/>
-      <c r="AB3" s="309"/>
-    </row>
-    <row r="4" spans="2:28" ht="53.25" customHeight="1">
+      <c r="AA3" s="186"/>
+      <c r="AB3" s="187"/>
+    </row>
+    <row r="4" spans="2:28" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="90" t="s">
         <v>192</v>
       </c>
@@ -7744,11 +7744,11 @@
       <c r="G4" s="93" t="s">
         <v>180</v>
       </c>
-      <c r="H4" s="256">
+      <c r="H4" s="216">
         <v>63</v>
       </c>
-      <c r="I4" s="257"/>
-      <c r="J4" s="258"/>
+      <c r="I4" s="217"/>
+      <c r="J4" s="218"/>
       <c r="L4" s="149" t="s">
         <v>211</v>
       </c>
@@ -7787,13 +7787,13 @@
       <c r="Y4" s="136" t="s">
         <v>282</v>
       </c>
-      <c r="Z4" s="310" t="s">
+      <c r="Z4" s="188" t="s">
         <v>285</v>
       </c>
-      <c r="AA4" s="219"/>
-      <c r="AB4" s="220"/>
-    </row>
-    <row r="5" spans="2:28" ht="47.25" customHeight="1">
+      <c r="AA4" s="189"/>
+      <c r="AB4" s="190"/>
+    </row>
+    <row r="5" spans="2:28" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="90" t="s">
         <v>193</v>
       </c>
@@ -7813,11 +7813,11 @@
       <c r="G5" s="93" t="s">
         <v>181</v>
       </c>
-      <c r="H5" s="256">
+      <c r="H5" s="216">
         <v>31</v>
       </c>
-      <c r="I5" s="257"/>
-      <c r="J5" s="258"/>
+      <c r="I5" s="217"/>
+      <c r="J5" s="218"/>
       <c r="L5" s="147" t="s">
         <v>220</v>
       </c>
@@ -7856,11 +7856,11 @@
       <c r="Y5" s="133" t="s">
         <v>259</v>
       </c>
-      <c r="Z5" s="310"/>
-      <c r="AA5" s="219"/>
-      <c r="AB5" s="220"/>
-    </row>
-    <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
+      <c r="Z5" s="188"/>
+      <c r="AA5" s="189"/>
+      <c r="AB5" s="190"/>
+    </row>
+    <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="106" t="s">
         <v>241</v>
       </c>
@@ -7880,11 +7880,11 @@
       <c r="G6" s="94" t="s">
         <v>182</v>
       </c>
-      <c r="H6" s="276">
+      <c r="H6" s="213">
         <v>7</v>
       </c>
-      <c r="I6" s="277"/>
-      <c r="J6" s="278"/>
+      <c r="I6" s="214"/>
+      <c r="J6" s="215"/>
       <c r="L6" s="150" t="s">
         <v>206</v>
       </c>
@@ -7923,11 +7923,11 @@
       <c r="Y6" s="142" t="s">
         <v>281</v>
       </c>
-      <c r="Z6" s="311"/>
-      <c r="AA6" s="222"/>
-      <c r="AB6" s="223"/>
-    </row>
-    <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1">
+      <c r="Z6" s="191"/>
+      <c r="AA6" s="192"/>
+      <c r="AB6" s="193"/>
+    </row>
+    <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="89" t="s">
         <v>185</v>
       </c>
@@ -7947,12 +7947,12 @@
       <c r="G7" s="87" t="s">
         <v>239</v>
       </c>
-      <c r="H7" s="325" t="str">
+      <c r="H7" s="207" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12))</f>
         <v>E3FFF000</v>
       </c>
-      <c r="I7" s="326"/>
-      <c r="J7" s="327"/>
+      <c r="I7" s="208"/>
+      <c r="J7" s="209"/>
       <c r="L7" s="148" t="s">
         <v>231</v>
       </c>
@@ -7980,7 +7980,7 @@
       </c>
       <c r="U7" s="131"/>
     </row>
-    <row r="8" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
+    <row r="8" spans="2:28" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="90" t="s">
         <v>186</v>
       </c>
@@ -8000,18 +8000,18 @@
       <c r="G8" s="87" t="s">
         <v>184</v>
       </c>
-      <c r="H8" s="325" t="str">
+      <c r="H8" s="207" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12)+4095)</f>
         <v>E3FFFFFF</v>
       </c>
-      <c r="I8" s="326"/>
-      <c r="J8" s="327"/>
-      <c r="L8" s="191" t="s">
+      <c r="I8" s="208"/>
+      <c r="J8" s="209"/>
+      <c r="L8" s="225" t="s">
         <v>298</v>
       </c>
-      <c r="M8" s="227"/>
-      <c r="N8" s="227"/>
-      <c r="O8" s="192"/>
+      <c r="M8" s="226"/>
+      <c r="N8" s="226"/>
+      <c r="O8" s="227"/>
       <c r="P8" s="131"/>
       <c r="Q8" s="162" t="s">
         <v>251</v>
@@ -8030,7 +8030,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="9" spans="2:28" ht="65.25" customHeight="1" thickBot="1">
+    <row r="9" spans="2:28" ht="65.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="90" t="s">
         <v>187</v>
       </c>
@@ -8066,7 +8066,7 @@
       </c>
       <c r="U9" s="131"/>
     </row>
-    <row r="10" spans="2:28" ht="28.5" customHeight="1" thickBot="1">
+    <row r="10" spans="2:28" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="90" t="s">
         <v>188</v>
       </c>
@@ -8094,7 +8094,7 @@
       <c r="P10" s="131"/>
       <c r="U10" s="131"/>
     </row>
-    <row r="11" spans="2:28" ht="36.75" customHeight="1" thickBot="1">
+    <row r="11" spans="2:28" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="90" t="s">
         <v>189</v>
       </c>
@@ -8120,15 +8120,15 @@
       <c r="N11" s="131"/>
       <c r="O11" s="131"/>
       <c r="P11" s="131"/>
-      <c r="Q11" s="328" t="s">
+      <c r="Q11" s="222" t="s">
         <v>278</v>
       </c>
-      <c r="R11" s="329"/>
-      <c r="S11" s="329"/>
-      <c r="T11" s="330"/>
+      <c r="R11" s="223"/>
+      <c r="S11" s="223"/>
+      <c r="T11" s="224"/>
       <c r="U11" s="131"/>
     </row>
-    <row r="12" spans="2:28" ht="44.25" customHeight="1" thickBot="1">
+    <row r="12" spans="2:28" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="90" t="s">
         <v>190</v>
       </c>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="U12" s="131"/>
     </row>
-    <row r="13" spans="2:28" ht="51.75" customHeight="1" thickBot="1">
+    <row r="13" spans="2:28" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="91" t="s">
         <v>191</v>
       </c>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="U13" s="131"/>
     </row>
-    <row r="14" spans="2:28" ht="54" customHeight="1">
+    <row r="14" spans="2:28" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G14" s="15"/>
       <c r="H14" s="15"/>
       <c r="I14" s="15"/>
@@ -8232,7 +8232,7 @@
       </c>
       <c r="U14" s="131"/>
     </row>
-    <row r="15" spans="2:28" ht="87.75" customHeight="1" thickBot="1">
+    <row r="15" spans="2:28" ht="87.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
       <c r="D15" s="15"/>
@@ -8261,7 +8261,7 @@
       </c>
       <c r="U15" s="131"/>
     </row>
-    <row r="16" spans="2:28" ht="68.25" customHeight="1" thickBot="1">
+    <row r="16" spans="2:28" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="119" t="s">
         <v>194</v>
       </c>
@@ -8277,12 +8277,12 @@
       <c r="F16" s="122" t="s">
         <v>198</v>
       </c>
-      <c r="G16" s="249" t="s">
+      <c r="G16" s="228" t="s">
         <v>236</v>
       </c>
-      <c r="H16" s="250"/>
-      <c r="I16" s="250"/>
-      <c r="J16" s="251"/>
+      <c r="H16" s="229"/>
+      <c r="I16" s="229"/>
+      <c r="J16" s="230"/>
       <c r="Q16" s="165" t="s">
         <v>272</v>
       </c>
@@ -8296,11 +8296,11 @@
         <v>274</v>
       </c>
     </row>
-    <row r="17" spans="2:20" ht="60.75" customHeight="1" thickBot="1">
-      <c r="B17" s="317" t="s">
+    <row r="17" spans="2:20" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="199" t="s">
         <v>199</v>
       </c>
-      <c r="C17" s="315" t="s">
+      <c r="C17" s="197" t="s">
         <v>200</v>
       </c>
       <c r="D17" s="123" t="s">
@@ -8312,12 +8312,12 @@
       <c r="F17" s="125" t="s">
         <v>202</v>
       </c>
-      <c r="G17" s="331" t="s">
+      <c r="G17" s="231" t="s">
         <v>237</v>
       </c>
-      <c r="H17" s="332"/>
-      <c r="I17" s="332"/>
-      <c r="J17" s="333"/>
+      <c r="H17" s="232"/>
+      <c r="I17" s="232"/>
+      <c r="J17" s="233"/>
       <c r="Q17" s="166" t="s">
         <v>275</v>
       </c>
@@ -8331,9 +8331,9 @@
         <v>277</v>
       </c>
     </row>
-    <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B18" s="334"/>
-      <c r="C18" s="335"/>
+    <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="234"/>
+      <c r="C18" s="235"/>
       <c r="D18" s="110" t="s">
         <v>203</v>
       </c>
@@ -8343,16 +8343,16 @@
       <c r="F18" s="113" t="s">
         <v>205</v>
       </c>
-      <c r="G18" s="325" t="s">
+      <c r="G18" s="207" t="s">
         <v>238</v>
       </c>
-      <c r="H18" s="326"/>
-      <c r="I18" s="326"/>
-      <c r="J18" s="327"/>
-    </row>
-    <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B19" s="318"/>
-      <c r="C19" s="316"/>
+      <c r="H18" s="208"/>
+      <c r="I18" s="208"/>
+      <c r="J18" s="209"/>
+    </row>
+    <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="200"/>
+      <c r="C19" s="198"/>
       <c r="D19" s="115" t="s">
         <v>206</v>
       </c>
@@ -8367,11 +8367,11 @@
       <c r="I19" s="15"/>
       <c r="J19" s="15"/>
     </row>
-    <row r="20" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B20" s="317" t="s">
+    <row r="20" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="199" t="s">
         <v>209</v>
       </c>
-      <c r="C20" s="315" t="s">
+      <c r="C20" s="197" t="s">
         <v>210</v>
       </c>
       <c r="D20" s="123" t="s">
@@ -8388,9 +8388,9 @@
       <c r="I20" s="15"/>
       <c r="J20" s="15"/>
     </row>
-    <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B21" s="318"/>
-      <c r="C21" s="316"/>
+    <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="200"/>
+      <c r="C21" s="198"/>
       <c r="D21" s="115" t="s">
         <v>213</v>
       </c>
@@ -8405,11 +8405,11 @@
       <c r="I21" s="15"/>
       <c r="J21" s="15"/>
     </row>
-    <row r="22" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B22" s="317" t="s">
+    <row r="22" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="199" t="s">
         <v>215</v>
       </c>
-      <c r="C22" s="315" t="s">
+      <c r="C22" s="197" t="s">
         <v>216</v>
       </c>
       <c r="D22" s="123" t="s">
@@ -8426,9 +8426,9 @@
       <c r="I22" s="15"/>
       <c r="J22" s="15"/>
     </row>
-    <row r="23" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B23" s="318"/>
-      <c r="C23" s="316"/>
+    <row r="23" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="200"/>
+      <c r="C23" s="198"/>
       <c r="D23" s="115" t="s">
         <v>209</v>
       </c>
@@ -8443,11 +8443,11 @@
       <c r="I23" s="15"/>
       <c r="J23" s="15"/>
     </row>
-    <row r="24" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B24" s="317" t="s">
+    <row r="24" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="199" t="s">
         <v>220</v>
       </c>
-      <c r="C24" s="315" t="s">
+      <c r="C24" s="197" t="s">
         <v>221</v>
       </c>
       <c r="D24" s="123" t="s">
@@ -8464,9 +8464,9 @@
       <c r="I24" s="15"/>
       <c r="J24" s="15"/>
     </row>
-    <row r="25" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B25" s="318"/>
-      <c r="C25" s="316"/>
+    <row r="25" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="200"/>
+      <c r="C25" s="198"/>
       <c r="D25" s="115" t="s">
         <v>215</v>
       </c>
@@ -8481,7 +8481,7 @@
       <c r="I25" s="15"/>
       <c r="J25" s="15"/>
     </row>
-    <row r="26" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+    <row r="26" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="130" t="s">
         <v>224</v>
       </c>
@@ -8502,11 +8502,11 @@
       <c r="I26" s="15"/>
       <c r="J26" s="15"/>
     </row>
-    <row r="27" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B27" s="317" t="s">
+    <row r="27" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="199" t="s">
         <v>203</v>
       </c>
-      <c r="C27" s="315" t="s">
+      <c r="C27" s="197" t="s">
         <v>227</v>
       </c>
       <c r="D27" s="123" t="s">
@@ -8523,9 +8523,9 @@
       <c r="I27" s="15"/>
       <c r="J27" s="15"/>
     </row>
-    <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B28" s="318"/>
-      <c r="C28" s="316"/>
+    <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="200"/>
+      <c r="C28" s="198"/>
       <c r="D28" s="115" t="s">
         <v>220</v>
       </c>
@@ -8540,11 +8540,11 @@
       <c r="I28" s="15"/>
       <c r="J28" s="15"/>
     </row>
-    <row r="29" spans="2:20" ht="51.75" customHeight="1">
-      <c r="B29" s="317" t="s">
+    <row r="29" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="199" t="s">
         <v>231</v>
       </c>
-      <c r="C29" s="315" t="s">
+      <c r="C29" s="197" t="s">
         <v>232</v>
       </c>
       <c r="D29" s="123" t="s">
@@ -8561,9 +8561,9 @@
       <c r="I29" s="15"/>
       <c r="J29" s="15"/>
     </row>
-    <row r="30" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
-      <c r="B30" s="318"/>
-      <c r="C30" s="316"/>
+    <row r="30" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="200"/>
+      <c r="C30" s="198"/>
       <c r="D30" s="115" t="s">
         <v>224</v>
       </c>

</xml_diff>

<commit_message>
Se creo el programa de enumeración de buses de BIOS. Ademas se integro el ensamblador, y se hizo que el salto de fff0 sea directo a main
</commit_message>
<xml_diff>
--- a/Inst.xlsx
+++ b/Inst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yo\Escritorio\Procesador-32-bits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304592E3-A4AB-4023-8DA7-A3AFABA0F5C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0497493-F73C-49B4-900A-17287FCC50E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="603" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2260,7 +2260,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3366,7 +3366,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="346">
+  <cellXfs count="345">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3974,6 +3974,75 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4028,73 +4097,229 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4124,9 +4349,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4151,24 +4373,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4178,9 +4385,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="75" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4196,211 +4400,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4682,7 +4681,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:AI75"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="15"/>
     <col min="2" max="2" width="19.85546875" style="15" customWidth="1"/>
@@ -4718,64 +4717,64 @@
     <col min="36" max="16384" width="9.140625" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:35" ht="15.75" thickBot="1"/>
-    <row r="2" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B2" s="314" t="s">
+    <row r="1" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="276" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="326" t="s">
+      <c r="C2" s="285" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="327"/>
-      <c r="E2" s="328" t="s">
+      <c r="D2" s="286"/>
+      <c r="E2" s="287" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="328"/>
-      <c r="G2" s="329" t="s">
+      <c r="F2" s="287"/>
+      <c r="G2" s="288" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="328"/>
-      <c r="I2" s="328" t="s">
+      <c r="H2" s="287"/>
+      <c r="I2" s="287" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="328"/>
-      <c r="K2" s="330" t="s">
+      <c r="J2" s="287"/>
+      <c r="K2" s="289" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="328"/>
-      <c r="M2" s="328"/>
-      <c r="N2" s="328"/>
-      <c r="O2" s="328"/>
-      <c r="P2" s="331"/>
-      <c r="R2" s="311" t="s">
+      <c r="L2" s="287"/>
+      <c r="M2" s="287"/>
+      <c r="N2" s="287"/>
+      <c r="O2" s="287"/>
+      <c r="P2" s="290"/>
+      <c r="R2" s="293" t="s">
         <v>61</v>
       </c>
-      <c r="S2" s="309" t="s">
+      <c r="S2" s="245" t="s">
         <v>62</v>
       </c>
-      <c r="T2" s="302" t="s">
+      <c r="T2" s="297" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="303"/>
-      <c r="V2" s="303"/>
-      <c r="W2" s="303"/>
-      <c r="X2" s="303"/>
-      <c r="Y2" s="303"/>
-      <c r="Z2" s="303"/>
-      <c r="AA2" s="303"/>
-      <c r="AB2" s="303" t="s">
+      <c r="U2" s="298"/>
+      <c r="V2" s="298"/>
+      <c r="W2" s="298"/>
+      <c r="X2" s="298"/>
+      <c r="Y2" s="298"/>
+      <c r="Z2" s="298"/>
+      <c r="AA2" s="298"/>
+      <c r="AB2" s="298" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="303"/>
-      <c r="AD2" s="303"/>
-      <c r="AE2" s="303"/>
-      <c r="AF2" s="303"/>
-      <c r="AG2" s="303"/>
-      <c r="AH2" s="303"/>
-      <c r="AI2" s="304"/>
-    </row>
-    <row r="3" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B3" s="315"/>
+      <c r="AC2" s="298"/>
+      <c r="AD2" s="298"/>
+      <c r="AE2" s="298"/>
+      <c r="AF2" s="298"/>
+      <c r="AG2" s="298"/>
+      <c r="AH2" s="298"/>
+      <c r="AI2" s="299"/>
+    </row>
+    <row r="3" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="277"/>
       <c r="C3" s="16" t="s">
         <v>75</v>
       </c>
@@ -4800,21 +4799,21 @@
       <c r="J3" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="293"/>
-      <c r="L3" s="325"/>
-      <c r="M3" s="325"/>
-      <c r="N3" s="325"/>
-      <c r="O3" s="325"/>
-      <c r="P3" s="294"/>
-      <c r="R3" s="312"/>
-      <c r="S3" s="253"/>
+      <c r="K3" s="282"/>
+      <c r="L3" s="283"/>
+      <c r="M3" s="283"/>
+      <c r="N3" s="283"/>
+      <c r="O3" s="283"/>
+      <c r="P3" s="284"/>
+      <c r="R3" s="294"/>
+      <c r="S3" s="291"/>
       <c r="T3" s="18">
         <v>15</v>
       </c>
-      <c r="U3" s="335" t="s">
+      <c r="U3" s="263" t="s">
         <v>79</v>
       </c>
-      <c r="V3" s="335"/>
+      <c r="V3" s="263"/>
       <c r="W3" s="19">
         <v>12</v>
       </c>
@@ -4827,10 +4826,10 @@
       <c r="Z3" s="19">
         <v>9</v>
       </c>
-      <c r="AA3" s="301" t="s">
+      <c r="AA3" s="296" t="s">
         <v>70</v>
       </c>
-      <c r="AB3" s="301"/>
+      <c r="AB3" s="296"/>
       <c r="AC3" s="19">
         <v>6</v>
       </c>
@@ -4853,22 +4852,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:35" ht="15.75" thickBot="1">
-      <c r="B4" s="316"/>
+    <row r="4" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="278"/>
       <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="305" t="s">
+      <c r="E4" s="264" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="242"/>
-      <c r="G4" s="242"/>
-      <c r="H4" s="242"/>
-      <c r="I4" s="242"/>
-      <c r="J4" s="243"/>
+      <c r="F4" s="210"/>
+      <c r="G4" s="210"/>
+      <c r="H4" s="210"/>
+      <c r="I4" s="210"/>
+      <c r="J4" s="211"/>
       <c r="K4" s="5" t="s">
         <v>7</v>
       </c>
@@ -4878,20 +4877,20 @@
       <c r="M4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="305" t="s">
+      <c r="N4" s="264" t="s">
         <v>312</v>
       </c>
-      <c r="O4" s="242"/>
-      <c r="P4" s="243"/>
-      <c r="R4" s="313"/>
-      <c r="S4" s="310"/>
+      <c r="O4" s="210"/>
+      <c r="P4" s="211"/>
+      <c r="R4" s="295"/>
+      <c r="S4" s="292"/>
       <c r="T4" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="U4" s="305" t="s">
+      <c r="U4" s="264" t="s">
         <v>71</v>
       </c>
-      <c r="V4" s="306"/>
+      <c r="V4" s="265"/>
       <c r="W4" s="7" t="s">
         <v>67</v>
       </c>
@@ -4904,10 +4903,10 @@
       <c r="Z4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AA4" s="305" t="s">
+      <c r="AA4" s="264" t="s">
         <v>68</v>
       </c>
-      <c r="AB4" s="306"/>
+      <c r="AB4" s="265"/>
       <c r="AC4" s="7" t="s">
         <v>11</v>
       </c>
@@ -4930,7 +4929,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="2:35" ht="15.75" thickBot="1">
+    <row r="5" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
         <v>0</v>
       </c>
@@ -4939,22 +4938,22 @@
         <f t="shared" ref="D5:D28" si="0">DEC2BIN(B5,5)</f>
         <v>00000</v>
       </c>
-      <c r="E5" s="332"/>
-      <c r="F5" s="333"/>
-      <c r="G5" s="333"/>
-      <c r="H5" s="333"/>
-      <c r="I5" s="333"/>
-      <c r="J5" s="334"/>
+      <c r="E5" s="268"/>
+      <c r="F5" s="269"/>
+      <c r="G5" s="269"/>
+      <c r="H5" s="269"/>
+      <c r="I5" s="269"/>
+      <c r="J5" s="270"/>
       <c r="K5" s="25" t="s">
         <v>9</v>
       </c>
       <c r="L5" s="23"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="232" t="s">
+      <c r="N5" s="223" t="s">
         <v>49</v>
       </c>
-      <c r="O5" s="233"/>
-      <c r="P5" s="234"/>
+      <c r="O5" s="224"/>
+      <c r="P5" s="225"/>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -4964,10 +4963,10 @@
       <c r="T5" s="27">
         <v>0</v>
       </c>
-      <c r="U5" s="307" t="s">
+      <c r="U5" s="266" t="s">
         <v>69</v>
       </c>
-      <c r="V5" s="308"/>
+      <c r="V5" s="267"/>
       <c r="W5" s="28">
         <v>0</v>
       </c>
@@ -4980,10 +4979,10 @@
       <c r="Z5" s="28">
         <v>0</v>
       </c>
-      <c r="AA5" s="307" t="s">
+      <c r="AA5" s="266" t="s">
         <v>69</v>
       </c>
-      <c r="AB5" s="308"/>
+      <c r="AB5" s="267"/>
       <c r="AC5" s="28">
         <v>0</v>
       </c>
@@ -5006,7 +5005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:35" ht="15.75" thickBot="1">
+    <row r="6" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2">
         <v>1</v>
       </c>
@@ -5015,12 +5014,12 @@
         <f t="shared" si="0"/>
         <v>00001</v>
       </c>
-      <c r="E6" s="323"/>
-      <c r="F6" s="318"/>
-      <c r="G6" s="318"/>
-      <c r="H6" s="318"/>
-      <c r="I6" s="318"/>
-      <c r="J6" s="319"/>
+      <c r="E6" s="275"/>
+      <c r="F6" s="272"/>
+      <c r="G6" s="272"/>
+      <c r="H6" s="272"/>
+      <c r="I6" s="272"/>
+      <c r="J6" s="273"/>
       <c r="K6" s="31" t="s">
         <v>10</v>
       </c>
@@ -5028,11 +5027,11 @@
         <v>131</v>
       </c>
       <c r="M6" s="35"/>
-      <c r="N6" s="229" t="s">
+      <c r="N6" s="220" t="s">
         <v>313</v>
       </c>
-      <c r="O6" s="230"/>
-      <c r="P6" s="231"/>
+      <c r="O6" s="221"/>
+      <c r="P6" s="222"/>
       <c r="R6" s="2">
         <v>1</v>
       </c>
@@ -5042,10 +5041,10 @@
       <c r="T6" s="33">
         <v>0</v>
       </c>
-      <c r="U6" s="297" t="s">
+      <c r="U6" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V6" s="298"/>
+      <c r="V6" s="262"/>
       <c r="W6" s="34">
         <v>0</v>
       </c>
@@ -5058,10 +5057,10 @@
       <c r="Z6" s="34">
         <v>0</v>
       </c>
-      <c r="AA6" s="297" t="s">
+      <c r="AA6" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB6" s="298"/>
+      <c r="AB6" s="262"/>
       <c r="AC6" s="34">
         <v>0</v>
       </c>
@@ -5084,7 +5083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:35" ht="15.75" thickBot="1">
+    <row r="7" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2">
         <v>2</v>
       </c>
@@ -5104,9 +5103,9 @@
       <c r="G7" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="317"/>
-      <c r="I7" s="318"/>
-      <c r="J7" s="319"/>
+      <c r="H7" s="271"/>
+      <c r="I7" s="272"/>
+      <c r="J7" s="273"/>
       <c r="K7" s="25" t="s">
         <v>12</v>
       </c>
@@ -5114,11 +5113,11 @@
       <c r="M7" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N7" s="229" t="s">
+      <c r="N7" s="220" t="s">
         <v>50</v>
       </c>
-      <c r="O7" s="230"/>
-      <c r="P7" s="231"/>
+      <c r="O7" s="221"/>
+      <c r="P7" s="222"/>
       <c r="R7" s="2">
         <v>2</v>
       </c>
@@ -5128,10 +5127,10 @@
       <c r="T7" s="33">
         <v>0</v>
       </c>
-      <c r="U7" s="297" t="s">
+      <c r="U7" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V7" s="298"/>
+      <c r="V7" s="262"/>
       <c r="W7" s="34">
         <v>0</v>
       </c>
@@ -5144,10 +5143,10 @@
       <c r="Z7" s="34">
         <v>0</v>
       </c>
-      <c r="AA7" s="297" t="s">
+      <c r="AA7" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB7" s="298"/>
+      <c r="AB7" s="262"/>
       <c r="AC7" s="34">
         <v>0</v>
       </c>
@@ -5170,7 +5169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:35" ht="15.75" thickBot="1">
+    <row r="8" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2">
         <v>3</v>
       </c>
@@ -5190,9 +5189,9 @@
       <c r="G8" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H8" s="317"/>
-      <c r="I8" s="318"/>
-      <c r="J8" s="319"/>
+      <c r="H8" s="271"/>
+      <c r="I8" s="272"/>
+      <c r="J8" s="273"/>
       <c r="K8" s="37" t="s">
         <v>13</v>
       </c>
@@ -5200,11 +5199,11 @@
       <c r="M8" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N8" s="229" t="s">
+      <c r="N8" s="220" t="s">
         <v>51</v>
       </c>
-      <c r="O8" s="230"/>
-      <c r="P8" s="231"/>
+      <c r="O8" s="221"/>
+      <c r="P8" s="222"/>
       <c r="R8" s="2">
         <v>3</v>
       </c>
@@ -5214,10 +5213,10 @@
       <c r="T8" s="33">
         <v>0</v>
       </c>
-      <c r="U8" s="297" t="s">
+      <c r="U8" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V8" s="298"/>
+      <c r="V8" s="262"/>
       <c r="W8" s="34">
         <v>0</v>
       </c>
@@ -5230,10 +5229,10 @@
       <c r="Z8" s="34">
         <v>0</v>
       </c>
-      <c r="AA8" s="297" t="s">
+      <c r="AA8" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB8" s="298"/>
+      <c r="AB8" s="262"/>
       <c r="AC8" s="34">
         <v>0</v>
       </c>
@@ -5256,7 +5255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:35" ht="15.75" thickBot="1">
+    <row r="9" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
         <v>4</v>
       </c>
@@ -5276,9 +5275,9 @@
       <c r="G9" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H9" s="317"/>
-      <c r="I9" s="318"/>
-      <c r="J9" s="319"/>
+      <c r="H9" s="271"/>
+      <c r="I9" s="272"/>
+      <c r="J9" s="273"/>
       <c r="K9" s="37" t="s">
         <v>46</v>
       </c>
@@ -5286,11 +5285,11 @@
       <c r="M9" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N9" s="229" t="s">
+      <c r="N9" s="220" t="s">
         <v>52</v>
       </c>
-      <c r="O9" s="230"/>
-      <c r="P9" s="231"/>
+      <c r="O9" s="221"/>
+      <c r="P9" s="222"/>
       <c r="R9" s="1">
         <v>4</v>
       </c>
@@ -5300,10 +5299,10 @@
       <c r="T9" s="33">
         <v>0</v>
       </c>
-      <c r="U9" s="297" t="s">
+      <c r="U9" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V9" s="298"/>
+      <c r="V9" s="262"/>
       <c r="W9" s="34">
         <v>0</v>
       </c>
@@ -5316,10 +5315,10 @@
       <c r="Z9" s="34">
         <v>0</v>
       </c>
-      <c r="AA9" s="297" t="s">
+      <c r="AA9" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB9" s="298"/>
+      <c r="AB9" s="262"/>
       <c r="AC9" s="34">
         <v>0</v>
       </c>
@@ -5342,7 +5341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:35" ht="15.75" thickBot="1">
+    <row r="10" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2">
         <v>5</v>
       </c>
@@ -5362,9 +5361,9 @@
       <c r="G10" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="317"/>
-      <c r="I10" s="318"/>
-      <c r="J10" s="319"/>
+      <c r="H10" s="271"/>
+      <c r="I10" s="272"/>
+      <c r="J10" s="273"/>
       <c r="K10" s="37" t="s">
         <v>47</v>
       </c>
@@ -5372,11 +5371,11 @@
       <c r="M10" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N10" s="229" t="s">
+      <c r="N10" s="220" t="s">
         <v>53</v>
       </c>
-      <c r="O10" s="230"/>
-      <c r="P10" s="231"/>
+      <c r="O10" s="221"/>
+      <c r="P10" s="222"/>
       <c r="R10" s="2">
         <v>5</v>
       </c>
@@ -5386,10 +5385,10 @@
       <c r="T10" s="33">
         <v>0</v>
       </c>
-      <c r="U10" s="297" t="s">
+      <c r="U10" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V10" s="298"/>
+      <c r="V10" s="262"/>
       <c r="W10" s="34">
         <v>0</v>
       </c>
@@ -5402,10 +5401,10 @@
       <c r="Z10" s="34">
         <v>0</v>
       </c>
-      <c r="AA10" s="297" t="s">
+      <c r="AA10" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB10" s="298"/>
+      <c r="AB10" s="262"/>
       <c r="AC10" s="34">
         <v>0</v>
       </c>
@@ -5428,7 +5427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:35" ht="15.75" thickBot="1">
+    <row r="11" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2">
         <v>6</v>
       </c>
@@ -5448,9 +5447,9 @@
       <c r="G11" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H11" s="317"/>
-      <c r="I11" s="318"/>
-      <c r="J11" s="319"/>
+      <c r="H11" s="271"/>
+      <c r="I11" s="272"/>
+      <c r="J11" s="273"/>
       <c r="K11" s="37" t="s">
         <v>14</v>
       </c>
@@ -5458,11 +5457,11 @@
       <c r="M11" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N11" s="229" t="s">
+      <c r="N11" s="220" t="s">
         <v>54</v>
       </c>
-      <c r="O11" s="230"/>
-      <c r="P11" s="231"/>
+      <c r="O11" s="221"/>
+      <c r="P11" s="222"/>
       <c r="R11" s="2">
         <v>6</v>
       </c>
@@ -5472,10 +5471,10 @@
       <c r="T11" s="33">
         <v>0</v>
       </c>
-      <c r="U11" s="297" t="s">
+      <c r="U11" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V11" s="298"/>
+      <c r="V11" s="262"/>
       <c r="W11" s="34">
         <v>0</v>
       </c>
@@ -5488,10 +5487,10 @@
       <c r="Z11" s="34">
         <v>0</v>
       </c>
-      <c r="AA11" s="297" t="s">
+      <c r="AA11" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB11" s="298"/>
+      <c r="AB11" s="262"/>
       <c r="AC11" s="34">
         <v>0</v>
       </c>
@@ -5514,7 +5513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:35" ht="15.75" thickBot="1">
+    <row r="12" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2">
         <v>7</v>
       </c>
@@ -5534,9 +5533,9 @@
       <c r="G12" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H12" s="317"/>
-      <c r="I12" s="318"/>
-      <c r="J12" s="319"/>
+      <c r="H12" s="271"/>
+      <c r="I12" s="272"/>
+      <c r="J12" s="273"/>
       <c r="K12" s="37" t="s">
         <v>15</v>
       </c>
@@ -5544,11 +5543,11 @@
       <c r="M12" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N12" s="229" t="s">
+      <c r="N12" s="220" t="s">
         <v>55</v>
       </c>
-      <c r="O12" s="230"/>
-      <c r="P12" s="231"/>
+      <c r="O12" s="221"/>
+      <c r="P12" s="222"/>
       <c r="R12" s="2">
         <v>7</v>
       </c>
@@ -5558,10 +5557,10 @@
       <c r="T12" s="33">
         <v>0</v>
       </c>
-      <c r="U12" s="297" t="s">
+      <c r="U12" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V12" s="298"/>
+      <c r="V12" s="262"/>
       <c r="W12" s="34">
         <v>0</v>
       </c>
@@ -5574,10 +5573,10 @@
       <c r="Z12" s="34">
         <v>0</v>
       </c>
-      <c r="AA12" s="297" t="s">
+      <c r="AA12" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB12" s="298"/>
+      <c r="AB12" s="262"/>
       <c r="AC12" s="34">
         <v>0</v>
       </c>
@@ -5600,7 +5599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:35" ht="15.75" thickBot="1">
+    <row r="13" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="1">
         <v>8</v>
       </c>
@@ -5620,9 +5619,9 @@
       <c r="G13" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="317"/>
-      <c r="I13" s="318"/>
-      <c r="J13" s="319"/>
+      <c r="H13" s="271"/>
+      <c r="I13" s="272"/>
+      <c r="J13" s="273"/>
       <c r="K13" s="37" t="s">
         <v>16</v>
       </c>
@@ -5630,11 +5629,11 @@
       <c r="M13" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N13" s="229" t="s">
+      <c r="N13" s="220" t="s">
         <v>56</v>
       </c>
-      <c r="O13" s="230"/>
-      <c r="P13" s="231"/>
+      <c r="O13" s="221"/>
+      <c r="P13" s="222"/>
       <c r="R13" s="1">
         <v>8</v>
       </c>
@@ -5644,10 +5643,10 @@
       <c r="T13" s="33">
         <v>0</v>
       </c>
-      <c r="U13" s="297" t="s">
+      <c r="U13" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V13" s="298"/>
+      <c r="V13" s="262"/>
       <c r="W13" s="34">
         <v>0</v>
       </c>
@@ -5660,10 +5659,10 @@
       <c r="Z13" s="34">
         <v>0</v>
       </c>
-      <c r="AA13" s="297" t="s">
+      <c r="AA13" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB13" s="298"/>
+      <c r="AB13" s="262"/>
       <c r="AC13" s="34">
         <v>0</v>
       </c>
@@ -5686,7 +5685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:35" ht="15.75" thickBot="1">
+    <row r="14" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2">
         <v>9</v>
       </c>
@@ -5706,9 +5705,9 @@
       <c r="G14" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H14" s="317"/>
-      <c r="I14" s="318"/>
-      <c r="J14" s="319"/>
+      <c r="H14" s="271"/>
+      <c r="I14" s="272"/>
+      <c r="J14" s="273"/>
       <c r="K14" s="37" t="s">
         <v>17</v>
       </c>
@@ -5716,11 +5715,11 @@
       <c r="M14" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N14" s="229" t="s">
+      <c r="N14" s="220" t="s">
         <v>314</v>
       </c>
-      <c r="O14" s="230"/>
-      <c r="P14" s="231"/>
+      <c r="O14" s="221"/>
+      <c r="P14" s="222"/>
       <c r="R14" s="2">
         <v>9</v>
       </c>
@@ -5730,10 +5729,10 @@
       <c r="T14" s="33">
         <v>0</v>
       </c>
-      <c r="U14" s="297" t="s">
+      <c r="U14" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V14" s="298"/>
+      <c r="V14" s="262"/>
       <c r="W14" s="34">
         <v>0</v>
       </c>
@@ -5746,10 +5745,10 @@
       <c r="Z14" s="34">
         <v>0</v>
       </c>
-      <c r="AA14" s="297" t="s">
+      <c r="AA14" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB14" s="298"/>
+      <c r="AB14" s="262"/>
       <c r="AC14" s="34">
         <v>0</v>
       </c>
@@ -5772,7 +5771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:35" ht="15.75" thickBot="1">
+    <row r="15" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2">
         <v>10</v>
       </c>
@@ -5792,9 +5791,9 @@
       <c r="G15" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H15" s="317"/>
-      <c r="I15" s="318"/>
-      <c r="J15" s="319"/>
+      <c r="H15" s="271"/>
+      <c r="I15" s="272"/>
+      <c r="J15" s="273"/>
       <c r="K15" s="31" t="s">
         <v>18</v>
       </c>
@@ -5802,11 +5801,11 @@
       <c r="M15" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N15" s="229" t="s">
+      <c r="N15" s="220" t="s">
         <v>315</v>
       </c>
-      <c r="O15" s="230"/>
-      <c r="P15" s="231"/>
+      <c r="O15" s="221"/>
+      <c r="P15" s="222"/>
       <c r="R15" s="2">
         <v>10</v>
       </c>
@@ -5816,10 +5815,10 @@
       <c r="T15" s="33">
         <v>0</v>
       </c>
-      <c r="U15" s="297" t="s">
+      <c r="U15" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V15" s="298"/>
+      <c r="V15" s="262"/>
       <c r="W15" s="34">
         <v>0</v>
       </c>
@@ -5832,10 +5831,10 @@
       <c r="Z15" s="34">
         <v>0</v>
       </c>
-      <c r="AA15" s="297" t="s">
+      <c r="AA15" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB15" s="298"/>
+      <c r="AB15" s="262"/>
       <c r="AC15" s="34">
         <v>0</v>
       </c>
@@ -5858,7 +5857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:35" ht="15.75" thickBot="1">
+    <row r="16" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="2">
         <v>11</v>
       </c>
@@ -5872,21 +5871,21 @@
       <c r="E16" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="F16" s="317"/>
-      <c r="G16" s="318"/>
-      <c r="H16" s="318"/>
-      <c r="I16" s="318"/>
-      <c r="J16" s="319"/>
+      <c r="F16" s="271"/>
+      <c r="G16" s="272"/>
+      <c r="H16" s="272"/>
+      <c r="I16" s="272"/>
+      <c r="J16" s="273"/>
       <c r="K16" s="40" t="s">
         <v>48</v>
       </c>
       <c r="L16" s="43"/>
       <c r="M16" s="35"/>
-      <c r="N16" s="229" t="s">
+      <c r="N16" s="220" t="s">
         <v>316</v>
       </c>
-      <c r="O16" s="230"/>
-      <c r="P16" s="231"/>
+      <c r="O16" s="221"/>
+      <c r="P16" s="222"/>
       <c r="R16" s="2">
         <v>11</v>
       </c>
@@ -5896,10 +5895,10 @@
       <c r="T16" s="33">
         <v>0</v>
       </c>
-      <c r="U16" s="297" t="s">
+      <c r="U16" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V16" s="298"/>
+      <c r="V16" s="262"/>
       <c r="W16" s="34">
         <v>0</v>
       </c>
@@ -5912,10 +5911,10 @@
       <c r="Z16" s="34">
         <v>0</v>
       </c>
-      <c r="AA16" s="297" t="s">
+      <c r="AA16" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB16" s="298"/>
+      <c r="AB16" s="262"/>
       <c r="AC16" s="34">
         <v>0</v>
       </c>
@@ -5938,7 +5937,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:35" ht="15.75" thickBot="1">
+    <row r="17" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="2">
         <v>12</v>
       </c>
@@ -5953,22 +5952,22 @@
         <v>27</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="324" t="s">
+      <c r="G17" s="274" t="s">
         <v>72</v>
       </c>
-      <c r="H17" s="230"/>
-      <c r="I17" s="230"/>
-      <c r="J17" s="231"/>
+      <c r="H17" s="221"/>
+      <c r="I17" s="221"/>
+      <c r="J17" s="222"/>
       <c r="K17" s="25" t="s">
         <v>19</v>
       </c>
       <c r="L17" s="43"/>
       <c r="M17" s="35"/>
-      <c r="N17" s="229" t="s">
+      <c r="N17" s="220" t="s">
         <v>60</v>
       </c>
-      <c r="O17" s="230"/>
-      <c r="P17" s="231"/>
+      <c r="O17" s="221"/>
+      <c r="P17" s="222"/>
       <c r="R17" s="2">
         <v>12</v>
       </c>
@@ -5978,10 +5977,10 @@
       <c r="T17" s="33">
         <v>0</v>
       </c>
-      <c r="U17" s="297" t="s">
+      <c r="U17" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V17" s="298"/>
+      <c r="V17" s="262"/>
       <c r="W17" s="34">
         <v>0</v>
       </c>
@@ -5994,10 +5993,10 @@
       <c r="Z17" s="34">
         <v>0</v>
       </c>
-      <c r="AA17" s="297" t="s">
+      <c r="AA17" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB17" s="298"/>
+      <c r="AB17" s="262"/>
       <c r="AC17" s="34">
         <v>0</v>
       </c>
@@ -6020,7 +6019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:35" ht="15.75" thickBot="1">
+    <row r="18" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="2">
         <v>13</v>
       </c>
@@ -6035,12 +6034,12 @@
         <v>27</v>
       </c>
       <c r="F18" s="42"/>
-      <c r="G18" s="324" t="s">
+      <c r="G18" s="274" t="s">
         <v>72</v>
       </c>
-      <c r="H18" s="230"/>
-      <c r="I18" s="230"/>
-      <c r="J18" s="231"/>
+      <c r="H18" s="221"/>
+      <c r="I18" s="221"/>
+      <c r="J18" s="222"/>
       <c r="K18" s="40" t="s">
         <v>20</v>
       </c>
@@ -6048,11 +6047,11 @@
       <c r="M18" s="55" t="s">
         <v>131</v>
       </c>
-      <c r="N18" s="229" t="s">
+      <c r="N18" s="220" t="s">
         <v>57</v>
       </c>
-      <c r="O18" s="230"/>
-      <c r="P18" s="231"/>
+      <c r="O18" s="221"/>
+      <c r="P18" s="222"/>
       <c r="R18" s="2">
         <v>13</v>
       </c>
@@ -6062,10 +6061,10 @@
       <c r="T18" s="33">
         <v>0</v>
       </c>
-      <c r="U18" s="297" t="s">
+      <c r="U18" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V18" s="298"/>
+      <c r="V18" s="262"/>
       <c r="W18" s="34">
         <v>0</v>
       </c>
@@ -6078,10 +6077,10 @@
       <c r="Z18" s="34">
         <v>0</v>
       </c>
-      <c r="AA18" s="297" t="s">
+      <c r="AA18" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB18" s="298"/>
+      <c r="AB18" s="262"/>
       <c r="AC18" s="34">
         <v>0</v>
       </c>
@@ -6104,7 +6103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:35" ht="15.75" thickBot="1">
+    <row r="19" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="2">
         <v>14</v>
       </c>
@@ -6117,20 +6116,20 @@
       <c r="F19" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G19" s="317"/>
-      <c r="H19" s="318"/>
-      <c r="I19" s="318"/>
-      <c r="J19" s="319"/>
+      <c r="G19" s="271"/>
+      <c r="H19" s="272"/>
+      <c r="I19" s="272"/>
+      <c r="J19" s="273"/>
       <c r="K19" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L19" s="43"/>
       <c r="M19" s="35"/>
-      <c r="N19" s="229" t="s">
+      <c r="N19" s="220" t="s">
         <v>317</v>
       </c>
-      <c r="O19" s="230"/>
-      <c r="P19" s="231"/>
+      <c r="O19" s="221"/>
+      <c r="P19" s="222"/>
       <c r="R19" s="2">
         <v>14</v>
       </c>
@@ -6140,10 +6139,10 @@
       <c r="T19" s="33">
         <v>0</v>
       </c>
-      <c r="U19" s="297" t="s">
+      <c r="U19" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V19" s="298"/>
+      <c r="V19" s="262"/>
       <c r="W19" s="34">
         <v>0</v>
       </c>
@@ -6156,10 +6155,10 @@
       <c r="Z19" s="34">
         <v>0</v>
       </c>
-      <c r="AA19" s="297" t="s">
+      <c r="AA19" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB19" s="298"/>
+      <c r="AB19" s="262"/>
       <c r="AC19" s="34">
         <v>0</v>
       </c>
@@ -6182,7 +6181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:35" ht="15.75" thickBot="1">
+    <row r="20" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="2">
         <v>15</v>
       </c>
@@ -6197,20 +6196,20 @@
       <c r="F20" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G20" s="317"/>
-      <c r="H20" s="318"/>
-      <c r="I20" s="318"/>
-      <c r="J20" s="319"/>
+      <c r="G20" s="271"/>
+      <c r="H20" s="272"/>
+      <c r="I20" s="272"/>
+      <c r="J20" s="273"/>
       <c r="K20" s="37" t="s">
         <v>22</v>
       </c>
       <c r="L20" s="43"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="229" t="s">
+      <c r="N20" s="220" t="s">
         <v>318</v>
       </c>
-      <c r="O20" s="230"/>
-      <c r="P20" s="231"/>
+      <c r="O20" s="221"/>
+      <c r="P20" s="222"/>
       <c r="R20" s="2">
         <v>15</v>
       </c>
@@ -6220,10 +6219,10 @@
       <c r="T20" s="33">
         <v>0</v>
       </c>
-      <c r="U20" s="297" t="s">
+      <c r="U20" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V20" s="298"/>
+      <c r="V20" s="262"/>
       <c r="W20" s="34">
         <v>0</v>
       </c>
@@ -6236,10 +6235,10 @@
       <c r="Z20" s="34">
         <v>0</v>
       </c>
-      <c r="AA20" s="297" t="s">
+      <c r="AA20" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB20" s="298"/>
+      <c r="AB20" s="262"/>
       <c r="AC20" s="34">
         <v>0</v>
       </c>
@@ -6262,7 +6261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:35" ht="15.75" thickBot="1">
+    <row r="21" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="2">
         <v>16</v>
       </c>
@@ -6277,20 +6276,20 @@
       <c r="F21" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G21" s="317"/>
-      <c r="H21" s="318"/>
-      <c r="I21" s="318"/>
-      <c r="J21" s="319"/>
+      <c r="G21" s="271"/>
+      <c r="H21" s="272"/>
+      <c r="I21" s="272"/>
+      <c r="J21" s="273"/>
       <c r="K21" s="44" t="s">
         <v>23</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="229" t="s">
+      <c r="N21" s="220" t="s">
         <v>58</v>
       </c>
-      <c r="O21" s="230"/>
-      <c r="P21" s="231"/>
+      <c r="O21" s="221"/>
+      <c r="P21" s="222"/>
       <c r="R21" s="2">
         <v>16</v>
       </c>
@@ -6300,10 +6299,10 @@
       <c r="T21" s="33">
         <v>0</v>
       </c>
-      <c r="U21" s="297" t="s">
+      <c r="U21" s="261" t="s">
         <v>88</v>
       </c>
-      <c r="V21" s="298"/>
+      <c r="V21" s="262"/>
       <c r="W21" s="34">
         <v>0</v>
       </c>
@@ -6316,10 +6315,10 @@
       <c r="Z21" s="34">
         <v>0</v>
       </c>
-      <c r="AA21" s="297" t="s">
+      <c r="AA21" s="261" t="s">
         <v>90</v>
       </c>
-      <c r="AB21" s="298"/>
+      <c r="AB21" s="262"/>
       <c r="AC21" s="34">
         <v>0</v>
       </c>
@@ -6342,7 +6341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:35" ht="15.75" thickBot="1">
+    <row r="22" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="2">
         <v>17</v>
       </c>
@@ -6353,22 +6352,22 @@
         <f t="shared" si="0"/>
         <v>10001</v>
       </c>
-      <c r="E22" s="323"/>
-      <c r="F22" s="318"/>
-      <c r="G22" s="318"/>
-      <c r="H22" s="318"/>
-      <c r="I22" s="318"/>
-      <c r="J22" s="319"/>
+      <c r="E22" s="275"/>
+      <c r="F22" s="272"/>
+      <c r="G22" s="272"/>
+      <c r="H22" s="272"/>
+      <c r="I22" s="272"/>
+      <c r="J22" s="273"/>
       <c r="K22" s="40" t="s">
         <v>24</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="35"/>
-      <c r="N22" s="229" t="s">
+      <c r="N22" s="220" t="s">
         <v>59</v>
       </c>
-      <c r="O22" s="230"/>
-      <c r="P22" s="231"/>
+      <c r="O22" s="221"/>
+      <c r="P22" s="222"/>
       <c r="R22" s="2">
         <v>17</v>
       </c>
@@ -6378,10 +6377,10 @@
       <c r="T22" s="33">
         <v>0</v>
       </c>
-      <c r="U22" s="297" t="s">
+      <c r="U22" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V22" s="298"/>
+      <c r="V22" s="262"/>
       <c r="W22" s="34">
         <v>0</v>
       </c>
@@ -6394,10 +6393,10 @@
       <c r="Z22" s="34">
         <v>1</v>
       </c>
-      <c r="AA22" s="297" t="s">
+      <c r="AA22" s="261" t="s">
         <v>88</v>
       </c>
-      <c r="AB22" s="298"/>
+      <c r="AB22" s="262"/>
       <c r="AC22" s="34">
         <v>0</v>
       </c>
@@ -6420,7 +6419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:35" ht="15.75" thickBot="1">
+    <row r="23" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="2">
         <v>18</v>
       </c>
@@ -6437,22 +6436,22 @@
       <c r="F23" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G23" s="324" t="s">
+      <c r="G23" s="274" t="s">
         <v>73</v>
       </c>
-      <c r="H23" s="230"/>
-      <c r="I23" s="230"/>
-      <c r="J23" s="231"/>
+      <c r="H23" s="221"/>
+      <c r="I23" s="221"/>
+      <c r="J23" s="222"/>
       <c r="K23" s="44" t="s">
         <v>25</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="35"/>
-      <c r="N23" s="229" t="s">
+      <c r="N23" s="220" t="s">
         <v>78</v>
       </c>
-      <c r="O23" s="230"/>
-      <c r="P23" s="231"/>
+      <c r="O23" s="221"/>
+      <c r="P23" s="222"/>
       <c r="R23" s="2">
         <v>18</v>
       </c>
@@ -6462,10 +6461,10 @@
       <c r="T23" s="33">
         <v>0</v>
       </c>
-      <c r="U23" s="297" t="s">
+      <c r="U23" s="261" t="s">
         <v>89</v>
       </c>
-      <c r="V23" s="298"/>
+      <c r="V23" s="262"/>
       <c r="W23" s="34">
         <v>0</v>
       </c>
@@ -6478,10 +6477,10 @@
       <c r="Z23" s="34">
         <v>0</v>
       </c>
-      <c r="AA23" s="297" t="s">
+      <c r="AA23" s="261" t="s">
         <v>88</v>
       </c>
-      <c r="AB23" s="298"/>
+      <c r="AB23" s="262"/>
       <c r="AC23" s="34">
         <v>0</v>
       </c>
@@ -6504,7 +6503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:35" ht="15.75" thickBot="1">
+    <row r="24" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="2">
         <v>19</v>
       </c>
@@ -6521,22 +6520,22 @@
       <c r="F24" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="G24" s="324" t="s">
+      <c r="G24" s="274" t="s">
         <v>73</v>
       </c>
-      <c r="H24" s="230"/>
-      <c r="I24" s="230"/>
-      <c r="J24" s="231"/>
+      <c r="H24" s="221"/>
+      <c r="I24" s="221"/>
+      <c r="J24" s="222"/>
       <c r="K24" s="31" t="s">
         <v>26</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="56"/>
-      <c r="N24" s="229" t="s">
+      <c r="N24" s="220" t="s">
         <v>77</v>
       </c>
-      <c r="O24" s="230"/>
-      <c r="P24" s="231"/>
+      <c r="O24" s="221"/>
+      <c r="P24" s="222"/>
       <c r="R24" s="2">
         <v>19</v>
       </c>
@@ -6546,10 +6545,10 @@
       <c r="T24" s="33">
         <v>0</v>
       </c>
-      <c r="U24" s="297" t="s">
+      <c r="U24" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V24" s="298"/>
+      <c r="V24" s="262"/>
       <c r="W24" s="34">
         <v>0</v>
       </c>
@@ -6562,10 +6561,10 @@
       <c r="Z24" s="34">
         <v>0</v>
       </c>
-      <c r="AA24" s="297" t="s">
+      <c r="AA24" s="261" t="s">
         <v>90</v>
       </c>
-      <c r="AB24" s="298"/>
+      <c r="AB24" s="262"/>
       <c r="AC24" s="34">
         <v>0</v>
       </c>
@@ -6588,7 +6587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:35" ht="15.75" thickBot="1">
+    <row r="25" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="2">
         <v>20</v>
       </c>
@@ -6603,10 +6602,10 @@
       <c r="F25" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="G25" s="317"/>
-      <c r="H25" s="318"/>
-      <c r="I25" s="318"/>
-      <c r="J25" s="319"/>
+      <c r="G25" s="271"/>
+      <c r="H25" s="272"/>
+      <c r="I25" s="272"/>
+      <c r="J25" s="273"/>
       <c r="K25" s="49" t="s">
         <v>38</v>
       </c>
@@ -6614,11 +6613,11 @@
         <v>131</v>
       </c>
       <c r="M25" s="56"/>
-      <c r="N25" s="229" t="s">
+      <c r="N25" s="220" t="s">
         <v>40</v>
       </c>
-      <c r="O25" s="230"/>
-      <c r="P25" s="231"/>
+      <c r="O25" s="221"/>
+      <c r="P25" s="222"/>
       <c r="R25" s="2">
         <v>20</v>
       </c>
@@ -6628,10 +6627,10 @@
       <c r="T25" s="33">
         <v>1</v>
       </c>
-      <c r="U25" s="297" t="s">
+      <c r="U25" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V25" s="298"/>
+      <c r="V25" s="262"/>
       <c r="W25" s="34">
         <v>0</v>
       </c>
@@ -6644,10 +6643,10 @@
       <c r="Z25" s="34">
         <v>0</v>
       </c>
-      <c r="AA25" s="297" t="s">
+      <c r="AA25" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB25" s="298"/>
+      <c r="AB25" s="262"/>
       <c r="AC25" s="34">
         <v>0</v>
       </c>
@@ -6670,7 +6669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:35" ht="15.75" thickBot="1">
+    <row r="26" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="2">
         <v>21</v>
       </c>
@@ -6685,10 +6684,10 @@
       <c r="F26" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="G26" s="317"/>
-      <c r="H26" s="318"/>
-      <c r="I26" s="318"/>
-      <c r="J26" s="319"/>
+      <c r="G26" s="271"/>
+      <c r="H26" s="272"/>
+      <c r="I26" s="272"/>
+      <c r="J26" s="273"/>
       <c r="K26" s="31" t="s">
         <v>39</v>
       </c>
@@ -6696,11 +6695,11 @@
         <v>131</v>
       </c>
       <c r="M26" s="56"/>
-      <c r="N26" s="229" t="s">
+      <c r="N26" s="220" t="s">
         <v>41</v>
       </c>
-      <c r="O26" s="230"/>
-      <c r="P26" s="231"/>
+      <c r="O26" s="221"/>
+      <c r="P26" s="222"/>
       <c r="R26" s="2">
         <v>21</v>
       </c>
@@ -6710,10 +6709,10 @@
       <c r="T26" s="33">
         <v>0</v>
       </c>
-      <c r="U26" s="297" t="s">
+      <c r="U26" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V26" s="298"/>
+      <c r="V26" s="262"/>
       <c r="W26" s="34">
         <v>1</v>
       </c>
@@ -6726,10 +6725,10 @@
       <c r="Z26" s="34">
         <v>0</v>
       </c>
-      <c r="AA26" s="297" t="s">
+      <c r="AA26" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB26" s="298"/>
+      <c r="AB26" s="262"/>
       <c r="AC26" s="34">
         <v>0</v>
       </c>
@@ -6752,7 +6751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:35" ht="15.75" thickBot="1">
+    <row r="27" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="3">
         <v>22</v>
       </c>
@@ -6761,22 +6760,22 @@
         <f t="shared" si="0"/>
         <v>10110</v>
       </c>
-      <c r="E27" s="323"/>
-      <c r="F27" s="318"/>
-      <c r="G27" s="318"/>
-      <c r="H27" s="318"/>
-      <c r="I27" s="318"/>
-      <c r="J27" s="319"/>
+      <c r="E27" s="275"/>
+      <c r="F27" s="272"/>
+      <c r="G27" s="272"/>
+      <c r="H27" s="272"/>
+      <c r="I27" s="272"/>
+      <c r="J27" s="273"/>
       <c r="K27" s="25" t="s">
         <v>43</v>
       </c>
       <c r="L27" s="39"/>
       <c r="M27" s="56"/>
-      <c r="N27" s="229" t="s">
+      <c r="N27" s="220" t="s">
         <v>45</v>
       </c>
-      <c r="O27" s="230"/>
-      <c r="P27" s="231"/>
+      <c r="O27" s="221"/>
+      <c r="P27" s="222"/>
       <c r="R27" s="3">
         <v>22</v>
       </c>
@@ -6786,10 +6785,10 @@
       <c r="T27" s="33">
         <v>0</v>
       </c>
-      <c r="U27" s="297" t="s">
+      <c r="U27" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="V27" s="298"/>
+      <c r="V27" s="262"/>
       <c r="W27" s="34">
         <v>0</v>
       </c>
@@ -6802,10 +6801,10 @@
       <c r="Z27" s="34">
         <v>0</v>
       </c>
-      <c r="AA27" s="297" t="s">
+      <c r="AA27" s="261" t="s">
         <v>69</v>
       </c>
-      <c r="AB27" s="298"/>
+      <c r="AB27" s="262"/>
       <c r="AC27" s="34">
         <v>1</v>
       </c>
@@ -6828,7 +6827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:35" ht="15.75" thickBot="1">
+    <row r="28" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="4">
         <v>23</v>
       </c>
@@ -6837,12 +6836,12 @@
         <f t="shared" si="0"/>
         <v>10111</v>
       </c>
-      <c r="E28" s="320"/>
-      <c r="F28" s="321"/>
-      <c r="G28" s="321"/>
-      <c r="H28" s="321"/>
-      <c r="I28" s="321"/>
-      <c r="J28" s="322"/>
+      <c r="E28" s="279"/>
+      <c r="F28" s="280"/>
+      <c r="G28" s="280"/>
+      <c r="H28" s="280"/>
+      <c r="I28" s="280"/>
+      <c r="J28" s="281"/>
       <c r="K28" s="52" t="s">
         <v>44</v>
       </c>
@@ -6850,11 +6849,11 @@
         <v>131</v>
       </c>
       <c r="M28" s="14"/>
-      <c r="N28" s="226" t="s">
+      <c r="N28" s="217" t="s">
         <v>319</v>
       </c>
-      <c r="O28" s="227"/>
-      <c r="P28" s="228"/>
+      <c r="O28" s="218"/>
+      <c r="P28" s="219"/>
       <c r="R28" s="4">
         <v>23</v>
       </c>
@@ -6864,10 +6863,10 @@
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="299" t="s">
+      <c r="U28" s="308" t="s">
         <v>69</v>
       </c>
-      <c r="V28" s="300"/>
+      <c r="V28" s="309"/>
       <c r="W28" s="54">
         <v>0</v>
       </c>
@@ -6880,10 +6879,10 @@
       <c r="Z28" s="54">
         <v>0</v>
       </c>
-      <c r="AA28" s="299" t="s">
+      <c r="AA28" s="308" t="s">
         <v>69</v>
       </c>
-      <c r="AB28" s="300"/>
+      <c r="AB28" s="309"/>
       <c r="AC28" s="13">
         <v>1</v>
       </c>
@@ -6906,8 +6905,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:35" ht="15.75" thickBot="1"/>
-    <row r="30" spans="2:35" ht="21.75" customHeight="1" thickBot="1">
+    <row r="29" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="2:35" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="66" t="s">
         <v>80</v>
       </c>
@@ -6960,20 +6959,20 @@
       <c r="S30" s="75" t="s">
         <v>132</v>
       </c>
-      <c r="T30" s="336" t="s">
+      <c r="T30" s="244" t="s">
         <v>133</v>
       </c>
-      <c r="U30" s="336"/>
-      <c r="V30" s="336"/>
-      <c r="W30" s="336"/>
-      <c r="X30" s="336"/>
-      <c r="Y30" s="336"/>
-      <c r="Z30" s="336"/>
-      <c r="AA30" s="336"/>
-      <c r="AB30" s="336"/>
-      <c r="AC30" s="309"/>
-    </row>
-    <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
+      <c r="U30" s="244"/>
+      <c r="V30" s="244"/>
+      <c r="W30" s="244"/>
+      <c r="X30" s="244"/>
+      <c r="Y30" s="244"/>
+      <c r="Z30" s="244"/>
+      <c r="AA30" s="244"/>
+      <c r="AB30" s="244"/>
+      <c r="AC30" s="245"/>
+    </row>
+    <row r="31" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="67" t="s">
         <v>68</v>
       </c>
@@ -7012,20 +7011,20 @@
       <c r="S31" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="T31" s="232" t="s">
+      <c r="T31" s="223" t="s">
         <v>138</v>
       </c>
-      <c r="U31" s="233"/>
-      <c r="V31" s="233"/>
-      <c r="W31" s="233"/>
-      <c r="X31" s="233"/>
-      <c r="Y31" s="233"/>
-      <c r="Z31" s="233"/>
-      <c r="AA31" s="233"/>
-      <c r="AB31" s="233"/>
-      <c r="AC31" s="234"/>
-    </row>
-    <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1">
+      <c r="U31" s="224"/>
+      <c r="V31" s="224"/>
+      <c r="W31" s="224"/>
+      <c r="X31" s="224"/>
+      <c r="Y31" s="224"/>
+      <c r="Z31" s="224"/>
+      <c r="AA31" s="224"/>
+      <c r="AB31" s="224"/>
+      <c r="AC31" s="225"/>
+    </row>
+    <row r="32" spans="2:35" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="4" t="s">
         <v>71</v>
       </c>
@@ -7047,20 +7046,20 @@
       <c r="S32" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="T32" s="229" t="s">
+      <c r="T32" s="220" t="s">
         <v>139</v>
       </c>
-      <c r="U32" s="230"/>
-      <c r="V32" s="230"/>
-      <c r="W32" s="230"/>
-      <c r="X32" s="230"/>
-      <c r="Y32" s="230"/>
-      <c r="Z32" s="230"/>
-      <c r="AA32" s="230"/>
-      <c r="AB32" s="230"/>
-      <c r="AC32" s="231"/>
-    </row>
-    <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1">
+      <c r="U32" s="221"/>
+      <c r="V32" s="221"/>
+      <c r="W32" s="221"/>
+      <c r="X32" s="221"/>
+      <c r="Y32" s="221"/>
+      <c r="Z32" s="221"/>
+      <c r="AA32" s="221"/>
+      <c r="AB32" s="221"/>
+      <c r="AC32" s="222"/>
+    </row>
+    <row r="33" spans="2:29" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H33" s="84" t="s">
         <v>165</v>
       </c>
@@ -7094,31 +7093,31 @@
       <c r="S33" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="T33" s="229" t="s">
+      <c r="T33" s="220" t="s">
         <v>140</v>
       </c>
-      <c r="U33" s="230"/>
-      <c r="V33" s="230"/>
-      <c r="W33" s="230"/>
-      <c r="X33" s="230"/>
-      <c r="Y33" s="230"/>
-      <c r="Z33" s="230"/>
-      <c r="AA33" s="230"/>
-      <c r="AB33" s="230"/>
-      <c r="AC33" s="231"/>
-    </row>
-    <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B34" s="295" t="s">
+      <c r="U33" s="221"/>
+      <c r="V33" s="221"/>
+      <c r="W33" s="221"/>
+      <c r="X33" s="221"/>
+      <c r="Y33" s="221"/>
+      <c r="Z33" s="221"/>
+      <c r="AA33" s="221"/>
+      <c r="AB33" s="221"/>
+      <c r="AC33" s="222"/>
+    </row>
+    <row r="34" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="306" t="s">
         <v>95</v>
       </c>
-      <c r="C34" s="293" t="s">
+      <c r="C34" s="282" t="s">
         <v>100</v>
       </c>
-      <c r="D34" s="294"/>
-      <c r="E34" s="293" t="s">
+      <c r="D34" s="284"/>
+      <c r="E34" s="282" t="s">
         <v>101</v>
       </c>
-      <c r="F34" s="294"/>
+      <c r="F34" s="284"/>
       <c r="H34" s="77" t="s">
         <v>61</v>
       </c>
@@ -7146,21 +7145,21 @@
       <c r="S34" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="T34" s="229" t="s">
+      <c r="T34" s="220" t="s">
         <v>141</v>
       </c>
-      <c r="U34" s="230"/>
-      <c r="V34" s="230"/>
-      <c r="W34" s="230"/>
-      <c r="X34" s="230"/>
-      <c r="Y34" s="230"/>
-      <c r="Z34" s="230"/>
-      <c r="AA34" s="230"/>
-      <c r="AB34" s="230"/>
-      <c r="AC34" s="231"/>
-    </row>
-    <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1">
-      <c r="B35" s="296"/>
+      <c r="U34" s="221"/>
+      <c r="V34" s="221"/>
+      <c r="W34" s="221"/>
+      <c r="X34" s="221"/>
+      <c r="Y34" s="221"/>
+      <c r="Z34" s="221"/>
+      <c r="AA34" s="221"/>
+      <c r="AB34" s="221"/>
+      <c r="AC34" s="222"/>
+    </row>
+    <row r="35" spans="2:29" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="307"/>
       <c r="C35" s="64" t="s">
         <v>91</v>
       </c>
@@ -7179,20 +7178,20 @@
       <c r="S35" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="T35" s="229" t="s">
+      <c r="T35" s="220" t="s">
         <v>142</v>
       </c>
-      <c r="U35" s="230"/>
-      <c r="V35" s="230"/>
-      <c r="W35" s="230"/>
-      <c r="X35" s="230"/>
-      <c r="Y35" s="230"/>
-      <c r="Z35" s="230"/>
-      <c r="AA35" s="230"/>
-      <c r="AB35" s="230"/>
-      <c r="AC35" s="231"/>
-    </row>
-    <row r="36" spans="2:29" ht="36" customHeight="1" thickBot="1">
+      <c r="U35" s="221"/>
+      <c r="V35" s="221"/>
+      <c r="W35" s="221"/>
+      <c r="X35" s="221"/>
+      <c r="Y35" s="221"/>
+      <c r="Z35" s="221"/>
+      <c r="AA35" s="221"/>
+      <c r="AB35" s="221"/>
+      <c r="AC35" s="222"/>
+    </row>
+    <row r="36" spans="2:29" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="1">
         <v>0</v>
       </c>
@@ -7241,20 +7240,20 @@
       <c r="S36" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="T36" s="229" t="s">
+      <c r="T36" s="220" t="s">
         <v>143</v>
       </c>
-      <c r="U36" s="230"/>
-      <c r="V36" s="230"/>
-      <c r="W36" s="230"/>
-      <c r="X36" s="230"/>
-      <c r="Y36" s="230"/>
-      <c r="Z36" s="230"/>
-      <c r="AA36" s="230"/>
-      <c r="AB36" s="230"/>
-      <c r="AC36" s="231"/>
-    </row>
-    <row r="37" spans="2:29" ht="36.75" customHeight="1" thickBot="1">
+      <c r="U36" s="221"/>
+      <c r="V36" s="221"/>
+      <c r="W36" s="221"/>
+      <c r="X36" s="221"/>
+      <c r="Y36" s="221"/>
+      <c r="Z36" s="221"/>
+      <c r="AA36" s="221"/>
+      <c r="AB36" s="221"/>
+      <c r="AC36" s="222"/>
+    </row>
+    <row r="37" spans="2:29" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="2">
         <v>1</v>
       </c>
@@ -7295,20 +7294,20 @@
       <c r="S37" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="T37" s="229" t="s">
+      <c r="T37" s="220" t="s">
         <v>163</v>
       </c>
-      <c r="U37" s="230"/>
-      <c r="V37" s="230"/>
-      <c r="W37" s="230"/>
-      <c r="X37" s="230"/>
-      <c r="Y37" s="230"/>
-      <c r="Z37" s="230"/>
-      <c r="AA37" s="230"/>
-      <c r="AB37" s="230"/>
-      <c r="AC37" s="231"/>
-    </row>
-    <row r="38" spans="2:29" ht="15.75" thickBot="1">
+      <c r="U37" s="221"/>
+      <c r="V37" s="221"/>
+      <c r="W37" s="221"/>
+      <c r="X37" s="221"/>
+      <c r="Y37" s="221"/>
+      <c r="Z37" s="221"/>
+      <c r="AA37" s="221"/>
+      <c r="AB37" s="221"/>
+      <c r="AC37" s="222"/>
+    </row>
+    <row r="38" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="2">
         <v>2</v>
       </c>
@@ -7327,23 +7326,23 @@
       <c r="R38" s="2">
         <v>7</v>
       </c>
-      <c r="S38" s="337" t="s">
+      <c r="S38" s="246" t="s">
         <v>68</v>
       </c>
-      <c r="T38" s="339" t="s">
+      <c r="T38" s="248" t="s">
         <v>144</v>
       </c>
-      <c r="U38" s="340"/>
-      <c r="V38" s="340"/>
-      <c r="W38" s="340"/>
-      <c r="X38" s="340"/>
-      <c r="Y38" s="340"/>
-      <c r="Z38" s="340"/>
-      <c r="AA38" s="340"/>
-      <c r="AB38" s="340"/>
-      <c r="AC38" s="341"/>
-    </row>
-    <row r="39" spans="2:29" ht="15" customHeight="1">
+      <c r="U38" s="249"/>
+      <c r="V38" s="249"/>
+      <c r="W38" s="249"/>
+      <c r="X38" s="249"/>
+      <c r="Y38" s="249"/>
+      <c r="Z38" s="249"/>
+      <c r="AA38" s="249"/>
+      <c r="AB38" s="249"/>
+      <c r="AC38" s="250"/>
+    </row>
+    <row r="39" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="2">
         <v>3</v>
       </c>
@@ -7359,28 +7358,28 @@
       <c r="F39" s="35" t="s">
         <v>97</v>
       </c>
-      <c r="G39" s="282" t="s">
+      <c r="G39" s="254" t="s">
         <v>153</v>
       </c>
-      <c r="H39" s="224"/>
-      <c r="I39" s="224"/>
-      <c r="J39" s="225"/>
+      <c r="H39" s="215"/>
+      <c r="I39" s="215"/>
+      <c r="J39" s="216"/>
       <c r="R39" s="2">
         <v>8</v>
       </c>
-      <c r="S39" s="338"/>
-      <c r="T39" s="342"/>
-      <c r="U39" s="343"/>
-      <c r="V39" s="343"/>
-      <c r="W39" s="343"/>
-      <c r="X39" s="343"/>
-      <c r="Y39" s="343"/>
-      <c r="Z39" s="343"/>
-      <c r="AA39" s="343"/>
-      <c r="AB39" s="343"/>
-      <c r="AC39" s="344"/>
-    </row>
-    <row r="40" spans="2:29" ht="37.5" customHeight="1">
+      <c r="S39" s="247"/>
+      <c r="T39" s="251"/>
+      <c r="U39" s="252"/>
+      <c r="V39" s="252"/>
+      <c r="W39" s="252"/>
+      <c r="X39" s="252"/>
+      <c r="Y39" s="252"/>
+      <c r="Z39" s="252"/>
+      <c r="AA39" s="252"/>
+      <c r="AB39" s="252"/>
+      <c r="AC39" s="253"/>
+    </row>
+    <row r="40" spans="2:29" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="2">
         <v>4</v>
       </c>
@@ -7396,30 +7395,30 @@
       <c r="F40" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="G40" s="283"/>
-      <c r="H40" s="284"/>
-      <c r="I40" s="284"/>
-      <c r="J40" s="285"/>
+      <c r="G40" s="258"/>
+      <c r="H40" s="259"/>
+      <c r="I40" s="259"/>
+      <c r="J40" s="260"/>
       <c r="R40" s="2">
         <v>9</v>
       </c>
       <c r="S40" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="T40" s="229" t="s">
+      <c r="T40" s="220" t="s">
         <v>323</v>
       </c>
-      <c r="U40" s="230"/>
-      <c r="V40" s="230"/>
-      <c r="W40" s="230"/>
-      <c r="X40" s="230"/>
-      <c r="Y40" s="230"/>
-      <c r="Z40" s="230"/>
-      <c r="AA40" s="230"/>
-      <c r="AB40" s="230"/>
-      <c r="AC40" s="231"/>
-    </row>
-    <row r="41" spans="2:29" ht="30" customHeight="1">
+      <c r="U40" s="221"/>
+      <c r="V40" s="221"/>
+      <c r="W40" s="221"/>
+      <c r="X40" s="221"/>
+      <c r="Y40" s="221"/>
+      <c r="Z40" s="221"/>
+      <c r="AA40" s="221"/>
+      <c r="AB40" s="221"/>
+      <c r="AC40" s="222"/>
+    </row>
+    <row r="41" spans="2:29" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="2">
         <v>5</v>
       </c>
@@ -7435,30 +7434,30 @@
       <c r="F41" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="G41" s="283"/>
-      <c r="H41" s="284"/>
-      <c r="I41" s="284"/>
-      <c r="J41" s="285"/>
+      <c r="G41" s="258"/>
+      <c r="H41" s="259"/>
+      <c r="I41" s="259"/>
+      <c r="J41" s="260"/>
       <c r="R41" s="2">
         <v>10</v>
       </c>
       <c r="S41" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="T41" s="229" t="s">
+      <c r="T41" s="220" t="s">
         <v>326</v>
       </c>
-      <c r="U41" s="230"/>
-      <c r="V41" s="230"/>
-      <c r="W41" s="230"/>
-      <c r="X41" s="230"/>
-      <c r="Y41" s="230"/>
-      <c r="Z41" s="230"/>
-      <c r="AA41" s="230"/>
-      <c r="AB41" s="230"/>
-      <c r="AC41" s="231"/>
-    </row>
-    <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1">
+      <c r="U41" s="221"/>
+      <c r="V41" s="221"/>
+      <c r="W41" s="221"/>
+      <c r="X41" s="221"/>
+      <c r="Y41" s="221"/>
+      <c r="Z41" s="221"/>
+      <c r="AA41" s="221"/>
+      <c r="AB41" s="221"/>
+      <c r="AC41" s="222"/>
+    </row>
+    <row r="42" spans="2:29" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="2">
         <v>6</v>
       </c>
@@ -7474,30 +7473,30 @@
       <c r="F42" s="76" t="s">
         <v>148</v>
       </c>
-      <c r="G42" s="286"/>
-      <c r="H42" s="287"/>
-      <c r="I42" s="287"/>
-      <c r="J42" s="288"/>
+      <c r="G42" s="255"/>
+      <c r="H42" s="256"/>
+      <c r="I42" s="256"/>
+      <c r="J42" s="257"/>
       <c r="R42" s="2">
         <v>11</v>
       </c>
       <c r="S42" s="37" t="s">
         <v>136</v>
       </c>
-      <c r="T42" s="229" t="s">
+      <c r="T42" s="220" t="s">
         <v>145</v>
       </c>
-      <c r="U42" s="230"/>
-      <c r="V42" s="230"/>
-      <c r="W42" s="230"/>
-      <c r="X42" s="230"/>
-      <c r="Y42" s="230"/>
-      <c r="Z42" s="230"/>
-      <c r="AA42" s="230"/>
-      <c r="AB42" s="230"/>
-      <c r="AC42" s="231"/>
-    </row>
-    <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1">
+      <c r="U42" s="221"/>
+      <c r="V42" s="221"/>
+      <c r="W42" s="221"/>
+      <c r="X42" s="221"/>
+      <c r="Y42" s="221"/>
+      <c r="Z42" s="221"/>
+      <c r="AA42" s="221"/>
+      <c r="AB42" s="221"/>
+      <c r="AC42" s="222"/>
+    </row>
+    <row r="43" spans="2:29" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="2">
         <v>7</v>
       </c>
@@ -7513,32 +7512,32 @@
       <c r="F43" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="G43" s="238" t="s">
+      <c r="G43" s="206" t="s">
         <v>330</v>
       </c>
-      <c r="H43" s="239"/>
-      <c r="I43" s="239"/>
-      <c r="J43" s="240"/>
+      <c r="H43" s="207"/>
+      <c r="I43" s="207"/>
+      <c r="J43" s="208"/>
       <c r="R43" s="2">
         <v>12</v>
       </c>
       <c r="S43" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="T43" s="229" t="s">
+      <c r="T43" s="220" t="s">
         <v>146</v>
       </c>
-      <c r="U43" s="230"/>
-      <c r="V43" s="230"/>
-      <c r="W43" s="230"/>
-      <c r="X43" s="230"/>
-      <c r="Y43" s="230"/>
-      <c r="Z43" s="230"/>
-      <c r="AA43" s="230"/>
-      <c r="AB43" s="230"/>
-      <c r="AC43" s="231"/>
-    </row>
-    <row r="44" spans="2:29" ht="45.75" thickBot="1">
+      <c r="U43" s="221"/>
+      <c r="V43" s="221"/>
+      <c r="W43" s="221"/>
+      <c r="X43" s="221"/>
+      <c r="Y43" s="221"/>
+      <c r="Z43" s="221"/>
+      <c r="AA43" s="221"/>
+      <c r="AB43" s="221"/>
+      <c r="AC43" s="222"/>
+    </row>
+    <row r="44" spans="2:29" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="2">
         <v>8</v>
       </c>
@@ -7557,23 +7556,23 @@
       <c r="R44" s="2">
         <v>13</v>
       </c>
-      <c r="S44" s="337" t="s">
+      <c r="S44" s="246" t="s">
         <v>71</v>
       </c>
-      <c r="T44" s="339" t="s">
+      <c r="T44" s="248" t="s">
         <v>332</v>
       </c>
-      <c r="U44" s="340"/>
-      <c r="V44" s="340"/>
-      <c r="W44" s="340"/>
-      <c r="X44" s="340"/>
-      <c r="Y44" s="340"/>
-      <c r="Z44" s="340"/>
-      <c r="AA44" s="340"/>
-      <c r="AB44" s="340"/>
-      <c r="AC44" s="341"/>
-    </row>
-    <row r="45" spans="2:29" ht="30.75" customHeight="1">
+      <c r="U44" s="249"/>
+      <c r="V44" s="249"/>
+      <c r="W44" s="249"/>
+      <c r="X44" s="249"/>
+      <c r="Y44" s="249"/>
+      <c r="Z44" s="249"/>
+      <c r="AA44" s="249"/>
+      <c r="AB44" s="249"/>
+      <c r="AC44" s="250"/>
+    </row>
+    <row r="45" spans="2:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="2">
         <v>9</v>
       </c>
@@ -7589,28 +7588,28 @@
       <c r="F45" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="G45" s="282" t="s">
+      <c r="G45" s="254" t="s">
         <v>152</v>
       </c>
-      <c r="H45" s="224"/>
-      <c r="I45" s="224"/>
-      <c r="J45" s="225"/>
+      <c r="H45" s="215"/>
+      <c r="I45" s="215"/>
+      <c r="J45" s="216"/>
       <c r="R45" s="2">
         <v>14</v>
       </c>
-      <c r="S45" s="338"/>
-      <c r="T45" s="342"/>
-      <c r="U45" s="343"/>
-      <c r="V45" s="343"/>
-      <c r="W45" s="343"/>
-      <c r="X45" s="343"/>
-      <c r="Y45" s="343"/>
-      <c r="Z45" s="343"/>
-      <c r="AA45" s="343"/>
-      <c r="AB45" s="343"/>
-      <c r="AC45" s="344"/>
-    </row>
-    <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1">
+      <c r="S45" s="247"/>
+      <c r="T45" s="251"/>
+      <c r="U45" s="252"/>
+      <c r="V45" s="252"/>
+      <c r="W45" s="252"/>
+      <c r="X45" s="252"/>
+      <c r="Y45" s="252"/>
+      <c r="Z45" s="252"/>
+      <c r="AA45" s="252"/>
+      <c r="AB45" s="252"/>
+      <c r="AC45" s="253"/>
+    </row>
+    <row r="46" spans="2:29" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B46" s="2">
         <v>10</v>
       </c>
@@ -7626,30 +7625,30 @@
       <c r="F46" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="G46" s="286"/>
-      <c r="H46" s="287"/>
-      <c r="I46" s="287"/>
-      <c r="J46" s="288"/>
+      <c r="G46" s="255"/>
+      <c r="H46" s="256"/>
+      <c r="I46" s="256"/>
+      <c r="J46" s="257"/>
       <c r="R46" s="4">
         <v>15</v>
       </c>
       <c r="S46" s="40" t="s">
         <v>127</v>
       </c>
-      <c r="T46" s="226" t="s">
+      <c r="T46" s="217" t="s">
         <v>147</v>
       </c>
-      <c r="U46" s="227"/>
-      <c r="V46" s="227"/>
-      <c r="W46" s="227"/>
-      <c r="X46" s="227"/>
-      <c r="Y46" s="227"/>
-      <c r="Z46" s="227"/>
-      <c r="AA46" s="227"/>
-      <c r="AB46" s="227"/>
-      <c r="AC46" s="228"/>
-    </row>
-    <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1">
+      <c r="U46" s="218"/>
+      <c r="V46" s="218"/>
+      <c r="W46" s="218"/>
+      <c r="X46" s="218"/>
+      <c r="Y46" s="218"/>
+      <c r="Z46" s="218"/>
+      <c r="AA46" s="218"/>
+      <c r="AB46" s="218"/>
+      <c r="AC46" s="219"/>
+    </row>
+    <row r="47" spans="2:29" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="2">
         <v>11</v>
       </c>
@@ -7665,14 +7664,14 @@
       <c r="F47" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="G47" s="239" t="s">
+      <c r="G47" s="207" t="s">
         <v>334</v>
       </c>
-      <c r="H47" s="239"/>
-      <c r="I47" s="239"/>
-      <c r="J47" s="240"/>
-    </row>
-    <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1">
+      <c r="H47" s="207"/>
+      <c r="I47" s="207"/>
+      <c r="J47" s="208"/>
+    </row>
+    <row r="48" spans="2:29" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B48" s="2">
         <v>12</v>
       </c>
@@ -7715,13 +7714,13 @@
       <c r="Z48" s="72">
         <v>0</v>
       </c>
-      <c r="AA48" s="244" t="s">
+      <c r="AA48" s="319" t="s">
         <v>336</v>
       </c>
-      <c r="AB48" s="245"/>
-      <c r="AC48" s="246"/>
-    </row>
-    <row r="49" spans="2:29" ht="35.25" customHeight="1" thickBot="1">
+      <c r="AB48" s="320"/>
+      <c r="AC48" s="321"/>
+    </row>
+    <row r="49" spans="2:29" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B49" s="2">
         <v>13</v>
       </c>
@@ -7737,12 +7736,12 @@
       <c r="F49" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="G49" s="282" t="s">
+      <c r="G49" s="254" t="s">
         <v>338</v>
       </c>
-      <c r="H49" s="224"/>
-      <c r="I49" s="224"/>
-      <c r="J49" s="225"/>
+      <c r="H49" s="215"/>
+      <c r="I49" s="215"/>
+      <c r="J49" s="216"/>
       <c r="R49" s="77" t="s">
         <v>61</v>
       </c>
@@ -7758,11 +7757,11 @@
       <c r="Z49" s="80" t="s">
         <v>298</v>
       </c>
-      <c r="AA49" s="247"/>
-      <c r="AB49" s="248"/>
-      <c r="AC49" s="249"/>
-    </row>
-    <row r="50" spans="2:29" ht="30" customHeight="1" thickBot="1">
+      <c r="AA49" s="322"/>
+      <c r="AB49" s="323"/>
+      <c r="AC49" s="324"/>
+    </row>
+    <row r="50" spans="2:29" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B50" s="2">
         <v>14</v>
       </c>
@@ -7778,12 +7777,12 @@
       <c r="F50" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="G50" s="283"/>
-      <c r="H50" s="284"/>
-      <c r="I50" s="284"/>
-      <c r="J50" s="285"/>
-    </row>
-    <row r="51" spans="2:29" ht="20.25" customHeight="1" thickBot="1">
+      <c r="G50" s="258"/>
+      <c r="H50" s="259"/>
+      <c r="I50" s="259"/>
+      <c r="J50" s="260"/>
+    </row>
+    <row r="51" spans="2:29" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" s="4">
         <v>15</v>
       </c>
@@ -7799,447 +7798,566 @@
       <c r="F51" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="G51" s="286"/>
-      <c r="H51" s="287"/>
-      <c r="I51" s="287"/>
-      <c r="J51" s="288"/>
-      <c r="R51" s="262" t="s">
+      <c r="G51" s="255"/>
+      <c r="H51" s="256"/>
+      <c r="I51" s="256"/>
+      <c r="J51" s="257"/>
+      <c r="R51" s="316" t="s">
         <v>301</v>
       </c>
-      <c r="S51" s="264" t="s">
+      <c r="S51" s="300" t="s">
         <v>156</v>
       </c>
-      <c r="T51" s="266" t="s">
+      <c r="T51" s="312" t="s">
         <v>155</v>
       </c>
-      <c r="U51" s="266"/>
-      <c r="V51" s="267"/>
-    </row>
-    <row r="52" spans="2:29" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B52" s="241" t="s">
+      <c r="U51" s="312"/>
+      <c r="V51" s="313"/>
+    </row>
+    <row r="52" spans="2:29" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="209" t="s">
         <v>339</v>
       </c>
-      <c r="C52" s="242"/>
-      <c r="D52" s="242"/>
-      <c r="E52" s="242"/>
-      <c r="F52" s="243"/>
-      <c r="R52" s="263"/>
-      <c r="S52" s="265"/>
-      <c r="T52" s="268"/>
-      <c r="U52" s="268"/>
-      <c r="V52" s="269"/>
-    </row>
-    <row r="53" spans="2:29" ht="48" customHeight="1" thickBot="1">
+      <c r="C52" s="210"/>
+      <c r="D52" s="210"/>
+      <c r="E52" s="210"/>
+      <c r="F52" s="211"/>
+      <c r="R52" s="336"/>
+      <c r="S52" s="318"/>
+      <c r="T52" s="337"/>
+      <c r="U52" s="337"/>
+      <c r="V52" s="338"/>
+    </row>
+    <row r="53" spans="2:29" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="R53" s="165" t="s">
         <v>195</v>
       </c>
       <c r="S53" s="166" t="s">
         <v>302</v>
       </c>
-      <c r="T53" s="257" t="s">
+      <c r="T53" s="331" t="s">
         <v>340</v>
       </c>
-      <c r="U53" s="257"/>
-      <c r="V53" s="258"/>
-    </row>
-    <row r="54" spans="2:29" ht="36.75" customHeight="1">
-      <c r="B54" s="291" t="s">
+      <c r="U53" s="331"/>
+      <c r="V53" s="332"/>
+    </row>
+    <row r="54" spans="2:29" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="302" t="s">
         <v>154</v>
       </c>
-      <c r="C54" s="264" t="s">
+      <c r="C54" s="300" t="s">
         <v>156</v>
       </c>
-      <c r="D54" s="266" t="s">
+      <c r="D54" s="312" t="s">
         <v>155</v>
       </c>
-      <c r="E54" s="267"/>
-      <c r="H54" s="262" t="s">
+      <c r="E54" s="313"/>
+      <c r="H54" s="316" t="s">
         <v>292</v>
       </c>
-      <c r="I54" s="264" t="s">
+      <c r="I54" s="300" t="s">
         <v>156</v>
       </c>
-      <c r="J54" s="250" t="s">
+      <c r="J54" s="325" t="s">
         <v>155</v>
       </c>
-      <c r="K54" s="251"/>
-      <c r="L54" s="252"/>
+      <c r="K54" s="326"/>
+      <c r="L54" s="327"/>
       <c r="R54" s="163" t="s">
         <v>204</v>
       </c>
       <c r="S54" s="161" t="s">
         <v>303</v>
       </c>
-      <c r="T54" s="270" t="s">
+      <c r="T54" s="339" t="s">
         <v>309</v>
       </c>
-      <c r="U54" s="270"/>
-      <c r="V54" s="271"/>
-    </row>
-    <row r="55" spans="2:29" ht="24" customHeight="1" thickBot="1">
-      <c r="B55" s="292"/>
-      <c r="C55" s="290"/>
-      <c r="D55" s="280"/>
-      <c r="E55" s="281"/>
-      <c r="H55" s="289"/>
-      <c r="I55" s="265"/>
-      <c r="J55" s="253"/>
-      <c r="K55" s="254"/>
-      <c r="L55" s="255"/>
+      <c r="U54" s="339"/>
+      <c r="V54" s="305"/>
+    </row>
+    <row r="55" spans="2:29" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B55" s="303"/>
+      <c r="C55" s="301"/>
+      <c r="D55" s="314"/>
+      <c r="E55" s="315"/>
+      <c r="H55" s="317"/>
+      <c r="I55" s="318"/>
+      <c r="J55" s="291"/>
+      <c r="K55" s="328"/>
+      <c r="L55" s="329"/>
       <c r="R55" s="163" t="s">
         <v>190</v>
       </c>
       <c r="S55" s="161" t="s">
         <v>304</v>
       </c>
-      <c r="T55" s="270" t="s">
+      <c r="T55" s="339" t="s">
         <v>341</v>
       </c>
-      <c r="U55" s="270"/>
-      <c r="V55" s="271"/>
-    </row>
-    <row r="56" spans="2:29" ht="60.75" customHeight="1" thickBot="1">
+      <c r="U55" s="339"/>
+      <c r="V55" s="305"/>
+    </row>
+    <row r="56" spans="2:29" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B56" s="81">
         <v>0</v>
       </c>
       <c r="C56" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="D56" s="232" t="s">
+      <c r="D56" s="223" t="s">
         <v>170</v>
       </c>
-      <c r="E56" s="234"/>
+      <c r="E56" s="225"/>
       <c r="H56" s="81" t="s">
         <v>295</v>
       </c>
       <c r="I56" s="45" t="s">
         <v>290</v>
       </c>
-      <c r="J56" s="256" t="s">
+      <c r="J56" s="330" t="s">
         <v>293</v>
       </c>
-      <c r="K56" s="257"/>
-      <c r="L56" s="258"/>
-      <c r="M56" s="238" t="s">
+      <c r="K56" s="331"/>
+      <c r="L56" s="332"/>
+      <c r="M56" s="206" t="s">
         <v>342</v>
       </c>
-      <c r="N56" s="240"/>
+      <c r="N56" s="208"/>
       <c r="R56" s="163" t="s">
         <v>215</v>
       </c>
       <c r="S56" s="161" t="s">
         <v>305</v>
       </c>
-      <c r="T56" s="270" t="s">
+      <c r="T56" s="339" t="s">
         <v>343</v>
       </c>
-      <c r="U56" s="270"/>
-      <c r="V56" s="271"/>
-    </row>
-    <row r="57" spans="2:29" ht="49.5" customHeight="1" thickBot="1">
+      <c r="U56" s="339"/>
+      <c r="V56" s="305"/>
+    </row>
+    <row r="57" spans="2:29" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B57" s="82">
         <v>1</v>
       </c>
       <c r="C57" s="85" t="s">
         <v>288</v>
       </c>
-      <c r="D57" s="277" t="s">
+      <c r="D57" s="304" t="s">
         <v>289</v>
       </c>
-      <c r="E57" s="271"/>
-      <c r="F57" s="238" t="s">
+      <c r="E57" s="305"/>
+      <c r="F57" s="206" t="s">
         <v>344</v>
       </c>
-      <c r="G57" s="240"/>
+      <c r="G57" s="208"/>
       <c r="H57" s="82">
         <v>0</v>
       </c>
       <c r="I57" s="85" t="s">
         <v>294</v>
       </c>
-      <c r="J57" s="259" t="s">
+      <c r="J57" s="333" t="s">
         <v>345</v>
       </c>
-      <c r="K57" s="260"/>
-      <c r="L57" s="261"/>
+      <c r="K57" s="334"/>
+      <c r="L57" s="335"/>
       <c r="R57" s="163" t="s">
         <v>229</v>
       </c>
       <c r="S57" s="36" t="s">
         <v>310</v>
       </c>
-      <c r="T57" s="270" t="s">
+      <c r="T57" s="339" t="s">
         <v>346</v>
       </c>
-      <c r="U57" s="270"/>
-      <c r="V57" s="271"/>
-    </row>
-    <row r="58" spans="2:29" ht="60" customHeight="1">
+      <c r="U57" s="339"/>
+      <c r="V57" s="305"/>
+    </row>
+    <row r="58" spans="2:29" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="82">
         <v>2</v>
       </c>
       <c r="C58" s="85" t="s">
         <v>164</v>
       </c>
-      <c r="D58" s="277" t="s">
+      <c r="D58" s="304" t="s">
         <v>347</v>
       </c>
-      <c r="E58" s="271"/>
+      <c r="E58" s="305"/>
       <c r="H58" s="82">
         <v>1</v>
       </c>
       <c r="I58" s="85" t="s">
         <v>348</v>
       </c>
-      <c r="J58" s="259" t="s">
+      <c r="J58" s="333" t="s">
         <v>349</v>
       </c>
-      <c r="K58" s="260"/>
-      <c r="L58" s="261"/>
+      <c r="K58" s="334"/>
+      <c r="L58" s="335"/>
       <c r="R58" s="163" t="s">
         <v>230</v>
       </c>
       <c r="S58" s="36" t="s">
         <v>306</v>
       </c>
-      <c r="T58" s="270" t="s">
+      <c r="T58" s="339" t="s">
         <v>350</v>
       </c>
-      <c r="U58" s="270"/>
-      <c r="V58" s="271"/>
-    </row>
-    <row r="59" spans="2:29" ht="61.5" customHeight="1">
+      <c r="U58" s="339"/>
+      <c r="V58" s="305"/>
+    </row>
+    <row r="59" spans="2:29" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="82">
         <v>3</v>
       </c>
       <c r="C59" s="85" t="s">
         <v>351</v>
       </c>
-      <c r="D59" s="277" t="s">
+      <c r="D59" s="304" t="s">
         <v>159</v>
       </c>
-      <c r="E59" s="271"/>
+      <c r="E59" s="305"/>
       <c r="H59" s="82">
         <v>2</v>
       </c>
       <c r="I59" s="85" t="s">
         <v>291</v>
       </c>
-      <c r="J59" s="259" t="s">
+      <c r="J59" s="333" t="s">
         <v>352</v>
       </c>
-      <c r="K59" s="260"/>
-      <c r="L59" s="261"/>
+      <c r="K59" s="334"/>
+      <c r="L59" s="335"/>
       <c r="R59" s="163" t="s">
         <v>231</v>
       </c>
       <c r="S59" s="36" t="s">
         <v>307</v>
       </c>
-      <c r="T59" s="270" t="s">
+      <c r="T59" s="339" t="s">
         <v>353</v>
       </c>
-      <c r="U59" s="270"/>
-      <c r="V59" s="271"/>
+      <c r="U59" s="339"/>
+      <c r="V59" s="305"/>
       <c r="X59" s="167"/>
     </row>
-    <row r="60" spans="2:29" ht="45.75" customHeight="1">
+    <row r="60" spans="2:29" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="82">
         <v>4</v>
       </c>
       <c r="C60" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="D60" s="277" t="s">
+      <c r="D60" s="304" t="s">
         <v>160</v>
       </c>
-      <c r="E60" s="271"/>
+      <c r="E60" s="305"/>
       <c r="H60" s="82">
         <v>3</v>
       </c>
       <c r="I60" s="38" t="s">
         <v>296</v>
       </c>
-      <c r="J60" s="259" t="s">
+      <c r="J60" s="333" t="s">
         <v>311</v>
       </c>
-      <c r="K60" s="260"/>
-      <c r="L60" s="261"/>
+      <c r="K60" s="334"/>
+      <c r="L60" s="335"/>
       <c r="R60" s="163" t="s">
         <v>232</v>
       </c>
       <c r="S60" s="161" t="s">
         <v>308</v>
       </c>
-      <c r="T60" s="272" t="s">
+      <c r="T60" s="340" t="s">
         <v>355</v>
       </c>
-      <c r="U60" s="273"/>
-      <c r="V60" s="274"/>
-    </row>
-    <row r="61" spans="2:29" ht="40.5" customHeight="1">
+      <c r="U60" s="341"/>
+      <c r="V60" s="342"/>
+    </row>
+    <row r="61" spans="2:29" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="82">
         <v>5</v>
       </c>
       <c r="C61" s="38" t="s">
         <v>158</v>
       </c>
-      <c r="D61" s="277" t="s">
+      <c r="D61" s="304" t="s">
         <v>161</v>
       </c>
-      <c r="E61" s="271"/>
+      <c r="E61" s="305"/>
       <c r="H61" s="82">
         <v>4</v>
       </c>
       <c r="I61" s="38"/>
-      <c r="J61" s="259"/>
-      <c r="K61" s="260"/>
-      <c r="L61" s="261"/>
+      <c r="J61" s="333"/>
+      <c r="K61" s="334"/>
+      <c r="L61" s="335"/>
       <c r="R61" s="163" t="s">
         <v>233</v>
       </c>
       <c r="S61" s="161" t="s">
         <v>308</v>
       </c>
-      <c r="T61" s="275"/>
-      <c r="U61" s="207"/>
-      <c r="V61" s="208"/>
-    </row>
-    <row r="62" spans="2:29" ht="53.25" customHeight="1">
+      <c r="T61" s="343"/>
+      <c r="U61" s="230"/>
+      <c r="V61" s="231"/>
+    </row>
+    <row r="62" spans="2:29" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="82">
         <v>6</v>
       </c>
       <c r="C62" s="38"/>
-      <c r="D62" s="277"/>
-      <c r="E62" s="271"/>
+      <c r="D62" s="304"/>
+      <c r="E62" s="305"/>
       <c r="H62" s="82">
         <v>5</v>
       </c>
       <c r="I62" s="38"/>
-      <c r="J62" s="259"/>
-      <c r="K62" s="260"/>
-      <c r="L62" s="261"/>
+      <c r="J62" s="333"/>
+      <c r="K62" s="334"/>
+      <c r="L62" s="335"/>
       <c r="R62" s="163" t="s">
         <v>265</v>
       </c>
       <c r="S62" s="161" t="s">
         <v>308</v>
       </c>
-      <c r="T62" s="275"/>
-      <c r="U62" s="207"/>
-      <c r="V62" s="208"/>
-    </row>
-    <row r="63" spans="2:29" ht="36" customHeight="1" thickBot="1">
+      <c r="T62" s="343"/>
+      <c r="U62" s="230"/>
+      <c r="V62" s="231"/>
+    </row>
+    <row r="63" spans="2:29" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B63" s="82">
         <v>7</v>
       </c>
       <c r="C63" s="85"/>
-      <c r="D63" s="277"/>
-      <c r="E63" s="271"/>
+      <c r="D63" s="304"/>
+      <c r="E63" s="305"/>
       <c r="H63" s="82">
         <v>6</v>
       </c>
       <c r="I63" s="85"/>
-      <c r="J63" s="259"/>
-      <c r="K63" s="260"/>
-      <c r="L63" s="261"/>
+      <c r="J63" s="333"/>
+      <c r="K63" s="334"/>
+      <c r="L63" s="335"/>
       <c r="R63" s="164" t="s">
         <v>354</v>
       </c>
       <c r="S63" s="162" t="s">
         <v>308</v>
       </c>
-      <c r="T63" s="276"/>
-      <c r="U63" s="210"/>
-      <c r="V63" s="211"/>
-    </row>
-    <row r="64" spans="2:29" ht="40.5" customHeight="1">
+      <c r="T63" s="344"/>
+      <c r="U63" s="233"/>
+      <c r="V63" s="234"/>
+    </row>
+    <row r="64" spans="2:29" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="82">
         <v>8</v>
       </c>
       <c r="C64" s="85"/>
-      <c r="D64" s="277"/>
-      <c r="E64" s="271"/>
-    </row>
-    <row r="65" spans="2:5">
+      <c r="D64" s="304"/>
+      <c r="E64" s="305"/>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="82">
         <v>9</v>
       </c>
       <c r="C65" s="85"/>
-      <c r="D65" s="277"/>
-      <c r="E65" s="271"/>
-    </row>
-    <row r="66" spans="2:5" ht="30" customHeight="1">
+      <c r="D65" s="304"/>
+      <c r="E65" s="305"/>
+    </row>
+    <row r="66" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="82">
         <v>10</v>
       </c>
       <c r="C66" s="85"/>
-      <c r="D66" s="277"/>
-      <c r="E66" s="271"/>
-    </row>
-    <row r="67" spans="2:5">
+      <c r="D66" s="304"/>
+      <c r="E66" s="305"/>
+    </row>
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" s="82">
         <v>11</v>
       </c>
       <c r="C67" s="85"/>
-      <c r="D67" s="277"/>
-      <c r="E67" s="271"/>
-    </row>
-    <row r="68" spans="2:5">
+      <c r="D67" s="304"/>
+      <c r="E67" s="305"/>
+    </row>
+    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" s="82">
         <v>12</v>
       </c>
       <c r="C68" s="85"/>
-      <c r="D68" s="277"/>
-      <c r="E68" s="271"/>
-    </row>
-    <row r="69" spans="2:5">
+      <c r="D68" s="304"/>
+      <c r="E68" s="305"/>
+    </row>
+    <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69" s="82">
         <v>13</v>
       </c>
       <c r="C69" s="85"/>
-      <c r="D69" s="277"/>
-      <c r="E69" s="271"/>
-    </row>
-    <row r="70" spans="2:5" ht="30" customHeight="1">
+      <c r="D69" s="304"/>
+      <c r="E69" s="305"/>
+    </row>
+    <row r="70" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="82">
         <v>14</v>
       </c>
       <c r="C70" s="85"/>
-      <c r="D70" s="277"/>
-      <c r="E70" s="271"/>
-    </row>
-    <row r="71" spans="2:5" ht="15.75" thickBot="1">
+      <c r="D70" s="304"/>
+      <c r="E70" s="305"/>
+    </row>
+    <row r="71" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B71" s="83">
         <v>15</v>
       </c>
       <c r="C71" s="86"/>
-      <c r="D71" s="278"/>
-      <c r="E71" s="279"/>
-    </row>
-    <row r="75" spans="2:5" ht="72" customHeight="1"/>
+      <c r="D71" s="310"/>
+      <c r="E71" s="311"/>
+    </row>
+    <row r="75" spans="2:5" ht="72" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="183">
-    <mergeCell ref="T30:AC30"/>
-    <mergeCell ref="T31:AC31"/>
-    <mergeCell ref="T32:AC32"/>
-    <mergeCell ref="T33:AC33"/>
-    <mergeCell ref="T34:AC34"/>
-    <mergeCell ref="T35:AC35"/>
-    <mergeCell ref="T36:AC36"/>
-    <mergeCell ref="T37:AC37"/>
-    <mergeCell ref="G47:J47"/>
-    <mergeCell ref="S38:S39"/>
-    <mergeCell ref="T38:AC39"/>
-    <mergeCell ref="S44:S45"/>
-    <mergeCell ref="T44:AC45"/>
-    <mergeCell ref="T40:AC40"/>
-    <mergeCell ref="T41:AC41"/>
-    <mergeCell ref="T42:AC42"/>
-    <mergeCell ref="T43:AC43"/>
-    <mergeCell ref="T46:AC46"/>
-    <mergeCell ref="G45:J46"/>
-    <mergeCell ref="G39:J42"/>
+    <mergeCell ref="AA48:AC49"/>
+    <mergeCell ref="M56:N56"/>
+    <mergeCell ref="J54:L55"/>
+    <mergeCell ref="J56:L56"/>
+    <mergeCell ref="J57:L57"/>
+    <mergeCell ref="J58:L58"/>
+    <mergeCell ref="J59:L59"/>
+    <mergeCell ref="J60:L60"/>
+    <mergeCell ref="J61:L61"/>
+    <mergeCell ref="R51:R52"/>
+    <mergeCell ref="S51:S52"/>
+    <mergeCell ref="T51:V52"/>
+    <mergeCell ref="T53:V53"/>
+    <mergeCell ref="T54:V54"/>
+    <mergeCell ref="T55:V55"/>
+    <mergeCell ref="T56:V56"/>
+    <mergeCell ref="T57:V57"/>
+    <mergeCell ref="T58:V58"/>
+    <mergeCell ref="T59:V59"/>
+    <mergeCell ref="T60:V63"/>
+    <mergeCell ref="J62:L62"/>
+    <mergeCell ref="J63:L63"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D54:E55"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="G49:J51"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="H54:H55"/>
+    <mergeCell ref="I54:I55"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="AA7:AB7"/>
+    <mergeCell ref="AA28:AB28"/>
+    <mergeCell ref="AA12:AB12"/>
+    <mergeCell ref="AA13:AB13"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AA25:AB25"/>
+    <mergeCell ref="AA26:AB26"/>
+    <mergeCell ref="U27:V27"/>
+    <mergeCell ref="AA27:AB27"/>
+    <mergeCell ref="U12:V12"/>
+    <mergeCell ref="AA14:AB14"/>
+    <mergeCell ref="U28:V28"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="N20:P20"/>
+    <mergeCell ref="N21:P21"/>
+    <mergeCell ref="N23:P23"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AA4:AB4"/>
+    <mergeCell ref="AA5:AB5"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="AA11:AB11"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="N26:P26"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="N24:P24"/>
+    <mergeCell ref="E27:J27"/>
+    <mergeCell ref="E22:J22"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K2:P2"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AA17:AB17"/>
+    <mergeCell ref="AA18:AB18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="N13:P13"/>
     <mergeCell ref="AA20:AB20"/>
     <mergeCell ref="AA21:AB21"/>
     <mergeCell ref="AA22:AB22"/>
@@ -8264,145 +8382,26 @@
     <mergeCell ref="U11:V11"/>
     <mergeCell ref="AA23:AB23"/>
     <mergeCell ref="AA6:AB6"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AA17:AB17"/>
-    <mergeCell ref="AA18:AB18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="AA19:AB19"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="N28:P28"/>
-    <mergeCell ref="N27:P27"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="E28:J28"/>
-    <mergeCell ref="N24:P24"/>
-    <mergeCell ref="E27:J27"/>
-    <mergeCell ref="E22:J22"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K2:P2"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="R2:R4"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AA4:AB4"/>
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="AA11:AB11"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B52:F52"/>
-    <mergeCell ref="AA7:AB7"/>
-    <mergeCell ref="AA28:AB28"/>
-    <mergeCell ref="AA12:AB12"/>
-    <mergeCell ref="AA13:AB13"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AA25:AB25"/>
-    <mergeCell ref="AA26:AB26"/>
-    <mergeCell ref="U27:V27"/>
-    <mergeCell ref="AA27:AB27"/>
-    <mergeCell ref="U12:V12"/>
-    <mergeCell ref="AA14:AB14"/>
-    <mergeCell ref="U28:V28"/>
-    <mergeCell ref="N17:P17"/>
-    <mergeCell ref="N19:P19"/>
-    <mergeCell ref="N20:P20"/>
-    <mergeCell ref="N21:P21"/>
-    <mergeCell ref="N23:P23"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D54:E55"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="G49:J51"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="F57:G57"/>
-    <mergeCell ref="H54:H55"/>
-    <mergeCell ref="I54:I55"/>
-    <mergeCell ref="AA48:AC49"/>
-    <mergeCell ref="M56:N56"/>
-    <mergeCell ref="J54:L55"/>
-    <mergeCell ref="J56:L56"/>
-    <mergeCell ref="J57:L57"/>
-    <mergeCell ref="J58:L58"/>
-    <mergeCell ref="J59:L59"/>
-    <mergeCell ref="J60:L60"/>
-    <mergeCell ref="J61:L61"/>
-    <mergeCell ref="R51:R52"/>
-    <mergeCell ref="S51:S52"/>
-    <mergeCell ref="T51:V52"/>
-    <mergeCell ref="T53:V53"/>
-    <mergeCell ref="T54:V54"/>
-    <mergeCell ref="T55:V55"/>
-    <mergeCell ref="T56:V56"/>
-    <mergeCell ref="T57:V57"/>
-    <mergeCell ref="T58:V58"/>
-    <mergeCell ref="T59:V59"/>
-    <mergeCell ref="T60:V63"/>
-    <mergeCell ref="J62:L62"/>
-    <mergeCell ref="J63:L63"/>
+    <mergeCell ref="T30:AC30"/>
+    <mergeCell ref="T31:AC31"/>
+    <mergeCell ref="T32:AC32"/>
+    <mergeCell ref="T33:AC33"/>
+    <mergeCell ref="T34:AC34"/>
+    <mergeCell ref="T35:AC35"/>
+    <mergeCell ref="T36:AC36"/>
+    <mergeCell ref="T37:AC37"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="S38:S39"/>
+    <mergeCell ref="T38:AC39"/>
+    <mergeCell ref="S44:S45"/>
+    <mergeCell ref="T44:AC45"/>
+    <mergeCell ref="T40:AC40"/>
+    <mergeCell ref="T41:AC41"/>
+    <mergeCell ref="T42:AC42"/>
+    <mergeCell ref="T43:AC43"/>
+    <mergeCell ref="T46:AC46"/>
+    <mergeCell ref="G45:J46"/>
+    <mergeCell ref="G39:J42"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8417,7 +8416,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CBBBEA-E421-4197-9F44-CA2E8EC0215F}">
   <dimension ref="B1:AB33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
@@ -8439,8 +8438,8 @@
     <col min="26" max="28" width="7.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" ht="15.75" thickBot="1"/>
-    <row r="2" spans="2:28" ht="45" customHeight="1" thickBot="1">
+    <row r="1" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:28" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="194" t="s">
         <v>358</v>
       </c>
@@ -8456,37 +8455,37 @@
       <c r="F2" s="188" t="s">
         <v>361</v>
       </c>
-      <c r="G2" s="224" t="s">
+      <c r="G2" s="215" t="s">
         <v>171</v>
       </c>
-      <c r="H2" s="224"/>
-      <c r="I2" s="224"/>
-      <c r="J2" s="225"/>
-      <c r="L2" s="215" t="s">
+      <c r="H2" s="215"/>
+      <c r="I2" s="215"/>
+      <c r="J2" s="216"/>
+      <c r="L2" s="238" t="s">
         <v>276</v>
       </c>
-      <c r="M2" s="216"/>
-      <c r="N2" s="216"/>
-      <c r="O2" s="217"/>
+      <c r="M2" s="239"/>
+      <c r="N2" s="239"/>
+      <c r="O2" s="240"/>
       <c r="P2" s="114"/>
-      <c r="Q2" s="218" t="s">
+      <c r="Q2" s="241" t="s">
         <v>238</v>
       </c>
-      <c r="R2" s="219"/>
-      <c r="S2" s="219"/>
-      <c r="T2" s="220"/>
+      <c r="R2" s="242"/>
+      <c r="S2" s="242"/>
+      <c r="T2" s="243"/>
       <c r="U2" s="114"/>
-      <c r="V2" s="212" t="s">
+      <c r="V2" s="235" t="s">
         <v>261</v>
       </c>
-      <c r="W2" s="213"/>
-      <c r="X2" s="213"/>
-      <c r="Y2" s="213"/>
-      <c r="Z2" s="213"/>
-      <c r="AA2" s="213"/>
-      <c r="AB2" s="214"/>
-    </row>
-    <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
+      <c r="W2" s="236"/>
+      <c r="X2" s="236"/>
+      <c r="Y2" s="236"/>
+      <c r="Z2" s="236"/>
+      <c r="AA2" s="236"/>
+      <c r="AB2" s="237"/>
+    </row>
+    <row r="3" spans="2:28" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="195" t="s">
         <v>362</v>
       </c>
@@ -8505,11 +8504,11 @@
       <c r="G3" s="88" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="232" t="s">
+      <c r="H3" s="223" t="s">
         <v>176</v>
       </c>
-      <c r="I3" s="233"/>
-      <c r="J3" s="234"/>
+      <c r="I3" s="224"/>
+      <c r="J3" s="225"/>
       <c r="L3" s="126" t="s">
         <v>224</v>
       </c>
@@ -8548,13 +8547,13 @@
       <c r="Y3" s="152" t="s">
         <v>227</v>
       </c>
-      <c r="Z3" s="203" t="s">
+      <c r="Z3" s="226" t="s">
         <v>266</v>
       </c>
-      <c r="AA3" s="204"/>
-      <c r="AB3" s="205"/>
-    </row>
-    <row r="4" spans="2:28" ht="53.25" customHeight="1">
+      <c r="AA3" s="227"/>
+      <c r="AB3" s="228"/>
+    </row>
+    <row r="4" spans="2:28" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="196" t="s">
         <v>367</v>
       </c>
@@ -8573,11 +8572,11 @@
       <c r="G4" s="89" t="s">
         <v>173</v>
       </c>
-      <c r="H4" s="229">
+      <c r="H4" s="220">
         <v>63</v>
       </c>
-      <c r="I4" s="230"/>
-      <c r="J4" s="231"/>
+      <c r="I4" s="221"/>
+      <c r="J4" s="222"/>
       <c r="L4" s="132" t="s">
         <v>195</v>
       </c>
@@ -8616,13 +8615,13 @@
       <c r="Y4" s="119" t="s">
         <v>264</v>
       </c>
-      <c r="Z4" s="206" t="s">
+      <c r="Z4" s="229" t="s">
         <v>424</v>
       </c>
-      <c r="AA4" s="207"/>
-      <c r="AB4" s="208"/>
-    </row>
-    <row r="5" spans="2:28" ht="47.25" customHeight="1">
+      <c r="AA4" s="230"/>
+      <c r="AB4" s="231"/>
+    </row>
+    <row r="5" spans="2:28" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="197" t="s">
         <v>372</v>
       </c>
@@ -8641,11 +8640,11 @@
       <c r="G5" s="89" t="s">
         <v>174</v>
       </c>
-      <c r="H5" s="229">
+      <c r="H5" s="220">
         <v>31</v>
       </c>
-      <c r="I5" s="230"/>
-      <c r="J5" s="231"/>
+      <c r="I5" s="221"/>
+      <c r="J5" s="222"/>
       <c r="L5" s="130" t="s">
         <v>204</v>
       </c>
@@ -8684,11 +8683,11 @@
       <c r="Y5" s="116" t="s">
         <v>241</v>
       </c>
-      <c r="Z5" s="206"/>
-      <c r="AA5" s="207"/>
-      <c r="AB5" s="208"/>
-    </row>
-    <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
+      <c r="Z5" s="229"/>
+      <c r="AA5" s="230"/>
+      <c r="AB5" s="231"/>
+    </row>
+    <row r="6" spans="2:28" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="196" t="s">
         <v>376</v>
       </c>
@@ -8707,11 +8706,11 @@
       <c r="G6" s="90" t="s">
         <v>175</v>
       </c>
-      <c r="H6" s="226">
+      <c r="H6" s="217">
         <v>7</v>
       </c>
-      <c r="I6" s="227"/>
-      <c r="J6" s="228"/>
+      <c r="I6" s="218"/>
+      <c r="J6" s="219"/>
       <c r="L6" s="133" t="s">
         <v>190</v>
       </c>
@@ -8750,11 +8749,11 @@
       <c r="Y6" s="125" t="s">
         <v>263</v>
       </c>
-      <c r="Z6" s="209"/>
-      <c r="AA6" s="210"/>
-      <c r="AB6" s="211"/>
-    </row>
-    <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1">
+      <c r="Z6" s="232"/>
+      <c r="AA6" s="233"/>
+      <c r="AB6" s="234"/>
+    </row>
+    <row r="7" spans="2:28" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="197" t="s">
         <v>380</v>
       </c>
@@ -8773,12 +8772,12 @@
       <c r="G7" s="87" t="s">
         <v>223</v>
       </c>
-      <c r="H7" s="221" t="str">
+      <c r="H7" s="212" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12))</f>
         <v>E3FFF000</v>
       </c>
-      <c r="I7" s="222"/>
-      <c r="J7" s="223"/>
+      <c r="I7" s="213"/>
+      <c r="J7" s="214"/>
       <c r="L7" s="131" t="s">
         <v>190</v>
       </c>
@@ -8805,9 +8804,8 @@
         <v>239</v>
       </c>
       <c r="U7" s="114"/>
-      <c r="Z7" s="345"/>
-    </row>
-    <row r="8" spans="2:28" ht="43.5" customHeight="1" thickBot="1">
+    </row>
+    <row r="8" spans="2:28" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="196" t="s">
         <v>384</v>
       </c>
@@ -8826,18 +8824,18 @@
       <c r="G8" s="87" t="s">
         <v>177</v>
       </c>
-      <c r="H8" s="221" t="str">
+      <c r="H8" s="212" t="str">
         <f>DEC2HEX(HEX2DEC($H$3)+_xlfn.BITLSHIFT(H4,20)+_xlfn.BITLSHIFT(H5,15)+_xlfn.BITLSHIFT(H6,12)+4095)</f>
         <v>E3FFFFFF</v>
       </c>
-      <c r="I8" s="222"/>
-      <c r="J8" s="223"/>
-      <c r="L8" s="238" t="s">
+      <c r="I8" s="213"/>
+      <c r="J8" s="214"/>
+      <c r="L8" s="206" t="s">
         <v>420</v>
       </c>
-      <c r="M8" s="239"/>
-      <c r="N8" s="239"/>
-      <c r="O8" s="240"/>
+      <c r="M8" s="207"/>
+      <c r="N8" s="207"/>
+      <c r="O8" s="208"/>
       <c r="P8" s="114"/>
       <c r="Q8" s="145" t="s">
         <v>233</v>
@@ -8856,7 +8854,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="9" spans="2:28" ht="65.25" customHeight="1" thickBot="1">
+    <row r="9" spans="2:28" ht="65.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="196" t="s">
         <v>388</v>
       </c>
@@ -8891,7 +8889,7 @@
       </c>
       <c r="U9" s="114"/>
     </row>
-    <row r="10" spans="2:28" ht="76.5" customHeight="1" thickBot="1">
+    <row r="10" spans="2:28" ht="76.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="196" t="s">
         <v>393</v>
       </c>
@@ -8918,7 +8916,7 @@
       <c r="P10" s="114"/>
       <c r="U10" s="114"/>
     </row>
-    <row r="11" spans="2:28" ht="74.25" customHeight="1" thickBot="1">
+    <row r="11" spans="2:28" ht="74.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="196" t="s">
         <v>397</v>
       </c>
@@ -8943,15 +8941,15 @@
       <c r="N11" s="114"/>
       <c r="O11" s="114"/>
       <c r="P11" s="114"/>
-      <c r="Q11" s="235" t="s">
+      <c r="Q11" s="203" t="s">
         <v>260</v>
       </c>
-      <c r="R11" s="236"/>
-      <c r="S11" s="236"/>
-      <c r="T11" s="237"/>
+      <c r="R11" s="204"/>
+      <c r="S11" s="204"/>
+      <c r="T11" s="205"/>
       <c r="U11" s="114"/>
     </row>
-    <row r="12" spans="2:28" ht="47.25" customHeight="1" thickBot="1">
+    <row r="12" spans="2:28" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="196" t="s">
         <v>401</v>
       </c>
@@ -8988,7 +8986,7 @@
       </c>
       <c r="U12" s="114"/>
     </row>
-    <row r="13" spans="2:28" ht="47.25" customHeight="1">
+    <row r="13" spans="2:28" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="196" t="s">
         <v>404</v>
       </c>
@@ -9025,7 +9023,7 @@
       </c>
       <c r="U13" s="114"/>
     </row>
-    <row r="14" spans="2:28" ht="47.25" customHeight="1">
+    <row r="14" spans="2:28" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="196" t="s">
         <v>407</v>
       </c>
@@ -9062,7 +9060,7 @@
       </c>
       <c r="U14" s="114"/>
     </row>
-    <row r="15" spans="2:28" ht="69" customHeight="1">
+    <row r="15" spans="2:28" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="196" t="s">
         <v>410</v>
       </c>
@@ -9099,7 +9097,7 @@
       </c>
       <c r="U15" s="114"/>
     </row>
-    <row r="16" spans="2:28" ht="62.25" customHeight="1">
+    <row r="16" spans="2:28" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="196" t="s">
         <v>413</v>
       </c>
@@ -9126,7 +9124,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="17" spans="2:20" ht="69.75" customHeight="1" thickBot="1">
+    <row r="17" spans="2:20" ht="69.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="198" t="s">
         <v>416</v>
       </c>
@@ -9153,8 +9151,8 @@
         <v>259</v>
       </c>
     </row>
-    <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1"/>
-    <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+    <row r="18" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="102" t="s">
         <v>178</v>
       </c>
@@ -9170,14 +9168,14 @@
       <c r="F19" s="105" t="s">
         <v>182</v>
       </c>
-      <c r="G19" s="241" t="s">
+      <c r="G19" s="209" t="s">
         <v>220</v>
       </c>
-      <c r="H19" s="242"/>
-      <c r="I19" s="242"/>
-      <c r="J19" s="243"/>
-    </row>
-    <row r="20" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+      <c r="H19" s="210"/>
+      <c r="I19" s="210"/>
+      <c r="J19" s="211"/>
+    </row>
+    <row r="20" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="170" t="s">
         <v>183</v>
       </c>
@@ -9200,7 +9198,7 @@
       <c r="I20" s="175"/>
       <c r="J20" s="176"/>
     </row>
-    <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+    <row r="21" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="177"/>
       <c r="C21" s="178"/>
       <c r="D21" s="94" t="s">
@@ -9219,7 +9217,7 @@
       <c r="I21" s="172"/>
       <c r="J21" s="173"/>
     </row>
-    <row r="22" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+    <row r="22" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="171"/>
       <c r="C22" s="169"/>
       <c r="D22" s="99" t="s">
@@ -9236,7 +9234,7 @@
       <c r="I22" s="15"/>
       <c r="J22" s="15"/>
     </row>
-    <row r="23" spans="2:20" ht="51.75" customHeight="1">
+    <row r="23" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="170" t="s">
         <v>193</v>
       </c>
@@ -9257,7 +9255,7 @@
       <c r="I23" s="15"/>
       <c r="J23" s="15"/>
     </row>
-    <row r="24" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+    <row r="24" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="171"/>
       <c r="C24" s="169"/>
       <c r="D24" s="99" t="s">
@@ -9274,7 +9272,7 @@
       <c r="I24" s="15"/>
       <c r="J24" s="15"/>
     </row>
-    <row r="25" spans="2:20" ht="51.75" customHeight="1">
+    <row r="25" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="170" t="s">
         <v>199</v>
       </c>
@@ -9295,7 +9293,7 @@
       <c r="I25" s="15"/>
       <c r="J25" s="15"/>
     </row>
-    <row r="26" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+    <row r="26" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="171"/>
       <c r="C26" s="169"/>
       <c r="D26" s="99" t="s">
@@ -9312,7 +9310,7 @@
       <c r="I26" s="15"/>
       <c r="J26" s="15"/>
     </row>
-    <row r="27" spans="2:20" ht="51.75" customHeight="1">
+    <row r="27" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="170" t="s">
         <v>204</v>
       </c>
@@ -9333,7 +9331,7 @@
       <c r="I27" s="15"/>
       <c r="J27" s="15"/>
     </row>
-    <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+    <row r="28" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="171"/>
       <c r="C28" s="169"/>
       <c r="D28" s="99" t="s">
@@ -9350,7 +9348,7 @@
       <c r="I28" s="15"/>
       <c r="J28" s="15"/>
     </row>
-    <row r="29" spans="2:20" ht="51.75" customHeight="1" thickBot="1">
+    <row r="29" spans="2:20" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="113" t="s">
         <v>208</v>
       </c>
@@ -9371,7 +9369,7 @@
       <c r="I29" s="15"/>
       <c r="J29" s="15"/>
     </row>
-    <row r="30" spans="2:20" ht="51.75" customHeight="1">
+    <row r="30" spans="2:20" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="170" t="s">
         <v>187</v>
       </c>
@@ -9392,7 +9390,7 @@
       <c r="I30" s="15"/>
       <c r="J30" s="15"/>
     </row>
-    <row r="31" spans="2:20" ht="45.75" thickBot="1">
+    <row r="31" spans="2:20" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="171"/>
       <c r="C31" s="169"/>
       <c r="D31" s="99" t="s">
@@ -9409,7 +9407,7 @@
       <c r="I31" s="15"/>
       <c r="J31" s="15"/>
     </row>
-    <row r="32" spans="2:20" ht="30">
+    <row r="32" spans="2:20" ht="30" x14ac:dyDescent="0.25">
       <c r="B32" s="170" t="s">
         <v>215</v>
       </c>
@@ -9430,7 +9428,7 @@
       <c r="I32" s="15"/>
       <c r="J32" s="15"/>
     </row>
-    <row r="33" spans="2:10" ht="57.75" thickBot="1">
+    <row r="33" spans="2:10" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="171"/>
       <c r="C33" s="169"/>
       <c r="D33" s="99" t="s">
@@ -9449,6 +9447,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="Z4:AB6"/>
+    <mergeCell ref="V2:AB2"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="Q2:T2"/>
     <mergeCell ref="Q11:T11"/>
     <mergeCell ref="L8:O8"/>
     <mergeCell ref="G19:J19"/>
@@ -9459,11 +9462,6 @@
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="H7:J7"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="Z4:AB6"/>
-    <mergeCell ref="V2:AB2"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="Q2:T2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>